<commit_message>
Update news log — 2026-03-24
</commit_message>
<xml_diff>
--- a/news_log.xlsx
+++ b/news_log.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -87,6 +87,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -453,8 +456,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
@@ -580,6 +583,34 @@
       </c>
       <c r="F4" s="3" t="inlineStr"/>
     </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update news log — 2026-03-25
</commit_message>
<xml_diff>
--- a/news_log.xlsx
+++ b/news_log.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -87,6 +87,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -474,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -518,7 +521,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -528,17 +531,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E2" s="9" t="inlineStr">
+      <c r="E2" s="10" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -546,7 +549,7 @@
       <c r="F2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -556,17 +559,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="10" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -574,7 +577,7 @@
       <c r="F3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -584,17 +587,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -602,7 +605,7 @@
       <c r="F4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -612,17 +615,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -630,7 +633,7 @@
       <c r="F5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -640,17 +643,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -658,7 +661,7 @@
       <c r="F6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -668,17 +671,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -686,7 +689,7 @@
       <c r="F7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -696,17 +699,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -714,7 +717,7 @@
       <c r="F8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -724,17 +727,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -742,7 +745,7 @@
       <c r="F9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -752,17 +755,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -770,7 +773,7 @@
       <c r="F10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -780,17 +783,17 @@
           <t>Zarraffa’s Coffee celebrates 30 years, eyes nationwide growth</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOcXNzUkRLemZEOWtOZjhvRUtzcUZrSTdzV0s0LUJTd2NGRk1Gb1NSLUR5Rlh3NUdWQUJkVWctb0toUFBRajlMcWV3VnNyTUtydy1PSUoyb1NCOGVtMUZqRVN0MzFkVkNlOUZNVXlHN2kzREhSdWJQUnJqa0pnUzExTVZSc1NCVFZSNlBSUWNfWnZ3MC01aUx0UWF5SkNOaHI3ZkE?oc=5</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -798,7 +801,7 @@
       <c r="F11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -808,17 +811,17 @@
           <t>Zarraffa’s Coffee eyes 200 outlets ahead of 2032 Olympics</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPMUFjRTlGVFBqYzlPWXdzQ0dKVVlhWGxncUQxTDd1R0VHcThlV3ExVmo4SlBGSHVuUGZrMGNqSVo1YVpDWHViMm5KZWIxcHNMMHo0b1FQcmxUNElDR2lEeWRuLWZIN2lyQUV0VndEUWNkNU42Z3AzNXRlbm50NzhtTXZ0Q245dF9hNzBxOENuMXZsVlU4Z0JGVElR?oc=5</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -826,7 +829,7 @@
       <c r="F12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -836,17 +839,17 @@
           <t>Aware Super appoints new head of private equity</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNVHJXNWEtdEZZUW1fZzdYMTB4RklBTUh6dUNKQ3BrTlpYUnBwRURIVGZjWTV0OUxScnhGMVNSczhLUjVqOEwzbkR2WWlEbmF4ZkNUdHNQY0J1djI0REctbHd2SVhUNlNCa2M5bFhOQ0JPU0RHOVVTQkEzRDdGMjRZbVFDOUdlTXNNczlmZWF6bXlfbEFGRE0xbkZQaw?oc=5</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -854,7 +857,7 @@
       <c r="F13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -864,17 +867,17 @@
           <t>Commission wrinkle over UP Education sale</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxNSV9GMjhqM2ZSanI2X0w2OVlQVFRQTUoxYzAxaXVZMmU1REVTcHlUeEltdXJtaXZrcUJWdDZxNGpYTTZYSFE2TkZHeG9OaVRZakoxV0s1U01TVjJpWlhaSENfNVhucG5NVzFMbTVBY25zWGRSODBtRGtkS1owVTlJWnNfcTJ5alFnbVl1SU9aUDF1QWxJLTBSQ3kxUUFlZnpJMlVEQndFSGRGbDF6WVBUVHlCcDM5Qnh3R2xBMG9xN2FLckNzbUFOWDI1aVF1YV90d0twd0ZmMnUySDBMdG1R0gHkAUFVX3lxTE5EWVp6VzZWb01TRmlHSS0wMExldkJwSHJjdlZXdElsRlpBTEtVMkd6VzNQa1RpVDNsOFQzaGZ2VHpzUnBDYk82RmZGQWJuTmVQMXhxLXVmdVFxTVZOZTBsOHZ0V3cyVVVkNWUwVUxSc0xNSU92ZktpdFRfYnQ4WHBTX3A5bFhXZ1YwZXNrc1BSZEU4LVYybnNBd0dCdk92OFUwclJCMzdoU0ctX1pEdTAwY0JiTWQ4S01QRE00TW5EUEJwR2YtczZ0T005bTJnN1RDY2p6NFF1SndfLUo4QzJUWk1tRg?oc=5</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -882,7 +885,7 @@
       <c r="F14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -892,17 +895,17 @@
           <t>Gloria Jean’s owner has an angry shareholder on its case</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPTnZwUVBCdTFJZWkwc0YtVmJqMkNPcUR5RktjMlVURmhROFZkYUpXM01iRUh3SnJEUElxRGlSNk9DQjZSdTdNdmZwWWpONjlmR1hoMl92cUNmd3M4cnJhVkNqc095MmN6WXBYUmdEblB0eERtVDdlUU4yNGFjXzVnT19rOERIRzVPNzY3VDNNRS1tVGVTX3pKMVRpTXZVR1ROLURBLWtJbVZhY0lSU09DNkE2NzFLbEFU?oc=5</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -910,7 +913,7 @@
       <c r="F15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -920,17 +923,17 @@
           <t>Oporto-owner Craveable Brands hires new CEO from Domino’s</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNNmxfQVc2Umc4QWwzSTdsZTFvejRzTzZxXy1ScGlhXzh6bm5JS3IyX0xTNDVBNjh0cXpPbGhxNU5xUHhQN3EtRF9aV3FEc2JoSG5QTU1WeU1TLUJfZzVUT2N6dXloQXhZaHB5djB3dDFKN1llVmI3UVpKNjJTNlcyV0ZDcG9GdVdSdW41ZkN1b1N3SFFIUzcwRkQ3UHY2TmxERmZwTlA0RzU?oc=5</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -938,7 +941,7 @@
       <c r="F16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -948,17 +951,17 @@
           <t>Brookfield, BGH Capital rub shoulders in ScotPac’s data room</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPMVlxbzlQNnFXWnJFNU11Y1BhTTVqbjN4RG1nbkZuN0pkdDFFaUhJN0RaVnUtWDlZSGJWR1ozQXk5UUx6RVdOcjBPU2t5UzN4T0JvUFJISnNvVWxQemd3blNHZjRQVVVZQk1nZER0Y0JfY3VvQ0t1a09sM1RTS2c1YTJyUmdzYWh1WGRUNjl2dkdzYTJJeHVhMTdqR3Y5WVlHVEtSZHp1cmVYYmM?oc=5</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -966,7 +969,7 @@
       <c r="F17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -976,17 +979,17 @@
           <t>Payments player Pay.com.au hits the road(show) for $850m IPO</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOMFZleXZrbU53TzBlakI2ZmJKTjlrN3BoQlRaWjQ5cXFzTllKWmFoRm1UT2xDUHBtNC1QNTNiX1BwSzllMkRZdHIzRlAteDREaUczN1JTNTByTW1jNnR3d2NnR0RxUDBxeHYyWU1CSUs5MEZad2JqSGF6ZUxHZUNtZmFQaTJZZVJVZ1B4MkZ6V09QMWIxaUNHQmVzTDhvWVA1Ty1UbHgtQnRrQQ?oc=5</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -994,7 +997,7 @@
       <c r="F18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1004,17 +1007,17 @@
           <t>Another year, another IPO cold shower for investors</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNeEhzYzQzdjR5MDJCWkd6Q2VLdEZzbzRoWnNOcXFlQjNfMlV4Q0NQRjExMlNhT2NPcnRBbW1sZUkteXo4N0dGaHNNeGZJOEZ2aXFvdmZiN2V2QzdOMzFteFRnY1RVRm1rQXltWmY5VFZOdFVNNVpudVp1dTlrcFM5b1k5SmlWQllDMVFXSjA4ZVpSZHgtV2JpWDJ4SkFRbVE?oc=5</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E19" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1022,7 +1025,7 @@
       <c r="F19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1032,17 +1035,17 @@
           <t>Priceline Pharmacy franchisee sale narrows to final four bidders</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNR294am9sYWNiQ3FVT1B6YlV5ejMyeHAyT0FibTFVbU5pcjZyaVRyazEzbFkxd0lrcnpZNGpTYUx4Ykl1Xy1sZF93M2Nid19ydUFwbUJ3ZHozaURaNkRoOE9OMnRBRGZfQVdCVWZCaVhhNnZSRjlwYUdDVnp2WU9HUkJxbE1QMV8zdWxYRTNBQWktR0xSOFU4dmtXZWk0am9SSU92NWp6QUZmTVU5TzJEOEJNak5fQUtN?oc=5</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1050,7 +1053,7 @@
       <c r="F20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1060,17 +1063,17 @@
           <t>Private equity gets better image of Qscan</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D21" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxPRjVmT0hDRjZLblB1VHdPRmRGeXhKdDJHdWxDTzV4RDZ0VzdHaUFfOVlnZjRQMWhKcWMxby1oRDR6N2lQZkI1UDE1REppS3c4LTVmU3p5b2wtblRCWnhNajFnZGNHaGRJUHFMUGRtTHAyQmIxOHhNNTgwRWVSeWp6ZWRxbUY0WVhiUnhMRUpDLXNwS1RuelJldTk0Z1R0WHg0XzNXNTA5Rk5TRFZhU1RNVnN2TlZuaFE4OWtIYXQ5a2VGSW1UWmt5Rlc4Q2lIXzF3YlkwNVhfUzJDV0dQdVAxa2RKc08wRGR6TlB2Vi14QV9BdlhyaTZsM2pEVGZycTjSAYQCQVVfeXFMTWpnb0lWQmZ6MTFnRGhWNTNqczk1TWhTcUFEMVpDNnJ4ZWVxVlRUODhJXy03NHdGZVJlMmhyUHM0Nlh4NlZtTzRhQ0xxRDFLVHNzUVNfbWxhS3BLUEQteEMzZHRrc0F1eFRzYmxVNDZlSURyZDB5bF9wQTNRRU5yZEs1Z3pFRTdwcFBaMkNlN0JvT1NEYkFWVUJNcHJqcEM5RVJYa0JFUVl6cThyQXloaERzQjhkTUVPakJqb0hzNVlwSWxNS0dmZkNFSG9Gb3dNUnVvUnV0d3MxSmpzdFZKTHJ2RTQwRUoyMEVLLWMwT1NnOHdXVl9lRXNDWEFndzJFSDlZU0o?oc=5</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1078,7 +1081,7 @@
       <c r="F21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1088,17 +1091,17 @@
           <t>Oporto CEO’s first year reshapes brand and network strategy</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D22" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPY25mNTJfT3FiVlBPZE5CcVNkR1UzR2xWaUtJSmxhU3EwcEMzQi1ISDFSajlCQWk1UUJpZVJ1Q19ZV3Jjd0Noc0l3OExpMXhSQUVVdHhCLTBlOXNoZzA3UXZBdkR1VHBvMmVsZkNhUFJndm1DdGpnX2w0ZVViU2phZ1RmYXY1SlhwUnhKSUxBQVZZUXpqNHQxQmo0Rk1iV0g0OW9qUS16eWRSNW5FaW1yQQ?oc=5</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="E22" s="10" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1106,7 +1109,7 @@
       <c r="F22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1116,17 +1119,17 @@
           <t>The Melbourne restaurant our reviewer grew to love</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOc3YxQTljcHJXVWtRX2ZGM2lpM2pILWNwSFg0MFJrNmNWX0ZxRG9nV0J5N19qRWh4U0hPXzNmVVZwWk9wT2kzaFNrTlV3NEQ1Q3JpaXVIYlBHb216Q3VYVWdSRXMwdDl0SmYzdnRlSDFUYVRmRGJyZVlRZDJKTHpJOUctYlF1RDZSYjloY0hfZy13QmFTLU9UNjkwTHc1bjlGcGxoZ0ZLVU1GWTctZkdLZU9zSGhEZEpKbXJnaWJfZjd2OWs3?oc=5</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1134,7 +1137,7 @@
       <c r="F23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1144,17 +1147,17 @@
           <t>Crescent Capital strikes Benson Radiology deal for close to $400m</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C24" s="10" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOLTNrWG1ZZlFoU3pDZ3E2SEgwMlhzQkdtQUYzaHZTZmYwU3ZhMnE0dlkza005VkZmZ09NMExlWDVncnBmYVVISXJ6X1ZjNHhpM2RnSlprY1dnbndJNUczcDVtNXNRY3pVNW12bm5rUVdqVmR4R0JlVHFuN0RwTlFkR2xrbFFpSl9jcm5oSjk3aFM1clBSVDhnbkhoWUREeUhsbVpvQW90d05xOTdfOV9nbW5POFdmelJkVlpsUlRuYl9odmRNVUV2S0pCMFBMTS0tcVhGVGFYU0h2d9IB3wFBVV95cUxPWEs4R2pxdThPbHJHb0dBT183SkRHTTlXNzdWazcxdkd1eGx2VlAyM2VVbEtEbWxTZ1R0TlBFRmRMZTFoalgxSmVVRUJFR0c0RFYzZVJFODg3dWxicU9pOHppeFhjaVp0WWlyTnUzV1dyZXdkMHBDVHI4LUVQdjc0cWpheU55NTlvdWdCZmVoODB0Mm5fbGNCTmQwLUhMZ0psQVpzb3BEUnJpSkRnOUM0c0VCdUp5N3g5MkhaM01vTHJ3NWd0ay02UXZUUG9nVkxicVc1Z0xjWGhjUDRDVjlN?oc=5</t>
         </is>
       </c>
-      <c r="E24" s="9" t="inlineStr">
+      <c r="E24" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1162,7 +1165,7 @@
       <c r="F24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1172,17 +1175,17 @@
           <t>Dual-listed giant Capstone Copper flirts with $600m-plus carve-out</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNcVh4blRkQnoyaG1TajhVV0lrOEJRaHdTZWtzUnJHaEdaSXNRWThGTHlVdGl4dGJ1cTMwZ2pLcVNzUXRYNlZzVzhvaXdkNGtVUG0wN0FrMHB0R1I2Ry1jcEgtSWUtajI0cTFMRTlfdzBuMWtrZmJOLVUtMkl5dW85dFp6dEhEOHhTNzdfOFNFSGtlT0MwQnRlY0VhcUZBNE9RYzhQcDdOQUFnYkgzd0V0N253SQ?oc=5</t>
         </is>
       </c>
-      <c r="E25" s="9" t="inlineStr">
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1190,7 +1193,7 @@
       <c r="F25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="inlineStr">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1200,17 +1203,17 @@
           <t>Guzman y Gomez unveils a new menu under $4</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="C26" s="10" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPMjRjRTV2a3BJc3AzdDNOQktoYjBvLVZSODVsc3lKQ3pET0lxUlpkc05NcVlKRlZITjVJbjkwLS1DUFJNMGJ1amJKTlp3S3VqMWJaU3YtUENEN01rUEJiV1FNZTRXYjcyV08zZzlxNDVOSlVOTlJDOGV3QzBQcUpKa2Zab1ItNlI3ajZVVTF3?oc=5</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="E26" s="10" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1218,7 +1221,7 @@
       <c r="F26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1228,17 +1231,17 @@
           <t>Can Sydney’s burrito king conquer the $676b US fast food market?</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNM0ZFcUpLN1dUZWUyaE1LMnNZVGlEbkNNQUQ4Wmd6QVFlTy0wZDVHdnlja1gzMEZTbVpKU1Ftb3VKZ2pzajcyWU16NUtUTmR0TlZMOVhMRUNqZXZiX2d2NWY0YlJDOFhhYUE0SkhMRUprNndXak8tWGdERU90cmMxTkFjcFFVSTd5VlZ3NFVKOXN3M255MFhzZThmbi1VUGMyQ3E4d2pYcFlJckY3QlVBdVJJeF9qUQ?oc=5</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="E27" s="10" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1246,7 +1249,7 @@
       <c r="F27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="inlineStr">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1256,17 +1259,17 @@
           <t>Drone maker Innovaero prepares for ASX float, taps Euroz Hartleys</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNU3JrejNRZ1VBZVNVV29NMkFPVmRsWE4yMVZPcjk2aUNUTHFJUGFyQ1VnZEZiZlIzQW9VVzRNNDNRR01jcHo3X0tqZjB4bzhMTTI0Y3BwYUh6OGRUUGt2REIxV09oRnJoVWlVelZWaUlWUmlPQ3dJdi1TejcyaXB1Z0x1MEJRSlB3SGMwVGdXaXJJNm9TVllPOG5JZC1feEV3TVhTeExGeHR2RHFIWlVCOXh3?oc=5</t>
         </is>
       </c>
-      <c r="E28" s="9" t="inlineStr">
+      <c r="E28" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1274,7 +1277,7 @@
       <c r="F28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1284,17 +1287,17 @@
           <t>Bain flaunts Estia 2.0 as IPO roadshow gets under way</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNTEN1cGsxNDN2c1NqUzB6UmJ4TFl0NGZjZVN3U3oxMlVFWTF4WUZLQS13dUxMV0N2ek1XN2VURTNVWms1NjdXSm0waEdaTXQwdTdWY1MxZ1V3ZnpEcVJtczdOWGNNZ0RQNzRZLU1MTTgtRW5DZkctbXBGMmVXVXdPZW5pNThiRHEzWnB2eFZzTFZTb1ZkeW9LendkNDd0cXRid05ZSGZYbW9NZXdOLVZWODdZU3hVcTA?oc=5</t>
         </is>
       </c>
-      <c r="E29" s="9" t="inlineStr">
+      <c r="E29" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1302,7 +1305,7 @@
       <c r="F29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="9" t="inlineStr">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1312,17 +1315,17 @@
           <t>Carl’s Jr. Australia unveils nationwide freebies for Happiness Day</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
+      <c r="C30" s="10" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="D30" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNVWgwdjU1NDFWalBfMTFYX1dQOWNDbG1FVUdlcS1LTVlHZVRRTVBWTjhSMnpkTXRXNlFJdllGQUp5Mm5ObWpIazd1d0RJa3QtdFBZN1hOenBmVzBEU05wM0gtNUxPeWpsYkxyVnhWWFFOU2Y3R0tXcmNkeWhpWDh2eDZBdjNCMHhuc1lHYTZHblBPVkpfRXpKd051UWlNc1hm?oc=5</t>
         </is>
       </c>
-      <c r="E30" s="9" t="inlineStr">
+      <c r="E30" s="10" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1330,7 +1333,7 @@
       <c r="F30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="9" t="inlineStr">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1340,17 +1343,17 @@
           <t>BHP and Woodside appoint new CEOs in major mining shake-up</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
+      <c r="C31" s="10" t="inlineStr">
         <is>
           <t>ABC News</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D31" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQbTg5VFJLbWJfcy1uV3ZReTJkTndzX01qZ2MxNWkzaWZRckNLZUR1Y1VsMVRNc2FySC13U0NzalFEb3k1R3BaUEhfcTV0N1M4Q1dpSlo0YXI0UFhrMGRab2RiYV9DQVNVX01ycFc5ZFZrZWZqc1VRZXoxLVEzSDJLclJLSWg5bzN3R1I0bG9lWjVDaHE4?oc=5</t>
         </is>
       </c>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="E31" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1358,7 +1361,7 @@
       <c r="F31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="9" t="inlineStr">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1368,17 +1371,17 @@
           <t>Next Capital sells Enviropacific unit to French waste management giant</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D32" s="9" t="inlineStr">
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPR3lFbERLR2FtdmJUU3BDU2thZk00YmFHRFhXR2VBVXhQSURTeE5ONVJKczBwbzlFMnR5cmhxMnM0bzlJbWo4SXl1dHpqYWxxMUJBRjZHVUtab1RYZjZMTnpGc3FzMWQ2NjNEdGU3NTZwa0diM1lJS1haYllwTldLZlpZbXp0YzlxcDh0ekcwTy03dDdPcnk4b29HZVdqbHhZY2JPR2drM2puSVpjUzZkVjNpZUE4dVMwYlE?oc=5</t>
         </is>
       </c>
-      <c r="E32" s="9" t="inlineStr">
+      <c r="E32" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1386,7 +1389,7 @@
       <c r="F32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="9" t="inlineStr">
+      <c r="A33" s="10" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1396,17 +1399,17 @@
           <t>Future Fund private equity and real assets chiefs head for the door</t>
         </is>
       </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPUHNHRFhFMVdwVld6RFRZUFd3QWNOd1kzeS1QdnJxMERFSnE5LTdZcDhDYlVGcWZMeWxlR0FSRWF6YkZoQVZrZU9TQ1E4YTEydUJnOFE3enV5Rmk5UnF5VEdYZ1FMUWpKVjdjMlZZUGFsU0tKcV9Vbl8zcHp5aVF5Z2JMOUZocHJqRXNRaEp4Nm5CbDM1WkdIMHdQS2xqQnE2Tnh3?oc=5</t>
         </is>
       </c>
-      <c r="E33" s="9" t="inlineStr">
+      <c r="E33" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1414,7 +1417,7 @@
       <c r="F33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="inlineStr">
+      <c r="A34" s="10" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1424,17 +1427,17 @@
           <t>‘I actually started to die’: the new billionaire’s epiphany</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="D34" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxPblkxbHVrdnVKY1pqQzNyWGNMZm9UYmY3dzlPaGQ4Yi1tc0U1akhrVWdIaXBpM05aZXRwTXE1eDBITlZpbDkwRXNrWjJ2YXBzX0VCY2JSLWhrVmpjSTE5eE5rLWgtc2pRZEdXbmhhWU1KeFExZDBGS2pjSkIwV0FGbndBZVAyQkg4WFRsengzSGYyZkFfQnJsQ18tUHJGNDd2T0pzZElPSVJTQkl2Rm5QTExJNHhmU2dHOHJGdTdzU08yNHRtd1R3Q0cyOF8taDktQTZvVXVBVjN1d0NHMmtFOHBWZXBFcUFWa1IyWGNDTDZUT3lQSXJHOVhxTFQ3b3RH0gGGAkFVX3lxTFBZQ3BFQWl5dEwwLW5yVWJuMU8zcXBPdE9pamRVSWVkbWNyVzgydGVOaDBROUN6RlBDbjdld05DVmZyb0R1eEN0UERubzZRU2NiMTQtVV9XNS1wYmlvZ1paM3RaOUlrTzJka0tXVVJEamFESGlSdXg2bDk1aUdhUVhBcXpnN01fX0Y0cTNvcm5DdEFFLVVERDFKTWxKZFR0UzAyblJqVHBua2JoYUdzeUNMb053ZVczWUFQU1AtVHV1d3lSSDFfZFh2cEkxSGw2MEdicEVsb2pLQ1RuQmdaRl9xNUROS3pKR2s2T2wxTTZ5bEwtTUNQNU04djFHTHlPbXVLSW9YSUE?oc=5</t>
         </is>
       </c>
-      <c r="E34" s="9" t="inlineStr">
+      <c r="E34" s="10" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1442,7 +1445,7 @@
       <c r="F34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="inlineStr">
+      <c r="A35" s="10" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1452,17 +1455,17 @@
           <t>Ironbark shuns private equity as it hunts for cash injection</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
+      <c r="C35" s="10" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D35" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxQZWFaeVhldi00VkV5ZmEtS2tjcWdFWG55OGpCX3IyN25Rb3ZFV0ZKVm1aSE1WbThoYVY4ZEdfODVGX0RaUDV2Ul9HS1JQMDFCT05Fc2FaU0RINTMwbDRveWFsOFJSM2ZqTU9tVGxJSEl2ZmhhUHFHT3dqYkk5TUtvMUQySnZzTWw1MzFNWl9aVzhkSEZ4Q3YyWjRMUmpIdmJkdUVKWE54Nkt6bTd2dGFSUFoyNkgxTHh2TGVGak9ja0dFZ0xQM2g0S1lmQkZiWWtUcTVNdHhBdC1KeVRQcDA2dnpmeHRkWEnSAewBQVVfeXFMTWtYRDRSaHNULW1HanowRnpMdFF2VVMtZW1SV2ViZXlGaW02WlIwUzRZMGg5WDNrOUR4eDlGOEt5eGlqV0pfVDFhb0JEcS1faEJodWxyRnB3MkozOVJyT3NvM1I5MzdDcXNnUFNSdkRDamUzZTRQYlk0c1VIQUNMZ2ZzOWVCb2V2MC1aSTZLWkFkbW9GYk05b3RmN1htWENTeDh3SU1WYWJMcWx2eGUzZmwwVXF6czlnRGdXbE1vRElyVG0yM0ZzXzZ5TFh1YlRGNU9MQ1p3NnVZSFB0M0xBcGlueVZILXlVaXdqUkU?oc=5</t>
         </is>
       </c>
-      <c r="E35" s="9" t="inlineStr">
+      <c r="E35" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1470,7 +1473,7 @@
       <c r="F35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="inlineStr">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1480,17 +1483,17 @@
           <t>Minister leaps to fix food chain</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="D36" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxOd2NqakVWRnQ4anFZNkl4Zy03MkloX08tUkktRTZqeEtQWFZJeVhkMUJIb0FxUjc2UjhCQ3MxbmNxczNxblJIZ09IeTBGNFM4Wkh4ZE1qNkhJMjIwU2RtX1JxcEV1Y0NjWXF6eHpVdTN4ZUlYMGIwcDJzMXZMTk94VzFlcjhpcVZVSTJFMjhsQjVGWEJQYTQ3aTFyNmNEZ1F1b3NGTWd5WnFJWmxXSTJ2NlRLcjJHNWkwaTZ2YVR6S0w5WVo1Vlg0VWdxcWZoa3VaTmcxY2NVcnR2bFRWNGNvZ1M2Tlg5NzlvVXZFZm9B0gHzAUFVX3lxTE1uNERoR3p2dXRIa0g0RXI2MWR6N0c5U3NGcjFDQVMtdEpyNDI2bk8yOS1qUnFOazdiODl0Ymo5R1pwRVJ0UFFVdzlhYjRDSUFCU0FRak4xcVVrTHphdTdxcHNIMnEyRVZud1FURmh5T0JLOHpRM3lFbDRuRnZMYmtaRnRFTXh3dkszTFhFUmZlRmoydnlEbW1fZTlmUzh4NXNyeTZTeUhOSktvclJVc0NTZTVYMkdJZEUyY2RmVC1kQ1hwVEloSEtVMEo5QnNTUXQyME5IN1BPd1NOS3oyR1JtMHBFVTZEbzhEQmdrWUk1ZnZVTQ?oc=5</t>
         </is>
       </c>
-      <c r="E36" s="9" t="inlineStr">
+      <c r="E36" s="10" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1498,7 +1501,7 @@
       <c r="F36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="inlineStr">
+      <c r="A37" s="10" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1508,17 +1511,17 @@
           <t>‘Brace for swings on every tweet’: Investors bamboozled by peace talks</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D37" s="9" t="inlineStr">
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOczZHTWFmTW9FZ1ZwSnc5Z3ZacGpsVDQ3LWw1a1BFT0tjRkphek41MlhNOU84emYzZUVwNV9xM0hyc1FUR0NHck14Qnh6c2JvQks5ZE02ZTNLWDI0dy1STi1HbDFDWW9yMDhGQXVVVzdkMzFXcnNNMVZHVXFMUXUteGtsVGhPVmhLcVZPQzlhTWNoYVVRMHF0cFhybWxzek13Y3ZjcjlXWjZJM2VYbm0tTmk4NExLQzQzX1ZPMVlhcnJxQkZx?oc=5</t>
         </is>
       </c>
-      <c r="E37" s="9" t="inlineStr">
+      <c r="E37" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1526,7 +1529,7 @@
       <c r="F37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="inlineStr">
+      <c r="A38" s="10" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1536,17 +1539,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D38" s="9" t="inlineStr">
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5</t>
         </is>
       </c>
-      <c r="E38" s="9" t="inlineStr">
+      <c r="E38" s="10" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1554,7 +1557,7 @@
       <c r="F38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="9" t="inlineStr">
+      <c r="A39" s="10" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1564,17 +1567,17 @@
           <t>Wirth’s Myer rescue mission is caught in the eye of the storm</t>
         </is>
       </c>
-      <c r="C39" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D39" s="9" t="inlineStr">
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNTlQ4NDRnWE91VG1YNENpSTUxNnBjZkljOGdYaGV0aVB5dkVOaEJ6SjZ1bVA4NXE1S1hjV1NjcVhQTEVpWEVNV0UtbzhQTFZLOWxIenZiaF9QM3F6bmJYRy1lbXVMczZ3TnBHNy1aLUtVcnBDdkl4TE0zRGN4U0FwSjNPY1M5S3AtdUQ3UUNmR0x4MlU2YXRuUDJEUm01SmZWakx2UjFvY04zRHk4Smc?oc=5</t>
         </is>
       </c>
-      <c r="E39" s="9" t="inlineStr">
+      <c r="E39" s="10" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1582,7 +1585,7 @@
       <c r="F39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="9" t="inlineStr">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1592,17 +1595,17 @@
           <t>‘Darling, I’m not going anywhere’: The rise of at-home care</t>
         </is>
       </c>
-      <c r="C40" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D40" s="9" t="inlineStr">
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQS2k0M2otaldpNVFXdHRTMVNtZVhyUDV4VTNIcE5FSnFRaHNubGNQQzBVbllnNTktNGhrZ1lndzV5V1FpUS01SklRaTZmZHJkRzVsQmlsdEVmenZ4U2x6U01NeXdIMktBUW94TUE3R3FoLUxVcVhsVFI0SjVQVUFaZldnd3prMWMyaVRWX2J4aUdfQ25KWHpaLUlqSnhvQmM2TTRRQldGbm8tclFYRDA0TVdnU2g3QQ?oc=5</t>
         </is>
       </c>
-      <c r="E40" s="9" t="inlineStr">
+      <c r="E40" s="10" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1610,7 +1613,7 @@
       <c r="F40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="9" t="inlineStr">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1620,17 +1623,17 @@
           <t>Iran targets Israel and Gulf states as Trump looks to calm markets</t>
         </is>
       </c>
-      <c r="C41" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D41" s="9" t="inlineStr">
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPLXBITXU3WTRtc0NYdnhTZHFaUTBCSXdldTBuSHliTlY1dlJONW43Qkd6Nl9pNmY1eDhzaHZoX19xYjBxMXR5UEhkVUg2M2k1MmhuVEwyY0JxbnJyemxVYUZjbk5BbkN4ajhPbW9ZeDhlRDRYTW1hN3k2d084c2djMEJUZTV3NVdPbllKUmFlU2JsaDV3Zk9CVFF0VDFkV09JSloycWdOUlVrREptQTJfa25LUEx5djA2SjNMMFY0RjM?oc=5</t>
         </is>
       </c>
-      <c r="E41" s="9" t="inlineStr">
+      <c r="E41" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1638,7 +1641,7 @@
       <c r="F41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="9" t="inlineStr">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1648,17 +1651,17 @@
           <t>Meet Christian Louboutin, footwear’s most famous billionaire</t>
         </is>
       </c>
-      <c r="C42" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D42" s="9" t="inlineStr">
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPcXdGd0tMckYxbjZ5TVJmQ0Q4NFl2RkhHMHdlZDZsdGZ6cVQ0cUpaLWJTNlVoc2ZOQmtXNlFTRnJVMnVDTGc1NFNZN2g1VnotQlNQbzhlM1BJV3ZwQktOcGtac3RwSHRLZkR0b2l0eGIyVVlYdHJrc2hpT0pJbDR3LURPTnowZk54LThObndtMVkwV2VWQkluNVlWY0p4QVJGbE1hSGMzOW8zdkJZOWdocEZQWFBhTllNR1ZBSEg1TWRXUWd3X0t6TVcyY05PM0pF?oc=5</t>
         </is>
       </c>
-      <c r="E42" s="9" t="inlineStr">
+      <c r="E42" s="10" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1666,7 +1669,7 @@
       <c r="F42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="9" t="inlineStr">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1676,17 +1679,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C43" s="9" t="inlineStr">
+      <c r="C43" s="10" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D43" s="9" t="inlineStr">
+      <c r="D43" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQbHdYM2pSM2xkdmZ3OHhQc2tVUmhzclJWaVJ0aEwtUkNBR0ZUd3p1emF1M21jbTF1ejlKSkdDMnotcVNjZE1CYUlKako3WXR4MTJhdWNlSXZMbTBYanlmTWFzRGFIandXRUQ3UjN6SEV1bThvZjN2bDY0eFdpaTdMODN6TGFTdE5rd05TUll3MmNfTDhkQldoNDIwVlpoSl85aVRwcTd5Ymh3TDl4enZhZ2p4OExGY1ZaOFNEWFBB?oc=5</t>
         </is>
       </c>
-      <c r="E43" s="9" t="inlineStr">
+      <c r="E43" s="10" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1694,7 +1697,7 @@
       <c r="F43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="9" t="inlineStr">
+      <c r="A44" s="10" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1704,17 +1707,17 @@
           <t>Sembcorp Picks Banks for $2 Billion Alinta Loan in Aussie Push</t>
         </is>
       </c>
-      <c r="C44" s="9" t="inlineStr">
+      <c r="C44" s="10" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D44" s="9" t="inlineStr">
+      <c r="D44" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOdS1aaXZjT2VnSDl2TDdzZ3NfRElDWXdUXzZQYjFQMEZJOGlpaE5CNGdQMlZ2UFVHbUtfOXF1ZVBReExrdF85M0RWLWlBY2Y5dlRtWVdXLWp0Y1VrRmF4UGQzVUhxaHA4UHd1SUdFV21QcVFITXFHRlhzekdSUS1PdHlYRjdUbUQydU8wSktKVHRJQ0NaWE9sU1l6YXhtSWtBd3RwTERacnV4VzB6YlFhUE1QcXNDVXVESFcyeWY3cGhHUkRJcDhrYUtpTEY2UQ?oc=5</t>
         </is>
       </c>
-      <c r="E44" s="9" t="inlineStr">
+      <c r="E44" s="10" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1722,7 +1725,7 @@
       <c r="F44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="9" t="inlineStr">
+      <c r="A45" s="10" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1732,17 +1735,17 @@
           <t>Navis targets June for $1bn-plus med-tech auction</t>
         </is>
       </c>
-      <c r="C45" s="9" t="inlineStr">
+      <c r="C45" s="10" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D45" s="9" t="inlineStr">
+      <c r="D45" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxPNHRXaU5tNUVkd2MtcTg5M0EyQllrM0owMkZobGxLaUJxYUN2MUg0ZkdKdzU2YmxfanR3QU53cHZzNDI1WXgzRUcxOE9EZlluNmtNRUUzTGJPRnpfVVVOeFM3bFRNQmp6VHFBdi1mTnU4UDBvOEpMaHZPNXFtdUIyTlhuRExIVElSeVRUMGxjU0k5VnVxaWFfd3htWngydlhuR2E5aTQ5VW1LS01ac05rMGZoVFdOZzVyTzFhUDVsYkNrc0VQZmhubERSaTNwelk3WEhYUjF5d2ptMktYeEhzOHpWazFQZXphd0xfUFdhbkVGMVR2Z1dtVtIB_gFBVV95cUxObEwzeHd6RmZtNUp2dXVVV0plOVQ4WlNqQXNJU0thd1BEWE8yWkxxVTZjTkpsVGxxWGxpQzN0OERZbk91ai1fZkdtc0JoM1h5NERLTVdDbVJ4Y2k4djdQcWlVcDF6NjMyVDQzZWMzUFZxWjVRWllMZHVSOF9jQ2U1REFfNUlhM2EwYloxb1MwSTJjODdWdlZwX2h2N0xiQWNhallHUTNPZEtLaXhsY3dBZy0xM1VITXhLUERXS1JxR0R3OUpBTVBPZ2dPZTRUTVpvbFBNMjFUSTJuWS1XLWdhUS11UTRzVTVqaEhfMDhqWHlTMlJGekU2QzJVcFdodw?oc=5</t>
         </is>
       </c>
-      <c r="E45" s="9" t="inlineStr">
+      <c r="E45" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1750,7 +1753,7 @@
       <c r="F45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="9" t="inlineStr">
+      <c r="A46" s="10" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1760,17 +1763,17 @@
           <t>ExxonMobil eyes New Zealand market exit</t>
         </is>
       </c>
-      <c r="C46" s="9" t="inlineStr">
+      <c r="C46" s="10" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D46" s="9" t="inlineStr">
+      <c r="D46" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxPanlvR1V1eVVpdmYxNVNGMnd6UjJFd0J6Zk9IU1lhOW1GbmVTcjY4QkJCYkl3Y3NOU25VRTBUekwtS3plV0NVdlZtOTZZRHJWZ0FVdDl3S05aMlFWeEZiYzdwYmQtVnJxZEw0NktHaFZMNlZkUC16empqRGxxMEhhZGwxRzVEek5FelB3aE9UWFhGQW42b21MRnJHUXV2ZGJYUXJIMnVFWGZsSnEwazNGNUdVcjVoekp0NEZCN1J3cTlaZldFa1pMUkJTbVZYeFljVkRqQmlZV1M2aXh0ZjI5dEI1NDB0UElPUERsbUljMlA3OHBnYmtJTXFWZWkyUdIBgwJBVV95cUxNWFBRQ05GUDdwTWJ2ZVFJUS00ZUh0QkpZQVNNcU9JYXRTN21sMS1VZTlOSTh2LVFuZHh6UVk2djlrdWFsd3MwcDFCNmhwUlVLTlpjVF8wSmt1YnBWRE9tNVpKQlk2YXJWdmwzZWlLX0xpaWxSMUpsX3ZjYXhmRmE2YlAtSFJGRG5pQnVmMnViQXlsVFV3OU1hZFVrY3ZITHQxcTR5UkZ5U1pReHVJMGZGM2FCZWliSFZQZmpVLThSdExWMW14OElodmVVSC05SUh1d1hBenJoY3BUZGxoM0NTbTExdERmM3pjZGd4VzgyV3BNOG11TElBQ3NsRGhtSEc3YzJz?oc=5</t>
         </is>
       </c>
-      <c r="E46" s="9" t="inlineStr">
+      <c r="E46" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1778,7 +1781,7 @@
       <c r="F46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="9" t="inlineStr">
+      <c r="A47" s="10" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1788,17 +1791,17 @@
           <t>PAC Capital’s Clayton Larcombe charged with assaulting wife</t>
         </is>
       </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D47" s="9" t="inlineStr">
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D47" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOLXNDU2xjMWpyeEZwWGwtZkV0TjNSbGtWS3ZidUo3a0dvV1hrTnJiVXBXSkJNWlhXYXFHZkNTa3g4a1ZfMjRPM3BtWTZUNGg3S09kbGI2TTRGd0Jkc1A4WFAycjlpVC1URjFvNnBraWprRkhaT0VOWkh6N0xkUjNXNUw0dGx2N1JtTDVsREdtZDhraXVsSkxhR2ozamFUSGR5VHBBRm1Zcmx1c2RDaUIxQkVpeUpfWjFNeTRLWVRtYjluZ3ZncGZIMQ?oc=5</t>
         </is>
       </c>
-      <c r="E47" s="9" t="inlineStr">
+      <c r="E47" s="10" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1806,7 +1809,7 @@
       <c r="F47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="9" t="inlineStr">
+      <c r="A48" s="10" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1816,17 +1819,17 @@
           <t>China touts itself as ‘harbour of stability’ to global CEOs</t>
         </is>
       </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D48" s="9" t="inlineStr">
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPUzBWeVk0elBOZ0l5QU44TUJvU0RvSmtPdmVyT2VuQTczaEdzbkktT25ZT2Y0Nzh0bVBhQW96TUhpWkdEOEJMVVk2UWxLOENKZGk3X2tQcDNsWGZtU0JkM2U0N3VfUWFBclhUSUZya0NwRTJOWmZJdWlhT3JtY1EtSkJ6TmlsV3dzOXpDaVFMNlBaa3RfRHBjc3Q0cjk0eVdPV2MwcjlHNA?oc=5</t>
         </is>
       </c>
-      <c r="E48" s="9" t="inlineStr">
+      <c r="E48" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1834,7 +1837,7 @@
       <c r="F48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="9" t="inlineStr">
+      <c r="A49" s="10" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1844,17 +1847,17 @@
           <t>Eyes on 3D Energi as oil and gas giant Conoco flexes buy-out rights</t>
         </is>
       </c>
-      <c r="C49" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D49" s="9" t="inlineStr">
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWVU1QmhTUGFkYlpTQkw1WUFPTHhmbk5lbnE4T1haQUswSi1ITHlhVmhyM3ZYS3N4cVd6ZkwzdGdhT1lvM1JJek4yLXFpSWoxUnRtR2JRLTZWa2dlTDVTakE3b2xvazFWX0kzRHFZWVB4OUh0XzFFd3JVSVlfelpVa21qTldCVHdvcmJYcGNjZ1RrdElWS3Yzck9KYzRvbzloWkNqMnQ3dmtHbzNuc21ZSXNYeEFlZw?oc=5</t>
         </is>
       </c>
-      <c r="E49" s="9" t="inlineStr">
+      <c r="E49" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1862,7 +1865,7 @@
       <c r="F49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="9" t="inlineStr">
+      <c r="A50" s="10" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1872,17 +1875,17 @@
           <t>Blackstone tempted by $900m payday for Sydney’s JPMorgan tower</t>
         </is>
       </c>
-      <c r="C50" s="9" t="inlineStr">
+      <c r="C50" s="10" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D50" s="9" t="inlineStr">
+      <c r="D50" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxQNEZTZjY0S2YzcUxsb25RSDk2NHd1N1VOVlpMbi1JNGEzbUt5ajlYZFhvLWNBTkNQVXNuWERfTkl0Z2o4R1U0Zk5jVE1FTW5TTUJGZnNJc2NqMm1fT2dmYTVwRGU2TkZ0c3BjZVBGS29fWFJvZ2F0MWNLa0pYY0RNME5xYS1vOGZmMDVBcDBaLV9MWF9od0EwekFyb0ZCOEdkNTFaN3ZXckJwd25zS0FsdzU4OW1UODlueGNyZVBDSDZkeHQwelV5ZXVDVlcyUkhKWDZfVlRacEJHSElmNnhKSXk4ZHJHWHhPTEV5NGNkcmhyU0hjV3J4dVBXbnRGQdIBgwJBVV95cUxPME4ySFF5RWNrejVlWW1yeW56N244RGpyeVJUZEgyTjFNcE10YjVpMmJyeWsxTENzZFhPRlpsbl9pVXl0NGJvUlZFT216NE1KRFNwOHVZVXMzanNKNXFmWEdsMndsd1cza3NTTzUyUUZfaDEyWHJwZEtQbTdJRmkyU3A0RGh4QlAtT1lRVXk2SGoyaTI1NUpwVExYSkZJNmVFNjdXTDJTNURFOEh4Y1dnUDVGdjBpaDlWVWJtUHZiRDdGTmE5R1R6TDBwWFFnT2MwQ1lmT2w5bDF6eVU0R20tYnpnT3JCZlJod2s0UndyZTM5M2xLZC02a3E0NmJRdFV0Qkow?oc=5</t>
         </is>
       </c>
-      <c r="E50" s="9" t="inlineStr">
+      <c r="E50" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1890,7 +1893,7 @@
       <c r="F50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="9" t="inlineStr">
+      <c r="A51" s="10" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1900,17 +1903,17 @@
           <t>I-MED attracts mystery suitor as Permira weighs sale or IPO</t>
         </is>
       </c>
-      <c r="C51" s="9" t="inlineStr">
+      <c r="C51" s="10" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D51" s="9" t="inlineStr">
+      <c r="D51" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxNaGlwS3d5MGFMbEg2U2hnZUxMQmdqaWI4bS1lblNZOFhkSnRMcUotRkZMTjhFZkRUQWxUUDVtYml6TVAxUXkyZmx3SHRFb0gzVHRST2ZQUThKa25aWlhlcGprSU9tWktXZjZRaC12bFpkaVVWZHhIMERyeVNNWEswYTJ2ZHdnRFVRaFhod2U5N011TkQ0NG5MYVhoT3MwRUVZdVB2UVhKZExvdFIyXzNNUGt2SHJUanQxRkI3bXlLSlNJQTF4NXQ1YlZDaGVBM0EzNUhYQVp6NkFWRzU4bnRPWTgtXy1HVnB0ZlN0Uy1rY2FuWlNfN1U4WXVHQnRzVkNG0gGGAkFVX3lxTE1GaDJJdTJlOXFEZUtDTmdXMmsyLXlpaUxzQXpycHk4MTdHZng0dVczYWVwdWRzdFFCMlNLWkZpMm5Zd2RpN0Y0Zmo3Q1FOZFBZQlh5LVl6aVZ3X284UmpxM0pVRzZmMmpjaUdNWnJPZGV4V3lNai1CTllCcW5oUEVxaG0zejB5anc5YnJEZzZPT2d2QklCWjl2MjRBc25jUndqZkVadllKaUZScG12bEozT1NKUUJYR0pHTGtJZVc0ZHZLNHVSYlhzcTE0SkZmMXNlVGJ4YWJ1cThxcGlZTDMzRUMxLVM5VHh2OW5tRW1PT3VyRUhDbV8tRzUzVzRzVWZPZ2w1bnc?oc=5</t>
         </is>
       </c>
-      <c r="E51" s="9" t="inlineStr">
+      <c r="E51" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1918,7 +1921,7 @@
       <c r="F51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="9" t="inlineStr">
+      <c r="A52" s="10" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1928,17 +1931,17 @@
           <t>The stagflationary mix that has billionaire Solomon Lew worried</t>
         </is>
       </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D52" s="9" t="inlineStr">
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPWTh3S05XQWpTQm03WjhBT1pWc2cyOFRMd2ZraHhPUHlDRW1tWkZvdkhQWHE0MHVMRUpaOFRoX0JsYWhJV21nVkpIM2RBSmlZRUtEbFAydzZfOTh1S05oNEZPOGgyZDJRMS1uLThWYWRVT3VEVGhtYkVLN3J2OWsyX0VVdTUteFBCOVNKZ28xUTRPTk1SUkMxZ1NJc1B6NXRrUEEzOG01YnZOYjk2cWlFZA?oc=5</t>
         </is>
       </c>
-      <c r="E52" s="9" t="inlineStr">
+      <c r="E52" s="10" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1946,7 +1949,7 @@
       <c r="F52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="9" t="inlineStr">
+      <c r="A53" s="10" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1956,17 +1959,17 @@
           <t>Oliver Curtis on Firmus: From prison barber to AI billionaire</t>
         </is>
       </c>
-      <c r="C53" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D53" s="9" t="inlineStr">
+      <c r="C53" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D53" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQek9VTlV1b2hVb2RoZ0Fya0REb3E3YlBCR2NYZldXcEh2VEY0LXg5bjd6RzlnZDI0OUJJd2cydTBwTm9tdHpiZ1lSMnhtcmJSYVRKbzJFMjdDaEJyZExSQVJVRDh1c00yMjFMaVlPdnRuV3VkTjNxdzFRbW1yeGltSF8tVXlJVXJzTEJXS2FTYkJTVkdKbmdPTTd6YzRtYV9nN0JzOVZNTzhUdUk?oc=5</t>
         </is>
       </c>
-      <c r="E53" s="9" t="inlineStr">
+      <c r="E53" s="10" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1974,7 +1977,7 @@
       <c r="F53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="9" t="inlineStr">
+      <c r="A54" s="10" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1984,17 +1987,17 @@
           <t>Three startups that raised $161 million this week</t>
         </is>
       </c>
-      <c r="C54" s="9" t="inlineStr">
+      <c r="C54" s="10" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D54" s="9" t="inlineStr">
+      <c r="D54" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNRGVZMF9DeGJjX29vN3B0blVoM3RKSlJJTllrMThKUDJNZzdPNFNnT2JyTElUOUYxMHlsUm9yM2dBQnZfaVNZblpqb3NzTXdHVlpQNkRqR3NBZHdzODdjN3RKMTZhSVRqUEM5d3JRc3F2OG9hWmZJdU5rakg4ck8wLXlMTnZSU0lNaERmQmswbkVGWW8?oc=5</t>
         </is>
       </c>
-      <c r="E54" s="9" t="inlineStr">
+      <c r="E54" s="10" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2002,7 +2005,7 @@
       <c r="F54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="9" t="inlineStr">
+      <c r="A55" s="10" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2012,17 +2015,17 @@
           <t>Iran eyes ‘plenty more’ vulnerable energy targets in costly war</t>
         </is>
       </c>
-      <c r="C55" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D55" s="9" t="inlineStr">
+      <c r="C55" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D55" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNLUN1MHlZaTNfVHhVX0RnTXp5QW83RmM4WVZkWW1PSnNaZF93VkY5ZF81anB3NDNmX0kyMkVSdkxNSURvSEh6enloWnRVcTlsR0JPTjVzNFR1YjRsSm52VnA1XzFFUlUtODJjYy15YWRRdWZZRkdjRXpCcEFSVURmV3VpSTFhTjVUb1d5bmw3NHNlT3VQZU9ieEYwM1J1TGEyZnlnWXNIWFJUMEtIOVZad0dxRWZBdw?oc=5</t>
         </is>
       </c>
-      <c r="E55" s="9" t="inlineStr">
+      <c r="E55" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2030,7 +2033,7 @@
       <c r="F55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="9" t="inlineStr">
+      <c r="A56" s="10" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2040,17 +2043,17 @@
           <t>Don’t take it personally: Bain Special Sits hits hurdle at Infinity</t>
         </is>
       </c>
-      <c r="C56" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D56" s="9" t="inlineStr">
+      <c r="C56" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D56" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQRjdwTk0xTHVIRHNkdG9tVk1EQ0hiQjJ6dGcxaWZRZ0hZV1U4YjJDU0tnTUlWSkQ1S2dUTHJVNk0tNWQ2cVd4dkw0M25leXRreWJtdlBKYTAtNzRocTJUazh1dnRzSVlYZThySTBNVjg5X0xYWUxCMC1SelltSHVSUEV5U3B1bTA2NjAzMGFZLW1CNkQ3aWU0S1JxS0d0YmZiZjBKQVRNVUpzYno5R1pvbTBsaTM?oc=5</t>
         </is>
       </c>
-      <c r="E56" s="9" t="inlineStr">
+      <c r="E56" s="10" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2058,7 +2061,7 @@
       <c r="F56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="9" t="inlineStr">
+      <c r="A57" s="10" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2068,17 +2071,17 @@
           <t>Drill, baby, drill: It’s boom time for mineral and petroleum explorers</t>
         </is>
       </c>
-      <c r="C57" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D57" s="9" t="inlineStr">
+      <c r="C57" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D57" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNdlFOWld5ZWhPVnFRa2xidWlUVzluQzkxUTgxR0t0Rmg2S1BzNjdINnhwS3VLRkNjRVJLX0RHU0h4VFVRY2RfSHBudEhfNVNjeE50ZUxQenJNSlJtWFRlcnNsZm1iLXlxM2RmVDViWEtjNDloaTBhUDVxYkNfOWFCTjV6cExEVlFCMzNfWnVwRDJHYWxWV0hOR2V2S0VlV2NyS2s5cWNmREtWXzlMMDRQNW1tVlBOblp3SHBEVg?oc=5</t>
         </is>
       </c>
-      <c r="E57" s="9" t="inlineStr">
+      <c r="E57" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2086,7 +2089,7 @@
       <c r="F57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="9" t="inlineStr">
+      <c r="A58" s="10" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2096,17 +2099,17 @@
           <t>‘Wake up’: Fury as farming crisis looms</t>
         </is>
       </c>
-      <c r="C58" s="9" t="inlineStr">
+      <c r="C58" s="10" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D58" s="9" t="inlineStr">
+      <c r="D58" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNelJvMXFPX3MwUVRMN2xqbzE1MWdvOF92Zy02YmIyZW9SQXRNQVZsS0xVVG9UdkFPaTV6ZC1tV05SZWNqblNFZ3Y1VGNaVVBaaEl6aFJqQ09ONDVkNUs4TzNvVjV5eHNjUk9xaDRFZTM0alpuYUdvWGtLRzRhYXN5alZ1QWdsZTEyODdQVnZoazkya29WeTJZVmpxLVBCdWxfY0dTN2Z3WFZlSy1sVW44RDlvZFAzYlhnQ0N6UWhKSU02eF9iZllIU3g5MWtSbkJzZGxWLUxHNERzdUlLTF9VYmpJSTRLY3U4NlVVaDhmc09uOWwtUGtlb0I2M05DR1dnRWxGSFV2NEJXaEF4c00tN9IBlgJBVV95cUxOSzZ5NXZMTTlZa3BSNjZyTUxUMjRhYWJhN0hMa3dDcW9CWGstNnI5MzV5U0hJSTdKLTFwa2E5YUItZnFRbW5RbzVuYW91MmZaYXN3R25hWVpUbW9oUU9fVktPRHROVDYyd2dSLXJVZWQtY016bkVxY0VPbkY3Zkgtb1liWGMxeEpyYmloS1V0TVJMMWZaeWRZX3FQRjBmVzJwdkkwMEVDSXV1MTdReUhGZ0Z3dENyMEFkLUl1aXhtRkFLRFFXcEdMZzFuT3NxRDFMOGVaY2YzeXBQc09fY3YwcFp4MVczRVN3d3dJZWJfTFFscjF0cUtRWHdzTUptaHowNDhYWXZXTHhYTHNTdlZGUmNlamRTdw?oc=5</t>
         </is>
       </c>
-      <c r="E58" s="9" t="inlineStr">
+      <c r="E58" s="10" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2114,7 +2117,7 @@
       <c r="F58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="9" t="inlineStr">
+      <c r="A59" s="10" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2124,17 +2127,17 @@
           <t>Construction giant FDC road tests IPO pitch</t>
         </is>
       </c>
-      <c r="C59" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D59" s="9" t="inlineStr">
+      <c r="C59" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D59" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxON3p5Y3VPM01XZFk4a3g0R3JnQkZXbHVGV3BKdDB6M3NRb0M0SEl3V0R5RmhCQ3dnaHB0ZHp5N2hCMUFsNU1ZNWZ4YWdNZWdETkUyZmdoeW81amwtTWNFZlc5WlNpMkJwRzk0QklORGhlLWNEalh2d0JCX0lhVHhhUF9ibVlxcHAwOW9ENndVOTY0enBYUWc?oc=5</t>
         </is>
       </c>
-      <c r="E59" s="9" t="inlineStr">
+      <c r="E59" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2142,7 +2145,7 @@
       <c r="F59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="9" t="inlineStr">
+      <c r="A60" s="10" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2152,17 +2155,17 @@
           <t>Austal suitor Arlington Capital Partners buys Eptec’s defence unit</t>
         </is>
       </c>
-      <c r="C60" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D60" s="9" t="inlineStr">
+      <c r="C60" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D60" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNM01qb1ZRZVBIdmp3cFc3R3RLaTdmZk1JOFo4anRtSm95Z1hJc0N0S3VranBTV29IdlViT0FkSm92eHdtbDBqdU5HTHNMaXo0dGRWMkpDdjk3LVRBVU1rZC1YejZJMkhyNmpZZFJodGoxWlB1dkRhYTJVRlljMlV0dUllQ3EtOHZkNFdSUWJLSW9Xemw1XzFzU2RHV1o0RTViOXp0bDZFQTZycWhpNElLU0FZQVI?oc=5</t>
         </is>
       </c>
-      <c r="E60" s="9" t="inlineStr">
+      <c r="E60" s="10" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2170,7 +2173,7 @@
       <c r="F60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="9" t="inlineStr">
+      <c r="A61" s="10" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2180,17 +2183,17 @@
           <t>Eyes on Tom Wallace as clock ticks on Adgemis pub deal</t>
         </is>
       </c>
-      <c r="C61" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D61" s="9" t="inlineStr">
+      <c r="C61" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D61" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxNSExQeDlENWlHb0prRnRldjZ5YWhKVUZ5eVdsYjZmbVRWRWQ0WnZXWkU3UHZJdElnQ21jMU9zNnhnc3JlNDczVGQ5Y0FGV2J3QUp3NXdZTXZMNm5tVC1vWDFtOFN3aS04QVJZb3FZV2VsUmJ2aVgwbUhTaFVGdHg0UjRyTXVVUnFhQmE5eFYwMGR6T1R2U3Q3WEdZclVKNWJiby1IRg?oc=5</t>
         </is>
       </c>
-      <c r="E61" s="9" t="inlineStr">
+      <c r="E61" s="10" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2198,7 +2201,7 @@
       <c r="F61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="9" t="inlineStr">
+      <c r="A62" s="10" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2208,17 +2211,17 @@
           <t>UBS names head of APAC leveraged capital markets</t>
         </is>
       </c>
-      <c r="C62" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D62" s="9" t="inlineStr">
+      <c r="C62" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D62" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNMm9WZ2ZKVFBvX2pYMk16VmY1WFZnZ2J5N0F2bHduTVM0Sjg4STVtTGFLQVdzeFloVHg3clRic0owTDMwYVpXdDVjdjFOWjQxdkdxdFY5MEY1Q1U2Q0R5dFBJWTNtUzgyd3RXcm9uM0hKdEZ3b3JjXzcwQ2VpRm5SS0hYT2gxSU9iVFRlR05Xd2EtM2JOQjBGUzlKdnE?oc=5</t>
         </is>
       </c>
-      <c r="E62" s="9" t="inlineStr">
+      <c r="E62" s="10" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2226,7 +2229,7 @@
       <c r="F62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="9" t="inlineStr">
+      <c r="A63" s="10" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2236,17 +2239,17 @@
           <t>BHP, Woodside rise after new CEOs named; Future Fund chiefs exit; Sandilands ‘doesn’t accept’ termination</t>
         </is>
       </c>
-      <c r="C63" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D63" s="9" t="inlineStr">
+      <c r="C63" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D63" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNUHhZeHNHemtiLW1IOHN1OTZXOGpsM0ZtUG1MVHRCT1hUT1k5S2lEOXlXRENWOXNlMEZadThQR18xSTJfTVlQM3BtX0ptX1J0bk80SzNLUVRtbkJITGgtb0lsSVdJTWt2S1E1WUlXdUdsbEV0V1RpNWlyRXBoc0dPVDl1OXRrSlM3SHlDazg2UlcxenVzNzlhQldhUGhfNE5IV2xrVmVBNzhhSE9qY042Z3pzMEVzd0VyVmZudXgxcTgwWGJXSWZKZ0FyNVhjcmhjTm5DYUVjLUdDRmxUQkZuTDFlUXVaV0ZoSWp5WHMyR3c?oc=5</t>
         </is>
       </c>
-      <c r="E63" s="9" t="inlineStr">
+      <c r="E63" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2254,7 +2257,7 @@
       <c r="F63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="9" t="inlineStr">
+      <c r="A64" s="10" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2264,17 +2267,17 @@
           <t>BHP’s new CEO will shift the Big Australian’s centre of gravity</t>
         </is>
       </c>
-      <c r="C64" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D64" s="9" t="inlineStr">
+      <c r="C64" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D64" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPQnZpWndNZzZvN1VsOHBmRDVLRHVTNkxLeDVDelpOMURjOTRDSDZfN2dPZlZqaW05WEZuZXMyRTJZeVZnV0poT2UxRkVfZ1RZSjdvUjVKblhoSU5Cd1plRTVNNTRaNWZmbm1yUGZkblVpYkctNzVRRkVQQm4zX1FtRG1KV2Y0djUtOURianJ3dElqeXBUMFp4aWFEWVFYelVjYTluSWpOM1FlbHpIaUxXdnBn?oc=5</t>
         </is>
       </c>
-      <c r="E64" s="9" t="inlineStr">
+      <c r="E64" s="10" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2282,7 +2285,7 @@
       <c r="F64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="9" t="inlineStr">
+      <c r="A65" s="10" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2292,17 +2295,17 @@
           <t>How philanthropy became the sandbox of succession</t>
         </is>
       </c>
-      <c r="C65" s="9" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D65" s="9" t="inlineStr">
+      <c r="C65" s="10" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D65" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxObnBPb2MzQ1RvSVVCbmNzYWFBMlFjU0dQRmpPakNfdkxtMWc1bFdVNXNlZmRKQnNlWEtUUDNSTHpTLVV4Skx0V2otbTZsTTdvT1VaUDhMZFZoMFFab1RoS2pCcno1WGlNQlY4eXQ0OFEtLXJTay1MUkFSSEJ2MVVScUpjUkhJOThISy1QbHIzTzFlWVhOc29fWWs0V19sQ25hRW9MSGhBVVNKWUp6dUo3NS1SWlk?oc=5</t>
         </is>
       </c>
-      <c r="E65" s="9" t="inlineStr">
+      <c r="E65" s="10" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2310,7 +2313,7 @@
       <c r="F65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="9" t="inlineStr">
+      <c r="A66" s="10" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2320,17 +2323,17 @@
           <t>Advanced Navigation raises $158 million Series C round with NRFC backing</t>
         </is>
       </c>
-      <c r="C66" s="9" t="inlineStr">
+      <c r="C66" s="10" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D66" s="9" t="inlineStr">
+      <c r="D66" s="10" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNTXhwVlVLUy1pWEpFdzFCazNTY0dkczd4WW9oeW14cUtTaDZRTGlVQXBPaHN4WTBkNW1zOGxvN0tVWl9JSFdVNXlQMzVxbk4zbDZFUjNOcUxSamNaSnFCckMzWEk1VlNoSHJHQ3VWdGltVWZCV0c0NmU4UlN6YU55Q0J2TkQtUzBzOW96UXRxem5Zb3M2SUljNURISlRkQmJD?oc=5</t>
         </is>
       </c>
-      <c r="E66" s="9" t="inlineStr">
+      <c r="E66" s="10" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2476,6 +2479,454 @@
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Gentlemen at Melbourne’s exclusive The Australian Club sweat another election</t>
+        </is>
+      </c>
+      <c r="C72" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D72" s="11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPcEwyU01BOXF4TzlmREhYbTFEWklxdWZqWmZybDVnOWtLQ2dTU2dNQ2t5M3BVT2stN08xYkFmazVkY29oT3RVc2xUZmZINFJURGtIRTg4RGsxOURBdWEybTUwU2NUODQ2eDNBbTdPT3QxeXRFNHlSc014T0g1aG4xZ1A0U0FWMTB1Wm1CSHlQU0ZJb3lMYkE?oc=5</t>
+        </is>
+      </c>
+      <c r="E72" s="11" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Inside Fortescue’s AI ‘hive’ that could save the mining giant billions</t>
+        </is>
+      </c>
+      <c r="C73" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D73" s="11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOSVVCbGpzcVcxTGlZZ2dTUkxXdVVvVU1ONEtUS0t1R1VkWWRNeUF1UmlHbXd6clR3QVRuWGxrUGQwVG1OeUxZb2RqTzdYOEVGQ1N6eDFta3VOZDdHNThYbUEwWEVHZlZBVzNpZ1Foak1kLURZTWpJVzZLekczdzFrdHMtLVZwMUZnYmkxSVc0czFqWnFaSGZiT2pIVW5rdVZmdThreFlRZWVEU0xoa1VFOV9MTjE2UHFOcWhqUzVB?oc=5</t>
+        </is>
+      </c>
+      <c r="E73" s="11" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Tiny house maker Elsewhere Pods seeks cash after Bunnings debut</t>
+        </is>
+      </c>
+      <c r="C74" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D74" s="11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM0ZpVnBTS21Ib25qa09CaU52Z29kZWhTU0FJLW5VR2JCLVFPTVlZTmpYX3lZVWdtMDVTYTJkWHlPUmhXa0Rua2ZXTTBWQU1VdmFrV21KOGlrdjJ3TTdxbGlvZVBUZUxUWE1uelpWMGxWWk04UndJTXVKQjBZUEtoX3lodmdpMWZKNUc1YTIxVFZLYkFKT1QwbS01WU01ZUZTTlczY2ZpLXlpTjNJTWpsUg?oc=5</t>
+        </is>
+      </c>
+      <c r="E74" s="11" t="inlineStr">
+        <is>
+          <t>Retail &amp; Consumer</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Chinese consortium emerges as dark horse in Made Group sale</t>
+        </is>
+      </c>
+      <c r="C75" s="11" t="inlineStr">
+        <is>
+          <t>The Australian</t>
+        </is>
+      </c>
+      <c r="D75" s="11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQYlpEY0hxNm5lalIxSTUzbDE4UEF5QTNpMTl4dWNPMkRrMU1yQnltZ25WcUkwOU13V2Y2RGItVW5QTXotSnBZRUJMdGJySGw0NVVxc3ZLZmVEcTlfU193Vkd5UVVuTFVYWFNtd185eGlVQW5RRElHdk5pMjhUR24wd1k0T0I3cW9qTG5Lcjg2bV9aNWsya0FYODRjeURyMW1EeHdYT05iZHZhLVFrUVNoV25idnZYZ2lpZEhta2JxOWFJb0M2SE9hbFF6NlVWYTM3QmF5anpWOEZackZiTDBfN2gtX1luQkxFOUxSSNIB8gFBVV95cUxOQklMYWl1ZkRqZGUwN0ppeXFubzZWNTNmeE5GY1BfcS13N2dFT096YW9JSndVX1EzTlBKdWZIemdKZnRIME9SQk5aT1M2WnRESjJxckFTaUdOSEd6eG9hRVBjdlhBbWQyWGpUS1kwQXJsdlpkLXJpXzJZX2xiUC1FSlNnNTFoVXQ4bF9JeUp3UGRWdUFOUVRrNUtsRzRxaUczb1p2LVVucFBNazhuZFNDaUZDR2ZQUVdObmVtTnBndGlkazZqeHVheVNzSE9RY3Bad0lrckxDSWY5QXBWS0hwVzZvSTZjaGEtNkNncW1RRE5uUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E75" s="11" t="inlineStr">
+        <is>
+          <t>Retail &amp; Consumer</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>KMD faces uphill battle in capital raise as key shareholder baulks</t>
+        </is>
+      </c>
+      <c r="C76" s="11" t="inlineStr">
+        <is>
+          <t>The Australian</t>
+        </is>
+      </c>
+      <c r="D76" s="11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxOVTU0OGNfRURNcDdzYUtIcG8tR3N4OFFYalhKNWJBaUd6ZlQwNU5MZVZYbUZVSzB3WmdOOFdTZHlBOXBzSGdYUVV6eGt1UndHN296bENxZzNUM2NoaV93LXZaZFNNOXJ2YlA4RHNFS2FDb1ltNWpPWUdRR3VGMWoxaU5qYm9VSW9yUW5kS1NaN2RSc2YtcHZRSTB6aE9Zdkl3NG5nbVRzODRfQVYtelo5M3g4R2JEbnpraFpWbENOZzE2Qndla2t3MXRPWkU1dXg4NmZRME1jT3pOOHZOVlpTZGloNENUZllaSTFmWUV1Y2JLck02ZDhnTHJ5bUPSAYICQVVfeXFMUEFXR29tQjlTbTdMRVNDWUlGNFNOQjVhX0FiSkl0U2stbml5VHR4d1g3bDFqMUw2TzR1eHhYOU5ZUmJpZ2xBY2NzcmJRX3MwaEQ0YmpzMUFnV1BQNGxmcnlXUzVvbHpwNEo5dWFnZlduZ0Z2dGZGRFRKRTNCUzctZDNCd0FMNEkzTm84dmZOM2NKYk81RERsVnlZN1VZaXp5TW5QRVAzOHNXQTFWdVlKdGtFX0FmcU1EbElZSm52alBQeWx4VnlvOFRwNk1ia2lZYXlpemQ4cFdmckotMmMyRGE4ZXN0dThQYmxxUkpvMzAwRXBBcVJuRnp0QkZ3b2tqMWF3?oc=5</t>
+        </is>
+      </c>
+      <c r="E76" s="11" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>AustralianSuper claims another listed M&amp;A kill with Pepper Money</t>
+        </is>
+      </c>
+      <c r="C77" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D77" s="11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOY0RwcnpWZlhfOHA2MG13MkJUX1RDNF9wN2RxZGU2cEpzS1RKTjJDeUl0OERFOGhFRXJaSXNETEhHbW9PS0lua283RnFVbHJvTlRva0djQ2lRSGc2RENJYmt0OEsyYTRVSzFGeE9jWVhKMVRnd240WXVNTVdac2lOUGJSZlc4UVZ5RXo0OTlQbUd6NWRSek1HZG9fZGk2aDhDelhGVmk4YkRKeVV1M0VHZ2hZNmFVdXM?oc=5</t>
+        </is>
+      </c>
+      <c r="E77" s="11" t="inlineStr">
+        <is>
+          <t>Australian Economy &amp; Markets</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Apollo to Acquire Nippon Sheet Glass in $3.7 Billion Deal</t>
+        </is>
+      </c>
+      <c r="C78" s="11" t="inlineStr">
+        <is>
+          <t>Wall Street Journal</t>
+        </is>
+      </c>
+      <c r="D78" s="11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOanpORVBremoyamJyZ2FqQWVOcDcxa2NpempBUmNYcktMLUl1Mzg5VDloWmlVbUdNUnplVk90WEUzXzJjNGxENk9LcGF0enVSdlFpWU9nd244YWNTS0ZHd1JTZEtlbjRQTmJUU0dzWmlDOVFhR1ZRSFJkNXN4a3FHdGozcUcwdHRseXpYMFREUzBNcXRmQ1VCN056SWlEa1l5VVE?oc=5</t>
+        </is>
+      </c>
+      <c r="E78" s="11" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Estee Lauder in talks to combine with Jean Paul Gaultier owner Puig</t>
+        </is>
+      </c>
+      <c r="C79" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D79" s="11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPSjN6QnFVbmdHWFoteURWaU5VaWZmRmpTT3QtYm1tZUFyNUZyLUdheGdfWlRBTlJyTlp4THIwVDA4U3BnWFNpT2FpZlZzX1lJSDV0MkRGVjYtNVc0b0lOQy1RSnFGTWhCTWE2ZFFPYlFQX05yaVlfZF9IUEN2ZWkzQ0VFMUxxdHF2ODNQY09xdWlqWEczSC1CZk5wYU9QQlAyaTMyelJnaVM0cmN4M0paNzlBdzM1RndoZE8yRHN4UnZqaXVhVmx5NFpqS3hmUHhUdlpF?oc=5</t>
+        </is>
+      </c>
+      <c r="E79" s="11" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>David Jones accused of squeezing suppliers as losses mount</t>
+        </is>
+      </c>
+      <c r="C80" s="11" t="inlineStr">
+        <is>
+          <t>The Age</t>
+        </is>
+      </c>
+      <c r="D80" s="11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPdUtyNWs5YmxJMXNsNWtaMi1WMm5SVHd6ci1ReURLajdYd1IzWGJMZmE2MzJsSzAxQWtSTm8xMUEwNTh4Vy1zTmFsWFBKTkJ0YXc3ZkcwOVk2a2VNRWVGUS0yQzZhSXlCWmpDYUx6RmpTTlNhS0xIQklyVFdIVXJRZTNPaVB4TG4yQ1R1ZWF2MWpmSG81TVRaRzdtMXpydWhBS2w0a3ZPZFI5MnFKOW5tN21oUDB3NkNtQmR4LVVBWW9BUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E80" s="11" t="inlineStr">
+        <is>
+          <t>Retail &amp; Consumer</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>Australia’s new millionaire factory: Start-up to $1.6b in five years</t>
+        </is>
+      </c>
+      <c r="C81" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D81" s="11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOVkl5N1NGWS1XWWZSc0pHXzE3MUNERmV5SUgyQ3o2MmJ3U3Y2YlNwUXNSTGlQenBwVFdnMWhoT2FrcDAwUHNVU0RQbjFHMjJiLU1TRC1nemdrX3hPTG93VWZUQUx3Wk9HT3lYd055Z2FtREFpOWRlYXFDb2hwV0cyWFMwaHpsLU0ta2VVQlpid1dlYks0ZHg5YTY3Ykt6Um5YaF9MR2tIRzd1Tk1IRnBrWVhxVjZNSUl1OE9iRlZzYmQ3QUVnZmhYVGxoOA?oc=5</t>
+        </is>
+      </c>
+      <c r="E81" s="11" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Social Media Wrap: Genki Sushi Singapore's loyalty benefits; Dunkin Philippines launches new collectible; Burger King Malaysia unveils new Korean inspired burger</t>
+        </is>
+      </c>
+      <c r="C82" s="11" t="inlineStr">
+        <is>
+          <t>QSR Media</t>
+        </is>
+      </c>
+      <c r="D82" s="11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxPbFR6eHVTRWZNcUw1TTBJdE1JTFpmbk5iWndKZnRoU3Fmc3cxcF80TnVhRERmY0poM09zTFpCaEVnMGo5aktxY0ExV1ZlZVpHYUtldXBoOUh6bm14SURHNmhnUE9tYnI5YlpXQ3pRZlp0Ni1wM2lYQmdxdjk4SDl0aFN0R1VBbGxpbFVzOHV0TFY3YjJZbDg4Vk1HMTBkQk5LRHd1ZEVpRnBsT1U0Nm1IbVFkZEUybmpabEhuLUNLOGhicUxXZG5UalRLOE5DSzcxRncyNjVRdk8zclhJNkVQcTRkQTZYSEdN?oc=5</t>
+        </is>
+      </c>
+      <c r="E82" s="11" t="inlineStr">
+        <is>
+          <t>QSR &amp; Franchising</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Copyright ‘status quo’ not working in AI boom times, says Charlton</t>
+        </is>
+      </c>
+      <c r="C83" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D83" s="11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNVVgwdEQ2YUt0eFo3THcxOXZHbUFYZ091VTFKZDZHX0szYWQ2dnZ1dkJma3VZcGk1LUM2SUtQSWhxMGpCUlFZVzdKNmdoSGEycm1oYlBUdEZ5R0ZlU2hrWHpFWXdSN1lCZnZzb3hZc2twVVlWdTNNVXhaR0Nza0FiaUNveXZWQWQ1ZE45MU1HbGNmWlU2aUdha2FyZllzNWdONEpsM2RrdGRFSFl2UlpJUnQ4WGpleGs?oc=5</t>
+        </is>
+      </c>
+      <c r="E83" s="11" t="inlineStr">
+        <is>
+          <t>Australian Economy &amp; Markets</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>The unapologetically analogue 4WD for off-roaders with $120k to spare</t>
+        </is>
+      </c>
+      <c r="C84" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D84" s="11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxPSFJ4ZnNLT3U1REp3MWI2WDFaQm5vZlp6QWN6c0hZamtYVU95WmpkUERwR1dwc0NQN1dEc0FNbHlaMTdLclVHb1JTc2VZNExENGYyUE9OR1BkQ244YXRVeWNwbkxia2VrckVqSy00WV9UNWlvZWJHOG9ibUthaTlpVmRBOGZjLWFzMU8yS2Q5Um05SWIzY2dKajhoMWFUcmFrbTMzai1CdVBNLWczTWRvbTBwSDRfUzNwOHhqQm5hTDdhM0xLWEpNQTRyRXZjU1FLdGhRMUxtOTg?oc=5</t>
+        </is>
+      </c>
+      <c r="E84" s="11" t="inlineStr">
+        <is>
+          <t>Retail &amp; Consumer</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Junk room to become jazz club with priceless Melbourne view</t>
+        </is>
+      </c>
+      <c r="C85" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D85" s="11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQbHN4My1nOGtueVJQZWM0LXNjLTR3MmhuemRJMUEwN09FTUZhZk1lbV9MbnVWblgyUXFEMEl3LUtsOGVqdGUweFR0MXF0ZEo0XzNhWVRqb2pGRUdiNTlLc1dFcXFmdnctQU1wQkRSdHN0T3J6VGt3MU1iNENydGlsOEpsT0ttZmJVZ0FUZmFXSUd3alVzUTQxMzVmcEVXSlV2dWdQd3JsMUZ0d3ZZYlBHaGhKTm9rM01SUmdseE9hT1prbHZtMlhv?oc=5</t>
+        </is>
+      </c>
+      <c r="E85" s="11" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Zimmermann fashion label appoints new CEO Roberto Eggs to replace Chris Olliver</t>
+        </is>
+      </c>
+      <c r="C86" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D86" s="11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM2M5QU1scVoyNHBmV2lwQ0VQS1Z6d2Qwa1ZkZ0M2WVIzdXR3QnZwVWhUSDRCUEdRZkc5QzFQSFFhNzZ4VE9lWXBTcGhpS01JdG12TlQxSHhValZfbWt3MUdFZGl3RlBtdnlrel83TjNjNFZ0SUpvSDNQbThpU3FLa3Atd0dNU04zQm9OSk5uNHpTVE84aWZpaVlKWkdOQjJjRTZSd1MwMEZ1b3pENkRCQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E86" s="11" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>Construction giant FDC road tests IPO pitch - AFR</t>
+        </is>
+      </c>
+      <c r="C87" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D87" s="11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNTnRScHFhQlpkdEdSb2x1bExxQm96ZE5zSV9wTDNDV2pxYjFQdUtoYmNBell3SFlTTFEzMUhpeXlmNERSeDd6VGppM2szQ1NHVE9PY1R3MTN0SUZLWkF5em8tQ3IycUZ2RmswX0tnN1IwOHl1ZFo4UUtMUDlQbXRjTnRCWFB5cU1RZFhsdDdaWGpMZzh3d29CWWZvZGtnTjl0T1k5ZHFHSUg5XzFSSF9TSUxTYkU0QkFheFlLZUY3S2tCSWRLZWlBbUpxUjc3TXBQQ01V?oc=5</t>
+        </is>
+      </c>
+      <c r="E87" s="11" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>

</xml_diff>

<commit_message>
Update news log — 2026-03-26
</commit_message>
<xml_diff>
--- a/news_log.xlsx
+++ b/news_log.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -87,6 +87,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -477,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -521,7 +524,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -531,17 +534,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -549,7 +552,7 @@
       <c r="F2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -559,17 +562,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -577,7 +580,7 @@
       <c r="F3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -587,17 +590,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -605,7 +608,7 @@
       <c r="F4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -615,17 +618,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -633,7 +636,7 @@
       <c r="F5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -643,17 +646,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -661,7 +664,7 @@
       <c r="F6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -671,17 +674,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -689,7 +692,7 @@
       <c r="F7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -699,17 +702,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -717,7 +720,7 @@
       <c r="F8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -727,17 +730,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="11" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -745,7 +748,7 @@
       <c r="F9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -755,17 +758,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -773,7 +776,7 @@
       <c r="F10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -783,17 +786,17 @@
           <t>Zarraffa’s Coffee celebrates 30 years, eyes nationwide growth</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOcXNzUkRLemZEOWtOZjhvRUtzcUZrSTdzV0s0LUJTd2NGRk1Gb1NSLUR5Rlh3NUdWQUJkVWctb0toUFBRajlMcWV3VnNyTUtydy1PSUoyb1NCOGVtMUZqRVN0MzFkVkNlOUZNVXlHN2kzREhSdWJQUnJqa0pnUzExTVZSc1NCVFZSNlBSUWNfWnZ3MC01aUx0UWF5SkNOaHI3ZkE?oc=5</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -801,7 +804,7 @@
       <c r="F11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -811,17 +814,17 @@
           <t>Zarraffa’s Coffee eyes 200 outlets ahead of 2032 Olympics</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPMUFjRTlGVFBqYzlPWXdzQ0dKVVlhWGxncUQxTDd1R0VHcThlV3ExVmo4SlBGSHVuUGZrMGNqSVo1YVpDWHViMm5KZWIxcHNMMHo0b1FQcmxUNElDR2lEeWRuLWZIN2lyQUV0VndEUWNkNU42Z3AzNXRlbm50NzhtTXZ0Q245dF9hNzBxOENuMXZsVlU4Z0JGVElR?oc=5</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -829,7 +832,7 @@
       <c r="F12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -839,17 +842,17 @@
           <t>Aware Super appoints new head of private equity</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNVHJXNWEtdEZZUW1fZzdYMTB4RklBTUh6dUNKQ3BrTlpYUnBwRURIVGZjWTV0OUxScnhGMVNSczhLUjVqOEwzbkR2WWlEbmF4ZkNUdHNQY0J1djI0REctbHd2SVhUNlNCa2M5bFhOQ0JPU0RHOVVTQkEzRDdGMjRZbVFDOUdlTXNNczlmZWF6bXlfbEFGRE0xbkZQaw?oc=5</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -857,7 +860,7 @@
       <c r="F13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -867,17 +870,17 @@
           <t>Commission wrinkle over UP Education sale</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxNSV9GMjhqM2ZSanI2X0w2OVlQVFRQTUoxYzAxaXVZMmU1REVTcHlUeEltdXJtaXZrcUJWdDZxNGpYTTZYSFE2TkZHeG9OaVRZakoxV0s1U01TVjJpWlhaSENfNVhucG5NVzFMbTVBY25zWGRSODBtRGtkS1owVTlJWnNfcTJ5alFnbVl1SU9aUDF1QWxJLTBSQ3kxUUFlZnpJMlVEQndFSGRGbDF6WVBUVHlCcDM5Qnh3R2xBMG9xN2FLckNzbUFOWDI1aVF1YV90d0twd0ZmMnUySDBMdG1R0gHkAUFVX3lxTE5EWVp6VzZWb01TRmlHSS0wMExldkJwSHJjdlZXdElsRlpBTEtVMkd6VzNQa1RpVDNsOFQzaGZ2VHpzUnBDYk82RmZGQWJuTmVQMXhxLXVmdVFxTVZOZTBsOHZ0V3cyVVVkNWUwVUxSc0xNSU92ZktpdFRfYnQ4WHBTX3A5bFhXZ1YwZXNrc1BSZEU4LVYybnNBd0dCdk92OFUwclJCMzdoU0ctX1pEdTAwY0JiTWQ4S01QRE00TW5EUEJwR2YtczZ0T005bTJnN1RDY2p6NFF1SndfLUo4QzJUWk1tRg?oc=5</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -885,7 +888,7 @@
       <c r="F14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -895,17 +898,17 @@
           <t>Gloria Jean’s owner has an angry shareholder on its case</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPTnZwUVBCdTFJZWkwc0YtVmJqMkNPcUR5RktjMlVURmhROFZkYUpXM01iRUh3SnJEUElxRGlSNk9DQjZSdTdNdmZwWWpONjlmR1hoMl92cUNmd3M4cnJhVkNqc095MmN6WXBYUmdEblB0eERtVDdlUU4yNGFjXzVnT19rOERIRzVPNzY3VDNNRS1tVGVTX3pKMVRpTXZVR1ROLURBLWtJbVZhY0lSU09DNkE2NzFLbEFU?oc=5</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -913,7 +916,7 @@
       <c r="F15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -923,17 +926,17 @@
           <t>Oporto-owner Craveable Brands hires new CEO from Domino’s</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNNmxfQVc2Umc4QWwzSTdsZTFvejRzTzZxXy1ScGlhXzh6bm5JS3IyX0xTNDVBNjh0cXpPbGhxNU5xUHhQN3EtRF9aV3FEc2JoSG5QTU1WeU1TLUJfZzVUT2N6dXloQXhZaHB5djB3dDFKN1llVmI3UVpKNjJTNlcyV0ZDcG9GdVdSdW41ZkN1b1N3SFFIUzcwRkQ3UHY2TmxERmZwTlA0RzU?oc=5</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -941,7 +944,7 @@
       <c r="F16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -951,17 +954,17 @@
           <t>Brookfield, BGH Capital rub shoulders in ScotPac’s data room</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPMVlxbzlQNnFXWnJFNU11Y1BhTTVqbjN4RG1nbkZuN0pkdDFFaUhJN0RaVnUtWDlZSGJWR1ozQXk5UUx6RVdOcjBPU2t5UzN4T0JvUFJISnNvVWxQemd3blNHZjRQVVVZQk1nZER0Y0JfY3VvQ0t1a09sM1RTS2c1YTJyUmdzYWh1WGRUNjl2dkdzYTJJeHVhMTdqR3Y5WVlHVEtSZHp1cmVYYmM?oc=5</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -969,7 +972,7 @@
       <c r="F17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -979,17 +982,17 @@
           <t>Payments player Pay.com.au hits the road(show) for $850m IPO</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOMFZleXZrbU53TzBlakI2ZmJKTjlrN3BoQlRaWjQ5cXFzTllKWmFoRm1UT2xDUHBtNC1QNTNiX1BwSzllMkRZdHIzRlAteDREaUczN1JTNTByTW1jNnR3d2NnR0RxUDBxeHYyWU1CSUs5MEZad2JqSGF6ZUxHZUNtZmFQaTJZZVJVZ1B4MkZ6V09QMWIxaUNHQmVzTDhvWVA1Ty1UbHgtQnRrQQ?oc=5</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -997,7 +1000,7 @@
       <c r="F18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1007,17 +1010,17 @@
           <t>Another year, another IPO cold shower for investors</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNeEhzYzQzdjR5MDJCWkd6Q2VLdEZzbzRoWnNOcXFlQjNfMlV4Q0NQRjExMlNhT2NPcnRBbW1sZUkteXo4N0dGaHNNeGZJOEZ2aXFvdmZiN2V2QzdOMzFteFRnY1RVRm1rQXltWmY5VFZOdFVNNVpudVp1dTlrcFM5b1k5SmlWQllDMVFXSjA4ZVpSZHgtV2JpWDJ4SkFRbVE?oc=5</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1025,7 +1028,7 @@
       <c r="F19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1035,17 +1038,17 @@
           <t>Priceline Pharmacy franchisee sale narrows to final four bidders</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNR294am9sYWNiQ3FVT1B6YlV5ejMyeHAyT0FibTFVbU5pcjZyaVRyazEzbFkxd0lrcnpZNGpTYUx4Ykl1Xy1sZF93M2Nid19ydUFwbUJ3ZHozaURaNkRoOE9OMnRBRGZfQVdCVWZCaVhhNnZSRjlwYUdDVnp2WU9HUkJxbE1QMV8zdWxYRTNBQWktR0xSOFU4dmtXZWk0am9SSU92NWp6QUZmTVU5TzJEOEJNak5fQUtN?oc=5</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1053,7 +1056,7 @@
       <c r="F20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1063,17 +1066,17 @@
           <t>Private equity gets better image of Qscan</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxPRjVmT0hDRjZLblB1VHdPRmRGeXhKdDJHdWxDTzV4RDZ0VzdHaUFfOVlnZjRQMWhKcWMxby1oRDR6N2lQZkI1UDE1REppS3c4LTVmU3p5b2wtblRCWnhNajFnZGNHaGRJUHFMUGRtTHAyQmIxOHhNNTgwRWVSeWp6ZWRxbUY0WVhiUnhMRUpDLXNwS1RuelJldTk0Z1R0WHg0XzNXNTA5Rk5TRFZhU1RNVnN2TlZuaFE4OWtIYXQ5a2VGSW1UWmt5Rlc4Q2lIXzF3YlkwNVhfUzJDV0dQdVAxa2RKc08wRGR6TlB2Vi14QV9BdlhyaTZsM2pEVGZycTjSAYQCQVVfeXFMTWpnb0lWQmZ6MTFnRGhWNTNqczk1TWhTcUFEMVpDNnJ4ZWVxVlRUODhJXy03NHdGZVJlMmhyUHM0Nlh4NlZtTzRhQ0xxRDFLVHNzUVNfbWxhS3BLUEQteEMzZHRrc0F1eFRzYmxVNDZlSURyZDB5bF9wQTNRRU5yZEs1Z3pFRTdwcFBaMkNlN0JvT1NEYkFWVUJNcHJqcEM5RVJYa0JFUVl6cThyQXloaERzQjhkTUVPakJqb0hzNVlwSWxNS0dmZkNFSG9Gb3dNUnVvUnV0d3MxSmpzdFZKTHJ2RTQwRUoyMEVLLWMwT1NnOHdXVl9lRXNDWEFndzJFSDlZU0o?oc=5</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1081,7 +1084,7 @@
       <c r="F21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1091,17 +1094,17 @@
           <t>Oporto CEO’s first year reshapes brand and network strategy</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D22" s="10" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPY25mNTJfT3FiVlBPZE5CcVNkR1UzR2xWaUtJSmxhU3EwcEMzQi1ISDFSajlCQWk1UUJpZVJ1Q19ZV3Jjd0Noc0l3OExpMXhSQUVVdHhCLTBlOXNoZzA3UXZBdkR1VHBvMmVsZkNhUFJndm1DdGpnX2w0ZVViU2phZ1RmYXY1SlhwUnhKSUxBQVZZUXpqNHQxQmo0Rk1iV0g0OW9qUS16eWRSNW5FaW1yQQ?oc=5</t>
         </is>
       </c>
-      <c r="E22" s="10" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1109,7 +1112,7 @@
       <c r="F22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1119,17 +1122,17 @@
           <t>The Melbourne restaurant our reviewer grew to love</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOc3YxQTljcHJXVWtRX2ZGM2lpM2pILWNwSFg0MFJrNmNWX0ZxRG9nV0J5N19qRWh4U0hPXzNmVVZwWk9wT2kzaFNrTlV3NEQ1Q3JpaXVIYlBHb216Q3VYVWdSRXMwdDl0SmYzdnRlSDFUYVRmRGJyZVlRZDJKTHpJOUctYlF1RDZSYjloY0hfZy13QmFTLU9UNjkwTHc1bjlGcGxoZ0ZLVU1GWTctZkdLZU9zSGhEZEpKbXJnaWJfZjd2OWs3?oc=5</t>
         </is>
       </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="E23" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1137,7 +1140,7 @@
       <c r="F23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1147,17 +1150,17 @@
           <t>Crescent Capital strikes Benson Radiology deal for close to $400m</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D24" s="10" t="inlineStr">
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOLTNrWG1ZZlFoU3pDZ3E2SEgwMlhzQkdtQUYzaHZTZmYwU3ZhMnE0dlkza005VkZmZ09NMExlWDVncnBmYVVISXJ6X1ZjNHhpM2RnSlprY1dnbndJNUczcDVtNXNRY3pVNW12bm5rUVdqVmR4R0JlVHFuN0RwTlFkR2xrbFFpSl9jcm5oSjk3aFM1clBSVDhnbkhoWUREeUhsbVpvQW90d05xOTdfOV9nbW5POFdmelJkVlpsUlRuYl9odmRNVUV2S0pCMFBMTS0tcVhGVGFYU0h2d9IB3wFBVV95cUxPWEs4R2pxdThPbHJHb0dBT183SkRHTTlXNzdWazcxdkd1eGx2VlAyM2VVbEtEbWxTZ1R0TlBFRmRMZTFoalgxSmVVRUJFR0c0RFYzZVJFODg3dWxicU9pOHppeFhjaVp0WWlyTnUzV1dyZXdkMHBDVHI4LUVQdjc0cWpheU55NTlvdWdCZmVoODB0Mm5fbGNCTmQwLUhMZ0psQVpzb3BEUnJpSkRnOUM0c0VCdUp5N3g5MkhaM01vTHJ3NWd0ay02UXZUUG9nVkxicVc1Z0xjWGhjUDRDVjlN?oc=5</t>
         </is>
       </c>
-      <c r="E24" s="10" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1165,7 +1168,7 @@
       <c r="F24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1175,17 +1178,17 @@
           <t>Dual-listed giant Capstone Copper flirts with $600m-plus carve-out</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNcVh4blRkQnoyaG1TajhVV0lrOEJRaHdTZWtzUnJHaEdaSXNRWThGTHlVdGl4dGJ1cTMwZ2pLcVNzUXRYNlZzVzhvaXdkNGtVUG0wN0FrMHB0R1I2Ry1jcEgtSWUtajI0cTFMRTlfdzBuMWtrZmJOLVUtMkl5dW85dFp6dEhEOHhTNzdfOFNFSGtlT0MwQnRlY0VhcUZBNE9RYzhQcDdOQUFnYkgzd0V0N253SQ?oc=5</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1193,7 +1196,7 @@
       <c r="F25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1203,17 +1206,17 @@
           <t>Guzman y Gomez unveils a new menu under $4</t>
         </is>
       </c>
-      <c r="C26" s="10" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D26" s="10" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPMjRjRTV2a3BJc3AzdDNOQktoYjBvLVZSODVsc3lKQ3pET0lxUlpkc05NcVlKRlZITjVJbjkwLS1DUFJNMGJ1amJKTlp3S3VqMWJaU3YtUENEN01rUEJiV1FNZTRXYjcyV08zZzlxNDVOSlVOTlJDOGV3QzBQcUpKa2Zab1ItNlI3ajZVVTF3?oc=5</t>
         </is>
       </c>
-      <c r="E26" s="10" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1221,7 +1224,7 @@
       <c r="F26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1231,17 +1234,17 @@
           <t>Can Sydney’s burrito king conquer the $676b US fast food market?</t>
         </is>
       </c>
-      <c r="C27" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="inlineStr">
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNM0ZFcUpLN1dUZWUyaE1LMnNZVGlEbkNNQUQ4Wmd6QVFlTy0wZDVHdnlja1gzMEZTbVpKU1Ftb3VKZ2pzajcyWU16NUtUTmR0TlZMOVhMRUNqZXZiX2d2NWY0YlJDOFhhYUE0SkhMRUprNndXak8tWGdERU90cmMxTkFjcFFVSTd5VlZ3NFVKOXN3M255MFhzZThmbi1VUGMyQ3E4d2pYcFlJckY3QlVBdVJJeF9qUQ?oc=5</t>
         </is>
       </c>
-      <c r="E27" s="10" t="inlineStr">
+      <c r="E27" s="11" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1249,7 +1252,7 @@
       <c r="F27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1259,17 +1262,17 @@
           <t>Drone maker Innovaero prepares for ASX float, taps Euroz Hartleys</t>
         </is>
       </c>
-      <c r="C28" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D28" s="10" t="inlineStr">
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNU3JrejNRZ1VBZVNVV29NMkFPVmRsWE4yMVZPcjk2aUNUTHFJUGFyQ1VnZEZiZlIzQW9VVzRNNDNRR01jcHo3X0tqZjB4bzhMTTI0Y3BwYUh6OGRUUGt2REIxV09oRnJoVWlVelZWaUlWUmlPQ3dJdi1TejcyaXB1Z0x1MEJRSlB3SGMwVGdXaXJJNm9TVllPOG5JZC1feEV3TVhTeExGeHR2RHFIWlVCOXh3?oc=5</t>
         </is>
       </c>
-      <c r="E28" s="10" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1277,7 +1280,7 @@
       <c r="F28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="inlineStr">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1287,17 +1290,17 @@
           <t>Bain flaunts Estia 2.0 as IPO roadshow gets under way</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D29" s="10" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNTEN1cGsxNDN2c1NqUzB6UmJ4TFl0NGZjZVN3U3oxMlVFWTF4WUZLQS13dUxMV0N2ek1XN2VURTNVWms1NjdXSm0waEdaTXQwdTdWY1MxZ1V3ZnpEcVJtczdOWGNNZ0RQNzRZLU1MTTgtRW5DZkctbXBGMmVXVXdPZW5pNThiRHEzWnB2eFZzTFZTb1ZkeW9LendkNDd0cXRid05ZSGZYbW9NZXdOLVZWODdZU3hVcTA?oc=5</t>
         </is>
       </c>
-      <c r="E29" s="10" t="inlineStr">
+      <c r="E29" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1305,7 +1308,7 @@
       <c r="F29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="inlineStr">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1315,17 +1318,17 @@
           <t>Carl’s Jr. Australia unveils nationwide freebies for Happiness Day</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
+      <c r="C30" s="11" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D30" s="10" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNVWgwdjU1NDFWalBfMTFYX1dQOWNDbG1FVUdlcS1LTVlHZVRRTVBWTjhSMnpkTXRXNlFJdllGQUp5Mm5ObWpIazd1d0RJa3QtdFBZN1hOenBmVzBEU05wM0gtNUxPeWpsYkxyVnhWWFFOU2Y3R0tXcmNkeWhpWDh2eDZBdjNCMHhuc1lHYTZHblBPVkpfRXpKd051UWlNc1hm?oc=5</t>
         </is>
       </c>
-      <c r="E30" s="10" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1333,7 +1336,7 @@
       <c r="F30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="inlineStr">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1343,17 +1346,17 @@
           <t>BHP and Woodside appoint new CEOs in major mining shake-up</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
         <is>
           <t>ABC News</t>
         </is>
       </c>
-      <c r="D31" s="10" t="inlineStr">
+      <c r="D31" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQbTg5VFJLbWJfcy1uV3ZReTJkTndzX01qZ2MxNWkzaWZRckNLZUR1Y1VsMVRNc2FySC13U0NzalFEb3k1R3BaUEhfcTV0N1M4Q1dpSlo0YXI0UFhrMGRab2RiYV9DQVNVX01ycFc5ZFZrZWZqc1VRZXoxLVEzSDJLclJLSWg5bzN3R1I0bG9lWjVDaHE4?oc=5</t>
         </is>
       </c>
-      <c r="E31" s="10" t="inlineStr">
+      <c r="E31" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1361,7 +1364,7 @@
       <c r="F31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="inlineStr">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1371,17 +1374,17 @@
           <t>Next Capital sells Enviropacific unit to French waste management giant</t>
         </is>
       </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPR3lFbERLR2FtdmJUU3BDU2thZk00YmFHRFhXR2VBVXhQSURTeE5ONVJKczBwbzlFMnR5cmhxMnM0bzlJbWo4SXl1dHpqYWxxMUJBRjZHVUtab1RYZjZMTnpGc3FzMWQ2NjNEdGU3NTZwa0diM1lJS1haYllwTldLZlpZbXp0YzlxcDh0ekcwTy03dDdPcnk4b29HZVdqbHhZY2JPR2drM2puSVpjUzZkVjNpZUE4dVMwYlE?oc=5</t>
         </is>
       </c>
-      <c r="E32" s="10" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1389,7 +1392,7 @@
       <c r="F32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="inlineStr">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1399,17 +1402,17 @@
           <t>Future Fund private equity and real assets chiefs head for the door</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D33" s="10" t="inlineStr">
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPUHNHRFhFMVdwVld6RFRZUFd3QWNOd1kzeS1QdnJxMERFSnE5LTdZcDhDYlVGcWZMeWxlR0FSRWF6YkZoQVZrZU9TQ1E4YTEydUJnOFE3enV5Rmk5UnF5VEdYZ1FMUWpKVjdjMlZZUGFsU0tKcV9Vbl8zcHp5aVF5Z2JMOUZocHJqRXNRaEp4Nm5CbDM1WkdIMHdQS2xqQnE2Tnh3?oc=5</t>
         </is>
       </c>
-      <c r="E33" s="10" t="inlineStr">
+      <c r="E33" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1417,7 +1420,7 @@
       <c r="F33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="inlineStr">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1427,17 +1430,17 @@
           <t>‘I actually started to die’: the new billionaire’s epiphany</t>
         </is>
       </c>
-      <c r="C34" s="10" t="inlineStr">
+      <c r="C34" s="11" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D34" s="10" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxPblkxbHVrdnVKY1pqQzNyWGNMZm9UYmY3dzlPaGQ4Yi1tc0U1akhrVWdIaXBpM05aZXRwTXE1eDBITlZpbDkwRXNrWjJ2YXBzX0VCY2JSLWhrVmpjSTE5eE5rLWgtc2pRZEdXbmhhWU1KeFExZDBGS2pjSkIwV0FGbndBZVAyQkg4WFRsengzSGYyZkFfQnJsQ18tUHJGNDd2T0pzZElPSVJTQkl2Rm5QTExJNHhmU2dHOHJGdTdzU08yNHRtd1R3Q0cyOF8taDktQTZvVXVBVjN1d0NHMmtFOHBWZXBFcUFWa1IyWGNDTDZUT3lQSXJHOVhxTFQ3b3RH0gGGAkFVX3lxTFBZQ3BFQWl5dEwwLW5yVWJuMU8zcXBPdE9pamRVSWVkbWNyVzgydGVOaDBROUN6RlBDbjdld05DVmZyb0R1eEN0UERubzZRU2NiMTQtVV9XNS1wYmlvZ1paM3RaOUlrTzJka0tXVVJEamFESGlSdXg2bDk1aUdhUVhBcXpnN01fX0Y0cTNvcm5DdEFFLVVERDFKTWxKZFR0UzAyblJqVHBua2JoYUdzeUNMb053ZVczWUFQU1AtVHV1d3lSSDFfZFh2cEkxSGw2MEdicEVsb2pLQ1RuQmdaRl9xNUROS3pKR2s2T2wxTTZ5bEwtTUNQNU04djFHTHlPbXVLSW9YSUE?oc=5</t>
         </is>
       </c>
-      <c r="E34" s="10" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1445,7 +1448,7 @@
       <c r="F34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="inlineStr">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1455,17 +1458,17 @@
           <t>Ironbark shuns private equity as it hunts for cash injection</t>
         </is>
       </c>
-      <c r="C35" s="10" t="inlineStr">
+      <c r="C35" s="11" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D35" s="10" t="inlineStr">
+      <c r="D35" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxQZWFaeVhldi00VkV5ZmEtS2tjcWdFWG55OGpCX3IyN25Rb3ZFV0ZKVm1aSE1WbThoYVY4ZEdfODVGX0RaUDV2Ul9HS1JQMDFCT05Fc2FaU0RINTMwbDRveWFsOFJSM2ZqTU9tVGxJSEl2ZmhhUHFHT3dqYkk5TUtvMUQySnZzTWw1MzFNWl9aVzhkSEZ4Q3YyWjRMUmpIdmJkdUVKWE54Nkt6bTd2dGFSUFoyNkgxTHh2TGVGak9ja0dFZ0xQM2g0S1lmQkZiWWtUcTVNdHhBdC1KeVRQcDA2dnpmeHRkWEnSAewBQVVfeXFMTWtYRDRSaHNULW1HanowRnpMdFF2VVMtZW1SV2ViZXlGaW02WlIwUzRZMGg5WDNrOUR4eDlGOEt5eGlqV0pfVDFhb0JEcS1faEJodWxyRnB3MkozOVJyT3NvM1I5MzdDcXNnUFNSdkRDamUzZTRQYlk0c1VIQUNMZ2ZzOWVCb2V2MC1aSTZLWkFkbW9GYk05b3RmN1htWENTeDh3SU1WYWJMcWx2eGUzZmwwVXF6czlnRGdXbE1vRElyVG0yM0ZzXzZ5TFh1YlRGNU9MQ1p3NnVZSFB0M0xBcGlueVZILXlVaXdqUkU?oc=5</t>
         </is>
       </c>
-      <c r="E35" s="10" t="inlineStr">
+      <c r="E35" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1473,7 +1476,7 @@
       <c r="F35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="inlineStr">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1483,17 +1486,17 @@
           <t>Minister leaps to fix food chain</t>
         </is>
       </c>
-      <c r="C36" s="10" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D36" s="10" t="inlineStr">
+      <c r="D36" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxOd2NqakVWRnQ4anFZNkl4Zy03MkloX08tUkktRTZqeEtQWFZJeVhkMUJIb0FxUjc2UjhCQ3MxbmNxczNxblJIZ09IeTBGNFM4Wkh4ZE1qNkhJMjIwU2RtX1JxcEV1Y0NjWXF6eHpVdTN4ZUlYMGIwcDJzMXZMTk94VzFlcjhpcVZVSTJFMjhsQjVGWEJQYTQ3aTFyNmNEZ1F1b3NGTWd5WnFJWmxXSTJ2NlRLcjJHNWkwaTZ2YVR6S0w5WVo1Vlg0VWdxcWZoa3VaTmcxY2NVcnR2bFRWNGNvZ1M2Tlg5NzlvVXZFZm9B0gHzAUFVX3lxTE1uNERoR3p2dXRIa0g0RXI2MWR6N0c5U3NGcjFDQVMtdEpyNDI2bk8yOS1qUnFOazdiODl0Ymo5R1pwRVJ0UFFVdzlhYjRDSUFCU0FRak4xcVVrTHphdTdxcHNIMnEyRVZud1FURmh5T0JLOHpRM3lFbDRuRnZMYmtaRnRFTXh3dkszTFhFUmZlRmoydnlEbW1fZTlmUzh4NXNyeTZTeUhOSktvclJVc0NTZTVYMkdJZEUyY2RmVC1kQ1hwVEloSEtVMEo5QnNTUXQyME5IN1BPd1NOS3oyR1JtMHBFVTZEbzhEQmdrWUk1ZnZVTQ?oc=5</t>
         </is>
       </c>
-      <c r="E36" s="10" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1501,7 +1504,7 @@
       <c r="F36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="inlineStr">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1511,17 +1514,17 @@
           <t>‘Brace for swings on every tweet’: Investors bamboozled by peace talks</t>
         </is>
       </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D37" s="10" t="inlineStr">
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOczZHTWFmTW9FZ1ZwSnc5Z3ZacGpsVDQ3LWw1a1BFT0tjRkphek41MlhNOU84emYzZUVwNV9xM0hyc1FUR0NHck14Qnh6c2JvQks5ZE02ZTNLWDI0dy1STi1HbDFDWW9yMDhGQXVVVzdkMzFXcnNNMVZHVXFMUXUteGtsVGhPVmhLcVZPQzlhTWNoYVVRMHF0cFhybWxzek13Y3ZjcjlXWjZJM2VYbm0tTmk4NExLQzQzX1ZPMVlhcnJxQkZx?oc=5</t>
         </is>
       </c>
-      <c r="E37" s="10" t="inlineStr">
+      <c r="E37" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1529,7 +1532,7 @@
       <c r="F37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="inlineStr">
+      <c r="A38" s="11" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1539,17 +1542,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C38" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D38" s="10" t="inlineStr">
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5</t>
         </is>
       </c>
-      <c r="E38" s="10" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1557,7 +1560,7 @@
       <c r="F38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="10" t="inlineStr">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1567,17 +1570,17 @@
           <t>Wirth’s Myer rescue mission is caught in the eye of the storm</t>
         </is>
       </c>
-      <c r="C39" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D39" s="10" t="inlineStr">
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNTlQ4NDRnWE91VG1YNENpSTUxNnBjZkljOGdYaGV0aVB5dkVOaEJ6SjZ1bVA4NXE1S1hjV1NjcVhQTEVpWEVNV0UtbzhQTFZLOWxIenZiaF9QM3F6bmJYRy1lbXVMczZ3TnBHNy1aLUtVcnBDdkl4TE0zRGN4U0FwSjNPY1M5S3AtdUQ3UUNmR0x4MlU2YXRuUDJEUm01SmZWakx2UjFvY04zRHk4Smc?oc=5</t>
         </is>
       </c>
-      <c r="E39" s="10" t="inlineStr">
+      <c r="E39" s="11" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1585,7 +1588,7 @@
       <c r="F39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="inlineStr">
+      <c r="A40" s="11" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1595,17 +1598,17 @@
           <t>‘Darling, I’m not going anywhere’: The rise of at-home care</t>
         </is>
       </c>
-      <c r="C40" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D40" s="10" t="inlineStr">
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQS2k0M2otaldpNVFXdHRTMVNtZVhyUDV4VTNIcE5FSnFRaHNubGNQQzBVbllnNTktNGhrZ1lndzV5V1FpUS01SklRaTZmZHJkRzVsQmlsdEVmenZ4U2x6U01NeXdIMktBUW94TUE3R3FoLUxVcVhsVFI0SjVQVUFaZldnd3prMWMyaVRWX2J4aUdfQ25KWHpaLUlqSnhvQmM2TTRRQldGbm8tclFYRDA0TVdnU2g3QQ?oc=5</t>
         </is>
       </c>
-      <c r="E40" s="10" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1613,7 +1616,7 @@
       <c r="F40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="10" t="inlineStr">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1623,17 +1626,17 @@
           <t>Iran targets Israel and Gulf states as Trump looks to calm markets</t>
         </is>
       </c>
-      <c r="C41" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D41" s="10" t="inlineStr">
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPLXBITXU3WTRtc0NYdnhTZHFaUTBCSXdldTBuSHliTlY1dlJONW43Qkd6Nl9pNmY1eDhzaHZoX19xYjBxMXR5UEhkVUg2M2k1MmhuVEwyY0JxbnJyemxVYUZjbk5BbkN4ajhPbW9ZeDhlRDRYTW1hN3k2d084c2djMEJUZTV3NVdPbllKUmFlU2JsaDV3Zk9CVFF0VDFkV09JSloycWdOUlVrREptQTJfa25LUEx5djA2SjNMMFY0RjM?oc=5</t>
         </is>
       </c>
-      <c r="E41" s="10" t="inlineStr">
+      <c r="E41" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1641,7 +1644,7 @@
       <c r="F41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="10" t="inlineStr">
+      <c r="A42" s="11" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1651,17 +1654,17 @@
           <t>Meet Christian Louboutin, footwear’s most famous billionaire</t>
         </is>
       </c>
-      <c r="C42" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D42" s="10" t="inlineStr">
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPcXdGd0tMckYxbjZ5TVJmQ0Q4NFl2RkhHMHdlZDZsdGZ6cVQ0cUpaLWJTNlVoc2ZOQmtXNlFTRnJVMnVDTGc1NFNZN2g1VnotQlNQbzhlM1BJV3ZwQktOcGtac3RwSHRLZkR0b2l0eGIyVVlYdHJrc2hpT0pJbDR3LURPTnowZk54LThObndtMVkwV2VWQkluNVlWY0p4QVJGbE1hSGMzOW8zdkJZOWdocEZQWFBhTllNR1ZBSEg1TWRXUWd3X0t6TVcyY05PM0pF?oc=5</t>
         </is>
       </c>
-      <c r="E42" s="10" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1669,7 +1672,7 @@
       <c r="F42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="10" t="inlineStr">
+      <c r="A43" s="11" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1679,17 +1682,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C43" s="10" t="inlineStr">
+      <c r="C43" s="11" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D43" s="10" t="inlineStr">
+      <c r="D43" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQbHdYM2pSM2xkdmZ3OHhQc2tVUmhzclJWaVJ0aEwtUkNBR0ZUd3p1emF1M21jbTF1ejlKSkdDMnotcVNjZE1CYUlKako3WXR4MTJhdWNlSXZMbTBYanlmTWFzRGFIandXRUQ3UjN6SEV1bThvZjN2bDY0eFdpaTdMODN6TGFTdE5rd05TUll3MmNfTDhkQldoNDIwVlpoSl85aVRwcTd5Ymh3TDl4enZhZ2p4OExGY1ZaOFNEWFBB?oc=5</t>
         </is>
       </c>
-      <c r="E43" s="10" t="inlineStr">
+      <c r="E43" s="11" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1697,7 +1700,7 @@
       <c r="F43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="10" t="inlineStr">
+      <c r="A44" s="11" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1707,17 +1710,17 @@
           <t>Sembcorp Picks Banks for $2 Billion Alinta Loan in Aussie Push</t>
         </is>
       </c>
-      <c r="C44" s="10" t="inlineStr">
+      <c r="C44" s="11" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D44" s="10" t="inlineStr">
+      <c r="D44" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOdS1aaXZjT2VnSDl2TDdzZ3NfRElDWXdUXzZQYjFQMEZJOGlpaE5CNGdQMlZ2UFVHbUtfOXF1ZVBReExrdF85M0RWLWlBY2Y5dlRtWVdXLWp0Y1VrRmF4UGQzVUhxaHA4UHd1SUdFV21QcVFITXFHRlhzekdSUS1PdHlYRjdUbUQydU8wSktKVHRJQ0NaWE9sU1l6YXhtSWtBd3RwTERacnV4VzB6YlFhUE1QcXNDVXVESFcyeWY3cGhHUkRJcDhrYUtpTEY2UQ?oc=5</t>
         </is>
       </c>
-      <c r="E44" s="10" t="inlineStr">
+      <c r="E44" s="11" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1725,7 +1728,7 @@
       <c r="F44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="10" t="inlineStr">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1735,17 +1738,17 @@
           <t>Navis targets June for $1bn-plus med-tech auction</t>
         </is>
       </c>
-      <c r="C45" s="10" t="inlineStr">
+      <c r="C45" s="11" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D45" s="10" t="inlineStr">
+      <c r="D45" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxPNHRXaU5tNUVkd2MtcTg5M0EyQllrM0owMkZobGxLaUJxYUN2MUg0ZkdKdzU2YmxfanR3QU53cHZzNDI1WXgzRUcxOE9EZlluNmtNRUUzTGJPRnpfVVVOeFM3bFRNQmp6VHFBdi1mTnU4UDBvOEpMaHZPNXFtdUIyTlhuRExIVElSeVRUMGxjU0k5VnVxaWFfd3htWngydlhuR2E5aTQ5VW1LS01ac05rMGZoVFdOZzVyTzFhUDVsYkNrc0VQZmhubERSaTNwelk3WEhYUjF5d2ptMktYeEhzOHpWazFQZXphd0xfUFdhbkVGMVR2Z1dtVtIB_gFBVV95cUxObEwzeHd6RmZtNUp2dXVVV0plOVQ4WlNqQXNJU0thd1BEWE8yWkxxVTZjTkpsVGxxWGxpQzN0OERZbk91ai1fZkdtc0JoM1h5NERLTVdDbVJ4Y2k4djdQcWlVcDF6NjMyVDQzZWMzUFZxWjVRWllMZHVSOF9jQ2U1REFfNUlhM2EwYloxb1MwSTJjODdWdlZwX2h2N0xiQWNhallHUTNPZEtLaXhsY3dBZy0xM1VITXhLUERXS1JxR0R3OUpBTVBPZ2dPZTRUTVpvbFBNMjFUSTJuWS1XLWdhUS11UTRzVTVqaEhfMDhqWHlTMlJGekU2QzJVcFdodw?oc=5</t>
         </is>
       </c>
-      <c r="E45" s="10" t="inlineStr">
+      <c r="E45" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1753,7 +1756,7 @@
       <c r="F45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="10" t="inlineStr">
+      <c r="A46" s="11" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1763,17 +1766,17 @@
           <t>ExxonMobil eyes New Zealand market exit</t>
         </is>
       </c>
-      <c r="C46" s="10" t="inlineStr">
+      <c r="C46" s="11" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D46" s="10" t="inlineStr">
+      <c r="D46" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxPanlvR1V1eVVpdmYxNVNGMnd6UjJFd0J6Zk9IU1lhOW1GbmVTcjY4QkJCYkl3Y3NOU25VRTBUekwtS3plV0NVdlZtOTZZRHJWZ0FVdDl3S05aMlFWeEZiYzdwYmQtVnJxZEw0NktHaFZMNlZkUC16empqRGxxMEhhZGwxRzVEek5FelB3aE9UWFhGQW42b21MRnJHUXV2ZGJYUXJIMnVFWGZsSnEwazNGNUdVcjVoekp0NEZCN1J3cTlaZldFa1pMUkJTbVZYeFljVkRqQmlZV1M2aXh0ZjI5dEI1NDB0UElPUERsbUljMlA3OHBnYmtJTXFWZWkyUdIBgwJBVV95cUxNWFBRQ05GUDdwTWJ2ZVFJUS00ZUh0QkpZQVNNcU9JYXRTN21sMS1VZTlOSTh2LVFuZHh6UVk2djlrdWFsd3MwcDFCNmhwUlVLTlpjVF8wSmt1YnBWRE9tNVpKQlk2YXJWdmwzZWlLX0xpaWxSMUpsX3ZjYXhmRmE2YlAtSFJGRG5pQnVmMnViQXlsVFV3OU1hZFVrY3ZITHQxcTR5UkZ5U1pReHVJMGZGM2FCZWliSFZQZmpVLThSdExWMW14OElodmVVSC05SUh1d1hBenJoY3BUZGxoM0NTbTExdERmM3pjZGd4VzgyV3BNOG11TElBQ3NsRGhtSEc3YzJz?oc=5</t>
         </is>
       </c>
-      <c r="E46" s="10" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1781,7 +1784,7 @@
       <c r="F46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="10" t="inlineStr">
+      <c r="A47" s="11" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1791,17 +1794,17 @@
           <t>PAC Capital’s Clayton Larcombe charged with assaulting wife</t>
         </is>
       </c>
-      <c r="C47" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D47" s="10" t="inlineStr">
+      <c r="C47" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D47" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOLXNDU2xjMWpyeEZwWGwtZkV0TjNSbGtWS3ZidUo3a0dvV1hrTnJiVXBXSkJNWlhXYXFHZkNTa3g4a1ZfMjRPM3BtWTZUNGg3S09kbGI2TTRGd0Jkc1A4WFAycjlpVC1URjFvNnBraWprRkhaT0VOWkh6N0xkUjNXNUw0dGx2N1JtTDVsREdtZDhraXVsSkxhR2ozamFUSGR5VHBBRm1Zcmx1c2RDaUIxQkVpeUpfWjFNeTRLWVRtYjluZ3ZncGZIMQ?oc=5</t>
         </is>
       </c>
-      <c r="E47" s="10" t="inlineStr">
+      <c r="E47" s="11" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1809,7 +1812,7 @@
       <c r="F47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="10" t="inlineStr">
+      <c r="A48" s="11" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1819,17 +1822,17 @@
           <t>China touts itself as ‘harbour of stability’ to global CEOs</t>
         </is>
       </c>
-      <c r="C48" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D48" s="10" t="inlineStr">
+      <c r="C48" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPUzBWeVk0elBOZ0l5QU44TUJvU0RvSmtPdmVyT2VuQTczaEdzbkktT25ZT2Y0Nzh0bVBhQW96TUhpWkdEOEJMVVk2UWxLOENKZGk3X2tQcDNsWGZtU0JkM2U0N3VfUWFBclhUSUZya0NwRTJOWmZJdWlhT3JtY1EtSkJ6TmlsV3dzOXpDaVFMNlBaa3RfRHBjc3Q0cjk0eVdPV2MwcjlHNA?oc=5</t>
         </is>
       </c>
-      <c r="E48" s="10" t="inlineStr">
+      <c r="E48" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1837,7 +1840,7 @@
       <c r="F48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="10" t="inlineStr">
+      <c r="A49" s="11" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1847,17 +1850,17 @@
           <t>Eyes on 3D Energi as oil and gas giant Conoco flexes buy-out rights</t>
         </is>
       </c>
-      <c r="C49" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D49" s="10" t="inlineStr">
+      <c r="C49" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWVU1QmhTUGFkYlpTQkw1WUFPTHhmbk5lbnE4T1haQUswSi1ITHlhVmhyM3ZYS3N4cVd6ZkwzdGdhT1lvM1JJek4yLXFpSWoxUnRtR2JRLTZWa2dlTDVTakE3b2xvazFWX0kzRHFZWVB4OUh0XzFFd3JVSVlfelpVa21qTldCVHdvcmJYcGNjZ1RrdElWS3Yzck9KYzRvbzloWkNqMnQ3dmtHbzNuc21ZSXNYeEFlZw?oc=5</t>
         </is>
       </c>
-      <c r="E49" s="10" t="inlineStr">
+      <c r="E49" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1865,7 +1868,7 @@
       <c r="F49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="10" t="inlineStr">
+      <c r="A50" s="11" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1875,17 +1878,17 @@
           <t>Blackstone tempted by $900m payday for Sydney’s JPMorgan tower</t>
         </is>
       </c>
-      <c r="C50" s="10" t="inlineStr">
+      <c r="C50" s="11" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D50" s="10" t="inlineStr">
+      <c r="D50" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxQNEZTZjY0S2YzcUxsb25RSDk2NHd1N1VOVlpMbi1JNGEzbUt5ajlYZFhvLWNBTkNQVXNuWERfTkl0Z2o4R1U0Zk5jVE1FTW5TTUJGZnNJc2NqMm1fT2dmYTVwRGU2TkZ0c3BjZVBGS29fWFJvZ2F0MWNLa0pYY0RNME5xYS1vOGZmMDVBcDBaLV9MWF9od0EwekFyb0ZCOEdkNTFaN3ZXckJwd25zS0FsdzU4OW1UODlueGNyZVBDSDZkeHQwelV5ZXVDVlcyUkhKWDZfVlRacEJHSElmNnhKSXk4ZHJHWHhPTEV5NGNkcmhyU0hjV3J4dVBXbnRGQdIBgwJBVV95cUxPME4ySFF5RWNrejVlWW1yeW56N244RGpyeVJUZEgyTjFNcE10YjVpMmJyeWsxTENzZFhPRlpsbl9pVXl0NGJvUlZFT216NE1KRFNwOHVZVXMzanNKNXFmWEdsMndsd1cza3NTTzUyUUZfaDEyWHJwZEtQbTdJRmkyU3A0RGh4QlAtT1lRVXk2SGoyaTI1NUpwVExYSkZJNmVFNjdXTDJTNURFOEh4Y1dnUDVGdjBpaDlWVWJtUHZiRDdGTmE5R1R6TDBwWFFnT2MwQ1lmT2w5bDF6eVU0R20tYnpnT3JCZlJod2s0UndyZTM5M2xLZC02a3E0NmJRdFV0Qkow?oc=5</t>
         </is>
       </c>
-      <c r="E50" s="10" t="inlineStr">
+      <c r="E50" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1893,7 +1896,7 @@
       <c r="F50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="10" t="inlineStr">
+      <c r="A51" s="11" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1903,17 +1906,17 @@
           <t>I-MED attracts mystery suitor as Permira weighs sale or IPO</t>
         </is>
       </c>
-      <c r="C51" s="10" t="inlineStr">
+      <c r="C51" s="11" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D51" s="10" t="inlineStr">
+      <c r="D51" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxNaGlwS3d5MGFMbEg2U2hnZUxMQmdqaWI4bS1lblNZOFhkSnRMcUotRkZMTjhFZkRUQWxUUDVtYml6TVAxUXkyZmx3SHRFb0gzVHRST2ZQUThKa25aWlhlcGprSU9tWktXZjZRaC12bFpkaVVWZHhIMERyeVNNWEswYTJ2ZHdnRFVRaFhod2U5N011TkQ0NG5MYVhoT3MwRUVZdVB2UVhKZExvdFIyXzNNUGt2SHJUanQxRkI3bXlLSlNJQTF4NXQ1YlZDaGVBM0EzNUhYQVp6NkFWRzU4bnRPWTgtXy1HVnB0ZlN0Uy1rY2FuWlNfN1U4WXVHQnRzVkNG0gGGAkFVX3lxTE1GaDJJdTJlOXFEZUtDTmdXMmsyLXlpaUxzQXpycHk4MTdHZng0dVczYWVwdWRzdFFCMlNLWkZpMm5Zd2RpN0Y0Zmo3Q1FOZFBZQlh5LVl6aVZ3X284UmpxM0pVRzZmMmpjaUdNWnJPZGV4V3lNai1CTllCcW5oUEVxaG0zejB5anc5YnJEZzZPT2d2QklCWjl2MjRBc25jUndqZkVadllKaUZScG12bEozT1NKUUJYR0pHTGtJZVc0ZHZLNHVSYlhzcTE0SkZmMXNlVGJ4YWJ1cThxcGlZTDMzRUMxLVM5VHh2OW5tRW1PT3VyRUhDbV8tRzUzVzRzVWZPZ2w1bnc?oc=5</t>
         </is>
       </c>
-      <c r="E51" s="10" t="inlineStr">
+      <c r="E51" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1921,7 +1924,7 @@
       <c r="F51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="10" t="inlineStr">
+      <c r="A52" s="11" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1931,17 +1934,17 @@
           <t>The stagflationary mix that has billionaire Solomon Lew worried</t>
         </is>
       </c>
-      <c r="C52" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D52" s="10" t="inlineStr">
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPWTh3S05XQWpTQm03WjhBT1pWc2cyOFRMd2ZraHhPUHlDRW1tWkZvdkhQWHE0MHVMRUpaOFRoX0JsYWhJV21nVkpIM2RBSmlZRUtEbFAydzZfOTh1S05oNEZPOGgyZDJRMS1uLThWYWRVT3VEVGhtYkVLN3J2OWsyX0VVdTUteFBCOVNKZ28xUTRPTk1SUkMxZ1NJc1B6NXRrUEEzOG01YnZOYjk2cWlFZA?oc=5</t>
         </is>
       </c>
-      <c r="E52" s="10" t="inlineStr">
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1949,7 +1952,7 @@
       <c r="F52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="10" t="inlineStr">
+      <c r="A53" s="11" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1959,17 +1962,17 @@
           <t>Oliver Curtis on Firmus: From prison barber to AI billionaire</t>
         </is>
       </c>
-      <c r="C53" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D53" s="10" t="inlineStr">
+      <c r="C53" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D53" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQek9VTlV1b2hVb2RoZ0Fya0REb3E3YlBCR2NYZldXcEh2VEY0LXg5bjd6RzlnZDI0OUJJd2cydTBwTm9tdHpiZ1lSMnhtcmJSYVRKbzJFMjdDaEJyZExSQVJVRDh1c00yMjFMaVlPdnRuV3VkTjNxdzFRbW1yeGltSF8tVXlJVXJzTEJXS2FTYkJTVkdKbmdPTTd6YzRtYV9nN0JzOVZNTzhUdUk?oc=5</t>
         </is>
       </c>
-      <c r="E53" s="10" t="inlineStr">
+      <c r="E53" s="11" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1977,7 +1980,7 @@
       <c r="F53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="10" t="inlineStr">
+      <c r="A54" s="11" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1987,17 +1990,17 @@
           <t>Three startups that raised $161 million this week</t>
         </is>
       </c>
-      <c r="C54" s="10" t="inlineStr">
+      <c r="C54" s="11" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D54" s="10" t="inlineStr">
+      <c r="D54" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNRGVZMF9DeGJjX29vN3B0blVoM3RKSlJJTllrMThKUDJNZzdPNFNnT2JyTElUOUYxMHlsUm9yM2dBQnZfaVNZblpqb3NzTXdHVlpQNkRqR3NBZHdzODdjN3RKMTZhSVRqUEM5d3JRc3F2OG9hWmZJdU5rakg4ck8wLXlMTnZSU0lNaERmQmswbkVGWW8?oc=5</t>
         </is>
       </c>
-      <c r="E54" s="10" t="inlineStr">
+      <c r="E54" s="11" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2005,7 +2008,7 @@
       <c r="F54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="10" t="inlineStr">
+      <c r="A55" s="11" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2015,17 +2018,17 @@
           <t>Iran eyes ‘plenty more’ vulnerable energy targets in costly war</t>
         </is>
       </c>
-      <c r="C55" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D55" s="10" t="inlineStr">
+      <c r="C55" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNLUN1MHlZaTNfVHhVX0RnTXp5QW83RmM4WVZkWW1PSnNaZF93VkY5ZF81anB3NDNmX0kyMkVSdkxNSURvSEh6enloWnRVcTlsR0JPTjVzNFR1YjRsSm52VnA1XzFFUlUtODJjYy15YWRRdWZZRkdjRXpCcEFSVURmV3VpSTFhTjVUb1d5bmw3NHNlT3VQZU9ieEYwM1J1TGEyZnlnWXNIWFJUMEtIOVZad0dxRWZBdw?oc=5</t>
         </is>
       </c>
-      <c r="E55" s="10" t="inlineStr">
+      <c r="E55" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2033,7 +2036,7 @@
       <c r="F55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="10" t="inlineStr">
+      <c r="A56" s="11" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2043,17 +2046,17 @@
           <t>Don’t take it personally: Bain Special Sits hits hurdle at Infinity</t>
         </is>
       </c>
-      <c r="C56" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D56" s="10" t="inlineStr">
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQRjdwTk0xTHVIRHNkdG9tVk1EQ0hiQjJ6dGcxaWZRZ0hZV1U4YjJDU0tnTUlWSkQ1S2dUTHJVNk0tNWQ2cVd4dkw0M25leXRreWJtdlBKYTAtNzRocTJUazh1dnRzSVlYZThySTBNVjg5X0xYWUxCMC1SelltSHVSUEV5U3B1bTA2NjAzMGFZLW1CNkQ3aWU0S1JxS0d0YmZiZjBKQVRNVUpzYno5R1pvbTBsaTM?oc=5</t>
         </is>
       </c>
-      <c r="E56" s="10" t="inlineStr">
+      <c r="E56" s="11" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2061,7 +2064,7 @@
       <c r="F56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="10" t="inlineStr">
+      <c r="A57" s="11" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2071,17 +2074,17 @@
           <t>Drill, baby, drill: It’s boom time for mineral and petroleum explorers</t>
         </is>
       </c>
-      <c r="C57" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D57" s="10" t="inlineStr">
+      <c r="C57" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNdlFOWld5ZWhPVnFRa2xidWlUVzluQzkxUTgxR0t0Rmg2S1BzNjdINnhwS3VLRkNjRVJLX0RHU0h4VFVRY2RfSHBudEhfNVNjeE50ZUxQenJNSlJtWFRlcnNsZm1iLXlxM2RmVDViWEtjNDloaTBhUDVxYkNfOWFCTjV6cExEVlFCMzNfWnVwRDJHYWxWV0hOR2V2S0VlV2NyS2s5cWNmREtWXzlMMDRQNW1tVlBOblp3SHBEVg?oc=5</t>
         </is>
       </c>
-      <c r="E57" s="10" t="inlineStr">
+      <c r="E57" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2089,7 +2092,7 @@
       <c r="F57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="10" t="inlineStr">
+      <c r="A58" s="11" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2099,17 +2102,17 @@
           <t>‘Wake up’: Fury as farming crisis looms</t>
         </is>
       </c>
-      <c r="C58" s="10" t="inlineStr">
+      <c r="C58" s="11" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D58" s="10" t="inlineStr">
+      <c r="D58" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNelJvMXFPX3MwUVRMN2xqbzE1MWdvOF92Zy02YmIyZW9SQXRNQVZsS0xVVG9UdkFPaTV6ZC1tV05SZWNqblNFZ3Y1VGNaVVBaaEl6aFJqQ09ONDVkNUs4TzNvVjV5eHNjUk9xaDRFZTM0alpuYUdvWGtLRzRhYXN5alZ1QWdsZTEyODdQVnZoazkya29WeTJZVmpxLVBCdWxfY0dTN2Z3WFZlSy1sVW44RDlvZFAzYlhnQ0N6UWhKSU02eF9iZllIU3g5MWtSbkJzZGxWLUxHNERzdUlLTF9VYmpJSTRLY3U4NlVVaDhmc09uOWwtUGtlb0I2M05DR1dnRWxGSFV2NEJXaEF4c00tN9IBlgJBVV95cUxOSzZ5NXZMTTlZa3BSNjZyTUxUMjRhYWJhN0hMa3dDcW9CWGstNnI5MzV5U0hJSTdKLTFwa2E5YUItZnFRbW5RbzVuYW91MmZaYXN3R25hWVpUbW9oUU9fVktPRHROVDYyd2dSLXJVZWQtY016bkVxY0VPbkY3Zkgtb1liWGMxeEpyYmloS1V0TVJMMWZaeWRZX3FQRjBmVzJwdkkwMEVDSXV1MTdReUhGZ0Z3dENyMEFkLUl1aXhtRkFLRFFXcEdMZzFuT3NxRDFMOGVaY2YzeXBQc09fY3YwcFp4MVczRVN3d3dJZWJfTFFscjF0cUtRWHdzTUptaHowNDhYWXZXTHhYTHNTdlZGUmNlamRTdw?oc=5</t>
         </is>
       </c>
-      <c r="E58" s="10" t="inlineStr">
+      <c r="E58" s="11" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2117,7 +2120,7 @@
       <c r="F58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="10" t="inlineStr">
+      <c r="A59" s="11" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2127,17 +2130,17 @@
           <t>Construction giant FDC road tests IPO pitch</t>
         </is>
       </c>
-      <c r="C59" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D59" s="10" t="inlineStr">
+      <c r="C59" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D59" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxON3p5Y3VPM01XZFk4a3g0R3JnQkZXbHVGV3BKdDB6M3NRb0M0SEl3V0R5RmhCQ3dnaHB0ZHp5N2hCMUFsNU1ZNWZ4YWdNZWdETkUyZmdoeW81amwtTWNFZlc5WlNpMkJwRzk0QklORGhlLWNEalh2d0JCX0lhVHhhUF9ibVlxcHAwOW9ENndVOTY0enBYUWc?oc=5</t>
         </is>
       </c>
-      <c r="E59" s="10" t="inlineStr">
+      <c r="E59" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2145,7 +2148,7 @@
       <c r="F59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="10" t="inlineStr">
+      <c r="A60" s="11" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2155,17 +2158,17 @@
           <t>Austal suitor Arlington Capital Partners buys Eptec’s defence unit</t>
         </is>
       </c>
-      <c r="C60" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D60" s="10" t="inlineStr">
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNM01qb1ZRZVBIdmp3cFc3R3RLaTdmZk1JOFo4anRtSm95Z1hJc0N0S3VranBTV29IdlViT0FkSm92eHdtbDBqdU5HTHNMaXo0dGRWMkpDdjk3LVRBVU1rZC1YejZJMkhyNmpZZFJodGoxWlB1dkRhYTJVRlljMlV0dUllQ3EtOHZkNFdSUWJLSW9Xemw1XzFzU2RHV1o0RTViOXp0bDZFQTZycWhpNElLU0FZQVI?oc=5</t>
         </is>
       </c>
-      <c r="E60" s="10" t="inlineStr">
+      <c r="E60" s="11" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2173,7 +2176,7 @@
       <c r="F60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="10" t="inlineStr">
+      <c r="A61" s="11" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2183,17 +2186,17 @@
           <t>Eyes on Tom Wallace as clock ticks on Adgemis pub deal</t>
         </is>
       </c>
-      <c r="C61" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D61" s="10" t="inlineStr">
+      <c r="C61" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D61" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxNSExQeDlENWlHb0prRnRldjZ5YWhKVUZ5eVdsYjZmbVRWRWQ0WnZXWkU3UHZJdElnQ21jMU9zNnhnc3JlNDczVGQ5Y0FGV2J3QUp3NXdZTXZMNm5tVC1vWDFtOFN3aS04QVJZb3FZV2VsUmJ2aVgwbUhTaFVGdHg0UjRyTXVVUnFhQmE5eFYwMGR6T1R2U3Q3WEdZclVKNWJiby1IRg?oc=5</t>
         </is>
       </c>
-      <c r="E61" s="10" t="inlineStr">
+      <c r="E61" s="11" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2201,7 +2204,7 @@
       <c r="F61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="10" t="inlineStr">
+      <c r="A62" s="11" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2211,17 +2214,17 @@
           <t>UBS names head of APAC leveraged capital markets</t>
         </is>
       </c>
-      <c r="C62" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D62" s="10" t="inlineStr">
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNMm9WZ2ZKVFBvX2pYMk16VmY1WFZnZ2J5N0F2bHduTVM0Sjg4STVtTGFLQVdzeFloVHg3clRic0owTDMwYVpXdDVjdjFOWjQxdkdxdFY5MEY1Q1U2Q0R5dFBJWTNtUzgyd3RXcm9uM0hKdEZ3b3JjXzcwQ2VpRm5SS0hYT2gxSU9iVFRlR05Xd2EtM2JOQjBGUzlKdnE?oc=5</t>
         </is>
       </c>
-      <c r="E62" s="10" t="inlineStr">
+      <c r="E62" s="11" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2229,7 +2232,7 @@
       <c r="F62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="10" t="inlineStr">
+      <c r="A63" s="11" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2239,17 +2242,17 @@
           <t>BHP, Woodside rise after new CEOs named; Future Fund chiefs exit; Sandilands ‘doesn’t accept’ termination</t>
         </is>
       </c>
-      <c r="C63" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D63" s="10" t="inlineStr">
+      <c r="C63" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D63" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNUHhZeHNHemtiLW1IOHN1OTZXOGpsM0ZtUG1MVHRCT1hUT1k5S2lEOXlXRENWOXNlMEZadThQR18xSTJfTVlQM3BtX0ptX1J0bk80SzNLUVRtbkJITGgtb0lsSVdJTWt2S1E1WUlXdUdsbEV0V1RpNWlyRXBoc0dPVDl1OXRrSlM3SHlDazg2UlcxenVzNzlhQldhUGhfNE5IV2xrVmVBNzhhSE9qY042Z3pzMEVzd0VyVmZudXgxcTgwWGJXSWZKZ0FyNVhjcmhjTm5DYUVjLUdDRmxUQkZuTDFlUXVaV0ZoSWp5WHMyR3c?oc=5</t>
         </is>
       </c>
-      <c r="E63" s="10" t="inlineStr">
+      <c r="E63" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2257,7 +2260,7 @@
       <c r="F63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="10" t="inlineStr">
+      <c r="A64" s="11" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2267,17 +2270,17 @@
           <t>BHP’s new CEO will shift the Big Australian’s centre of gravity</t>
         </is>
       </c>
-      <c r="C64" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D64" s="10" t="inlineStr">
+      <c r="C64" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPQnZpWndNZzZvN1VsOHBmRDVLRHVTNkxLeDVDelpOMURjOTRDSDZfN2dPZlZqaW05WEZuZXMyRTJZeVZnV0poT2UxRkVfZ1RZSjdvUjVKblhoSU5Cd1plRTVNNTRaNWZmbm1yUGZkblVpYkctNzVRRkVQQm4zX1FtRG1KV2Y0djUtOURianJ3dElqeXBUMFp4aWFEWVFYelVjYTluSWpOM1FlbHpIaUxXdnBn?oc=5</t>
         </is>
       </c>
-      <c r="E64" s="10" t="inlineStr">
+      <c r="E64" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2285,7 +2288,7 @@
       <c r="F64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="10" t="inlineStr">
+      <c r="A65" s="11" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2295,17 +2298,17 @@
           <t>How philanthropy became the sandbox of succession</t>
         </is>
       </c>
-      <c r="C65" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D65" s="10" t="inlineStr">
+      <c r="C65" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D65" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxObnBPb2MzQ1RvSVVCbmNzYWFBMlFjU0dQRmpPakNfdkxtMWc1bFdVNXNlZmRKQnNlWEtUUDNSTHpTLVV4Skx0V2otbTZsTTdvT1VaUDhMZFZoMFFab1RoS2pCcno1WGlNQlY4eXQ0OFEtLXJTay1MUkFSSEJ2MVVScUpjUkhJOThISy1QbHIzTzFlWVhOc29fWWs0V19sQ25hRW9MSGhBVVNKWUp6dUo3NS1SWlk?oc=5</t>
         </is>
       </c>
-      <c r="E65" s="10" t="inlineStr">
+      <c r="E65" s="11" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2313,7 +2316,7 @@
       <c r="F65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="10" t="inlineStr">
+      <c r="A66" s="11" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2323,17 +2326,17 @@
           <t>Advanced Navigation raises $158 million Series C round with NRFC backing</t>
         </is>
       </c>
-      <c r="C66" s="10" t="inlineStr">
+      <c r="C66" s="11" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D66" s="10" t="inlineStr">
+      <c r="D66" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNTXhwVlVLUy1pWEpFdzFCazNTY0dkczd4WW9oeW14cUtTaDZRTGlVQXBPaHN4WTBkNW1zOGxvN0tVWl9JSFdVNXlQMzVxbk4zbDZFUjNOcUxSamNaSnFCckMzWEk1VlNoSHJHQ3VWdGltVWZCV0c0NmU4UlN6YU55Q0J2TkQtUzBzOW96UXRxem5Zb3M2SUljNURISlRkQmJD?oc=5</t>
         </is>
       </c>
-      <c r="E66" s="10" t="inlineStr">
+      <c r="E66" s="11" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2341,7 +2344,7 @@
       <c r="F66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="10" t="inlineStr">
+      <c r="A67" s="11" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2351,17 +2354,17 @@
           <t>Kal Somani-led consortium buys Rajasthan Royals for USD 1.63 billion</t>
         </is>
       </c>
-      <c r="C67" s="10" t="inlineStr">
+      <c r="C67" s="11" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D67" s="10" t="inlineStr">
+      <c r="D67" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOX3lmdG5aTmk4TEpBa3ROdWZ1aDJHUElBQXktVmlKaHFmTUhPX1QxX1dKLXZfaHRDQjBnWm9McTZjTjJtTWFETTRNMHgzN0tTTm1xY0JpMF84Q2lNaFQyZGVjaHN4bkVmcDN5Qy1ta3FtYnpMSVVyYm0ydWpTRUdZU1hoYXpaNkZUQzlPc1QycjZ6aG5QVHRqY213?oc=5</t>
         </is>
       </c>
-      <c r="E67" s="10" t="inlineStr">
+      <c r="E67" s="11" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2369,7 +2372,7 @@
       <c r="F67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="10" t="inlineStr">
+      <c r="A68" s="11" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2379,17 +2382,17 @@
           <t>KMD says Rip Curl demerger proposal delivers investors ‘no value’</t>
         </is>
       </c>
-      <c r="C68" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D68" s="10" t="inlineStr">
+      <c r="C68" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D68" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPTXhBdHByWE9EbllFdDA2OW1UTUZEMVJfV2xsNFdURFRKX2JrODJReVRuQlFoakpWbTBKcjhNLUVsNE9sdG5LUElLZlVrbFNERS1QZTN6bEZIWEhXZ1pTWG5GWEw3ZmNETTdDUDUzYzR5M0E3ZGVlTWpSUnVlVU56dDNFZUtZN3liZ1dKNzJhLWU1S0M1ZnlKd1JNWXlxSlkyU3pGS1lhS05hTUJPRkxucldabzFucGs?oc=5</t>
         </is>
       </c>
-      <c r="E68" s="10" t="inlineStr">
+      <c r="E68" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2397,7 +2400,7 @@
       <c r="F68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="10" t="inlineStr">
+      <c r="A69" s="11" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2407,17 +2410,17 @@
           <t>Ex-Macquarie banker drives mortgage broker roll-up Recludo towards IPO</t>
         </is>
       </c>
-      <c r="C69" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D69" s="10" t="inlineStr">
+      <c r="C69" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D69" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxNQms5X1F2aTNhOExDbW42TlZOLVJwVWxna1JYSW9vWF9Na1RZa1ViTFdZc0tCcXRZZkRudTlsTzNuZGgwSENyYi03Zjdfc0lZTXp0NmJRZnhzb2pWRXRIOUdJN2lQM2h3ZFFtTXlSWHVWOFBIaW1Na3FQMjBCck1nVlhUcmRkLW9LOHpKWXQwTm9LcWR5M2FfdjFiRW04TndoanR5NmJvMENGalNuUGNINy1Qc20xR1J4d21ncHNNSUZqa1BXNnI4STIxSUFkZXdU?oc=5</t>
         </is>
       </c>
-      <c r="E69" s="10" t="inlineStr">
+      <c r="E69" s="11" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2425,7 +2428,7 @@
       <c r="F69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="10" t="inlineStr">
+      <c r="A70" s="11" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2435,17 +2438,17 @@
           <t>Coles reviews truck fuel charges as crisis worsens</t>
         </is>
       </c>
-      <c r="C70" s="10" t="inlineStr">
+      <c r="C70" s="11" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D70" s="10" t="inlineStr">
+      <c r="D70" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxOSGpBM3RjLVJ3LVlmR1QydnY2dm50WlVxcG43ajRFZ25QS1hDNTBONU8tY3Z2TklzbUNla0ttZk1GZzFaLUZRakFjSUpUQWItQ0VqVTVwS1B0QS1ObVEzNzdRT1l6aU9pVm5jSlhna1N6QmFKT3k1RkhMZGNTVnVLcDVIcXZmRjdjLWRpYVlRQUVmcVRtM21BSjVhTGNaaThyZkhLS2NWdkNCSkZKTlloUVdtbzRnYjFKbllOZXhOd3lkcFZEYURwUFVNQzVnSWRyM1RlOGd2M1pMZXI3c0NIa0Y0MNIB6AFBVV95cUxNSjB3Z0hoTGxwOHJQQ09xb3BmRmhCYjBCc2E0OHA2elFDRE45UGpaTEVDc1Y2VnRvVmZQUzRHbng4QTMwNGZZNGpmaVlHRmV6bnhiZ0FReU50TnRiQ0NZMEtoM3dBZ0hXbFBZMVJQNXd4LVdXRDVyTDAxNS1zeVdvcFVvend2N3J5R2pLYmhxNVFfd19rUlRsNWNndlptMUVkcS1CaUN6UXRHVzByTU5BMW1TdktOZUJYck5xMEJucmR6czIySEMycDA5cmR1MXB0N25Xc0JDUG9zN29YWklVc1BUMzl3UVhn?oc=5</t>
         </is>
       </c>
-      <c r="E70" s="10" t="inlineStr">
+      <c r="E70" s="11" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2453,7 +2456,7 @@
       <c r="F70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="10" t="inlineStr">
+      <c r="A71" s="11" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2463,17 +2466,17 @@
           <t>Sam Arnaout’s Midas touch turns suburban pubs into pokie gold mines</t>
         </is>
       </c>
-      <c r="C71" s="10" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D71" s="10" t="inlineStr">
+      <c r="C71" s="11" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D71" s="11" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQV2xlTTdYOFpIMzNmVVRnMlJRbTdGTC1jelVCd1V3UjN5cHQ1VzhWZzhrNW1PNm1RX3FlZmU3UkRycjF4WDlQUzRMcVVYY1g3UTZqQ0hxRnl2Ti1IQ0owVmZjN3Jod1BFbmhPVUwxNjhsTGh6d0kzdU01N0hmempRZ044ZmZNUllnenhyc3djRGJOdEtrekx5UVFoaFFMWDdqMHMwdng1SFg4TzZHY1hQNFJNN3huZXpWYWFtQ0ZJakhkVFlQcl9SQlRfZkQ?oc=5</t>
         </is>
       </c>
-      <c r="E71" s="10" t="inlineStr">
+      <c r="E71" s="11" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2927,6 +2930,258 @@
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>David Jones is trying to defy retail gravity. It’s causing problems</t>
+        </is>
+      </c>
+      <c r="C88" s="12" t="inlineStr">
+        <is>
+          <t>SMH</t>
+        </is>
+      </c>
+      <c r="D88" s="12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPZy14UldWZDRrSjI3R0lzdGlKamlkVnU1WWVjTWRUTlpya1ZpVW80WHlrT0FQTUUwMzkzM19xQWpwTnVLOF8zeTFXamhTZFRQVjl5TTlXbE1RRWY2NW03dlpmZ25qdkgyN1IwbDdjRlhxd1MzSGkxeG45M214OVlESWF5WWh5TjM0STQtOXdieWIyOUI2NzRsaDhiS0ROUU5YQ185aWtObUY2S0dOSTBROVlwSVB1VkNqTkZTTllkZmtMYmxjNVdlTA?oc=5</t>
+        </is>
+      </c>
+      <c r="E88" s="12" t="inlineStr">
+        <is>
+          <t>Retail &amp; Consumer</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Jefferies’ Australian ambitions in focus as Sumitomo circles</t>
+        </is>
+      </c>
+      <c r="C89" s="12" t="inlineStr">
+        <is>
+          <t>The Australian</t>
+        </is>
+      </c>
+      <c r="D89" s="12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxNUTd0LXFPQmZXSldrTmZHTkIwUWQ3MmlCUmFOUGRkcVVjRXV6YXZJUTcyMG5FV3I0dWY2NXh6MnduVjNxZmhJMHdDVGw5VzFxTEFzN2FBdlNvS1JGSDltQmlzVS1QRDdCeWdfSHZ2VlZDMlBnN1Y0d2JxbnlGejhWVjJpWGZLejdCTUt2Uk9ENmhyRkd4dDJjd0RlUnBlZXhOTmUtOG9ITE05VHJ3dTBRSWZneURuUW1NYkExVXpfWXlsMzZ1WUlyNE84SThQX1JJTFlXOHc4ZnB0aXRmdVhaaG1qSEJRZUhuU3RibHAzbHVNLWFLUF9NNTFoUXV3NGQzelcwcNIBigJBVV95cUxPMkhEeDJpNzg0NTlDZmF2LUFPSEs4cmZ5U2p6bWVZSTYwcXVUUGVIb0FLVnhZV0cta01CLVpfQzQzYzdvTWdxR0o4bGJDWDVBb1lnOGx0bWROdTdjcHhwLUpPMW9MQ0RVM2NUOUt6UGpTd05JYzhuVmgybGp2LVpORFF0SHpBTU5DUTJEUmZKUFBNajlQdHJ4WkdHVV9QMjVwOWVlNWliVkFaM20yWGZhOEc4bldHRERJak1BWXlmSE0zdno1VTVSc0FMck0wSE1BR1RVaVRMSEdzU2FvcWpMYmp5ZTVJTWcyUGdXanhqSUNZU0tzTkNYWVg2SXpVMEoyS184VkxOeWtSUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E89" s="12" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Bain Gets Nearly $300 Million Loan for Australia Wealth Unit M&amp;A</t>
+        </is>
+      </c>
+      <c r="C90" s="12" t="inlineStr">
+        <is>
+          <t>Bloomberg</t>
+        </is>
+      </c>
+      <c r="D90" s="12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMUQ4WExYZFY1aFBwWENNR1JiVkw4OHFKWjY4NW4zQ3ZBalFiTU10Y2hic2p2VjFqOE1rMndNYmVoN0lPcnY0WmFOV1MtaEY5c2xvcW1PNGN2SzZVcThwc3ljWkYwV1Q4a2dIaUpBeXZpMkRUU3IxZzVBVkhydGU3OXEzNW1sdlVQeTRNRFY4bUJLOGpGYmJ0ZXpPc1YzY05TYWd2bF9oWVJ6Rks2dWlod1dGRU4?oc=5</t>
+        </is>
+      </c>
+      <c r="E90" s="12" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Fund managers caught up in Aware, TelstraSuper $237b merger</t>
+        </is>
+      </c>
+      <c r="C91" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D91" s="12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcFF4Q1A5X1VtNWFnYXZSVUlZX2JMRVoxaUJoeGhybmRrZkd4UlEzTURwMkx2d2I1Y1hMYmljbk05WUFzRl9JbF9JampqeDd2bXdYcUpHbVZYak1sYXFHS2VuUDJyTUhzSS1QTW15aVpfeHRuMGZHenlxOHJQRUdENkV0b2FMZXhOZWF1Yk5hR1lOYWFQc2Q0SEROUFNERXhKQUIzRkt6NTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E91" s="12" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Soul Patts defies private credit jitters with 15pc returns</t>
+        </is>
+      </c>
+      <c r="C92" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D92" s="12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPRkNINFJOai1NbUUtX3ZrcnJFS3EzRHZPbFRfVFE3SERudTVqbjIybWsyYUthOUJOUVFPb1U0UzlGTTRqbUxraFZfYlVtclQxeTBQU1M5YjJzMDVPU3RiX0cxbk8xOEd5YjV1R04zT0NNZjhNSi1meWo4RHM1ckFsUnNLd0JiQXFnZ0dtckNzdWxmanZoQUl3TEQ2a29nRkRDZ1lJd2Y5VGc2UWZHX0pkU1NObmRJTlZKS0E?oc=5</t>
+        </is>
+      </c>
+      <c r="E92" s="12" t="inlineStr">
+        <is>
+          <t>Retail &amp; Consumer</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>Ex-KKR China heads negotiate to buy Vitaco, owner of Musashi, Nutra-Life</t>
+        </is>
+      </c>
+      <c r="C93" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D93" s="12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQRmlCdTlFeHdBUGkyOS1CeEFIYTRSREdZM1JOZ3IyZThnNmNMdm9QeXVwRWtMbzU0em1vcDAyM1hodDlvalVRdThtNVhLR2FsaE1vV0xuWjkwMkVCUDk5SmVka1BURFJZNkl2bURLeC1GdzI0V2hEaVhrNlJZejlvc2gwRmtnUjd1NDFlX2trbGk2aXJiQ2FrTWtmVVpiOXhBc05JSkNYY2xLX2JEQUpWY2dlY1pDZw?oc=5</t>
+        </is>
+      </c>
+      <c r="E93" s="12" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Antipodes Global Investment Company</t>
+        </is>
+      </c>
+      <c r="C94" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D94" s="12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE5mdkJzN19XLTFQc25LOUk0ZGJBMER6djB2VnFvbGVrS1hlemRBRmlNY2JmMGlPTzktU0RRS3NNUW8tRXhtUE1QdE1JLWdUNVhibmZPZi1MRkJOWk95NzM2bXplS3JzeG13UU5henhza1ozeGRZZmlBNTNR?oc=5</t>
+        </is>
+      </c>
+      <c r="E94" s="12" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>AusSuper to lift insurance premiums by up to 40pc</t>
+        </is>
+      </c>
+      <c r="C95" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D95" s="12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQNEhYQkoyNnJFU2xBZG8wdXhEZWRSakRiWWNHOGZBTFhfaElxWkRsSWViaWxjenVjMF91cGdrbFZxSGJfbkR2SUZNdEJtYUVadlV6YVVrWU1VbVdsMWpyNUZ4bE13Mmo4cGQ3WWZlVFVrTTdyOGpSdkpUb0tkcjdQUFlsTnM0MnpOMDJNZlJ4YTlzZGpLS1QzMFluOFU2VUJya3lSclBLSnZkQ2Y0a2djNUpSYlo?oc=5</t>
+        </is>
+      </c>
+      <c r="E95" s="12" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>Unions want inflation-plus minimum wage rise due to ‘Trump and RBA’</t>
+        </is>
+      </c>
+      <c r="C96" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D96" s="12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNdzNhU0MzbFRFX2I3OVY4bFItd1h6OVE2Wnpqb01NM2tMYzNob21BeW02LTBfTFZIWnN6SG5DVnYxQTJGZWZaLTJpTXZGUnhmS3RPY3hQV01fd1RIYU9Ednc4a1hvalVRT19ESU5TX19sQjN4dVV3X29kQjliQjNFU19iaXFIS2l3blk5TWUwdHFrRmJtQ0JocDN0WEhWbXZOVUJzR3RaYnJPSHpIRFlYOVFObEtuT1d0TUo0MUVZTXdFZWR3WG1r?oc=5</t>
+        </is>
+      </c>
+      <c r="E96" s="12" t="inlineStr">
+        <is>
+          <t>Australian Economy &amp; Markets</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>

</xml_diff>

<commit_message>
Update news log — 2026-03-27
</commit_message>
<xml_diff>
--- a/news_log.xlsx
+++ b/news_log.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -87,6 +87,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -480,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:F107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -524,7 +527,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -534,17 +537,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D2" s="11" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -552,7 +555,7 @@
       <c r="F2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -562,17 +565,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="E3" s="12" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -580,7 +583,7 @@
       <c r="F3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -590,17 +593,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="12" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -608,7 +611,7 @@
       <c r="F4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -618,17 +621,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -636,7 +639,7 @@
       <c r="F5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -646,17 +649,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -664,7 +667,7 @@
       <c r="F6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -674,17 +677,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -692,7 +695,7 @@
       <c r="F7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -702,17 +705,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -720,7 +723,7 @@
       <c r="F8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -730,17 +733,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -748,7 +751,7 @@
       <c r="F9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -758,17 +761,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -776,7 +779,7 @@
       <c r="F10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -786,17 +789,17 @@
           <t>Zarraffa’s Coffee celebrates 30 years, eyes nationwide growth</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOcXNzUkRLemZEOWtOZjhvRUtzcUZrSTdzV0s0LUJTd2NGRk1Gb1NSLUR5Rlh3NUdWQUJkVWctb0toUFBRajlMcWV3VnNyTUtydy1PSUoyb1NCOGVtMUZqRVN0MzFkVkNlOUZNVXlHN2kzREhSdWJQUnJqa0pnUzExTVZSc1NCVFZSNlBSUWNfWnZ3MC01aUx0UWF5SkNOaHI3ZkE?oc=5</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -804,7 +807,7 @@
       <c r="F11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -814,17 +817,17 @@
           <t>Zarraffa’s Coffee eyes 200 outlets ahead of 2032 Olympics</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPMUFjRTlGVFBqYzlPWXdzQ0dKVVlhWGxncUQxTDd1R0VHcThlV3ExVmo4SlBGSHVuUGZrMGNqSVo1YVpDWHViMm5KZWIxcHNMMHo0b1FQcmxUNElDR2lEeWRuLWZIN2lyQUV0VndEUWNkNU42Z3AzNXRlbm50NzhtTXZ0Q245dF9hNzBxOENuMXZsVlU4Z0JGVElR?oc=5</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="12" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -832,7 +835,7 @@
       <c r="F12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -842,17 +845,17 @@
           <t>Aware Super appoints new head of private equity</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNVHJXNWEtdEZZUW1fZzdYMTB4RklBTUh6dUNKQ3BrTlpYUnBwRURIVGZjWTV0OUxScnhGMVNSczhLUjVqOEwzbkR2WWlEbmF4ZkNUdHNQY0J1djI0REctbHd2SVhUNlNCa2M5bFhOQ0JPU0RHOVVTQkEzRDdGMjRZbVFDOUdlTXNNczlmZWF6bXlfbEFGRE0xbkZQaw?oc=5</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -860,7 +863,7 @@
       <c r="F13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -870,17 +873,17 @@
           <t>Commission wrinkle over UP Education sale</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxNSV9GMjhqM2ZSanI2X0w2OVlQVFRQTUoxYzAxaXVZMmU1REVTcHlUeEltdXJtaXZrcUJWdDZxNGpYTTZYSFE2TkZHeG9OaVRZakoxV0s1U01TVjJpWlhaSENfNVhucG5NVzFMbTVBY25zWGRSODBtRGtkS1owVTlJWnNfcTJ5alFnbVl1SU9aUDF1QWxJLTBSQ3kxUUFlZnpJMlVEQndFSGRGbDF6WVBUVHlCcDM5Qnh3R2xBMG9xN2FLckNzbUFOWDI1aVF1YV90d0twd0ZmMnUySDBMdG1R0gHkAUFVX3lxTE5EWVp6VzZWb01TRmlHSS0wMExldkJwSHJjdlZXdElsRlpBTEtVMkd6VzNQa1RpVDNsOFQzaGZ2VHpzUnBDYk82RmZGQWJuTmVQMXhxLXVmdVFxTVZOZTBsOHZ0V3cyVVVkNWUwVUxSc0xNSU92ZktpdFRfYnQ4WHBTX3A5bFhXZ1YwZXNrc1BSZEU4LVYybnNBd0dCdk92OFUwclJCMzdoU0ctX1pEdTAwY0JiTWQ4S01QRE00TW5EUEJwR2YtczZ0T005bTJnN1RDY2p6NFF1SndfLUo4QzJUWk1tRg?oc=5</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
+      <c r="E14" s="12" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -888,7 +891,7 @@
       <c r="F14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -898,17 +901,17 @@
           <t>Gloria Jean’s owner has an angry shareholder on its case</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPTnZwUVBCdTFJZWkwc0YtVmJqMkNPcUR5RktjMlVURmhROFZkYUpXM01iRUh3SnJEUElxRGlSNk9DQjZSdTdNdmZwWWpONjlmR1hoMl92cUNmd3M4cnJhVkNqc095MmN6WXBYUmdEblB0eERtVDdlUU4yNGFjXzVnT19rOERIRzVPNzY3VDNNRS1tVGVTX3pKMVRpTXZVR1ROLURBLWtJbVZhY0lSU09DNkE2NzFLbEFU?oc=5</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -916,7 +919,7 @@
       <c r="F15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -926,17 +929,17 @@
           <t>Oporto-owner Craveable Brands hires new CEO from Domino’s</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNNmxfQVc2Umc4QWwzSTdsZTFvejRzTzZxXy1ScGlhXzh6bm5JS3IyX0xTNDVBNjh0cXpPbGhxNU5xUHhQN3EtRF9aV3FEc2JoSG5QTU1WeU1TLUJfZzVUT2N6dXloQXhZaHB5djB3dDFKN1llVmI3UVpKNjJTNlcyV0ZDcG9GdVdSdW41ZkN1b1N3SFFIUzcwRkQ3UHY2TmxERmZwTlA0RzU?oc=5</t>
         </is>
       </c>
-      <c r="E16" s="11" t="inlineStr">
+      <c r="E16" s="12" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -944,7 +947,7 @@
       <c r="F16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -954,17 +957,17 @@
           <t>Brookfield, BGH Capital rub shoulders in ScotPac’s data room</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPMVlxbzlQNnFXWnJFNU11Y1BhTTVqbjN4RG1nbkZuN0pkdDFFaUhJN0RaVnUtWDlZSGJWR1ozQXk5UUx6RVdOcjBPU2t5UzN4T0JvUFJISnNvVWxQemd3blNHZjRQVVVZQk1nZER0Y0JfY3VvQ0t1a09sM1RTS2c1YTJyUmdzYWh1WGRUNjl2dkdzYTJJeHVhMTdqR3Y5WVlHVEtSZHp1cmVYYmM?oc=5</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -972,7 +975,7 @@
       <c r="F17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -982,17 +985,17 @@
           <t>Payments player Pay.com.au hits the road(show) for $850m IPO</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOMFZleXZrbU53TzBlakI2ZmJKTjlrN3BoQlRaWjQ5cXFzTllKWmFoRm1UT2xDUHBtNC1QNTNiX1BwSzllMkRZdHIzRlAteDREaUczN1JTNTByTW1jNnR3d2NnR0RxUDBxeHYyWU1CSUs5MEZad2JqSGF6ZUxHZUNtZmFQaTJZZVJVZ1B4MkZ6V09QMWIxaUNHQmVzTDhvWVA1Ty1UbHgtQnRrQQ?oc=5</t>
         </is>
       </c>
-      <c r="E18" s="11" t="inlineStr">
+      <c r="E18" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1000,7 +1003,7 @@
       <c r="F18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1010,17 +1013,17 @@
           <t>Another year, another IPO cold shower for investors</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNeEhzYzQzdjR5MDJCWkd6Q2VLdEZzbzRoWnNOcXFlQjNfMlV4Q0NQRjExMlNhT2NPcnRBbW1sZUkteXo4N0dGaHNNeGZJOEZ2aXFvdmZiN2V2QzdOMzFteFRnY1RVRm1rQXltWmY5VFZOdFVNNVpudVp1dTlrcFM5b1k5SmlWQllDMVFXSjA4ZVpSZHgtV2JpWDJ4SkFRbVE?oc=5</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1028,7 +1031,7 @@
       <c r="F19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1038,17 +1041,17 @@
           <t>Priceline Pharmacy franchisee sale narrows to final four bidders</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNR294am9sYWNiQ3FVT1B6YlV5ejMyeHAyT0FibTFVbU5pcjZyaVRyazEzbFkxd0lrcnpZNGpTYUx4Ykl1Xy1sZF93M2Nid19ydUFwbUJ3ZHozaURaNkRoOE9OMnRBRGZfQVdCVWZCaVhhNnZSRjlwYUdDVnp2WU9HUkJxbE1QMV8zdWxYRTNBQWktR0xSOFU4dmtXZWk0am9SSU92NWp6QUZmTVU5TzJEOEJNak5fQUtN?oc=5</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="E20" s="12" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1056,7 +1059,7 @@
       <c r="F20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1066,17 +1069,17 @@
           <t>Private equity gets better image of Qscan</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D21" s="11" t="inlineStr">
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxPRjVmT0hDRjZLblB1VHdPRmRGeXhKdDJHdWxDTzV4RDZ0VzdHaUFfOVlnZjRQMWhKcWMxby1oRDR6N2lQZkI1UDE1REppS3c4LTVmU3p5b2wtblRCWnhNajFnZGNHaGRJUHFMUGRtTHAyQmIxOHhNNTgwRWVSeWp6ZWRxbUY0WVhiUnhMRUpDLXNwS1RuelJldTk0Z1R0WHg0XzNXNTA5Rk5TRFZhU1RNVnN2TlZuaFE4OWtIYXQ5a2VGSW1UWmt5Rlc4Q2lIXzF3YlkwNVhfUzJDV0dQdVAxa2RKc08wRGR6TlB2Vi14QV9BdlhyaTZsM2pEVGZycTjSAYQCQVVfeXFMTWpnb0lWQmZ6MTFnRGhWNTNqczk1TWhTcUFEMVpDNnJ4ZWVxVlRUODhJXy03NHdGZVJlMmhyUHM0Nlh4NlZtTzRhQ0xxRDFLVHNzUVNfbWxhS3BLUEQteEMzZHRrc0F1eFRzYmxVNDZlSURyZDB5bF9wQTNRRU5yZEs1Z3pFRTdwcFBaMkNlN0JvT1NEYkFWVUJNcHJqcEM5RVJYa0JFUVl6cThyQXloaERzQjhkTUVPakJqb0hzNVlwSWxNS0dmZkNFSG9Gb3dNUnVvUnV0d3MxSmpzdFZKTHJ2RTQwRUoyMEVLLWMwT1NnOHdXVl9lRXNDWEFndzJFSDlZU0o?oc=5</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1084,7 +1087,7 @@
       <c r="F21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1094,17 +1097,17 @@
           <t>Oporto CEO’s first year reshapes brand and network strategy</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="C22" s="12" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
+      <c r="D22" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPY25mNTJfT3FiVlBPZE5CcVNkR1UzR2xWaUtJSmxhU3EwcEMzQi1ISDFSajlCQWk1UUJpZVJ1Q19ZV3Jjd0Noc0l3OExpMXhSQUVVdHhCLTBlOXNoZzA3UXZBdkR1VHBvMmVsZkNhUFJndm1DdGpnX2w0ZVViU2phZ1RmYXY1SlhwUnhKSUxBQVZZUXpqNHQxQmo0Rk1iV0g0OW9qUS16eWRSNW5FaW1yQQ?oc=5</t>
         </is>
       </c>
-      <c r="E22" s="11" t="inlineStr">
+      <c r="E22" s="12" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1112,7 +1115,7 @@
       <c r="F22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1122,17 +1125,17 @@
           <t>The Melbourne restaurant our reviewer grew to love</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D23" s="11" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOc3YxQTljcHJXVWtRX2ZGM2lpM2pILWNwSFg0MFJrNmNWX0ZxRG9nV0J5N19qRWh4U0hPXzNmVVZwWk9wT2kzaFNrTlV3NEQ1Q3JpaXVIYlBHb216Q3VYVWdSRXMwdDl0SmYzdnRlSDFUYVRmRGJyZVlRZDJKTHpJOUctYlF1RDZSYjloY0hfZy13QmFTLU9UNjkwTHc1bjlGcGxoZ0ZLVU1GWTctZkdLZU9zSGhEZEpKbXJnaWJfZjd2OWs3?oc=5</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1140,7 +1143,7 @@
       <c r="F23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1150,17 +1153,17 @@
           <t>Crescent Capital strikes Benson Radiology deal for close to $400m</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr">
+      <c r="C24" s="12" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D24" s="11" t="inlineStr">
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOLTNrWG1ZZlFoU3pDZ3E2SEgwMlhzQkdtQUYzaHZTZmYwU3ZhMnE0dlkza005VkZmZ09NMExlWDVncnBmYVVISXJ6X1ZjNHhpM2RnSlprY1dnbndJNUczcDVtNXNRY3pVNW12bm5rUVdqVmR4R0JlVHFuN0RwTlFkR2xrbFFpSl9jcm5oSjk3aFM1clBSVDhnbkhoWUREeUhsbVpvQW90d05xOTdfOV9nbW5POFdmelJkVlpsUlRuYl9odmRNVUV2S0pCMFBMTS0tcVhGVGFYU0h2d9IB3wFBVV95cUxPWEs4R2pxdThPbHJHb0dBT183SkRHTTlXNzdWazcxdkd1eGx2VlAyM2VVbEtEbWxTZ1R0TlBFRmRMZTFoalgxSmVVRUJFR0c0RFYzZVJFODg3dWxicU9pOHppeFhjaVp0WWlyTnUzV1dyZXdkMHBDVHI4LUVQdjc0cWpheU55NTlvdWdCZmVoODB0Mm5fbGNCTmQwLUhMZ0psQVpzb3BEUnJpSkRnOUM0c0VCdUp5N3g5MkhaM01vTHJ3NWd0ay02UXZUUG9nVkxicVc1Z0xjWGhjUDRDVjlN?oc=5</t>
         </is>
       </c>
-      <c r="E24" s="11" t="inlineStr">
+      <c r="E24" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1168,7 +1171,7 @@
       <c r="F24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1178,17 +1181,17 @@
           <t>Dual-listed giant Capstone Copper flirts with $600m-plus carve-out</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D25" s="11" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNcVh4blRkQnoyaG1TajhVV0lrOEJRaHdTZWtzUnJHaEdaSXNRWThGTHlVdGl4dGJ1cTMwZ2pLcVNzUXRYNlZzVzhvaXdkNGtVUG0wN0FrMHB0R1I2Ry1jcEgtSWUtajI0cTFMRTlfdzBuMWtrZmJOLVUtMkl5dW85dFp6dEhEOHhTNzdfOFNFSGtlT0MwQnRlY0VhcUZBNE9RYzhQcDdOQUFnYkgzd0V0N253SQ?oc=5</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1196,7 +1199,7 @@
       <c r="F25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1206,17 +1209,17 @@
           <t>Guzman y Gomez unveils a new menu under $4</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
+      <c r="C26" s="12" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D26" s="11" t="inlineStr">
+      <c r="D26" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPMjRjRTV2a3BJc3AzdDNOQktoYjBvLVZSODVsc3lKQ3pET0lxUlpkc05NcVlKRlZITjVJbjkwLS1DUFJNMGJ1amJKTlp3S3VqMWJaU3YtUENEN01rUEJiV1FNZTRXYjcyV08zZzlxNDVOSlVOTlJDOGV3QzBQcUpKa2Zab1ItNlI3ajZVVTF3?oc=5</t>
         </is>
       </c>
-      <c r="E26" s="11" t="inlineStr">
+      <c r="E26" s="12" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1224,7 +1227,7 @@
       <c r="F26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1234,17 +1237,17 @@
           <t>Can Sydney’s burrito king conquer the $676b US fast food market?</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D27" s="11" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNM0ZFcUpLN1dUZWUyaE1LMnNZVGlEbkNNQUQ4Wmd6QVFlTy0wZDVHdnlja1gzMEZTbVpKU1Ftb3VKZ2pzajcyWU16NUtUTmR0TlZMOVhMRUNqZXZiX2d2NWY0YlJDOFhhYUE0SkhMRUprNndXak8tWGdERU90cmMxTkFjcFFVSTd5VlZ3NFVKOXN3M255MFhzZThmbi1VUGMyQ3E4d2pYcFlJckY3QlVBdVJJeF9qUQ?oc=5</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1252,7 +1255,7 @@
       <c r="F27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="inlineStr">
+      <c r="A28" s="12" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1262,17 +1265,17 @@
           <t>Drone maker Innovaero prepares for ASX float, taps Euroz Hartleys</t>
         </is>
       </c>
-      <c r="C28" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D28" s="11" t="inlineStr">
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNU3JrejNRZ1VBZVNVV29NMkFPVmRsWE4yMVZPcjk2aUNUTHFJUGFyQ1VnZEZiZlIzQW9VVzRNNDNRR01jcHo3X0tqZjB4bzhMTTI0Y3BwYUh6OGRUUGt2REIxV09oRnJoVWlVelZWaUlWUmlPQ3dJdi1TejcyaXB1Z0x1MEJRSlB3SGMwVGdXaXJJNm9TVllPOG5JZC1feEV3TVhTeExGeHR2RHFIWlVCOXh3?oc=5</t>
         </is>
       </c>
-      <c r="E28" s="11" t="inlineStr">
+      <c r="E28" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1280,7 +1283,7 @@
       <c r="F28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+      <c r="A29" s="12" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1290,17 +1293,17 @@
           <t>Bain flaunts Estia 2.0 as IPO roadshow gets under way</t>
         </is>
       </c>
-      <c r="C29" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNTEN1cGsxNDN2c1NqUzB6UmJ4TFl0NGZjZVN3U3oxMlVFWTF4WUZLQS13dUxMV0N2ek1XN2VURTNVWms1NjdXSm0waEdaTXQwdTdWY1MxZ1V3ZnpEcVJtczdOWGNNZ0RQNzRZLU1MTTgtRW5DZkctbXBGMmVXVXdPZW5pNThiRHEzWnB2eFZzTFZTb1ZkeW9LendkNDd0cXRid05ZSGZYbW9NZXdOLVZWODdZU3hVcTA?oc=5</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1308,7 +1311,7 @@
       <c r="F29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1318,17 +1321,17 @@
           <t>Carl’s Jr. Australia unveils nationwide freebies for Happiness Day</t>
         </is>
       </c>
-      <c r="C30" s="11" t="inlineStr">
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D30" s="11" t="inlineStr">
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNVWgwdjU1NDFWalBfMTFYX1dQOWNDbG1FVUdlcS1LTVlHZVRRTVBWTjhSMnpkTXRXNlFJdllGQUp5Mm5ObWpIazd1d0RJa3QtdFBZN1hOenBmVzBEU05wM0gtNUxPeWpsYkxyVnhWWFFOU2Y3R0tXcmNkeWhpWDh2eDZBdjNCMHhuc1lHYTZHblBPVkpfRXpKd051UWlNc1hm?oc=5</t>
         </is>
       </c>
-      <c r="E30" s="11" t="inlineStr">
+      <c r="E30" s="12" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1336,7 +1339,7 @@
       <c r="F30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1346,17 +1349,17 @@
           <t>BHP and Woodside appoint new CEOs in major mining shake-up</t>
         </is>
       </c>
-      <c r="C31" s="11" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>ABC News</t>
         </is>
       </c>
-      <c r="D31" s="11" t="inlineStr">
+      <c r="D31" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQbTg5VFJLbWJfcy1uV3ZReTJkTndzX01qZ2MxNWkzaWZRckNLZUR1Y1VsMVRNc2FySC13U0NzalFEb3k1R3BaUEhfcTV0N1M4Q1dpSlo0YXI0UFhrMGRab2RiYV9DQVNVX01ycFc5ZFZrZWZqc1VRZXoxLVEzSDJLclJLSWg5bzN3R1I0bG9lWjVDaHE4?oc=5</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1364,7 +1367,7 @@
       <c r="F31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1374,17 +1377,17 @@
           <t>Next Capital sells Enviropacific unit to French waste management giant</t>
         </is>
       </c>
-      <c r="C32" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D32" s="11" t="inlineStr">
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPR3lFbERLR2FtdmJUU3BDU2thZk00YmFHRFhXR2VBVXhQSURTeE5ONVJKczBwbzlFMnR5cmhxMnM0bzlJbWo4SXl1dHpqYWxxMUJBRjZHVUtab1RYZjZMTnpGc3FzMWQ2NjNEdGU3NTZwa0diM1lJS1haYllwTldLZlpZbXp0YzlxcDh0ekcwTy03dDdPcnk4b29HZVdqbHhZY2JPR2drM2puSVpjUzZkVjNpZUE4dVMwYlE?oc=5</t>
         </is>
       </c>
-      <c r="E32" s="11" t="inlineStr">
+      <c r="E32" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1392,7 +1395,7 @@
       <c r="F32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="inlineStr">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1402,17 +1405,17 @@
           <t>Future Fund private equity and real assets chiefs head for the door</t>
         </is>
       </c>
-      <c r="C33" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D33" s="11" t="inlineStr">
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPUHNHRFhFMVdwVld6RFRZUFd3QWNOd1kzeS1QdnJxMERFSnE5LTdZcDhDYlVGcWZMeWxlR0FSRWF6YkZoQVZrZU9TQ1E4YTEydUJnOFE3enV5Rmk5UnF5VEdYZ1FMUWpKVjdjMlZZUGFsU0tKcV9Vbl8zcHp5aVF5Z2JMOUZocHJqRXNRaEp4Nm5CbDM1WkdIMHdQS2xqQnE2Tnh3?oc=5</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1420,7 +1423,7 @@
       <c r="F33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="inlineStr">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1430,17 +1433,17 @@
           <t>‘I actually started to die’: the new billionaire’s epiphany</t>
         </is>
       </c>
-      <c r="C34" s="11" t="inlineStr">
+      <c r="C34" s="12" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D34" s="11" t="inlineStr">
+      <c r="D34" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxPblkxbHVrdnVKY1pqQzNyWGNMZm9UYmY3dzlPaGQ4Yi1tc0U1akhrVWdIaXBpM05aZXRwTXE1eDBITlZpbDkwRXNrWjJ2YXBzX0VCY2JSLWhrVmpjSTE5eE5rLWgtc2pRZEdXbmhhWU1KeFExZDBGS2pjSkIwV0FGbndBZVAyQkg4WFRsengzSGYyZkFfQnJsQ18tUHJGNDd2T0pzZElPSVJTQkl2Rm5QTExJNHhmU2dHOHJGdTdzU08yNHRtd1R3Q0cyOF8taDktQTZvVXVBVjN1d0NHMmtFOHBWZXBFcUFWa1IyWGNDTDZUT3lQSXJHOVhxTFQ3b3RH0gGGAkFVX3lxTFBZQ3BFQWl5dEwwLW5yVWJuMU8zcXBPdE9pamRVSWVkbWNyVzgydGVOaDBROUN6RlBDbjdld05DVmZyb0R1eEN0UERubzZRU2NiMTQtVV9XNS1wYmlvZ1paM3RaOUlrTzJka0tXVVJEamFESGlSdXg2bDk1aUdhUVhBcXpnN01fX0Y0cTNvcm5DdEFFLVVERDFKTWxKZFR0UzAyblJqVHBua2JoYUdzeUNMb053ZVczWUFQU1AtVHV1d3lSSDFfZFh2cEkxSGw2MEdicEVsb2pLQ1RuQmdaRl9xNUROS3pKR2s2T2wxTTZ5bEwtTUNQNU04djFHTHlPbXVLSW9YSUE?oc=5</t>
         </is>
       </c>
-      <c r="E34" s="11" t="inlineStr">
+      <c r="E34" s="12" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1448,7 +1451,7 @@
       <c r="F34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="inlineStr">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1458,17 +1461,17 @@
           <t>Ironbark shuns private equity as it hunts for cash injection</t>
         </is>
       </c>
-      <c r="C35" s="11" t="inlineStr">
+      <c r="C35" s="12" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D35" s="11" t="inlineStr">
+      <c r="D35" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxQZWFaeVhldi00VkV5ZmEtS2tjcWdFWG55OGpCX3IyN25Rb3ZFV0ZKVm1aSE1WbThoYVY4ZEdfODVGX0RaUDV2Ul9HS1JQMDFCT05Fc2FaU0RINTMwbDRveWFsOFJSM2ZqTU9tVGxJSEl2ZmhhUHFHT3dqYkk5TUtvMUQySnZzTWw1MzFNWl9aVzhkSEZ4Q3YyWjRMUmpIdmJkdUVKWE54Nkt6bTd2dGFSUFoyNkgxTHh2TGVGak9ja0dFZ0xQM2g0S1lmQkZiWWtUcTVNdHhBdC1KeVRQcDA2dnpmeHRkWEnSAewBQVVfeXFMTWtYRDRSaHNULW1HanowRnpMdFF2VVMtZW1SV2ViZXlGaW02WlIwUzRZMGg5WDNrOUR4eDlGOEt5eGlqV0pfVDFhb0JEcS1faEJodWxyRnB3MkozOVJyT3NvM1I5MzdDcXNnUFNSdkRDamUzZTRQYlk0c1VIQUNMZ2ZzOWVCb2V2MC1aSTZLWkFkbW9GYk05b3RmN1htWENTeDh3SU1WYWJMcWx2eGUzZmwwVXF6czlnRGdXbE1vRElyVG0yM0ZzXzZ5TFh1YlRGNU9MQ1p3NnVZSFB0M0xBcGlueVZILXlVaXdqUkU?oc=5</t>
         </is>
       </c>
-      <c r="E35" s="11" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1476,7 +1479,7 @@
       <c r="F35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="inlineStr">
+      <c r="A36" s="12" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1486,17 +1489,17 @@
           <t>Minister leaps to fix food chain</t>
         </is>
       </c>
-      <c r="C36" s="11" t="inlineStr">
+      <c r="C36" s="12" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D36" s="11" t="inlineStr">
+      <c r="D36" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxOd2NqakVWRnQ4anFZNkl4Zy03MkloX08tUkktRTZqeEtQWFZJeVhkMUJIb0FxUjc2UjhCQ3MxbmNxczNxblJIZ09IeTBGNFM4Wkh4ZE1qNkhJMjIwU2RtX1JxcEV1Y0NjWXF6eHpVdTN4ZUlYMGIwcDJzMXZMTk94VzFlcjhpcVZVSTJFMjhsQjVGWEJQYTQ3aTFyNmNEZ1F1b3NGTWd5WnFJWmxXSTJ2NlRLcjJHNWkwaTZ2YVR6S0w5WVo1Vlg0VWdxcWZoa3VaTmcxY2NVcnR2bFRWNGNvZ1M2Tlg5NzlvVXZFZm9B0gHzAUFVX3lxTE1uNERoR3p2dXRIa0g0RXI2MWR6N0c5U3NGcjFDQVMtdEpyNDI2bk8yOS1qUnFOazdiODl0Ymo5R1pwRVJ0UFFVdzlhYjRDSUFCU0FRak4xcVVrTHphdTdxcHNIMnEyRVZud1FURmh5T0JLOHpRM3lFbDRuRnZMYmtaRnRFTXh3dkszTFhFUmZlRmoydnlEbW1fZTlmUzh4NXNyeTZTeUhOSktvclJVc0NTZTVYMkdJZEUyY2RmVC1kQ1hwVEloSEtVMEo5QnNTUXQyME5IN1BPd1NOS3oyR1JtMHBFVTZEbzhEQmdrWUk1ZnZVTQ?oc=5</t>
         </is>
       </c>
-      <c r="E36" s="11" t="inlineStr">
+      <c r="E36" s="12" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1504,7 +1507,7 @@
       <c r="F36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="inlineStr">
+      <c r="A37" s="12" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1514,17 +1517,17 @@
           <t>‘Brace for swings on every tweet’: Investors bamboozled by peace talks</t>
         </is>
       </c>
-      <c r="C37" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D37" s="11" t="inlineStr">
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOczZHTWFmTW9FZ1ZwSnc5Z3ZacGpsVDQ3LWw1a1BFT0tjRkphek41MlhNOU84emYzZUVwNV9xM0hyc1FUR0NHck14Qnh6c2JvQks5ZE02ZTNLWDI0dy1STi1HbDFDWW9yMDhGQXVVVzdkMzFXcnNNMVZHVXFMUXUteGtsVGhPVmhLcVZPQzlhTWNoYVVRMHF0cFhybWxzek13Y3ZjcjlXWjZJM2VYbm0tTmk4NExLQzQzX1ZPMVlhcnJxQkZx?oc=5</t>
         </is>
       </c>
-      <c r="E37" s="11" t="inlineStr">
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1532,7 +1535,7 @@
       <c r="F37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="11" t="inlineStr">
+      <c r="A38" s="12" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1542,17 +1545,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C38" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D38" s="11" t="inlineStr">
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5</t>
         </is>
       </c>
-      <c r="E38" s="11" t="inlineStr">
+      <c r="E38" s="12" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1560,7 +1563,7 @@
       <c r="F38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="inlineStr">
+      <c r="A39" s="12" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1570,17 +1573,17 @@
           <t>Wirth’s Myer rescue mission is caught in the eye of the storm</t>
         </is>
       </c>
-      <c r="C39" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D39" s="11" t="inlineStr">
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNTlQ4NDRnWE91VG1YNENpSTUxNnBjZkljOGdYaGV0aVB5dkVOaEJ6SjZ1bVA4NXE1S1hjV1NjcVhQTEVpWEVNV0UtbzhQTFZLOWxIenZiaF9QM3F6bmJYRy1lbXVMczZ3TnBHNy1aLUtVcnBDdkl4TE0zRGN4U0FwSjNPY1M5S3AtdUQ3UUNmR0x4MlU2YXRuUDJEUm01SmZWakx2UjFvY04zRHk4Smc?oc=5</t>
         </is>
       </c>
-      <c r="E39" s="11" t="inlineStr">
+      <c r="E39" s="12" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1588,7 +1591,7 @@
       <c r="F39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="11" t="inlineStr">
+      <c r="A40" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1598,17 +1601,17 @@
           <t>‘Darling, I’m not going anywhere’: The rise of at-home care</t>
         </is>
       </c>
-      <c r="C40" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D40" s="11" t="inlineStr">
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D40" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQS2k0M2otaldpNVFXdHRTMVNtZVhyUDV4VTNIcE5FSnFRaHNubGNQQzBVbllnNTktNGhrZ1lndzV5V1FpUS01SklRaTZmZHJkRzVsQmlsdEVmenZ4U2x6U01NeXdIMktBUW94TUE3R3FoLUxVcVhsVFI0SjVQVUFaZldnd3prMWMyaVRWX2J4aUdfQ25KWHpaLUlqSnhvQmM2TTRRQldGbm8tclFYRDA0TVdnU2g3QQ?oc=5</t>
         </is>
       </c>
-      <c r="E40" s="11" t="inlineStr">
+      <c r="E40" s="12" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1616,7 +1619,7 @@
       <c r="F40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="inlineStr">
+      <c r="A41" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1626,17 +1629,17 @@
           <t>Iran targets Israel and Gulf states as Trump looks to calm markets</t>
         </is>
       </c>
-      <c r="C41" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D41" s="11" t="inlineStr">
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPLXBITXU3WTRtc0NYdnhTZHFaUTBCSXdldTBuSHliTlY1dlJONW43Qkd6Nl9pNmY1eDhzaHZoX19xYjBxMXR5UEhkVUg2M2k1MmhuVEwyY0JxbnJyemxVYUZjbk5BbkN4ajhPbW9ZeDhlRDRYTW1hN3k2d084c2djMEJUZTV3NVdPbllKUmFlU2JsaDV3Zk9CVFF0VDFkV09JSloycWdOUlVrREptQTJfa25LUEx5djA2SjNMMFY0RjM?oc=5</t>
         </is>
       </c>
-      <c r="E41" s="11" t="inlineStr">
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1644,7 +1647,7 @@
       <c r="F41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="11" t="inlineStr">
+      <c r="A42" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1654,17 +1657,17 @@
           <t>Meet Christian Louboutin, footwear’s most famous billionaire</t>
         </is>
       </c>
-      <c r="C42" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D42" s="11" t="inlineStr">
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPcXdGd0tMckYxbjZ5TVJmQ0Q4NFl2RkhHMHdlZDZsdGZ6cVQ0cUpaLWJTNlVoc2ZOQmtXNlFTRnJVMnVDTGc1NFNZN2g1VnotQlNQbzhlM1BJV3ZwQktOcGtac3RwSHRLZkR0b2l0eGIyVVlYdHJrc2hpT0pJbDR3LURPTnowZk54LThObndtMVkwV2VWQkluNVlWY0p4QVJGbE1hSGMzOW8zdkJZOWdocEZQWFBhTllNR1ZBSEg1TWRXUWd3X0t6TVcyY05PM0pF?oc=5</t>
         </is>
       </c>
-      <c r="E42" s="11" t="inlineStr">
+      <c r="E42" s="12" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1672,7 +1675,7 @@
       <c r="F42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="inlineStr">
+      <c r="A43" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1682,17 +1685,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C43" s="11" t="inlineStr">
+      <c r="C43" s="12" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D43" s="11" t="inlineStr">
+      <c r="D43" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQbHdYM2pSM2xkdmZ3OHhQc2tVUmhzclJWaVJ0aEwtUkNBR0ZUd3p1emF1M21jbTF1ejlKSkdDMnotcVNjZE1CYUlKako3WXR4MTJhdWNlSXZMbTBYanlmTWFzRGFIandXRUQ3UjN6SEV1bThvZjN2bDY0eFdpaTdMODN6TGFTdE5rd05TUll3MmNfTDhkQldoNDIwVlpoSl85aVRwcTd5Ymh3TDl4enZhZ2p4OExGY1ZaOFNEWFBB?oc=5</t>
         </is>
       </c>
-      <c r="E43" s="11" t="inlineStr">
+      <c r="E43" s="12" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1700,7 +1703,7 @@
       <c r="F43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="11" t="inlineStr">
+      <c r="A44" s="12" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1710,17 +1713,17 @@
           <t>Sembcorp Picks Banks for $2 Billion Alinta Loan in Aussie Push</t>
         </is>
       </c>
-      <c r="C44" s="11" t="inlineStr">
+      <c r="C44" s="12" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D44" s="11" t="inlineStr">
+      <c r="D44" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOdS1aaXZjT2VnSDl2TDdzZ3NfRElDWXdUXzZQYjFQMEZJOGlpaE5CNGdQMlZ2UFVHbUtfOXF1ZVBReExrdF85M0RWLWlBY2Y5dlRtWVdXLWp0Y1VrRmF4UGQzVUhxaHA4UHd1SUdFV21QcVFITXFHRlhzekdSUS1PdHlYRjdUbUQydU8wSktKVHRJQ0NaWE9sU1l6YXhtSWtBd3RwTERacnV4VzB6YlFhUE1QcXNDVXVESFcyeWY3cGhHUkRJcDhrYUtpTEY2UQ?oc=5</t>
         </is>
       </c>
-      <c r="E44" s="11" t="inlineStr">
+      <c r="E44" s="12" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1728,7 +1731,7 @@
       <c r="F44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="11" t="inlineStr">
+      <c r="A45" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1738,17 +1741,17 @@
           <t>Navis targets June for $1bn-plus med-tech auction</t>
         </is>
       </c>
-      <c r="C45" s="11" t="inlineStr">
+      <c r="C45" s="12" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D45" s="11" t="inlineStr">
+      <c r="D45" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxPNHRXaU5tNUVkd2MtcTg5M0EyQllrM0owMkZobGxLaUJxYUN2MUg0ZkdKdzU2YmxfanR3QU53cHZzNDI1WXgzRUcxOE9EZlluNmtNRUUzTGJPRnpfVVVOeFM3bFRNQmp6VHFBdi1mTnU4UDBvOEpMaHZPNXFtdUIyTlhuRExIVElSeVRUMGxjU0k5VnVxaWFfd3htWngydlhuR2E5aTQ5VW1LS01ac05rMGZoVFdOZzVyTzFhUDVsYkNrc0VQZmhubERSaTNwelk3WEhYUjF5d2ptMktYeEhzOHpWazFQZXphd0xfUFdhbkVGMVR2Z1dtVtIB_gFBVV95cUxObEwzeHd6RmZtNUp2dXVVV0plOVQ4WlNqQXNJU0thd1BEWE8yWkxxVTZjTkpsVGxxWGxpQzN0OERZbk91ai1fZkdtc0JoM1h5NERLTVdDbVJ4Y2k4djdQcWlVcDF6NjMyVDQzZWMzUFZxWjVRWllMZHVSOF9jQ2U1REFfNUlhM2EwYloxb1MwSTJjODdWdlZwX2h2N0xiQWNhallHUTNPZEtLaXhsY3dBZy0xM1VITXhLUERXS1JxR0R3OUpBTVBPZ2dPZTRUTVpvbFBNMjFUSTJuWS1XLWdhUS11UTRzVTVqaEhfMDhqWHlTMlJGekU2QzJVcFdodw?oc=5</t>
         </is>
       </c>
-      <c r="E45" s="11" t="inlineStr">
+      <c r="E45" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1756,7 +1759,7 @@
       <c r="F45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="11" t="inlineStr">
+      <c r="A46" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1766,17 +1769,17 @@
           <t>ExxonMobil eyes New Zealand market exit</t>
         </is>
       </c>
-      <c r="C46" s="11" t="inlineStr">
+      <c r="C46" s="12" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D46" s="11" t="inlineStr">
+      <c r="D46" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxPanlvR1V1eVVpdmYxNVNGMnd6UjJFd0J6Zk9IU1lhOW1GbmVTcjY4QkJCYkl3Y3NOU25VRTBUekwtS3plV0NVdlZtOTZZRHJWZ0FVdDl3S05aMlFWeEZiYzdwYmQtVnJxZEw0NktHaFZMNlZkUC16empqRGxxMEhhZGwxRzVEek5FelB3aE9UWFhGQW42b21MRnJHUXV2ZGJYUXJIMnVFWGZsSnEwazNGNUdVcjVoekp0NEZCN1J3cTlaZldFa1pMUkJTbVZYeFljVkRqQmlZV1M2aXh0ZjI5dEI1NDB0UElPUERsbUljMlA3OHBnYmtJTXFWZWkyUdIBgwJBVV95cUxNWFBRQ05GUDdwTWJ2ZVFJUS00ZUh0QkpZQVNNcU9JYXRTN21sMS1VZTlOSTh2LVFuZHh6UVk2djlrdWFsd3MwcDFCNmhwUlVLTlpjVF8wSmt1YnBWRE9tNVpKQlk2YXJWdmwzZWlLX0xpaWxSMUpsX3ZjYXhmRmE2YlAtSFJGRG5pQnVmMnViQXlsVFV3OU1hZFVrY3ZITHQxcTR5UkZ5U1pReHVJMGZGM2FCZWliSFZQZmpVLThSdExWMW14OElodmVVSC05SUh1d1hBenJoY3BUZGxoM0NTbTExdERmM3pjZGd4VzgyV3BNOG11TElBQ3NsRGhtSEc3YzJz?oc=5</t>
         </is>
       </c>
-      <c r="E46" s="11" t="inlineStr">
+      <c r="E46" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1784,7 +1787,7 @@
       <c r="F46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="11" t="inlineStr">
+      <c r="A47" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1794,17 +1797,17 @@
           <t>PAC Capital’s Clayton Larcombe charged with assaulting wife</t>
         </is>
       </c>
-      <c r="C47" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D47" s="11" t="inlineStr">
+      <c r="C47" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D47" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOLXNDU2xjMWpyeEZwWGwtZkV0TjNSbGtWS3ZidUo3a0dvV1hrTnJiVXBXSkJNWlhXYXFHZkNTa3g4a1ZfMjRPM3BtWTZUNGg3S09kbGI2TTRGd0Jkc1A4WFAycjlpVC1URjFvNnBraWprRkhaT0VOWkh6N0xkUjNXNUw0dGx2N1JtTDVsREdtZDhraXVsSkxhR2ozamFUSGR5VHBBRm1Zcmx1c2RDaUIxQkVpeUpfWjFNeTRLWVRtYjluZ3ZncGZIMQ?oc=5</t>
         </is>
       </c>
-      <c r="E47" s="11" t="inlineStr">
+      <c r="E47" s="12" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1812,7 +1815,7 @@
       <c r="F47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="11" t="inlineStr">
+      <c r="A48" s="12" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1822,17 +1825,17 @@
           <t>China touts itself as ‘harbour of stability’ to global CEOs</t>
         </is>
       </c>
-      <c r="C48" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D48" s="11" t="inlineStr">
+      <c r="C48" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPUzBWeVk0elBOZ0l5QU44TUJvU0RvSmtPdmVyT2VuQTczaEdzbkktT25ZT2Y0Nzh0bVBhQW96TUhpWkdEOEJMVVk2UWxLOENKZGk3X2tQcDNsWGZtU0JkM2U0N3VfUWFBclhUSUZya0NwRTJOWmZJdWlhT3JtY1EtSkJ6TmlsV3dzOXpDaVFMNlBaa3RfRHBjc3Q0cjk0eVdPV2MwcjlHNA?oc=5</t>
         </is>
       </c>
-      <c r="E48" s="11" t="inlineStr">
+      <c r="E48" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1840,7 +1843,7 @@
       <c r="F48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="11" t="inlineStr">
+      <c r="A49" s="12" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1850,17 +1853,17 @@
           <t>Eyes on 3D Energi as oil and gas giant Conoco flexes buy-out rights</t>
         </is>
       </c>
-      <c r="C49" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D49" s="11" t="inlineStr">
+      <c r="C49" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D49" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWVU1QmhTUGFkYlpTQkw1WUFPTHhmbk5lbnE4T1haQUswSi1ITHlhVmhyM3ZYS3N4cVd6ZkwzdGdhT1lvM1JJek4yLXFpSWoxUnRtR2JRLTZWa2dlTDVTakE3b2xvazFWX0kzRHFZWVB4OUh0XzFFd3JVSVlfelpVa21qTldCVHdvcmJYcGNjZ1RrdElWS3Yzck9KYzRvbzloWkNqMnQ3dmtHbzNuc21ZSXNYeEFlZw?oc=5</t>
         </is>
       </c>
-      <c r="E49" s="11" t="inlineStr">
+      <c r="E49" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1868,7 +1871,7 @@
       <c r="F49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="11" t="inlineStr">
+      <c r="A50" s="12" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1878,17 +1881,17 @@
           <t>Blackstone tempted by $900m payday for Sydney’s JPMorgan tower</t>
         </is>
       </c>
-      <c r="C50" s="11" t="inlineStr">
+      <c r="C50" s="12" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D50" s="11" t="inlineStr">
+      <c r="D50" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxQNEZTZjY0S2YzcUxsb25RSDk2NHd1N1VOVlpMbi1JNGEzbUt5ajlYZFhvLWNBTkNQVXNuWERfTkl0Z2o4R1U0Zk5jVE1FTW5TTUJGZnNJc2NqMm1fT2dmYTVwRGU2TkZ0c3BjZVBGS29fWFJvZ2F0MWNLa0pYY0RNME5xYS1vOGZmMDVBcDBaLV9MWF9od0EwekFyb0ZCOEdkNTFaN3ZXckJwd25zS0FsdzU4OW1UODlueGNyZVBDSDZkeHQwelV5ZXVDVlcyUkhKWDZfVlRacEJHSElmNnhKSXk4ZHJHWHhPTEV5NGNkcmhyU0hjV3J4dVBXbnRGQdIBgwJBVV95cUxPME4ySFF5RWNrejVlWW1yeW56N244RGpyeVJUZEgyTjFNcE10YjVpMmJyeWsxTENzZFhPRlpsbl9pVXl0NGJvUlZFT216NE1KRFNwOHVZVXMzanNKNXFmWEdsMndsd1cza3NTTzUyUUZfaDEyWHJwZEtQbTdJRmkyU3A0RGh4QlAtT1lRVXk2SGoyaTI1NUpwVExYSkZJNmVFNjdXTDJTNURFOEh4Y1dnUDVGdjBpaDlWVWJtUHZiRDdGTmE5R1R6TDBwWFFnT2MwQ1lmT2w5bDF6eVU0R20tYnpnT3JCZlJod2s0UndyZTM5M2xLZC02a3E0NmJRdFV0Qkow?oc=5</t>
         </is>
       </c>
-      <c r="E50" s="11" t="inlineStr">
+      <c r="E50" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1896,7 +1899,7 @@
       <c r="F50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="11" t="inlineStr">
+      <c r="A51" s="12" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1906,17 +1909,17 @@
           <t>I-MED attracts mystery suitor as Permira weighs sale or IPO</t>
         </is>
       </c>
-      <c r="C51" s="11" t="inlineStr">
+      <c r="C51" s="12" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D51" s="11" t="inlineStr">
+      <c r="D51" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxNaGlwS3d5MGFMbEg2U2hnZUxMQmdqaWI4bS1lblNZOFhkSnRMcUotRkZMTjhFZkRUQWxUUDVtYml6TVAxUXkyZmx3SHRFb0gzVHRST2ZQUThKa25aWlhlcGprSU9tWktXZjZRaC12bFpkaVVWZHhIMERyeVNNWEswYTJ2ZHdnRFVRaFhod2U5N011TkQ0NG5MYVhoT3MwRUVZdVB2UVhKZExvdFIyXzNNUGt2SHJUanQxRkI3bXlLSlNJQTF4NXQ1YlZDaGVBM0EzNUhYQVp6NkFWRzU4bnRPWTgtXy1HVnB0ZlN0Uy1rY2FuWlNfN1U4WXVHQnRzVkNG0gGGAkFVX3lxTE1GaDJJdTJlOXFEZUtDTmdXMmsyLXlpaUxzQXpycHk4MTdHZng0dVczYWVwdWRzdFFCMlNLWkZpMm5Zd2RpN0Y0Zmo3Q1FOZFBZQlh5LVl6aVZ3X284UmpxM0pVRzZmMmpjaUdNWnJPZGV4V3lNai1CTllCcW5oUEVxaG0zejB5anc5YnJEZzZPT2d2QklCWjl2MjRBc25jUndqZkVadllKaUZScG12bEozT1NKUUJYR0pHTGtJZVc0ZHZLNHVSYlhzcTE0SkZmMXNlVGJ4YWJ1cThxcGlZTDMzRUMxLVM5VHh2OW5tRW1PT3VyRUhDbV8tRzUzVzRzVWZPZ2w1bnc?oc=5</t>
         </is>
       </c>
-      <c r="E51" s="11" t="inlineStr">
+      <c r="E51" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1924,7 +1927,7 @@
       <c r="F51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="11" t="inlineStr">
+      <c r="A52" s="12" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1934,17 +1937,17 @@
           <t>The stagflationary mix that has billionaire Solomon Lew worried</t>
         </is>
       </c>
-      <c r="C52" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D52" s="11" t="inlineStr">
+      <c r="C52" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPWTh3S05XQWpTQm03WjhBT1pWc2cyOFRMd2ZraHhPUHlDRW1tWkZvdkhQWHE0MHVMRUpaOFRoX0JsYWhJV21nVkpIM2RBSmlZRUtEbFAydzZfOTh1S05oNEZPOGgyZDJRMS1uLThWYWRVT3VEVGhtYkVLN3J2OWsyX0VVdTUteFBCOVNKZ28xUTRPTk1SUkMxZ1NJc1B6NXRrUEEzOG01YnZOYjk2cWlFZA?oc=5</t>
         </is>
       </c>
-      <c r="E52" s="11" t="inlineStr">
+      <c r="E52" s="12" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1952,7 +1955,7 @@
       <c r="F52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="11" t="inlineStr">
+      <c r="A53" s="12" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1962,17 +1965,17 @@
           <t>Oliver Curtis on Firmus: From prison barber to AI billionaire</t>
         </is>
       </c>
-      <c r="C53" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D53" s="11" t="inlineStr">
+      <c r="C53" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D53" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQek9VTlV1b2hVb2RoZ0Fya0REb3E3YlBCR2NYZldXcEh2VEY0LXg5bjd6RzlnZDI0OUJJd2cydTBwTm9tdHpiZ1lSMnhtcmJSYVRKbzJFMjdDaEJyZExSQVJVRDh1c00yMjFMaVlPdnRuV3VkTjNxdzFRbW1yeGltSF8tVXlJVXJzTEJXS2FTYkJTVkdKbmdPTTd6YzRtYV9nN0JzOVZNTzhUdUk?oc=5</t>
         </is>
       </c>
-      <c r="E53" s="11" t="inlineStr">
+      <c r="E53" s="12" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1980,7 +1983,7 @@
       <c r="F53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="11" t="inlineStr">
+      <c r="A54" s="12" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1990,17 +1993,17 @@
           <t>Three startups that raised $161 million this week</t>
         </is>
       </c>
-      <c r="C54" s="11" t="inlineStr">
+      <c r="C54" s="12" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D54" s="11" t="inlineStr">
+      <c r="D54" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNRGVZMF9DeGJjX29vN3B0blVoM3RKSlJJTllrMThKUDJNZzdPNFNnT2JyTElUOUYxMHlsUm9yM2dBQnZfaVNZblpqb3NzTXdHVlpQNkRqR3NBZHdzODdjN3RKMTZhSVRqUEM5d3JRc3F2OG9hWmZJdU5rakg4ck8wLXlMTnZSU0lNaERmQmswbkVGWW8?oc=5</t>
         </is>
       </c>
-      <c r="E54" s="11" t="inlineStr">
+      <c r="E54" s="12" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2008,7 +2011,7 @@
       <c r="F54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="11" t="inlineStr">
+      <c r="A55" s="12" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2018,17 +2021,17 @@
           <t>Iran eyes ‘plenty more’ vulnerable energy targets in costly war</t>
         </is>
       </c>
-      <c r="C55" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D55" s="11" t="inlineStr">
+      <c r="C55" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D55" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNLUN1MHlZaTNfVHhVX0RnTXp5QW83RmM4WVZkWW1PSnNaZF93VkY5ZF81anB3NDNmX0kyMkVSdkxNSURvSEh6enloWnRVcTlsR0JPTjVzNFR1YjRsSm52VnA1XzFFUlUtODJjYy15YWRRdWZZRkdjRXpCcEFSVURmV3VpSTFhTjVUb1d5bmw3NHNlT3VQZU9ieEYwM1J1TGEyZnlnWXNIWFJUMEtIOVZad0dxRWZBdw?oc=5</t>
         </is>
       </c>
-      <c r="E55" s="11" t="inlineStr">
+      <c r="E55" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2036,7 +2039,7 @@
       <c r="F55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="11" t="inlineStr">
+      <c r="A56" s="12" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2046,17 +2049,17 @@
           <t>Don’t take it personally: Bain Special Sits hits hurdle at Infinity</t>
         </is>
       </c>
-      <c r="C56" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D56" s="11" t="inlineStr">
+      <c r="C56" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D56" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQRjdwTk0xTHVIRHNkdG9tVk1EQ0hiQjJ6dGcxaWZRZ0hZV1U4YjJDU0tnTUlWSkQ1S2dUTHJVNk0tNWQ2cVd4dkw0M25leXRreWJtdlBKYTAtNzRocTJUazh1dnRzSVlYZThySTBNVjg5X0xYWUxCMC1SelltSHVSUEV5U3B1bTA2NjAzMGFZLW1CNkQ3aWU0S1JxS0d0YmZiZjBKQVRNVUpzYno5R1pvbTBsaTM?oc=5</t>
         </is>
       </c>
-      <c r="E56" s="11" t="inlineStr">
+      <c r="E56" s="12" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2064,7 +2067,7 @@
       <c r="F56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="11" t="inlineStr">
+      <c r="A57" s="12" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2074,17 +2077,17 @@
           <t>Drill, baby, drill: It’s boom time for mineral and petroleum explorers</t>
         </is>
       </c>
-      <c r="C57" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D57" s="11" t="inlineStr">
+      <c r="C57" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D57" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNdlFOWld5ZWhPVnFRa2xidWlUVzluQzkxUTgxR0t0Rmg2S1BzNjdINnhwS3VLRkNjRVJLX0RHU0h4VFVRY2RfSHBudEhfNVNjeE50ZUxQenJNSlJtWFRlcnNsZm1iLXlxM2RmVDViWEtjNDloaTBhUDVxYkNfOWFCTjV6cExEVlFCMzNfWnVwRDJHYWxWV0hOR2V2S0VlV2NyS2s5cWNmREtWXzlMMDRQNW1tVlBOblp3SHBEVg?oc=5</t>
         </is>
       </c>
-      <c r="E57" s="11" t="inlineStr">
+      <c r="E57" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2092,7 +2095,7 @@
       <c r="F57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="11" t="inlineStr">
+      <c r="A58" s="12" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2102,17 +2105,17 @@
           <t>‘Wake up’: Fury as farming crisis looms</t>
         </is>
       </c>
-      <c r="C58" s="11" t="inlineStr">
+      <c r="C58" s="12" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D58" s="11" t="inlineStr">
+      <c r="D58" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNelJvMXFPX3MwUVRMN2xqbzE1MWdvOF92Zy02YmIyZW9SQXRNQVZsS0xVVG9UdkFPaTV6ZC1tV05SZWNqblNFZ3Y1VGNaVVBaaEl6aFJqQ09ONDVkNUs4TzNvVjV5eHNjUk9xaDRFZTM0alpuYUdvWGtLRzRhYXN5alZ1QWdsZTEyODdQVnZoazkya29WeTJZVmpxLVBCdWxfY0dTN2Z3WFZlSy1sVW44RDlvZFAzYlhnQ0N6UWhKSU02eF9iZllIU3g5MWtSbkJzZGxWLUxHNERzdUlLTF9VYmpJSTRLY3U4NlVVaDhmc09uOWwtUGtlb0I2M05DR1dnRWxGSFV2NEJXaEF4c00tN9IBlgJBVV95cUxOSzZ5NXZMTTlZa3BSNjZyTUxUMjRhYWJhN0hMa3dDcW9CWGstNnI5MzV5U0hJSTdKLTFwa2E5YUItZnFRbW5RbzVuYW91MmZaYXN3R25hWVpUbW9oUU9fVktPRHROVDYyd2dSLXJVZWQtY016bkVxY0VPbkY3Zkgtb1liWGMxeEpyYmloS1V0TVJMMWZaeWRZX3FQRjBmVzJwdkkwMEVDSXV1MTdReUhGZ0Z3dENyMEFkLUl1aXhtRkFLRFFXcEdMZzFuT3NxRDFMOGVaY2YzeXBQc09fY3YwcFp4MVczRVN3d3dJZWJfTFFscjF0cUtRWHdzTUptaHowNDhYWXZXTHhYTHNTdlZGUmNlamRTdw?oc=5</t>
         </is>
       </c>
-      <c r="E58" s="11" t="inlineStr">
+      <c r="E58" s="12" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2120,7 +2123,7 @@
       <c r="F58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="11" t="inlineStr">
+      <c r="A59" s="12" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2130,17 +2133,17 @@
           <t>Construction giant FDC road tests IPO pitch</t>
         </is>
       </c>
-      <c r="C59" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D59" s="11" t="inlineStr">
+      <c r="C59" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D59" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxON3p5Y3VPM01XZFk4a3g0R3JnQkZXbHVGV3BKdDB6M3NRb0M0SEl3V0R5RmhCQ3dnaHB0ZHp5N2hCMUFsNU1ZNWZ4YWdNZWdETkUyZmdoeW81amwtTWNFZlc5WlNpMkJwRzk0QklORGhlLWNEalh2d0JCX0lhVHhhUF9ibVlxcHAwOW9ENndVOTY0enBYUWc?oc=5</t>
         </is>
       </c>
-      <c r="E59" s="11" t="inlineStr">
+      <c r="E59" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2148,7 +2151,7 @@
       <c r="F59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="11" t="inlineStr">
+      <c r="A60" s="12" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2158,17 +2161,17 @@
           <t>Austal suitor Arlington Capital Partners buys Eptec’s defence unit</t>
         </is>
       </c>
-      <c r="C60" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D60" s="11" t="inlineStr">
+      <c r="C60" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D60" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNM01qb1ZRZVBIdmp3cFc3R3RLaTdmZk1JOFo4anRtSm95Z1hJc0N0S3VranBTV29IdlViT0FkSm92eHdtbDBqdU5HTHNMaXo0dGRWMkpDdjk3LVRBVU1rZC1YejZJMkhyNmpZZFJodGoxWlB1dkRhYTJVRlljMlV0dUllQ3EtOHZkNFdSUWJLSW9Xemw1XzFzU2RHV1o0RTViOXp0bDZFQTZycWhpNElLU0FZQVI?oc=5</t>
         </is>
       </c>
-      <c r="E60" s="11" t="inlineStr">
+      <c r="E60" s="12" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2176,7 +2179,7 @@
       <c r="F60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="11" t="inlineStr">
+      <c r="A61" s="12" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2186,17 +2189,17 @@
           <t>Eyes on Tom Wallace as clock ticks on Adgemis pub deal</t>
         </is>
       </c>
-      <c r="C61" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D61" s="11" t="inlineStr">
+      <c r="C61" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D61" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxNSExQeDlENWlHb0prRnRldjZ5YWhKVUZ5eVdsYjZmbVRWRWQ0WnZXWkU3UHZJdElnQ21jMU9zNnhnc3JlNDczVGQ5Y0FGV2J3QUp3NXdZTXZMNm5tVC1vWDFtOFN3aS04QVJZb3FZV2VsUmJ2aVgwbUhTaFVGdHg0UjRyTXVVUnFhQmE5eFYwMGR6T1R2U3Q3WEdZclVKNWJiby1IRg?oc=5</t>
         </is>
       </c>
-      <c r="E61" s="11" t="inlineStr">
+      <c r="E61" s="12" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2204,7 +2207,7 @@
       <c r="F61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="11" t="inlineStr">
+      <c r="A62" s="12" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2214,17 +2217,17 @@
           <t>UBS names head of APAC leveraged capital markets</t>
         </is>
       </c>
-      <c r="C62" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D62" s="11" t="inlineStr">
+      <c r="C62" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D62" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNMm9WZ2ZKVFBvX2pYMk16VmY1WFZnZ2J5N0F2bHduTVM0Sjg4STVtTGFLQVdzeFloVHg3clRic0owTDMwYVpXdDVjdjFOWjQxdkdxdFY5MEY1Q1U2Q0R5dFBJWTNtUzgyd3RXcm9uM0hKdEZ3b3JjXzcwQ2VpRm5SS0hYT2gxSU9iVFRlR05Xd2EtM2JOQjBGUzlKdnE?oc=5</t>
         </is>
       </c>
-      <c r="E62" s="11" t="inlineStr">
+      <c r="E62" s="12" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2232,7 +2235,7 @@
       <c r="F62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="11" t="inlineStr">
+      <c r="A63" s="12" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2242,17 +2245,17 @@
           <t>BHP, Woodside rise after new CEOs named; Future Fund chiefs exit; Sandilands ‘doesn’t accept’ termination</t>
         </is>
       </c>
-      <c r="C63" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D63" s="11" t="inlineStr">
+      <c r="C63" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D63" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNUHhZeHNHemtiLW1IOHN1OTZXOGpsM0ZtUG1MVHRCT1hUT1k5S2lEOXlXRENWOXNlMEZadThQR18xSTJfTVlQM3BtX0ptX1J0bk80SzNLUVRtbkJITGgtb0lsSVdJTWt2S1E1WUlXdUdsbEV0V1RpNWlyRXBoc0dPVDl1OXRrSlM3SHlDazg2UlcxenVzNzlhQldhUGhfNE5IV2xrVmVBNzhhSE9qY042Z3pzMEVzd0VyVmZudXgxcTgwWGJXSWZKZ0FyNVhjcmhjTm5DYUVjLUdDRmxUQkZuTDFlUXVaV0ZoSWp5WHMyR3c?oc=5</t>
         </is>
       </c>
-      <c r="E63" s="11" t="inlineStr">
+      <c r="E63" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2260,7 +2263,7 @@
       <c r="F63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="11" t="inlineStr">
+      <c r="A64" s="12" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2270,17 +2273,17 @@
           <t>BHP’s new CEO will shift the Big Australian’s centre of gravity</t>
         </is>
       </c>
-      <c r="C64" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D64" s="11" t="inlineStr">
+      <c r="C64" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D64" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPQnZpWndNZzZvN1VsOHBmRDVLRHVTNkxLeDVDelpOMURjOTRDSDZfN2dPZlZqaW05WEZuZXMyRTJZeVZnV0poT2UxRkVfZ1RZSjdvUjVKblhoSU5Cd1plRTVNNTRaNWZmbm1yUGZkblVpYkctNzVRRkVQQm4zX1FtRG1KV2Y0djUtOURianJ3dElqeXBUMFp4aWFEWVFYelVjYTluSWpOM1FlbHpIaUxXdnBn?oc=5</t>
         </is>
       </c>
-      <c r="E64" s="11" t="inlineStr">
+      <c r="E64" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2288,7 +2291,7 @@
       <c r="F64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="11" t="inlineStr">
+      <c r="A65" s="12" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2298,17 +2301,17 @@
           <t>How philanthropy became the sandbox of succession</t>
         </is>
       </c>
-      <c r="C65" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D65" s="11" t="inlineStr">
+      <c r="C65" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D65" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxObnBPb2MzQ1RvSVVCbmNzYWFBMlFjU0dQRmpPakNfdkxtMWc1bFdVNXNlZmRKQnNlWEtUUDNSTHpTLVV4Skx0V2otbTZsTTdvT1VaUDhMZFZoMFFab1RoS2pCcno1WGlNQlY4eXQ0OFEtLXJTay1MUkFSSEJ2MVVScUpjUkhJOThISy1QbHIzTzFlWVhOc29fWWs0V19sQ25hRW9MSGhBVVNKWUp6dUo3NS1SWlk?oc=5</t>
         </is>
       </c>
-      <c r="E65" s="11" t="inlineStr">
+      <c r="E65" s="12" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2316,7 +2319,7 @@
       <c r="F65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="11" t="inlineStr">
+      <c r="A66" s="12" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2326,17 +2329,17 @@
           <t>Advanced Navigation raises $158 million Series C round with NRFC backing</t>
         </is>
       </c>
-      <c r="C66" s="11" t="inlineStr">
+      <c r="C66" s="12" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D66" s="11" t="inlineStr">
+      <c r="D66" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNTXhwVlVLUy1pWEpFdzFCazNTY0dkczd4WW9oeW14cUtTaDZRTGlVQXBPaHN4WTBkNW1zOGxvN0tVWl9JSFdVNXlQMzVxbk4zbDZFUjNOcUxSamNaSnFCckMzWEk1VlNoSHJHQ3VWdGltVWZCV0c0NmU4UlN6YU55Q0J2TkQtUzBzOW96UXRxem5Zb3M2SUljNURISlRkQmJD?oc=5</t>
         </is>
       </c>
-      <c r="E66" s="11" t="inlineStr">
+      <c r="E66" s="12" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2344,7 +2347,7 @@
       <c r="F66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="11" t="inlineStr">
+      <c r="A67" s="12" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2354,17 +2357,17 @@
           <t>Kal Somani-led consortium buys Rajasthan Royals for USD 1.63 billion</t>
         </is>
       </c>
-      <c r="C67" s="11" t="inlineStr">
+      <c r="C67" s="12" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D67" s="11" t="inlineStr">
+      <c r="D67" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOX3lmdG5aTmk4TEpBa3ROdWZ1aDJHUElBQXktVmlKaHFmTUhPX1QxX1dKLXZfaHRDQjBnWm9McTZjTjJtTWFETTRNMHgzN0tTTm1xY0JpMF84Q2lNaFQyZGVjaHN4bkVmcDN5Qy1ta3FtYnpMSVVyYm0ydWpTRUdZU1hoYXpaNkZUQzlPc1QycjZ6aG5QVHRqY213?oc=5</t>
         </is>
       </c>
-      <c r="E67" s="11" t="inlineStr">
+      <c r="E67" s="12" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2372,7 +2375,7 @@
       <c r="F67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="11" t="inlineStr">
+      <c r="A68" s="12" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2382,17 +2385,17 @@
           <t>KMD says Rip Curl demerger proposal delivers investors ‘no value’</t>
         </is>
       </c>
-      <c r="C68" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D68" s="11" t="inlineStr">
+      <c r="C68" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D68" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPTXhBdHByWE9EbllFdDA2OW1UTUZEMVJfV2xsNFdURFRKX2JrODJReVRuQlFoakpWbTBKcjhNLUVsNE9sdG5LUElLZlVrbFNERS1QZTN6bEZIWEhXZ1pTWG5GWEw3ZmNETTdDUDUzYzR5M0E3ZGVlTWpSUnVlVU56dDNFZUtZN3liZ1dKNzJhLWU1S0M1ZnlKd1JNWXlxSlkyU3pGS1lhS05hTUJPRkxucldabzFucGs?oc=5</t>
         </is>
       </c>
-      <c r="E68" s="11" t="inlineStr">
+      <c r="E68" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2400,7 +2403,7 @@
       <c r="F68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="11" t="inlineStr">
+      <c r="A69" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2410,17 +2413,17 @@
           <t>Ex-Macquarie banker drives mortgage broker roll-up Recludo towards IPO</t>
         </is>
       </c>
-      <c r="C69" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D69" s="11" t="inlineStr">
+      <c r="C69" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D69" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxNQms5X1F2aTNhOExDbW42TlZOLVJwVWxna1JYSW9vWF9Na1RZa1ViTFdZc0tCcXRZZkRudTlsTzNuZGgwSENyYi03Zjdfc0lZTXp0NmJRZnhzb2pWRXRIOUdJN2lQM2h3ZFFtTXlSWHVWOFBIaW1Na3FQMjBCck1nVlhUcmRkLW9LOHpKWXQwTm9LcWR5M2FfdjFiRW04TndoanR5NmJvMENGalNuUGNINy1Qc20xR1J4d21ncHNNSUZqa1BXNnI4STIxSUFkZXdU?oc=5</t>
         </is>
       </c>
-      <c r="E69" s="11" t="inlineStr">
+      <c r="E69" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2428,7 +2431,7 @@
       <c r="F69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="11" t="inlineStr">
+      <c r="A70" s="12" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2438,17 +2441,17 @@
           <t>Coles reviews truck fuel charges as crisis worsens</t>
         </is>
       </c>
-      <c r="C70" s="11" t="inlineStr">
+      <c r="C70" s="12" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D70" s="11" t="inlineStr">
+      <c r="D70" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxOSGpBM3RjLVJ3LVlmR1QydnY2dm50WlVxcG43ajRFZ25QS1hDNTBONU8tY3Z2TklzbUNla0ttZk1GZzFaLUZRakFjSUpUQWItQ0VqVTVwS1B0QS1ObVEzNzdRT1l6aU9pVm5jSlhna1N6QmFKT3k1RkhMZGNTVnVLcDVIcXZmRjdjLWRpYVlRQUVmcVRtM21BSjVhTGNaaThyZkhLS2NWdkNCSkZKTlloUVdtbzRnYjFKbllOZXhOd3lkcFZEYURwUFVNQzVnSWRyM1RlOGd2M1pMZXI3c0NIa0Y0MNIB6AFBVV95cUxNSjB3Z0hoTGxwOHJQQ09xb3BmRmhCYjBCc2E0OHA2elFDRE45UGpaTEVDc1Y2VnRvVmZQUzRHbng4QTMwNGZZNGpmaVlHRmV6bnhiZ0FReU50TnRiQ0NZMEtoM3dBZ0hXbFBZMVJQNXd4LVdXRDVyTDAxNS1zeVdvcFVvend2N3J5R2pLYmhxNVFfd19rUlRsNWNndlptMUVkcS1CaUN6UXRHVzByTU5BMW1TdktOZUJYck5xMEJucmR6czIySEMycDA5cmR1MXB0N25Xc0JDUG9zN29YWklVc1BUMzl3UVhn?oc=5</t>
         </is>
       </c>
-      <c r="E70" s="11" t="inlineStr">
+      <c r="E70" s="12" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2456,7 +2459,7 @@
       <c r="F70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="11" t="inlineStr">
+      <c r="A71" s="12" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2466,17 +2469,17 @@
           <t>Sam Arnaout’s Midas touch turns suburban pubs into pokie gold mines</t>
         </is>
       </c>
-      <c r="C71" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D71" s="11" t="inlineStr">
+      <c r="C71" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D71" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQV2xlTTdYOFpIMzNmVVRnMlJRbTdGTC1jelVCd1V3UjN5cHQ1VzhWZzhrNW1PNm1RX3FlZmU3UkRycjF4WDlQUzRMcVVYY1g3UTZqQ0hxRnl2Ti1IQ0owVmZjN3Jod1BFbmhPVUwxNjhsTGh6d0kzdU01N0hmempRZ044ZmZNUllnenhyc3djRGJOdEtrekx5UVFoaFFMWDdqMHMwdng1SFg4TzZHY1hQNFJNN3huZXpWYWFtQ0ZJakhkVFlQcl9SQlRfZkQ?oc=5</t>
         </is>
       </c>
-      <c r="E71" s="11" t="inlineStr">
+      <c r="E71" s="12" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2484,7 +2487,7 @@
       <c r="F71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="11" t="inlineStr">
+      <c r="A72" s="12" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2494,17 +2497,17 @@
           <t>Gentlemen at Melbourne’s exclusive The Australian Club sweat another election</t>
         </is>
       </c>
-      <c r="C72" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D72" s="11" t="inlineStr">
+      <c r="C72" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D72" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPcEwyU01BOXF4TzlmREhYbTFEWklxdWZqWmZybDVnOWtLQ2dTU2dNQ2t5M3BVT2stN08xYkFmazVkY29oT3RVc2xUZmZINFJURGtIRTg4RGsxOURBdWEybTUwU2NUODQ2eDNBbTdPT3QxeXRFNHlSc014T0g1aG4xZ1A0U0FWMTB1Wm1CSHlQU0ZJb3lMYkE?oc=5</t>
         </is>
       </c>
-      <c r="E72" s="11" t="inlineStr">
+      <c r="E72" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2512,7 +2515,7 @@
       <c r="F72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="11" t="inlineStr">
+      <c r="A73" s="12" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2522,17 +2525,17 @@
           <t>Inside Fortescue’s AI ‘hive’ that could save the mining giant billions</t>
         </is>
       </c>
-      <c r="C73" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D73" s="11" t="inlineStr">
+      <c r="C73" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D73" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOSVVCbGpzcVcxTGlZZ2dTUkxXdVVvVU1ONEtUS0t1R1VkWWRNeUF1UmlHbXd6clR3QVRuWGxrUGQwVG1OeUxZb2RqTzdYOEVGQ1N6eDFta3VOZDdHNThYbUEwWEVHZlZBVzNpZ1Foak1kLURZTWpJVzZLekczdzFrdHMtLVZwMUZnYmkxSVc0czFqWnFaSGZiT2pIVW5rdVZmdThreFlRZWVEU0xoa1VFOV9MTjE2UHFOcWhqUzVB?oc=5</t>
         </is>
       </c>
-      <c r="E73" s="11" t="inlineStr">
+      <c r="E73" s="12" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2540,7 +2543,7 @@
       <c r="F73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="11" t="inlineStr">
+      <c r="A74" s="12" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2550,17 +2553,17 @@
           <t>Tiny house maker Elsewhere Pods seeks cash after Bunnings debut</t>
         </is>
       </c>
-      <c r="C74" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D74" s="11" t="inlineStr">
+      <c r="C74" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D74" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM0ZpVnBTS21Ib25qa09CaU52Z29kZWhTU0FJLW5VR2JCLVFPTVlZTmpYX3lZVWdtMDVTYTJkWHlPUmhXa0Rua2ZXTTBWQU1VdmFrV21KOGlrdjJ3TTdxbGlvZVBUZUxUWE1uelpWMGxWWk04UndJTXVKQjBZUEtoX3lodmdpMWZKNUc1YTIxVFZLYkFKT1QwbS01WU01ZUZTTlczY2ZpLXlpTjNJTWpsUg?oc=5</t>
         </is>
       </c>
-      <c r="E74" s="11" t="inlineStr">
+      <c r="E74" s="12" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2568,7 +2571,7 @@
       <c r="F74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="11" t="inlineStr">
+      <c r="A75" s="12" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2578,17 +2581,17 @@
           <t>Chinese consortium emerges as dark horse in Made Group sale</t>
         </is>
       </c>
-      <c r="C75" s="11" t="inlineStr">
+      <c r="C75" s="12" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D75" s="11" t="inlineStr">
+      <c r="D75" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQYlpEY0hxNm5lalIxSTUzbDE4UEF5QTNpMTl4dWNPMkRrMU1yQnltZ25WcUkwOU13V2Y2RGItVW5QTXotSnBZRUJMdGJySGw0NVVxc3ZLZmVEcTlfU193Vkd5UVVuTFVYWFNtd185eGlVQW5RRElHdk5pMjhUR24wd1k0T0I3cW9qTG5Lcjg2bV9aNWsya0FYODRjeURyMW1EeHdYT05iZHZhLVFrUVNoV25idnZYZ2lpZEhta2JxOWFJb0M2SE9hbFF6NlVWYTM3QmF5anpWOEZackZiTDBfN2gtX1luQkxFOUxSSNIB8gFBVV95cUxOQklMYWl1ZkRqZGUwN0ppeXFubzZWNTNmeE5GY1BfcS13N2dFT096YW9JSndVX1EzTlBKdWZIemdKZnRIME9SQk5aT1M2WnRESjJxckFTaUdOSEd6eG9hRVBjdlhBbWQyWGpUS1kwQXJsdlpkLXJpXzJZX2xiUC1FSlNnNTFoVXQ4bF9JeUp3UGRWdUFOUVRrNUtsRzRxaUczb1p2LVVucFBNazhuZFNDaUZDR2ZQUVdObmVtTnBndGlkazZqeHVheVNzSE9RY3Bad0lrckxDSWY5QXBWS0hwVzZvSTZjaGEtNkNncW1RRE5uUQ?oc=5</t>
         </is>
       </c>
-      <c r="E75" s="11" t="inlineStr">
+      <c r="E75" s="12" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2596,7 +2599,7 @@
       <c r="F75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="11" t="inlineStr">
+      <c r="A76" s="12" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2606,17 +2609,17 @@
           <t>KMD faces uphill battle in capital raise as key shareholder baulks</t>
         </is>
       </c>
-      <c r="C76" s="11" t="inlineStr">
+      <c r="C76" s="12" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D76" s="11" t="inlineStr">
+      <c r="D76" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxOVTU0OGNfRURNcDdzYUtIcG8tR3N4OFFYalhKNWJBaUd6ZlQwNU5MZVZYbUZVSzB3WmdOOFdTZHlBOXBzSGdYUVV6eGt1UndHN296bENxZzNUM2NoaV93LXZaZFNNOXJ2YlA4RHNFS2FDb1ltNWpPWUdRR3VGMWoxaU5qYm9VSW9yUW5kS1NaN2RSc2YtcHZRSTB6aE9Zdkl3NG5nbVRzODRfQVYtelo5M3g4R2JEbnpraFpWbENOZzE2Qndla2t3MXRPWkU1dXg4NmZRME1jT3pOOHZOVlpTZGloNENUZllaSTFmWUV1Y2JLck02ZDhnTHJ5bUPSAYICQVVfeXFMUEFXR29tQjlTbTdMRVNDWUlGNFNOQjVhX0FiSkl0U2stbml5VHR4d1g3bDFqMUw2TzR1eHhYOU5ZUmJpZ2xBY2NzcmJRX3MwaEQ0YmpzMUFnV1BQNGxmcnlXUzVvbHpwNEo5dWFnZlduZ0Z2dGZGRFRKRTNCUzctZDNCd0FMNEkzTm84dmZOM2NKYk81RERsVnlZN1VZaXp5TW5QRVAzOHNXQTFWdVlKdGtFX0FmcU1EbElZSm52alBQeWx4VnlvOFRwNk1ia2lZYXlpemQ4cFdmckotMmMyRGE4ZXN0dThQYmxxUkpvMzAwRXBBcVJuRnp0QkZ3b2tqMWF3?oc=5</t>
         </is>
       </c>
-      <c r="E76" s="11" t="inlineStr">
+      <c r="E76" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2624,7 +2627,7 @@
       <c r="F76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="11" t="inlineStr">
+      <c r="A77" s="12" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2634,17 +2637,17 @@
           <t>AustralianSuper claims another listed M&amp;A kill with Pepper Money</t>
         </is>
       </c>
-      <c r="C77" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D77" s="11" t="inlineStr">
+      <c r="C77" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D77" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOY0RwcnpWZlhfOHA2MG13MkJUX1RDNF9wN2RxZGU2cEpzS1RKTjJDeUl0OERFOGhFRXJaSXNETEhHbW9PS0lua283RnFVbHJvTlRva0djQ2lRSGc2RENJYmt0OEsyYTRVSzFGeE9jWVhKMVRnd240WXVNTVdac2lOUGJSZlc4UVZ5RXo0OTlQbUd6NWRSek1HZG9fZGk2aDhDelhGVmk4YkRKeVV1M0VHZ2hZNmFVdXM?oc=5</t>
         </is>
       </c>
-      <c r="E77" s="11" t="inlineStr">
+      <c r="E77" s="12" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2652,7 +2655,7 @@
       <c r="F77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="11" t="inlineStr">
+      <c r="A78" s="12" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2662,17 +2665,17 @@
           <t>Apollo to Acquire Nippon Sheet Glass in $3.7 Billion Deal</t>
         </is>
       </c>
-      <c r="C78" s="11" t="inlineStr">
+      <c r="C78" s="12" t="inlineStr">
         <is>
           <t>Wall Street Journal</t>
         </is>
       </c>
-      <c r="D78" s="11" t="inlineStr">
+      <c r="D78" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOanpORVBremoyamJyZ2FqQWVOcDcxa2NpempBUmNYcktMLUl1Mzg5VDloWmlVbUdNUnplVk90WEUzXzJjNGxENk9LcGF0enVSdlFpWU9nd244YWNTS0ZHd1JTZEtlbjRQTmJUU0dzWmlDOVFhR1ZRSFJkNXN4a3FHdGozcUcwdHRseXpYMFREUzBNcXRmQ1VCN056SWlEa1l5VVE?oc=5</t>
         </is>
       </c>
-      <c r="E78" s="11" t="inlineStr">
+      <c r="E78" s="12" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2680,7 +2683,7 @@
       <c r="F78" s="3" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="11" t="inlineStr">
+      <c r="A79" s="12" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2690,17 +2693,17 @@
           <t>Estee Lauder in talks to combine with Jean Paul Gaultier owner Puig</t>
         </is>
       </c>
-      <c r="C79" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D79" s="11" t="inlineStr">
+      <c r="C79" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D79" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPSjN6QnFVbmdHWFoteURWaU5VaWZmRmpTT3QtYm1tZUFyNUZyLUdheGdfWlRBTlJyTlp4THIwVDA4U3BnWFNpT2FpZlZzX1lJSDV0MkRGVjYtNVc0b0lOQy1RSnFGTWhCTWE2ZFFPYlFQX05yaVlfZF9IUEN2ZWkzQ0VFMUxxdHF2ODNQY09xdWlqWEczSC1CZk5wYU9QQlAyaTMyelJnaVM0cmN4M0paNzlBdzM1RndoZE8yRHN4UnZqaXVhVmx5NFpqS3hmUHhUdlpF?oc=5</t>
         </is>
       </c>
-      <c r="E79" s="11" t="inlineStr">
+      <c r="E79" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2708,7 +2711,7 @@
       <c r="F79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="11" t="inlineStr">
+      <c r="A80" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2718,17 +2721,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C80" s="11" t="inlineStr">
+      <c r="C80" s="12" t="inlineStr">
         <is>
           <t>The Age</t>
         </is>
       </c>
-      <c r="D80" s="11" t="inlineStr">
+      <c r="D80" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPdUtyNWs5YmxJMXNsNWtaMi1WMm5SVHd6ci1ReURLajdYd1IzWGJMZmE2MzJsSzAxQWtSTm8xMUEwNTh4Vy1zTmFsWFBKTkJ0YXc3ZkcwOVk2a2VNRWVGUS0yQzZhSXlCWmpDYUx6RmpTTlNhS0xIQklyVFdIVXJRZTNPaVB4TG4yQ1R1ZWF2MWpmSG81TVRaRzdtMXpydWhBS2w0a3ZPZFI5MnFKOW5tN21oUDB3NkNtQmR4LVVBWW9BUQ?oc=5</t>
         </is>
       </c>
-      <c r="E80" s="11" t="inlineStr">
+      <c r="E80" s="12" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2736,7 +2739,7 @@
       <c r="F80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="11" t="inlineStr">
+      <c r="A81" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2746,17 +2749,17 @@
           <t>Australia’s new millionaire factory: Start-up to $1.6b in five years</t>
         </is>
       </c>
-      <c r="C81" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D81" s="11" t="inlineStr">
+      <c r="C81" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D81" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOVkl5N1NGWS1XWWZSc0pHXzE3MUNERmV5SUgyQ3o2MmJ3U3Y2YlNwUXNSTGlQenBwVFdnMWhoT2FrcDAwUHNVU0RQbjFHMjJiLU1TRC1nemdrX3hPTG93VWZUQUx3Wk9HT3lYd055Z2FtREFpOWRlYXFDb2hwV0cyWFMwaHpsLU0ta2VVQlpid1dlYks0ZHg5YTY3Ykt6Um5YaF9MR2tIRzd1Tk1IRnBrWVhxVjZNSUl1OE9iRlZzYmQ3QUVnZmhYVGxoOA?oc=5</t>
         </is>
       </c>
-      <c r="E81" s="11" t="inlineStr">
+      <c r="E81" s="12" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2764,7 +2767,7 @@
       <c r="F81" s="3" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="11" t="inlineStr">
+      <c r="A82" s="12" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2774,17 +2777,17 @@
           <t>Social Media Wrap: Genki Sushi Singapore's loyalty benefits; Dunkin Philippines launches new collectible; Burger King Malaysia unveils new Korean inspired burger</t>
         </is>
       </c>
-      <c r="C82" s="11" t="inlineStr">
+      <c r="C82" s="12" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D82" s="11" t="inlineStr">
+      <c r="D82" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxPbFR6eHVTRWZNcUw1TTBJdE1JTFpmbk5iWndKZnRoU3Fmc3cxcF80TnVhRERmY0poM09zTFpCaEVnMGo5aktxY0ExV1ZlZVpHYUtldXBoOUh6bm14SURHNmhnUE9tYnI5YlpXQ3pRZlp0Ni1wM2lYQmdxdjk4SDl0aFN0R1VBbGxpbFVzOHV0TFY3YjJZbDg4Vk1HMTBkQk5LRHd1ZEVpRnBsT1U0Nm1IbVFkZEUybmpabEhuLUNLOGhicUxXZG5UalRLOE5DSzcxRncyNjVRdk8zclhJNkVQcTRkQTZYSEdN?oc=5</t>
         </is>
       </c>
-      <c r="E82" s="11" t="inlineStr">
+      <c r="E82" s="12" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -2792,7 +2795,7 @@
       <c r="F82" s="3" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="11" t="inlineStr">
+      <c r="A83" s="12" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -2802,17 +2805,17 @@
           <t>Copyright ‘status quo’ not working in AI boom times, says Charlton</t>
         </is>
       </c>
-      <c r="C83" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D83" s="11" t="inlineStr">
+      <c r="C83" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D83" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNVVgwdEQ2YUt0eFo3THcxOXZHbUFYZ091VTFKZDZHX0szYWQ2dnZ1dkJma3VZcGk1LUM2SUtQSWhxMGpCUlFZVzdKNmdoSGEycm1oYlBUdEZ5R0ZlU2hrWHpFWXdSN1lCZnZzb3hZc2twVVlWdTNNVXhaR0Nza0FiaUNveXZWQWQ1ZE45MU1HbGNmWlU2aUdha2FyZllzNWdONEpsM2RrdGRFSFl2UlpJUnQ4WGpleGs?oc=5</t>
         </is>
       </c>
-      <c r="E83" s="11" t="inlineStr">
+      <c r="E83" s="12" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2820,7 +2823,7 @@
       <c r="F83" s="3" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="11" t="inlineStr">
+      <c r="A84" s="12" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -2830,17 +2833,17 @@
           <t>The unapologetically analogue 4WD for off-roaders with $120k to spare</t>
         </is>
       </c>
-      <c r="C84" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D84" s="11" t="inlineStr">
+      <c r="C84" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D84" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxPSFJ4ZnNLT3U1REp3MWI2WDFaQm5vZlp6QWN6c0hZamtYVU95WmpkUERwR1dwc0NQN1dEc0FNbHlaMTdLclVHb1JTc2VZNExENGYyUE9OR1BkQ244YXRVeWNwbkxia2VrckVqSy00WV9UNWlvZWJHOG9ibUthaTlpVmRBOGZjLWFzMU8yS2Q5Um05SWIzY2dKajhoMWFUcmFrbTMzai1CdVBNLWczTWRvbTBwSDRfUzNwOHhqQm5hTDdhM0xLWEpNQTRyRXZjU1FLdGhRMUxtOTg?oc=5</t>
         </is>
       </c>
-      <c r="E84" s="11" t="inlineStr">
+      <c r="E84" s="12" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2848,7 +2851,7 @@
       <c r="F84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="11" t="inlineStr">
+      <c r="A85" s="12" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2858,17 +2861,17 @@
           <t>Junk room to become jazz club with priceless Melbourne view</t>
         </is>
       </c>
-      <c r="C85" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D85" s="11" t="inlineStr">
+      <c r="C85" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D85" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQbHN4My1nOGtueVJQZWM0LXNjLTR3MmhuemRJMUEwN09FTUZhZk1lbV9MbnVWblgyUXFEMEl3LUtsOGVqdGUweFR0MXF0ZEo0XzNhWVRqb2pGRUdiNTlLc1dFcXFmdnctQU1wQkRSdHN0T3J6VGt3MU1iNENydGlsOEpsT0ttZmJVZ0FUZmFXSUd3alVzUTQxMzVmcEVXSlV2dWdQd3JsMUZ0d3ZZYlBHaGhKTm9rM01SUmdseE9hT1prbHZtMlhv?oc=5</t>
         </is>
       </c>
-      <c r="E85" s="11" t="inlineStr">
+      <c r="E85" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2876,7 +2879,7 @@
       <c r="F85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="11" t="inlineStr">
+      <c r="A86" s="12" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2886,17 +2889,17 @@
           <t>Zimmermann fashion label appoints new CEO Roberto Eggs to replace Chris Olliver</t>
         </is>
       </c>
-      <c r="C86" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D86" s="11" t="inlineStr">
+      <c r="C86" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D86" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM2M5QU1scVoyNHBmV2lwQ0VQS1Z6d2Qwa1ZkZ0M2WVIzdXR3QnZwVWhUSDRCUEdRZkc5QzFQSFFhNzZ4VE9lWXBTcGhpS01JdG12TlQxSHhValZfbWt3MUdFZGl3RlBtdnlrel83TjNjNFZ0SUpvSDNQbThpU3FLa3Atd0dNU04zQm9OSk5uNHpTVE84aWZpaVlKWkdOQjJjRTZSd1MwMEZ1b3pENkRCQQ?oc=5</t>
         </is>
       </c>
-      <c r="E86" s="11" t="inlineStr">
+      <c r="E86" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2904,7 +2907,7 @@
       <c r="F86" s="3" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="11" t="inlineStr">
+      <c r="A87" s="12" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2914,17 +2917,17 @@
           <t>Construction giant FDC road tests IPO pitch - AFR</t>
         </is>
       </c>
-      <c r="C87" s="11" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D87" s="11" t="inlineStr">
+      <c r="C87" s="12" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D87" s="12" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNTnRScHFhQlpkdEdSb2x1bExxQm96ZE5zSV9wTDNDV2pxYjFQdUtoYmNBell3SFlTTFEzMUhpeXlmNERSeDd6VGppM2szQ1NHVE9PY1R3MTN0SUZLWkF5em8tQ3IycUZ2RmswX0tnN1IwOHl1ZFo4UUtMUDlQbXRjTnRCWFB5cU1RZFhsdDdaWGpMZzh3d29CWWZvZGtnTjl0T1k5ZHFHSUg5XzFSSF9TSUxTYkU0QkFheFlLZUY3S2tCSWRLZWlBbUpxUjc3TXBQQ01V?oc=5</t>
         </is>
       </c>
-      <c r="E87" s="11" t="inlineStr">
+      <c r="E87" s="12" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3182,6 +3185,314 @@
         </is>
       </c>
       <c r="F96" s="3" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>Firmus’ Oliver Curtis set for green light to run ASX-listed company</t>
+        </is>
+      </c>
+      <c r="C97" s="13" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D97" s="13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNR3VmQW9vNmUyeU9WbVRvRG9tcTNMYVlvRUhCd29wTkRZaVlEcG50Z0hIN29XcE5GUmxkUy1yMm0yTm94Q1BXMmNCcXBpZDlqVTRlZFpMX1QyMWh5Ym5XQ3VjYW1ZdDFtYWNyOERCOURuWXM5ZTV4WGthMVVjNUZlcmVTQ3JBUjQzUXRXYXRLQjlNeHpBMkVCVWpsd2Z1Vk42TjJxSlRiQ0ZtaTkzOTZtNmRHQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E97" s="13" t="inlineStr">
+        <is>
+          <t>Australian Economy &amp; Markets</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>Crisis Hit David Jones Chasing Funding As Retail Markets Come Under Pressure</t>
+        </is>
+      </c>
+      <c r="C98" s="13" t="inlineStr">
+        <is>
+          <t>News.com.au</t>
+        </is>
+      </c>
+      <c r="D98" s="13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNNjJSOUVQcTkwUmxXNXg4ZzljSGhnRlBJY0otSHRrX2ZIQXRqWmNDZlgxYW1jckhHd3BtdXJsUWhwTjQ5SGw2NUU3TnFtcmhYd2JVcThIR2VCLWJLU0h5RE8xaTV5TS03Mi1za19hcF9PcXRRSU9PX3ZxSktSV2FfY1ppcUFVV2w1TmF1UWVtZlBWSUhEcG9oRGlEVkEwR2ltQ2VMSTNlcENEYlY0?oc=5</t>
+        </is>
+      </c>
+      <c r="E98" s="13" t="inlineStr">
+        <is>
+          <t>Retail &amp; Consumer</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>Beirut Street Food eyes niche in Lebanese fast casual</t>
+        </is>
+      </c>
+      <c r="C99" s="13" t="inlineStr">
+        <is>
+          <t>QSR Media</t>
+        </is>
+      </c>
+      <c r="D99" s="13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNVlZVeTNGcXVOSXV1eklvTnFxYk1hb1A2VTQtNHkwdUpvdFF0YnlYU2RSWkZNV2dGQkEyZjRVQzVJZ2Uwc3gtZ0F1TGlSQlVna01HRnZOTTJnVUFxaWtOam1vZ245Z05jdlRnQURqbnQxaGtEcnFYS20wWmtvSDV0MW15c18zUE5ZN2JJWUpLV0RsZE1LSm5fcUNNeVZNTmdMQ2c?oc=5</t>
+        </is>
+      </c>
+      <c r="E99" s="13" t="inlineStr">
+        <is>
+          <t>QSR &amp; Franchising</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>Gami Chicken credits chip design for cult following across Australia</t>
+        </is>
+      </c>
+      <c r="C100" s="13" t="inlineStr">
+        <is>
+          <t>QSR Media</t>
+        </is>
+      </c>
+      <c r="D100" s="13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPTXg4T0dvQ1l4NFVxV25iUXQzY0F3MnFjYmE4X0NOcFdNZHgweUg4NmVZZjNJbTFMajNhNHBmVDE2MGNBZzhOTUJsaG5KejFZbk1Db0JyNTZJbUI2WnRZeVhXRFRMNXVBWVFMdGJ3WkN5dV85dEduQi1OVDhOSE9UOGVERXh3T2hCVmlDNVg5LTdLY2VHNEZJSzlrN3VuemhzX1B5blpYRGtwS0hrak5r?oc=5</t>
+        </is>
+      </c>
+      <c r="E100" s="13" t="inlineStr">
+        <is>
+          <t>QSR &amp; Franchising</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>The great fake meat meltdown is taking plant-based burgers with it</t>
+        </is>
+      </c>
+      <c r="C101" s="13" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D101" s="13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPRTVDNW5oaWJ5bHdKM21iYllEVnpJbHhSbWFzYy1RcEZCdnNGUlJOWVJCaDZacFVoRjlSUGpfa3N6ckQtMFYzZTNITW5tMy05Sk0tZmtlSWlESHdOMWIyUWpUbE5RQVlsTHp0VXg0cHJYM0lJVmw1ckRURkFPVHFabTRIUzlFX1FlbFNuYmQ5MVJwWHVOaVhVWTdPajZxdG1WOTliTE1qZ3k1dnFRbk9BNTZCcXRRSGlIXzJv?oc=5</t>
+        </is>
+      </c>
+      <c r="E101" s="13" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="F101" s="3" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>Solar for Cuba: How Xi is turning Trump’s war into a China win</t>
+        </is>
+      </c>
+      <c r="C102" s="13" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D102" s="13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQOFlUUnNZUWo0MTJRaDFIZHp5dUJudERrOWxCZmY1WjZmeXRTVzJkbENEbUFhSkZFUWV6WjNGNUJIejVYRXFPcmRNZjFZeTkzTmtaeFNlb2V1OFFnMGtkV2JfTVRUN2FSV2xxcUpDUDJQeUpqWE9DRHRmT2kyc1dIZE9jeUM2eV9KQjd2RkJuTkxYeEdISDZDejhRbVo?oc=5</t>
+        </is>
+      </c>
+      <c r="E102" s="13" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="F102" s="3" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>Beer Sectoral Group appoints Nigerian Breweries CEO Thibaut Boidin as Chairman</t>
+        </is>
+      </c>
+      <c r="C103" s="13" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D103" s="13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOamdsNTN1dkRUY19Yak0wUGxsdm9NZGhySUM0Vzc4blNCeldzdFBiRkxuSW1xbTlZQUJIWkNxdzI3Zi1zc3F3SmJvai1UVGlZdUhGTEJ0eF9mNHRwSGREbDktT2txWXA4OVBESTdPLXdxWmV2V3FPTEZaYjRWLTlMM1VaY1dCbGZudTczZlFEYzN1aE9HeWdObE1yZFduLUtNVXBheDNsUWlIcUxibml4YQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E103" s="13" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="F103" s="3" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>Hip pocket pain comes for shoppers – and for supermarket giants</t>
+        </is>
+      </c>
+      <c r="C104" s="13" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D104" s="13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOeTdfN2dwYlBWSTdGbFo0SWRJcTNYelFFM2FBRnlORWRNcGd0WUVCbVdHVWZ6TFdZQzFpM2h6TkU2OEtqeE5OYlRrNmhsRU43a0E0UXhtZEZyTWZidzhMUEVxSVdiMlpTYXQ4ZVRaNl9BSi1Mb3JRaXhvM2hlMmNDcnk1aFBvVXFQSmlPbkN4Z3o2R2RzV0drQWpKaVZpbXR4dHppa08wRFd0dlNwcDc1alRDSXg?oc=5</t>
+        </is>
+      </c>
+      <c r="E104" s="13" t="inlineStr">
+        <is>
+          <t>Retail &amp; Consumer</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>RBA calls for co-ordinated effort to unlock digital asset markets</t>
+        </is>
+      </c>
+      <c r="C105" s="13" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D105" s="13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOT3dEcEtwVUptWTZydTRYWFdCU1RhTjI1RkFWeU5HckRVZjBxc2lqRkNOT0stc1h2Q0E1YTkxTjk3NTB3TGxKZGIweGFQRGh2S05QWHRoVGNZRFR2SlI2bkEzWlRoY2t3WU16dDlhVEI4RTFWYzhKS25YbGYxSVRjdFpVQ2M0dVc5MFJuUExNMTJIMVJTYmZGbkNLR1BPeVFYSF95NkNnWEEzamg3NmRuRkx0U2NjbXlxY015UWljTzRWbXpKclAwUg?oc=5</t>
+        </is>
+      </c>
+      <c r="E105" s="13" t="inlineStr">
+        <is>
+          <t>Australian Economy &amp; Markets</t>
+        </is>
+      </c>
+      <c r="F105" s="3" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>Banks rebuff work from home calls as Wesfarmers pauses business travel</t>
+        </is>
+      </c>
+      <c r="C106" s="13" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D106" s="13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOTjFLNnZUNXZHeE85a3kyaG1IX29sWjFvZ2NzS041UnYxNkkwUF9YU3ZFYXhtQmlxY3Rmd0lUSTJrdTl1Y0ZobWp0M1lrZnZhZE9OSzV3Ql9Hb2UtUEpqWC1McjM0S2pESDJQVWJKQkw4enF5THJfeXFWRDZiMk5KMmVrazVUMzBNTk1tOXRVX1ZzVU1IUHBVSlhENEdEWFJpQnFXUGkyNVJGUnhzdXgyNW1WZXRkRmRaaVloZnpaMFdqVmk3elpFSkZ6ZmotZw?oc=5</t>
+        </is>
+      </c>
+      <c r="E106" s="13" t="inlineStr">
+        <is>
+          <t>Retail &amp; Consumer</t>
+        </is>
+      </c>
+      <c r="F106" s="3" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>This mine was fast-tracked to boost Australian solar. It’s exporting to China instead</t>
+        </is>
+      </c>
+      <c r="C107" s="13" t="inlineStr">
+        <is>
+          <t>The Australian</t>
+        </is>
+      </c>
+      <c r="D107" s="13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAJBVV95cUxPN1ZSdEMzSXBhMno2YzNkSFFtdlBOTTRGV3UtbnZtRktEd3Q0MHdmZHp0SDN5S0FZYmVKUllicHRMRkxTdmxtbkMtT2ZVN3hsUXdBVzAxdzhWcGFWRkxVdFY3NURqTVV2QVJQT0ZUT193R3JLLU9aZUw4YzlucjVUN0xyTzdoZlNjYXdyR2VWeDZrbW53cTJoRGZDd2kxbkxzMHBQWkRJMTFPMkNlX19wYjI2LVBZbnVJOVNsRjF3Tm0xUUFpY0ctczFZdWJFcHQyLUhwdDNiSGVtdHQzVVRtbExpcHJZak1SNkhWd2s4a0RtYWFNN2J2Q3FobTF1N0hWLXA4YUtaMXBScjZsUWt3alVVTVpJdVl0WDF5RTJLM1BKUl85dnhUUktkb2VwMzFkUWZ1ctIBugJBVV95cUxOOENIa2JzQzdxekNYTnJNVmRzdm9KTFpndnBybEJfNjBUR3VNMk92ZnhGY0JwVGZLeFRpdHJLMTQ0NjRNOFg5b3FESzhPLWlub2hSeFdidW0yS1h6ZXlGMjh3X3FhaWo1dHdneUZxS2NsaUJ6dWtfT1R6VndwSk52bVVNN2I5VlNYazBIelcwUkVBZHFlM0hiQVJ1a2NGWFpmR0c5R3Bna2RZMmJuSXB5WkQ1Zl94VDFtcjVEd2x6amIwSWdXUWtQVVo1Q0hpWVBLRVFycDAyU1NJV3N4YktlUlBtMTlkY2VNZjc1QVZhbnRrQ01OQnZqNzI5dTNNZ1VlNVVJcURycXlDRFZDYVo1aC15RXpwUFlvZWxlMHFybWJiM1YxT05lRElXYlZsbkJWUnI4VV9Da1lIUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E107" s="13" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F107" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>

</xml_diff>

<commit_message>
Update news log — 2026-03-28
</commit_message>
<xml_diff>
--- a/news_log.xlsx
+++ b/news_log.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -87,6 +87,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -486,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:F110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -530,7 +533,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -540,17 +543,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C2" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D2" s="13" t="inlineStr">
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E2" s="13" t="inlineStr">
+      <c r="E2" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -558,7 +561,7 @@
       <c r="F2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -568,17 +571,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="E3" s="14" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -586,7 +589,7 @@
       <c r="F3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -596,17 +599,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="D4" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="E4" s="14" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -614,7 +617,7 @@
       <c r="F4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -624,17 +627,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -642,7 +645,7 @@
       <c r="F5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -652,17 +655,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -670,7 +673,7 @@
       <c r="F6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -680,17 +683,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -698,7 +701,7 @@
       <c r="F7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -708,17 +711,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -726,7 +729,7 @@
       <c r="F8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -736,17 +739,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -754,7 +757,7 @@
       <c r="F9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -764,17 +767,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="14" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -782,7 +785,7 @@
       <c r="F10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -792,17 +795,17 @@
           <t>Zarraffa’s Coffee celebrates 30 years, eyes nationwide growth</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOcXNzUkRLemZEOWtOZjhvRUtzcUZrSTdzV0s0LUJTd2NGRk1Gb1NSLUR5Rlh3NUdWQUJkVWctb0toUFBRajlMcWV3VnNyTUtydy1PSUoyb1NCOGVtMUZqRVN0MzFkVkNlOUZNVXlHN2kzREhSdWJQUnJqa0pnUzExTVZSc1NCVFZSNlBSUWNfWnZ3MC01aUx0UWF5SkNOaHI3ZkE?oc=5</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -810,7 +813,7 @@
       <c r="F11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -820,17 +823,17 @@
           <t>Zarraffa’s Coffee eyes 200 outlets ahead of 2032 Olympics</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPMUFjRTlGVFBqYzlPWXdzQ0dKVVlhWGxncUQxTDd1R0VHcThlV3ExVmo4SlBGSHVuUGZrMGNqSVo1YVpDWHViMm5KZWIxcHNMMHo0b1FQcmxUNElDR2lEeWRuLWZIN2lyQUV0VndEUWNkNU42Z3AzNXRlbm50NzhtTXZ0Q245dF9hNzBxOENuMXZsVlU4Z0JGVElR?oc=5</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E12" s="14" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -838,7 +841,7 @@
       <c r="F12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -848,17 +851,17 @@
           <t>Aware Super appoints new head of private equity</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNVHJXNWEtdEZZUW1fZzdYMTB4RklBTUh6dUNKQ3BrTlpYUnBwRURIVGZjWTV0OUxScnhGMVNSczhLUjVqOEwzbkR2WWlEbmF4ZkNUdHNQY0J1djI0REctbHd2SVhUNlNCa2M5bFhOQ0JPU0RHOVVTQkEzRDdGMjRZbVFDOUdlTXNNczlmZWF6bXlfbEFGRE0xbkZQaw?oc=5</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -866,7 +869,7 @@
       <c r="F13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -876,17 +879,17 @@
           <t>Commission wrinkle over UP Education sale</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxNSV9GMjhqM2ZSanI2X0w2OVlQVFRQTUoxYzAxaXVZMmU1REVTcHlUeEltdXJtaXZrcUJWdDZxNGpYTTZYSFE2TkZHeG9OaVRZakoxV0s1U01TVjJpWlhaSENfNVhucG5NVzFMbTVBY25zWGRSODBtRGtkS1owVTlJWnNfcTJ5alFnbVl1SU9aUDF1QWxJLTBSQ3kxUUFlZnpJMlVEQndFSGRGbDF6WVBUVHlCcDM5Qnh3R2xBMG9xN2FLckNzbUFOWDI1aVF1YV90d0twd0ZmMnUySDBMdG1R0gHkAUFVX3lxTE5EWVp6VzZWb01TRmlHSS0wMExldkJwSHJjdlZXdElsRlpBTEtVMkd6VzNQa1RpVDNsOFQzaGZ2VHpzUnBDYk82RmZGQWJuTmVQMXhxLXVmdVFxTVZOZTBsOHZ0V3cyVVVkNWUwVUxSc0xNSU92ZktpdFRfYnQ4WHBTX3A5bFhXZ1YwZXNrc1BSZEU4LVYybnNBd0dCdk92OFUwclJCMzdoU0ctX1pEdTAwY0JiTWQ4S01QRE00TW5EUEJwR2YtczZ0T005bTJnN1RDY2p6NFF1SndfLUo4QzJUWk1tRg?oc=5</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="E14" s="14" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -894,7 +897,7 @@
       <c r="F14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -904,17 +907,17 @@
           <t>Gloria Jean’s owner has an angry shareholder on its case</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPTnZwUVBCdTFJZWkwc0YtVmJqMkNPcUR5RktjMlVURmhROFZkYUpXM01iRUh3SnJEUElxRGlSNk9DQjZSdTdNdmZwWWpONjlmR1hoMl92cUNmd3M4cnJhVkNqc095MmN6WXBYUmdEblB0eERtVDdlUU4yNGFjXzVnT19rOERIRzVPNzY3VDNNRS1tVGVTX3pKMVRpTXZVR1ROLURBLWtJbVZhY0lSU09DNkE2NzFLbEFU?oc=5</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -922,7 +925,7 @@
       <c r="F15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -932,17 +935,17 @@
           <t>Oporto-owner Craveable Brands hires new CEO from Domino’s</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNNmxfQVc2Umc4QWwzSTdsZTFvejRzTzZxXy1ScGlhXzh6bm5JS3IyX0xTNDVBNjh0cXpPbGhxNU5xUHhQN3EtRF9aV3FEc2JoSG5QTU1WeU1TLUJfZzVUT2N6dXloQXhZaHB5djB3dDFKN1llVmI3UVpKNjJTNlcyV0ZDcG9GdVdSdW41ZkN1b1N3SFFIUzcwRkQ3UHY2TmxERmZwTlA0RzU?oc=5</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr">
+      <c r="E16" s="14" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -950,7 +953,7 @@
       <c r="F16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -960,17 +963,17 @@
           <t>Brookfield, BGH Capital rub shoulders in ScotPac’s data room</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPMVlxbzlQNnFXWnJFNU11Y1BhTTVqbjN4RG1nbkZuN0pkdDFFaUhJN0RaVnUtWDlZSGJWR1ozQXk5UUx6RVdOcjBPU2t5UzN4T0JvUFJISnNvVWxQemd3blNHZjRQVVVZQk1nZER0Y0JfY3VvQ0t1a09sM1RTS2c1YTJyUmdzYWh1WGRUNjl2dkdzYTJJeHVhMTdqR3Y5WVlHVEtSZHp1cmVYYmM?oc=5</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="E17" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -978,7 +981,7 @@
       <c r="F17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -988,17 +991,17 @@
           <t>Payments player Pay.com.au hits the road(show) for $850m IPO</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOMFZleXZrbU53TzBlakI2ZmJKTjlrN3BoQlRaWjQ5cXFzTllKWmFoRm1UT2xDUHBtNC1QNTNiX1BwSzllMkRZdHIzRlAteDREaUczN1JTNTByTW1jNnR3d2NnR0RxUDBxeHYyWU1CSUs5MEZad2JqSGF6ZUxHZUNtZmFQaTJZZVJVZ1B4MkZ6V09QMWIxaUNHQmVzTDhvWVA1Ty1UbHgtQnRrQQ?oc=5</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="E18" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1006,7 +1009,7 @@
       <c r="F18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1016,17 +1019,17 @@
           <t>Another year, another IPO cold shower for investors</t>
         </is>
       </c>
-      <c r="C19" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="inlineStr">
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNeEhzYzQzdjR5MDJCWkd6Q2VLdEZzbzRoWnNOcXFlQjNfMlV4Q0NQRjExMlNhT2NPcnRBbW1sZUkteXo4N0dGaHNNeGZJOEZ2aXFvdmZiN2V2QzdOMzFteFRnY1RVRm1rQXltWmY5VFZOdFVNNVpudVp1dTlrcFM5b1k5SmlWQllDMVFXSjA4ZVpSZHgtV2JpWDJ4SkFRbVE?oc=5</t>
         </is>
       </c>
-      <c r="E19" s="13" t="inlineStr">
+      <c r="E19" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1034,7 +1037,7 @@
       <c r="F19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1044,17 +1047,17 @@
           <t>Priceline Pharmacy franchisee sale narrows to final four bidders</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNR294am9sYWNiQ3FVT1B6YlV5ejMyeHAyT0FibTFVbU5pcjZyaVRyazEzbFkxd0lrcnpZNGpTYUx4Ykl1Xy1sZF93M2Nid19ydUFwbUJ3ZHozaURaNkRoOE9OMnRBRGZfQVdCVWZCaVhhNnZSRjlwYUdDVnp2WU9HUkJxbE1QMV8zdWxYRTNBQWktR0xSOFU4dmtXZWk0am9SSU92NWp6QUZmTVU5TzJEOEJNak5fQUtN?oc=5</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
+      <c r="E20" s="14" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1062,7 +1065,7 @@
       <c r="F20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1072,17 +1075,17 @@
           <t>Private equity gets better image of Qscan</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="D21" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxPRjVmT0hDRjZLblB1VHdPRmRGeXhKdDJHdWxDTzV4RDZ0VzdHaUFfOVlnZjRQMWhKcWMxby1oRDR6N2lQZkI1UDE1REppS3c4LTVmU3p5b2wtblRCWnhNajFnZGNHaGRJUHFMUGRtTHAyQmIxOHhNNTgwRWVSeWp6ZWRxbUY0WVhiUnhMRUpDLXNwS1RuelJldTk0Z1R0WHg0XzNXNTA5Rk5TRFZhU1RNVnN2TlZuaFE4OWtIYXQ5a2VGSW1UWmt5Rlc4Q2lIXzF3YlkwNVhfUzJDV0dQdVAxa2RKc08wRGR6TlB2Vi14QV9BdlhyaTZsM2pEVGZycTjSAYQCQVVfeXFMTWpnb0lWQmZ6MTFnRGhWNTNqczk1TWhTcUFEMVpDNnJ4ZWVxVlRUODhJXy03NHdGZVJlMmhyUHM0Nlh4NlZtTzRhQ0xxRDFLVHNzUVNfbWxhS3BLUEQteEMzZHRrc0F1eFRzYmxVNDZlSURyZDB5bF9wQTNRRU5yZEs1Z3pFRTdwcFBaMkNlN0JvT1NEYkFWVUJNcHJqcEM5RVJYa0JFUVl6cThyQXloaERzQjhkTUVPakJqb0hzNVlwSWxNS0dmZkNFSG9Gb3dNUnVvUnV0d3MxSmpzdFZKTHJ2RTQwRUoyMEVLLWMwT1NnOHdXVl9lRXNDWEFndzJFSDlZU0o?oc=5</t>
         </is>
       </c>
-      <c r="E21" s="13" t="inlineStr">
+      <c r="E21" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1090,7 +1093,7 @@
       <c r="F21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1100,17 +1103,17 @@
           <t>Oporto CEO’s first year reshapes brand and network strategy</t>
         </is>
       </c>
-      <c r="C22" s="13" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="D22" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPY25mNTJfT3FiVlBPZE5CcVNkR1UzR2xWaUtJSmxhU3EwcEMzQi1ISDFSajlCQWk1UUJpZVJ1Q19ZV3Jjd0Noc0l3OExpMXhSQUVVdHhCLTBlOXNoZzA3UXZBdkR1VHBvMmVsZkNhUFJndm1DdGpnX2w0ZVViU2phZ1RmYXY1SlhwUnhKSUxBQVZZUXpqNHQxQmo0Rk1iV0g0OW9qUS16eWRSNW5FaW1yQQ?oc=5</t>
         </is>
       </c>
-      <c r="E22" s="13" t="inlineStr">
+      <c r="E22" s="14" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1118,7 +1121,7 @@
       <c r="F22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1128,17 +1131,17 @@
           <t>The Melbourne restaurant our reviewer grew to love</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOc3YxQTljcHJXVWtRX2ZGM2lpM2pILWNwSFg0MFJrNmNWX0ZxRG9nV0J5N19qRWh4U0hPXzNmVVZwWk9wT2kzaFNrTlV3NEQ1Q3JpaXVIYlBHb216Q3VYVWdSRXMwdDl0SmYzdnRlSDFUYVRmRGJyZVlRZDJKTHpJOUctYlF1RDZSYjloY0hfZy13QmFTLU9UNjkwTHc1bjlGcGxoZ0ZLVU1GWTctZkdLZU9zSGhEZEpKbXJnaWJfZjd2OWs3?oc=5</t>
         </is>
       </c>
-      <c r="E23" s="13" t="inlineStr">
+      <c r="E23" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1146,7 +1149,7 @@
       <c r="F23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1156,17 +1159,17 @@
           <t>Crescent Capital strikes Benson Radiology deal for close to $400m</t>
         </is>
       </c>
-      <c r="C24" s="13" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOLTNrWG1ZZlFoU3pDZ3E2SEgwMlhzQkdtQUYzaHZTZmYwU3ZhMnE0dlkza005VkZmZ09NMExlWDVncnBmYVVISXJ6X1ZjNHhpM2RnSlprY1dnbndJNUczcDVtNXNRY3pVNW12bm5rUVdqVmR4R0JlVHFuN0RwTlFkR2xrbFFpSl9jcm5oSjk3aFM1clBSVDhnbkhoWUREeUhsbVpvQW90d05xOTdfOV9nbW5POFdmelJkVlpsUlRuYl9odmRNVUV2S0pCMFBMTS0tcVhGVGFYU0h2d9IB3wFBVV95cUxPWEs4R2pxdThPbHJHb0dBT183SkRHTTlXNzdWazcxdkd1eGx2VlAyM2VVbEtEbWxTZ1R0TlBFRmRMZTFoalgxSmVVRUJFR0c0RFYzZVJFODg3dWxicU9pOHppeFhjaVp0WWlyTnUzV1dyZXdkMHBDVHI4LUVQdjc0cWpheU55NTlvdWdCZmVoODB0Mm5fbGNCTmQwLUhMZ0psQVpzb3BEUnJpSkRnOUM0c0VCdUp5N3g5MkhaM01vTHJ3NWd0ay02UXZUUG9nVkxicVc1Z0xjWGhjUDRDVjlN?oc=5</t>
         </is>
       </c>
-      <c r="E24" s="13" t="inlineStr">
+      <c r="E24" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1174,7 +1177,7 @@
       <c r="F24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1184,17 +1187,17 @@
           <t>Dual-listed giant Capstone Copper flirts with $600m-plus carve-out</t>
         </is>
       </c>
-      <c r="C25" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D25" s="13" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNcVh4blRkQnoyaG1TajhVV0lrOEJRaHdTZWtzUnJHaEdaSXNRWThGTHlVdGl4dGJ1cTMwZ2pLcVNzUXRYNlZzVzhvaXdkNGtVUG0wN0FrMHB0R1I2Ry1jcEgtSWUtajI0cTFMRTlfdzBuMWtrZmJOLVUtMkl5dW85dFp6dEhEOHhTNzdfOFNFSGtlT0MwQnRlY0VhcUZBNE9RYzhQcDdOQUFnYkgzd0V0N253SQ?oc=5</t>
         </is>
       </c>
-      <c r="E25" s="13" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1202,7 +1205,7 @@
       <c r="F25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="inlineStr">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1212,17 +1215,17 @@
           <t>Guzman y Gomez unveils a new menu under $4</t>
         </is>
       </c>
-      <c r="C26" s="13" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D26" s="13" t="inlineStr">
+      <c r="D26" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPMjRjRTV2a3BJc3AzdDNOQktoYjBvLVZSODVsc3lKQ3pET0lxUlpkc05NcVlKRlZITjVJbjkwLS1DUFJNMGJ1amJKTlp3S3VqMWJaU3YtUENEN01rUEJiV1FNZTRXYjcyV08zZzlxNDVOSlVOTlJDOGV3QzBQcUpKa2Zab1ItNlI3ajZVVTF3?oc=5</t>
         </is>
       </c>
-      <c r="E26" s="13" t="inlineStr">
+      <c r="E26" s="14" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1230,7 +1233,7 @@
       <c r="F26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1240,17 +1243,17 @@
           <t>Can Sydney’s burrito king conquer the $676b US fast food market?</t>
         </is>
       </c>
-      <c r="C27" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNM0ZFcUpLN1dUZWUyaE1LMnNZVGlEbkNNQUQ4Wmd6QVFlTy0wZDVHdnlja1gzMEZTbVpKU1Ftb3VKZ2pzajcyWU16NUtUTmR0TlZMOVhMRUNqZXZiX2d2NWY0YlJDOFhhYUE0SkhMRUprNndXak8tWGdERU90cmMxTkFjcFFVSTd5VlZ3NFVKOXN3M255MFhzZThmbi1VUGMyQ3E4d2pYcFlJckY3QlVBdVJJeF9qUQ?oc=5</t>
         </is>
       </c>
-      <c r="E27" s="13" t="inlineStr">
+      <c r="E27" s="14" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1258,7 +1261,7 @@
       <c r="F27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1268,17 +1271,17 @@
           <t>Drone maker Innovaero prepares for ASX float, taps Euroz Hartleys</t>
         </is>
       </c>
-      <c r="C28" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNU3JrejNRZ1VBZVNVV29NMkFPVmRsWE4yMVZPcjk2aUNUTHFJUGFyQ1VnZEZiZlIzQW9VVzRNNDNRR01jcHo3X0tqZjB4bzhMTTI0Y3BwYUh6OGRUUGt2REIxV09oRnJoVWlVelZWaUlWUmlPQ3dJdi1TejcyaXB1Z0x1MEJRSlB3SGMwVGdXaXJJNm9TVllPOG5JZC1feEV3TVhTeExGeHR2RHFIWlVCOXh3?oc=5</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr">
+      <c r="E28" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1286,7 +1289,7 @@
       <c r="F28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1296,17 +1299,17 @@
           <t>Bain flaunts Estia 2.0 as IPO roadshow gets under way</t>
         </is>
       </c>
-      <c r="C29" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNTEN1cGsxNDN2c1NqUzB6UmJ4TFl0NGZjZVN3U3oxMlVFWTF4WUZLQS13dUxMV0N2ek1XN2VURTNVWms1NjdXSm0waEdaTXQwdTdWY1MxZ1V3ZnpEcVJtczdOWGNNZ0RQNzRZLU1MTTgtRW5DZkctbXBGMmVXVXdPZW5pNThiRHEzWnB2eFZzTFZTb1ZkeW9LendkNDd0cXRid05ZSGZYbW9NZXdOLVZWODdZU3hVcTA?oc=5</t>
         </is>
       </c>
-      <c r="E29" s="13" t="inlineStr">
+      <c r="E29" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1314,7 +1317,7 @@
       <c r="F29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="inlineStr">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1324,17 +1327,17 @@
           <t>Carl’s Jr. Australia unveils nationwide freebies for Happiness Day</t>
         </is>
       </c>
-      <c r="C30" s="13" t="inlineStr">
+      <c r="C30" s="14" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNVWgwdjU1NDFWalBfMTFYX1dQOWNDbG1FVUdlcS1LTVlHZVRRTVBWTjhSMnpkTXRXNlFJdllGQUp5Mm5ObWpIazd1d0RJa3QtdFBZN1hOenBmVzBEU05wM0gtNUxPeWpsYkxyVnhWWFFOU2Y3R0tXcmNkeWhpWDh2eDZBdjNCMHhuc1lHYTZHblBPVkpfRXpKd051UWlNc1hm?oc=5</t>
         </is>
       </c>
-      <c r="E30" s="13" t="inlineStr">
+      <c r="E30" s="14" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1342,7 +1345,7 @@
       <c r="F30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="inlineStr">
+      <c r="A31" s="14" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1352,17 +1355,17 @@
           <t>BHP and Woodside appoint new CEOs in major mining shake-up</t>
         </is>
       </c>
-      <c r="C31" s="13" t="inlineStr">
+      <c r="C31" s="14" t="inlineStr">
         <is>
           <t>ABC News</t>
         </is>
       </c>
-      <c r="D31" s="13" t="inlineStr">
+      <c r="D31" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQbTg5VFJLbWJfcy1uV3ZReTJkTndzX01qZ2MxNWkzaWZRckNLZUR1Y1VsMVRNc2FySC13U0NzalFEb3k1R3BaUEhfcTV0N1M4Q1dpSlo0YXI0UFhrMGRab2RiYV9DQVNVX01ycFc5ZFZrZWZqc1VRZXoxLVEzSDJLclJLSWg5bzN3R1I0bG9lWjVDaHE4?oc=5</t>
         </is>
       </c>
-      <c r="E31" s="13" t="inlineStr">
+      <c r="E31" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1370,7 +1373,7 @@
       <c r="F31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="inlineStr">
+      <c r="A32" s="14" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1380,17 +1383,17 @@
           <t>Next Capital sells Enviropacific unit to French waste management giant</t>
         </is>
       </c>
-      <c r="C32" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D32" s="13" t="inlineStr">
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPR3lFbERLR2FtdmJUU3BDU2thZk00YmFHRFhXR2VBVXhQSURTeE5ONVJKczBwbzlFMnR5cmhxMnM0bzlJbWo4SXl1dHpqYWxxMUJBRjZHVUtab1RYZjZMTnpGc3FzMWQ2NjNEdGU3NTZwa0diM1lJS1haYllwTldLZlpZbXp0YzlxcDh0ekcwTy03dDdPcnk4b29HZVdqbHhZY2JPR2drM2puSVpjUzZkVjNpZUE4dVMwYlE?oc=5</t>
         </is>
       </c>
-      <c r="E32" s="13" t="inlineStr">
+      <c r="E32" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1398,7 +1401,7 @@
       <c r="F32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="A33" s="14" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1408,17 +1411,17 @@
           <t>Future Fund private equity and real assets chiefs head for the door</t>
         </is>
       </c>
-      <c r="C33" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPUHNHRFhFMVdwVld6RFRZUFd3QWNOd1kzeS1QdnJxMERFSnE5LTdZcDhDYlVGcWZMeWxlR0FSRWF6YkZoQVZrZU9TQ1E4YTEydUJnOFE3enV5Rmk5UnF5VEdYZ1FMUWpKVjdjMlZZUGFsU0tKcV9Vbl8zcHp5aVF5Z2JMOUZocHJqRXNRaEp4Nm5CbDM1WkdIMHdQS2xqQnE2Tnh3?oc=5</t>
         </is>
       </c>
-      <c r="E33" s="13" t="inlineStr">
+      <c r="E33" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1426,7 +1429,7 @@
       <c r="F33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="A34" s="14" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1436,17 +1439,17 @@
           <t>‘I actually started to die’: the new billionaire’s epiphany</t>
         </is>
       </c>
-      <c r="C34" s="13" t="inlineStr">
+      <c r="C34" s="14" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="D34" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxPblkxbHVrdnVKY1pqQzNyWGNMZm9UYmY3dzlPaGQ4Yi1tc0U1akhrVWdIaXBpM05aZXRwTXE1eDBITlZpbDkwRXNrWjJ2YXBzX0VCY2JSLWhrVmpjSTE5eE5rLWgtc2pRZEdXbmhhWU1KeFExZDBGS2pjSkIwV0FGbndBZVAyQkg4WFRsengzSGYyZkFfQnJsQ18tUHJGNDd2T0pzZElPSVJTQkl2Rm5QTExJNHhmU2dHOHJGdTdzU08yNHRtd1R3Q0cyOF8taDktQTZvVXVBVjN1d0NHMmtFOHBWZXBFcUFWa1IyWGNDTDZUT3lQSXJHOVhxTFQ3b3RH0gGGAkFVX3lxTFBZQ3BFQWl5dEwwLW5yVWJuMU8zcXBPdE9pamRVSWVkbWNyVzgydGVOaDBROUN6RlBDbjdld05DVmZyb0R1eEN0UERubzZRU2NiMTQtVV9XNS1wYmlvZ1paM3RaOUlrTzJka0tXVVJEamFESGlSdXg2bDk1aUdhUVhBcXpnN01fX0Y0cTNvcm5DdEFFLVVERDFKTWxKZFR0UzAyblJqVHBua2JoYUdzeUNMb053ZVczWUFQU1AtVHV1d3lSSDFfZFh2cEkxSGw2MEdicEVsb2pLQ1RuQmdaRl9xNUROS3pKR2s2T2wxTTZ5bEwtTUNQNU04djFHTHlPbXVLSW9YSUE?oc=5</t>
         </is>
       </c>
-      <c r="E34" s="13" t="inlineStr">
+      <c r="E34" s="14" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1454,7 +1457,7 @@
       <c r="F34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="inlineStr">
+      <c r="A35" s="14" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1464,17 +1467,17 @@
           <t>Ironbark shuns private equity as it hunts for cash injection</t>
         </is>
       </c>
-      <c r="C35" s="13" t="inlineStr">
+      <c r="C35" s="14" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="D35" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxQZWFaeVhldi00VkV5ZmEtS2tjcWdFWG55OGpCX3IyN25Rb3ZFV0ZKVm1aSE1WbThoYVY4ZEdfODVGX0RaUDV2Ul9HS1JQMDFCT05Fc2FaU0RINTMwbDRveWFsOFJSM2ZqTU9tVGxJSEl2ZmhhUHFHT3dqYkk5TUtvMUQySnZzTWw1MzFNWl9aVzhkSEZ4Q3YyWjRMUmpIdmJkdUVKWE54Nkt6bTd2dGFSUFoyNkgxTHh2TGVGak9ja0dFZ0xQM2g0S1lmQkZiWWtUcTVNdHhBdC1KeVRQcDA2dnpmeHRkWEnSAewBQVVfeXFMTWtYRDRSaHNULW1HanowRnpMdFF2VVMtZW1SV2ViZXlGaW02WlIwUzRZMGg5WDNrOUR4eDlGOEt5eGlqV0pfVDFhb0JEcS1faEJodWxyRnB3MkozOVJyT3NvM1I5MzdDcXNnUFNSdkRDamUzZTRQYlk0c1VIQUNMZ2ZzOWVCb2V2MC1aSTZLWkFkbW9GYk05b3RmN1htWENTeDh3SU1WYWJMcWx2eGUzZmwwVXF6czlnRGdXbE1vRElyVG0yM0ZzXzZ5TFh1YlRGNU9MQ1p3NnVZSFB0M0xBcGlueVZILXlVaXdqUkU?oc=5</t>
         </is>
       </c>
-      <c r="E35" s="13" t="inlineStr">
+      <c r="E35" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1482,7 +1485,7 @@
       <c r="F35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="13" t="inlineStr">
+      <c r="A36" s="14" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1492,17 +1495,17 @@
           <t>Minister leaps to fix food chain</t>
         </is>
       </c>
-      <c r="C36" s="13" t="inlineStr">
+      <c r="C36" s="14" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="D36" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxOd2NqakVWRnQ4anFZNkl4Zy03MkloX08tUkktRTZqeEtQWFZJeVhkMUJIb0FxUjc2UjhCQ3MxbmNxczNxblJIZ09IeTBGNFM4Wkh4ZE1qNkhJMjIwU2RtX1JxcEV1Y0NjWXF6eHpVdTN4ZUlYMGIwcDJzMXZMTk94VzFlcjhpcVZVSTJFMjhsQjVGWEJQYTQ3aTFyNmNEZ1F1b3NGTWd5WnFJWmxXSTJ2NlRLcjJHNWkwaTZ2YVR6S0w5WVo1Vlg0VWdxcWZoa3VaTmcxY2NVcnR2bFRWNGNvZ1M2Tlg5NzlvVXZFZm9B0gHzAUFVX3lxTE1uNERoR3p2dXRIa0g0RXI2MWR6N0c5U3NGcjFDQVMtdEpyNDI2bk8yOS1qUnFOazdiODl0Ymo5R1pwRVJ0UFFVdzlhYjRDSUFCU0FRak4xcVVrTHphdTdxcHNIMnEyRVZud1FURmh5T0JLOHpRM3lFbDRuRnZMYmtaRnRFTXh3dkszTFhFUmZlRmoydnlEbW1fZTlmUzh4NXNyeTZTeUhOSktvclJVc0NTZTVYMkdJZEUyY2RmVC1kQ1hwVEloSEtVMEo5QnNTUXQyME5IN1BPd1NOS3oyR1JtMHBFVTZEbzhEQmdrWUk1ZnZVTQ?oc=5</t>
         </is>
       </c>
-      <c r="E36" s="13" t="inlineStr">
+      <c r="E36" s="14" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1510,7 +1513,7 @@
       <c r="F36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="A37" s="14" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1520,17 +1523,17 @@
           <t>‘Brace for swings on every tweet’: Investors bamboozled by peace talks</t>
         </is>
       </c>
-      <c r="C37" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D37" s="13" t="inlineStr">
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOczZHTWFmTW9FZ1ZwSnc5Z3ZacGpsVDQ3LWw1a1BFT0tjRkphek41MlhNOU84emYzZUVwNV9xM0hyc1FUR0NHck14Qnh6c2JvQks5ZE02ZTNLWDI0dy1STi1HbDFDWW9yMDhGQXVVVzdkMzFXcnNNMVZHVXFMUXUteGtsVGhPVmhLcVZPQzlhTWNoYVVRMHF0cFhybWxzek13Y3ZjcjlXWjZJM2VYbm0tTmk4NExLQzQzX1ZPMVlhcnJxQkZx?oc=5</t>
         </is>
       </c>
-      <c r="E37" s="13" t="inlineStr">
+      <c r="E37" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1538,7 +1541,7 @@
       <c r="F37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="A38" s="14" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1548,17 +1551,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C38" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D38" s="13" t="inlineStr">
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5</t>
         </is>
       </c>
-      <c r="E38" s="13" t="inlineStr">
+      <c r="E38" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1566,7 +1569,7 @@
       <c r="F38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="A39" s="14" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1576,17 +1579,17 @@
           <t>Wirth’s Myer rescue mission is caught in the eye of the storm</t>
         </is>
       </c>
-      <c r="C39" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D39" s="13" t="inlineStr">
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNTlQ4NDRnWE91VG1YNENpSTUxNnBjZkljOGdYaGV0aVB5dkVOaEJ6SjZ1bVA4NXE1S1hjV1NjcVhQTEVpWEVNV0UtbzhQTFZLOWxIenZiaF9QM3F6bmJYRy1lbXVMczZ3TnBHNy1aLUtVcnBDdkl4TE0zRGN4U0FwSjNPY1M5S3AtdUQ3UUNmR0x4MlU2YXRuUDJEUm01SmZWakx2UjFvY04zRHk4Smc?oc=5</t>
         </is>
       </c>
-      <c r="E39" s="13" t="inlineStr">
+      <c r="E39" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1594,7 +1597,7 @@
       <c r="F39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="13" t="inlineStr">
+      <c r="A40" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1604,17 +1607,17 @@
           <t>‘Darling, I’m not going anywhere’: The rise of at-home care</t>
         </is>
       </c>
-      <c r="C40" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D40" s="13" t="inlineStr">
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQS2k0M2otaldpNVFXdHRTMVNtZVhyUDV4VTNIcE5FSnFRaHNubGNQQzBVbllnNTktNGhrZ1lndzV5V1FpUS01SklRaTZmZHJkRzVsQmlsdEVmenZ4U2x6U01NeXdIMktBUW94TUE3R3FoLUxVcVhsVFI0SjVQVUFaZldnd3prMWMyaVRWX2J4aUdfQ25KWHpaLUlqSnhvQmM2TTRRQldGbm8tclFYRDA0TVdnU2g3QQ?oc=5</t>
         </is>
       </c>
-      <c r="E40" s="13" t="inlineStr">
+      <c r="E40" s="14" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1622,7 +1625,7 @@
       <c r="F40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="13" t="inlineStr">
+      <c r="A41" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1632,17 +1635,17 @@
           <t>Iran targets Israel and Gulf states as Trump looks to calm markets</t>
         </is>
       </c>
-      <c r="C41" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D41" s="13" t="inlineStr">
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPLXBITXU3WTRtc0NYdnhTZHFaUTBCSXdldTBuSHliTlY1dlJONW43Qkd6Nl9pNmY1eDhzaHZoX19xYjBxMXR5UEhkVUg2M2k1MmhuVEwyY0JxbnJyemxVYUZjbk5BbkN4ajhPbW9ZeDhlRDRYTW1hN3k2d084c2djMEJUZTV3NVdPbllKUmFlU2JsaDV3Zk9CVFF0VDFkV09JSloycWdOUlVrREptQTJfa25LUEx5djA2SjNMMFY0RjM?oc=5</t>
         </is>
       </c>
-      <c r="E41" s="13" t="inlineStr">
+      <c r="E41" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1650,7 +1653,7 @@
       <c r="F41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="13" t="inlineStr">
+      <c r="A42" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1660,17 +1663,17 @@
           <t>Meet Christian Louboutin, footwear’s most famous billionaire</t>
         </is>
       </c>
-      <c r="C42" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D42" s="13" t="inlineStr">
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPcXdGd0tMckYxbjZ5TVJmQ0Q4NFl2RkhHMHdlZDZsdGZ6cVQ0cUpaLWJTNlVoc2ZOQmtXNlFTRnJVMnVDTGc1NFNZN2g1VnotQlNQbzhlM1BJV3ZwQktOcGtac3RwSHRLZkR0b2l0eGIyVVlYdHJrc2hpT0pJbDR3LURPTnowZk54LThObndtMVkwV2VWQkluNVlWY0p4QVJGbE1hSGMzOW8zdkJZOWdocEZQWFBhTllNR1ZBSEg1TWRXUWd3X0t6TVcyY05PM0pF?oc=5</t>
         </is>
       </c>
-      <c r="E42" s="13" t="inlineStr">
+      <c r="E42" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1678,7 +1681,7 @@
       <c r="F42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="13" t="inlineStr">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1688,17 +1691,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C43" s="13" t="inlineStr">
+      <c r="C43" s="14" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D43" s="13" t="inlineStr">
+      <c r="D43" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQbHdYM2pSM2xkdmZ3OHhQc2tVUmhzclJWaVJ0aEwtUkNBR0ZUd3p1emF1M21jbTF1ejlKSkdDMnotcVNjZE1CYUlKako3WXR4MTJhdWNlSXZMbTBYanlmTWFzRGFIandXRUQ3UjN6SEV1bThvZjN2bDY0eFdpaTdMODN6TGFTdE5rd05TUll3MmNfTDhkQldoNDIwVlpoSl85aVRwcTd5Ymh3TDl4enZhZ2p4OExGY1ZaOFNEWFBB?oc=5</t>
         </is>
       </c>
-      <c r="E43" s="13" t="inlineStr">
+      <c r="E43" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1706,7 +1709,7 @@
       <c r="F43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="13" t="inlineStr">
+      <c r="A44" s="14" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1716,17 +1719,17 @@
           <t>Sembcorp Picks Banks for $2 Billion Alinta Loan in Aussie Push</t>
         </is>
       </c>
-      <c r="C44" s="13" t="inlineStr">
+      <c r="C44" s="14" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D44" s="13" t="inlineStr">
+      <c r="D44" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOdS1aaXZjT2VnSDl2TDdzZ3NfRElDWXdUXzZQYjFQMEZJOGlpaE5CNGdQMlZ2UFVHbUtfOXF1ZVBReExrdF85M0RWLWlBY2Y5dlRtWVdXLWp0Y1VrRmF4UGQzVUhxaHA4UHd1SUdFV21QcVFITXFHRlhzekdSUS1PdHlYRjdUbUQydU8wSktKVHRJQ0NaWE9sU1l6YXhtSWtBd3RwTERacnV4VzB6YlFhUE1QcXNDVXVESFcyeWY3cGhHUkRJcDhrYUtpTEY2UQ?oc=5</t>
         </is>
       </c>
-      <c r="E44" s="13" t="inlineStr">
+      <c r="E44" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1734,7 +1737,7 @@
       <c r="F44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="13" t="inlineStr">
+      <c r="A45" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1744,17 +1747,17 @@
           <t>Navis targets June for $1bn-plus med-tech auction</t>
         </is>
       </c>
-      <c r="C45" s="13" t="inlineStr">
+      <c r="C45" s="14" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D45" s="13" t="inlineStr">
+      <c r="D45" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxPNHRXaU5tNUVkd2MtcTg5M0EyQllrM0owMkZobGxLaUJxYUN2MUg0ZkdKdzU2YmxfanR3QU53cHZzNDI1WXgzRUcxOE9EZlluNmtNRUUzTGJPRnpfVVVOeFM3bFRNQmp6VHFBdi1mTnU4UDBvOEpMaHZPNXFtdUIyTlhuRExIVElSeVRUMGxjU0k5VnVxaWFfd3htWngydlhuR2E5aTQ5VW1LS01ac05rMGZoVFdOZzVyTzFhUDVsYkNrc0VQZmhubERSaTNwelk3WEhYUjF5d2ptMktYeEhzOHpWazFQZXphd0xfUFdhbkVGMVR2Z1dtVtIB_gFBVV95cUxObEwzeHd6RmZtNUp2dXVVV0plOVQ4WlNqQXNJU0thd1BEWE8yWkxxVTZjTkpsVGxxWGxpQzN0OERZbk91ai1fZkdtc0JoM1h5NERLTVdDbVJ4Y2k4djdQcWlVcDF6NjMyVDQzZWMzUFZxWjVRWllMZHVSOF9jQ2U1REFfNUlhM2EwYloxb1MwSTJjODdWdlZwX2h2N0xiQWNhallHUTNPZEtLaXhsY3dBZy0xM1VITXhLUERXS1JxR0R3OUpBTVBPZ2dPZTRUTVpvbFBNMjFUSTJuWS1XLWdhUS11UTRzVTVqaEhfMDhqWHlTMlJGekU2QzJVcFdodw?oc=5</t>
         </is>
       </c>
-      <c r="E45" s="13" t="inlineStr">
+      <c r="E45" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1762,7 +1765,7 @@
       <c r="F45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="13" t="inlineStr">
+      <c r="A46" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1772,17 +1775,17 @@
           <t>ExxonMobil eyes New Zealand market exit</t>
         </is>
       </c>
-      <c r="C46" s="13" t="inlineStr">
+      <c r="C46" s="14" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D46" s="13" t="inlineStr">
+      <c r="D46" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxPanlvR1V1eVVpdmYxNVNGMnd6UjJFd0J6Zk9IU1lhOW1GbmVTcjY4QkJCYkl3Y3NOU25VRTBUekwtS3plV0NVdlZtOTZZRHJWZ0FVdDl3S05aMlFWeEZiYzdwYmQtVnJxZEw0NktHaFZMNlZkUC16empqRGxxMEhhZGwxRzVEek5FelB3aE9UWFhGQW42b21MRnJHUXV2ZGJYUXJIMnVFWGZsSnEwazNGNUdVcjVoekp0NEZCN1J3cTlaZldFa1pMUkJTbVZYeFljVkRqQmlZV1M2aXh0ZjI5dEI1NDB0UElPUERsbUljMlA3OHBnYmtJTXFWZWkyUdIBgwJBVV95cUxNWFBRQ05GUDdwTWJ2ZVFJUS00ZUh0QkpZQVNNcU9JYXRTN21sMS1VZTlOSTh2LVFuZHh6UVk2djlrdWFsd3MwcDFCNmhwUlVLTlpjVF8wSmt1YnBWRE9tNVpKQlk2YXJWdmwzZWlLX0xpaWxSMUpsX3ZjYXhmRmE2YlAtSFJGRG5pQnVmMnViQXlsVFV3OU1hZFVrY3ZITHQxcTR5UkZ5U1pReHVJMGZGM2FCZWliSFZQZmpVLThSdExWMW14OElodmVVSC05SUh1d1hBenJoY3BUZGxoM0NTbTExdERmM3pjZGd4VzgyV3BNOG11TElBQ3NsRGhtSEc3YzJz?oc=5</t>
         </is>
       </c>
-      <c r="E46" s="13" t="inlineStr">
+      <c r="E46" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1790,7 +1793,7 @@
       <c r="F46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="13" t="inlineStr">
+      <c r="A47" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1800,17 +1803,17 @@
           <t>PAC Capital’s Clayton Larcombe charged with assaulting wife</t>
         </is>
       </c>
-      <c r="C47" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D47" s="13" t="inlineStr">
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D47" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOLXNDU2xjMWpyeEZwWGwtZkV0TjNSbGtWS3ZidUo3a0dvV1hrTnJiVXBXSkJNWlhXYXFHZkNTa3g4a1ZfMjRPM3BtWTZUNGg3S09kbGI2TTRGd0Jkc1A4WFAycjlpVC1URjFvNnBraWprRkhaT0VOWkh6N0xkUjNXNUw0dGx2N1JtTDVsREdtZDhraXVsSkxhR2ozamFUSGR5VHBBRm1Zcmx1c2RDaUIxQkVpeUpfWjFNeTRLWVRtYjluZ3ZncGZIMQ?oc=5</t>
         </is>
       </c>
-      <c r="E47" s="13" t="inlineStr">
+      <c r="E47" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1818,7 +1821,7 @@
       <c r="F47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="13" t="inlineStr">
+      <c r="A48" s="14" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1828,17 +1831,17 @@
           <t>China touts itself as ‘harbour of stability’ to global CEOs</t>
         </is>
       </c>
-      <c r="C48" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D48" s="13" t="inlineStr">
+      <c r="C48" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D48" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPUzBWeVk0elBOZ0l5QU44TUJvU0RvSmtPdmVyT2VuQTczaEdzbkktT25ZT2Y0Nzh0bVBhQW96TUhpWkdEOEJMVVk2UWxLOENKZGk3X2tQcDNsWGZtU0JkM2U0N3VfUWFBclhUSUZya0NwRTJOWmZJdWlhT3JtY1EtSkJ6TmlsV3dzOXpDaVFMNlBaa3RfRHBjc3Q0cjk0eVdPV2MwcjlHNA?oc=5</t>
         </is>
       </c>
-      <c r="E48" s="13" t="inlineStr">
+      <c r="E48" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1846,7 +1849,7 @@
       <c r="F48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="13" t="inlineStr">
+      <c r="A49" s="14" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1856,17 +1859,17 @@
           <t>Eyes on 3D Energi as oil and gas giant Conoco flexes buy-out rights</t>
         </is>
       </c>
-      <c r="C49" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D49" s="13" t="inlineStr">
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D49" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWVU1QmhTUGFkYlpTQkw1WUFPTHhmbk5lbnE4T1haQUswSi1ITHlhVmhyM3ZYS3N4cVd6ZkwzdGdhT1lvM1JJek4yLXFpSWoxUnRtR2JRLTZWa2dlTDVTakE3b2xvazFWX0kzRHFZWVB4OUh0XzFFd3JVSVlfelpVa21qTldCVHdvcmJYcGNjZ1RrdElWS3Yzck9KYzRvbzloWkNqMnQ3dmtHbzNuc21ZSXNYeEFlZw?oc=5</t>
         </is>
       </c>
-      <c r="E49" s="13" t="inlineStr">
+      <c r="E49" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1874,7 +1877,7 @@
       <c r="F49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="13" t="inlineStr">
+      <c r="A50" s="14" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1884,17 +1887,17 @@
           <t>Blackstone tempted by $900m payday for Sydney’s JPMorgan tower</t>
         </is>
       </c>
-      <c r="C50" s="13" t="inlineStr">
+      <c r="C50" s="14" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D50" s="13" t="inlineStr">
+      <c r="D50" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxQNEZTZjY0S2YzcUxsb25RSDk2NHd1N1VOVlpMbi1JNGEzbUt5ajlYZFhvLWNBTkNQVXNuWERfTkl0Z2o4R1U0Zk5jVE1FTW5TTUJGZnNJc2NqMm1fT2dmYTVwRGU2TkZ0c3BjZVBGS29fWFJvZ2F0MWNLa0pYY0RNME5xYS1vOGZmMDVBcDBaLV9MWF9od0EwekFyb0ZCOEdkNTFaN3ZXckJwd25zS0FsdzU4OW1UODlueGNyZVBDSDZkeHQwelV5ZXVDVlcyUkhKWDZfVlRacEJHSElmNnhKSXk4ZHJHWHhPTEV5NGNkcmhyU0hjV3J4dVBXbnRGQdIBgwJBVV95cUxPME4ySFF5RWNrejVlWW1yeW56N244RGpyeVJUZEgyTjFNcE10YjVpMmJyeWsxTENzZFhPRlpsbl9pVXl0NGJvUlZFT216NE1KRFNwOHVZVXMzanNKNXFmWEdsMndsd1cza3NTTzUyUUZfaDEyWHJwZEtQbTdJRmkyU3A0RGh4QlAtT1lRVXk2SGoyaTI1NUpwVExYSkZJNmVFNjdXTDJTNURFOEh4Y1dnUDVGdjBpaDlWVWJtUHZiRDdGTmE5R1R6TDBwWFFnT2MwQ1lmT2w5bDF6eVU0R20tYnpnT3JCZlJod2s0UndyZTM5M2xLZC02a3E0NmJRdFV0Qkow?oc=5</t>
         </is>
       </c>
-      <c r="E50" s="13" t="inlineStr">
+      <c r="E50" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1902,7 +1905,7 @@
       <c r="F50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="13" t="inlineStr">
+      <c r="A51" s="14" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1912,17 +1915,17 @@
           <t>I-MED attracts mystery suitor as Permira weighs sale or IPO</t>
         </is>
       </c>
-      <c r="C51" s="13" t="inlineStr">
+      <c r="C51" s="14" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D51" s="13" t="inlineStr">
+      <c r="D51" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxNaGlwS3d5MGFMbEg2U2hnZUxMQmdqaWI4bS1lblNZOFhkSnRMcUotRkZMTjhFZkRUQWxUUDVtYml6TVAxUXkyZmx3SHRFb0gzVHRST2ZQUThKa25aWlhlcGprSU9tWktXZjZRaC12bFpkaVVWZHhIMERyeVNNWEswYTJ2ZHdnRFVRaFhod2U5N011TkQ0NG5MYVhoT3MwRUVZdVB2UVhKZExvdFIyXzNNUGt2SHJUanQxRkI3bXlLSlNJQTF4NXQ1YlZDaGVBM0EzNUhYQVp6NkFWRzU4bnRPWTgtXy1HVnB0ZlN0Uy1rY2FuWlNfN1U4WXVHQnRzVkNG0gGGAkFVX3lxTE1GaDJJdTJlOXFEZUtDTmdXMmsyLXlpaUxzQXpycHk4MTdHZng0dVczYWVwdWRzdFFCMlNLWkZpMm5Zd2RpN0Y0Zmo3Q1FOZFBZQlh5LVl6aVZ3X284UmpxM0pVRzZmMmpjaUdNWnJPZGV4V3lNai1CTllCcW5oUEVxaG0zejB5anc5YnJEZzZPT2d2QklCWjl2MjRBc25jUndqZkVadllKaUZScG12bEozT1NKUUJYR0pHTGtJZVc0ZHZLNHVSYlhzcTE0SkZmMXNlVGJ4YWJ1cThxcGlZTDMzRUMxLVM5VHh2OW5tRW1PT3VyRUhDbV8tRzUzVzRzVWZPZ2w1bnc?oc=5</t>
         </is>
       </c>
-      <c r="E51" s="13" t="inlineStr">
+      <c r="E51" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1930,7 +1933,7 @@
       <c r="F51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="13" t="inlineStr">
+      <c r="A52" s="14" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1940,17 +1943,17 @@
           <t>The stagflationary mix that has billionaire Solomon Lew worried</t>
         </is>
       </c>
-      <c r="C52" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D52" s="13" t="inlineStr">
+      <c r="C52" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D52" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPWTh3S05XQWpTQm03WjhBT1pWc2cyOFRMd2ZraHhPUHlDRW1tWkZvdkhQWHE0MHVMRUpaOFRoX0JsYWhJV21nVkpIM2RBSmlZRUtEbFAydzZfOTh1S05oNEZPOGgyZDJRMS1uLThWYWRVT3VEVGhtYkVLN3J2OWsyX0VVdTUteFBCOVNKZ28xUTRPTk1SUkMxZ1NJc1B6NXRrUEEzOG01YnZOYjk2cWlFZA?oc=5</t>
         </is>
       </c>
-      <c r="E52" s="13" t="inlineStr">
+      <c r="E52" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1958,7 +1961,7 @@
       <c r="F52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="13" t="inlineStr">
+      <c r="A53" s="14" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1968,17 +1971,17 @@
           <t>Oliver Curtis on Firmus: From prison barber to AI billionaire</t>
         </is>
       </c>
-      <c r="C53" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D53" s="13" t="inlineStr">
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D53" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQek9VTlV1b2hVb2RoZ0Fya0REb3E3YlBCR2NYZldXcEh2VEY0LXg5bjd6RzlnZDI0OUJJd2cydTBwTm9tdHpiZ1lSMnhtcmJSYVRKbzJFMjdDaEJyZExSQVJVRDh1c00yMjFMaVlPdnRuV3VkTjNxdzFRbW1yeGltSF8tVXlJVXJzTEJXS2FTYkJTVkdKbmdPTTd6YzRtYV9nN0JzOVZNTzhUdUk?oc=5</t>
         </is>
       </c>
-      <c r="E53" s="13" t="inlineStr">
+      <c r="E53" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1986,7 +1989,7 @@
       <c r="F53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="13" t="inlineStr">
+      <c r="A54" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1996,17 +1999,17 @@
           <t>Three startups that raised $161 million this week</t>
         </is>
       </c>
-      <c r="C54" s="13" t="inlineStr">
+      <c r="C54" s="14" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D54" s="13" t="inlineStr">
+      <c r="D54" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNRGVZMF9DeGJjX29vN3B0blVoM3RKSlJJTllrMThKUDJNZzdPNFNnT2JyTElUOUYxMHlsUm9yM2dBQnZfaVNZblpqb3NzTXdHVlpQNkRqR3NBZHdzODdjN3RKMTZhSVRqUEM5d3JRc3F2OG9hWmZJdU5rakg4ck8wLXlMTnZSU0lNaERmQmswbkVGWW8?oc=5</t>
         </is>
       </c>
-      <c r="E54" s="13" t="inlineStr">
+      <c r="E54" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2014,7 +2017,7 @@
       <c r="F54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="13" t="inlineStr">
+      <c r="A55" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2024,17 +2027,17 @@
           <t>Iran eyes ‘plenty more’ vulnerable energy targets in costly war</t>
         </is>
       </c>
-      <c r="C55" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D55" s="13" t="inlineStr">
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNLUN1MHlZaTNfVHhVX0RnTXp5QW83RmM4WVZkWW1PSnNaZF93VkY5ZF81anB3NDNmX0kyMkVSdkxNSURvSEh6enloWnRVcTlsR0JPTjVzNFR1YjRsSm52VnA1XzFFUlUtODJjYy15YWRRdWZZRkdjRXpCcEFSVURmV3VpSTFhTjVUb1d5bmw3NHNlT3VQZU9ieEYwM1J1TGEyZnlnWXNIWFJUMEtIOVZad0dxRWZBdw?oc=5</t>
         </is>
       </c>
-      <c r="E55" s="13" t="inlineStr">
+      <c r="E55" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2042,7 +2045,7 @@
       <c r="F55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="13" t="inlineStr">
+      <c r="A56" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2052,17 +2055,17 @@
           <t>Don’t take it personally: Bain Special Sits hits hurdle at Infinity</t>
         </is>
       </c>
-      <c r="C56" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D56" s="13" t="inlineStr">
+      <c r="C56" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQRjdwTk0xTHVIRHNkdG9tVk1EQ0hiQjJ6dGcxaWZRZ0hZV1U4YjJDU0tnTUlWSkQ1S2dUTHJVNk0tNWQ2cVd4dkw0M25leXRreWJtdlBKYTAtNzRocTJUazh1dnRzSVlYZThySTBNVjg5X0xYWUxCMC1SelltSHVSUEV5U3B1bTA2NjAzMGFZLW1CNkQ3aWU0S1JxS0d0YmZiZjBKQVRNVUpzYno5R1pvbTBsaTM?oc=5</t>
         </is>
       </c>
-      <c r="E56" s="13" t="inlineStr">
+      <c r="E56" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2070,7 +2073,7 @@
       <c r="F56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="13" t="inlineStr">
+      <c r="A57" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2080,17 +2083,17 @@
           <t>Drill, baby, drill: It’s boom time for mineral and petroleum explorers</t>
         </is>
       </c>
-      <c r="C57" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D57" s="13" t="inlineStr">
+      <c r="C57" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNdlFOWld5ZWhPVnFRa2xidWlUVzluQzkxUTgxR0t0Rmg2S1BzNjdINnhwS3VLRkNjRVJLX0RHU0h4VFVRY2RfSHBudEhfNVNjeE50ZUxQenJNSlJtWFRlcnNsZm1iLXlxM2RmVDViWEtjNDloaTBhUDVxYkNfOWFCTjV6cExEVlFCMzNfWnVwRDJHYWxWV0hOR2V2S0VlV2NyS2s5cWNmREtWXzlMMDRQNW1tVlBOblp3SHBEVg?oc=5</t>
         </is>
       </c>
-      <c r="E57" s="13" t="inlineStr">
+      <c r="E57" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2098,7 +2101,7 @@
       <c r="F57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="13" t="inlineStr">
+      <c r="A58" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2108,17 +2111,17 @@
           <t>‘Wake up’: Fury as farming crisis looms</t>
         </is>
       </c>
-      <c r="C58" s="13" t="inlineStr">
+      <c r="C58" s="14" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D58" s="13" t="inlineStr">
+      <c r="D58" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNelJvMXFPX3MwUVRMN2xqbzE1MWdvOF92Zy02YmIyZW9SQXRNQVZsS0xVVG9UdkFPaTV6ZC1tV05SZWNqblNFZ3Y1VGNaVVBaaEl6aFJqQ09ONDVkNUs4TzNvVjV5eHNjUk9xaDRFZTM0alpuYUdvWGtLRzRhYXN5alZ1QWdsZTEyODdQVnZoazkya29WeTJZVmpxLVBCdWxfY0dTN2Z3WFZlSy1sVW44RDlvZFAzYlhnQ0N6UWhKSU02eF9iZllIU3g5MWtSbkJzZGxWLUxHNERzdUlLTF9VYmpJSTRLY3U4NlVVaDhmc09uOWwtUGtlb0I2M05DR1dnRWxGSFV2NEJXaEF4c00tN9IBlgJBVV95cUxOSzZ5NXZMTTlZa3BSNjZyTUxUMjRhYWJhN0hMa3dDcW9CWGstNnI5MzV5U0hJSTdKLTFwa2E5YUItZnFRbW5RbzVuYW91MmZaYXN3R25hWVpUbW9oUU9fVktPRHROVDYyd2dSLXJVZWQtY016bkVxY0VPbkY3Zkgtb1liWGMxeEpyYmloS1V0TVJMMWZaeWRZX3FQRjBmVzJwdkkwMEVDSXV1MTdReUhGZ0Z3dENyMEFkLUl1aXhtRkFLRFFXcEdMZzFuT3NxRDFMOGVaY2YzeXBQc09fY3YwcFp4MVczRVN3d3dJZWJfTFFscjF0cUtRWHdzTUptaHowNDhYWXZXTHhYTHNTdlZGUmNlamRTdw?oc=5</t>
         </is>
       </c>
-      <c r="E58" s="13" t="inlineStr">
+      <c r="E58" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2126,7 +2129,7 @@
       <c r="F58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="13" t="inlineStr">
+      <c r="A59" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2136,17 +2139,17 @@
           <t>Construction giant FDC road tests IPO pitch</t>
         </is>
       </c>
-      <c r="C59" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D59" s="13" t="inlineStr">
+      <c r="C59" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxON3p5Y3VPM01XZFk4a3g0R3JnQkZXbHVGV3BKdDB6M3NRb0M0SEl3V0R5RmhCQ3dnaHB0ZHp5N2hCMUFsNU1ZNWZ4YWdNZWdETkUyZmdoeW81amwtTWNFZlc5WlNpMkJwRzk0QklORGhlLWNEalh2d0JCX0lhVHhhUF9ibVlxcHAwOW9ENndVOTY0enBYUWc?oc=5</t>
         </is>
       </c>
-      <c r="E59" s="13" t="inlineStr">
+      <c r="E59" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2154,7 +2157,7 @@
       <c r="F59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="13" t="inlineStr">
+      <c r="A60" s="14" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2164,17 +2167,17 @@
           <t>Austal suitor Arlington Capital Partners buys Eptec’s defence unit</t>
         </is>
       </c>
-      <c r="C60" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D60" s="13" t="inlineStr">
+      <c r="C60" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D60" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNM01qb1ZRZVBIdmp3cFc3R3RLaTdmZk1JOFo4anRtSm95Z1hJc0N0S3VranBTV29IdlViT0FkSm92eHdtbDBqdU5HTHNMaXo0dGRWMkpDdjk3LVRBVU1rZC1YejZJMkhyNmpZZFJodGoxWlB1dkRhYTJVRlljMlV0dUllQ3EtOHZkNFdSUWJLSW9Xemw1XzFzU2RHV1o0RTViOXp0bDZFQTZycWhpNElLU0FZQVI?oc=5</t>
         </is>
       </c>
-      <c r="E60" s="13" t="inlineStr">
+      <c r="E60" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2182,7 +2185,7 @@
       <c r="F60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="13" t="inlineStr">
+      <c r="A61" s="14" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2192,17 +2195,17 @@
           <t>Eyes on Tom Wallace as clock ticks on Adgemis pub deal</t>
         </is>
       </c>
-      <c r="C61" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D61" s="13" t="inlineStr">
+      <c r="C61" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D61" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxNSExQeDlENWlHb0prRnRldjZ5YWhKVUZ5eVdsYjZmbVRWRWQ0WnZXWkU3UHZJdElnQ21jMU9zNnhnc3JlNDczVGQ5Y0FGV2J3QUp3NXdZTXZMNm5tVC1vWDFtOFN3aS04QVJZb3FZV2VsUmJ2aVgwbUhTaFVGdHg0UjRyTXVVUnFhQmE5eFYwMGR6T1R2U3Q3WEdZclVKNWJiby1IRg?oc=5</t>
         </is>
       </c>
-      <c r="E61" s="13" t="inlineStr">
+      <c r="E61" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2210,7 +2213,7 @@
       <c r="F61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="13" t="inlineStr">
+      <c r="A62" s="14" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2220,17 +2223,17 @@
           <t>UBS names head of APAC leveraged capital markets</t>
         </is>
       </c>
-      <c r="C62" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D62" s="13" t="inlineStr">
+      <c r="C62" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D62" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNMm9WZ2ZKVFBvX2pYMk16VmY1WFZnZ2J5N0F2bHduTVM0Sjg4STVtTGFLQVdzeFloVHg3clRic0owTDMwYVpXdDVjdjFOWjQxdkdxdFY5MEY1Q1U2Q0R5dFBJWTNtUzgyd3RXcm9uM0hKdEZ3b3JjXzcwQ2VpRm5SS0hYT2gxSU9iVFRlR05Xd2EtM2JOQjBGUzlKdnE?oc=5</t>
         </is>
       </c>
-      <c r="E62" s="13" t="inlineStr">
+      <c r="E62" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2238,7 +2241,7 @@
       <c r="F62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="13" t="inlineStr">
+      <c r="A63" s="14" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2248,17 +2251,17 @@
           <t>BHP, Woodside rise after new CEOs named; Future Fund chiefs exit; Sandilands ‘doesn’t accept’ termination</t>
         </is>
       </c>
-      <c r="C63" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D63" s="13" t="inlineStr">
+      <c r="C63" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNUHhZeHNHemtiLW1IOHN1OTZXOGpsM0ZtUG1MVHRCT1hUT1k5S2lEOXlXRENWOXNlMEZadThQR18xSTJfTVlQM3BtX0ptX1J0bk80SzNLUVRtbkJITGgtb0lsSVdJTWt2S1E1WUlXdUdsbEV0V1RpNWlyRXBoc0dPVDl1OXRrSlM3SHlDazg2UlcxenVzNzlhQldhUGhfNE5IV2xrVmVBNzhhSE9qY042Z3pzMEVzd0VyVmZudXgxcTgwWGJXSWZKZ0FyNVhjcmhjTm5DYUVjLUdDRmxUQkZuTDFlUXVaV0ZoSWp5WHMyR3c?oc=5</t>
         </is>
       </c>
-      <c r="E63" s="13" t="inlineStr">
+      <c r="E63" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2266,7 +2269,7 @@
       <c r="F63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="13" t="inlineStr">
+      <c r="A64" s="14" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2276,17 +2279,17 @@
           <t>BHP’s new CEO will shift the Big Australian’s centre of gravity</t>
         </is>
       </c>
-      <c r="C64" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D64" s="13" t="inlineStr">
+      <c r="C64" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D64" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPQnZpWndNZzZvN1VsOHBmRDVLRHVTNkxLeDVDelpOMURjOTRDSDZfN2dPZlZqaW05WEZuZXMyRTJZeVZnV0poT2UxRkVfZ1RZSjdvUjVKblhoSU5Cd1plRTVNNTRaNWZmbm1yUGZkblVpYkctNzVRRkVQQm4zX1FtRG1KV2Y0djUtOURianJ3dElqeXBUMFp4aWFEWVFYelVjYTluSWpOM1FlbHpIaUxXdnBn?oc=5</t>
         </is>
       </c>
-      <c r="E64" s="13" t="inlineStr">
+      <c r="E64" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2294,7 +2297,7 @@
       <c r="F64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="13" t="inlineStr">
+      <c r="A65" s="14" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2304,17 +2307,17 @@
           <t>How philanthropy became the sandbox of succession</t>
         </is>
       </c>
-      <c r="C65" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D65" s="13" t="inlineStr">
+      <c r="C65" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D65" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxObnBPb2MzQ1RvSVVCbmNzYWFBMlFjU0dQRmpPakNfdkxtMWc1bFdVNXNlZmRKQnNlWEtUUDNSTHpTLVV4Skx0V2otbTZsTTdvT1VaUDhMZFZoMFFab1RoS2pCcno1WGlNQlY4eXQ0OFEtLXJTay1MUkFSSEJ2MVVScUpjUkhJOThISy1QbHIzTzFlWVhOc29fWWs0V19sQ25hRW9MSGhBVVNKWUp6dUo3NS1SWlk?oc=5</t>
         </is>
       </c>
-      <c r="E65" s="13" t="inlineStr">
+      <c r="E65" s="14" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2322,7 +2325,7 @@
       <c r="F65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="13" t="inlineStr">
+      <c r="A66" s="14" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2332,17 +2335,17 @@
           <t>Advanced Navigation raises $158 million Series C round with NRFC backing</t>
         </is>
       </c>
-      <c r="C66" s="13" t="inlineStr">
+      <c r="C66" s="14" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D66" s="13" t="inlineStr">
+      <c r="D66" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNTXhwVlVLUy1pWEpFdzFCazNTY0dkczd4WW9oeW14cUtTaDZRTGlVQXBPaHN4WTBkNW1zOGxvN0tVWl9JSFdVNXlQMzVxbk4zbDZFUjNOcUxSamNaSnFCckMzWEk1VlNoSHJHQ3VWdGltVWZCV0c0NmU4UlN6YU55Q0J2TkQtUzBzOW96UXRxem5Zb3M2SUljNURISlRkQmJD?oc=5</t>
         </is>
       </c>
-      <c r="E66" s="13" t="inlineStr">
+      <c r="E66" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2350,7 +2353,7 @@
       <c r="F66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="13" t="inlineStr">
+      <c r="A67" s="14" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2360,17 +2363,17 @@
           <t>Kal Somani-led consortium buys Rajasthan Royals for USD 1.63 billion</t>
         </is>
       </c>
-      <c r="C67" s="13" t="inlineStr">
+      <c r="C67" s="14" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D67" s="13" t="inlineStr">
+      <c r="D67" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOX3lmdG5aTmk4TEpBa3ROdWZ1aDJHUElBQXktVmlKaHFmTUhPX1QxX1dKLXZfaHRDQjBnWm9McTZjTjJtTWFETTRNMHgzN0tTTm1xY0JpMF84Q2lNaFQyZGVjaHN4bkVmcDN5Qy1ta3FtYnpMSVVyYm0ydWpTRUdZU1hoYXpaNkZUQzlPc1QycjZ6aG5QVHRqY213?oc=5</t>
         </is>
       </c>
-      <c r="E67" s="13" t="inlineStr">
+      <c r="E67" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2378,7 +2381,7 @@
       <c r="F67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="13" t="inlineStr">
+      <c r="A68" s="14" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2388,17 +2391,17 @@
           <t>KMD says Rip Curl demerger proposal delivers investors ‘no value’</t>
         </is>
       </c>
-      <c r="C68" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D68" s="13" t="inlineStr">
+      <c r="C68" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D68" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPTXhBdHByWE9EbllFdDA2OW1UTUZEMVJfV2xsNFdURFRKX2JrODJReVRuQlFoakpWbTBKcjhNLUVsNE9sdG5LUElLZlVrbFNERS1QZTN6bEZIWEhXZ1pTWG5GWEw3ZmNETTdDUDUzYzR5M0E3ZGVlTWpSUnVlVU56dDNFZUtZN3liZ1dKNzJhLWU1S0M1ZnlKd1JNWXlxSlkyU3pGS1lhS05hTUJPRkxucldabzFucGs?oc=5</t>
         </is>
       </c>
-      <c r="E68" s="13" t="inlineStr">
+      <c r="E68" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2406,7 +2409,7 @@
       <c r="F68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="13" t="inlineStr">
+      <c r="A69" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2416,17 +2419,17 @@
           <t>Ex-Macquarie banker drives mortgage broker roll-up Recludo towards IPO</t>
         </is>
       </c>
-      <c r="C69" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D69" s="13" t="inlineStr">
+      <c r="C69" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D69" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxNQms5X1F2aTNhOExDbW42TlZOLVJwVWxna1JYSW9vWF9Na1RZa1ViTFdZc0tCcXRZZkRudTlsTzNuZGgwSENyYi03Zjdfc0lZTXp0NmJRZnhzb2pWRXRIOUdJN2lQM2h3ZFFtTXlSWHVWOFBIaW1Na3FQMjBCck1nVlhUcmRkLW9LOHpKWXQwTm9LcWR5M2FfdjFiRW04TndoanR5NmJvMENGalNuUGNINy1Qc20xR1J4d21ncHNNSUZqa1BXNnI4STIxSUFkZXdU?oc=5</t>
         </is>
       </c>
-      <c r="E69" s="13" t="inlineStr">
+      <c r="E69" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2434,7 +2437,7 @@
       <c r="F69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="13" t="inlineStr">
+      <c r="A70" s="14" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2444,17 +2447,17 @@
           <t>Coles reviews truck fuel charges as crisis worsens</t>
         </is>
       </c>
-      <c r="C70" s="13" t="inlineStr">
+      <c r="C70" s="14" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D70" s="13" t="inlineStr">
+      <c r="D70" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxOSGpBM3RjLVJ3LVlmR1QydnY2dm50WlVxcG43ajRFZ25QS1hDNTBONU8tY3Z2TklzbUNla0ttZk1GZzFaLUZRakFjSUpUQWItQ0VqVTVwS1B0QS1ObVEzNzdRT1l6aU9pVm5jSlhna1N6QmFKT3k1RkhMZGNTVnVLcDVIcXZmRjdjLWRpYVlRQUVmcVRtM21BSjVhTGNaaThyZkhLS2NWdkNCSkZKTlloUVdtbzRnYjFKbllOZXhOd3lkcFZEYURwUFVNQzVnSWRyM1RlOGd2M1pMZXI3c0NIa0Y0MNIB6AFBVV95cUxNSjB3Z0hoTGxwOHJQQ09xb3BmRmhCYjBCc2E0OHA2elFDRE45UGpaTEVDc1Y2VnRvVmZQUzRHbng4QTMwNGZZNGpmaVlHRmV6bnhiZ0FReU50TnRiQ0NZMEtoM3dBZ0hXbFBZMVJQNXd4LVdXRDVyTDAxNS1zeVdvcFVvend2N3J5R2pLYmhxNVFfd19rUlRsNWNndlptMUVkcS1CaUN6UXRHVzByTU5BMW1TdktOZUJYck5xMEJucmR6czIySEMycDA5cmR1MXB0N25Xc0JDUG9zN29YWklVc1BUMzl3UVhn?oc=5</t>
         </is>
       </c>
-      <c r="E70" s="13" t="inlineStr">
+      <c r="E70" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2462,7 +2465,7 @@
       <c r="F70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="13" t="inlineStr">
+      <c r="A71" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2472,17 +2475,17 @@
           <t>Sam Arnaout’s Midas touch turns suburban pubs into pokie gold mines</t>
         </is>
       </c>
-      <c r="C71" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D71" s="13" t="inlineStr">
+      <c r="C71" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D71" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQV2xlTTdYOFpIMzNmVVRnMlJRbTdGTC1jelVCd1V3UjN5cHQ1VzhWZzhrNW1PNm1RX3FlZmU3UkRycjF4WDlQUzRMcVVYY1g3UTZqQ0hxRnl2Ti1IQ0owVmZjN3Jod1BFbmhPVUwxNjhsTGh6d0kzdU01N0hmempRZ044ZmZNUllnenhyc3djRGJOdEtrekx5UVFoaFFMWDdqMHMwdng1SFg4TzZHY1hQNFJNN3huZXpWYWFtQ0ZJakhkVFlQcl9SQlRfZkQ?oc=5</t>
         </is>
       </c>
-      <c r="E71" s="13" t="inlineStr">
+      <c r="E71" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2490,7 +2493,7 @@
       <c r="F71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="13" t="inlineStr">
+      <c r="A72" s="14" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2500,17 +2503,17 @@
           <t>Gentlemen at Melbourne’s exclusive The Australian Club sweat another election</t>
         </is>
       </c>
-      <c r="C72" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D72" s="13" t="inlineStr">
+      <c r="C72" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D72" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPcEwyU01BOXF4TzlmREhYbTFEWklxdWZqWmZybDVnOWtLQ2dTU2dNQ2t5M3BVT2stN08xYkFmazVkY29oT3RVc2xUZmZINFJURGtIRTg4RGsxOURBdWEybTUwU2NUODQ2eDNBbTdPT3QxeXRFNHlSc014T0g1aG4xZ1A0U0FWMTB1Wm1CSHlQU0ZJb3lMYkE?oc=5</t>
         </is>
       </c>
-      <c r="E72" s="13" t="inlineStr">
+      <c r="E72" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2518,7 +2521,7 @@
       <c r="F72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="13" t="inlineStr">
+      <c r="A73" s="14" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2528,17 +2531,17 @@
           <t>Inside Fortescue’s AI ‘hive’ that could save the mining giant billions</t>
         </is>
       </c>
-      <c r="C73" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D73" s="13" t="inlineStr">
+      <c r="C73" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D73" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOSVVCbGpzcVcxTGlZZ2dTUkxXdVVvVU1ONEtUS0t1R1VkWWRNeUF1UmlHbXd6clR3QVRuWGxrUGQwVG1OeUxZb2RqTzdYOEVGQ1N6eDFta3VOZDdHNThYbUEwWEVHZlZBVzNpZ1Foak1kLURZTWpJVzZLekczdzFrdHMtLVZwMUZnYmkxSVc0czFqWnFaSGZiT2pIVW5rdVZmdThreFlRZWVEU0xoa1VFOV9MTjE2UHFOcWhqUzVB?oc=5</t>
         </is>
       </c>
-      <c r="E73" s="13" t="inlineStr">
+      <c r="E73" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2546,7 +2549,7 @@
       <c r="F73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="13" t="inlineStr">
+      <c r="A74" s="14" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2556,17 +2559,17 @@
           <t>Tiny house maker Elsewhere Pods seeks cash after Bunnings debut</t>
         </is>
       </c>
-      <c r="C74" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D74" s="13" t="inlineStr">
+      <c r="C74" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D74" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM0ZpVnBTS21Ib25qa09CaU52Z29kZWhTU0FJLW5VR2JCLVFPTVlZTmpYX3lZVWdtMDVTYTJkWHlPUmhXa0Rua2ZXTTBWQU1VdmFrV21KOGlrdjJ3TTdxbGlvZVBUZUxUWE1uelpWMGxWWk04UndJTXVKQjBZUEtoX3lodmdpMWZKNUc1YTIxVFZLYkFKT1QwbS01WU01ZUZTTlczY2ZpLXlpTjNJTWpsUg?oc=5</t>
         </is>
       </c>
-      <c r="E74" s="13" t="inlineStr">
+      <c r="E74" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2574,7 +2577,7 @@
       <c r="F74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="13" t="inlineStr">
+      <c r="A75" s="14" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2584,17 +2587,17 @@
           <t>Chinese consortium emerges as dark horse in Made Group sale</t>
         </is>
       </c>
-      <c r="C75" s="13" t="inlineStr">
+      <c r="C75" s="14" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D75" s="13" t="inlineStr">
+      <c r="D75" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQYlpEY0hxNm5lalIxSTUzbDE4UEF5QTNpMTl4dWNPMkRrMU1yQnltZ25WcUkwOU13V2Y2RGItVW5QTXotSnBZRUJMdGJySGw0NVVxc3ZLZmVEcTlfU193Vkd5UVVuTFVYWFNtd185eGlVQW5RRElHdk5pMjhUR24wd1k0T0I3cW9qTG5Lcjg2bV9aNWsya0FYODRjeURyMW1EeHdYT05iZHZhLVFrUVNoV25idnZYZ2lpZEhta2JxOWFJb0M2SE9hbFF6NlVWYTM3QmF5anpWOEZackZiTDBfN2gtX1luQkxFOUxSSNIB8gFBVV95cUxOQklMYWl1ZkRqZGUwN0ppeXFubzZWNTNmeE5GY1BfcS13N2dFT096YW9JSndVX1EzTlBKdWZIemdKZnRIME9SQk5aT1M2WnRESjJxckFTaUdOSEd6eG9hRVBjdlhBbWQyWGpUS1kwQXJsdlpkLXJpXzJZX2xiUC1FSlNnNTFoVXQ4bF9JeUp3UGRWdUFOUVRrNUtsRzRxaUczb1p2LVVucFBNazhuZFNDaUZDR2ZQUVdObmVtTnBndGlkazZqeHVheVNzSE9RY3Bad0lrckxDSWY5QXBWS0hwVzZvSTZjaGEtNkNncW1RRE5uUQ?oc=5</t>
         </is>
       </c>
-      <c r="E75" s="13" t="inlineStr">
+      <c r="E75" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2602,7 +2605,7 @@
       <c r="F75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="13" t="inlineStr">
+      <c r="A76" s="14" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2612,17 +2615,17 @@
           <t>KMD faces uphill battle in capital raise as key shareholder baulks</t>
         </is>
       </c>
-      <c r="C76" s="13" t="inlineStr">
+      <c r="C76" s="14" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D76" s="13" t="inlineStr">
+      <c r="D76" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxOVTU0OGNfRURNcDdzYUtIcG8tR3N4OFFYalhKNWJBaUd6ZlQwNU5MZVZYbUZVSzB3WmdOOFdTZHlBOXBzSGdYUVV6eGt1UndHN296bENxZzNUM2NoaV93LXZaZFNNOXJ2YlA4RHNFS2FDb1ltNWpPWUdRR3VGMWoxaU5qYm9VSW9yUW5kS1NaN2RSc2YtcHZRSTB6aE9Zdkl3NG5nbVRzODRfQVYtelo5M3g4R2JEbnpraFpWbENOZzE2Qndla2t3MXRPWkU1dXg4NmZRME1jT3pOOHZOVlpTZGloNENUZllaSTFmWUV1Y2JLck02ZDhnTHJ5bUPSAYICQVVfeXFMUEFXR29tQjlTbTdMRVNDWUlGNFNOQjVhX0FiSkl0U2stbml5VHR4d1g3bDFqMUw2TzR1eHhYOU5ZUmJpZ2xBY2NzcmJRX3MwaEQ0YmpzMUFnV1BQNGxmcnlXUzVvbHpwNEo5dWFnZlduZ0Z2dGZGRFRKRTNCUzctZDNCd0FMNEkzTm84dmZOM2NKYk81RERsVnlZN1VZaXp5TW5QRVAzOHNXQTFWdVlKdGtFX0FmcU1EbElZSm52alBQeWx4VnlvOFRwNk1ia2lZYXlpemQ4cFdmckotMmMyRGE4ZXN0dThQYmxxUkpvMzAwRXBBcVJuRnp0QkZ3b2tqMWF3?oc=5</t>
         </is>
       </c>
-      <c r="E76" s="13" t="inlineStr">
+      <c r="E76" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2630,7 +2633,7 @@
       <c r="F76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="13" t="inlineStr">
+      <c r="A77" s="14" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2640,17 +2643,17 @@
           <t>AustralianSuper claims another listed M&amp;A kill with Pepper Money</t>
         </is>
       </c>
-      <c r="C77" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D77" s="13" t="inlineStr">
+      <c r="C77" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D77" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOY0RwcnpWZlhfOHA2MG13MkJUX1RDNF9wN2RxZGU2cEpzS1RKTjJDeUl0OERFOGhFRXJaSXNETEhHbW9PS0lua283RnFVbHJvTlRva0djQ2lRSGc2RENJYmt0OEsyYTRVSzFGeE9jWVhKMVRnd240WXVNTVdac2lOUGJSZlc4UVZ5RXo0OTlQbUd6NWRSek1HZG9fZGk2aDhDelhGVmk4YkRKeVV1M0VHZ2hZNmFVdXM?oc=5</t>
         </is>
       </c>
-      <c r="E77" s="13" t="inlineStr">
+      <c r="E77" s="14" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2658,7 +2661,7 @@
       <c r="F77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="13" t="inlineStr">
+      <c r="A78" s="14" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2668,17 +2671,17 @@
           <t>Apollo to Acquire Nippon Sheet Glass in $3.7 Billion Deal</t>
         </is>
       </c>
-      <c r="C78" s="13" t="inlineStr">
+      <c r="C78" s="14" t="inlineStr">
         <is>
           <t>Wall Street Journal</t>
         </is>
       </c>
-      <c r="D78" s="13" t="inlineStr">
+      <c r="D78" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOanpORVBremoyamJyZ2FqQWVOcDcxa2NpempBUmNYcktMLUl1Mzg5VDloWmlVbUdNUnplVk90WEUzXzJjNGxENk9LcGF0enVSdlFpWU9nd244YWNTS0ZHd1JTZEtlbjRQTmJUU0dzWmlDOVFhR1ZRSFJkNXN4a3FHdGozcUcwdHRseXpYMFREUzBNcXRmQ1VCN056SWlEa1l5VVE?oc=5</t>
         </is>
       </c>
-      <c r="E78" s="13" t="inlineStr">
+      <c r="E78" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2686,7 +2689,7 @@
       <c r="F78" s="3" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="13" t="inlineStr">
+      <c r="A79" s="14" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2696,17 +2699,17 @@
           <t>Estee Lauder in talks to combine with Jean Paul Gaultier owner Puig</t>
         </is>
       </c>
-      <c r="C79" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D79" s="13" t="inlineStr">
+      <c r="C79" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D79" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPSjN6QnFVbmdHWFoteURWaU5VaWZmRmpTT3QtYm1tZUFyNUZyLUdheGdfWlRBTlJyTlp4THIwVDA4U3BnWFNpT2FpZlZzX1lJSDV0MkRGVjYtNVc0b0lOQy1RSnFGTWhCTWE2ZFFPYlFQX05yaVlfZF9IUEN2ZWkzQ0VFMUxxdHF2ODNQY09xdWlqWEczSC1CZk5wYU9QQlAyaTMyelJnaVM0cmN4M0paNzlBdzM1RndoZE8yRHN4UnZqaXVhVmx5NFpqS3hmUHhUdlpF?oc=5</t>
         </is>
       </c>
-      <c r="E79" s="13" t="inlineStr">
+      <c r="E79" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2714,7 +2717,7 @@
       <c r="F79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="13" t="inlineStr">
+      <c r="A80" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2724,17 +2727,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C80" s="13" t="inlineStr">
+      <c r="C80" s="14" t="inlineStr">
         <is>
           <t>The Age</t>
         </is>
       </c>
-      <c r="D80" s="13" t="inlineStr">
+      <c r="D80" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPdUtyNWs5YmxJMXNsNWtaMi1WMm5SVHd6ci1ReURLajdYd1IzWGJMZmE2MzJsSzAxQWtSTm8xMUEwNTh4Vy1zTmFsWFBKTkJ0YXc3ZkcwOVk2a2VNRWVGUS0yQzZhSXlCWmpDYUx6RmpTTlNhS0xIQklyVFdIVXJRZTNPaVB4TG4yQ1R1ZWF2MWpmSG81TVRaRzdtMXpydWhBS2w0a3ZPZFI5MnFKOW5tN21oUDB3NkNtQmR4LVVBWW9BUQ?oc=5</t>
         </is>
       </c>
-      <c r="E80" s="13" t="inlineStr">
+      <c r="E80" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2742,7 +2745,7 @@
       <c r="F80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="13" t="inlineStr">
+      <c r="A81" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2752,17 +2755,17 @@
           <t>Australia’s new millionaire factory: Start-up to $1.6b in five years</t>
         </is>
       </c>
-      <c r="C81" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D81" s="13" t="inlineStr">
+      <c r="C81" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D81" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOVkl5N1NGWS1XWWZSc0pHXzE3MUNERmV5SUgyQ3o2MmJ3U3Y2YlNwUXNSTGlQenBwVFdnMWhoT2FrcDAwUHNVU0RQbjFHMjJiLU1TRC1nemdrX3hPTG93VWZUQUx3Wk9HT3lYd055Z2FtREFpOWRlYXFDb2hwV0cyWFMwaHpsLU0ta2VVQlpid1dlYks0ZHg5YTY3Ykt6Um5YaF9MR2tIRzd1Tk1IRnBrWVhxVjZNSUl1OE9iRlZzYmQ3QUVnZmhYVGxoOA?oc=5</t>
         </is>
       </c>
-      <c r="E81" s="13" t="inlineStr">
+      <c r="E81" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2770,7 +2773,7 @@
       <c r="F81" s="3" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="13" t="inlineStr">
+      <c r="A82" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2780,17 +2783,17 @@
           <t>Social Media Wrap: Genki Sushi Singapore's loyalty benefits; Dunkin Philippines launches new collectible; Burger King Malaysia unveils new Korean inspired burger</t>
         </is>
       </c>
-      <c r="C82" s="13" t="inlineStr">
+      <c r="C82" s="14" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D82" s="13" t="inlineStr">
+      <c r="D82" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxPbFR6eHVTRWZNcUw1TTBJdE1JTFpmbk5iWndKZnRoU3Fmc3cxcF80TnVhRERmY0poM09zTFpCaEVnMGo5aktxY0ExV1ZlZVpHYUtldXBoOUh6bm14SURHNmhnUE9tYnI5YlpXQ3pRZlp0Ni1wM2lYQmdxdjk4SDl0aFN0R1VBbGxpbFVzOHV0TFY3YjJZbDg4Vk1HMTBkQk5LRHd1ZEVpRnBsT1U0Nm1IbVFkZEUybmpabEhuLUNLOGhicUxXZG5UalRLOE5DSzcxRncyNjVRdk8zclhJNkVQcTRkQTZYSEdN?oc=5</t>
         </is>
       </c>
-      <c r="E82" s="13" t="inlineStr">
+      <c r="E82" s="14" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -2798,7 +2801,7 @@
       <c r="F82" s="3" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="13" t="inlineStr">
+      <c r="A83" s="14" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -2808,17 +2811,17 @@
           <t>Copyright ‘status quo’ not working in AI boom times, says Charlton</t>
         </is>
       </c>
-      <c r="C83" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D83" s="13" t="inlineStr">
+      <c r="C83" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D83" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNVVgwdEQ2YUt0eFo3THcxOXZHbUFYZ091VTFKZDZHX0szYWQ2dnZ1dkJma3VZcGk1LUM2SUtQSWhxMGpCUlFZVzdKNmdoSGEycm1oYlBUdEZ5R0ZlU2hrWHpFWXdSN1lCZnZzb3hZc2twVVlWdTNNVXhaR0Nza0FiaUNveXZWQWQ1ZE45MU1HbGNmWlU2aUdha2FyZllzNWdONEpsM2RrdGRFSFl2UlpJUnQ4WGpleGs?oc=5</t>
         </is>
       </c>
-      <c r="E83" s="13" t="inlineStr">
+      <c r="E83" s="14" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2826,7 +2829,7 @@
       <c r="F83" s="3" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="13" t="inlineStr">
+      <c r="A84" s="14" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -2836,17 +2839,17 @@
           <t>The unapologetically analogue 4WD for off-roaders with $120k to spare</t>
         </is>
       </c>
-      <c r="C84" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D84" s="13" t="inlineStr">
+      <c r="C84" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D84" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxPSFJ4ZnNLT3U1REp3MWI2WDFaQm5vZlp6QWN6c0hZamtYVU95WmpkUERwR1dwc0NQN1dEc0FNbHlaMTdLclVHb1JTc2VZNExENGYyUE9OR1BkQ244YXRVeWNwbkxia2VrckVqSy00WV9UNWlvZWJHOG9ibUthaTlpVmRBOGZjLWFzMU8yS2Q5Um05SWIzY2dKajhoMWFUcmFrbTMzai1CdVBNLWczTWRvbTBwSDRfUzNwOHhqQm5hTDdhM0xLWEpNQTRyRXZjU1FLdGhRMUxtOTg?oc=5</t>
         </is>
       </c>
-      <c r="E84" s="13" t="inlineStr">
+      <c r="E84" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2854,7 +2857,7 @@
       <c r="F84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="13" t="inlineStr">
+      <c r="A85" s="14" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2864,17 +2867,17 @@
           <t>Junk room to become jazz club with priceless Melbourne view</t>
         </is>
       </c>
-      <c r="C85" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D85" s="13" t="inlineStr">
+      <c r="C85" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D85" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQbHN4My1nOGtueVJQZWM0LXNjLTR3MmhuemRJMUEwN09FTUZhZk1lbV9MbnVWblgyUXFEMEl3LUtsOGVqdGUweFR0MXF0ZEo0XzNhWVRqb2pGRUdiNTlLc1dFcXFmdnctQU1wQkRSdHN0T3J6VGt3MU1iNENydGlsOEpsT0ttZmJVZ0FUZmFXSUd3alVzUTQxMzVmcEVXSlV2dWdQd3JsMUZ0d3ZZYlBHaGhKTm9rM01SUmdseE9hT1prbHZtMlhv?oc=5</t>
         </is>
       </c>
-      <c r="E85" s="13" t="inlineStr">
+      <c r="E85" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2882,7 +2885,7 @@
       <c r="F85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="13" t="inlineStr">
+      <c r="A86" s="14" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2892,17 +2895,17 @@
           <t>Zimmermann fashion label appoints new CEO Roberto Eggs to replace Chris Olliver</t>
         </is>
       </c>
-      <c r="C86" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D86" s="13" t="inlineStr">
+      <c r="C86" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D86" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM2M5QU1scVoyNHBmV2lwQ0VQS1Z6d2Qwa1ZkZ0M2WVIzdXR3QnZwVWhUSDRCUEdRZkc5QzFQSFFhNzZ4VE9lWXBTcGhpS01JdG12TlQxSHhValZfbWt3MUdFZGl3RlBtdnlrel83TjNjNFZ0SUpvSDNQbThpU3FLa3Atd0dNU04zQm9OSk5uNHpTVE84aWZpaVlKWkdOQjJjRTZSd1MwMEZ1b3pENkRCQQ?oc=5</t>
         </is>
       </c>
-      <c r="E86" s="13" t="inlineStr">
+      <c r="E86" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2910,7 +2913,7 @@
       <c r="F86" s="3" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="13" t="inlineStr">
+      <c r="A87" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2920,17 +2923,17 @@
           <t>Construction giant FDC road tests IPO pitch - AFR</t>
         </is>
       </c>
-      <c r="C87" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D87" s="13" t="inlineStr">
+      <c r="C87" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D87" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNTnRScHFhQlpkdEdSb2x1bExxQm96ZE5zSV9wTDNDV2pxYjFQdUtoYmNBell3SFlTTFEzMUhpeXlmNERSeDd6VGppM2szQ1NHVE9PY1R3MTN0SUZLWkF5em8tQ3IycUZ2RmswX0tnN1IwOHl1ZFo4UUtMUDlQbXRjTnRCWFB5cU1RZFhsdDdaWGpMZzh3d29CWWZvZGtnTjl0T1k5ZHFHSUg5XzFSSF9TSUxTYkU0QkFheFlLZUY3S2tCSWRLZWlBbUpxUjc3TXBQQ01V?oc=5</t>
         </is>
       </c>
-      <c r="E87" s="13" t="inlineStr">
+      <c r="E87" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2938,7 +2941,7 @@
       <c r="F87" s="3" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="13" t="inlineStr">
+      <c r="A88" s="14" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -2948,17 +2951,17 @@
           <t>David Jones is trying to defy retail gravity. It’s causing problems</t>
         </is>
       </c>
-      <c r="C88" s="13" t="inlineStr">
+      <c r="C88" s="14" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D88" s="13" t="inlineStr">
+      <c r="D88" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPZy14UldWZDRrSjI3R0lzdGlKamlkVnU1WWVjTWRUTlpya1ZpVW80WHlrT0FQTUUwMzkzM19xQWpwTnVLOF8zeTFXamhTZFRQVjl5TTlXbE1RRWY2NW03dlpmZ25qdkgyN1IwbDdjRlhxd1MzSGkxeG45M214OVlESWF5WWh5TjM0STQtOXdieWIyOUI2NzRsaDhiS0ROUU5YQ185aWtObUY2S0dOSTBROVlwSVB1VkNqTkZTTllkZmtMYmxjNVdlTA?oc=5</t>
         </is>
       </c>
-      <c r="E88" s="13" t="inlineStr">
+      <c r="E88" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2966,7 +2969,7 @@
       <c r="F88" s="3" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="13" t="inlineStr">
+      <c r="A89" s="14" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -2976,17 +2979,17 @@
           <t>Jefferies’ Australian ambitions in focus as Sumitomo circles</t>
         </is>
       </c>
-      <c r="C89" s="13" t="inlineStr">
+      <c r="C89" s="14" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D89" s="13" t="inlineStr">
+      <c r="D89" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxNUTd0LXFPQmZXSldrTmZHTkIwUWQ3MmlCUmFOUGRkcVVjRXV6YXZJUTcyMG5FV3I0dWY2NXh6MnduVjNxZmhJMHdDVGw5VzFxTEFzN2FBdlNvS1JGSDltQmlzVS1QRDdCeWdfSHZ2VlZDMlBnN1Y0d2JxbnlGejhWVjJpWGZLejdCTUt2Uk9ENmhyRkd4dDJjd0RlUnBlZXhOTmUtOG9ITE05VHJ3dTBRSWZneURuUW1NYkExVXpfWXlsMzZ1WUlyNE84SThQX1JJTFlXOHc4ZnB0aXRmdVhaaG1qSEJRZUhuU3RibHAzbHVNLWFLUF9NNTFoUXV3NGQzelcwcNIBigJBVV95cUxPMkhEeDJpNzg0NTlDZmF2LUFPSEs4cmZ5U2p6bWVZSTYwcXVUUGVIb0FLVnhZV0cta01CLVpfQzQzYzdvTWdxR0o4bGJDWDVBb1lnOGx0bWROdTdjcHhwLUpPMW9MQ0RVM2NUOUt6UGpTd05JYzhuVmgybGp2LVpORFF0SHpBTU5DUTJEUmZKUFBNajlQdHJ4WkdHVV9QMjVwOWVlNWliVkFaM20yWGZhOEc4bldHRERJak1BWXlmSE0zdno1VTVSc0FMck0wSE1BR1RVaVRMSEdzU2FvcWpMYmp5ZTVJTWcyUGdXanhqSUNZU0tzTkNYWVg2SXpVMEoyS184VkxOeWtSUQ?oc=5</t>
         </is>
       </c>
-      <c r="E89" s="13" t="inlineStr">
+      <c r="E89" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2994,7 +2997,7 @@
       <c r="F89" s="3" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="13" t="inlineStr">
+      <c r="A90" s="14" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3004,17 +3007,17 @@
           <t>Bain Gets Nearly $300 Million Loan for Australia Wealth Unit M&amp;A</t>
         </is>
       </c>
-      <c r="C90" s="13" t="inlineStr">
+      <c r="C90" s="14" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D90" s="13" t="inlineStr">
+      <c r="D90" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMUQ4WExYZFY1aFBwWENNR1JiVkw4OHFKWjY4NW4zQ3ZBalFiTU10Y2hic2p2VjFqOE1rMndNYmVoN0lPcnY0WmFOV1MtaEY5c2xvcW1PNGN2SzZVcThwc3ljWkYwV1Q4a2dIaUpBeXZpMkRUU3IxZzVBVkhydGU3OXEzNW1sdlVQeTRNRFY4bUJLOGpGYmJ0ZXpPc1YzY05TYWd2bF9oWVJ6Rks2dWlod1dGRU4?oc=5</t>
         </is>
       </c>
-      <c r="E90" s="13" t="inlineStr">
+      <c r="E90" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3022,7 +3025,7 @@
       <c r="F90" s="3" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="13" t="inlineStr">
+      <c r="A91" s="14" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3032,17 +3035,17 @@
           <t>Fund managers caught up in Aware, TelstraSuper $237b merger</t>
         </is>
       </c>
-      <c r="C91" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D91" s="13" t="inlineStr">
+      <c r="C91" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D91" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcFF4Q1A5X1VtNWFnYXZSVUlZX2JMRVoxaUJoeGhybmRrZkd4UlEzTURwMkx2d2I1Y1hMYmljbk05WUFzRl9JbF9JampqeDd2bXdYcUpHbVZYak1sYXFHS2VuUDJyTUhzSS1QTW15aVpfeHRuMGZHenlxOHJQRUdENkV0b2FMZXhOZWF1Yk5hR1lOYWFQc2Q0SEROUFNERXhKQUIzRkt6NTQ?oc=5</t>
         </is>
       </c>
-      <c r="E91" s="13" t="inlineStr">
+      <c r="E91" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3050,7 +3053,7 @@
       <c r="F91" s="3" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="13" t="inlineStr">
+      <c r="A92" s="14" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3060,17 +3063,17 @@
           <t>Soul Patts defies private credit jitters with 15pc returns</t>
         </is>
       </c>
-      <c r="C92" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D92" s="13" t="inlineStr">
+      <c r="C92" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D92" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPRkNINFJOai1NbUUtX3ZrcnJFS3EzRHZPbFRfVFE3SERudTVqbjIybWsyYUthOUJOUVFPb1U0UzlGTTRqbUxraFZfYlVtclQxeTBQU1M5YjJzMDVPU3RiX0cxbk8xOEd5YjV1R04zT0NNZjhNSi1meWo4RHM1ckFsUnNLd0JiQXFnZ0dtckNzdWxmanZoQUl3TEQ2a29nRkRDZ1lJd2Y5VGc2UWZHX0pkU1NObmRJTlZKS0E?oc=5</t>
         </is>
       </c>
-      <c r="E92" s="13" t="inlineStr">
+      <c r="E92" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3078,7 +3081,7 @@
       <c r="F92" s="3" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" s="13" t="inlineStr">
+      <c r="A93" s="14" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3088,17 +3091,17 @@
           <t>Ex-KKR China heads negotiate to buy Vitaco, owner of Musashi, Nutra-Life</t>
         </is>
       </c>
-      <c r="C93" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D93" s="13" t="inlineStr">
+      <c r="C93" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D93" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQRmlCdTlFeHdBUGkyOS1CeEFIYTRSREdZM1JOZ3IyZThnNmNMdm9QeXVwRWtMbzU0em1vcDAyM1hodDlvalVRdThtNVhLR2FsaE1vV0xuWjkwMkVCUDk5SmVka1BURFJZNkl2bURLeC1GdzI0V2hEaVhrNlJZejlvc2gwRmtnUjd1NDFlX2trbGk2aXJiQ2FrTWtmVVpiOXhBc05JSkNYY2xLX2JEQUpWY2dlY1pDZw?oc=5</t>
         </is>
       </c>
-      <c r="E93" s="13" t="inlineStr">
+      <c r="E93" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3106,7 +3109,7 @@
       <c r="F93" s="3" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="13" t="inlineStr">
+      <c r="A94" s="14" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3116,17 +3119,17 @@
           <t>Antipodes Global Investment Company</t>
         </is>
       </c>
-      <c r="C94" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D94" s="13" t="inlineStr">
+      <c r="C94" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D94" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE5mdkJzN19XLTFQc25LOUk0ZGJBMER6djB2VnFvbGVrS1hlemRBRmlNY2JmMGlPTzktU0RRS3NNUW8tRXhtUE1QdE1JLWdUNVhibmZPZi1MRkJOWk95NzM2bXplS3JzeG13UU5henhza1ozeGRZZmlBNTNR?oc=5</t>
         </is>
       </c>
-      <c r="E94" s="13" t="inlineStr">
+      <c r="E94" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3134,7 +3137,7 @@
       <c r="F94" s="3" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="13" t="inlineStr">
+      <c r="A95" s="14" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3144,17 +3147,17 @@
           <t>AusSuper to lift insurance premiums by up to 40pc</t>
         </is>
       </c>
-      <c r="C95" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D95" s="13" t="inlineStr">
+      <c r="C95" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D95" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQNEhYQkoyNnJFU2xBZG8wdXhEZWRSakRiWWNHOGZBTFhfaElxWkRsSWViaWxjenVjMF91cGdrbFZxSGJfbkR2SUZNdEJtYUVadlV6YVVrWU1VbVdsMWpyNUZ4bE13Mmo4cGQ3WWZlVFVrTTdyOGpSdkpUb0tkcjdQUFlsTnM0MnpOMDJNZlJ4YTlzZGpLS1QzMFluOFU2VUJya3lSclBLSnZkQ2Y0a2djNUpSYlo?oc=5</t>
         </is>
       </c>
-      <c r="E95" s="13" t="inlineStr">
+      <c r="E95" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3162,7 +3165,7 @@
       <c r="F95" s="3" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" s="13" t="inlineStr">
+      <c r="A96" s="14" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -3172,17 +3175,17 @@
           <t>Unions want inflation-plus minimum wage rise due to ‘Trump and RBA’</t>
         </is>
       </c>
-      <c r="C96" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D96" s="13" t="inlineStr">
+      <c r="C96" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D96" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNdzNhU0MzbFRFX2I3OVY4bFItd1h6OVE2Wnpqb01NM2tMYzNob21BeW02LTBfTFZIWnN6SG5DVnYxQTJGZWZaLTJpTXZGUnhmS3RPY3hQV01fd1RIYU9Ednc4a1hvalVRT19ESU5TX19sQjN4dVV3X29kQjliQjNFU19iaXFIS2l3blk5TWUwdHFrRmJtQ0JocDN0WEhWbXZOVUJzR3RaYnJPSHpIRFlYOVFObEtuT1d0TUo0MUVZTXdFZWR3WG1r?oc=5</t>
         </is>
       </c>
-      <c r="E96" s="13" t="inlineStr">
+      <c r="E96" s="14" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3190,7 +3193,7 @@
       <c r="F96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" s="13" t="inlineStr">
+      <c r="A97" s="14" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3200,17 +3203,17 @@
           <t>Firmus’ Oliver Curtis set for green light to run ASX-listed company</t>
         </is>
       </c>
-      <c r="C97" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D97" s="13" t="inlineStr">
+      <c r="C97" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D97" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNR3VmQW9vNmUyeU9WbVRvRG9tcTNMYVlvRUhCd29wTkRZaVlEcG50Z0hIN29XcE5GUmxkUy1yMm0yTm94Q1BXMmNCcXBpZDlqVTRlZFpMX1QyMWh5Ym5XQ3VjYW1ZdDFtYWNyOERCOURuWXM5ZTV4WGthMVVjNUZlcmVTQ3JBUjQzUXRXYXRLQjlNeHpBMkVCVWpsd2Z1Vk42TjJxSlRiQ0ZtaTkzOTZtNmRHQQ?oc=5</t>
         </is>
       </c>
-      <c r="E97" s="13" t="inlineStr">
+      <c r="E97" s="14" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3218,7 +3221,7 @@
       <c r="F97" s="3" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" s="13" t="inlineStr">
+      <c r="A98" s="14" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3228,17 +3231,17 @@
           <t>Crisis Hit David Jones Chasing Funding As Retail Markets Come Under Pressure</t>
         </is>
       </c>
-      <c r="C98" s="13" t="inlineStr">
+      <c r="C98" s="14" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D98" s="13" t="inlineStr">
+      <c r="D98" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNNjJSOUVQcTkwUmxXNXg4ZzljSGhnRlBJY0otSHRrX2ZIQXRqWmNDZlgxYW1jckhHd3BtdXJsUWhwTjQ5SGw2NUU3TnFtcmhYd2JVcThIR2VCLWJLU0h5RE8xaTV5TS03Mi1za19hcF9PcXRRSU9PX3ZxSktSV2FfY1ppcUFVV2w1TmF1UWVtZlBWSUhEcG9oRGlEVkEwR2ltQ2VMSTNlcENEYlY0?oc=5</t>
         </is>
       </c>
-      <c r="E98" s="13" t="inlineStr">
+      <c r="E98" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3246,7 +3249,7 @@
       <c r="F98" s="3" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" s="13" t="inlineStr">
+      <c r="A99" s="14" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3256,17 +3259,17 @@
           <t>Beirut Street Food eyes niche in Lebanese fast casual</t>
         </is>
       </c>
-      <c r="C99" s="13" t="inlineStr">
+      <c r="C99" s="14" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D99" s="13" t="inlineStr">
+      <c r="D99" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNVlZVeTNGcXVOSXV1eklvTnFxYk1hb1A2VTQtNHkwdUpvdFF0YnlYU2RSWkZNV2dGQkEyZjRVQzVJZ2Uwc3gtZ0F1TGlSQlVna01HRnZOTTJnVUFxaWtOam1vZ245Z05jdlRnQURqbnQxaGtEcnFYS20wWmtvSDV0MW15c18zUE5ZN2JJWUpLV0RsZE1LSm5fcUNNeVZNTmdMQ2c?oc=5</t>
         </is>
       </c>
-      <c r="E99" s="13" t="inlineStr">
+      <c r="E99" s="14" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3274,7 +3277,7 @@
       <c r="F99" s="3" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" s="13" t="inlineStr">
+      <c r="A100" s="14" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3284,17 +3287,17 @@
           <t>Gami Chicken credits chip design for cult following across Australia</t>
         </is>
       </c>
-      <c r="C100" s="13" t="inlineStr">
+      <c r="C100" s="14" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D100" s="13" t="inlineStr">
+      <c r="D100" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPTXg4T0dvQ1l4NFVxV25iUXQzY0F3MnFjYmE4X0NOcFdNZHgweUg4NmVZZjNJbTFMajNhNHBmVDE2MGNBZzhOTUJsaG5KejFZbk1Db0JyNTZJbUI2WnRZeVhXRFRMNXVBWVFMdGJ3WkN5dV85dEduQi1OVDhOSE9UOGVERXh3T2hCVmlDNVg5LTdLY2VHNEZJSzlrN3VuemhzX1B5blpYRGtwS0hrak5r?oc=5</t>
         </is>
       </c>
-      <c r="E100" s="13" t="inlineStr">
+      <c r="E100" s="14" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3302,7 +3305,7 @@
       <c r="F100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" s="13" t="inlineStr">
+      <c r="A101" s="14" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3312,17 +3315,17 @@
           <t>The great fake meat meltdown is taking plant-based burgers with it</t>
         </is>
       </c>
-      <c r="C101" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D101" s="13" t="inlineStr">
+      <c r="C101" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D101" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPRTVDNW5oaWJ5bHdKM21iYllEVnpJbHhSbWFzYy1RcEZCdnNGUlJOWVJCaDZacFVoRjlSUGpfa3N6ckQtMFYzZTNITW5tMy05Sk0tZmtlSWlESHdOMWIyUWpUbE5RQVlsTHp0VXg0cHJYM0lJVmw1ckRURkFPVHFabTRIUzlFX1FlbFNuYmQ5MVJwWHVOaVhVWTdPajZxdG1WOTliTE1qZ3k1dnFRbk9BNTZCcXRRSGlIXzJv?oc=5</t>
         </is>
       </c>
-      <c r="E101" s="13" t="inlineStr">
+      <c r="E101" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3330,7 +3333,7 @@
       <c r="F101" s="3" t="inlineStr"/>
     </row>
     <row r="102">
-      <c r="A102" s="13" t="inlineStr">
+      <c r="A102" s="14" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3340,17 +3343,17 @@
           <t>Solar for Cuba: How Xi is turning Trump’s war into a China win</t>
         </is>
       </c>
-      <c r="C102" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D102" s="13" t="inlineStr">
+      <c r="C102" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D102" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQOFlUUnNZUWo0MTJRaDFIZHp5dUJudERrOWxCZmY1WjZmeXRTVzJkbENEbUFhSkZFUWV6WjNGNUJIejVYRXFPcmRNZjFZeTkzTmtaeFNlb2V1OFFnMGtkV2JfTVRUN2FSV2xxcUpDUDJQeUpqWE9DRHRmT2kyc1dIZE9jeUM2eV9KQjd2RkJuTkxYeEdISDZDejhRbVo?oc=5</t>
         </is>
       </c>
-      <c r="E102" s="13" t="inlineStr">
+      <c r="E102" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3358,7 +3361,7 @@
       <c r="F102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" s="13" t="inlineStr">
+      <c r="A103" s="14" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3368,17 +3371,17 @@
           <t>Beer Sectoral Group appoints Nigerian Breweries CEO Thibaut Boidin as Chairman</t>
         </is>
       </c>
-      <c r="C103" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D103" s="13" t="inlineStr">
+      <c r="C103" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D103" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOamdsNTN1dkRUY19Yak0wUGxsdm9NZGhySUM0Vzc4blNCeldzdFBiRkxuSW1xbTlZQUJIWkNxdzI3Zi1zc3F3SmJvai1UVGlZdUhGTEJ0eF9mNHRwSGREbDktT2txWXA4OVBESTdPLXdxWmV2V3FPTEZaYjRWLTlMM1VaY1dCbGZudTczZlFEYzN1aE9HeWdObE1yZFduLUtNVXBheDNsUWlIcUxibml4YQ?oc=5</t>
         </is>
       </c>
-      <c r="E103" s="13" t="inlineStr">
+      <c r="E103" s="14" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3386,7 +3389,7 @@
       <c r="F103" s="3" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" s="13" t="inlineStr">
+      <c r="A104" s="14" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3396,17 +3399,17 @@
           <t>Hip pocket pain comes for shoppers – and for supermarket giants</t>
         </is>
       </c>
-      <c r="C104" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D104" s="13" t="inlineStr">
+      <c r="C104" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D104" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOeTdfN2dwYlBWSTdGbFo0SWRJcTNYelFFM2FBRnlORWRNcGd0WUVCbVdHVWZ6TFdZQzFpM2h6TkU2OEtqeE5OYlRrNmhsRU43a0E0UXhtZEZyTWZidzhMUEVxSVdiMlpTYXQ4ZVRaNl9BSi1Mb3JRaXhvM2hlMmNDcnk1aFBvVXFQSmlPbkN4Z3o2R2RzV0drQWpKaVZpbXR4dHppa08wRFd0dlNwcDc1alRDSXg?oc=5</t>
         </is>
       </c>
-      <c r="E104" s="13" t="inlineStr">
+      <c r="E104" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3414,7 +3417,7 @@
       <c r="F104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
-      <c r="A105" s="13" t="inlineStr">
+      <c r="A105" s="14" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3424,17 +3427,17 @@
           <t>RBA calls for co-ordinated effort to unlock digital asset markets</t>
         </is>
       </c>
-      <c r="C105" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D105" s="13" t="inlineStr">
+      <c r="C105" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D105" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOT3dEcEtwVUptWTZydTRYWFdCU1RhTjI1RkFWeU5HckRVZjBxc2lqRkNOT0stc1h2Q0E1YTkxTjk3NTB3TGxKZGIweGFQRGh2S05QWHRoVGNZRFR2SlI2bkEzWlRoY2t3WU16dDlhVEI4RTFWYzhKS25YbGYxSVRjdFpVQ2M0dVc5MFJuUExNMTJIMVJTYmZGbkNLR1BPeVFYSF95NkNnWEEzamg3NmRuRkx0U2NjbXlxY015UWljTzRWbXpKclAwUg?oc=5</t>
         </is>
       </c>
-      <c r="E105" s="13" t="inlineStr">
+      <c r="E105" s="14" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3442,7 +3445,7 @@
       <c r="F105" s="3" t="inlineStr"/>
     </row>
     <row r="106">
-      <c r="A106" s="13" t="inlineStr">
+      <c r="A106" s="14" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -3452,17 +3455,17 @@
           <t>Banks rebuff work from home calls as Wesfarmers pauses business travel</t>
         </is>
       </c>
-      <c r="C106" s="13" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D106" s="13" t="inlineStr">
+      <c r="C106" s="14" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D106" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOTjFLNnZUNXZHeE85a3kyaG1IX29sWjFvZ2NzS041UnYxNkkwUF9YU3ZFYXhtQmlxY3Rmd0lUSTJrdTl1Y0ZobWp0M1lrZnZhZE9OSzV3Ql9Hb2UtUEpqWC1McjM0S2pESDJQVWJKQkw4enF5THJfeXFWRDZiMk5KMmVrazVUMzBNTk1tOXRVX1ZzVU1IUHBVSlhENEdEWFJpQnFXUGkyNVJGUnhzdXgyNW1WZXRkRmRaaVloZnpaMFdqVmk3elpFSkZ6ZmotZw?oc=5</t>
         </is>
       </c>
-      <c r="E106" s="13" t="inlineStr">
+      <c r="E106" s="14" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3470,7 +3473,7 @@
       <c r="F106" s="3" t="inlineStr"/>
     </row>
     <row r="107">
-      <c r="A107" s="13" t="inlineStr">
+      <c r="A107" s="14" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -3480,17 +3483,17 @@
           <t>This mine was fast-tracked to boost Australian solar. It’s exporting to China instead</t>
         </is>
       </c>
-      <c r="C107" s="13" t="inlineStr">
+      <c r="C107" s="14" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D107" s="13" t="inlineStr">
+      <c r="D107" s="14" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAJBVV95cUxPN1ZSdEMzSXBhMno2YzNkSFFtdlBOTTRGV3UtbnZtRktEd3Q0MHdmZHp0SDN5S0FZYmVKUllicHRMRkxTdmxtbkMtT2ZVN3hsUXdBVzAxdzhWcGFWRkxVdFY3NURqTVV2QVJQT0ZUT193R3JLLU9aZUw4YzlucjVUN0xyTzdoZlNjYXdyR2VWeDZrbW53cTJoRGZDd2kxbkxzMHBQWkRJMTFPMkNlX19wYjI2LVBZbnVJOVNsRjF3Tm0xUUFpY0ctczFZdWJFcHQyLUhwdDNiSGVtdHQzVVRtbExpcHJZak1SNkhWd2s4a0RtYWFNN2J2Q3FobTF1N0hWLXA4YUtaMXBScjZsUWt3alVVTVpJdVl0WDF5RTJLM1BKUl85dnhUUktkb2VwMzFkUWZ1ctIBugJBVV95cUxOOENIa2JzQzdxekNYTnJNVmRzdm9KTFpndnBybEJfNjBUR3VNMk92ZnhGY0JwVGZLeFRpdHJLMTQ0NjRNOFg5b3FESzhPLWlub2hSeFdidW0yS1h6ZXlGMjh3X3FhaWo1dHdneUZxS2NsaUJ6dWtfT1R6VndwSk52bVVNN2I5VlNYazBIelcwUkVBZHFlM0hiQVJ1a2NGWFpmR0c5R3Bna2RZMmJuSXB5WkQ1Zl94VDFtcjVEd2x6amIwSWdXUWtQVVo1Q0hpWVBLRVFycDAyU1NJV3N4YktlUlBtMTlkY2VNZjc1QVZhbnRrQ01OQnZqNzI5dTNNZ1VlNVVJcURycXlDRFZDYVo1aC15RXpwUFlvZWxlMHFybWJiM1YxT05lRElXYlZsbkJWUnI4VV9Da1lIUQ?oc=5</t>
         </is>
       </c>
-      <c r="E107" s="13" t="inlineStr">
+      <c r="E107" s="14" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3552,6 +3555,34 @@
         </is>
       </c>
       <c r="F109" s="3" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="15" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>The Right Amount to Pay for Sushi</t>
+        </is>
+      </c>
+      <c r="C110" s="15" t="inlineStr">
+        <is>
+          <t>Bloomberg</t>
+        </is>
+      </c>
+      <c r="D110" s="15" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOLUljQ1FWeHk0N21FcnpCTzdNVW1WZmxfbDFucXRNYlBMSzR6aTh4WlNrdnFuT1VSWWpKWlJValZrbTE5RlllanJkcHNHeEVwVkxldnZSdjdLc2c1SHJTVG1hMHBKd2xtZXptV1FmcGZ0cXUwVXFMWjJiRFhhYTlKRkNBNHZQekVRcnRicXlNM2NQdXJaZkVRbTZta0hDRlV5YVN5NG9TYzltUFZucXNXc29Wc1Y?oc=5</t>
+        </is>
+      </c>
+      <c r="E110" s="15" t="inlineStr">
+        <is>
+          <t>Retail &amp; Consumer</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>

</xml_diff>

<commit_message>
Update news log — 2026-03-29
</commit_message>
<xml_diff>
--- a/news_log.xlsx
+++ b/news_log.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -87,6 +87,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -489,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F110"/>
+  <dimension ref="A1:F112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -533,7 +536,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -543,17 +546,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -561,7 +564,7 @@
       <c r="F2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -571,17 +574,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -589,7 +592,7 @@
       <c r="F3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -599,17 +602,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -617,7 +620,7 @@
       <c r="F4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -627,17 +630,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -645,7 +648,7 @@
       <c r="F5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -655,17 +658,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -673,7 +676,7 @@
       <c r="F6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -683,17 +686,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -701,7 +704,7 @@
       <c r="F7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -711,17 +714,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="E8" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -729,7 +732,7 @@
       <c r="F8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -739,17 +742,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -757,7 +760,7 @@
       <c r="F9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -767,17 +770,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="E10" s="15" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -785,7 +788,7 @@
       <c r="F10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -795,17 +798,17 @@
           <t>Zarraffa’s Coffee celebrates 30 years, eyes nationwide growth</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOcXNzUkRLemZEOWtOZjhvRUtzcUZrSTdzV0s0LUJTd2NGRk1Gb1NSLUR5Rlh3NUdWQUJkVWctb0toUFBRajlMcWV3VnNyTUtydy1PSUoyb1NCOGVtMUZqRVN0MzFkVkNlOUZNVXlHN2kzREhSdWJQUnJqa0pnUzExTVZSc1NCVFZSNlBSUWNfWnZ3MC01aUx0UWF5SkNOaHI3ZkE?oc=5</t>
         </is>
       </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="E11" s="15" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -813,7 +816,7 @@
       <c r="F11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -823,17 +826,17 @@
           <t>Zarraffa’s Coffee eyes 200 outlets ahead of 2032 Olympics</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPMUFjRTlGVFBqYzlPWXdzQ0dKVVlhWGxncUQxTDd1R0VHcThlV3ExVmo4SlBGSHVuUGZrMGNqSVo1YVpDWHViMm5KZWIxcHNMMHo0b1FQcmxUNElDR2lEeWRuLWZIN2lyQUV0VndEUWNkNU42Z3AzNXRlbm50NzhtTXZ0Q245dF9hNzBxOENuMXZsVlU4Z0JGVElR?oc=5</t>
         </is>
       </c>
-      <c r="E12" s="14" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -841,7 +844,7 @@
       <c r="F12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -851,17 +854,17 @@
           <t>Aware Super appoints new head of private equity</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNVHJXNWEtdEZZUW1fZzdYMTB4RklBTUh6dUNKQ3BrTlpYUnBwRURIVGZjWTV0OUxScnhGMVNSczhLUjVqOEwzbkR2WWlEbmF4ZkNUdHNQY0J1djI0REctbHd2SVhUNlNCa2M5bFhOQ0JPU0RHOVVTQkEzRDdGMjRZbVFDOUdlTXNNczlmZWF6bXlfbEFGRE0xbkZQaw?oc=5</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="E13" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -869,7 +872,7 @@
       <c r="F13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -879,17 +882,17 @@
           <t>Commission wrinkle over UP Education sale</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxNSV9GMjhqM2ZSanI2X0w2OVlQVFRQTUoxYzAxaXVZMmU1REVTcHlUeEltdXJtaXZrcUJWdDZxNGpYTTZYSFE2TkZHeG9OaVRZakoxV0s1U01TVjJpWlhaSENfNVhucG5NVzFMbTVBY25zWGRSODBtRGtkS1owVTlJWnNfcTJ5alFnbVl1SU9aUDF1QWxJLTBSQ3kxUUFlZnpJMlVEQndFSGRGbDF6WVBUVHlCcDM5Qnh3R2xBMG9xN2FLckNzbUFOWDI1aVF1YV90d0twd0ZmMnUySDBMdG1R0gHkAUFVX3lxTE5EWVp6VzZWb01TRmlHSS0wMExldkJwSHJjdlZXdElsRlpBTEtVMkd6VzNQa1RpVDNsOFQzaGZ2VHpzUnBDYk82RmZGQWJuTmVQMXhxLXVmdVFxTVZOZTBsOHZ0V3cyVVVkNWUwVUxSc0xNSU92ZktpdFRfYnQ4WHBTX3A5bFhXZ1YwZXNrc1BSZEU4LVYybnNBd0dCdk92OFUwclJCMzdoU0ctX1pEdTAwY0JiTWQ4S01QRE00TW5EUEJwR2YtczZ0T005bTJnN1RDY2p6NFF1SndfLUo4QzJUWk1tRg?oc=5</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E14" s="15" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -897,7 +900,7 @@
       <c r="F14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -907,17 +910,17 @@
           <t>Gloria Jean’s owner has an angry shareholder on its case</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPTnZwUVBCdTFJZWkwc0YtVmJqMkNPcUR5RktjMlVURmhROFZkYUpXM01iRUh3SnJEUElxRGlSNk9DQjZSdTdNdmZwWWpONjlmR1hoMl92cUNmd3M4cnJhVkNqc095MmN6WXBYUmdEblB0eERtVDdlUU4yNGFjXzVnT19rOERIRzVPNzY3VDNNRS1tVGVTX3pKMVRpTXZVR1ROLURBLWtJbVZhY0lSU09DNkE2NzFLbEFU?oc=5</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E15" s="15" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -925,7 +928,7 @@
       <c r="F15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -935,17 +938,17 @@
           <t>Oporto-owner Craveable Brands hires new CEO from Domino’s</t>
         </is>
       </c>
-      <c r="C16" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="inlineStr">
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNNmxfQVc2Umc4QWwzSTdsZTFvejRzTzZxXy1ScGlhXzh6bm5JS3IyX0xTNDVBNjh0cXpPbGhxNU5xUHhQN3EtRF9aV3FEc2JoSG5QTU1WeU1TLUJfZzVUT2N6dXloQXhZaHB5djB3dDFKN1llVmI3UVpKNjJTNlcyV0ZDcG9GdVdSdW41ZkN1b1N3SFFIUzcwRkQ3UHY2TmxERmZwTlA0RzU?oc=5</t>
         </is>
       </c>
-      <c r="E16" s="14" t="inlineStr">
+      <c r="E16" s="15" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -953,7 +956,7 @@
       <c r="F16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -963,17 +966,17 @@
           <t>Brookfield, BGH Capital rub shoulders in ScotPac’s data room</t>
         </is>
       </c>
-      <c r="C17" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPMVlxbzlQNnFXWnJFNU11Y1BhTTVqbjN4RG1nbkZuN0pkdDFFaUhJN0RaVnUtWDlZSGJWR1ozQXk5UUx6RVdOcjBPU2t5UzN4T0JvUFJISnNvVWxQemd3blNHZjRQVVVZQk1nZER0Y0JfY3VvQ0t1a09sM1RTS2c1YTJyUmdzYWh1WGRUNjl2dkdzYTJJeHVhMTdqR3Y5WVlHVEtSZHp1cmVYYmM?oc=5</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="E17" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -981,7 +984,7 @@
       <c r="F17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -991,17 +994,17 @@
           <t>Payments player Pay.com.au hits the road(show) for $850m IPO</t>
         </is>
       </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOMFZleXZrbU53TzBlakI2ZmJKTjlrN3BoQlRaWjQ5cXFzTllKWmFoRm1UT2xDUHBtNC1QNTNiX1BwSzllMkRZdHIzRlAteDREaUczN1JTNTByTW1jNnR3d2NnR0RxUDBxeHYyWU1CSUs5MEZad2JqSGF6ZUxHZUNtZmFQaTJZZVJVZ1B4MkZ6V09QMWIxaUNHQmVzTDhvWVA1Ty1UbHgtQnRrQQ?oc=5</t>
         </is>
       </c>
-      <c r="E18" s="14" t="inlineStr">
+      <c r="E18" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1009,7 +1012,7 @@
       <c r="F18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1019,17 +1022,17 @@
           <t>Another year, another IPO cold shower for investors</t>
         </is>
       </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNeEhzYzQzdjR5MDJCWkd6Q2VLdEZzbzRoWnNOcXFlQjNfMlV4Q0NQRjExMlNhT2NPcnRBbW1sZUkteXo4N0dGaHNNeGZJOEZ2aXFvdmZiN2V2QzdOMzFteFRnY1RVRm1rQXltWmY5VFZOdFVNNVpudVp1dTlrcFM5b1k5SmlWQllDMVFXSjA4ZVpSZHgtV2JpWDJ4SkFRbVE?oc=5</t>
         </is>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E19" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1037,7 +1040,7 @@
       <c r="F19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1047,17 +1050,17 @@
           <t>Priceline Pharmacy franchisee sale narrows to final four bidders</t>
         </is>
       </c>
-      <c r="C20" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNR294am9sYWNiQ3FVT1B6YlV5ejMyeHAyT0FibTFVbU5pcjZyaVRyazEzbFkxd0lrcnpZNGpTYUx4Ykl1Xy1sZF93M2Nid19ydUFwbUJ3ZHozaURaNkRoOE9OMnRBRGZfQVdCVWZCaVhhNnZSRjlwYUdDVnp2WU9HUkJxbE1QMV8zdWxYRTNBQWktR0xSOFU4dmtXZWk0am9SSU92NWp6QUZmTVU5TzJEOEJNak5fQUtN?oc=5</t>
         </is>
       </c>
-      <c r="E20" s="14" t="inlineStr">
+      <c r="E20" s="15" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1065,7 +1068,7 @@
       <c r="F20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1075,17 +1078,17 @@
           <t>Private equity gets better image of Qscan</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="C21" s="15" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="D21" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxPRjVmT0hDRjZLblB1VHdPRmRGeXhKdDJHdWxDTzV4RDZ0VzdHaUFfOVlnZjRQMWhKcWMxby1oRDR6N2lQZkI1UDE1REppS3c4LTVmU3p5b2wtblRCWnhNajFnZGNHaGRJUHFMUGRtTHAyQmIxOHhNNTgwRWVSeWp6ZWRxbUY0WVhiUnhMRUpDLXNwS1RuelJldTk0Z1R0WHg0XzNXNTA5Rk5TRFZhU1RNVnN2TlZuaFE4OWtIYXQ5a2VGSW1UWmt5Rlc4Q2lIXzF3YlkwNVhfUzJDV0dQdVAxa2RKc08wRGR6TlB2Vi14QV9BdlhyaTZsM2pEVGZycTjSAYQCQVVfeXFMTWpnb0lWQmZ6MTFnRGhWNTNqczk1TWhTcUFEMVpDNnJ4ZWVxVlRUODhJXy03NHdGZVJlMmhyUHM0Nlh4NlZtTzRhQ0xxRDFLVHNzUVNfbWxhS3BLUEQteEMzZHRrc0F1eFRzYmxVNDZlSURyZDB5bF9wQTNRRU5yZEs1Z3pFRTdwcFBaMkNlN0JvT1NEYkFWVUJNcHJqcEM5RVJYa0JFUVl6cThyQXloaERzQjhkTUVPakJqb0hzNVlwSWxNS0dmZkNFSG9Gb3dNUnVvUnV0d3MxSmpzdFZKTHJ2RTQwRUoyMEVLLWMwT1NnOHdXVl9lRXNDWEFndzJFSDlZU0o?oc=5</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E21" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1093,7 +1096,7 @@
       <c r="F21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1103,17 +1106,17 @@
           <t>Oporto CEO’s first year reshapes brand and network strategy</t>
         </is>
       </c>
-      <c r="C22" s="14" t="inlineStr">
+      <c r="C22" s="15" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr">
+      <c r="D22" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPY25mNTJfT3FiVlBPZE5CcVNkR1UzR2xWaUtJSmxhU3EwcEMzQi1ISDFSajlCQWk1UUJpZVJ1Q19ZV3Jjd0Noc0l3OExpMXhSQUVVdHhCLTBlOXNoZzA3UXZBdkR1VHBvMmVsZkNhUFJndm1DdGpnX2w0ZVViU2phZ1RmYXY1SlhwUnhKSUxBQVZZUXpqNHQxQmo0Rk1iV0g0OW9qUS16eWRSNW5FaW1yQQ?oc=5</t>
         </is>
       </c>
-      <c r="E22" s="14" t="inlineStr">
+      <c r="E22" s="15" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1121,7 +1124,7 @@
       <c r="F22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1131,17 +1134,17 @@
           <t>The Melbourne restaurant our reviewer grew to love</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOc3YxQTljcHJXVWtRX2ZGM2lpM2pILWNwSFg0MFJrNmNWX0ZxRG9nV0J5N19qRWh4U0hPXzNmVVZwWk9wT2kzaFNrTlV3NEQ1Q3JpaXVIYlBHb216Q3VYVWdSRXMwdDl0SmYzdnRlSDFUYVRmRGJyZVlRZDJKTHpJOUctYlF1RDZSYjloY0hfZy13QmFTLU9UNjkwTHc1bjlGcGxoZ0ZLVU1GWTctZkdLZU9zSGhEZEpKbXJnaWJfZjd2OWs3?oc=5</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E23" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1149,7 +1152,7 @@
       <c r="F23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1159,17 +1162,17 @@
           <t>Crescent Capital strikes Benson Radiology deal for close to $400m</t>
         </is>
       </c>
-      <c r="C24" s="14" t="inlineStr">
+      <c r="C24" s="15" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr">
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOLTNrWG1ZZlFoU3pDZ3E2SEgwMlhzQkdtQUYzaHZTZmYwU3ZhMnE0dlkza005VkZmZ09NMExlWDVncnBmYVVISXJ6X1ZjNHhpM2RnSlprY1dnbndJNUczcDVtNXNRY3pVNW12bm5rUVdqVmR4R0JlVHFuN0RwTlFkR2xrbFFpSl9jcm5oSjk3aFM1clBSVDhnbkhoWUREeUhsbVpvQW90d05xOTdfOV9nbW5POFdmelJkVlpsUlRuYl9odmRNVUV2S0pCMFBMTS0tcVhGVGFYU0h2d9IB3wFBVV95cUxPWEs4R2pxdThPbHJHb0dBT183SkRHTTlXNzdWazcxdkd1eGx2VlAyM2VVbEtEbWxTZ1R0TlBFRmRMZTFoalgxSmVVRUJFR0c0RFYzZVJFODg3dWxicU9pOHppeFhjaVp0WWlyTnUzV1dyZXdkMHBDVHI4LUVQdjc0cWpheU55NTlvdWdCZmVoODB0Mm5fbGNCTmQwLUhMZ0psQVpzb3BEUnJpSkRnOUM0c0VCdUp5N3g5MkhaM01vTHJ3NWd0ay02UXZUUG9nVkxicVc1Z0xjWGhjUDRDVjlN?oc=5</t>
         </is>
       </c>
-      <c r="E24" s="14" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1177,7 +1180,7 @@
       <c r="F24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="14" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1187,17 +1190,17 @@
           <t>Dual-listed giant Capstone Copper flirts with $600m-plus carve-out</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNcVh4blRkQnoyaG1TajhVV0lrOEJRaHdTZWtzUnJHaEdaSXNRWThGTHlVdGl4dGJ1cTMwZ2pLcVNzUXRYNlZzVzhvaXdkNGtVUG0wN0FrMHB0R1I2Ry1jcEgtSWUtajI0cTFMRTlfdzBuMWtrZmJOLVUtMkl5dW85dFp6dEhEOHhTNzdfOFNFSGtlT0MwQnRlY0VhcUZBNE9RYzhQcDdOQUFnYkgzd0V0N253SQ?oc=5</t>
         </is>
       </c>
-      <c r="E25" s="14" t="inlineStr">
+      <c r="E25" s="15" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1205,7 +1208,7 @@
       <c r="F25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="14" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1215,17 +1218,17 @@
           <t>Guzman y Gomez unveils a new menu under $4</t>
         </is>
       </c>
-      <c r="C26" s="14" t="inlineStr">
+      <c r="C26" s="15" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr">
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPMjRjRTV2a3BJc3AzdDNOQktoYjBvLVZSODVsc3lKQ3pET0lxUlpkc05NcVlKRlZITjVJbjkwLS1DUFJNMGJ1amJKTlp3S3VqMWJaU3YtUENEN01rUEJiV1FNZTRXYjcyV08zZzlxNDVOSlVOTlJDOGV3QzBQcUpKa2Zab1ItNlI3ajZVVTF3?oc=5</t>
         </is>
       </c>
-      <c r="E26" s="14" t="inlineStr">
+      <c r="E26" s="15" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1233,7 +1236,7 @@
       <c r="F26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="14" t="inlineStr">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1243,17 +1246,17 @@
           <t>Can Sydney’s burrito king conquer the $676b US fast food market?</t>
         </is>
       </c>
-      <c r="C27" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr">
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNM0ZFcUpLN1dUZWUyaE1LMnNZVGlEbkNNQUQ4Wmd6QVFlTy0wZDVHdnlja1gzMEZTbVpKU1Ftb3VKZ2pzajcyWU16NUtUTmR0TlZMOVhMRUNqZXZiX2d2NWY0YlJDOFhhYUE0SkhMRUprNndXak8tWGdERU90cmMxTkFjcFFVSTd5VlZ3NFVKOXN3M255MFhzZThmbi1VUGMyQ3E4d2pYcFlJckY3QlVBdVJJeF9qUQ?oc=5</t>
         </is>
       </c>
-      <c r="E27" s="14" t="inlineStr">
+      <c r="E27" s="15" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1261,7 +1264,7 @@
       <c r="F27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="14" t="inlineStr">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1271,17 +1274,17 @@
           <t>Drone maker Innovaero prepares for ASX float, taps Euroz Hartleys</t>
         </is>
       </c>
-      <c r="C28" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="inlineStr">
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNU3JrejNRZ1VBZVNVV29NMkFPVmRsWE4yMVZPcjk2aUNUTHFJUGFyQ1VnZEZiZlIzQW9VVzRNNDNRR01jcHo3X0tqZjB4bzhMTTI0Y3BwYUh6OGRUUGt2REIxV09oRnJoVWlVelZWaUlWUmlPQ3dJdi1TejcyaXB1Z0x1MEJRSlB3SGMwVGdXaXJJNm9TVllPOG5JZC1feEV3TVhTeExGeHR2RHFIWlVCOXh3?oc=5</t>
         </is>
       </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="E28" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1289,7 +1292,7 @@
       <c r="F28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="inlineStr">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1299,17 +1302,17 @@
           <t>Bain flaunts Estia 2.0 as IPO roadshow gets under way</t>
         </is>
       </c>
-      <c r="C29" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D29" s="14" t="inlineStr">
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNTEN1cGsxNDN2c1NqUzB6UmJ4TFl0NGZjZVN3U3oxMlVFWTF4WUZLQS13dUxMV0N2ek1XN2VURTNVWms1NjdXSm0waEdaTXQwdTdWY1MxZ1V3ZnpEcVJtczdOWGNNZ0RQNzRZLU1MTTgtRW5DZkctbXBGMmVXVXdPZW5pNThiRHEzWnB2eFZzTFZTb1ZkeW9LendkNDd0cXRid05ZSGZYbW9NZXdOLVZWODdZU3hVcTA?oc=5</t>
         </is>
       </c>
-      <c r="E29" s="14" t="inlineStr">
+      <c r="E29" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1317,7 +1320,7 @@
       <c r="F29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="14" t="inlineStr">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1327,17 +1330,17 @@
           <t>Carl’s Jr. Australia unveils nationwide freebies for Happiness Day</t>
         </is>
       </c>
-      <c r="C30" s="14" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D30" s="14" t="inlineStr">
+      <c r="D30" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNVWgwdjU1NDFWalBfMTFYX1dQOWNDbG1FVUdlcS1LTVlHZVRRTVBWTjhSMnpkTXRXNlFJdllGQUp5Mm5ObWpIazd1d0RJa3QtdFBZN1hOenBmVzBEU05wM0gtNUxPeWpsYkxyVnhWWFFOU2Y3R0tXcmNkeWhpWDh2eDZBdjNCMHhuc1lHYTZHblBPVkpfRXpKd051UWlNc1hm?oc=5</t>
         </is>
       </c>
-      <c r="E30" s="14" t="inlineStr">
+      <c r="E30" s="15" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1345,7 +1348,7 @@
       <c r="F30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="14" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1355,17 +1358,17 @@
           <t>BHP and Woodside appoint new CEOs in major mining shake-up</t>
         </is>
       </c>
-      <c r="C31" s="14" t="inlineStr">
+      <c r="C31" s="15" t="inlineStr">
         <is>
           <t>ABC News</t>
         </is>
       </c>
-      <c r="D31" s="14" t="inlineStr">
+      <c r="D31" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQbTg5VFJLbWJfcy1uV3ZReTJkTndzX01qZ2MxNWkzaWZRckNLZUR1Y1VsMVRNc2FySC13U0NzalFEb3k1R3BaUEhfcTV0N1M4Q1dpSlo0YXI0UFhrMGRab2RiYV9DQVNVX01ycFc5ZFZrZWZqc1VRZXoxLVEzSDJLclJLSWg5bzN3R1I0bG9lWjVDaHE4?oc=5</t>
         </is>
       </c>
-      <c r="E31" s="14" t="inlineStr">
+      <c r="E31" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1373,7 +1376,7 @@
       <c r="F31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="14" t="inlineStr">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1383,17 +1386,17 @@
           <t>Next Capital sells Enviropacific unit to French waste management giant</t>
         </is>
       </c>
-      <c r="C32" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D32" s="14" t="inlineStr">
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPR3lFbERLR2FtdmJUU3BDU2thZk00YmFHRFhXR2VBVXhQSURTeE5ONVJKczBwbzlFMnR5cmhxMnM0bzlJbWo4SXl1dHpqYWxxMUJBRjZHVUtab1RYZjZMTnpGc3FzMWQ2NjNEdGU3NTZwa0diM1lJS1haYllwTldLZlpZbXp0YzlxcDh0ekcwTy03dDdPcnk4b29HZVdqbHhZY2JPR2drM2puSVpjUzZkVjNpZUE4dVMwYlE?oc=5</t>
         </is>
       </c>
-      <c r="E32" s="14" t="inlineStr">
+      <c r="E32" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1401,7 +1404,7 @@
       <c r="F32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="14" t="inlineStr">
+      <c r="A33" s="15" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1411,17 +1414,17 @@
           <t>Future Fund private equity and real assets chiefs head for the door</t>
         </is>
       </c>
-      <c r="C33" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D33" s="14" t="inlineStr">
+      <c r="C33" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPUHNHRFhFMVdwVld6RFRZUFd3QWNOd1kzeS1QdnJxMERFSnE5LTdZcDhDYlVGcWZMeWxlR0FSRWF6YkZoQVZrZU9TQ1E4YTEydUJnOFE3enV5Rmk5UnF5VEdYZ1FMUWpKVjdjMlZZUGFsU0tKcV9Vbl8zcHp5aVF5Z2JMOUZocHJqRXNRaEp4Nm5CbDM1WkdIMHdQS2xqQnE2Tnh3?oc=5</t>
         </is>
       </c>
-      <c r="E33" s="14" t="inlineStr">
+      <c r="E33" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1429,7 +1432,7 @@
       <c r="F33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="14" t="inlineStr">
+      <c r="A34" s="15" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1439,17 +1442,17 @@
           <t>‘I actually started to die’: the new billionaire’s epiphany</t>
         </is>
       </c>
-      <c r="C34" s="14" t="inlineStr">
+      <c r="C34" s="15" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D34" s="14" t="inlineStr">
+      <c r="D34" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxPblkxbHVrdnVKY1pqQzNyWGNMZm9UYmY3dzlPaGQ4Yi1tc0U1akhrVWdIaXBpM05aZXRwTXE1eDBITlZpbDkwRXNrWjJ2YXBzX0VCY2JSLWhrVmpjSTE5eE5rLWgtc2pRZEdXbmhhWU1KeFExZDBGS2pjSkIwV0FGbndBZVAyQkg4WFRsengzSGYyZkFfQnJsQ18tUHJGNDd2T0pzZElPSVJTQkl2Rm5QTExJNHhmU2dHOHJGdTdzU08yNHRtd1R3Q0cyOF8taDktQTZvVXVBVjN1d0NHMmtFOHBWZXBFcUFWa1IyWGNDTDZUT3lQSXJHOVhxTFQ3b3RH0gGGAkFVX3lxTFBZQ3BFQWl5dEwwLW5yVWJuMU8zcXBPdE9pamRVSWVkbWNyVzgydGVOaDBROUN6RlBDbjdld05DVmZyb0R1eEN0UERubzZRU2NiMTQtVV9XNS1wYmlvZ1paM3RaOUlrTzJka0tXVVJEamFESGlSdXg2bDk1aUdhUVhBcXpnN01fX0Y0cTNvcm5DdEFFLVVERDFKTWxKZFR0UzAyblJqVHBua2JoYUdzeUNMb053ZVczWUFQU1AtVHV1d3lSSDFfZFh2cEkxSGw2MEdicEVsb2pLQ1RuQmdaRl9xNUROS3pKR2s2T2wxTTZ5bEwtTUNQNU04djFHTHlPbXVLSW9YSUE?oc=5</t>
         </is>
       </c>
-      <c r="E34" s="14" t="inlineStr">
+      <c r="E34" s="15" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1457,7 +1460,7 @@
       <c r="F34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="14" t="inlineStr">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1467,17 +1470,17 @@
           <t>Ironbark shuns private equity as it hunts for cash injection</t>
         </is>
       </c>
-      <c r="C35" s="14" t="inlineStr">
+      <c r="C35" s="15" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D35" s="14" t="inlineStr">
+      <c r="D35" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxQZWFaeVhldi00VkV5ZmEtS2tjcWdFWG55OGpCX3IyN25Rb3ZFV0ZKVm1aSE1WbThoYVY4ZEdfODVGX0RaUDV2Ul9HS1JQMDFCT05Fc2FaU0RINTMwbDRveWFsOFJSM2ZqTU9tVGxJSEl2ZmhhUHFHT3dqYkk5TUtvMUQySnZzTWw1MzFNWl9aVzhkSEZ4Q3YyWjRMUmpIdmJkdUVKWE54Nkt6bTd2dGFSUFoyNkgxTHh2TGVGak9ja0dFZ0xQM2g0S1lmQkZiWWtUcTVNdHhBdC1KeVRQcDA2dnpmeHRkWEnSAewBQVVfeXFMTWtYRDRSaHNULW1HanowRnpMdFF2VVMtZW1SV2ViZXlGaW02WlIwUzRZMGg5WDNrOUR4eDlGOEt5eGlqV0pfVDFhb0JEcS1faEJodWxyRnB3MkozOVJyT3NvM1I5MzdDcXNnUFNSdkRDamUzZTRQYlk0c1VIQUNMZ2ZzOWVCb2V2MC1aSTZLWkFkbW9GYk05b3RmN1htWENTeDh3SU1WYWJMcWx2eGUzZmwwVXF6czlnRGdXbE1vRElyVG0yM0ZzXzZ5TFh1YlRGNU9MQ1p3NnVZSFB0M0xBcGlueVZILXlVaXdqUkU?oc=5</t>
         </is>
       </c>
-      <c r="E35" s="14" t="inlineStr">
+      <c r="E35" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1485,7 +1488,7 @@
       <c r="F35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="14" t="inlineStr">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1495,17 +1498,17 @@
           <t>Minister leaps to fix food chain</t>
         </is>
       </c>
-      <c r="C36" s="14" t="inlineStr">
+      <c r="C36" s="15" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D36" s="14" t="inlineStr">
+      <c r="D36" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxOd2NqakVWRnQ4anFZNkl4Zy03MkloX08tUkktRTZqeEtQWFZJeVhkMUJIb0FxUjc2UjhCQ3MxbmNxczNxblJIZ09IeTBGNFM4Wkh4ZE1qNkhJMjIwU2RtX1JxcEV1Y0NjWXF6eHpVdTN4ZUlYMGIwcDJzMXZMTk94VzFlcjhpcVZVSTJFMjhsQjVGWEJQYTQ3aTFyNmNEZ1F1b3NGTWd5WnFJWmxXSTJ2NlRLcjJHNWkwaTZ2YVR6S0w5WVo1Vlg0VWdxcWZoa3VaTmcxY2NVcnR2bFRWNGNvZ1M2Tlg5NzlvVXZFZm9B0gHzAUFVX3lxTE1uNERoR3p2dXRIa0g0RXI2MWR6N0c5U3NGcjFDQVMtdEpyNDI2bk8yOS1qUnFOazdiODl0Ymo5R1pwRVJ0UFFVdzlhYjRDSUFCU0FRak4xcVVrTHphdTdxcHNIMnEyRVZud1FURmh5T0JLOHpRM3lFbDRuRnZMYmtaRnRFTXh3dkszTFhFUmZlRmoydnlEbW1fZTlmUzh4NXNyeTZTeUhOSktvclJVc0NTZTVYMkdJZEUyY2RmVC1kQ1hwVEloSEtVMEo5QnNTUXQyME5IN1BPd1NOS3oyR1JtMHBFVTZEbzhEQmdrWUk1ZnZVTQ?oc=5</t>
         </is>
       </c>
-      <c r="E36" s="14" t="inlineStr">
+      <c r="E36" s="15" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1513,7 +1516,7 @@
       <c r="F36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="14" t="inlineStr">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1523,17 +1526,17 @@
           <t>‘Brace for swings on every tweet’: Investors bamboozled by peace talks</t>
         </is>
       </c>
-      <c r="C37" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D37" s="14" t="inlineStr">
+      <c r="C37" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOczZHTWFmTW9FZ1ZwSnc5Z3ZacGpsVDQ3LWw1a1BFT0tjRkphek41MlhNOU84emYzZUVwNV9xM0hyc1FUR0NHck14Qnh6c2JvQks5ZE02ZTNLWDI0dy1STi1HbDFDWW9yMDhGQXVVVzdkMzFXcnNNMVZHVXFMUXUteGtsVGhPVmhLcVZPQzlhTWNoYVVRMHF0cFhybWxzek13Y3ZjcjlXWjZJM2VYbm0tTmk4NExLQzQzX1ZPMVlhcnJxQkZx?oc=5</t>
         </is>
       </c>
-      <c r="E37" s="14" t="inlineStr">
+      <c r="E37" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1541,7 +1544,7 @@
       <c r="F37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="14" t="inlineStr">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1551,17 +1554,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C38" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D38" s="14" t="inlineStr">
+      <c r="C38" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D38" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5</t>
         </is>
       </c>
-      <c r="E38" s="14" t="inlineStr">
+      <c r="E38" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1569,7 +1572,7 @@
       <c r="F38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="14" t="inlineStr">
+      <c r="A39" s="15" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1579,17 +1582,17 @@
           <t>Wirth’s Myer rescue mission is caught in the eye of the storm</t>
         </is>
       </c>
-      <c r="C39" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D39" s="14" t="inlineStr">
+      <c r="C39" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNTlQ4NDRnWE91VG1YNENpSTUxNnBjZkljOGdYaGV0aVB5dkVOaEJ6SjZ1bVA4NXE1S1hjV1NjcVhQTEVpWEVNV0UtbzhQTFZLOWxIenZiaF9QM3F6bmJYRy1lbXVMczZ3TnBHNy1aLUtVcnBDdkl4TE0zRGN4U0FwSjNPY1M5S3AtdUQ3UUNmR0x4MlU2YXRuUDJEUm01SmZWakx2UjFvY04zRHk4Smc?oc=5</t>
         </is>
       </c>
-      <c r="E39" s="14" t="inlineStr">
+      <c r="E39" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1597,7 +1600,7 @@
       <c r="F39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="14" t="inlineStr">
+      <c r="A40" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1607,17 +1610,17 @@
           <t>‘Darling, I’m not going anywhere’: The rise of at-home care</t>
         </is>
       </c>
-      <c r="C40" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D40" s="14" t="inlineStr">
+      <c r="C40" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQS2k0M2otaldpNVFXdHRTMVNtZVhyUDV4VTNIcE5FSnFRaHNubGNQQzBVbllnNTktNGhrZ1lndzV5V1FpUS01SklRaTZmZHJkRzVsQmlsdEVmenZ4U2x6U01NeXdIMktBUW94TUE3R3FoLUxVcVhsVFI0SjVQVUFaZldnd3prMWMyaVRWX2J4aUdfQ25KWHpaLUlqSnhvQmM2TTRRQldGbm8tclFYRDA0TVdnU2g3QQ?oc=5</t>
         </is>
       </c>
-      <c r="E40" s="14" t="inlineStr">
+      <c r="E40" s="15" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1625,7 +1628,7 @@
       <c r="F40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="14" t="inlineStr">
+      <c r="A41" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1635,17 +1638,17 @@
           <t>Iran targets Israel and Gulf states as Trump looks to calm markets</t>
         </is>
       </c>
-      <c r="C41" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D41" s="14" t="inlineStr">
+      <c r="C41" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPLXBITXU3WTRtc0NYdnhTZHFaUTBCSXdldTBuSHliTlY1dlJONW43Qkd6Nl9pNmY1eDhzaHZoX19xYjBxMXR5UEhkVUg2M2k1MmhuVEwyY0JxbnJyemxVYUZjbk5BbkN4ajhPbW9ZeDhlRDRYTW1hN3k2d084c2djMEJUZTV3NVdPbllKUmFlU2JsaDV3Zk9CVFF0VDFkV09JSloycWdOUlVrREptQTJfa25LUEx5djA2SjNMMFY0RjM?oc=5</t>
         </is>
       </c>
-      <c r="E41" s="14" t="inlineStr">
+      <c r="E41" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1653,7 +1656,7 @@
       <c r="F41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="14" t="inlineStr">
+      <c r="A42" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1663,17 +1666,17 @@
           <t>Meet Christian Louboutin, footwear’s most famous billionaire</t>
         </is>
       </c>
-      <c r="C42" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D42" s="14" t="inlineStr">
+      <c r="C42" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPcXdGd0tMckYxbjZ5TVJmQ0Q4NFl2RkhHMHdlZDZsdGZ6cVQ0cUpaLWJTNlVoc2ZOQmtXNlFTRnJVMnVDTGc1NFNZN2g1VnotQlNQbzhlM1BJV3ZwQktOcGtac3RwSHRLZkR0b2l0eGIyVVlYdHJrc2hpT0pJbDR3LURPTnowZk54LThObndtMVkwV2VWQkluNVlWY0p4QVJGbE1hSGMzOW8zdkJZOWdocEZQWFBhTllNR1ZBSEg1TWRXUWd3X0t6TVcyY05PM0pF?oc=5</t>
         </is>
       </c>
-      <c r="E42" s="14" t="inlineStr">
+      <c r="E42" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1681,7 +1684,7 @@
       <c r="F42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="14" t="inlineStr">
+      <c r="A43" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1691,17 +1694,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C43" s="14" t="inlineStr">
+      <c r="C43" s="15" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D43" s="14" t="inlineStr">
+      <c r="D43" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQbHdYM2pSM2xkdmZ3OHhQc2tVUmhzclJWaVJ0aEwtUkNBR0ZUd3p1emF1M21jbTF1ejlKSkdDMnotcVNjZE1CYUlKako3WXR4MTJhdWNlSXZMbTBYanlmTWFzRGFIandXRUQ3UjN6SEV1bThvZjN2bDY0eFdpaTdMODN6TGFTdE5rd05TUll3MmNfTDhkQldoNDIwVlpoSl85aVRwcTd5Ymh3TDl4enZhZ2p4OExGY1ZaOFNEWFBB?oc=5</t>
         </is>
       </c>
-      <c r="E43" s="14" t="inlineStr">
+      <c r="E43" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1709,7 +1712,7 @@
       <c r="F43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="14" t="inlineStr">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1719,17 +1722,17 @@
           <t>Sembcorp Picks Banks for $2 Billion Alinta Loan in Aussie Push</t>
         </is>
       </c>
-      <c r="C44" s="14" t="inlineStr">
+      <c r="C44" s="15" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D44" s="14" t="inlineStr">
+      <c r="D44" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOdS1aaXZjT2VnSDl2TDdzZ3NfRElDWXdUXzZQYjFQMEZJOGlpaE5CNGdQMlZ2UFVHbUtfOXF1ZVBReExrdF85M0RWLWlBY2Y5dlRtWVdXLWp0Y1VrRmF4UGQzVUhxaHA4UHd1SUdFV21QcVFITXFHRlhzekdSUS1PdHlYRjdUbUQydU8wSktKVHRJQ0NaWE9sU1l6YXhtSWtBd3RwTERacnV4VzB6YlFhUE1QcXNDVXVESFcyeWY3cGhHUkRJcDhrYUtpTEY2UQ?oc=5</t>
         </is>
       </c>
-      <c r="E44" s="14" t="inlineStr">
+      <c r="E44" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1737,7 +1740,7 @@
       <c r="F44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="14" t="inlineStr">
+      <c r="A45" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1747,17 +1750,17 @@
           <t>Navis targets June for $1bn-plus med-tech auction</t>
         </is>
       </c>
-      <c r="C45" s="14" t="inlineStr">
+      <c r="C45" s="15" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D45" s="14" t="inlineStr">
+      <c r="D45" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxPNHRXaU5tNUVkd2MtcTg5M0EyQllrM0owMkZobGxLaUJxYUN2MUg0ZkdKdzU2YmxfanR3QU53cHZzNDI1WXgzRUcxOE9EZlluNmtNRUUzTGJPRnpfVVVOeFM3bFRNQmp6VHFBdi1mTnU4UDBvOEpMaHZPNXFtdUIyTlhuRExIVElSeVRUMGxjU0k5VnVxaWFfd3htWngydlhuR2E5aTQ5VW1LS01ac05rMGZoVFdOZzVyTzFhUDVsYkNrc0VQZmhubERSaTNwelk3WEhYUjF5d2ptMktYeEhzOHpWazFQZXphd0xfUFdhbkVGMVR2Z1dtVtIB_gFBVV95cUxObEwzeHd6RmZtNUp2dXVVV0plOVQ4WlNqQXNJU0thd1BEWE8yWkxxVTZjTkpsVGxxWGxpQzN0OERZbk91ai1fZkdtc0JoM1h5NERLTVdDbVJ4Y2k4djdQcWlVcDF6NjMyVDQzZWMzUFZxWjVRWllMZHVSOF9jQ2U1REFfNUlhM2EwYloxb1MwSTJjODdWdlZwX2h2N0xiQWNhallHUTNPZEtLaXhsY3dBZy0xM1VITXhLUERXS1JxR0R3OUpBTVBPZ2dPZTRUTVpvbFBNMjFUSTJuWS1XLWdhUS11UTRzVTVqaEhfMDhqWHlTMlJGekU2QzJVcFdodw?oc=5</t>
         </is>
       </c>
-      <c r="E45" s="14" t="inlineStr">
+      <c r="E45" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1765,7 +1768,7 @@
       <c r="F45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="14" t="inlineStr">
+      <c r="A46" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1775,17 +1778,17 @@
           <t>ExxonMobil eyes New Zealand market exit</t>
         </is>
       </c>
-      <c r="C46" s="14" t="inlineStr">
+      <c r="C46" s="15" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D46" s="14" t="inlineStr">
+      <c r="D46" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxPanlvR1V1eVVpdmYxNVNGMnd6UjJFd0J6Zk9IU1lhOW1GbmVTcjY4QkJCYkl3Y3NOU25VRTBUekwtS3plV0NVdlZtOTZZRHJWZ0FVdDl3S05aMlFWeEZiYzdwYmQtVnJxZEw0NktHaFZMNlZkUC16empqRGxxMEhhZGwxRzVEek5FelB3aE9UWFhGQW42b21MRnJHUXV2ZGJYUXJIMnVFWGZsSnEwazNGNUdVcjVoekp0NEZCN1J3cTlaZldFa1pMUkJTbVZYeFljVkRqQmlZV1M2aXh0ZjI5dEI1NDB0UElPUERsbUljMlA3OHBnYmtJTXFWZWkyUdIBgwJBVV95cUxNWFBRQ05GUDdwTWJ2ZVFJUS00ZUh0QkpZQVNNcU9JYXRTN21sMS1VZTlOSTh2LVFuZHh6UVk2djlrdWFsd3MwcDFCNmhwUlVLTlpjVF8wSmt1YnBWRE9tNVpKQlk2YXJWdmwzZWlLX0xpaWxSMUpsX3ZjYXhmRmE2YlAtSFJGRG5pQnVmMnViQXlsVFV3OU1hZFVrY3ZITHQxcTR5UkZ5U1pReHVJMGZGM2FCZWliSFZQZmpVLThSdExWMW14OElodmVVSC05SUh1d1hBenJoY3BUZGxoM0NTbTExdERmM3pjZGd4VzgyV3BNOG11TElBQ3NsRGhtSEc3YzJz?oc=5</t>
         </is>
       </c>
-      <c r="E46" s="14" t="inlineStr">
+      <c r="E46" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1793,7 +1796,7 @@
       <c r="F46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="14" t="inlineStr">
+      <c r="A47" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1803,17 +1806,17 @@
           <t>PAC Capital’s Clayton Larcombe charged with assaulting wife</t>
         </is>
       </c>
-      <c r="C47" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D47" s="14" t="inlineStr">
+      <c r="C47" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOLXNDU2xjMWpyeEZwWGwtZkV0TjNSbGtWS3ZidUo3a0dvV1hrTnJiVXBXSkJNWlhXYXFHZkNTa3g4a1ZfMjRPM3BtWTZUNGg3S09kbGI2TTRGd0Jkc1A4WFAycjlpVC1URjFvNnBraWprRkhaT0VOWkh6N0xkUjNXNUw0dGx2N1JtTDVsREdtZDhraXVsSkxhR2ozamFUSGR5VHBBRm1Zcmx1c2RDaUIxQkVpeUpfWjFNeTRLWVRtYjluZ3ZncGZIMQ?oc=5</t>
         </is>
       </c>
-      <c r="E47" s="14" t="inlineStr">
+      <c r="E47" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1821,7 +1824,7 @@
       <c r="F47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="14" t="inlineStr">
+      <c r="A48" s="15" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1831,17 +1834,17 @@
           <t>China touts itself as ‘harbour of stability’ to global CEOs</t>
         </is>
       </c>
-      <c r="C48" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D48" s="14" t="inlineStr">
+      <c r="C48" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D48" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPUzBWeVk0elBOZ0l5QU44TUJvU0RvSmtPdmVyT2VuQTczaEdzbkktT25ZT2Y0Nzh0bVBhQW96TUhpWkdEOEJMVVk2UWxLOENKZGk3X2tQcDNsWGZtU0JkM2U0N3VfUWFBclhUSUZya0NwRTJOWmZJdWlhT3JtY1EtSkJ6TmlsV3dzOXpDaVFMNlBaa3RfRHBjc3Q0cjk0eVdPV2MwcjlHNA?oc=5</t>
         </is>
       </c>
-      <c r="E48" s="14" t="inlineStr">
+      <c r="E48" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1849,7 +1852,7 @@
       <c r="F48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="14" t="inlineStr">
+      <c r="A49" s="15" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1859,17 +1862,17 @@
           <t>Eyes on 3D Energi as oil and gas giant Conoco flexes buy-out rights</t>
         </is>
       </c>
-      <c r="C49" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D49" s="14" t="inlineStr">
+      <c r="C49" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D49" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWVU1QmhTUGFkYlpTQkw1WUFPTHhmbk5lbnE4T1haQUswSi1ITHlhVmhyM3ZYS3N4cVd6ZkwzdGdhT1lvM1JJek4yLXFpSWoxUnRtR2JRLTZWa2dlTDVTakE3b2xvazFWX0kzRHFZWVB4OUh0XzFFd3JVSVlfelpVa21qTldCVHdvcmJYcGNjZ1RrdElWS3Yzck9KYzRvbzloWkNqMnQ3dmtHbzNuc21ZSXNYeEFlZw?oc=5</t>
         </is>
       </c>
-      <c r="E49" s="14" t="inlineStr">
+      <c r="E49" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1877,7 +1880,7 @@
       <c r="F49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="14" t="inlineStr">
+      <c r="A50" s="15" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1887,17 +1890,17 @@
           <t>Blackstone tempted by $900m payday for Sydney’s JPMorgan tower</t>
         </is>
       </c>
-      <c r="C50" s="14" t="inlineStr">
+      <c r="C50" s="15" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D50" s="14" t="inlineStr">
+      <c r="D50" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxQNEZTZjY0S2YzcUxsb25RSDk2NHd1N1VOVlpMbi1JNGEzbUt5ajlYZFhvLWNBTkNQVXNuWERfTkl0Z2o4R1U0Zk5jVE1FTW5TTUJGZnNJc2NqMm1fT2dmYTVwRGU2TkZ0c3BjZVBGS29fWFJvZ2F0MWNLa0pYY0RNME5xYS1vOGZmMDVBcDBaLV9MWF9od0EwekFyb0ZCOEdkNTFaN3ZXckJwd25zS0FsdzU4OW1UODlueGNyZVBDSDZkeHQwelV5ZXVDVlcyUkhKWDZfVlRacEJHSElmNnhKSXk4ZHJHWHhPTEV5NGNkcmhyU0hjV3J4dVBXbnRGQdIBgwJBVV95cUxPME4ySFF5RWNrejVlWW1yeW56N244RGpyeVJUZEgyTjFNcE10YjVpMmJyeWsxTENzZFhPRlpsbl9pVXl0NGJvUlZFT216NE1KRFNwOHVZVXMzanNKNXFmWEdsMndsd1cza3NTTzUyUUZfaDEyWHJwZEtQbTdJRmkyU3A0RGh4QlAtT1lRVXk2SGoyaTI1NUpwVExYSkZJNmVFNjdXTDJTNURFOEh4Y1dnUDVGdjBpaDlWVWJtUHZiRDdGTmE5R1R6TDBwWFFnT2MwQ1lmT2w5bDF6eVU0R20tYnpnT3JCZlJod2s0UndyZTM5M2xLZC02a3E0NmJRdFV0Qkow?oc=5</t>
         </is>
       </c>
-      <c r="E50" s="14" t="inlineStr">
+      <c r="E50" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1905,7 +1908,7 @@
       <c r="F50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="14" t="inlineStr">
+      <c r="A51" s="15" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1915,17 +1918,17 @@
           <t>I-MED attracts mystery suitor as Permira weighs sale or IPO</t>
         </is>
       </c>
-      <c r="C51" s="14" t="inlineStr">
+      <c r="C51" s="15" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D51" s="14" t="inlineStr">
+      <c r="D51" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxNaGlwS3d5MGFMbEg2U2hnZUxMQmdqaWI4bS1lblNZOFhkSnRMcUotRkZMTjhFZkRUQWxUUDVtYml6TVAxUXkyZmx3SHRFb0gzVHRST2ZQUThKa25aWlhlcGprSU9tWktXZjZRaC12bFpkaVVWZHhIMERyeVNNWEswYTJ2ZHdnRFVRaFhod2U5N011TkQ0NG5MYVhoT3MwRUVZdVB2UVhKZExvdFIyXzNNUGt2SHJUanQxRkI3bXlLSlNJQTF4NXQ1YlZDaGVBM0EzNUhYQVp6NkFWRzU4bnRPWTgtXy1HVnB0ZlN0Uy1rY2FuWlNfN1U4WXVHQnRzVkNG0gGGAkFVX3lxTE1GaDJJdTJlOXFEZUtDTmdXMmsyLXlpaUxzQXpycHk4MTdHZng0dVczYWVwdWRzdFFCMlNLWkZpMm5Zd2RpN0Y0Zmo3Q1FOZFBZQlh5LVl6aVZ3X284UmpxM0pVRzZmMmpjaUdNWnJPZGV4V3lNai1CTllCcW5oUEVxaG0zejB5anc5YnJEZzZPT2d2QklCWjl2MjRBc25jUndqZkVadllKaUZScG12bEozT1NKUUJYR0pHTGtJZVc0ZHZLNHVSYlhzcTE0SkZmMXNlVGJ4YWJ1cThxcGlZTDMzRUMxLVM5VHh2OW5tRW1PT3VyRUhDbV8tRzUzVzRzVWZPZ2w1bnc?oc=5</t>
         </is>
       </c>
-      <c r="E51" s="14" t="inlineStr">
+      <c r="E51" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1933,7 +1936,7 @@
       <c r="F51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="14" t="inlineStr">
+      <c r="A52" s="15" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1943,17 +1946,17 @@
           <t>The stagflationary mix that has billionaire Solomon Lew worried</t>
         </is>
       </c>
-      <c r="C52" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D52" s="14" t="inlineStr">
+      <c r="C52" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D52" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPWTh3S05XQWpTQm03WjhBT1pWc2cyOFRMd2ZraHhPUHlDRW1tWkZvdkhQWHE0MHVMRUpaOFRoX0JsYWhJV21nVkpIM2RBSmlZRUtEbFAydzZfOTh1S05oNEZPOGgyZDJRMS1uLThWYWRVT3VEVGhtYkVLN3J2OWsyX0VVdTUteFBCOVNKZ28xUTRPTk1SUkMxZ1NJc1B6NXRrUEEzOG01YnZOYjk2cWlFZA?oc=5</t>
         </is>
       </c>
-      <c r="E52" s="14" t="inlineStr">
+      <c r="E52" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1961,7 +1964,7 @@
       <c r="F52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="14" t="inlineStr">
+      <c r="A53" s="15" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1971,17 +1974,17 @@
           <t>Oliver Curtis on Firmus: From prison barber to AI billionaire</t>
         </is>
       </c>
-      <c r="C53" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D53" s="14" t="inlineStr">
+      <c r="C53" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D53" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQek9VTlV1b2hVb2RoZ0Fya0REb3E3YlBCR2NYZldXcEh2VEY0LXg5bjd6RzlnZDI0OUJJd2cydTBwTm9tdHpiZ1lSMnhtcmJSYVRKbzJFMjdDaEJyZExSQVJVRDh1c00yMjFMaVlPdnRuV3VkTjNxdzFRbW1yeGltSF8tVXlJVXJzTEJXS2FTYkJTVkdKbmdPTTd6YzRtYV9nN0JzOVZNTzhUdUk?oc=5</t>
         </is>
       </c>
-      <c r="E53" s="14" t="inlineStr">
+      <c r="E53" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1989,7 +1992,7 @@
       <c r="F53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="14" t="inlineStr">
+      <c r="A54" s="15" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1999,17 +2002,17 @@
           <t>Three startups that raised $161 million this week</t>
         </is>
       </c>
-      <c r="C54" s="14" t="inlineStr">
+      <c r="C54" s="15" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D54" s="14" t="inlineStr">
+      <c r="D54" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNRGVZMF9DeGJjX29vN3B0blVoM3RKSlJJTllrMThKUDJNZzdPNFNnT2JyTElUOUYxMHlsUm9yM2dBQnZfaVNZblpqb3NzTXdHVlpQNkRqR3NBZHdzODdjN3RKMTZhSVRqUEM5d3JRc3F2OG9hWmZJdU5rakg4ck8wLXlMTnZSU0lNaERmQmswbkVGWW8?oc=5</t>
         </is>
       </c>
-      <c r="E54" s="14" t="inlineStr">
+      <c r="E54" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2017,7 +2020,7 @@
       <c r="F54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="14" t="inlineStr">
+      <c r="A55" s="15" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2027,17 +2030,17 @@
           <t>Iran eyes ‘plenty more’ vulnerable energy targets in costly war</t>
         </is>
       </c>
-      <c r="C55" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D55" s="14" t="inlineStr">
+      <c r="C55" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D55" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNLUN1MHlZaTNfVHhVX0RnTXp5QW83RmM4WVZkWW1PSnNaZF93VkY5ZF81anB3NDNmX0kyMkVSdkxNSURvSEh6enloWnRVcTlsR0JPTjVzNFR1YjRsSm52VnA1XzFFUlUtODJjYy15YWRRdWZZRkdjRXpCcEFSVURmV3VpSTFhTjVUb1d5bmw3NHNlT3VQZU9ieEYwM1J1TGEyZnlnWXNIWFJUMEtIOVZad0dxRWZBdw?oc=5</t>
         </is>
       </c>
-      <c r="E55" s="14" t="inlineStr">
+      <c r="E55" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2045,7 +2048,7 @@
       <c r="F55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="14" t="inlineStr">
+      <c r="A56" s="15" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2055,17 +2058,17 @@
           <t>Don’t take it personally: Bain Special Sits hits hurdle at Infinity</t>
         </is>
       </c>
-      <c r="C56" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D56" s="14" t="inlineStr">
+      <c r="C56" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D56" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQRjdwTk0xTHVIRHNkdG9tVk1EQ0hiQjJ6dGcxaWZRZ0hZV1U4YjJDU0tnTUlWSkQ1S2dUTHJVNk0tNWQ2cVd4dkw0M25leXRreWJtdlBKYTAtNzRocTJUazh1dnRzSVlYZThySTBNVjg5X0xYWUxCMC1SelltSHVSUEV5U3B1bTA2NjAzMGFZLW1CNkQ3aWU0S1JxS0d0YmZiZjBKQVRNVUpzYno5R1pvbTBsaTM?oc=5</t>
         </is>
       </c>
-      <c r="E56" s="14" t="inlineStr">
+      <c r="E56" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2073,7 +2076,7 @@
       <c r="F56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="14" t="inlineStr">
+      <c r="A57" s="15" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2083,17 +2086,17 @@
           <t>Drill, baby, drill: It’s boom time for mineral and petroleum explorers</t>
         </is>
       </c>
-      <c r="C57" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D57" s="14" t="inlineStr">
+      <c r="C57" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D57" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNdlFOWld5ZWhPVnFRa2xidWlUVzluQzkxUTgxR0t0Rmg2S1BzNjdINnhwS3VLRkNjRVJLX0RHU0h4VFVRY2RfSHBudEhfNVNjeE50ZUxQenJNSlJtWFRlcnNsZm1iLXlxM2RmVDViWEtjNDloaTBhUDVxYkNfOWFCTjV6cExEVlFCMzNfWnVwRDJHYWxWV0hOR2V2S0VlV2NyS2s5cWNmREtWXzlMMDRQNW1tVlBOblp3SHBEVg?oc=5</t>
         </is>
       </c>
-      <c r="E57" s="14" t="inlineStr">
+      <c r="E57" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2101,7 +2104,7 @@
       <c r="F57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="14" t="inlineStr">
+      <c r="A58" s="15" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2111,17 +2114,17 @@
           <t>‘Wake up’: Fury as farming crisis looms</t>
         </is>
       </c>
-      <c r="C58" s="14" t="inlineStr">
+      <c r="C58" s="15" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D58" s="14" t="inlineStr">
+      <c r="D58" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNelJvMXFPX3MwUVRMN2xqbzE1MWdvOF92Zy02YmIyZW9SQXRNQVZsS0xVVG9UdkFPaTV6ZC1tV05SZWNqblNFZ3Y1VGNaVVBaaEl6aFJqQ09ONDVkNUs4TzNvVjV5eHNjUk9xaDRFZTM0alpuYUdvWGtLRzRhYXN5alZ1QWdsZTEyODdQVnZoazkya29WeTJZVmpxLVBCdWxfY0dTN2Z3WFZlSy1sVW44RDlvZFAzYlhnQ0N6UWhKSU02eF9iZllIU3g5MWtSbkJzZGxWLUxHNERzdUlLTF9VYmpJSTRLY3U4NlVVaDhmc09uOWwtUGtlb0I2M05DR1dnRWxGSFV2NEJXaEF4c00tN9IBlgJBVV95cUxOSzZ5NXZMTTlZa3BSNjZyTUxUMjRhYWJhN0hMa3dDcW9CWGstNnI5MzV5U0hJSTdKLTFwa2E5YUItZnFRbW5RbzVuYW91MmZaYXN3R25hWVpUbW9oUU9fVktPRHROVDYyd2dSLXJVZWQtY016bkVxY0VPbkY3Zkgtb1liWGMxeEpyYmloS1V0TVJMMWZaeWRZX3FQRjBmVzJwdkkwMEVDSXV1MTdReUhGZ0Z3dENyMEFkLUl1aXhtRkFLRFFXcEdMZzFuT3NxRDFMOGVaY2YzeXBQc09fY3YwcFp4MVczRVN3d3dJZWJfTFFscjF0cUtRWHdzTUptaHowNDhYWXZXTHhYTHNTdlZGUmNlamRTdw?oc=5</t>
         </is>
       </c>
-      <c r="E58" s="14" t="inlineStr">
+      <c r="E58" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2129,7 +2132,7 @@
       <c r="F58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="14" t="inlineStr">
+      <c r="A59" s="15" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2139,17 +2142,17 @@
           <t>Construction giant FDC road tests IPO pitch</t>
         </is>
       </c>
-      <c r="C59" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D59" s="14" t="inlineStr">
+      <c r="C59" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D59" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxON3p5Y3VPM01XZFk4a3g0R3JnQkZXbHVGV3BKdDB6M3NRb0M0SEl3V0R5RmhCQ3dnaHB0ZHp5N2hCMUFsNU1ZNWZ4YWdNZWdETkUyZmdoeW81amwtTWNFZlc5WlNpMkJwRzk0QklORGhlLWNEalh2d0JCX0lhVHhhUF9ibVlxcHAwOW9ENndVOTY0enBYUWc?oc=5</t>
         </is>
       </c>
-      <c r="E59" s="14" t="inlineStr">
+      <c r="E59" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2157,7 +2160,7 @@
       <c r="F59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="14" t="inlineStr">
+      <c r="A60" s="15" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2167,17 +2170,17 @@
           <t>Austal suitor Arlington Capital Partners buys Eptec’s defence unit</t>
         </is>
       </c>
-      <c r="C60" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D60" s="14" t="inlineStr">
+      <c r="C60" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D60" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNM01qb1ZRZVBIdmp3cFc3R3RLaTdmZk1JOFo4anRtSm95Z1hJc0N0S3VranBTV29IdlViT0FkSm92eHdtbDBqdU5HTHNMaXo0dGRWMkpDdjk3LVRBVU1rZC1YejZJMkhyNmpZZFJodGoxWlB1dkRhYTJVRlljMlV0dUllQ3EtOHZkNFdSUWJLSW9Xemw1XzFzU2RHV1o0RTViOXp0bDZFQTZycWhpNElLU0FZQVI?oc=5</t>
         </is>
       </c>
-      <c r="E60" s="14" t="inlineStr">
+      <c r="E60" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2185,7 +2188,7 @@
       <c r="F60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="14" t="inlineStr">
+      <c r="A61" s="15" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2195,17 +2198,17 @@
           <t>Eyes on Tom Wallace as clock ticks on Adgemis pub deal</t>
         </is>
       </c>
-      <c r="C61" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D61" s="14" t="inlineStr">
+      <c r="C61" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D61" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxNSExQeDlENWlHb0prRnRldjZ5YWhKVUZ5eVdsYjZmbVRWRWQ0WnZXWkU3UHZJdElnQ21jMU9zNnhnc3JlNDczVGQ5Y0FGV2J3QUp3NXdZTXZMNm5tVC1vWDFtOFN3aS04QVJZb3FZV2VsUmJ2aVgwbUhTaFVGdHg0UjRyTXVVUnFhQmE5eFYwMGR6T1R2U3Q3WEdZclVKNWJiby1IRg?oc=5</t>
         </is>
       </c>
-      <c r="E61" s="14" t="inlineStr">
+      <c r="E61" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2213,7 +2216,7 @@
       <c r="F61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="14" t="inlineStr">
+      <c r="A62" s="15" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2223,17 +2226,17 @@
           <t>UBS names head of APAC leveraged capital markets</t>
         </is>
       </c>
-      <c r="C62" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D62" s="14" t="inlineStr">
+      <c r="C62" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D62" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNMm9WZ2ZKVFBvX2pYMk16VmY1WFZnZ2J5N0F2bHduTVM0Sjg4STVtTGFLQVdzeFloVHg3clRic0owTDMwYVpXdDVjdjFOWjQxdkdxdFY5MEY1Q1U2Q0R5dFBJWTNtUzgyd3RXcm9uM0hKdEZ3b3JjXzcwQ2VpRm5SS0hYT2gxSU9iVFRlR05Xd2EtM2JOQjBGUzlKdnE?oc=5</t>
         </is>
       </c>
-      <c r="E62" s="14" t="inlineStr">
+      <c r="E62" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2241,7 +2244,7 @@
       <c r="F62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="14" t="inlineStr">
+      <c r="A63" s="15" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2251,17 +2254,17 @@
           <t>BHP, Woodside rise after new CEOs named; Future Fund chiefs exit; Sandilands ‘doesn’t accept’ termination</t>
         </is>
       </c>
-      <c r="C63" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D63" s="14" t="inlineStr">
+      <c r="C63" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D63" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNUHhZeHNHemtiLW1IOHN1OTZXOGpsM0ZtUG1MVHRCT1hUT1k5S2lEOXlXRENWOXNlMEZadThQR18xSTJfTVlQM3BtX0ptX1J0bk80SzNLUVRtbkJITGgtb0lsSVdJTWt2S1E1WUlXdUdsbEV0V1RpNWlyRXBoc0dPVDl1OXRrSlM3SHlDazg2UlcxenVzNzlhQldhUGhfNE5IV2xrVmVBNzhhSE9qY042Z3pzMEVzd0VyVmZudXgxcTgwWGJXSWZKZ0FyNVhjcmhjTm5DYUVjLUdDRmxUQkZuTDFlUXVaV0ZoSWp5WHMyR3c?oc=5</t>
         </is>
       </c>
-      <c r="E63" s="14" t="inlineStr">
+      <c r="E63" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2269,7 +2272,7 @@
       <c r="F63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="14" t="inlineStr">
+      <c r="A64" s="15" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2279,17 +2282,17 @@
           <t>BHP’s new CEO will shift the Big Australian’s centre of gravity</t>
         </is>
       </c>
-      <c r="C64" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D64" s="14" t="inlineStr">
+      <c r="C64" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D64" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPQnZpWndNZzZvN1VsOHBmRDVLRHVTNkxLeDVDelpOMURjOTRDSDZfN2dPZlZqaW05WEZuZXMyRTJZeVZnV0poT2UxRkVfZ1RZSjdvUjVKblhoSU5Cd1plRTVNNTRaNWZmbm1yUGZkblVpYkctNzVRRkVQQm4zX1FtRG1KV2Y0djUtOURianJ3dElqeXBUMFp4aWFEWVFYelVjYTluSWpOM1FlbHpIaUxXdnBn?oc=5</t>
         </is>
       </c>
-      <c r="E64" s="14" t="inlineStr">
+      <c r="E64" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2297,7 +2300,7 @@
       <c r="F64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="14" t="inlineStr">
+      <c r="A65" s="15" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2307,17 +2310,17 @@
           <t>How philanthropy became the sandbox of succession</t>
         </is>
       </c>
-      <c r="C65" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D65" s="14" t="inlineStr">
+      <c r="C65" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D65" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxObnBPb2MzQ1RvSVVCbmNzYWFBMlFjU0dQRmpPakNfdkxtMWc1bFdVNXNlZmRKQnNlWEtUUDNSTHpTLVV4Skx0V2otbTZsTTdvT1VaUDhMZFZoMFFab1RoS2pCcno1WGlNQlY4eXQ0OFEtLXJTay1MUkFSSEJ2MVVScUpjUkhJOThISy1QbHIzTzFlWVhOc29fWWs0V19sQ25hRW9MSGhBVVNKWUp6dUo3NS1SWlk?oc=5</t>
         </is>
       </c>
-      <c r="E65" s="14" t="inlineStr">
+      <c r="E65" s="15" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2325,7 +2328,7 @@
       <c r="F65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="14" t="inlineStr">
+      <c r="A66" s="15" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2335,17 +2338,17 @@
           <t>Advanced Navigation raises $158 million Series C round with NRFC backing</t>
         </is>
       </c>
-      <c r="C66" s="14" t="inlineStr">
+      <c r="C66" s="15" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D66" s="14" t="inlineStr">
+      <c r="D66" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNTXhwVlVLUy1pWEpFdzFCazNTY0dkczd4WW9oeW14cUtTaDZRTGlVQXBPaHN4WTBkNW1zOGxvN0tVWl9JSFdVNXlQMzVxbk4zbDZFUjNOcUxSamNaSnFCckMzWEk1VlNoSHJHQ3VWdGltVWZCV0c0NmU4UlN6YU55Q0J2TkQtUzBzOW96UXRxem5Zb3M2SUljNURISlRkQmJD?oc=5</t>
         </is>
       </c>
-      <c r="E66" s="14" t="inlineStr">
+      <c r="E66" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2353,7 +2356,7 @@
       <c r="F66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="14" t="inlineStr">
+      <c r="A67" s="15" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2363,17 +2366,17 @@
           <t>Kal Somani-led consortium buys Rajasthan Royals for USD 1.63 billion</t>
         </is>
       </c>
-      <c r="C67" s="14" t="inlineStr">
+      <c r="C67" s="15" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D67" s="14" t="inlineStr">
+      <c r="D67" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOX3lmdG5aTmk4TEpBa3ROdWZ1aDJHUElBQXktVmlKaHFmTUhPX1QxX1dKLXZfaHRDQjBnWm9McTZjTjJtTWFETTRNMHgzN0tTTm1xY0JpMF84Q2lNaFQyZGVjaHN4bkVmcDN5Qy1ta3FtYnpMSVVyYm0ydWpTRUdZU1hoYXpaNkZUQzlPc1QycjZ6aG5QVHRqY213?oc=5</t>
         </is>
       </c>
-      <c r="E67" s="14" t="inlineStr">
+      <c r="E67" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2381,7 +2384,7 @@
       <c r="F67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="14" t="inlineStr">
+      <c r="A68" s="15" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2391,17 +2394,17 @@
           <t>KMD says Rip Curl demerger proposal delivers investors ‘no value’</t>
         </is>
       </c>
-      <c r="C68" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D68" s="14" t="inlineStr">
+      <c r="C68" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D68" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPTXhBdHByWE9EbllFdDA2OW1UTUZEMVJfV2xsNFdURFRKX2JrODJReVRuQlFoakpWbTBKcjhNLUVsNE9sdG5LUElLZlVrbFNERS1QZTN6bEZIWEhXZ1pTWG5GWEw3ZmNETTdDUDUzYzR5M0E3ZGVlTWpSUnVlVU56dDNFZUtZN3liZ1dKNzJhLWU1S0M1ZnlKd1JNWXlxSlkyU3pGS1lhS05hTUJPRkxucldabzFucGs?oc=5</t>
         </is>
       </c>
-      <c r="E68" s="14" t="inlineStr">
+      <c r="E68" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2409,7 +2412,7 @@
       <c r="F68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="14" t="inlineStr">
+      <c r="A69" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2419,17 +2422,17 @@
           <t>Ex-Macquarie banker drives mortgage broker roll-up Recludo towards IPO</t>
         </is>
       </c>
-      <c r="C69" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D69" s="14" t="inlineStr">
+      <c r="C69" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D69" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxNQms5X1F2aTNhOExDbW42TlZOLVJwVWxna1JYSW9vWF9Na1RZa1ViTFdZc0tCcXRZZkRudTlsTzNuZGgwSENyYi03Zjdfc0lZTXp0NmJRZnhzb2pWRXRIOUdJN2lQM2h3ZFFtTXlSWHVWOFBIaW1Na3FQMjBCck1nVlhUcmRkLW9LOHpKWXQwTm9LcWR5M2FfdjFiRW04TndoanR5NmJvMENGalNuUGNINy1Qc20xR1J4d21ncHNNSUZqa1BXNnI4STIxSUFkZXdU?oc=5</t>
         </is>
       </c>
-      <c r="E69" s="14" t="inlineStr">
+      <c r="E69" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2437,7 +2440,7 @@
       <c r="F69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="14" t="inlineStr">
+      <c r="A70" s="15" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2447,17 +2450,17 @@
           <t>Coles reviews truck fuel charges as crisis worsens</t>
         </is>
       </c>
-      <c r="C70" s="14" t="inlineStr">
+      <c r="C70" s="15" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D70" s="14" t="inlineStr">
+      <c r="D70" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxOSGpBM3RjLVJ3LVlmR1QydnY2dm50WlVxcG43ajRFZ25QS1hDNTBONU8tY3Z2TklzbUNla0ttZk1GZzFaLUZRakFjSUpUQWItQ0VqVTVwS1B0QS1ObVEzNzdRT1l6aU9pVm5jSlhna1N6QmFKT3k1RkhMZGNTVnVLcDVIcXZmRjdjLWRpYVlRQUVmcVRtM21BSjVhTGNaaThyZkhLS2NWdkNCSkZKTlloUVdtbzRnYjFKbllOZXhOd3lkcFZEYURwUFVNQzVnSWRyM1RlOGd2M1pMZXI3c0NIa0Y0MNIB6AFBVV95cUxNSjB3Z0hoTGxwOHJQQ09xb3BmRmhCYjBCc2E0OHA2elFDRE45UGpaTEVDc1Y2VnRvVmZQUzRHbng4QTMwNGZZNGpmaVlHRmV6bnhiZ0FReU50TnRiQ0NZMEtoM3dBZ0hXbFBZMVJQNXd4LVdXRDVyTDAxNS1zeVdvcFVvend2N3J5R2pLYmhxNVFfd19rUlRsNWNndlptMUVkcS1CaUN6UXRHVzByTU5BMW1TdktOZUJYck5xMEJucmR6czIySEMycDA5cmR1MXB0N25Xc0JDUG9zN29YWklVc1BUMzl3UVhn?oc=5</t>
         </is>
       </c>
-      <c r="E70" s="14" t="inlineStr">
+      <c r="E70" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2465,7 +2468,7 @@
       <c r="F70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="14" t="inlineStr">
+      <c r="A71" s="15" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2475,17 +2478,17 @@
           <t>Sam Arnaout’s Midas touch turns suburban pubs into pokie gold mines</t>
         </is>
       </c>
-      <c r="C71" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D71" s="14" t="inlineStr">
+      <c r="C71" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D71" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQV2xlTTdYOFpIMzNmVVRnMlJRbTdGTC1jelVCd1V3UjN5cHQ1VzhWZzhrNW1PNm1RX3FlZmU3UkRycjF4WDlQUzRMcVVYY1g3UTZqQ0hxRnl2Ti1IQ0owVmZjN3Jod1BFbmhPVUwxNjhsTGh6d0kzdU01N0hmempRZ044ZmZNUllnenhyc3djRGJOdEtrekx5UVFoaFFMWDdqMHMwdng1SFg4TzZHY1hQNFJNN3huZXpWYWFtQ0ZJakhkVFlQcl9SQlRfZkQ?oc=5</t>
         </is>
       </c>
-      <c r="E71" s="14" t="inlineStr">
+      <c r="E71" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2493,7 +2496,7 @@
       <c r="F71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="14" t="inlineStr">
+      <c r="A72" s="15" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2503,17 +2506,17 @@
           <t>Gentlemen at Melbourne’s exclusive The Australian Club sweat another election</t>
         </is>
       </c>
-      <c r="C72" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D72" s="14" t="inlineStr">
+      <c r="C72" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D72" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPcEwyU01BOXF4TzlmREhYbTFEWklxdWZqWmZybDVnOWtLQ2dTU2dNQ2t5M3BVT2stN08xYkFmazVkY29oT3RVc2xUZmZINFJURGtIRTg4RGsxOURBdWEybTUwU2NUODQ2eDNBbTdPT3QxeXRFNHlSc014T0g1aG4xZ1A0U0FWMTB1Wm1CSHlQU0ZJb3lMYkE?oc=5</t>
         </is>
       </c>
-      <c r="E72" s="14" t="inlineStr">
+      <c r="E72" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2521,7 +2524,7 @@
       <c r="F72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="14" t="inlineStr">
+      <c r="A73" s="15" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2531,17 +2534,17 @@
           <t>Inside Fortescue’s AI ‘hive’ that could save the mining giant billions</t>
         </is>
       </c>
-      <c r="C73" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D73" s="14" t="inlineStr">
+      <c r="C73" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D73" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOSVVCbGpzcVcxTGlZZ2dTUkxXdVVvVU1ONEtUS0t1R1VkWWRNeUF1UmlHbXd6clR3QVRuWGxrUGQwVG1OeUxZb2RqTzdYOEVGQ1N6eDFta3VOZDdHNThYbUEwWEVHZlZBVzNpZ1Foak1kLURZTWpJVzZLekczdzFrdHMtLVZwMUZnYmkxSVc0czFqWnFaSGZiT2pIVW5rdVZmdThreFlRZWVEU0xoa1VFOV9MTjE2UHFOcWhqUzVB?oc=5</t>
         </is>
       </c>
-      <c r="E73" s="14" t="inlineStr">
+      <c r="E73" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2549,7 +2552,7 @@
       <c r="F73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="14" t="inlineStr">
+      <c r="A74" s="15" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2559,17 +2562,17 @@
           <t>Tiny house maker Elsewhere Pods seeks cash after Bunnings debut</t>
         </is>
       </c>
-      <c r="C74" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D74" s="14" t="inlineStr">
+      <c r="C74" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D74" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM0ZpVnBTS21Ib25qa09CaU52Z29kZWhTU0FJLW5VR2JCLVFPTVlZTmpYX3lZVWdtMDVTYTJkWHlPUmhXa0Rua2ZXTTBWQU1VdmFrV21KOGlrdjJ3TTdxbGlvZVBUZUxUWE1uelpWMGxWWk04UndJTXVKQjBZUEtoX3lodmdpMWZKNUc1YTIxVFZLYkFKT1QwbS01WU01ZUZTTlczY2ZpLXlpTjNJTWpsUg?oc=5</t>
         </is>
       </c>
-      <c r="E74" s="14" t="inlineStr">
+      <c r="E74" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2577,7 +2580,7 @@
       <c r="F74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="14" t="inlineStr">
+      <c r="A75" s="15" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2587,17 +2590,17 @@
           <t>Chinese consortium emerges as dark horse in Made Group sale</t>
         </is>
       </c>
-      <c r="C75" s="14" t="inlineStr">
+      <c r="C75" s="15" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D75" s="14" t="inlineStr">
+      <c r="D75" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQYlpEY0hxNm5lalIxSTUzbDE4UEF5QTNpMTl4dWNPMkRrMU1yQnltZ25WcUkwOU13V2Y2RGItVW5QTXotSnBZRUJMdGJySGw0NVVxc3ZLZmVEcTlfU193Vkd5UVVuTFVYWFNtd185eGlVQW5RRElHdk5pMjhUR24wd1k0T0I3cW9qTG5Lcjg2bV9aNWsya0FYODRjeURyMW1EeHdYT05iZHZhLVFrUVNoV25idnZYZ2lpZEhta2JxOWFJb0M2SE9hbFF6NlVWYTM3QmF5anpWOEZackZiTDBfN2gtX1luQkxFOUxSSNIB8gFBVV95cUxOQklMYWl1ZkRqZGUwN0ppeXFubzZWNTNmeE5GY1BfcS13N2dFT096YW9JSndVX1EzTlBKdWZIemdKZnRIME9SQk5aT1M2WnRESjJxckFTaUdOSEd6eG9hRVBjdlhBbWQyWGpUS1kwQXJsdlpkLXJpXzJZX2xiUC1FSlNnNTFoVXQ4bF9JeUp3UGRWdUFOUVRrNUtsRzRxaUczb1p2LVVucFBNazhuZFNDaUZDR2ZQUVdObmVtTnBndGlkazZqeHVheVNzSE9RY3Bad0lrckxDSWY5QXBWS0hwVzZvSTZjaGEtNkNncW1RRE5uUQ?oc=5</t>
         </is>
       </c>
-      <c r="E75" s="14" t="inlineStr">
+      <c r="E75" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2605,7 +2608,7 @@
       <c r="F75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="14" t="inlineStr">
+      <c r="A76" s="15" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2615,17 +2618,17 @@
           <t>KMD faces uphill battle in capital raise as key shareholder baulks</t>
         </is>
       </c>
-      <c r="C76" s="14" t="inlineStr">
+      <c r="C76" s="15" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D76" s="14" t="inlineStr">
+      <c r="D76" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxOVTU0OGNfRURNcDdzYUtIcG8tR3N4OFFYalhKNWJBaUd6ZlQwNU5MZVZYbUZVSzB3WmdOOFdTZHlBOXBzSGdYUVV6eGt1UndHN296bENxZzNUM2NoaV93LXZaZFNNOXJ2YlA4RHNFS2FDb1ltNWpPWUdRR3VGMWoxaU5qYm9VSW9yUW5kS1NaN2RSc2YtcHZRSTB6aE9Zdkl3NG5nbVRzODRfQVYtelo5M3g4R2JEbnpraFpWbENOZzE2Qndla2t3MXRPWkU1dXg4NmZRME1jT3pOOHZOVlpTZGloNENUZllaSTFmWUV1Y2JLck02ZDhnTHJ5bUPSAYICQVVfeXFMUEFXR29tQjlTbTdMRVNDWUlGNFNOQjVhX0FiSkl0U2stbml5VHR4d1g3bDFqMUw2TzR1eHhYOU5ZUmJpZ2xBY2NzcmJRX3MwaEQ0YmpzMUFnV1BQNGxmcnlXUzVvbHpwNEo5dWFnZlduZ0Z2dGZGRFRKRTNCUzctZDNCd0FMNEkzTm84dmZOM2NKYk81RERsVnlZN1VZaXp5TW5QRVAzOHNXQTFWdVlKdGtFX0FmcU1EbElZSm52alBQeWx4VnlvOFRwNk1ia2lZYXlpemQ4cFdmckotMmMyRGE4ZXN0dThQYmxxUkpvMzAwRXBBcVJuRnp0QkZ3b2tqMWF3?oc=5</t>
         </is>
       </c>
-      <c r="E76" s="14" t="inlineStr">
+      <c r="E76" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2633,7 +2636,7 @@
       <c r="F76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="14" t="inlineStr">
+      <c r="A77" s="15" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2643,17 +2646,17 @@
           <t>AustralianSuper claims another listed M&amp;A kill with Pepper Money</t>
         </is>
       </c>
-      <c r="C77" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D77" s="14" t="inlineStr">
+      <c r="C77" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D77" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOY0RwcnpWZlhfOHA2MG13MkJUX1RDNF9wN2RxZGU2cEpzS1RKTjJDeUl0OERFOGhFRXJaSXNETEhHbW9PS0lua283RnFVbHJvTlRva0djQ2lRSGc2RENJYmt0OEsyYTRVSzFGeE9jWVhKMVRnd240WXVNTVdac2lOUGJSZlc4UVZ5RXo0OTlQbUd6NWRSek1HZG9fZGk2aDhDelhGVmk4YkRKeVV1M0VHZ2hZNmFVdXM?oc=5</t>
         </is>
       </c>
-      <c r="E77" s="14" t="inlineStr">
+      <c r="E77" s="15" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2661,7 +2664,7 @@
       <c r="F77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="14" t="inlineStr">
+      <c r="A78" s="15" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2671,17 +2674,17 @@
           <t>Apollo to Acquire Nippon Sheet Glass in $3.7 Billion Deal</t>
         </is>
       </c>
-      <c r="C78" s="14" t="inlineStr">
+      <c r="C78" s="15" t="inlineStr">
         <is>
           <t>Wall Street Journal</t>
         </is>
       </c>
-      <c r="D78" s="14" t="inlineStr">
+      <c r="D78" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOanpORVBremoyamJyZ2FqQWVOcDcxa2NpempBUmNYcktMLUl1Mzg5VDloWmlVbUdNUnplVk90WEUzXzJjNGxENk9LcGF0enVSdlFpWU9nd244YWNTS0ZHd1JTZEtlbjRQTmJUU0dzWmlDOVFhR1ZRSFJkNXN4a3FHdGozcUcwdHRseXpYMFREUzBNcXRmQ1VCN056SWlEa1l5VVE?oc=5</t>
         </is>
       </c>
-      <c r="E78" s="14" t="inlineStr">
+      <c r="E78" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2689,7 +2692,7 @@
       <c r="F78" s="3" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="14" t="inlineStr">
+      <c r="A79" s="15" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2699,17 +2702,17 @@
           <t>Estee Lauder in talks to combine with Jean Paul Gaultier owner Puig</t>
         </is>
       </c>
-      <c r="C79" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D79" s="14" t="inlineStr">
+      <c r="C79" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D79" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPSjN6QnFVbmdHWFoteURWaU5VaWZmRmpTT3QtYm1tZUFyNUZyLUdheGdfWlRBTlJyTlp4THIwVDA4U3BnWFNpT2FpZlZzX1lJSDV0MkRGVjYtNVc0b0lOQy1RSnFGTWhCTWE2ZFFPYlFQX05yaVlfZF9IUEN2ZWkzQ0VFMUxxdHF2ODNQY09xdWlqWEczSC1CZk5wYU9QQlAyaTMyelJnaVM0cmN4M0paNzlBdzM1RndoZE8yRHN4UnZqaXVhVmx5NFpqS3hmUHhUdlpF?oc=5</t>
         </is>
       </c>
-      <c r="E79" s="14" t="inlineStr">
+      <c r="E79" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2717,7 +2720,7 @@
       <c r="F79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="14" t="inlineStr">
+      <c r="A80" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2727,17 +2730,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C80" s="14" t="inlineStr">
+      <c r="C80" s="15" t="inlineStr">
         <is>
           <t>The Age</t>
         </is>
       </c>
-      <c r="D80" s="14" t="inlineStr">
+      <c r="D80" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPdUtyNWs5YmxJMXNsNWtaMi1WMm5SVHd6ci1ReURLajdYd1IzWGJMZmE2MzJsSzAxQWtSTm8xMUEwNTh4Vy1zTmFsWFBKTkJ0YXc3ZkcwOVk2a2VNRWVGUS0yQzZhSXlCWmpDYUx6RmpTTlNhS0xIQklyVFdIVXJRZTNPaVB4TG4yQ1R1ZWF2MWpmSG81TVRaRzdtMXpydWhBS2w0a3ZPZFI5MnFKOW5tN21oUDB3NkNtQmR4LVVBWW9BUQ?oc=5</t>
         </is>
       </c>
-      <c r="E80" s="14" t="inlineStr">
+      <c r="E80" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2745,7 +2748,7 @@
       <c r="F80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="14" t="inlineStr">
+      <c r="A81" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2755,17 +2758,17 @@
           <t>Australia’s new millionaire factory: Start-up to $1.6b in five years</t>
         </is>
       </c>
-      <c r="C81" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D81" s="14" t="inlineStr">
+      <c r="C81" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D81" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOVkl5N1NGWS1XWWZSc0pHXzE3MUNERmV5SUgyQ3o2MmJ3U3Y2YlNwUXNSTGlQenBwVFdnMWhoT2FrcDAwUHNVU0RQbjFHMjJiLU1TRC1nemdrX3hPTG93VWZUQUx3Wk9HT3lYd055Z2FtREFpOWRlYXFDb2hwV0cyWFMwaHpsLU0ta2VVQlpid1dlYks0ZHg5YTY3Ykt6Um5YaF9MR2tIRzd1Tk1IRnBrWVhxVjZNSUl1OE9iRlZzYmQ3QUVnZmhYVGxoOA?oc=5</t>
         </is>
       </c>
-      <c r="E81" s="14" t="inlineStr">
+      <c r="E81" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2773,7 +2776,7 @@
       <c r="F81" s="3" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="14" t="inlineStr">
+      <c r="A82" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2783,17 +2786,17 @@
           <t>Social Media Wrap: Genki Sushi Singapore's loyalty benefits; Dunkin Philippines launches new collectible; Burger King Malaysia unveils new Korean inspired burger</t>
         </is>
       </c>
-      <c r="C82" s="14" t="inlineStr">
+      <c r="C82" s="15" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D82" s="14" t="inlineStr">
+      <c r="D82" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxPbFR6eHVTRWZNcUw1TTBJdE1JTFpmbk5iWndKZnRoU3Fmc3cxcF80TnVhRERmY0poM09zTFpCaEVnMGo5aktxY0ExV1ZlZVpHYUtldXBoOUh6bm14SURHNmhnUE9tYnI5YlpXQ3pRZlp0Ni1wM2lYQmdxdjk4SDl0aFN0R1VBbGxpbFVzOHV0TFY3YjJZbDg4Vk1HMTBkQk5LRHd1ZEVpRnBsT1U0Nm1IbVFkZEUybmpabEhuLUNLOGhicUxXZG5UalRLOE5DSzcxRncyNjVRdk8zclhJNkVQcTRkQTZYSEdN?oc=5</t>
         </is>
       </c>
-      <c r="E82" s="14" t="inlineStr">
+      <c r="E82" s="15" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -2801,7 +2804,7 @@
       <c r="F82" s="3" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="14" t="inlineStr">
+      <c r="A83" s="15" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -2811,17 +2814,17 @@
           <t>Copyright ‘status quo’ not working in AI boom times, says Charlton</t>
         </is>
       </c>
-      <c r="C83" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D83" s="14" t="inlineStr">
+      <c r="C83" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D83" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNVVgwdEQ2YUt0eFo3THcxOXZHbUFYZ091VTFKZDZHX0szYWQ2dnZ1dkJma3VZcGk1LUM2SUtQSWhxMGpCUlFZVzdKNmdoSGEycm1oYlBUdEZ5R0ZlU2hrWHpFWXdSN1lCZnZzb3hZc2twVVlWdTNNVXhaR0Nza0FiaUNveXZWQWQ1ZE45MU1HbGNmWlU2aUdha2FyZllzNWdONEpsM2RrdGRFSFl2UlpJUnQ4WGpleGs?oc=5</t>
         </is>
       </c>
-      <c r="E83" s="14" t="inlineStr">
+      <c r="E83" s="15" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2829,7 +2832,7 @@
       <c r="F83" s="3" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="14" t="inlineStr">
+      <c r="A84" s="15" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -2839,17 +2842,17 @@
           <t>The unapologetically analogue 4WD for off-roaders with $120k to spare</t>
         </is>
       </c>
-      <c r="C84" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D84" s="14" t="inlineStr">
+      <c r="C84" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D84" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxPSFJ4ZnNLT3U1REp3MWI2WDFaQm5vZlp6QWN6c0hZamtYVU95WmpkUERwR1dwc0NQN1dEc0FNbHlaMTdLclVHb1JTc2VZNExENGYyUE9OR1BkQ244YXRVeWNwbkxia2VrckVqSy00WV9UNWlvZWJHOG9ibUthaTlpVmRBOGZjLWFzMU8yS2Q5Um05SWIzY2dKajhoMWFUcmFrbTMzai1CdVBNLWczTWRvbTBwSDRfUzNwOHhqQm5hTDdhM0xLWEpNQTRyRXZjU1FLdGhRMUxtOTg?oc=5</t>
         </is>
       </c>
-      <c r="E84" s="14" t="inlineStr">
+      <c r="E84" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2857,7 +2860,7 @@
       <c r="F84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="14" t="inlineStr">
+      <c r="A85" s="15" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2867,17 +2870,17 @@
           <t>Junk room to become jazz club with priceless Melbourne view</t>
         </is>
       </c>
-      <c r="C85" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D85" s="14" t="inlineStr">
+      <c r="C85" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D85" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQbHN4My1nOGtueVJQZWM0LXNjLTR3MmhuemRJMUEwN09FTUZhZk1lbV9MbnVWblgyUXFEMEl3LUtsOGVqdGUweFR0MXF0ZEo0XzNhWVRqb2pGRUdiNTlLc1dFcXFmdnctQU1wQkRSdHN0T3J6VGt3MU1iNENydGlsOEpsT0ttZmJVZ0FUZmFXSUd3alVzUTQxMzVmcEVXSlV2dWdQd3JsMUZ0d3ZZYlBHaGhKTm9rM01SUmdseE9hT1prbHZtMlhv?oc=5</t>
         </is>
       </c>
-      <c r="E85" s="14" t="inlineStr">
+      <c r="E85" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2885,7 +2888,7 @@
       <c r="F85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="14" t="inlineStr">
+      <c r="A86" s="15" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2895,17 +2898,17 @@
           <t>Zimmermann fashion label appoints new CEO Roberto Eggs to replace Chris Olliver</t>
         </is>
       </c>
-      <c r="C86" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D86" s="14" t="inlineStr">
+      <c r="C86" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D86" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM2M5QU1scVoyNHBmV2lwQ0VQS1Z6d2Qwa1ZkZ0M2WVIzdXR3QnZwVWhUSDRCUEdRZkc5QzFQSFFhNzZ4VE9lWXBTcGhpS01JdG12TlQxSHhValZfbWt3MUdFZGl3RlBtdnlrel83TjNjNFZ0SUpvSDNQbThpU3FLa3Atd0dNU04zQm9OSk5uNHpTVE84aWZpaVlKWkdOQjJjRTZSd1MwMEZ1b3pENkRCQQ?oc=5</t>
         </is>
       </c>
-      <c r="E86" s="14" t="inlineStr">
+      <c r="E86" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2913,7 +2916,7 @@
       <c r="F86" s="3" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="14" t="inlineStr">
+      <c r="A87" s="15" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2923,17 +2926,17 @@
           <t>Construction giant FDC road tests IPO pitch - AFR</t>
         </is>
       </c>
-      <c r="C87" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D87" s="14" t="inlineStr">
+      <c r="C87" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D87" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNTnRScHFhQlpkdEdSb2x1bExxQm96ZE5zSV9wTDNDV2pxYjFQdUtoYmNBell3SFlTTFEzMUhpeXlmNERSeDd6VGppM2szQ1NHVE9PY1R3MTN0SUZLWkF5em8tQ3IycUZ2RmswX0tnN1IwOHl1ZFo4UUtMUDlQbXRjTnRCWFB5cU1RZFhsdDdaWGpMZzh3d29CWWZvZGtnTjl0T1k5ZHFHSUg5XzFSSF9TSUxTYkU0QkFheFlLZUY3S2tCSWRLZWlBbUpxUjc3TXBQQ01V?oc=5</t>
         </is>
       </c>
-      <c r="E87" s="14" t="inlineStr">
+      <c r="E87" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2941,7 +2944,7 @@
       <c r="F87" s="3" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="14" t="inlineStr">
+      <c r="A88" s="15" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -2951,17 +2954,17 @@
           <t>David Jones is trying to defy retail gravity. It’s causing problems</t>
         </is>
       </c>
-      <c r="C88" s="14" t="inlineStr">
+      <c r="C88" s="15" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D88" s="14" t="inlineStr">
+      <c r="D88" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPZy14UldWZDRrSjI3R0lzdGlKamlkVnU1WWVjTWRUTlpya1ZpVW80WHlrT0FQTUUwMzkzM19xQWpwTnVLOF8zeTFXamhTZFRQVjl5TTlXbE1RRWY2NW03dlpmZ25qdkgyN1IwbDdjRlhxd1MzSGkxeG45M214OVlESWF5WWh5TjM0STQtOXdieWIyOUI2NzRsaDhiS0ROUU5YQ185aWtObUY2S0dOSTBROVlwSVB1VkNqTkZTTllkZmtMYmxjNVdlTA?oc=5</t>
         </is>
       </c>
-      <c r="E88" s="14" t="inlineStr">
+      <c r="E88" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2969,7 +2972,7 @@
       <c r="F88" s="3" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="14" t="inlineStr">
+      <c r="A89" s="15" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -2979,17 +2982,17 @@
           <t>Jefferies’ Australian ambitions in focus as Sumitomo circles</t>
         </is>
       </c>
-      <c r="C89" s="14" t="inlineStr">
+      <c r="C89" s="15" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D89" s="14" t="inlineStr">
+      <c r="D89" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxNUTd0LXFPQmZXSldrTmZHTkIwUWQ3MmlCUmFOUGRkcVVjRXV6YXZJUTcyMG5FV3I0dWY2NXh6MnduVjNxZmhJMHdDVGw5VzFxTEFzN2FBdlNvS1JGSDltQmlzVS1QRDdCeWdfSHZ2VlZDMlBnN1Y0d2JxbnlGejhWVjJpWGZLejdCTUt2Uk9ENmhyRkd4dDJjd0RlUnBlZXhOTmUtOG9ITE05VHJ3dTBRSWZneURuUW1NYkExVXpfWXlsMzZ1WUlyNE84SThQX1JJTFlXOHc4ZnB0aXRmdVhaaG1qSEJRZUhuU3RibHAzbHVNLWFLUF9NNTFoUXV3NGQzelcwcNIBigJBVV95cUxPMkhEeDJpNzg0NTlDZmF2LUFPSEs4cmZ5U2p6bWVZSTYwcXVUUGVIb0FLVnhZV0cta01CLVpfQzQzYzdvTWdxR0o4bGJDWDVBb1lnOGx0bWROdTdjcHhwLUpPMW9MQ0RVM2NUOUt6UGpTd05JYzhuVmgybGp2LVpORFF0SHpBTU5DUTJEUmZKUFBNajlQdHJ4WkdHVV9QMjVwOWVlNWliVkFaM20yWGZhOEc4bldHRERJak1BWXlmSE0zdno1VTVSc0FMck0wSE1BR1RVaVRMSEdzU2FvcWpMYmp5ZTVJTWcyUGdXanhqSUNZU0tzTkNYWVg2SXpVMEoyS184VkxOeWtSUQ?oc=5</t>
         </is>
       </c>
-      <c r="E89" s="14" t="inlineStr">
+      <c r="E89" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2997,7 +3000,7 @@
       <c r="F89" s="3" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="14" t="inlineStr">
+      <c r="A90" s="15" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3007,17 +3010,17 @@
           <t>Bain Gets Nearly $300 Million Loan for Australia Wealth Unit M&amp;A</t>
         </is>
       </c>
-      <c r="C90" s="14" t="inlineStr">
+      <c r="C90" s="15" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D90" s="14" t="inlineStr">
+      <c r="D90" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMUQ4WExYZFY1aFBwWENNR1JiVkw4OHFKWjY4NW4zQ3ZBalFiTU10Y2hic2p2VjFqOE1rMndNYmVoN0lPcnY0WmFOV1MtaEY5c2xvcW1PNGN2SzZVcThwc3ljWkYwV1Q4a2dIaUpBeXZpMkRUU3IxZzVBVkhydGU3OXEzNW1sdlVQeTRNRFY4bUJLOGpGYmJ0ZXpPc1YzY05TYWd2bF9oWVJ6Rks2dWlod1dGRU4?oc=5</t>
         </is>
       </c>
-      <c r="E90" s="14" t="inlineStr">
+      <c r="E90" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3025,7 +3028,7 @@
       <c r="F90" s="3" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="14" t="inlineStr">
+      <c r="A91" s="15" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3035,17 +3038,17 @@
           <t>Fund managers caught up in Aware, TelstraSuper $237b merger</t>
         </is>
       </c>
-      <c r="C91" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D91" s="14" t="inlineStr">
+      <c r="C91" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D91" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcFF4Q1A5X1VtNWFnYXZSVUlZX2JMRVoxaUJoeGhybmRrZkd4UlEzTURwMkx2d2I1Y1hMYmljbk05WUFzRl9JbF9JampqeDd2bXdYcUpHbVZYak1sYXFHS2VuUDJyTUhzSS1QTW15aVpfeHRuMGZHenlxOHJQRUdENkV0b2FMZXhOZWF1Yk5hR1lOYWFQc2Q0SEROUFNERXhKQUIzRkt6NTQ?oc=5</t>
         </is>
       </c>
-      <c r="E91" s="14" t="inlineStr">
+      <c r="E91" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3053,7 +3056,7 @@
       <c r="F91" s="3" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="14" t="inlineStr">
+      <c r="A92" s="15" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3063,17 +3066,17 @@
           <t>Soul Patts defies private credit jitters with 15pc returns</t>
         </is>
       </c>
-      <c r="C92" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D92" s="14" t="inlineStr">
+      <c r="C92" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D92" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPRkNINFJOai1NbUUtX3ZrcnJFS3EzRHZPbFRfVFE3SERudTVqbjIybWsyYUthOUJOUVFPb1U0UzlGTTRqbUxraFZfYlVtclQxeTBQU1M5YjJzMDVPU3RiX0cxbk8xOEd5YjV1R04zT0NNZjhNSi1meWo4RHM1ckFsUnNLd0JiQXFnZ0dtckNzdWxmanZoQUl3TEQ2a29nRkRDZ1lJd2Y5VGc2UWZHX0pkU1NObmRJTlZKS0E?oc=5</t>
         </is>
       </c>
-      <c r="E92" s="14" t="inlineStr">
+      <c r="E92" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3081,7 +3084,7 @@
       <c r="F92" s="3" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" s="14" t="inlineStr">
+      <c r="A93" s="15" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3091,17 +3094,17 @@
           <t>Ex-KKR China heads negotiate to buy Vitaco, owner of Musashi, Nutra-Life</t>
         </is>
       </c>
-      <c r="C93" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D93" s="14" t="inlineStr">
+      <c r="C93" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D93" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQRmlCdTlFeHdBUGkyOS1CeEFIYTRSREdZM1JOZ3IyZThnNmNMdm9QeXVwRWtMbzU0em1vcDAyM1hodDlvalVRdThtNVhLR2FsaE1vV0xuWjkwMkVCUDk5SmVka1BURFJZNkl2bURLeC1GdzI0V2hEaVhrNlJZejlvc2gwRmtnUjd1NDFlX2trbGk2aXJiQ2FrTWtmVVpiOXhBc05JSkNYY2xLX2JEQUpWY2dlY1pDZw?oc=5</t>
         </is>
       </c>
-      <c r="E93" s="14" t="inlineStr">
+      <c r="E93" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3109,7 +3112,7 @@
       <c r="F93" s="3" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="14" t="inlineStr">
+      <c r="A94" s="15" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3119,17 +3122,17 @@
           <t>Antipodes Global Investment Company</t>
         </is>
       </c>
-      <c r="C94" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D94" s="14" t="inlineStr">
+      <c r="C94" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D94" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE5mdkJzN19XLTFQc25LOUk0ZGJBMER6djB2VnFvbGVrS1hlemRBRmlNY2JmMGlPTzktU0RRS3NNUW8tRXhtUE1QdE1JLWdUNVhibmZPZi1MRkJOWk95NzM2bXplS3JzeG13UU5henhza1ozeGRZZmlBNTNR?oc=5</t>
         </is>
       </c>
-      <c r="E94" s="14" t="inlineStr">
+      <c r="E94" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3137,7 +3140,7 @@
       <c r="F94" s="3" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="14" t="inlineStr">
+      <c r="A95" s="15" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3147,17 +3150,17 @@
           <t>AusSuper to lift insurance premiums by up to 40pc</t>
         </is>
       </c>
-      <c r="C95" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D95" s="14" t="inlineStr">
+      <c r="C95" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D95" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQNEhYQkoyNnJFU2xBZG8wdXhEZWRSakRiWWNHOGZBTFhfaElxWkRsSWViaWxjenVjMF91cGdrbFZxSGJfbkR2SUZNdEJtYUVadlV6YVVrWU1VbVdsMWpyNUZ4bE13Mmo4cGQ3WWZlVFVrTTdyOGpSdkpUb0tkcjdQUFlsTnM0MnpOMDJNZlJ4YTlzZGpLS1QzMFluOFU2VUJya3lSclBLSnZkQ2Y0a2djNUpSYlo?oc=5</t>
         </is>
       </c>
-      <c r="E95" s="14" t="inlineStr">
+      <c r="E95" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3165,7 +3168,7 @@
       <c r="F95" s="3" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" s="14" t="inlineStr">
+      <c r="A96" s="15" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -3175,17 +3178,17 @@
           <t>Unions want inflation-plus minimum wage rise due to ‘Trump and RBA’</t>
         </is>
       </c>
-      <c r="C96" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D96" s="14" t="inlineStr">
+      <c r="C96" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D96" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNdzNhU0MzbFRFX2I3OVY4bFItd1h6OVE2Wnpqb01NM2tMYzNob21BeW02LTBfTFZIWnN6SG5DVnYxQTJGZWZaLTJpTXZGUnhmS3RPY3hQV01fd1RIYU9Ednc4a1hvalVRT19ESU5TX19sQjN4dVV3X29kQjliQjNFU19iaXFIS2l3blk5TWUwdHFrRmJtQ0JocDN0WEhWbXZOVUJzR3RaYnJPSHpIRFlYOVFObEtuT1d0TUo0MUVZTXdFZWR3WG1r?oc=5</t>
         </is>
       </c>
-      <c r="E96" s="14" t="inlineStr">
+      <c r="E96" s="15" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3193,7 +3196,7 @@
       <c r="F96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" s="14" t="inlineStr">
+      <c r="A97" s="15" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3203,17 +3206,17 @@
           <t>Firmus’ Oliver Curtis set for green light to run ASX-listed company</t>
         </is>
       </c>
-      <c r="C97" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D97" s="14" t="inlineStr">
+      <c r="C97" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D97" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNR3VmQW9vNmUyeU9WbVRvRG9tcTNMYVlvRUhCd29wTkRZaVlEcG50Z0hIN29XcE5GUmxkUy1yMm0yTm94Q1BXMmNCcXBpZDlqVTRlZFpMX1QyMWh5Ym5XQ3VjYW1ZdDFtYWNyOERCOURuWXM5ZTV4WGthMVVjNUZlcmVTQ3JBUjQzUXRXYXRLQjlNeHpBMkVCVWpsd2Z1Vk42TjJxSlRiQ0ZtaTkzOTZtNmRHQQ?oc=5</t>
         </is>
       </c>
-      <c r="E97" s="14" t="inlineStr">
+      <c r="E97" s="15" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3221,7 +3224,7 @@
       <c r="F97" s="3" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" s="14" t="inlineStr">
+      <c r="A98" s="15" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3231,17 +3234,17 @@
           <t>Crisis Hit David Jones Chasing Funding As Retail Markets Come Under Pressure</t>
         </is>
       </c>
-      <c r="C98" s="14" t="inlineStr">
+      <c r="C98" s="15" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D98" s="14" t="inlineStr">
+      <c r="D98" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNNjJSOUVQcTkwUmxXNXg4ZzljSGhnRlBJY0otSHRrX2ZIQXRqWmNDZlgxYW1jckhHd3BtdXJsUWhwTjQ5SGw2NUU3TnFtcmhYd2JVcThIR2VCLWJLU0h5RE8xaTV5TS03Mi1za19hcF9PcXRRSU9PX3ZxSktSV2FfY1ppcUFVV2w1TmF1UWVtZlBWSUhEcG9oRGlEVkEwR2ltQ2VMSTNlcENEYlY0?oc=5</t>
         </is>
       </c>
-      <c r="E98" s="14" t="inlineStr">
+      <c r="E98" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3249,7 +3252,7 @@
       <c r="F98" s="3" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" s="14" t="inlineStr">
+      <c r="A99" s="15" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3259,17 +3262,17 @@
           <t>Beirut Street Food eyes niche in Lebanese fast casual</t>
         </is>
       </c>
-      <c r="C99" s="14" t="inlineStr">
+      <c r="C99" s="15" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D99" s="14" t="inlineStr">
+      <c r="D99" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNVlZVeTNGcXVOSXV1eklvTnFxYk1hb1A2VTQtNHkwdUpvdFF0YnlYU2RSWkZNV2dGQkEyZjRVQzVJZ2Uwc3gtZ0F1TGlSQlVna01HRnZOTTJnVUFxaWtOam1vZ245Z05jdlRnQURqbnQxaGtEcnFYS20wWmtvSDV0MW15c18zUE5ZN2JJWUpLV0RsZE1LSm5fcUNNeVZNTmdMQ2c?oc=5</t>
         </is>
       </c>
-      <c r="E99" s="14" t="inlineStr">
+      <c r="E99" s="15" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3277,7 +3280,7 @@
       <c r="F99" s="3" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" s="14" t="inlineStr">
+      <c r="A100" s="15" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3287,17 +3290,17 @@
           <t>Gami Chicken credits chip design for cult following across Australia</t>
         </is>
       </c>
-      <c r="C100" s="14" t="inlineStr">
+      <c r="C100" s="15" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D100" s="14" t="inlineStr">
+      <c r="D100" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPTXg4T0dvQ1l4NFVxV25iUXQzY0F3MnFjYmE4X0NOcFdNZHgweUg4NmVZZjNJbTFMajNhNHBmVDE2MGNBZzhOTUJsaG5KejFZbk1Db0JyNTZJbUI2WnRZeVhXRFRMNXVBWVFMdGJ3WkN5dV85dEduQi1OVDhOSE9UOGVERXh3T2hCVmlDNVg5LTdLY2VHNEZJSzlrN3VuemhzX1B5blpYRGtwS0hrak5r?oc=5</t>
         </is>
       </c>
-      <c r="E100" s="14" t="inlineStr">
+      <c r="E100" s="15" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3305,7 +3308,7 @@
       <c r="F100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" s="14" t="inlineStr">
+      <c r="A101" s="15" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3315,17 +3318,17 @@
           <t>The great fake meat meltdown is taking plant-based burgers with it</t>
         </is>
       </c>
-      <c r="C101" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D101" s="14" t="inlineStr">
+      <c r="C101" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D101" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPRTVDNW5oaWJ5bHdKM21iYllEVnpJbHhSbWFzYy1RcEZCdnNGUlJOWVJCaDZacFVoRjlSUGpfa3N6ckQtMFYzZTNITW5tMy05Sk0tZmtlSWlESHdOMWIyUWpUbE5RQVlsTHp0VXg0cHJYM0lJVmw1ckRURkFPVHFabTRIUzlFX1FlbFNuYmQ5MVJwWHVOaVhVWTdPajZxdG1WOTliTE1qZ3k1dnFRbk9BNTZCcXRRSGlIXzJv?oc=5</t>
         </is>
       </c>
-      <c r="E101" s="14" t="inlineStr">
+      <c r="E101" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3333,7 +3336,7 @@
       <c r="F101" s="3" t="inlineStr"/>
     </row>
     <row r="102">
-      <c r="A102" s="14" t="inlineStr">
+      <c r="A102" s="15" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3343,17 +3346,17 @@
           <t>Solar for Cuba: How Xi is turning Trump’s war into a China win</t>
         </is>
       </c>
-      <c r="C102" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D102" s="14" t="inlineStr">
+      <c r="C102" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D102" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQOFlUUnNZUWo0MTJRaDFIZHp5dUJudERrOWxCZmY1WjZmeXRTVzJkbENEbUFhSkZFUWV6WjNGNUJIejVYRXFPcmRNZjFZeTkzTmtaeFNlb2V1OFFnMGtkV2JfTVRUN2FSV2xxcUpDUDJQeUpqWE9DRHRmT2kyc1dIZE9jeUM2eV9KQjd2RkJuTkxYeEdISDZDejhRbVo?oc=5</t>
         </is>
       </c>
-      <c r="E102" s="14" t="inlineStr">
+      <c r="E102" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3361,7 +3364,7 @@
       <c r="F102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" s="14" t="inlineStr">
+      <c r="A103" s="15" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3371,17 +3374,17 @@
           <t>Beer Sectoral Group appoints Nigerian Breweries CEO Thibaut Boidin as Chairman</t>
         </is>
       </c>
-      <c r="C103" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D103" s="14" t="inlineStr">
+      <c r="C103" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D103" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOamdsNTN1dkRUY19Yak0wUGxsdm9NZGhySUM0Vzc4blNCeldzdFBiRkxuSW1xbTlZQUJIWkNxdzI3Zi1zc3F3SmJvai1UVGlZdUhGTEJ0eF9mNHRwSGREbDktT2txWXA4OVBESTdPLXdxWmV2V3FPTEZaYjRWLTlMM1VaY1dCbGZudTczZlFEYzN1aE9HeWdObE1yZFduLUtNVXBheDNsUWlIcUxibml4YQ?oc=5</t>
         </is>
       </c>
-      <c r="E103" s="14" t="inlineStr">
+      <c r="E103" s="15" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3389,7 +3392,7 @@
       <c r="F103" s="3" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" s="14" t="inlineStr">
+      <c r="A104" s="15" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3399,17 +3402,17 @@
           <t>Hip pocket pain comes for shoppers – and for supermarket giants</t>
         </is>
       </c>
-      <c r="C104" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D104" s="14" t="inlineStr">
+      <c r="C104" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D104" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOeTdfN2dwYlBWSTdGbFo0SWRJcTNYelFFM2FBRnlORWRNcGd0WUVCbVdHVWZ6TFdZQzFpM2h6TkU2OEtqeE5OYlRrNmhsRU43a0E0UXhtZEZyTWZidzhMUEVxSVdiMlpTYXQ4ZVRaNl9BSi1Mb3JRaXhvM2hlMmNDcnk1aFBvVXFQSmlPbkN4Z3o2R2RzV0drQWpKaVZpbXR4dHppa08wRFd0dlNwcDc1alRDSXg?oc=5</t>
         </is>
       </c>
-      <c r="E104" s="14" t="inlineStr">
+      <c r="E104" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3417,7 +3420,7 @@
       <c r="F104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
-      <c r="A105" s="14" t="inlineStr">
+      <c r="A105" s="15" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3427,17 +3430,17 @@
           <t>RBA calls for co-ordinated effort to unlock digital asset markets</t>
         </is>
       </c>
-      <c r="C105" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D105" s="14" t="inlineStr">
+      <c r="C105" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D105" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOT3dEcEtwVUptWTZydTRYWFdCU1RhTjI1RkFWeU5HckRVZjBxc2lqRkNOT0stc1h2Q0E1YTkxTjk3NTB3TGxKZGIweGFQRGh2S05QWHRoVGNZRFR2SlI2bkEzWlRoY2t3WU16dDlhVEI4RTFWYzhKS25YbGYxSVRjdFpVQ2M0dVc5MFJuUExNMTJIMVJTYmZGbkNLR1BPeVFYSF95NkNnWEEzamg3NmRuRkx0U2NjbXlxY015UWljTzRWbXpKclAwUg?oc=5</t>
         </is>
       </c>
-      <c r="E105" s="14" t="inlineStr">
+      <c r="E105" s="15" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3445,7 +3448,7 @@
       <c r="F105" s="3" t="inlineStr"/>
     </row>
     <row r="106">
-      <c r="A106" s="14" t="inlineStr">
+      <c r="A106" s="15" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -3455,17 +3458,17 @@
           <t>Banks rebuff work from home calls as Wesfarmers pauses business travel</t>
         </is>
       </c>
-      <c r="C106" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D106" s="14" t="inlineStr">
+      <c r="C106" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D106" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOTjFLNnZUNXZHeE85a3kyaG1IX29sWjFvZ2NzS041UnYxNkkwUF9YU3ZFYXhtQmlxY3Rmd0lUSTJrdTl1Y0ZobWp0M1lrZnZhZE9OSzV3Ql9Hb2UtUEpqWC1McjM0S2pESDJQVWJKQkw4enF5THJfeXFWRDZiMk5KMmVrazVUMzBNTk1tOXRVX1ZzVU1IUHBVSlhENEdEWFJpQnFXUGkyNVJGUnhzdXgyNW1WZXRkRmRaaVloZnpaMFdqVmk3elpFSkZ6ZmotZw?oc=5</t>
         </is>
       </c>
-      <c r="E106" s="14" t="inlineStr">
+      <c r="E106" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3473,7 +3476,7 @@
       <c r="F106" s="3" t="inlineStr"/>
     </row>
     <row r="107">
-      <c r="A107" s="14" t="inlineStr">
+      <c r="A107" s="15" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -3483,17 +3486,17 @@
           <t>This mine was fast-tracked to boost Australian solar. It’s exporting to China instead</t>
         </is>
       </c>
-      <c r="C107" s="14" t="inlineStr">
+      <c r="C107" s="15" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D107" s="14" t="inlineStr">
+      <c r="D107" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAJBVV95cUxPN1ZSdEMzSXBhMno2YzNkSFFtdlBOTTRGV3UtbnZtRktEd3Q0MHdmZHp0SDN5S0FZYmVKUllicHRMRkxTdmxtbkMtT2ZVN3hsUXdBVzAxdzhWcGFWRkxVdFY3NURqTVV2QVJQT0ZUT193R3JLLU9aZUw4YzlucjVUN0xyTzdoZlNjYXdyR2VWeDZrbW53cTJoRGZDd2kxbkxzMHBQWkRJMTFPMkNlX19wYjI2LVBZbnVJOVNsRjF3Tm0xUUFpY0ctczFZdWJFcHQyLUhwdDNiSGVtdHQzVVRtbExpcHJZak1SNkhWd2s4a0RtYWFNN2J2Q3FobTF1N0hWLXA4YUtaMXBScjZsUWt3alVVTVpJdVl0WDF5RTJLM1BKUl85dnhUUktkb2VwMzFkUWZ1ctIBugJBVV95cUxOOENIa2JzQzdxekNYTnJNVmRzdm9KTFpndnBybEJfNjBUR3VNMk92ZnhGY0JwVGZLeFRpdHJLMTQ0NjRNOFg5b3FESzhPLWlub2hSeFdidW0yS1h6ZXlGMjh3X3FhaWo1dHdneUZxS2NsaUJ6dWtfT1R6VndwSk52bVVNN2I5VlNYazBIelcwUkVBZHFlM0hiQVJ1a2NGWFpmR0c5R3Bna2RZMmJuSXB5WkQ1Zl94VDFtcjVEd2x6amIwSWdXUWtQVVo1Q0hpWVBLRVFycDAyU1NJV3N4YktlUlBtMTlkY2VNZjc1QVZhbnRrQ01OQnZqNzI5dTNNZ1VlNVVJcURycXlDRFZDYVo1aC15RXpwUFlvZWxlMHFybWJiM1YxT05lRElXYlZsbkJWUnI4VV9Da1lIUQ?oc=5</t>
         </is>
       </c>
-      <c r="E107" s="14" t="inlineStr">
+      <c r="E107" s="15" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3501,7 +3504,7 @@
       <c r="F107" s="3" t="inlineStr"/>
     </row>
     <row r="108">
-      <c r="A108" s="14" t="inlineStr">
+      <c r="A108" s="15" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3511,17 +3514,17 @@
           <t>A $600m dream or a dangerous gamble for cricket?</t>
         </is>
       </c>
-      <c r="C108" s="14" t="inlineStr">
+      <c r="C108" s="15" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D108" s="14" t="inlineStr">
+      <c r="D108" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxOYnpVaTZiU3hGMWY1UVVmYk9nRTJaRTVFYUE2ZklLYmJIQkdXZzFMbWs3MVRJb0l4bUpPeThwRnhOSmh0bzNBdzhpeXpuS1RrZ0tNVVJ4eU8tRVIwR2FyYmUtNG1UVmN2OXRsZm1mVy1LZDVERkpXQURMUk1HRE9Hc3F3RWQzYmFvbHRCVGhFOTQ3M2xnVGcxTWxtT3cydW84NTNPc3BXQURodmY0azBOUllOQjhrbzJ6WmI3bjY5dk5RRzlDQ0JlYzg0VzRsdWtIblZJelRSamFyQnNweHdHLTRTMTFOcy1Jd3ZtQWFodEcxOThVeVVz0gH3AUFVX3lxTE5ielVpNmJTeEYxZjVRVWZiT2dFMlpFNUVhQTZmSUtiYkhCR1dnMUxtazcxVElvSXhtSk95OHBGeE5KaHRvM0F3OGl5em5LVGtnS01VUnh5Ty1FUjBHYXJiZS00bVRWY3Y5dGxmbWZXLUtkNURGSldBRExSTUdET0dzcXdFZDNiYW9sdEJUaEU5NDczbGdUZzFNbG1PdzJ1bzg1M09zcFdBRGh2ZjRrME5SWU5COGtvMnpaYjduNjl2TlFHOUNDQmVjODRXNGx1a0huVkl6VFJqYXJCc3B4d0ctNFMxMU5zLUl3dm1BYWh0RzE5OFV5VXM?oc=5</t>
         </is>
       </c>
-      <c r="E108" s="14" t="inlineStr">
+      <c r="E108" s="15" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3529,7 +3532,7 @@
       <c r="F108" s="3" t="inlineStr"/>
     </row>
     <row r="109">
-      <c r="A109" s="14" t="inlineStr">
+      <c r="A109" s="15" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3539,17 +3542,17 @@
           <t>Why these people decided to vote for One Nation</t>
         </is>
       </c>
-      <c r="C109" s="14" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D109" s="14" t="inlineStr">
+      <c r="C109" s="15" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D109" s="15" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOQmNaOHZXWEEwZzRmdTBVT2FiS2hsYUhFczgxaFJaeEQzMGlfSnRoUWo0ZXl3cWhhbTU2NDRLUjh1c2Jxd3ZoR2pJOHVNemI2cTFrdU9oVkFCNXN4WV94TER4VmtIX1JCblhKNTl4VHlMdFBDRHVBUFhkS1AtR05RMG5QVGJFaTlWaVpMZERIa3Ntbmh0V0xnVVhYNDdMWWlpSWc?oc=5</t>
         </is>
       </c>
-      <c r="E109" s="14" t="inlineStr">
+      <c r="E109" s="15" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3583,6 +3586,62 @@
         </is>
       </c>
       <c r="F110" s="3" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="16" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>Blackstone-backed $2b Xpansiv kicks off raise</t>
+        </is>
+      </c>
+      <c r="C111" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D111" s="16" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOOGIxbEhpZjgwbk5XampWenBXbGZmbzFQbnJhUjU1Z2FtT1FGVk40SHExMUJBZHZoRDBRVXZHS3ZlR3o5RGU0c1o0Y0E2MXVKZ3U2ZFBBRm1NbVJPRk1pMGp3dV96ZTlMNERlMFBPRDNROXpNZlNmLV83VGV2QVNzWkhtV1kxY2x6TUQ3QkhlcVNPNTlyMUQ0?oc=5</t>
+        </is>
+      </c>
+      <c r="E111" s="16" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="16" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>Elon Musk puts a $2.5 trillion rocket up Wall Street convention</t>
+        </is>
+      </c>
+      <c r="C112" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D112" s="16" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPeE52VS03NHBqZ3hvc1Q4V2laUElCcmxKem9SSzM0d1Uyd09ZSFl4SjZmUDl1Sl85WXp3TWtGX3hydFRwZG0xQmFlOVUtdEtaNmtYWFkzVDYyZGI0SWFZRWtYR2tGODdPVUNhLXBzVVpzYnVRYmZNZW8xbEpreGZMVzU5c1JrWDY1Nk9uWk53a3FCOHpQTDBCT0h6QllmbW1wc3FmVU4yTUlxSmRhTUdF?oc=5</t>
+        </is>
+      </c>
+      <c r="E112" s="16" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>

</xml_diff>

<commit_message>
Update news log — 2026-03-30
</commit_message>
<xml_diff>
--- a/news_log.xlsx
+++ b/news_log.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -87,6 +87,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -492,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F112"/>
+  <dimension ref="A1:F126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -536,7 +539,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -546,17 +549,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C2" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D2" s="15" t="inlineStr">
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E2" s="15" t="inlineStr">
+      <c r="E2" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -564,7 +567,7 @@
       <c r="F2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -574,17 +577,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C3" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D3" s="15" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E3" s="15" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -592,7 +595,7 @@
       <c r="F3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -602,17 +605,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -620,7 +623,7 @@
       <c r="F4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -630,17 +633,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -648,7 +651,7 @@
       <c r="F5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -658,17 +661,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -676,7 +679,7 @@
       <c r="F6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -686,17 +689,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D7" s="15" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5</t>
         </is>
       </c>
-      <c r="E7" s="15" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -704,7 +707,7 @@
       <c r="F7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -714,17 +717,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -732,7 +735,7 @@
       <c r="F8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -742,17 +745,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5</t>
         </is>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -760,7 +763,7 @@
       <c r="F9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -770,17 +773,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr">
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5</t>
         </is>
       </c>
-      <c r="E10" s="15" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -788,7 +791,7 @@
       <c r="F10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -798,17 +801,17 @@
           <t>Zarraffa’s Coffee celebrates 30 years, eyes nationwide growth</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOcXNzUkRLemZEOWtOZjhvRUtzcUZrSTdzV0s0LUJTd2NGRk1Gb1NSLUR5Rlh3NUdWQUJkVWctb0toUFBRajlMcWV3VnNyTUtydy1PSUoyb1NCOGVtMUZqRVN0MzFkVkNlOUZNVXlHN2kzREhSdWJQUnJqa0pnUzExTVZSc1NCVFZSNlBSUWNfWnZ3MC01aUx0UWF5SkNOaHI3ZkE?oc=5</t>
         </is>
       </c>
-      <c r="E11" s="15" t="inlineStr">
+      <c r="E11" s="16" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -816,7 +819,7 @@
       <c r="F11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -826,17 +829,17 @@
           <t>Zarraffa’s Coffee eyes 200 outlets ahead of 2032 Olympics</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="C12" s="16" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="D12" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPMUFjRTlGVFBqYzlPWXdzQ0dKVVlhWGxncUQxTDd1R0VHcThlV3ExVmo4SlBGSHVuUGZrMGNqSVo1YVpDWHViMm5KZWIxcHNMMHo0b1FQcmxUNElDR2lEeWRuLWZIN2lyQUV0VndEUWNkNU42Z3AzNXRlbm50NzhtTXZ0Q245dF9hNzBxOENuMXZsVlU4Z0JGVElR?oc=5</t>
         </is>
       </c>
-      <c r="E12" s="15" t="inlineStr">
+      <c r="E12" s="16" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -844,7 +847,7 @@
       <c r="F12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -854,17 +857,17 @@
           <t>Aware Super appoints new head of private equity</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNVHJXNWEtdEZZUW1fZzdYMTB4RklBTUh6dUNKQ3BrTlpYUnBwRURIVGZjWTV0OUxScnhGMVNSczhLUjVqOEwzbkR2WWlEbmF4ZkNUdHNQY0J1djI0REctbHd2SVhUNlNCa2M5bFhOQ0JPU0RHOVVTQkEzRDdGMjRZbVFDOUdlTXNNczlmZWF6bXlfbEFGRE0xbkZQaw?oc=5</t>
         </is>
       </c>
-      <c r="E13" s="15" t="inlineStr">
+      <c r="E13" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -872,7 +875,7 @@
       <c r="F13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -882,17 +885,17 @@
           <t>Commission wrinkle over UP Education sale</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxNSV9GMjhqM2ZSanI2X0w2OVlQVFRQTUoxYzAxaXVZMmU1REVTcHlUeEltdXJtaXZrcUJWdDZxNGpYTTZYSFE2TkZHeG9OaVRZakoxV0s1U01TVjJpWlhaSENfNVhucG5NVzFMbTVBY25zWGRSODBtRGtkS1owVTlJWnNfcTJ5alFnbVl1SU9aUDF1QWxJLTBSQ3kxUUFlZnpJMlVEQndFSGRGbDF6WVBUVHlCcDM5Qnh3R2xBMG9xN2FLckNzbUFOWDI1aVF1YV90d0twd0ZmMnUySDBMdG1R0gHkAUFVX3lxTE5EWVp6VzZWb01TRmlHSS0wMExldkJwSHJjdlZXdElsRlpBTEtVMkd6VzNQa1RpVDNsOFQzaGZ2VHpzUnBDYk82RmZGQWJuTmVQMXhxLXVmdVFxTVZOZTBsOHZ0V3cyVVVkNWUwVUxSc0xNSU92ZktpdFRfYnQ4WHBTX3A5bFhXZ1YwZXNrc1BSZEU4LVYybnNBd0dCdk92OFUwclJCMzdoU0ctX1pEdTAwY0JiTWQ4S01QRE00TW5EUEJwR2YtczZ0T005bTJnN1RDY2p6NFF1SndfLUo4QzJUWk1tRg?oc=5</t>
         </is>
       </c>
-      <c r="E14" s="15" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -900,7 +903,7 @@
       <c r="F14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -910,17 +913,17 @@
           <t>Gloria Jean’s owner has an angry shareholder on its case</t>
         </is>
       </c>
-      <c r="C15" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D15" s="15" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPTnZwUVBCdTFJZWkwc0YtVmJqMkNPcUR5RktjMlVURmhROFZkYUpXM01iRUh3SnJEUElxRGlSNk9DQjZSdTdNdmZwWWpONjlmR1hoMl92cUNmd3M4cnJhVkNqc095MmN6WXBYUmdEblB0eERtVDdlUU4yNGFjXzVnT19rOERIRzVPNzY3VDNNRS1tVGVTX3pKMVRpTXZVR1ROLURBLWtJbVZhY0lSU09DNkE2NzFLbEFU?oc=5</t>
         </is>
       </c>
-      <c r="E15" s="15" t="inlineStr">
+      <c r="E15" s="16" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -928,7 +931,7 @@
       <c r="F15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -938,17 +941,17 @@
           <t>Oporto-owner Craveable Brands hires new CEO from Domino’s</t>
         </is>
       </c>
-      <c r="C16" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D16" s="15" t="inlineStr">
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNNmxfQVc2Umc4QWwzSTdsZTFvejRzTzZxXy1ScGlhXzh6bm5JS3IyX0xTNDVBNjh0cXpPbGhxNU5xUHhQN3EtRF9aV3FEc2JoSG5QTU1WeU1TLUJfZzVUT2N6dXloQXhZaHB5djB3dDFKN1llVmI3UVpKNjJTNlcyV0ZDcG9GdVdSdW41ZkN1b1N3SFFIUzcwRkQ3UHY2TmxERmZwTlA0RzU?oc=5</t>
         </is>
       </c>
-      <c r="E16" s="15" t="inlineStr">
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -956,7 +959,7 @@
       <c r="F16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -966,17 +969,17 @@
           <t>Brookfield, BGH Capital rub shoulders in ScotPac’s data room</t>
         </is>
       </c>
-      <c r="C17" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D17" s="15" t="inlineStr">
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPMVlxbzlQNnFXWnJFNU11Y1BhTTVqbjN4RG1nbkZuN0pkdDFFaUhJN0RaVnUtWDlZSGJWR1ozQXk5UUx6RVdOcjBPU2t5UzN4T0JvUFJISnNvVWxQemd3blNHZjRQVVVZQk1nZER0Y0JfY3VvQ0t1a09sM1RTS2c1YTJyUmdzYWh1WGRUNjl2dkdzYTJJeHVhMTdqR3Y5WVlHVEtSZHp1cmVYYmM?oc=5</t>
         </is>
       </c>
-      <c r="E17" s="15" t="inlineStr">
+      <c r="E17" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -984,7 +987,7 @@
       <c r="F17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -994,17 +997,17 @@
           <t>Payments player Pay.com.au hits the road(show) for $850m IPO</t>
         </is>
       </c>
-      <c r="C18" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D18" s="15" t="inlineStr">
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOMFZleXZrbU53TzBlakI2ZmJKTjlrN3BoQlRaWjQ5cXFzTllKWmFoRm1UT2xDUHBtNC1QNTNiX1BwSzllMkRZdHIzRlAteDREaUczN1JTNTByTW1jNnR3d2NnR0RxUDBxeHYyWU1CSUs5MEZad2JqSGF6ZUxHZUNtZmFQaTJZZVJVZ1B4MkZ6V09QMWIxaUNHQmVzTDhvWVA1Ty1UbHgtQnRrQQ?oc=5</t>
         </is>
       </c>
-      <c r="E18" s="15" t="inlineStr">
+      <c r="E18" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1012,7 +1015,7 @@
       <c r="F18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1022,17 +1025,17 @@
           <t>Another year, another IPO cold shower for investors</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D19" s="15" t="inlineStr">
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNeEhzYzQzdjR5MDJCWkd6Q2VLdEZzbzRoWnNOcXFlQjNfMlV4Q0NQRjExMlNhT2NPcnRBbW1sZUkteXo4N0dGaHNNeGZJOEZ2aXFvdmZiN2V2QzdOMzFteFRnY1RVRm1rQXltWmY5VFZOdFVNNVpudVp1dTlrcFM5b1k5SmlWQllDMVFXSjA4ZVpSZHgtV2JpWDJ4SkFRbVE?oc=5</t>
         </is>
       </c>
-      <c r="E19" s="15" t="inlineStr">
+      <c r="E19" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1040,7 +1043,7 @@
       <c r="F19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1050,17 +1053,17 @@
           <t>Priceline Pharmacy franchisee sale narrows to final four bidders</t>
         </is>
       </c>
-      <c r="C20" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D20" s="15" t="inlineStr">
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNR294am9sYWNiQ3FVT1B6YlV5ejMyeHAyT0FibTFVbU5pcjZyaVRyazEzbFkxd0lrcnpZNGpTYUx4Ykl1Xy1sZF93M2Nid19ydUFwbUJ3ZHozaURaNkRoOE9OMnRBRGZfQVdCVWZCaVhhNnZSRjlwYUdDVnp2WU9HUkJxbE1QMV8zdWxYRTNBQWktR0xSOFU4dmtXZWk0am9SSU92NWp6QUZmTVU5TzJEOEJNak5fQUtN?oc=5</t>
         </is>
       </c>
-      <c r="E20" s="15" t="inlineStr">
+      <c r="E20" s="16" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1068,7 +1071,7 @@
       <c r="F20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1078,17 +1081,17 @@
           <t>Private equity gets better image of Qscan</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C21" s="16" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="D21" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxPRjVmT0hDRjZLblB1VHdPRmRGeXhKdDJHdWxDTzV4RDZ0VzdHaUFfOVlnZjRQMWhKcWMxby1oRDR6N2lQZkI1UDE1REppS3c4LTVmU3p5b2wtblRCWnhNajFnZGNHaGRJUHFMUGRtTHAyQmIxOHhNNTgwRWVSeWp6ZWRxbUY0WVhiUnhMRUpDLXNwS1RuelJldTk0Z1R0WHg0XzNXNTA5Rk5TRFZhU1RNVnN2TlZuaFE4OWtIYXQ5a2VGSW1UWmt5Rlc4Q2lIXzF3YlkwNVhfUzJDV0dQdVAxa2RKc08wRGR6TlB2Vi14QV9BdlhyaTZsM2pEVGZycTjSAYQCQVVfeXFMTWpnb0lWQmZ6MTFnRGhWNTNqczk1TWhTcUFEMVpDNnJ4ZWVxVlRUODhJXy03NHdGZVJlMmhyUHM0Nlh4NlZtTzRhQ0xxRDFLVHNzUVNfbWxhS3BLUEQteEMzZHRrc0F1eFRzYmxVNDZlSURyZDB5bF9wQTNRRU5yZEs1Z3pFRTdwcFBaMkNlN0JvT1NEYkFWVUJNcHJqcEM5RVJYa0JFUVl6cThyQXloaERzQjhkTUVPakJqb0hzNVlwSWxNS0dmZkNFSG9Gb3dNUnVvUnV0d3MxSmpzdFZKTHJ2RTQwRUoyMEVLLWMwT1NnOHdXVl9lRXNDWEFndzJFSDlZU0o?oc=5</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
+      <c r="E21" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1096,7 +1099,7 @@
       <c r="F21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1106,17 +1109,17 @@
           <t>Oporto CEO’s first year reshapes brand and network strategy</t>
         </is>
       </c>
-      <c r="C22" s="15" t="inlineStr">
+      <c r="C22" s="16" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D22" s="15" t="inlineStr">
+      <c r="D22" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPY25mNTJfT3FiVlBPZE5CcVNkR1UzR2xWaUtJSmxhU3EwcEMzQi1ISDFSajlCQWk1UUJpZVJ1Q19ZV3Jjd0Noc0l3OExpMXhSQUVVdHhCLTBlOXNoZzA3UXZBdkR1VHBvMmVsZkNhUFJndm1DdGpnX2w0ZVViU2phZ1RmYXY1SlhwUnhKSUxBQVZZUXpqNHQxQmo0Rk1iV0g0OW9qUS16eWRSNW5FaW1yQQ?oc=5</t>
         </is>
       </c>
-      <c r="E22" s="15" t="inlineStr">
+      <c r="E22" s="16" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1124,7 +1127,7 @@
       <c r="F22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1134,17 +1137,17 @@
           <t>The Melbourne restaurant our reviewer grew to love</t>
         </is>
       </c>
-      <c r="C23" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D23" s="15" t="inlineStr">
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOc3YxQTljcHJXVWtRX2ZGM2lpM2pILWNwSFg0MFJrNmNWX0ZxRG9nV0J5N19qRWh4U0hPXzNmVVZwWk9wT2kzaFNrTlV3NEQ1Q3JpaXVIYlBHb216Q3VYVWdSRXMwdDl0SmYzdnRlSDFUYVRmRGJyZVlRZDJKTHpJOUctYlF1RDZSYjloY0hfZy13QmFTLU9UNjkwTHc1bjlGcGxoZ0ZLVU1GWTctZkdLZU9zSGhEZEpKbXJnaWJfZjd2OWs3?oc=5</t>
         </is>
       </c>
-      <c r="E23" s="15" t="inlineStr">
+      <c r="E23" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1152,7 +1155,7 @@
       <c r="F23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1162,17 +1165,17 @@
           <t>Crescent Capital strikes Benson Radiology deal for close to $400m</t>
         </is>
       </c>
-      <c r="C24" s="15" t="inlineStr">
+      <c r="C24" s="16" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D24" s="15" t="inlineStr">
+      <c r="D24" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOLTNrWG1ZZlFoU3pDZ3E2SEgwMlhzQkdtQUYzaHZTZmYwU3ZhMnE0dlkza005VkZmZ09NMExlWDVncnBmYVVISXJ6X1ZjNHhpM2RnSlprY1dnbndJNUczcDVtNXNRY3pVNW12bm5rUVdqVmR4R0JlVHFuN0RwTlFkR2xrbFFpSl9jcm5oSjk3aFM1clBSVDhnbkhoWUREeUhsbVpvQW90d05xOTdfOV9nbW5POFdmelJkVlpsUlRuYl9odmRNVUV2S0pCMFBMTS0tcVhGVGFYU0h2d9IB3wFBVV95cUxPWEs4R2pxdThPbHJHb0dBT183SkRHTTlXNzdWazcxdkd1eGx2VlAyM2VVbEtEbWxTZ1R0TlBFRmRMZTFoalgxSmVVRUJFR0c0RFYzZVJFODg3dWxicU9pOHppeFhjaVp0WWlyTnUzV1dyZXdkMHBDVHI4LUVQdjc0cWpheU55NTlvdWdCZmVoODB0Mm5fbGNCTmQwLUhMZ0psQVpzb3BEUnJpSkRnOUM0c0VCdUp5N3g5MkhaM01vTHJ3NWd0ay02UXZUUG9nVkxicVc1Z0xjWGhjUDRDVjlN?oc=5</t>
         </is>
       </c>
-      <c r="E24" s="15" t="inlineStr">
+      <c r="E24" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1180,7 +1183,7 @@
       <c r="F24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="inlineStr">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1190,17 +1193,17 @@
           <t>Dual-listed giant Capstone Copper flirts with $600m-plus carve-out</t>
         </is>
       </c>
-      <c r="C25" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D25" s="15" t="inlineStr">
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNcVh4blRkQnoyaG1TajhVV0lrOEJRaHdTZWtzUnJHaEdaSXNRWThGTHlVdGl4dGJ1cTMwZ2pLcVNzUXRYNlZzVzhvaXdkNGtVUG0wN0FrMHB0R1I2Ry1jcEgtSWUtajI0cTFMRTlfdzBuMWtrZmJOLVUtMkl5dW85dFp6dEhEOHhTNzdfOFNFSGtlT0MwQnRlY0VhcUZBNE9RYzhQcDdOQUFnYkgzd0V0N253SQ?oc=5</t>
         </is>
       </c>
-      <c r="E25" s="15" t="inlineStr">
+      <c r="E25" s="16" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1208,7 +1211,7 @@
       <c r="F25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="inlineStr">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1218,17 +1221,17 @@
           <t>Guzman y Gomez unveils a new menu under $4</t>
         </is>
       </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="C26" s="16" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D26" s="15" t="inlineStr">
+      <c r="D26" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPMjRjRTV2a3BJc3AzdDNOQktoYjBvLVZSODVsc3lKQ3pET0lxUlpkc05NcVlKRlZITjVJbjkwLS1DUFJNMGJ1amJKTlp3S3VqMWJaU3YtUENEN01rUEJiV1FNZTRXYjcyV08zZzlxNDVOSlVOTlJDOGV3QzBQcUpKa2Zab1ItNlI3ajZVVTF3?oc=5</t>
         </is>
       </c>
-      <c r="E26" s="15" t="inlineStr">
+      <c r="E26" s="16" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1236,7 +1239,7 @@
       <c r="F26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="inlineStr">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1246,17 +1249,17 @@
           <t>Can Sydney’s burrito king conquer the $676b US fast food market?</t>
         </is>
       </c>
-      <c r="C27" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D27" s="15" t="inlineStr">
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNM0ZFcUpLN1dUZWUyaE1LMnNZVGlEbkNNQUQ4Wmd6QVFlTy0wZDVHdnlja1gzMEZTbVpKU1Ftb3VKZ2pzajcyWU16NUtUTmR0TlZMOVhMRUNqZXZiX2d2NWY0YlJDOFhhYUE0SkhMRUprNndXak8tWGdERU90cmMxTkFjcFFVSTd5VlZ3NFVKOXN3M255MFhzZThmbi1VUGMyQ3E4d2pYcFlJckY3QlVBdVJJeF9qUQ?oc=5</t>
         </is>
       </c>
-      <c r="E27" s="15" t="inlineStr">
+      <c r="E27" s="16" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1264,7 +1267,7 @@
       <c r="F27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="inlineStr">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1274,17 +1277,17 @@
           <t>Drone maker Innovaero prepares for ASX float, taps Euroz Hartleys</t>
         </is>
       </c>
-      <c r="C28" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D28" s="15" t="inlineStr">
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNU3JrejNRZ1VBZVNVV29NMkFPVmRsWE4yMVZPcjk2aUNUTHFJUGFyQ1VnZEZiZlIzQW9VVzRNNDNRR01jcHo3X0tqZjB4bzhMTTI0Y3BwYUh6OGRUUGt2REIxV09oRnJoVWlVelZWaUlWUmlPQ3dJdi1TejcyaXB1Z0x1MEJRSlB3SGMwVGdXaXJJNm9TVllPOG5JZC1feEV3TVhTeExGeHR2RHFIWlVCOXh3?oc=5</t>
         </is>
       </c>
-      <c r="E28" s="15" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1292,7 +1295,7 @@
       <c r="F28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="inlineStr">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1302,17 +1305,17 @@
           <t>Bain flaunts Estia 2.0 as IPO roadshow gets under way</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D29" s="15" t="inlineStr">
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNTEN1cGsxNDN2c1NqUzB6UmJ4TFl0NGZjZVN3U3oxMlVFWTF4WUZLQS13dUxMV0N2ek1XN2VURTNVWms1NjdXSm0waEdaTXQwdTdWY1MxZ1V3ZnpEcVJtczdOWGNNZ0RQNzRZLU1MTTgtRW5DZkctbXBGMmVXVXdPZW5pNThiRHEzWnB2eFZzTFZTb1ZkeW9LendkNDd0cXRid05ZSGZYbW9NZXdOLVZWODdZU3hVcTA?oc=5</t>
         </is>
       </c>
-      <c r="E29" s="15" t="inlineStr">
+      <c r="E29" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1320,7 +1323,7 @@
       <c r="F29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="inlineStr">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1330,17 +1333,17 @@
           <t>Carl’s Jr. Australia unveils nationwide freebies for Happiness Day</t>
         </is>
       </c>
-      <c r="C30" s="15" t="inlineStr">
+      <c r="C30" s="16" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D30" s="15" t="inlineStr">
+      <c r="D30" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNVWgwdjU1NDFWalBfMTFYX1dQOWNDbG1FVUdlcS1LTVlHZVRRTVBWTjhSMnpkTXRXNlFJdllGQUp5Mm5ObWpIazd1d0RJa3QtdFBZN1hOenBmVzBEU05wM0gtNUxPeWpsYkxyVnhWWFFOU2Y3R0tXcmNkeWhpWDh2eDZBdjNCMHhuc1lHYTZHblBPVkpfRXpKd051UWlNc1hm?oc=5</t>
         </is>
       </c>
-      <c r="E30" s="15" t="inlineStr">
+      <c r="E30" s="16" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1348,7 +1351,7 @@
       <c r="F30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="15" t="inlineStr">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1358,17 +1361,17 @@
           <t>BHP and Woodside appoint new CEOs in major mining shake-up</t>
         </is>
       </c>
-      <c r="C31" s="15" t="inlineStr">
+      <c r="C31" s="16" t="inlineStr">
         <is>
           <t>ABC News</t>
         </is>
       </c>
-      <c r="D31" s="15" t="inlineStr">
+      <c r="D31" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQbTg5VFJLbWJfcy1uV3ZReTJkTndzX01qZ2MxNWkzaWZRckNLZUR1Y1VsMVRNc2FySC13U0NzalFEb3k1R3BaUEhfcTV0N1M4Q1dpSlo0YXI0UFhrMGRab2RiYV9DQVNVX01ycFc5ZFZrZWZqc1VRZXoxLVEzSDJLclJLSWg5bzN3R1I0bG9lWjVDaHE4?oc=5</t>
         </is>
       </c>
-      <c r="E31" s="15" t="inlineStr">
+      <c r="E31" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1376,7 +1379,7 @@
       <c r="F31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="15" t="inlineStr">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1386,17 +1389,17 @@
           <t>Next Capital sells Enviropacific unit to French waste management giant</t>
         </is>
       </c>
-      <c r="C32" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D32" s="15" t="inlineStr">
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPR3lFbERLR2FtdmJUU3BDU2thZk00YmFHRFhXR2VBVXhQSURTeE5ONVJKczBwbzlFMnR5cmhxMnM0bzlJbWo4SXl1dHpqYWxxMUJBRjZHVUtab1RYZjZMTnpGc3FzMWQ2NjNEdGU3NTZwa0diM1lJS1haYllwTldLZlpZbXp0YzlxcDh0ekcwTy03dDdPcnk4b29HZVdqbHhZY2JPR2drM2puSVpjUzZkVjNpZUE4dVMwYlE?oc=5</t>
         </is>
       </c>
-      <c r="E32" s="15" t="inlineStr">
+      <c r="E32" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1404,7 +1407,7 @@
       <c r="F32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1414,17 +1417,17 @@
           <t>Future Fund private equity and real assets chiefs head for the door</t>
         </is>
       </c>
-      <c r="C33" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D33" s="15" t="inlineStr">
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPUHNHRFhFMVdwVld6RFRZUFd3QWNOd1kzeS1QdnJxMERFSnE5LTdZcDhDYlVGcWZMeWxlR0FSRWF6YkZoQVZrZU9TQ1E4YTEydUJnOFE3enV5Rmk5UnF5VEdYZ1FMUWpKVjdjMlZZUGFsU0tKcV9Vbl8zcHp5aVF5Z2JMOUZocHJqRXNRaEp4Nm5CbDM1WkdIMHdQS2xqQnE2Tnh3?oc=5</t>
         </is>
       </c>
-      <c r="E33" s="15" t="inlineStr">
+      <c r="E33" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1432,7 +1435,7 @@
       <c r="F33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="15" t="inlineStr">
+      <c r="A34" s="16" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1442,17 +1445,17 @@
           <t>‘I actually started to die’: the new billionaire’s epiphany</t>
         </is>
       </c>
-      <c r="C34" s="15" t="inlineStr">
+      <c r="C34" s="16" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D34" s="15" t="inlineStr">
+      <c r="D34" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxPblkxbHVrdnVKY1pqQzNyWGNMZm9UYmY3dzlPaGQ4Yi1tc0U1akhrVWdIaXBpM05aZXRwTXE1eDBITlZpbDkwRXNrWjJ2YXBzX0VCY2JSLWhrVmpjSTE5eE5rLWgtc2pRZEdXbmhhWU1KeFExZDBGS2pjSkIwV0FGbndBZVAyQkg4WFRsengzSGYyZkFfQnJsQ18tUHJGNDd2T0pzZElPSVJTQkl2Rm5QTExJNHhmU2dHOHJGdTdzU08yNHRtd1R3Q0cyOF8taDktQTZvVXVBVjN1d0NHMmtFOHBWZXBFcUFWa1IyWGNDTDZUT3lQSXJHOVhxTFQ3b3RH0gGGAkFVX3lxTFBZQ3BFQWl5dEwwLW5yVWJuMU8zcXBPdE9pamRVSWVkbWNyVzgydGVOaDBROUN6RlBDbjdld05DVmZyb0R1eEN0UERubzZRU2NiMTQtVV9XNS1wYmlvZ1paM3RaOUlrTzJka0tXVVJEamFESGlSdXg2bDk1aUdhUVhBcXpnN01fX0Y0cTNvcm5DdEFFLVVERDFKTWxKZFR0UzAyblJqVHBua2JoYUdzeUNMb053ZVczWUFQU1AtVHV1d3lSSDFfZFh2cEkxSGw2MEdicEVsb2pLQ1RuQmdaRl9xNUROS3pKR2s2T2wxTTZ5bEwtTUNQNU04djFHTHlPbXVLSW9YSUE?oc=5</t>
         </is>
       </c>
-      <c r="E34" s="15" t="inlineStr">
+      <c r="E34" s="16" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1460,7 +1463,7 @@
       <c r="F34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="15" t="inlineStr">
+      <c r="A35" s="16" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1470,17 +1473,17 @@
           <t>Ironbark shuns private equity as it hunts for cash injection</t>
         </is>
       </c>
-      <c r="C35" s="15" t="inlineStr">
+      <c r="C35" s="16" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D35" s="15" t="inlineStr">
+      <c r="D35" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxQZWFaeVhldi00VkV5ZmEtS2tjcWdFWG55OGpCX3IyN25Rb3ZFV0ZKVm1aSE1WbThoYVY4ZEdfODVGX0RaUDV2Ul9HS1JQMDFCT05Fc2FaU0RINTMwbDRveWFsOFJSM2ZqTU9tVGxJSEl2ZmhhUHFHT3dqYkk5TUtvMUQySnZzTWw1MzFNWl9aVzhkSEZ4Q3YyWjRMUmpIdmJkdUVKWE54Nkt6bTd2dGFSUFoyNkgxTHh2TGVGak9ja0dFZ0xQM2g0S1lmQkZiWWtUcTVNdHhBdC1KeVRQcDA2dnpmeHRkWEnSAewBQVVfeXFMTWtYRDRSaHNULW1HanowRnpMdFF2VVMtZW1SV2ViZXlGaW02WlIwUzRZMGg5WDNrOUR4eDlGOEt5eGlqV0pfVDFhb0JEcS1faEJodWxyRnB3MkozOVJyT3NvM1I5MzdDcXNnUFNSdkRDamUzZTRQYlk0c1VIQUNMZ2ZzOWVCb2V2MC1aSTZLWkFkbW9GYk05b3RmN1htWENTeDh3SU1WYWJMcWx2eGUzZmwwVXF6czlnRGdXbE1vRElyVG0yM0ZzXzZ5TFh1YlRGNU9MQ1p3NnVZSFB0M0xBcGlueVZILXlVaXdqUkU?oc=5</t>
         </is>
       </c>
-      <c r="E35" s="15" t="inlineStr">
+      <c r="E35" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1488,7 +1491,7 @@
       <c r="F35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="15" t="inlineStr">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1498,17 +1501,17 @@
           <t>Minister leaps to fix food chain</t>
         </is>
       </c>
-      <c r="C36" s="15" t="inlineStr">
+      <c r="C36" s="16" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D36" s="15" t="inlineStr">
+      <c r="D36" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxOd2NqakVWRnQ4anFZNkl4Zy03MkloX08tUkktRTZqeEtQWFZJeVhkMUJIb0FxUjc2UjhCQ3MxbmNxczNxblJIZ09IeTBGNFM4Wkh4ZE1qNkhJMjIwU2RtX1JxcEV1Y0NjWXF6eHpVdTN4ZUlYMGIwcDJzMXZMTk94VzFlcjhpcVZVSTJFMjhsQjVGWEJQYTQ3aTFyNmNEZ1F1b3NGTWd5WnFJWmxXSTJ2NlRLcjJHNWkwaTZ2YVR6S0w5WVo1Vlg0VWdxcWZoa3VaTmcxY2NVcnR2bFRWNGNvZ1M2Tlg5NzlvVXZFZm9B0gHzAUFVX3lxTE1uNERoR3p2dXRIa0g0RXI2MWR6N0c5U3NGcjFDQVMtdEpyNDI2bk8yOS1qUnFOazdiODl0Ymo5R1pwRVJ0UFFVdzlhYjRDSUFCU0FRak4xcVVrTHphdTdxcHNIMnEyRVZud1FURmh5T0JLOHpRM3lFbDRuRnZMYmtaRnRFTXh3dkszTFhFUmZlRmoydnlEbW1fZTlmUzh4NXNyeTZTeUhOSktvclJVc0NTZTVYMkdJZEUyY2RmVC1kQ1hwVEloSEtVMEo5QnNTUXQyME5IN1BPd1NOS3oyR1JtMHBFVTZEbzhEQmdrWUk1ZnZVTQ?oc=5</t>
         </is>
       </c>
-      <c r="E36" s="15" t="inlineStr">
+      <c r="E36" s="16" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1516,7 +1519,7 @@
       <c r="F36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="15" t="inlineStr">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1526,17 +1529,17 @@
           <t>‘Brace for swings on every tweet’: Investors bamboozled by peace talks</t>
         </is>
       </c>
-      <c r="C37" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D37" s="15" t="inlineStr">
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOczZHTWFmTW9FZ1ZwSnc5Z3ZacGpsVDQ3LWw1a1BFT0tjRkphek41MlhNOU84emYzZUVwNV9xM0hyc1FUR0NHck14Qnh6c2JvQks5ZE02ZTNLWDI0dy1STi1HbDFDWW9yMDhGQXVVVzdkMzFXcnNNMVZHVXFMUXUteGtsVGhPVmhLcVZPQzlhTWNoYVVRMHF0cFhybWxzek13Y3ZjcjlXWjZJM2VYbm0tTmk4NExLQzQzX1ZPMVlhcnJxQkZx?oc=5</t>
         </is>
       </c>
-      <c r="E37" s="15" t="inlineStr">
+      <c r="E37" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1544,7 +1547,7 @@
       <c r="F37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="15" t="inlineStr">
+      <c r="A38" s="16" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1554,17 +1557,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C38" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D38" s="15" t="inlineStr">
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D38" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5</t>
         </is>
       </c>
-      <c r="E38" s="15" t="inlineStr">
+      <c r="E38" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1572,7 +1575,7 @@
       <c r="F38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="15" t="inlineStr">
+      <c r="A39" s="16" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1582,17 +1585,17 @@
           <t>Wirth’s Myer rescue mission is caught in the eye of the storm</t>
         </is>
       </c>
-      <c r="C39" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D39" s="15" t="inlineStr">
+      <c r="C39" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D39" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNTlQ4NDRnWE91VG1YNENpSTUxNnBjZkljOGdYaGV0aVB5dkVOaEJ6SjZ1bVA4NXE1S1hjV1NjcVhQTEVpWEVNV0UtbzhQTFZLOWxIenZiaF9QM3F6bmJYRy1lbXVMczZ3TnBHNy1aLUtVcnBDdkl4TE0zRGN4U0FwSjNPY1M5S3AtdUQ3UUNmR0x4MlU2YXRuUDJEUm01SmZWakx2UjFvY04zRHk4Smc?oc=5</t>
         </is>
       </c>
-      <c r="E39" s="15" t="inlineStr">
+      <c r="E39" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1600,7 +1603,7 @@
       <c r="F39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="15" t="inlineStr">
+      <c r="A40" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1610,17 +1613,17 @@
           <t>‘Darling, I’m not going anywhere’: The rise of at-home care</t>
         </is>
       </c>
-      <c r="C40" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D40" s="15" t="inlineStr">
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQS2k0M2otaldpNVFXdHRTMVNtZVhyUDV4VTNIcE5FSnFRaHNubGNQQzBVbllnNTktNGhrZ1lndzV5V1FpUS01SklRaTZmZHJkRzVsQmlsdEVmenZ4U2x6U01NeXdIMktBUW94TUE3R3FoLUxVcVhsVFI0SjVQVUFaZldnd3prMWMyaVRWX2J4aUdfQ25KWHpaLUlqSnhvQmM2TTRRQldGbm8tclFYRDA0TVdnU2g3QQ?oc=5</t>
         </is>
       </c>
-      <c r="E40" s="15" t="inlineStr">
+      <c r="E40" s="16" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1628,7 +1631,7 @@
       <c r="F40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="15" t="inlineStr">
+      <c r="A41" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1638,17 +1641,17 @@
           <t>Iran targets Israel and Gulf states as Trump looks to calm markets</t>
         </is>
       </c>
-      <c r="C41" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D41" s="15" t="inlineStr">
+      <c r="C41" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D41" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPLXBITXU3WTRtc0NYdnhTZHFaUTBCSXdldTBuSHliTlY1dlJONW43Qkd6Nl9pNmY1eDhzaHZoX19xYjBxMXR5UEhkVUg2M2k1MmhuVEwyY0JxbnJyemxVYUZjbk5BbkN4ajhPbW9ZeDhlRDRYTW1hN3k2d084c2djMEJUZTV3NVdPbllKUmFlU2JsaDV3Zk9CVFF0VDFkV09JSloycWdOUlVrREptQTJfa25LUEx5djA2SjNMMFY0RjM?oc=5</t>
         </is>
       </c>
-      <c r="E41" s="15" t="inlineStr">
+      <c r="E41" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1656,7 +1659,7 @@
       <c r="F41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="15" t="inlineStr">
+      <c r="A42" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1666,17 +1669,17 @@
           <t>Meet Christian Louboutin, footwear’s most famous billionaire</t>
         </is>
       </c>
-      <c r="C42" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D42" s="15" t="inlineStr">
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPcXdGd0tMckYxbjZ5TVJmQ0Q4NFl2RkhHMHdlZDZsdGZ6cVQ0cUpaLWJTNlVoc2ZOQmtXNlFTRnJVMnVDTGc1NFNZN2g1VnotQlNQbzhlM1BJV3ZwQktOcGtac3RwSHRLZkR0b2l0eGIyVVlYdHJrc2hpT0pJbDR3LURPTnowZk54LThObndtMVkwV2VWQkluNVlWY0p4QVJGbE1hSGMzOW8zdkJZOWdocEZQWFBhTllNR1ZBSEg1TWRXUWd3X0t6TVcyY05PM0pF?oc=5</t>
         </is>
       </c>
-      <c r="E42" s="15" t="inlineStr">
+      <c r="E42" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1684,7 +1687,7 @@
       <c r="F42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="15" t="inlineStr">
+      <c r="A43" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1694,17 +1697,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C43" s="15" t="inlineStr">
+      <c r="C43" s="16" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D43" s="15" t="inlineStr">
+      <c r="D43" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQbHdYM2pSM2xkdmZ3OHhQc2tVUmhzclJWaVJ0aEwtUkNBR0ZUd3p1emF1M21jbTF1ejlKSkdDMnotcVNjZE1CYUlKako3WXR4MTJhdWNlSXZMbTBYanlmTWFzRGFIandXRUQ3UjN6SEV1bThvZjN2bDY0eFdpaTdMODN6TGFTdE5rd05TUll3MmNfTDhkQldoNDIwVlpoSl85aVRwcTd5Ymh3TDl4enZhZ2p4OExGY1ZaOFNEWFBB?oc=5</t>
         </is>
       </c>
-      <c r="E43" s="15" t="inlineStr">
+      <c r="E43" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1712,7 +1715,7 @@
       <c r="F43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="15" t="inlineStr">
+      <c r="A44" s="16" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1722,17 +1725,17 @@
           <t>Sembcorp Picks Banks for $2 Billion Alinta Loan in Aussie Push</t>
         </is>
       </c>
-      <c r="C44" s="15" t="inlineStr">
+      <c r="C44" s="16" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D44" s="15" t="inlineStr">
+      <c r="D44" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOdS1aaXZjT2VnSDl2TDdzZ3NfRElDWXdUXzZQYjFQMEZJOGlpaE5CNGdQMlZ2UFVHbUtfOXF1ZVBReExrdF85M0RWLWlBY2Y5dlRtWVdXLWp0Y1VrRmF4UGQzVUhxaHA4UHd1SUdFV21QcVFITXFHRlhzekdSUS1PdHlYRjdUbUQydU8wSktKVHRJQ0NaWE9sU1l6YXhtSWtBd3RwTERacnV4VzB6YlFhUE1QcXNDVXVESFcyeWY3cGhHUkRJcDhrYUtpTEY2UQ?oc=5</t>
         </is>
       </c>
-      <c r="E44" s="15" t="inlineStr">
+      <c r="E44" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1740,7 +1743,7 @@
       <c r="F44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="15" t="inlineStr">
+      <c r="A45" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1750,17 +1753,17 @@
           <t>Navis targets June for $1bn-plus med-tech auction</t>
         </is>
       </c>
-      <c r="C45" s="15" t="inlineStr">
+      <c r="C45" s="16" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D45" s="15" t="inlineStr">
+      <c r="D45" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxPNHRXaU5tNUVkd2MtcTg5M0EyQllrM0owMkZobGxLaUJxYUN2MUg0ZkdKdzU2YmxfanR3QU53cHZzNDI1WXgzRUcxOE9EZlluNmtNRUUzTGJPRnpfVVVOeFM3bFRNQmp6VHFBdi1mTnU4UDBvOEpMaHZPNXFtdUIyTlhuRExIVElSeVRUMGxjU0k5VnVxaWFfd3htWngydlhuR2E5aTQ5VW1LS01ac05rMGZoVFdOZzVyTzFhUDVsYkNrc0VQZmhubERSaTNwelk3WEhYUjF5d2ptMktYeEhzOHpWazFQZXphd0xfUFdhbkVGMVR2Z1dtVtIB_gFBVV95cUxObEwzeHd6RmZtNUp2dXVVV0plOVQ4WlNqQXNJU0thd1BEWE8yWkxxVTZjTkpsVGxxWGxpQzN0OERZbk91ai1fZkdtc0JoM1h5NERLTVdDbVJ4Y2k4djdQcWlVcDF6NjMyVDQzZWMzUFZxWjVRWllMZHVSOF9jQ2U1REFfNUlhM2EwYloxb1MwSTJjODdWdlZwX2h2N0xiQWNhallHUTNPZEtLaXhsY3dBZy0xM1VITXhLUERXS1JxR0R3OUpBTVBPZ2dPZTRUTVpvbFBNMjFUSTJuWS1XLWdhUS11UTRzVTVqaEhfMDhqWHlTMlJGekU2QzJVcFdodw?oc=5</t>
         </is>
       </c>
-      <c r="E45" s="15" t="inlineStr">
+      <c r="E45" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1768,7 +1771,7 @@
       <c r="F45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="15" t="inlineStr">
+      <c r="A46" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1778,17 +1781,17 @@
           <t>ExxonMobil eyes New Zealand market exit</t>
         </is>
       </c>
-      <c r="C46" s="15" t="inlineStr">
+      <c r="C46" s="16" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D46" s="15" t="inlineStr">
+      <c r="D46" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxPanlvR1V1eVVpdmYxNVNGMnd6UjJFd0J6Zk9IU1lhOW1GbmVTcjY4QkJCYkl3Y3NOU25VRTBUekwtS3plV0NVdlZtOTZZRHJWZ0FVdDl3S05aMlFWeEZiYzdwYmQtVnJxZEw0NktHaFZMNlZkUC16empqRGxxMEhhZGwxRzVEek5FelB3aE9UWFhGQW42b21MRnJHUXV2ZGJYUXJIMnVFWGZsSnEwazNGNUdVcjVoekp0NEZCN1J3cTlaZldFa1pMUkJTbVZYeFljVkRqQmlZV1M2aXh0ZjI5dEI1NDB0UElPUERsbUljMlA3OHBnYmtJTXFWZWkyUdIBgwJBVV95cUxNWFBRQ05GUDdwTWJ2ZVFJUS00ZUh0QkpZQVNNcU9JYXRTN21sMS1VZTlOSTh2LVFuZHh6UVk2djlrdWFsd3MwcDFCNmhwUlVLTlpjVF8wSmt1YnBWRE9tNVpKQlk2YXJWdmwzZWlLX0xpaWxSMUpsX3ZjYXhmRmE2YlAtSFJGRG5pQnVmMnViQXlsVFV3OU1hZFVrY3ZITHQxcTR5UkZ5U1pReHVJMGZGM2FCZWliSFZQZmpVLThSdExWMW14OElodmVVSC05SUh1d1hBenJoY3BUZGxoM0NTbTExdERmM3pjZGd4VzgyV3BNOG11TElBQ3NsRGhtSEc3YzJz?oc=5</t>
         </is>
       </c>
-      <c r="E46" s="15" t="inlineStr">
+      <c r="E46" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1796,7 +1799,7 @@
       <c r="F46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="15" t="inlineStr">
+      <c r="A47" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1806,17 +1809,17 @@
           <t>PAC Capital’s Clayton Larcombe charged with assaulting wife</t>
         </is>
       </c>
-      <c r="C47" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D47" s="15" t="inlineStr">
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOLXNDU2xjMWpyeEZwWGwtZkV0TjNSbGtWS3ZidUo3a0dvV1hrTnJiVXBXSkJNWlhXYXFHZkNTa3g4a1ZfMjRPM3BtWTZUNGg3S09kbGI2TTRGd0Jkc1A4WFAycjlpVC1URjFvNnBraWprRkhaT0VOWkh6N0xkUjNXNUw0dGx2N1JtTDVsREdtZDhraXVsSkxhR2ozamFUSGR5VHBBRm1Zcmx1c2RDaUIxQkVpeUpfWjFNeTRLWVRtYjluZ3ZncGZIMQ?oc=5</t>
         </is>
       </c>
-      <c r="E47" s="15" t="inlineStr">
+      <c r="E47" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1824,7 +1827,7 @@
       <c r="F47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="15" t="inlineStr">
+      <c r="A48" s="16" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1834,17 +1837,17 @@
           <t>China touts itself as ‘harbour of stability’ to global CEOs</t>
         </is>
       </c>
-      <c r="C48" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D48" s="15" t="inlineStr">
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPUzBWeVk0elBOZ0l5QU44TUJvU0RvSmtPdmVyT2VuQTczaEdzbkktT25ZT2Y0Nzh0bVBhQW96TUhpWkdEOEJMVVk2UWxLOENKZGk3X2tQcDNsWGZtU0JkM2U0N3VfUWFBclhUSUZya0NwRTJOWmZJdWlhT3JtY1EtSkJ6TmlsV3dzOXpDaVFMNlBaa3RfRHBjc3Q0cjk0eVdPV2MwcjlHNA?oc=5</t>
         </is>
       </c>
-      <c r="E48" s="15" t="inlineStr">
+      <c r="E48" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1852,7 +1855,7 @@
       <c r="F48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="15" t="inlineStr">
+      <c r="A49" s="16" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1862,17 +1865,17 @@
           <t>Eyes on 3D Energi as oil and gas giant Conoco flexes buy-out rights</t>
         </is>
       </c>
-      <c r="C49" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D49" s="15" t="inlineStr">
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWVU1QmhTUGFkYlpTQkw1WUFPTHhmbk5lbnE4T1haQUswSi1ITHlhVmhyM3ZYS3N4cVd6ZkwzdGdhT1lvM1JJek4yLXFpSWoxUnRtR2JRLTZWa2dlTDVTakE3b2xvazFWX0kzRHFZWVB4OUh0XzFFd3JVSVlfelpVa21qTldCVHdvcmJYcGNjZ1RrdElWS3Yzck9KYzRvbzloWkNqMnQ3dmtHbzNuc21ZSXNYeEFlZw?oc=5</t>
         </is>
       </c>
-      <c r="E49" s="15" t="inlineStr">
+      <c r="E49" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1880,7 +1883,7 @@
       <c r="F49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="15" t="inlineStr">
+      <c r="A50" s="16" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1890,17 +1893,17 @@
           <t>Blackstone tempted by $900m payday for Sydney’s JPMorgan tower</t>
         </is>
       </c>
-      <c r="C50" s="15" t="inlineStr">
+      <c r="C50" s="16" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D50" s="15" t="inlineStr">
+      <c r="D50" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxQNEZTZjY0S2YzcUxsb25RSDk2NHd1N1VOVlpMbi1JNGEzbUt5ajlYZFhvLWNBTkNQVXNuWERfTkl0Z2o4R1U0Zk5jVE1FTW5TTUJGZnNJc2NqMm1fT2dmYTVwRGU2TkZ0c3BjZVBGS29fWFJvZ2F0MWNLa0pYY0RNME5xYS1vOGZmMDVBcDBaLV9MWF9od0EwekFyb0ZCOEdkNTFaN3ZXckJwd25zS0FsdzU4OW1UODlueGNyZVBDSDZkeHQwelV5ZXVDVlcyUkhKWDZfVlRacEJHSElmNnhKSXk4ZHJHWHhPTEV5NGNkcmhyU0hjV3J4dVBXbnRGQdIBgwJBVV95cUxPME4ySFF5RWNrejVlWW1yeW56N244RGpyeVJUZEgyTjFNcE10YjVpMmJyeWsxTENzZFhPRlpsbl9pVXl0NGJvUlZFT216NE1KRFNwOHVZVXMzanNKNXFmWEdsMndsd1cza3NTTzUyUUZfaDEyWHJwZEtQbTdJRmkyU3A0RGh4QlAtT1lRVXk2SGoyaTI1NUpwVExYSkZJNmVFNjdXTDJTNURFOEh4Y1dnUDVGdjBpaDlWVWJtUHZiRDdGTmE5R1R6TDBwWFFnT2MwQ1lmT2w5bDF6eVU0R20tYnpnT3JCZlJod2s0UndyZTM5M2xLZC02a3E0NmJRdFV0Qkow?oc=5</t>
         </is>
       </c>
-      <c r="E50" s="15" t="inlineStr">
+      <c r="E50" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1908,7 +1911,7 @@
       <c r="F50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="15" t="inlineStr">
+      <c r="A51" s="16" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1918,17 +1921,17 @@
           <t>I-MED attracts mystery suitor as Permira weighs sale or IPO</t>
         </is>
       </c>
-      <c r="C51" s="15" t="inlineStr">
+      <c r="C51" s="16" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D51" s="15" t="inlineStr">
+      <c r="D51" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxNaGlwS3d5MGFMbEg2U2hnZUxMQmdqaWI4bS1lblNZOFhkSnRMcUotRkZMTjhFZkRUQWxUUDVtYml6TVAxUXkyZmx3SHRFb0gzVHRST2ZQUThKa25aWlhlcGprSU9tWktXZjZRaC12bFpkaVVWZHhIMERyeVNNWEswYTJ2ZHdnRFVRaFhod2U5N011TkQ0NG5MYVhoT3MwRUVZdVB2UVhKZExvdFIyXzNNUGt2SHJUanQxRkI3bXlLSlNJQTF4NXQ1YlZDaGVBM0EzNUhYQVp6NkFWRzU4bnRPWTgtXy1HVnB0ZlN0Uy1rY2FuWlNfN1U4WXVHQnRzVkNG0gGGAkFVX3lxTE1GaDJJdTJlOXFEZUtDTmdXMmsyLXlpaUxzQXpycHk4MTdHZng0dVczYWVwdWRzdFFCMlNLWkZpMm5Zd2RpN0Y0Zmo3Q1FOZFBZQlh5LVl6aVZ3X284UmpxM0pVRzZmMmpjaUdNWnJPZGV4V3lNai1CTllCcW5oUEVxaG0zejB5anc5YnJEZzZPT2d2QklCWjl2MjRBc25jUndqZkVadllKaUZScG12bEozT1NKUUJYR0pHTGtJZVc0ZHZLNHVSYlhzcTE0SkZmMXNlVGJ4YWJ1cThxcGlZTDMzRUMxLVM5VHh2OW5tRW1PT3VyRUhDbV8tRzUzVzRzVWZPZ2w1bnc?oc=5</t>
         </is>
       </c>
-      <c r="E51" s="15" t="inlineStr">
+      <c r="E51" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1936,7 +1939,7 @@
       <c r="F51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="15" t="inlineStr">
+      <c r="A52" s="16" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1946,17 +1949,17 @@
           <t>The stagflationary mix that has billionaire Solomon Lew worried</t>
         </is>
       </c>
-      <c r="C52" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D52" s="15" t="inlineStr">
+      <c r="C52" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D52" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPWTh3S05XQWpTQm03WjhBT1pWc2cyOFRMd2ZraHhPUHlDRW1tWkZvdkhQWHE0MHVMRUpaOFRoX0JsYWhJV21nVkpIM2RBSmlZRUtEbFAydzZfOTh1S05oNEZPOGgyZDJRMS1uLThWYWRVT3VEVGhtYkVLN3J2OWsyX0VVdTUteFBCOVNKZ28xUTRPTk1SUkMxZ1NJc1B6NXRrUEEzOG01YnZOYjk2cWlFZA?oc=5</t>
         </is>
       </c>
-      <c r="E52" s="15" t="inlineStr">
+      <c r="E52" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1964,7 +1967,7 @@
       <c r="F52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="15" t="inlineStr">
+      <c r="A53" s="16" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1974,17 +1977,17 @@
           <t>Oliver Curtis on Firmus: From prison barber to AI billionaire</t>
         </is>
       </c>
-      <c r="C53" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D53" s="15" t="inlineStr">
+      <c r="C53" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D53" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQek9VTlV1b2hVb2RoZ0Fya0REb3E3YlBCR2NYZldXcEh2VEY0LXg5bjd6RzlnZDI0OUJJd2cydTBwTm9tdHpiZ1lSMnhtcmJSYVRKbzJFMjdDaEJyZExSQVJVRDh1c00yMjFMaVlPdnRuV3VkTjNxdzFRbW1yeGltSF8tVXlJVXJzTEJXS2FTYkJTVkdKbmdPTTd6YzRtYV9nN0JzOVZNTzhUdUk?oc=5</t>
         </is>
       </c>
-      <c r="E53" s="15" t="inlineStr">
+      <c r="E53" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1992,7 +1995,7 @@
       <c r="F53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="15" t="inlineStr">
+      <c r="A54" s="16" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2002,17 +2005,17 @@
           <t>Three startups that raised $161 million this week</t>
         </is>
       </c>
-      <c r="C54" s="15" t="inlineStr">
+      <c r="C54" s="16" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D54" s="15" t="inlineStr">
+      <c r="D54" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNRGVZMF9DeGJjX29vN3B0blVoM3RKSlJJTllrMThKUDJNZzdPNFNnT2JyTElUOUYxMHlsUm9yM2dBQnZfaVNZblpqb3NzTXdHVlpQNkRqR3NBZHdzODdjN3RKMTZhSVRqUEM5d3JRc3F2OG9hWmZJdU5rakg4ck8wLXlMTnZSU0lNaERmQmswbkVGWW8?oc=5</t>
         </is>
       </c>
-      <c r="E54" s="15" t="inlineStr">
+      <c r="E54" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2020,7 +2023,7 @@
       <c r="F54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="15" t="inlineStr">
+      <c r="A55" s="16" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2030,17 +2033,17 @@
           <t>Iran eyes ‘plenty more’ vulnerable energy targets in costly war</t>
         </is>
       </c>
-      <c r="C55" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D55" s="15" t="inlineStr">
+      <c r="C55" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D55" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNLUN1MHlZaTNfVHhVX0RnTXp5QW83RmM4WVZkWW1PSnNaZF93VkY5ZF81anB3NDNmX0kyMkVSdkxNSURvSEh6enloWnRVcTlsR0JPTjVzNFR1YjRsSm52VnA1XzFFUlUtODJjYy15YWRRdWZZRkdjRXpCcEFSVURmV3VpSTFhTjVUb1d5bmw3NHNlT3VQZU9ieEYwM1J1TGEyZnlnWXNIWFJUMEtIOVZad0dxRWZBdw?oc=5</t>
         </is>
       </c>
-      <c r="E55" s="15" t="inlineStr">
+      <c r="E55" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2048,7 +2051,7 @@
       <c r="F55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="15" t="inlineStr">
+      <c r="A56" s="16" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2058,17 +2061,17 @@
           <t>Don’t take it personally: Bain Special Sits hits hurdle at Infinity</t>
         </is>
       </c>
-      <c r="C56" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D56" s="15" t="inlineStr">
+      <c r="C56" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D56" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQRjdwTk0xTHVIRHNkdG9tVk1EQ0hiQjJ6dGcxaWZRZ0hZV1U4YjJDU0tnTUlWSkQ1S2dUTHJVNk0tNWQ2cVd4dkw0M25leXRreWJtdlBKYTAtNzRocTJUazh1dnRzSVlYZThySTBNVjg5X0xYWUxCMC1SelltSHVSUEV5U3B1bTA2NjAzMGFZLW1CNkQ3aWU0S1JxS0d0YmZiZjBKQVRNVUpzYno5R1pvbTBsaTM?oc=5</t>
         </is>
       </c>
-      <c r="E56" s="15" t="inlineStr">
+      <c r="E56" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2076,7 +2079,7 @@
       <c r="F56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="15" t="inlineStr">
+      <c r="A57" s="16" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2086,17 +2089,17 @@
           <t>Drill, baby, drill: It’s boom time for mineral and petroleum explorers</t>
         </is>
       </c>
-      <c r="C57" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D57" s="15" t="inlineStr">
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D57" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNdlFOWld5ZWhPVnFRa2xidWlUVzluQzkxUTgxR0t0Rmg2S1BzNjdINnhwS3VLRkNjRVJLX0RHU0h4VFVRY2RfSHBudEhfNVNjeE50ZUxQenJNSlJtWFRlcnNsZm1iLXlxM2RmVDViWEtjNDloaTBhUDVxYkNfOWFCTjV6cExEVlFCMzNfWnVwRDJHYWxWV0hOR2V2S0VlV2NyS2s5cWNmREtWXzlMMDRQNW1tVlBOblp3SHBEVg?oc=5</t>
         </is>
       </c>
-      <c r="E57" s="15" t="inlineStr">
+      <c r="E57" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2104,7 +2107,7 @@
       <c r="F57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="15" t="inlineStr">
+      <c r="A58" s="16" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2114,17 +2117,17 @@
           <t>‘Wake up’: Fury as farming crisis looms</t>
         </is>
       </c>
-      <c r="C58" s="15" t="inlineStr">
+      <c r="C58" s="16" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D58" s="15" t="inlineStr">
+      <c r="D58" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNelJvMXFPX3MwUVRMN2xqbzE1MWdvOF92Zy02YmIyZW9SQXRNQVZsS0xVVG9UdkFPaTV6ZC1tV05SZWNqblNFZ3Y1VGNaVVBaaEl6aFJqQ09ONDVkNUs4TzNvVjV5eHNjUk9xaDRFZTM0alpuYUdvWGtLRzRhYXN5alZ1QWdsZTEyODdQVnZoazkya29WeTJZVmpxLVBCdWxfY0dTN2Z3WFZlSy1sVW44RDlvZFAzYlhnQ0N6UWhKSU02eF9iZllIU3g5MWtSbkJzZGxWLUxHNERzdUlLTF9VYmpJSTRLY3U4NlVVaDhmc09uOWwtUGtlb0I2M05DR1dnRWxGSFV2NEJXaEF4c00tN9IBlgJBVV95cUxOSzZ5NXZMTTlZa3BSNjZyTUxUMjRhYWJhN0hMa3dDcW9CWGstNnI5MzV5U0hJSTdKLTFwa2E5YUItZnFRbW5RbzVuYW91MmZaYXN3R25hWVpUbW9oUU9fVktPRHROVDYyd2dSLXJVZWQtY016bkVxY0VPbkY3Zkgtb1liWGMxeEpyYmloS1V0TVJMMWZaeWRZX3FQRjBmVzJwdkkwMEVDSXV1MTdReUhGZ0Z3dENyMEFkLUl1aXhtRkFLRFFXcEdMZzFuT3NxRDFMOGVaY2YzeXBQc09fY3YwcFp4MVczRVN3d3dJZWJfTFFscjF0cUtRWHdzTUptaHowNDhYWXZXTHhYTHNTdlZGUmNlamRTdw?oc=5</t>
         </is>
       </c>
-      <c r="E58" s="15" t="inlineStr">
+      <c r="E58" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2132,7 +2135,7 @@
       <c r="F58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="15" t="inlineStr">
+      <c r="A59" s="16" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2142,17 +2145,17 @@
           <t>Construction giant FDC road tests IPO pitch</t>
         </is>
       </c>
-      <c r="C59" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D59" s="15" t="inlineStr">
+      <c r="C59" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D59" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxON3p5Y3VPM01XZFk4a3g0R3JnQkZXbHVGV3BKdDB6M3NRb0M0SEl3V0R5RmhCQ3dnaHB0ZHp5N2hCMUFsNU1ZNWZ4YWdNZWdETkUyZmdoeW81amwtTWNFZlc5WlNpMkJwRzk0QklORGhlLWNEalh2d0JCX0lhVHhhUF9ibVlxcHAwOW9ENndVOTY0enBYUWc?oc=5</t>
         </is>
       </c>
-      <c r="E59" s="15" t="inlineStr">
+      <c r="E59" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2160,7 +2163,7 @@
       <c r="F59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="15" t="inlineStr">
+      <c r="A60" s="16" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2170,17 +2173,17 @@
           <t>Austal suitor Arlington Capital Partners buys Eptec’s defence unit</t>
         </is>
       </c>
-      <c r="C60" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D60" s="15" t="inlineStr">
+      <c r="C60" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D60" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNM01qb1ZRZVBIdmp3cFc3R3RLaTdmZk1JOFo4anRtSm95Z1hJc0N0S3VranBTV29IdlViT0FkSm92eHdtbDBqdU5HTHNMaXo0dGRWMkpDdjk3LVRBVU1rZC1YejZJMkhyNmpZZFJodGoxWlB1dkRhYTJVRlljMlV0dUllQ3EtOHZkNFdSUWJLSW9Xemw1XzFzU2RHV1o0RTViOXp0bDZFQTZycWhpNElLU0FZQVI?oc=5</t>
         </is>
       </c>
-      <c r="E60" s="15" t="inlineStr">
+      <c r="E60" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2188,7 +2191,7 @@
       <c r="F60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="15" t="inlineStr">
+      <c r="A61" s="16" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2198,17 +2201,17 @@
           <t>Eyes on Tom Wallace as clock ticks on Adgemis pub deal</t>
         </is>
       </c>
-      <c r="C61" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D61" s="15" t="inlineStr">
+      <c r="C61" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D61" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxNSExQeDlENWlHb0prRnRldjZ5YWhKVUZ5eVdsYjZmbVRWRWQ0WnZXWkU3UHZJdElnQ21jMU9zNnhnc3JlNDczVGQ5Y0FGV2J3QUp3NXdZTXZMNm5tVC1vWDFtOFN3aS04QVJZb3FZV2VsUmJ2aVgwbUhTaFVGdHg0UjRyTXVVUnFhQmE5eFYwMGR6T1R2U3Q3WEdZclVKNWJiby1IRg?oc=5</t>
         </is>
       </c>
-      <c r="E61" s="15" t="inlineStr">
+      <c r="E61" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2216,7 +2219,7 @@
       <c r="F61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="15" t="inlineStr">
+      <c r="A62" s="16" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2226,17 +2229,17 @@
           <t>UBS names head of APAC leveraged capital markets</t>
         </is>
       </c>
-      <c r="C62" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D62" s="15" t="inlineStr">
+      <c r="C62" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D62" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNMm9WZ2ZKVFBvX2pYMk16VmY1WFZnZ2J5N0F2bHduTVM0Sjg4STVtTGFLQVdzeFloVHg3clRic0owTDMwYVpXdDVjdjFOWjQxdkdxdFY5MEY1Q1U2Q0R5dFBJWTNtUzgyd3RXcm9uM0hKdEZ3b3JjXzcwQ2VpRm5SS0hYT2gxSU9iVFRlR05Xd2EtM2JOQjBGUzlKdnE?oc=5</t>
         </is>
       </c>
-      <c r="E62" s="15" t="inlineStr">
+      <c r="E62" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2244,7 +2247,7 @@
       <c r="F62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="15" t="inlineStr">
+      <c r="A63" s="16" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2254,17 +2257,17 @@
           <t>BHP, Woodside rise after new CEOs named; Future Fund chiefs exit; Sandilands ‘doesn’t accept’ termination</t>
         </is>
       </c>
-      <c r="C63" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D63" s="15" t="inlineStr">
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNUHhZeHNHemtiLW1IOHN1OTZXOGpsM0ZtUG1MVHRCT1hUT1k5S2lEOXlXRENWOXNlMEZadThQR18xSTJfTVlQM3BtX0ptX1J0bk80SzNLUVRtbkJITGgtb0lsSVdJTWt2S1E1WUlXdUdsbEV0V1RpNWlyRXBoc0dPVDl1OXRrSlM3SHlDazg2UlcxenVzNzlhQldhUGhfNE5IV2xrVmVBNzhhSE9qY042Z3pzMEVzd0VyVmZudXgxcTgwWGJXSWZKZ0FyNVhjcmhjTm5DYUVjLUdDRmxUQkZuTDFlUXVaV0ZoSWp5WHMyR3c?oc=5</t>
         </is>
       </c>
-      <c r="E63" s="15" t="inlineStr">
+      <c r="E63" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2272,7 +2275,7 @@
       <c r="F63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="15" t="inlineStr">
+      <c r="A64" s="16" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2282,17 +2285,17 @@
           <t>BHP’s new CEO will shift the Big Australian’s centre of gravity</t>
         </is>
       </c>
-      <c r="C64" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D64" s="15" t="inlineStr">
+      <c r="C64" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D64" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPQnZpWndNZzZvN1VsOHBmRDVLRHVTNkxLeDVDelpOMURjOTRDSDZfN2dPZlZqaW05WEZuZXMyRTJZeVZnV0poT2UxRkVfZ1RZSjdvUjVKblhoSU5Cd1plRTVNNTRaNWZmbm1yUGZkblVpYkctNzVRRkVQQm4zX1FtRG1KV2Y0djUtOURianJ3dElqeXBUMFp4aWFEWVFYelVjYTluSWpOM1FlbHpIaUxXdnBn?oc=5</t>
         </is>
       </c>
-      <c r="E64" s="15" t="inlineStr">
+      <c r="E64" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2300,7 +2303,7 @@
       <c r="F64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="15" t="inlineStr">
+      <c r="A65" s="16" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2310,17 +2313,17 @@
           <t>How philanthropy became the sandbox of succession</t>
         </is>
       </c>
-      <c r="C65" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D65" s="15" t="inlineStr">
+      <c r="C65" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D65" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxObnBPb2MzQ1RvSVVCbmNzYWFBMlFjU0dQRmpPakNfdkxtMWc1bFdVNXNlZmRKQnNlWEtUUDNSTHpTLVV4Skx0V2otbTZsTTdvT1VaUDhMZFZoMFFab1RoS2pCcno1WGlNQlY4eXQ0OFEtLXJTay1MUkFSSEJ2MVVScUpjUkhJOThISy1QbHIzTzFlWVhOc29fWWs0V19sQ25hRW9MSGhBVVNKWUp6dUo3NS1SWlk?oc=5</t>
         </is>
       </c>
-      <c r="E65" s="15" t="inlineStr">
+      <c r="E65" s="16" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2328,7 +2331,7 @@
       <c r="F65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="15" t="inlineStr">
+      <c r="A66" s="16" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2338,17 +2341,17 @@
           <t>Advanced Navigation raises $158 million Series C round with NRFC backing</t>
         </is>
       </c>
-      <c r="C66" s="15" t="inlineStr">
+      <c r="C66" s="16" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D66" s="15" t="inlineStr">
+      <c r="D66" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNTXhwVlVLUy1pWEpFdzFCazNTY0dkczd4WW9oeW14cUtTaDZRTGlVQXBPaHN4WTBkNW1zOGxvN0tVWl9JSFdVNXlQMzVxbk4zbDZFUjNOcUxSamNaSnFCckMzWEk1VlNoSHJHQ3VWdGltVWZCV0c0NmU4UlN6YU55Q0J2TkQtUzBzOW96UXRxem5Zb3M2SUljNURISlRkQmJD?oc=5</t>
         </is>
       </c>
-      <c r="E66" s="15" t="inlineStr">
+      <c r="E66" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2356,7 +2359,7 @@
       <c r="F66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="15" t="inlineStr">
+      <c r="A67" s="16" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2366,17 +2369,17 @@
           <t>Kal Somani-led consortium buys Rajasthan Royals for USD 1.63 billion</t>
         </is>
       </c>
-      <c r="C67" s="15" t="inlineStr">
+      <c r="C67" s="16" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D67" s="15" t="inlineStr">
+      <c r="D67" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOX3lmdG5aTmk4TEpBa3ROdWZ1aDJHUElBQXktVmlKaHFmTUhPX1QxX1dKLXZfaHRDQjBnWm9McTZjTjJtTWFETTRNMHgzN0tTTm1xY0JpMF84Q2lNaFQyZGVjaHN4bkVmcDN5Qy1ta3FtYnpMSVVyYm0ydWpTRUdZU1hoYXpaNkZUQzlPc1QycjZ6aG5QVHRqY213?oc=5</t>
         </is>
       </c>
-      <c r="E67" s="15" t="inlineStr">
+      <c r="E67" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2384,7 +2387,7 @@
       <c r="F67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="15" t="inlineStr">
+      <c r="A68" s="16" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2394,17 +2397,17 @@
           <t>KMD says Rip Curl demerger proposal delivers investors ‘no value’</t>
         </is>
       </c>
-      <c r="C68" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D68" s="15" t="inlineStr">
+      <c r="C68" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D68" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPTXhBdHByWE9EbllFdDA2OW1UTUZEMVJfV2xsNFdURFRKX2JrODJReVRuQlFoakpWbTBKcjhNLUVsNE9sdG5LUElLZlVrbFNERS1QZTN6bEZIWEhXZ1pTWG5GWEw3ZmNETTdDUDUzYzR5M0E3ZGVlTWpSUnVlVU56dDNFZUtZN3liZ1dKNzJhLWU1S0M1ZnlKd1JNWXlxSlkyU3pGS1lhS05hTUJPRkxucldabzFucGs?oc=5</t>
         </is>
       </c>
-      <c r="E68" s="15" t="inlineStr">
+      <c r="E68" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2412,7 +2415,7 @@
       <c r="F68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="15" t="inlineStr">
+      <c r="A69" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2422,17 +2425,17 @@
           <t>Ex-Macquarie banker drives mortgage broker roll-up Recludo towards IPO</t>
         </is>
       </c>
-      <c r="C69" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D69" s="15" t="inlineStr">
+      <c r="C69" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D69" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxNQms5X1F2aTNhOExDbW42TlZOLVJwVWxna1JYSW9vWF9Na1RZa1ViTFdZc0tCcXRZZkRudTlsTzNuZGgwSENyYi03Zjdfc0lZTXp0NmJRZnhzb2pWRXRIOUdJN2lQM2h3ZFFtTXlSWHVWOFBIaW1Na3FQMjBCck1nVlhUcmRkLW9LOHpKWXQwTm9LcWR5M2FfdjFiRW04TndoanR5NmJvMENGalNuUGNINy1Qc20xR1J4d21ncHNNSUZqa1BXNnI4STIxSUFkZXdU?oc=5</t>
         </is>
       </c>
-      <c r="E69" s="15" t="inlineStr">
+      <c r="E69" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2440,7 +2443,7 @@
       <c r="F69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="15" t="inlineStr">
+      <c r="A70" s="16" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2450,17 +2453,17 @@
           <t>Coles reviews truck fuel charges as crisis worsens</t>
         </is>
       </c>
-      <c r="C70" s="15" t="inlineStr">
+      <c r="C70" s="16" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D70" s="15" t="inlineStr">
+      <c r="D70" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxOSGpBM3RjLVJ3LVlmR1QydnY2dm50WlVxcG43ajRFZ25QS1hDNTBONU8tY3Z2TklzbUNla0ttZk1GZzFaLUZRakFjSUpUQWItQ0VqVTVwS1B0QS1ObVEzNzdRT1l6aU9pVm5jSlhna1N6QmFKT3k1RkhMZGNTVnVLcDVIcXZmRjdjLWRpYVlRQUVmcVRtM21BSjVhTGNaaThyZkhLS2NWdkNCSkZKTlloUVdtbzRnYjFKbllOZXhOd3lkcFZEYURwUFVNQzVnSWRyM1RlOGd2M1pMZXI3c0NIa0Y0MNIB6AFBVV95cUxNSjB3Z0hoTGxwOHJQQ09xb3BmRmhCYjBCc2E0OHA2elFDRE45UGpaTEVDc1Y2VnRvVmZQUzRHbng4QTMwNGZZNGpmaVlHRmV6bnhiZ0FReU50TnRiQ0NZMEtoM3dBZ0hXbFBZMVJQNXd4LVdXRDVyTDAxNS1zeVdvcFVvend2N3J5R2pLYmhxNVFfd19rUlRsNWNndlptMUVkcS1CaUN6UXRHVzByTU5BMW1TdktOZUJYck5xMEJucmR6czIySEMycDA5cmR1MXB0N25Xc0JDUG9zN29YWklVc1BUMzl3UVhn?oc=5</t>
         </is>
       </c>
-      <c r="E70" s="15" t="inlineStr">
+      <c r="E70" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2468,7 +2471,7 @@
       <c r="F70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="15" t="inlineStr">
+      <c r="A71" s="16" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2478,17 +2481,17 @@
           <t>Sam Arnaout’s Midas touch turns suburban pubs into pokie gold mines</t>
         </is>
       </c>
-      <c r="C71" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D71" s="15" t="inlineStr">
+      <c r="C71" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D71" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQV2xlTTdYOFpIMzNmVVRnMlJRbTdGTC1jelVCd1V3UjN5cHQ1VzhWZzhrNW1PNm1RX3FlZmU3UkRycjF4WDlQUzRMcVVYY1g3UTZqQ0hxRnl2Ti1IQ0owVmZjN3Jod1BFbmhPVUwxNjhsTGh6d0kzdU01N0hmempRZ044ZmZNUllnenhyc3djRGJOdEtrekx5UVFoaFFMWDdqMHMwdng1SFg4TzZHY1hQNFJNN3huZXpWYWFtQ0ZJakhkVFlQcl9SQlRfZkQ?oc=5</t>
         </is>
       </c>
-      <c r="E71" s="15" t="inlineStr">
+      <c r="E71" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2496,7 +2499,7 @@
       <c r="F71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="15" t="inlineStr">
+      <c r="A72" s="16" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2506,17 +2509,17 @@
           <t>Gentlemen at Melbourne’s exclusive The Australian Club sweat another election</t>
         </is>
       </c>
-      <c r="C72" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D72" s="15" t="inlineStr">
+      <c r="C72" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D72" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPcEwyU01BOXF4TzlmREhYbTFEWklxdWZqWmZybDVnOWtLQ2dTU2dNQ2t5M3BVT2stN08xYkFmazVkY29oT3RVc2xUZmZINFJURGtIRTg4RGsxOURBdWEybTUwU2NUODQ2eDNBbTdPT3QxeXRFNHlSc014T0g1aG4xZ1A0U0FWMTB1Wm1CSHlQU0ZJb3lMYkE?oc=5</t>
         </is>
       </c>
-      <c r="E72" s="15" t="inlineStr">
+      <c r="E72" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2524,7 +2527,7 @@
       <c r="F72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="15" t="inlineStr">
+      <c r="A73" s="16" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2534,17 +2537,17 @@
           <t>Inside Fortescue’s AI ‘hive’ that could save the mining giant billions</t>
         </is>
       </c>
-      <c r="C73" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D73" s="15" t="inlineStr">
+      <c r="C73" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D73" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOSVVCbGpzcVcxTGlZZ2dTUkxXdVVvVU1ONEtUS0t1R1VkWWRNeUF1UmlHbXd6clR3QVRuWGxrUGQwVG1OeUxZb2RqTzdYOEVGQ1N6eDFta3VOZDdHNThYbUEwWEVHZlZBVzNpZ1Foak1kLURZTWpJVzZLekczdzFrdHMtLVZwMUZnYmkxSVc0czFqWnFaSGZiT2pIVW5rdVZmdThreFlRZWVEU0xoa1VFOV9MTjE2UHFOcWhqUzVB?oc=5</t>
         </is>
       </c>
-      <c r="E73" s="15" t="inlineStr">
+      <c r="E73" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2552,7 +2555,7 @@
       <c r="F73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="15" t="inlineStr">
+      <c r="A74" s="16" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2562,17 +2565,17 @@
           <t>Tiny house maker Elsewhere Pods seeks cash after Bunnings debut</t>
         </is>
       </c>
-      <c r="C74" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D74" s="15" t="inlineStr">
+      <c r="C74" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D74" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM0ZpVnBTS21Ib25qa09CaU52Z29kZWhTU0FJLW5VR2JCLVFPTVlZTmpYX3lZVWdtMDVTYTJkWHlPUmhXa0Rua2ZXTTBWQU1VdmFrV21KOGlrdjJ3TTdxbGlvZVBUZUxUWE1uelpWMGxWWk04UndJTXVKQjBZUEtoX3lodmdpMWZKNUc1YTIxVFZLYkFKT1QwbS01WU01ZUZTTlczY2ZpLXlpTjNJTWpsUg?oc=5</t>
         </is>
       </c>
-      <c r="E74" s="15" t="inlineStr">
+      <c r="E74" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2580,7 +2583,7 @@
       <c r="F74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="15" t="inlineStr">
+      <c r="A75" s="16" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2590,17 +2593,17 @@
           <t>Chinese consortium emerges as dark horse in Made Group sale</t>
         </is>
       </c>
-      <c r="C75" s="15" t="inlineStr">
+      <c r="C75" s="16" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D75" s="15" t="inlineStr">
+      <c r="D75" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQYlpEY0hxNm5lalIxSTUzbDE4UEF5QTNpMTl4dWNPMkRrMU1yQnltZ25WcUkwOU13V2Y2RGItVW5QTXotSnBZRUJMdGJySGw0NVVxc3ZLZmVEcTlfU193Vkd5UVVuTFVYWFNtd185eGlVQW5RRElHdk5pMjhUR24wd1k0T0I3cW9qTG5Lcjg2bV9aNWsya0FYODRjeURyMW1EeHdYT05iZHZhLVFrUVNoV25idnZYZ2lpZEhta2JxOWFJb0M2SE9hbFF6NlVWYTM3QmF5anpWOEZackZiTDBfN2gtX1luQkxFOUxSSNIB8gFBVV95cUxOQklMYWl1ZkRqZGUwN0ppeXFubzZWNTNmeE5GY1BfcS13N2dFT096YW9JSndVX1EzTlBKdWZIemdKZnRIME9SQk5aT1M2WnRESjJxckFTaUdOSEd6eG9hRVBjdlhBbWQyWGpUS1kwQXJsdlpkLXJpXzJZX2xiUC1FSlNnNTFoVXQ4bF9JeUp3UGRWdUFOUVRrNUtsRzRxaUczb1p2LVVucFBNazhuZFNDaUZDR2ZQUVdObmVtTnBndGlkazZqeHVheVNzSE9RY3Bad0lrckxDSWY5QXBWS0hwVzZvSTZjaGEtNkNncW1RRE5uUQ?oc=5</t>
         </is>
       </c>
-      <c r="E75" s="15" t="inlineStr">
+      <c r="E75" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2608,7 +2611,7 @@
       <c r="F75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="15" t="inlineStr">
+      <c r="A76" s="16" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2618,17 +2621,17 @@
           <t>KMD faces uphill battle in capital raise as key shareholder baulks</t>
         </is>
       </c>
-      <c r="C76" s="15" t="inlineStr">
+      <c r="C76" s="16" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D76" s="15" t="inlineStr">
+      <c r="D76" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxOVTU0OGNfRURNcDdzYUtIcG8tR3N4OFFYalhKNWJBaUd6ZlQwNU5MZVZYbUZVSzB3WmdOOFdTZHlBOXBzSGdYUVV6eGt1UndHN296bENxZzNUM2NoaV93LXZaZFNNOXJ2YlA4RHNFS2FDb1ltNWpPWUdRR3VGMWoxaU5qYm9VSW9yUW5kS1NaN2RSc2YtcHZRSTB6aE9Zdkl3NG5nbVRzODRfQVYtelo5M3g4R2JEbnpraFpWbENOZzE2Qndla2t3MXRPWkU1dXg4NmZRME1jT3pOOHZOVlpTZGloNENUZllaSTFmWUV1Y2JLck02ZDhnTHJ5bUPSAYICQVVfeXFMUEFXR29tQjlTbTdMRVNDWUlGNFNOQjVhX0FiSkl0U2stbml5VHR4d1g3bDFqMUw2TzR1eHhYOU5ZUmJpZ2xBY2NzcmJRX3MwaEQ0YmpzMUFnV1BQNGxmcnlXUzVvbHpwNEo5dWFnZlduZ0Z2dGZGRFRKRTNCUzctZDNCd0FMNEkzTm84dmZOM2NKYk81RERsVnlZN1VZaXp5TW5QRVAzOHNXQTFWdVlKdGtFX0FmcU1EbElZSm52alBQeWx4VnlvOFRwNk1ia2lZYXlpemQ4cFdmckotMmMyRGE4ZXN0dThQYmxxUkpvMzAwRXBBcVJuRnp0QkZ3b2tqMWF3?oc=5</t>
         </is>
       </c>
-      <c r="E76" s="15" t="inlineStr">
+      <c r="E76" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2636,7 +2639,7 @@
       <c r="F76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="15" t="inlineStr">
+      <c r="A77" s="16" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2646,17 +2649,17 @@
           <t>AustralianSuper claims another listed M&amp;A kill with Pepper Money</t>
         </is>
       </c>
-      <c r="C77" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D77" s="15" t="inlineStr">
+      <c r="C77" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D77" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOY0RwcnpWZlhfOHA2MG13MkJUX1RDNF9wN2RxZGU2cEpzS1RKTjJDeUl0OERFOGhFRXJaSXNETEhHbW9PS0lua283RnFVbHJvTlRva0djQ2lRSGc2RENJYmt0OEsyYTRVSzFGeE9jWVhKMVRnd240WXVNTVdac2lOUGJSZlc4UVZ5RXo0OTlQbUd6NWRSek1HZG9fZGk2aDhDelhGVmk4YkRKeVV1M0VHZ2hZNmFVdXM?oc=5</t>
         </is>
       </c>
-      <c r="E77" s="15" t="inlineStr">
+      <c r="E77" s="16" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2664,7 +2667,7 @@
       <c r="F77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="15" t="inlineStr">
+      <c r="A78" s="16" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2674,17 +2677,17 @@
           <t>Apollo to Acquire Nippon Sheet Glass in $3.7 Billion Deal</t>
         </is>
       </c>
-      <c r="C78" s="15" t="inlineStr">
+      <c r="C78" s="16" t="inlineStr">
         <is>
           <t>Wall Street Journal</t>
         </is>
       </c>
-      <c r="D78" s="15" t="inlineStr">
+      <c r="D78" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOanpORVBremoyamJyZ2FqQWVOcDcxa2NpempBUmNYcktMLUl1Mzg5VDloWmlVbUdNUnplVk90WEUzXzJjNGxENk9LcGF0enVSdlFpWU9nd244YWNTS0ZHd1JTZEtlbjRQTmJUU0dzWmlDOVFhR1ZRSFJkNXN4a3FHdGozcUcwdHRseXpYMFREUzBNcXRmQ1VCN056SWlEa1l5VVE?oc=5</t>
         </is>
       </c>
-      <c r="E78" s="15" t="inlineStr">
+      <c r="E78" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2692,7 +2695,7 @@
       <c r="F78" s="3" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="15" t="inlineStr">
+      <c r="A79" s="16" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2702,17 +2705,17 @@
           <t>Estee Lauder in talks to combine with Jean Paul Gaultier owner Puig</t>
         </is>
       </c>
-      <c r="C79" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D79" s="15" t="inlineStr">
+      <c r="C79" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D79" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPSjN6QnFVbmdHWFoteURWaU5VaWZmRmpTT3QtYm1tZUFyNUZyLUdheGdfWlRBTlJyTlp4THIwVDA4U3BnWFNpT2FpZlZzX1lJSDV0MkRGVjYtNVc0b0lOQy1RSnFGTWhCTWE2ZFFPYlFQX05yaVlfZF9IUEN2ZWkzQ0VFMUxxdHF2ODNQY09xdWlqWEczSC1CZk5wYU9QQlAyaTMyelJnaVM0cmN4M0paNzlBdzM1RndoZE8yRHN4UnZqaXVhVmx5NFpqS3hmUHhUdlpF?oc=5</t>
         </is>
       </c>
-      <c r="E79" s="15" t="inlineStr">
+      <c r="E79" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2720,7 +2723,7 @@
       <c r="F79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="15" t="inlineStr">
+      <c r="A80" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2730,17 +2733,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C80" s="15" t="inlineStr">
+      <c r="C80" s="16" t="inlineStr">
         <is>
           <t>The Age</t>
         </is>
       </c>
-      <c r="D80" s="15" t="inlineStr">
+      <c r="D80" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPdUtyNWs5YmxJMXNsNWtaMi1WMm5SVHd6ci1ReURLajdYd1IzWGJMZmE2MzJsSzAxQWtSTm8xMUEwNTh4Vy1zTmFsWFBKTkJ0YXc3ZkcwOVk2a2VNRWVGUS0yQzZhSXlCWmpDYUx6RmpTTlNhS0xIQklyVFdIVXJRZTNPaVB4TG4yQ1R1ZWF2MWpmSG81TVRaRzdtMXpydWhBS2w0a3ZPZFI5MnFKOW5tN21oUDB3NkNtQmR4LVVBWW9BUQ?oc=5</t>
         </is>
       </c>
-      <c r="E80" s="15" t="inlineStr">
+      <c r="E80" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2748,7 +2751,7 @@
       <c r="F80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="15" t="inlineStr">
+      <c r="A81" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2758,17 +2761,17 @@
           <t>Australia’s new millionaire factory: Start-up to $1.6b in five years</t>
         </is>
       </c>
-      <c r="C81" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D81" s="15" t="inlineStr">
+      <c r="C81" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D81" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOVkl5N1NGWS1XWWZSc0pHXzE3MUNERmV5SUgyQ3o2MmJ3U3Y2YlNwUXNSTGlQenBwVFdnMWhoT2FrcDAwUHNVU0RQbjFHMjJiLU1TRC1nemdrX3hPTG93VWZUQUx3Wk9HT3lYd055Z2FtREFpOWRlYXFDb2hwV0cyWFMwaHpsLU0ta2VVQlpid1dlYks0ZHg5YTY3Ykt6Um5YaF9MR2tIRzd1Tk1IRnBrWVhxVjZNSUl1OE9iRlZzYmQ3QUVnZmhYVGxoOA?oc=5</t>
         </is>
       </c>
-      <c r="E81" s="15" t="inlineStr">
+      <c r="E81" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2776,7 +2779,7 @@
       <c r="F81" s="3" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="15" t="inlineStr">
+      <c r="A82" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2786,17 +2789,17 @@
           <t>Social Media Wrap: Genki Sushi Singapore's loyalty benefits; Dunkin Philippines launches new collectible; Burger King Malaysia unveils new Korean inspired burger</t>
         </is>
       </c>
-      <c r="C82" s="15" t="inlineStr">
+      <c r="C82" s="16" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D82" s="15" t="inlineStr">
+      <c r="D82" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxPbFR6eHVTRWZNcUw1TTBJdE1JTFpmbk5iWndKZnRoU3Fmc3cxcF80TnVhRERmY0poM09zTFpCaEVnMGo5aktxY0ExV1ZlZVpHYUtldXBoOUh6bm14SURHNmhnUE9tYnI5YlpXQ3pRZlp0Ni1wM2lYQmdxdjk4SDl0aFN0R1VBbGxpbFVzOHV0TFY3YjJZbDg4Vk1HMTBkQk5LRHd1ZEVpRnBsT1U0Nm1IbVFkZEUybmpabEhuLUNLOGhicUxXZG5UalRLOE5DSzcxRncyNjVRdk8zclhJNkVQcTRkQTZYSEdN?oc=5</t>
         </is>
       </c>
-      <c r="E82" s="15" t="inlineStr">
+      <c r="E82" s="16" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -2804,7 +2807,7 @@
       <c r="F82" s="3" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="15" t="inlineStr">
+      <c r="A83" s="16" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -2814,17 +2817,17 @@
           <t>Copyright ‘status quo’ not working in AI boom times, says Charlton</t>
         </is>
       </c>
-      <c r="C83" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D83" s="15" t="inlineStr">
+      <c r="C83" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D83" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNVVgwdEQ2YUt0eFo3THcxOXZHbUFYZ091VTFKZDZHX0szYWQ2dnZ1dkJma3VZcGk1LUM2SUtQSWhxMGpCUlFZVzdKNmdoSGEycm1oYlBUdEZ5R0ZlU2hrWHpFWXdSN1lCZnZzb3hZc2twVVlWdTNNVXhaR0Nza0FiaUNveXZWQWQ1ZE45MU1HbGNmWlU2aUdha2FyZllzNWdONEpsM2RrdGRFSFl2UlpJUnQ4WGpleGs?oc=5</t>
         </is>
       </c>
-      <c r="E83" s="15" t="inlineStr">
+      <c r="E83" s="16" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2832,7 +2835,7 @@
       <c r="F83" s="3" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="15" t="inlineStr">
+      <c r="A84" s="16" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -2842,17 +2845,17 @@
           <t>The unapologetically analogue 4WD for off-roaders with $120k to spare</t>
         </is>
       </c>
-      <c r="C84" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D84" s="15" t="inlineStr">
+      <c r="C84" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D84" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxPSFJ4ZnNLT3U1REp3MWI2WDFaQm5vZlp6QWN6c0hZamtYVU95WmpkUERwR1dwc0NQN1dEc0FNbHlaMTdLclVHb1JTc2VZNExENGYyUE9OR1BkQ244YXRVeWNwbkxia2VrckVqSy00WV9UNWlvZWJHOG9ibUthaTlpVmRBOGZjLWFzMU8yS2Q5Um05SWIzY2dKajhoMWFUcmFrbTMzai1CdVBNLWczTWRvbTBwSDRfUzNwOHhqQm5hTDdhM0xLWEpNQTRyRXZjU1FLdGhRMUxtOTg?oc=5</t>
         </is>
       </c>
-      <c r="E84" s="15" t="inlineStr">
+      <c r="E84" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2860,7 +2863,7 @@
       <c r="F84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="15" t="inlineStr">
+      <c r="A85" s="16" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2870,17 +2873,17 @@
           <t>Junk room to become jazz club with priceless Melbourne view</t>
         </is>
       </c>
-      <c r="C85" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D85" s="15" t="inlineStr">
+      <c r="C85" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D85" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQbHN4My1nOGtueVJQZWM0LXNjLTR3MmhuemRJMUEwN09FTUZhZk1lbV9MbnVWblgyUXFEMEl3LUtsOGVqdGUweFR0MXF0ZEo0XzNhWVRqb2pGRUdiNTlLc1dFcXFmdnctQU1wQkRSdHN0T3J6VGt3MU1iNENydGlsOEpsT0ttZmJVZ0FUZmFXSUd3alVzUTQxMzVmcEVXSlV2dWdQd3JsMUZ0d3ZZYlBHaGhKTm9rM01SUmdseE9hT1prbHZtMlhv?oc=5</t>
         </is>
       </c>
-      <c r="E85" s="15" t="inlineStr">
+      <c r="E85" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2888,7 +2891,7 @@
       <c r="F85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="15" t="inlineStr">
+      <c r="A86" s="16" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2898,17 +2901,17 @@
           <t>Zimmermann fashion label appoints new CEO Roberto Eggs to replace Chris Olliver</t>
         </is>
       </c>
-      <c r="C86" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D86" s="15" t="inlineStr">
+      <c r="C86" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D86" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM2M5QU1scVoyNHBmV2lwQ0VQS1Z6d2Qwa1ZkZ0M2WVIzdXR3QnZwVWhUSDRCUEdRZkc5QzFQSFFhNzZ4VE9lWXBTcGhpS01JdG12TlQxSHhValZfbWt3MUdFZGl3RlBtdnlrel83TjNjNFZ0SUpvSDNQbThpU3FLa3Atd0dNU04zQm9OSk5uNHpTVE84aWZpaVlKWkdOQjJjRTZSd1MwMEZ1b3pENkRCQQ?oc=5</t>
         </is>
       </c>
-      <c r="E86" s="15" t="inlineStr">
+      <c r="E86" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2916,7 +2919,7 @@
       <c r="F86" s="3" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="15" t="inlineStr">
+      <c r="A87" s="16" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2926,17 +2929,17 @@
           <t>Construction giant FDC road tests IPO pitch - AFR</t>
         </is>
       </c>
-      <c r="C87" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D87" s="15" t="inlineStr">
+      <c r="C87" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D87" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNTnRScHFhQlpkdEdSb2x1bExxQm96ZE5zSV9wTDNDV2pxYjFQdUtoYmNBell3SFlTTFEzMUhpeXlmNERSeDd6VGppM2szQ1NHVE9PY1R3MTN0SUZLWkF5em8tQ3IycUZ2RmswX0tnN1IwOHl1ZFo4UUtMUDlQbXRjTnRCWFB5cU1RZFhsdDdaWGpMZzh3d29CWWZvZGtnTjl0T1k5ZHFHSUg5XzFSSF9TSUxTYkU0QkFheFlLZUY3S2tCSWRLZWlBbUpxUjc3TXBQQ01V?oc=5</t>
         </is>
       </c>
-      <c r="E87" s="15" t="inlineStr">
+      <c r="E87" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2944,7 +2947,7 @@
       <c r="F87" s="3" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="15" t="inlineStr">
+      <c r="A88" s="16" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -2954,17 +2957,17 @@
           <t>David Jones is trying to defy retail gravity. It’s causing problems</t>
         </is>
       </c>
-      <c r="C88" s="15" t="inlineStr">
+      <c r="C88" s="16" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D88" s="15" t="inlineStr">
+      <c r="D88" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPZy14UldWZDRrSjI3R0lzdGlKamlkVnU1WWVjTWRUTlpya1ZpVW80WHlrT0FQTUUwMzkzM19xQWpwTnVLOF8zeTFXamhTZFRQVjl5TTlXbE1RRWY2NW03dlpmZ25qdkgyN1IwbDdjRlhxd1MzSGkxeG45M214OVlESWF5WWh5TjM0STQtOXdieWIyOUI2NzRsaDhiS0ROUU5YQ185aWtObUY2S0dOSTBROVlwSVB1VkNqTkZTTllkZmtMYmxjNVdlTA?oc=5</t>
         </is>
       </c>
-      <c r="E88" s="15" t="inlineStr">
+      <c r="E88" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2972,7 +2975,7 @@
       <c r="F88" s="3" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="15" t="inlineStr">
+      <c r="A89" s="16" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -2982,17 +2985,17 @@
           <t>Jefferies’ Australian ambitions in focus as Sumitomo circles</t>
         </is>
       </c>
-      <c r="C89" s="15" t="inlineStr">
+      <c r="C89" s="16" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D89" s="15" t="inlineStr">
+      <c r="D89" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxNUTd0LXFPQmZXSldrTmZHTkIwUWQ3MmlCUmFOUGRkcVVjRXV6YXZJUTcyMG5FV3I0dWY2NXh6MnduVjNxZmhJMHdDVGw5VzFxTEFzN2FBdlNvS1JGSDltQmlzVS1QRDdCeWdfSHZ2VlZDMlBnN1Y0d2JxbnlGejhWVjJpWGZLejdCTUt2Uk9ENmhyRkd4dDJjd0RlUnBlZXhOTmUtOG9ITE05VHJ3dTBRSWZneURuUW1NYkExVXpfWXlsMzZ1WUlyNE84SThQX1JJTFlXOHc4ZnB0aXRmdVhaaG1qSEJRZUhuU3RibHAzbHVNLWFLUF9NNTFoUXV3NGQzelcwcNIBigJBVV95cUxPMkhEeDJpNzg0NTlDZmF2LUFPSEs4cmZ5U2p6bWVZSTYwcXVUUGVIb0FLVnhZV0cta01CLVpfQzQzYzdvTWdxR0o4bGJDWDVBb1lnOGx0bWROdTdjcHhwLUpPMW9MQ0RVM2NUOUt6UGpTd05JYzhuVmgybGp2LVpORFF0SHpBTU5DUTJEUmZKUFBNajlQdHJ4WkdHVV9QMjVwOWVlNWliVkFaM20yWGZhOEc4bldHRERJak1BWXlmSE0zdno1VTVSc0FMck0wSE1BR1RVaVRMSEdzU2FvcWpMYmp5ZTVJTWcyUGdXanhqSUNZU0tzTkNYWVg2SXpVMEoyS184VkxOeWtSUQ?oc=5</t>
         </is>
       </c>
-      <c r="E89" s="15" t="inlineStr">
+      <c r="E89" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3000,7 +3003,7 @@
       <c r="F89" s="3" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="15" t="inlineStr">
+      <c r="A90" s="16" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3010,17 +3013,17 @@
           <t>Bain Gets Nearly $300 Million Loan for Australia Wealth Unit M&amp;A</t>
         </is>
       </c>
-      <c r="C90" s="15" t="inlineStr">
+      <c r="C90" s="16" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D90" s="15" t="inlineStr">
+      <c r="D90" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMUQ4WExYZFY1aFBwWENNR1JiVkw4OHFKWjY4NW4zQ3ZBalFiTU10Y2hic2p2VjFqOE1rMndNYmVoN0lPcnY0WmFOV1MtaEY5c2xvcW1PNGN2SzZVcThwc3ljWkYwV1Q4a2dIaUpBeXZpMkRUU3IxZzVBVkhydGU3OXEzNW1sdlVQeTRNRFY4bUJLOGpGYmJ0ZXpPc1YzY05TYWd2bF9oWVJ6Rks2dWlod1dGRU4?oc=5</t>
         </is>
       </c>
-      <c r="E90" s="15" t="inlineStr">
+      <c r="E90" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3028,7 +3031,7 @@
       <c r="F90" s="3" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="15" t="inlineStr">
+      <c r="A91" s="16" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3038,17 +3041,17 @@
           <t>Fund managers caught up in Aware, TelstraSuper $237b merger</t>
         </is>
       </c>
-      <c r="C91" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D91" s="15" t="inlineStr">
+      <c r="C91" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D91" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcFF4Q1A5X1VtNWFnYXZSVUlZX2JMRVoxaUJoeGhybmRrZkd4UlEzTURwMkx2d2I1Y1hMYmljbk05WUFzRl9JbF9JampqeDd2bXdYcUpHbVZYak1sYXFHS2VuUDJyTUhzSS1QTW15aVpfeHRuMGZHenlxOHJQRUdENkV0b2FMZXhOZWF1Yk5hR1lOYWFQc2Q0SEROUFNERXhKQUIzRkt6NTQ?oc=5</t>
         </is>
       </c>
-      <c r="E91" s="15" t="inlineStr">
+      <c r="E91" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3056,7 +3059,7 @@
       <c r="F91" s="3" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="15" t="inlineStr">
+      <c r="A92" s="16" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3066,17 +3069,17 @@
           <t>Soul Patts defies private credit jitters with 15pc returns</t>
         </is>
       </c>
-      <c r="C92" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D92" s="15" t="inlineStr">
+      <c r="C92" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D92" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPRkNINFJOai1NbUUtX3ZrcnJFS3EzRHZPbFRfVFE3SERudTVqbjIybWsyYUthOUJOUVFPb1U0UzlGTTRqbUxraFZfYlVtclQxeTBQU1M5YjJzMDVPU3RiX0cxbk8xOEd5YjV1R04zT0NNZjhNSi1meWo4RHM1ckFsUnNLd0JiQXFnZ0dtckNzdWxmanZoQUl3TEQ2a29nRkRDZ1lJd2Y5VGc2UWZHX0pkU1NObmRJTlZKS0E?oc=5</t>
         </is>
       </c>
-      <c r="E92" s="15" t="inlineStr">
+      <c r="E92" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3084,7 +3087,7 @@
       <c r="F92" s="3" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" s="15" t="inlineStr">
+      <c r="A93" s="16" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3094,17 +3097,17 @@
           <t>Ex-KKR China heads negotiate to buy Vitaco, owner of Musashi, Nutra-Life</t>
         </is>
       </c>
-      <c r="C93" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D93" s="15" t="inlineStr">
+      <c r="C93" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D93" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQRmlCdTlFeHdBUGkyOS1CeEFIYTRSREdZM1JOZ3IyZThnNmNMdm9QeXVwRWtMbzU0em1vcDAyM1hodDlvalVRdThtNVhLR2FsaE1vV0xuWjkwMkVCUDk5SmVka1BURFJZNkl2bURLeC1GdzI0V2hEaVhrNlJZejlvc2gwRmtnUjd1NDFlX2trbGk2aXJiQ2FrTWtmVVpiOXhBc05JSkNYY2xLX2JEQUpWY2dlY1pDZw?oc=5</t>
         </is>
       </c>
-      <c r="E93" s="15" t="inlineStr">
+      <c r="E93" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3112,7 +3115,7 @@
       <c r="F93" s="3" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="15" t="inlineStr">
+      <c r="A94" s="16" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3122,17 +3125,17 @@
           <t>Antipodes Global Investment Company</t>
         </is>
       </c>
-      <c r="C94" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D94" s="15" t="inlineStr">
+      <c r="C94" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D94" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE5mdkJzN19XLTFQc25LOUk0ZGJBMER6djB2VnFvbGVrS1hlemRBRmlNY2JmMGlPTzktU0RRS3NNUW8tRXhtUE1QdE1JLWdUNVhibmZPZi1MRkJOWk95NzM2bXplS3JzeG13UU5henhza1ozeGRZZmlBNTNR?oc=5</t>
         </is>
       </c>
-      <c r="E94" s="15" t="inlineStr">
+      <c r="E94" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3140,7 +3143,7 @@
       <c r="F94" s="3" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="15" t="inlineStr">
+      <c r="A95" s="16" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3150,17 +3153,17 @@
           <t>AusSuper to lift insurance premiums by up to 40pc</t>
         </is>
       </c>
-      <c r="C95" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D95" s="15" t="inlineStr">
+      <c r="C95" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D95" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQNEhYQkoyNnJFU2xBZG8wdXhEZWRSakRiWWNHOGZBTFhfaElxWkRsSWViaWxjenVjMF91cGdrbFZxSGJfbkR2SUZNdEJtYUVadlV6YVVrWU1VbVdsMWpyNUZ4bE13Mmo4cGQ3WWZlVFVrTTdyOGpSdkpUb0tkcjdQUFlsTnM0MnpOMDJNZlJ4YTlzZGpLS1QzMFluOFU2VUJya3lSclBLSnZkQ2Y0a2djNUpSYlo?oc=5</t>
         </is>
       </c>
-      <c r="E95" s="15" t="inlineStr">
+      <c r="E95" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3168,7 +3171,7 @@
       <c r="F95" s="3" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" s="15" t="inlineStr">
+      <c r="A96" s="16" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -3178,17 +3181,17 @@
           <t>Unions want inflation-plus minimum wage rise due to ‘Trump and RBA’</t>
         </is>
       </c>
-      <c r="C96" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D96" s="15" t="inlineStr">
+      <c r="C96" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D96" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNdzNhU0MzbFRFX2I3OVY4bFItd1h6OVE2Wnpqb01NM2tMYzNob21BeW02LTBfTFZIWnN6SG5DVnYxQTJGZWZaLTJpTXZGUnhmS3RPY3hQV01fd1RIYU9Ednc4a1hvalVRT19ESU5TX19sQjN4dVV3X29kQjliQjNFU19iaXFIS2l3blk5TWUwdHFrRmJtQ0JocDN0WEhWbXZOVUJzR3RaYnJPSHpIRFlYOVFObEtuT1d0TUo0MUVZTXdFZWR3WG1r?oc=5</t>
         </is>
       </c>
-      <c r="E96" s="15" t="inlineStr">
+      <c r="E96" s="16" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3196,7 +3199,7 @@
       <c r="F96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" s="15" t="inlineStr">
+      <c r="A97" s="16" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3206,17 +3209,17 @@
           <t>Firmus’ Oliver Curtis set for green light to run ASX-listed company</t>
         </is>
       </c>
-      <c r="C97" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D97" s="15" t="inlineStr">
+      <c r="C97" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D97" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNR3VmQW9vNmUyeU9WbVRvRG9tcTNMYVlvRUhCd29wTkRZaVlEcG50Z0hIN29XcE5GUmxkUy1yMm0yTm94Q1BXMmNCcXBpZDlqVTRlZFpMX1QyMWh5Ym5XQ3VjYW1ZdDFtYWNyOERCOURuWXM5ZTV4WGthMVVjNUZlcmVTQ3JBUjQzUXRXYXRLQjlNeHpBMkVCVWpsd2Z1Vk42TjJxSlRiQ0ZtaTkzOTZtNmRHQQ?oc=5</t>
         </is>
       </c>
-      <c r="E97" s="15" t="inlineStr">
+      <c r="E97" s="16" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3224,7 +3227,7 @@
       <c r="F97" s="3" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" s="15" t="inlineStr">
+      <c r="A98" s="16" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3234,17 +3237,17 @@
           <t>Crisis Hit David Jones Chasing Funding As Retail Markets Come Under Pressure</t>
         </is>
       </c>
-      <c r="C98" s="15" t="inlineStr">
+      <c r="C98" s="16" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D98" s="15" t="inlineStr">
+      <c r="D98" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNNjJSOUVQcTkwUmxXNXg4ZzljSGhnRlBJY0otSHRrX2ZIQXRqWmNDZlgxYW1jckhHd3BtdXJsUWhwTjQ5SGw2NUU3TnFtcmhYd2JVcThIR2VCLWJLU0h5RE8xaTV5TS03Mi1za19hcF9PcXRRSU9PX3ZxSktSV2FfY1ppcUFVV2w1TmF1UWVtZlBWSUhEcG9oRGlEVkEwR2ltQ2VMSTNlcENEYlY0?oc=5</t>
         </is>
       </c>
-      <c r="E98" s="15" t="inlineStr">
+      <c r="E98" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3252,7 +3255,7 @@
       <c r="F98" s="3" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" s="15" t="inlineStr">
+      <c r="A99" s="16" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3262,17 +3265,17 @@
           <t>Beirut Street Food eyes niche in Lebanese fast casual</t>
         </is>
       </c>
-      <c r="C99" s="15" t="inlineStr">
+      <c r="C99" s="16" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D99" s="15" t="inlineStr">
+      <c r="D99" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNVlZVeTNGcXVOSXV1eklvTnFxYk1hb1A2VTQtNHkwdUpvdFF0YnlYU2RSWkZNV2dGQkEyZjRVQzVJZ2Uwc3gtZ0F1TGlSQlVna01HRnZOTTJnVUFxaWtOam1vZ245Z05jdlRnQURqbnQxaGtEcnFYS20wWmtvSDV0MW15c18zUE5ZN2JJWUpLV0RsZE1LSm5fcUNNeVZNTmdMQ2c?oc=5</t>
         </is>
       </c>
-      <c r="E99" s="15" t="inlineStr">
+      <c r="E99" s="16" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3280,7 +3283,7 @@
       <c r="F99" s="3" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" s="15" t="inlineStr">
+      <c r="A100" s="16" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3290,17 +3293,17 @@
           <t>Gami Chicken credits chip design for cult following across Australia</t>
         </is>
       </c>
-      <c r="C100" s="15" t="inlineStr">
+      <c r="C100" s="16" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D100" s="15" t="inlineStr">
+      <c r="D100" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPTXg4T0dvQ1l4NFVxV25iUXQzY0F3MnFjYmE4X0NOcFdNZHgweUg4NmVZZjNJbTFMajNhNHBmVDE2MGNBZzhOTUJsaG5KejFZbk1Db0JyNTZJbUI2WnRZeVhXRFRMNXVBWVFMdGJ3WkN5dV85dEduQi1OVDhOSE9UOGVERXh3T2hCVmlDNVg5LTdLY2VHNEZJSzlrN3VuemhzX1B5blpYRGtwS0hrak5r?oc=5</t>
         </is>
       </c>
-      <c r="E100" s="15" t="inlineStr">
+      <c r="E100" s="16" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3308,7 +3311,7 @@
       <c r="F100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" s="15" t="inlineStr">
+      <c r="A101" s="16" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3318,17 +3321,17 @@
           <t>The great fake meat meltdown is taking plant-based burgers with it</t>
         </is>
       </c>
-      <c r="C101" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D101" s="15" t="inlineStr">
+      <c r="C101" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D101" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPRTVDNW5oaWJ5bHdKM21iYllEVnpJbHhSbWFzYy1RcEZCdnNGUlJOWVJCaDZacFVoRjlSUGpfa3N6ckQtMFYzZTNITW5tMy05Sk0tZmtlSWlESHdOMWIyUWpUbE5RQVlsTHp0VXg0cHJYM0lJVmw1ckRURkFPVHFabTRIUzlFX1FlbFNuYmQ5MVJwWHVOaVhVWTdPajZxdG1WOTliTE1qZ3k1dnFRbk9BNTZCcXRRSGlIXzJv?oc=5</t>
         </is>
       </c>
-      <c r="E101" s="15" t="inlineStr">
+      <c r="E101" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3336,7 +3339,7 @@
       <c r="F101" s="3" t="inlineStr"/>
     </row>
     <row r="102">
-      <c r="A102" s="15" t="inlineStr">
+      <c r="A102" s="16" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3346,17 +3349,17 @@
           <t>Solar for Cuba: How Xi is turning Trump’s war into a China win</t>
         </is>
       </c>
-      <c r="C102" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D102" s="15" t="inlineStr">
+      <c r="C102" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D102" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQOFlUUnNZUWo0MTJRaDFIZHp5dUJudERrOWxCZmY1WjZmeXRTVzJkbENEbUFhSkZFUWV6WjNGNUJIejVYRXFPcmRNZjFZeTkzTmtaeFNlb2V1OFFnMGtkV2JfTVRUN2FSV2xxcUpDUDJQeUpqWE9DRHRmT2kyc1dIZE9jeUM2eV9KQjd2RkJuTkxYeEdISDZDejhRbVo?oc=5</t>
         </is>
       </c>
-      <c r="E102" s="15" t="inlineStr">
+      <c r="E102" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3364,7 +3367,7 @@
       <c r="F102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" s="15" t="inlineStr">
+      <c r="A103" s="16" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3374,17 +3377,17 @@
           <t>Beer Sectoral Group appoints Nigerian Breweries CEO Thibaut Boidin as Chairman</t>
         </is>
       </c>
-      <c r="C103" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D103" s="15" t="inlineStr">
+      <c r="C103" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D103" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOamdsNTN1dkRUY19Yak0wUGxsdm9NZGhySUM0Vzc4blNCeldzdFBiRkxuSW1xbTlZQUJIWkNxdzI3Zi1zc3F3SmJvai1UVGlZdUhGTEJ0eF9mNHRwSGREbDktT2txWXA4OVBESTdPLXdxWmV2V3FPTEZaYjRWLTlMM1VaY1dCbGZudTczZlFEYzN1aE9HeWdObE1yZFduLUtNVXBheDNsUWlIcUxibml4YQ?oc=5</t>
         </is>
       </c>
-      <c r="E103" s="15" t="inlineStr">
+      <c r="E103" s="16" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3392,7 +3395,7 @@
       <c r="F103" s="3" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" s="15" t="inlineStr">
+      <c r="A104" s="16" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3402,17 +3405,17 @@
           <t>Hip pocket pain comes for shoppers – and for supermarket giants</t>
         </is>
       </c>
-      <c r="C104" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D104" s="15" t="inlineStr">
+      <c r="C104" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D104" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOeTdfN2dwYlBWSTdGbFo0SWRJcTNYelFFM2FBRnlORWRNcGd0WUVCbVdHVWZ6TFdZQzFpM2h6TkU2OEtqeE5OYlRrNmhsRU43a0E0UXhtZEZyTWZidzhMUEVxSVdiMlpTYXQ4ZVRaNl9BSi1Mb3JRaXhvM2hlMmNDcnk1aFBvVXFQSmlPbkN4Z3o2R2RzV0drQWpKaVZpbXR4dHppa08wRFd0dlNwcDc1alRDSXg?oc=5</t>
         </is>
       </c>
-      <c r="E104" s="15" t="inlineStr">
+      <c r="E104" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3420,7 +3423,7 @@
       <c r="F104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
-      <c r="A105" s="15" t="inlineStr">
+      <c r="A105" s="16" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3430,17 +3433,17 @@
           <t>RBA calls for co-ordinated effort to unlock digital asset markets</t>
         </is>
       </c>
-      <c r="C105" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D105" s="15" t="inlineStr">
+      <c r="C105" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D105" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOT3dEcEtwVUptWTZydTRYWFdCU1RhTjI1RkFWeU5HckRVZjBxc2lqRkNOT0stc1h2Q0E1YTkxTjk3NTB3TGxKZGIweGFQRGh2S05QWHRoVGNZRFR2SlI2bkEzWlRoY2t3WU16dDlhVEI4RTFWYzhKS25YbGYxSVRjdFpVQ2M0dVc5MFJuUExNMTJIMVJTYmZGbkNLR1BPeVFYSF95NkNnWEEzamg3NmRuRkx0U2NjbXlxY015UWljTzRWbXpKclAwUg?oc=5</t>
         </is>
       </c>
-      <c r="E105" s="15" t="inlineStr">
+      <c r="E105" s="16" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3448,7 +3451,7 @@
       <c r="F105" s="3" t="inlineStr"/>
     </row>
     <row r="106">
-      <c r="A106" s="15" t="inlineStr">
+      <c r="A106" s="16" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -3458,17 +3461,17 @@
           <t>Banks rebuff work from home calls as Wesfarmers pauses business travel</t>
         </is>
       </c>
-      <c r="C106" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D106" s="15" t="inlineStr">
+      <c r="C106" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D106" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOTjFLNnZUNXZHeE85a3kyaG1IX29sWjFvZ2NzS041UnYxNkkwUF9YU3ZFYXhtQmlxY3Rmd0lUSTJrdTl1Y0ZobWp0M1lrZnZhZE9OSzV3Ql9Hb2UtUEpqWC1McjM0S2pESDJQVWJKQkw4enF5THJfeXFWRDZiMk5KMmVrazVUMzBNTk1tOXRVX1ZzVU1IUHBVSlhENEdEWFJpQnFXUGkyNVJGUnhzdXgyNW1WZXRkRmRaaVloZnpaMFdqVmk3elpFSkZ6ZmotZw?oc=5</t>
         </is>
       </c>
-      <c r="E106" s="15" t="inlineStr">
+      <c r="E106" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3476,7 +3479,7 @@
       <c r="F106" s="3" t="inlineStr"/>
     </row>
     <row r="107">
-      <c r="A107" s="15" t="inlineStr">
+      <c r="A107" s="16" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -3486,17 +3489,17 @@
           <t>This mine was fast-tracked to boost Australian solar. It’s exporting to China instead</t>
         </is>
       </c>
-      <c r="C107" s="15" t="inlineStr">
+      <c r="C107" s="16" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D107" s="15" t="inlineStr">
+      <c r="D107" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAJBVV95cUxPN1ZSdEMzSXBhMno2YzNkSFFtdlBOTTRGV3UtbnZtRktEd3Q0MHdmZHp0SDN5S0FZYmVKUllicHRMRkxTdmxtbkMtT2ZVN3hsUXdBVzAxdzhWcGFWRkxVdFY3NURqTVV2QVJQT0ZUT193R3JLLU9aZUw4YzlucjVUN0xyTzdoZlNjYXdyR2VWeDZrbW53cTJoRGZDd2kxbkxzMHBQWkRJMTFPMkNlX19wYjI2LVBZbnVJOVNsRjF3Tm0xUUFpY0ctczFZdWJFcHQyLUhwdDNiSGVtdHQzVVRtbExpcHJZak1SNkhWd2s4a0RtYWFNN2J2Q3FobTF1N0hWLXA4YUtaMXBScjZsUWt3alVVTVpJdVl0WDF5RTJLM1BKUl85dnhUUktkb2VwMzFkUWZ1ctIBugJBVV95cUxOOENIa2JzQzdxekNYTnJNVmRzdm9KTFpndnBybEJfNjBUR3VNMk92ZnhGY0JwVGZLeFRpdHJLMTQ0NjRNOFg5b3FESzhPLWlub2hSeFdidW0yS1h6ZXlGMjh3X3FhaWo1dHdneUZxS2NsaUJ6dWtfT1R6VndwSk52bVVNN2I5VlNYazBIelcwUkVBZHFlM0hiQVJ1a2NGWFpmR0c5R3Bna2RZMmJuSXB5WkQ1Zl94VDFtcjVEd2x6amIwSWdXUWtQVVo1Q0hpWVBLRVFycDAyU1NJV3N4YktlUlBtMTlkY2VNZjc1QVZhbnRrQ01OQnZqNzI5dTNNZ1VlNVVJcURycXlDRFZDYVo1aC15RXpwUFlvZWxlMHFybWJiM1YxT05lRElXYlZsbkJWUnI4VV9Da1lIUQ?oc=5</t>
         </is>
       </c>
-      <c r="E107" s="15" t="inlineStr">
+      <c r="E107" s="16" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3504,7 +3507,7 @@
       <c r="F107" s="3" t="inlineStr"/>
     </row>
     <row r="108">
-      <c r="A108" s="15" t="inlineStr">
+      <c r="A108" s="16" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3514,17 +3517,17 @@
           <t>A $600m dream or a dangerous gamble for cricket?</t>
         </is>
       </c>
-      <c r="C108" s="15" t="inlineStr">
+      <c r="C108" s="16" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D108" s="15" t="inlineStr">
+      <c r="D108" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxOYnpVaTZiU3hGMWY1UVVmYk9nRTJaRTVFYUE2ZklLYmJIQkdXZzFMbWs3MVRJb0l4bUpPeThwRnhOSmh0bzNBdzhpeXpuS1RrZ0tNVVJ4eU8tRVIwR2FyYmUtNG1UVmN2OXRsZm1mVy1LZDVERkpXQURMUk1HRE9Hc3F3RWQzYmFvbHRCVGhFOTQ3M2xnVGcxTWxtT3cydW84NTNPc3BXQURodmY0azBOUllOQjhrbzJ6WmI3bjY5dk5RRzlDQ0JlYzg0VzRsdWtIblZJelRSamFyQnNweHdHLTRTMTFOcy1Jd3ZtQWFodEcxOThVeVVz0gH3AUFVX3lxTE5ielVpNmJTeEYxZjVRVWZiT2dFMlpFNUVhQTZmSUtiYkhCR1dnMUxtazcxVElvSXhtSk95OHBGeE5KaHRvM0F3OGl5em5LVGtnS01VUnh5Ty1FUjBHYXJiZS00bVRWY3Y5dGxmbWZXLUtkNURGSldBRExSTUdET0dzcXdFZDNiYW9sdEJUaEU5NDczbGdUZzFNbG1PdzJ1bzg1M09zcFdBRGh2ZjRrME5SWU5COGtvMnpaYjduNjl2TlFHOUNDQmVjODRXNGx1a0huVkl6VFJqYXJCc3B4d0ctNFMxMU5zLUl3dm1BYWh0RzE5OFV5VXM?oc=5</t>
         </is>
       </c>
-      <c r="E108" s="15" t="inlineStr">
+      <c r="E108" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3532,7 +3535,7 @@
       <c r="F108" s="3" t="inlineStr"/>
     </row>
     <row r="109">
-      <c r="A109" s="15" t="inlineStr">
+      <c r="A109" s="16" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3542,17 +3545,17 @@
           <t>Why these people decided to vote for One Nation</t>
         </is>
       </c>
-      <c r="C109" s="15" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D109" s="15" t="inlineStr">
+      <c r="C109" s="16" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D109" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOQmNaOHZXWEEwZzRmdTBVT2FiS2hsYUhFczgxaFJaeEQzMGlfSnRoUWo0ZXl3cWhhbTU2NDRLUjh1c2Jxd3ZoR2pJOHVNemI2cTFrdU9oVkFCNXN4WV94TER4VmtIX1JCblhKNTl4VHlMdFBDRHVBUFhkS1AtR05RMG5QVGJFaTlWaVpMZERIa3Ntbmh0V0xnVVhYNDdMWWlpSWc?oc=5</t>
         </is>
       </c>
-      <c r="E109" s="15" t="inlineStr">
+      <c r="E109" s="16" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3560,7 +3563,7 @@
       <c r="F109" s="3" t="inlineStr"/>
     </row>
     <row r="110">
-      <c r="A110" s="15" t="inlineStr">
+      <c r="A110" s="16" t="inlineStr">
         <is>
           <t>2026-03-28</t>
         </is>
@@ -3570,17 +3573,17 @@
           <t>The Right Amount to Pay for Sushi</t>
         </is>
       </c>
-      <c r="C110" s="15" t="inlineStr">
+      <c r="C110" s="16" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D110" s="15" t="inlineStr">
+      <c r="D110" s="16" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOLUljQ1FWeHk0N21FcnpCTzdNVW1WZmxfbDFucXRNYlBMSzR6aTh4WlNrdnFuT1VSWWpKWlJValZrbTE5RlllanJkcHNHeEVwVkxldnZSdjdLc2c1SHJTVG1hMHBKd2xtZXptV1FmcGZ0cXUwVXFMWjJiRFhhYTlKRkNBNHZQekVRcnRicXlNM2NQdXJaZkVRbTZta0hDRlV5YVN5NG9TYzltUFZucXNXc29Wc1Y?oc=5</t>
         </is>
       </c>
-      <c r="E110" s="15" t="inlineStr">
+      <c r="E110" s="16" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3642,6 +3645,398 @@
         </is>
       </c>
       <c r="F112" s="3" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="17" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>KMD Brands makes emergency capital raise, chairman David Kirk to exit</t>
+        </is>
+      </c>
+      <c r="C113" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D113" s="17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNb1JhRUM4dDhXM1hoajdzQkNLQk12LURQbkp5LWdqQXpEczBxdVhySHphaUhiLVRiYVh1R25kbHRidy1TbjhCOEk0MXk5a2VWWlhHcUt5aXpfNjZWNnd6LVpQUkZNbFFXSWJHTmFaM2x2aS0tbG9TeXFxUWI1NF9uazJKa3BrZHFwclB1OVR3cWhXU2dJNFhaZmpVRVlwWUdiX2hrX0thQ3RDOWdFTF9BOGdHTG1JSlF6RVRZdnZn?oc=5</t>
+        </is>
+      </c>
+      <c r="E113" s="17" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="17" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>RBA green lights credit card surcharge ban</t>
+        </is>
+      </c>
+      <c r="C114" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D114" s="17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOcTB6SlhfdTQ5ZWdqNDExZVhOcVVybW5mbmxOVktCS3ljTndLY3ItWldSNDIyeEkwQmdBZ3p1X1o5S3ktZXI3MFM3eVkwWWc4cGtUTUw3aWM4azM3VGdrcGZjTjZMN1diWHZ0N3pna0tJZHZNU1FaN2VZbVNwMmozSFNBb253OUcya0duaEMtZnNQaFYwUFBhTGthaGhyTWY0NHpPTTFubmZOWEk?oc=5</t>
+        </is>
+      </c>
+      <c r="E114" s="17" t="inlineStr">
+        <is>
+          <t>Australian Economy &amp; Markets</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="17" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>Constellation Brands to acquire Hop Wtr, expanding non-alcoholic beverage portfolio</t>
+        </is>
+      </c>
+      <c r="C115" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D115" s="17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPcjdPYWlEWWF6dkY2Y3RPWUh6M0pXYUw1NFNabUdXTS01TVBMWGtBMUpxTXFRekJINGNFOE5oVEI0WjR4Z2kzTUR6emJHUUYxWjA0MGVlWFNPR25xNmJJWkN2RHIzcWNxUHRFQXcwdWN5cHNZRVVYV3JTdXRJUFg1MWJKODNOdjJ5UEd4dWZEbVFyWlNaRkJPcnlyQW5janktSDVwYWRVRGJqTFdPTEdUSUFvRXI4QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E115" s="17" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="F115" s="3" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="17" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>David Jones races to secure $150m survival deal</t>
+        </is>
+      </c>
+      <c r="C116" s="17" t="inlineStr">
+        <is>
+          <t>The Australian</t>
+        </is>
+      </c>
+      <c r="D116" s="17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxONHp5S2RtcFJkYWVxakc1ZDE4UzZUVWlHSlBMTHJqVnVaRHJrcEwyV3BHWk9TdXdkOUlocWY2ZlN4NklobGVuYWhRc1BvdWppWlNFTm9wcGZoMG1UMEtjLS1scmx4cVNhNkZQYWw0M1VUQTJfOTJrYWMtTlpJYnl0N01QTWxZZDZPOEpfcTM1dFRVMDBTOEthcFU2Z0U4WFFBaE1GM2V6VHJVb2Z5ekxJWmUwQlphbXRlTS02NWNJV2p1Ym5Ca2JxNS0xQWZpbHJ4UFVtbDBCXy1IV2NXMlFOY25HSVkzTjYxbXZB0gHwAUFVX3lxTFBDVlc2X3JNcnNNWjlUV2RkeEdtSFBJRFNtTXVHcmZERW1vZURfeDFvRGo0b1Z5SlVOVGNJTXB4MVc3d3hWY3FVOENwbEJ1MERBalhlc2EwNnktcUprSjZQLUxNTVlqYzc0enZtQ0FOUFVTWHBCZVF1SWs2Y0ZKRllXblI4MVRrXzZUMHNicmxqeFhUUld4VzM0TGNtcl9fTG4wbEJPWDg4RWpjMUdHOUxlczdEend1MkZLRTZuUjdkV0xGRlR6RVlXdVUxdUhndmozTHNtT2czTjJzRUs0bFc2QnMxS0V1X3QwcjVNeGVjcQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E116" s="17" t="inlineStr">
+        <is>
+          <t>Retail &amp; Consumer</t>
+        </is>
+      </c>
+      <c r="F116" s="3" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="17" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>Newly listed Advanced Innergy targets smaller rival</t>
+        </is>
+      </c>
+      <c r="C117" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D117" s="17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPamkyYnZfT0NwamdES3JPYklaaXFYdUp5cHJPOTZUNklqcUlral9ObHFPY1VROHJSdm1tOS1KZlZJWFA0Q1l2UUZhOThleHFsWDJTSVdTUnhlbE1OeVhBTXVQQjVIdHZHTFBHOUxGOGx3MWc1UmVIWUV6Q3RhTDR6WHRfRy05a25VX01lcWZOV3BWX1JyQVI0WlQ3dTQwNHhxWXJCQmV0VQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E117" s="17" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F117" s="3" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="17" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>Aussie eyewear giant’s costly $20k mistake</t>
+        </is>
+      </c>
+      <c r="C118" s="17" t="inlineStr">
+        <is>
+          <t>The Australian</t>
+        </is>
+      </c>
+      <c r="D118" s="17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAJBVV95cUxOTmtzblUxcW5WbDZLeEJXSWVuVW5qVzdpRkc1Rkoxc1pVT0FIaHdmR0p4ZzljcVpST2tHdTBwVEdqbmF2TVhlV0VaMDFiMVk2ZEZkUTZMNFQ1a1lUbWRCdGwySkJtbmRfTXFmUy1VVU1tU1dzMldON3lEUFVVVFI4T000b2NJLVhobDBBUzQyLTRGLXNPT3ptZ2tlUU8wNG5nNFAyUVo1elpTeDd1TW01YzB4eUI2eE9YQjZxNTJBSVpLYy0yR1BzSVFiWWxib1g0YmlzREFGTEV0bkRucmNLa3U4dXhkTC1aRkhnUHN1d0hjVUFuZFlWWG9xVUtMT0hKMjhmNkZzLWpMS2MzYWp1OVN0cV9IYnBRZG5OdWwwcErSAaYCQVVfeXFMTzBFMkJ2TU5EZGZYLVF5WHBJanYzeFJqS1owbk5EUUNOZFNiam5PcEZ1aDBFelJ5MjFzM0E0NlZRdGI4Rjdnb1RYVmVSN1Z1OWd1SFdweVB0ZEY5akVqOHBsTHpJaXZKNnhUMmd2YVVxTzUtUEJKcWpOY0VHeHlTbXNCbHFDdnlndzJFT2ZDcnlZWXYxNUFNekVUZWU1UTFnOXZXUERMWjdjYl9wVVl6OURodW1JSUI2ejJDTktfaTRCY2xEeHVBRW9tNmM3YXBHU201WXpHYjFYbU1sYnB1MjlLNjI0eTRWVElXU2ZqMDNNRW5LMVQyS2M5Z2tPSHJneGlkUkxFYXhDdWM1MGtkUUExT1hBSlU1ZkgtRlM4YnV3b1hkM2NR?oc=5</t>
+        </is>
+      </c>
+      <c r="E118" s="17" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="17" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>Rio Tinto bankers up for infrastructure sale; eyes on Pilbara power</t>
+        </is>
+      </c>
+      <c r="C119" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D119" s="17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPQTRxenprUFZmM2JIMDNPZGVVV09IakN5STI4ZFJVQmEtemVQUlJCRjdtbGpKWEZFOWVRd2ZYZk4xNkNHclpMSEFZLUpBVHhKaFN5Q0Y2bmhRWERpc2N4NEhua0VSQnFpVmpxa29tSlFNOHJRaFROMS1mTHBGdzZ6UlhLaVpqaUJhOEs3Y0Iyc29KY01XUXR3R1gwOXJHQUp2QVpNYi03NTZhLVgxN3VlODY4T0E?oc=5</t>
+        </is>
+      </c>
+      <c r="E119" s="17" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="17" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>Luke’s Bánh Mí launches budget mini meal deal</t>
+        </is>
+      </c>
+      <c r="C120" s="17" t="inlineStr">
+        <is>
+          <t>QSR Media</t>
+        </is>
+      </c>
+      <c r="D120" s="17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPQmh4NzlPa29pOXFmeTlKVFVUenNqdTF0VGU2REVwaWRsR3dKSEs3NFlTcGlscFRhRWRtV1JtVmFNTzJCb1d4d1NrUm9mMzBKcDBmM2JBbWZPTEVNdWZ1ZlVZZW93bW14Ull1UTNLUDh6WlZ2RUdBTS1NZEg2dmRZc3BEd2dfTFRFUERwdERnZnZwMFRR?oc=5</t>
+        </is>
+      </c>
+      <c r="E120" s="17" t="inlineStr">
+        <is>
+          <t>QSR &amp; Franchising</t>
+        </is>
+      </c>
+      <c r="F120" s="3" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="17" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>Zeus Street Greek sets sights on drive-thru as next phase of growth</t>
+        </is>
+      </c>
+      <c r="C121" s="17" t="inlineStr">
+        <is>
+          <t>QSR Media</t>
+        </is>
+      </c>
+      <c r="D121" s="17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNTEEzZ2VJMDdRek9JdGZCVVpJRGZoSjNIWjNiN3h2OHR2RjUwUG42SzViRUpteXRURFZzbFBpR0Q4TFdianc0SjZkc09DU01MY0hMLWRNbXQyYUVNai1BMUxFM0pZRWJaT0cwcmFna3pRS253R1FUY3UxOURmRkcwN3Fmd0VfLWVONzJJXzBzX1U5TFBQTFMtSURtZUV0TDhu?oc=5</t>
+        </is>
+      </c>
+      <c r="E121" s="17" t="inlineStr">
+        <is>
+          <t>QSR &amp; Franchising</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="17" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>From $5bn to $50bn: The end of an era at Blackstone</t>
+        </is>
+      </c>
+      <c r="C122" s="17" t="inlineStr">
+        <is>
+          <t>The Australian</t>
+        </is>
+      </c>
+      <c r="D122" s="17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgJBVV95cUxQc251ZVp0SEY1TnpWc2g4WERmLU9INk5VTUJHa3RGWGRmbWYzLV9MQW9rZmQ3bjVTRVI3R3NDbVNPdW9GTksxNUdrdkk1eTk0VXNFZmR2V2FBQWtnZGRmZkVMbm5QTUo4dFUxSGlOS0FSRmZZcThBVnlqWTN0eEUwUjFPdjhFb29BTXFWTTdHODRYelQwWUNBbXdNOElkQ2UzRU51VjM3SC1HZmpEUlNJUFFKRmdPWnhqNlEtVkNUaUtCbEc3ZWo2NFVIVktNMTQyd21lekpHVjlXOGV5WEhIZWJrU0ZTTFlrSkZnYlUxOWdUYnhna2JZTlhGYlAwMmhDYlJfZ1o3bVVDTnppS1HSAZMCQVVfeXFMT2E5cHJhVE9FUlVLN3RPakxmMHZKN3JLVUEwM3FSdmlfR0o0X2tybDFQWTg3NmZsYkE5LVRjX1dQMHVhNHBXNkhVRl9kd3lGeFdIWUV2QVFyYVgzWXU1Z2dpLXd6OGtUR0Z5SkdZc2VVM0tDU2MydXZSbGZOZjhUOEg0YXlBN2EtVDk3Z2FUM3pGY2JkTXdGZ2I5U2otVkJ1S3NhTXRBVVNqS1FvYzdPeHdaY3dqNlJmdkhwWHZCdjVsMXNibEc3aDFBR3NkRkZpdVRzU3Nad3Y0N2gyaHRQWlY0cGV2SUh3T1NwdEJEZTh3T3laM1B6YXlzVHlRRXdHc09tOFVKUTFfYjU0aFpJMDRlSTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E122" s="17" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F122" s="3" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="17" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>Starbucks opens first retail outlet at new Town Hall Station</t>
+        </is>
+      </c>
+      <c r="C123" s="17" t="inlineStr">
+        <is>
+          <t>News.com.au</t>
+        </is>
+      </c>
+      <c r="D123" s="17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOTnJ1YVF6V1dqMm9HbmdUZEk3NlQtdjRxT28ya19fbjRKMlJRb3hsam5zdDg1cnEycHc4STRPdENPQnlMQldBbTh3NXlYb0tUNW9WS201NTZ0M0xvRE8zRkVYcFlNSmdOeVZvbXRMVzJMMkV6czFPX2djSFdKNlhWbUQtNUpMcnhFNnpfa1RPY3Q?oc=5</t>
+        </is>
+      </c>
+      <c r="E123" s="17" t="inlineStr">
+        <is>
+          <t>Retail &amp; Consumer</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="17" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>The ex-Platinum quant who has won billionaire Kerr Neilson’s backing</t>
+        </is>
+      </c>
+      <c r="C124" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D124" s="17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNMkpmVTVUVU1WZUZiRWlJUkRId3BhS1hqM09aM0FSODBFNE96SDlKWG11Qkw2bjVSNFFrc0oyWHBBVXNYclBYQklIdnZBNEZ3b2NvZzdHZWNrV1JhbWI5aUpBLXRqTjIwSnhRSlFtdUlTU3VUbVMxcmtYZzlnVEsxellFb0dwb1hhME9QbERGcU9aXy1rOEtyQ0pXZW9KcENIem5TMjhUZ1VydFlrVWI3cWN6aGJROGFwWUFlNjQweTdqYkptcHc?oc=5</t>
+        </is>
+      </c>
+      <c r="E124" s="17" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="F124" s="3" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="17" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>Media bosses: ‘Australia shouldn’t be held to ransom’ by AI giants</t>
+        </is>
+      </c>
+      <c r="C125" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D125" s="17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPSGdRM3JDVld4OG5UWk5RdlVZVlU2LTFKUjdzVy1HejgyaUxMWHhmUlJnN1FrY2dSTTczczU0Tno2TUVPWDFiZk9TTjJTNlQ4Yi03MWpfdVEwWGFaQm9ydjJpaGFkekZHME1xNUswcWF4b2Y4TUxkOUpOa0dFTjlYVmhVMnFPMXlEcGJjeXZBR0tFaDZUa3Ixd1lIai1qcml5OE9SM1dTcUVkWW1HdFJTUFBJZUU0Nzg?oc=5</t>
+        </is>
+      </c>
+      <c r="E125" s="17" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="17" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>PLI scheme for food processing industries sees Rs 9,207 crore investment</t>
+        </is>
+      </c>
+      <c r="C126" s="17" t="inlineStr">
+        <is>
+          <t>News.com.au</t>
+        </is>
+      </c>
+      <c r="D126" s="17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOcUwtamFxVTZ0YTdEOTBsN1gxNlphTV84aGJoRnFFTkFkZDhaT2VzVkFDT29hMU1Xa3BLeWFiRWlXT3Noc3VVVkg3WkphSFMwS3k2aWI4ZlhfcDN2LTV6Q3E0YnNXbEFVZFdUU3U0R293aEtlUmxlLXdFWXl5MHh0X2hWYnNvbU5MLUNCRm53aVpJa0E4OUxuNnN3X1FwUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E126" s="17" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="F126" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>

</xml_diff>

<commit_message>
Update news log — 2026-03-31
</commit_message>
<xml_diff>
--- a/news_log.xlsx
+++ b/news_log.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -87,6 +87,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -495,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F126"/>
+  <dimension ref="A1:F146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -539,7 +542,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -549,17 +552,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C2" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D2" s="16" t="inlineStr">
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D2" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E2" s="16" t="inlineStr">
+      <c r="E2" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -567,7 +570,7 @@
       <c r="F2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -577,17 +580,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C3" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D3" s="16" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E3" s="16" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -595,7 +598,7 @@
       <c r="F3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -605,17 +608,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E4" s="16" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -623,7 +626,7 @@
       <c r="F4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -633,17 +636,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E5" s="16" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -651,7 +654,7 @@
       <c r="F5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -661,17 +664,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -679,7 +682,7 @@
       <c r="F6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -689,17 +692,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -707,7 +710,7 @@
       <c r="F7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -717,17 +720,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5</t>
         </is>
       </c>
-      <c r="E8" s="16" t="inlineStr">
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -735,7 +738,7 @@
       <c r="F8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -745,17 +748,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5</t>
         </is>
       </c>
-      <c r="E9" s="16" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -763,7 +766,7 @@
       <c r="F9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -773,17 +776,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D10" s="16" t="inlineStr">
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5</t>
         </is>
       </c>
-      <c r="E10" s="16" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -791,7 +794,7 @@
       <c r="F10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -801,17 +804,17 @@
           <t>Zarraffa’s Coffee celebrates 30 years, eyes nationwide growth</t>
         </is>
       </c>
-      <c r="C11" s="16" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOcXNzUkRLemZEOWtOZjhvRUtzcUZrSTdzV0s0LUJTd2NGRk1Gb1NSLUR5Rlh3NUdWQUJkVWctb0toUFBRajlMcWV3VnNyTUtydy1PSUoyb1NCOGVtMUZqRVN0MzFkVkNlOUZNVXlHN2kzREhSdWJQUnJqa0pnUzExTVZSc1NCVFZSNlBSUWNfWnZ3MC01aUx0UWF5SkNOaHI3ZkE?oc=5</t>
         </is>
       </c>
-      <c r="E11" s="16" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -819,7 +822,7 @@
       <c r="F11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -829,17 +832,17 @@
           <t>Zarraffa’s Coffee eyes 200 outlets ahead of 2032 Olympics</t>
         </is>
       </c>
-      <c r="C12" s="16" t="inlineStr">
+      <c r="C12" s="17" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D12" s="16" t="inlineStr">
+      <c r="D12" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPMUFjRTlGVFBqYzlPWXdzQ0dKVVlhWGxncUQxTDd1R0VHcThlV3ExVmo4SlBGSHVuUGZrMGNqSVo1YVpDWHViMm5KZWIxcHNMMHo0b1FQcmxUNElDR2lEeWRuLWZIN2lyQUV0VndEUWNkNU42Z3AzNXRlbm50NzhtTXZ0Q245dF9hNzBxOENuMXZsVlU4Z0JGVElR?oc=5</t>
         </is>
       </c>
-      <c r="E12" s="16" t="inlineStr">
+      <c r="E12" s="17" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -847,7 +850,7 @@
       <c r="F12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -857,17 +860,17 @@
           <t>Aware Super appoints new head of private equity</t>
         </is>
       </c>
-      <c r="C13" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D13" s="16" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNVHJXNWEtdEZZUW1fZzdYMTB4RklBTUh6dUNKQ3BrTlpYUnBwRURIVGZjWTV0OUxScnhGMVNSczhLUjVqOEwzbkR2WWlEbmF4ZkNUdHNQY0J1djI0REctbHd2SVhUNlNCa2M5bFhOQ0JPU0RHOVVTQkEzRDdGMjRZbVFDOUdlTXNNczlmZWF6bXlfbEFGRE0xbkZQaw?oc=5</t>
         </is>
       </c>
-      <c r="E13" s="16" t="inlineStr">
+      <c r="E13" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -875,7 +878,7 @@
       <c r="F13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -885,17 +888,17 @@
           <t>Commission wrinkle over UP Education sale</t>
         </is>
       </c>
-      <c r="C14" s="16" t="inlineStr">
+      <c r="C14" s="17" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D14" s="16" t="inlineStr">
+      <c r="D14" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxNSV9GMjhqM2ZSanI2X0w2OVlQVFRQTUoxYzAxaXVZMmU1REVTcHlUeEltdXJtaXZrcUJWdDZxNGpYTTZYSFE2TkZHeG9OaVRZakoxV0s1U01TVjJpWlhaSENfNVhucG5NVzFMbTVBY25zWGRSODBtRGtkS1owVTlJWnNfcTJ5alFnbVl1SU9aUDF1QWxJLTBSQ3kxUUFlZnpJMlVEQndFSGRGbDF6WVBUVHlCcDM5Qnh3R2xBMG9xN2FLckNzbUFOWDI1aVF1YV90d0twd0ZmMnUySDBMdG1R0gHkAUFVX3lxTE5EWVp6VzZWb01TRmlHSS0wMExldkJwSHJjdlZXdElsRlpBTEtVMkd6VzNQa1RpVDNsOFQzaGZ2VHpzUnBDYk82RmZGQWJuTmVQMXhxLXVmdVFxTVZOZTBsOHZ0V3cyVVVkNWUwVUxSc0xNSU92ZktpdFRfYnQ4WHBTX3A5bFhXZ1YwZXNrc1BSZEU4LVYybnNBd0dCdk92OFUwclJCMzdoU0ctX1pEdTAwY0JiTWQ4S01QRE00TW5EUEJwR2YtczZ0T005bTJnN1RDY2p6NFF1SndfLUo4QzJUWk1tRg?oc=5</t>
         </is>
       </c>
-      <c r="E14" s="16" t="inlineStr">
+      <c r="E14" s="17" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -903,7 +906,7 @@
       <c r="F14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -913,17 +916,17 @@
           <t>Gloria Jean’s owner has an angry shareholder on its case</t>
         </is>
       </c>
-      <c r="C15" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D15" s="16" t="inlineStr">
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPTnZwUVBCdTFJZWkwc0YtVmJqMkNPcUR5RktjMlVURmhROFZkYUpXM01iRUh3SnJEUElxRGlSNk9DQjZSdTdNdmZwWWpONjlmR1hoMl92cUNmd3M4cnJhVkNqc095MmN6WXBYUmdEblB0eERtVDdlUU4yNGFjXzVnT19rOERIRzVPNzY3VDNNRS1tVGVTX3pKMVRpTXZVR1ROLURBLWtJbVZhY0lSU09DNkE2NzFLbEFU?oc=5</t>
         </is>
       </c>
-      <c r="E15" s="16" t="inlineStr">
+      <c r="E15" s="17" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -931,7 +934,7 @@
       <c r="F15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -941,17 +944,17 @@
           <t>Oporto-owner Craveable Brands hires new CEO from Domino’s</t>
         </is>
       </c>
-      <c r="C16" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D16" s="16" t="inlineStr">
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNNmxfQVc2Umc4QWwzSTdsZTFvejRzTzZxXy1ScGlhXzh6bm5JS3IyX0xTNDVBNjh0cXpPbGhxNU5xUHhQN3EtRF9aV3FEc2JoSG5QTU1WeU1TLUJfZzVUT2N6dXloQXhZaHB5djB3dDFKN1llVmI3UVpKNjJTNlcyV0ZDcG9GdVdSdW41ZkN1b1N3SFFIUzcwRkQ3UHY2TmxERmZwTlA0RzU?oc=5</t>
         </is>
       </c>
-      <c r="E16" s="16" t="inlineStr">
+      <c r="E16" s="17" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -959,7 +962,7 @@
       <c r="F16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -969,17 +972,17 @@
           <t>Brookfield, BGH Capital rub shoulders in ScotPac’s data room</t>
         </is>
       </c>
-      <c r="C17" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D17" s="16" t="inlineStr">
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPMVlxbzlQNnFXWnJFNU11Y1BhTTVqbjN4RG1nbkZuN0pkdDFFaUhJN0RaVnUtWDlZSGJWR1ozQXk5UUx6RVdOcjBPU2t5UzN4T0JvUFJISnNvVWxQemd3blNHZjRQVVVZQk1nZER0Y0JfY3VvQ0t1a09sM1RTS2c1YTJyUmdzYWh1WGRUNjl2dkdzYTJJeHVhMTdqR3Y5WVlHVEtSZHp1cmVYYmM?oc=5</t>
         </is>
       </c>
-      <c r="E17" s="16" t="inlineStr">
+      <c r="E17" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -987,7 +990,7 @@
       <c r="F17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -997,17 +1000,17 @@
           <t>Payments player Pay.com.au hits the road(show) for $850m IPO</t>
         </is>
       </c>
-      <c r="C18" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D18" s="16" t="inlineStr">
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOMFZleXZrbU53TzBlakI2ZmJKTjlrN3BoQlRaWjQ5cXFzTllKWmFoRm1UT2xDUHBtNC1QNTNiX1BwSzllMkRZdHIzRlAteDREaUczN1JTNTByTW1jNnR3d2NnR0RxUDBxeHYyWU1CSUs5MEZad2JqSGF6ZUxHZUNtZmFQaTJZZVJVZ1B4MkZ6V09QMWIxaUNHQmVzTDhvWVA1Ty1UbHgtQnRrQQ?oc=5</t>
         </is>
       </c>
-      <c r="E18" s="16" t="inlineStr">
+      <c r="E18" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1015,7 +1018,7 @@
       <c r="F18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1025,17 +1028,17 @@
           <t>Another year, another IPO cold shower for investors</t>
         </is>
       </c>
-      <c r="C19" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNeEhzYzQzdjR5MDJCWkd6Q2VLdEZzbzRoWnNOcXFlQjNfMlV4Q0NQRjExMlNhT2NPcnRBbW1sZUkteXo4N0dGaHNNeGZJOEZ2aXFvdmZiN2V2QzdOMzFteFRnY1RVRm1rQXltWmY5VFZOdFVNNVpudVp1dTlrcFM5b1k5SmlWQllDMVFXSjA4ZVpSZHgtV2JpWDJ4SkFRbVE?oc=5</t>
         </is>
       </c>
-      <c r="E19" s="16" t="inlineStr">
+      <c r="E19" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1043,7 +1046,7 @@
       <c r="F19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1053,17 +1056,17 @@
           <t>Priceline Pharmacy franchisee sale narrows to final four bidders</t>
         </is>
       </c>
-      <c r="C20" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D20" s="16" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNR294am9sYWNiQ3FVT1B6YlV5ejMyeHAyT0FibTFVbU5pcjZyaVRyazEzbFkxd0lrcnpZNGpTYUx4Ykl1Xy1sZF93M2Nid19ydUFwbUJ3ZHozaURaNkRoOE9OMnRBRGZfQVdCVWZCaVhhNnZSRjlwYUdDVnp2WU9HUkJxbE1QMV8zdWxYRTNBQWktR0xSOFU4dmtXZWk0am9SSU92NWp6QUZmTVU5TzJEOEJNak5fQUtN?oc=5</t>
         </is>
       </c>
-      <c r="E20" s="16" t="inlineStr">
+      <c r="E20" s="17" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1071,7 +1074,7 @@
       <c r="F20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1081,17 +1084,17 @@
           <t>Private equity gets better image of Qscan</t>
         </is>
       </c>
-      <c r="C21" s="16" t="inlineStr">
+      <c r="C21" s="17" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D21" s="16" t="inlineStr">
+      <c r="D21" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxPRjVmT0hDRjZLblB1VHdPRmRGeXhKdDJHdWxDTzV4RDZ0VzdHaUFfOVlnZjRQMWhKcWMxby1oRDR6N2lQZkI1UDE1REppS3c4LTVmU3p5b2wtblRCWnhNajFnZGNHaGRJUHFMUGRtTHAyQmIxOHhNNTgwRWVSeWp6ZWRxbUY0WVhiUnhMRUpDLXNwS1RuelJldTk0Z1R0WHg0XzNXNTA5Rk5TRFZhU1RNVnN2TlZuaFE4OWtIYXQ5a2VGSW1UWmt5Rlc4Q2lIXzF3YlkwNVhfUzJDV0dQdVAxa2RKc08wRGR6TlB2Vi14QV9BdlhyaTZsM2pEVGZycTjSAYQCQVVfeXFMTWpnb0lWQmZ6MTFnRGhWNTNqczk1TWhTcUFEMVpDNnJ4ZWVxVlRUODhJXy03NHdGZVJlMmhyUHM0Nlh4NlZtTzRhQ0xxRDFLVHNzUVNfbWxhS3BLUEQteEMzZHRrc0F1eFRzYmxVNDZlSURyZDB5bF9wQTNRRU5yZEs1Z3pFRTdwcFBaMkNlN0JvT1NEYkFWVUJNcHJqcEM5RVJYa0JFUVl6cThyQXloaERzQjhkTUVPakJqb0hzNVlwSWxNS0dmZkNFSG9Gb3dNUnVvUnV0d3MxSmpzdFZKTHJ2RTQwRUoyMEVLLWMwT1NnOHdXVl9lRXNDWEFndzJFSDlZU0o?oc=5</t>
         </is>
       </c>
-      <c r="E21" s="16" t="inlineStr">
+      <c r="E21" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1099,7 +1102,7 @@
       <c r="F21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1109,17 +1112,17 @@
           <t>Oporto CEO’s first year reshapes brand and network strategy</t>
         </is>
       </c>
-      <c r="C22" s="16" t="inlineStr">
+      <c r="C22" s="17" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D22" s="16" t="inlineStr">
+      <c r="D22" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPY25mNTJfT3FiVlBPZE5CcVNkR1UzR2xWaUtJSmxhU3EwcEMzQi1ISDFSajlCQWk1UUJpZVJ1Q19ZV3Jjd0Noc0l3OExpMXhSQUVVdHhCLTBlOXNoZzA3UXZBdkR1VHBvMmVsZkNhUFJndm1DdGpnX2w0ZVViU2phZ1RmYXY1SlhwUnhKSUxBQVZZUXpqNHQxQmo0Rk1iV0g0OW9qUS16eWRSNW5FaW1yQQ?oc=5</t>
         </is>
       </c>
-      <c r="E22" s="16" t="inlineStr">
+      <c r="E22" s="17" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1127,7 +1130,7 @@
       <c r="F22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1137,17 +1140,17 @@
           <t>The Melbourne restaurant our reviewer grew to love</t>
         </is>
       </c>
-      <c r="C23" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D23" s="16" t="inlineStr">
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOc3YxQTljcHJXVWtRX2ZGM2lpM2pILWNwSFg0MFJrNmNWX0ZxRG9nV0J5N19qRWh4U0hPXzNmVVZwWk9wT2kzaFNrTlV3NEQ1Q3JpaXVIYlBHb216Q3VYVWdSRXMwdDl0SmYzdnRlSDFUYVRmRGJyZVlRZDJKTHpJOUctYlF1RDZSYjloY0hfZy13QmFTLU9UNjkwTHc1bjlGcGxoZ0ZLVU1GWTctZkdLZU9zSGhEZEpKbXJnaWJfZjd2OWs3?oc=5</t>
         </is>
       </c>
-      <c r="E23" s="16" t="inlineStr">
+      <c r="E23" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1155,7 +1158,7 @@
       <c r="F23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1165,17 +1168,17 @@
           <t>Crescent Capital strikes Benson Radiology deal for close to $400m</t>
         </is>
       </c>
-      <c r="C24" s="16" t="inlineStr">
+      <c r="C24" s="17" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D24" s="16" t="inlineStr">
+      <c r="D24" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOLTNrWG1ZZlFoU3pDZ3E2SEgwMlhzQkdtQUYzaHZTZmYwU3ZhMnE0dlkza005VkZmZ09NMExlWDVncnBmYVVISXJ6X1ZjNHhpM2RnSlprY1dnbndJNUczcDVtNXNRY3pVNW12bm5rUVdqVmR4R0JlVHFuN0RwTlFkR2xrbFFpSl9jcm5oSjk3aFM1clBSVDhnbkhoWUREeUhsbVpvQW90d05xOTdfOV9nbW5POFdmelJkVlpsUlRuYl9odmRNVUV2S0pCMFBMTS0tcVhGVGFYU0h2d9IB3wFBVV95cUxPWEs4R2pxdThPbHJHb0dBT183SkRHTTlXNzdWazcxdkd1eGx2VlAyM2VVbEtEbWxTZ1R0TlBFRmRMZTFoalgxSmVVRUJFR0c0RFYzZVJFODg3dWxicU9pOHppeFhjaVp0WWlyTnUzV1dyZXdkMHBDVHI4LUVQdjc0cWpheU55NTlvdWdCZmVoODB0Mm5fbGNCTmQwLUhMZ0psQVpzb3BEUnJpSkRnOUM0c0VCdUp5N3g5MkhaM01vTHJ3NWd0ay02UXZUUG9nVkxicVc1Z0xjWGhjUDRDVjlN?oc=5</t>
         </is>
       </c>
-      <c r="E24" s="16" t="inlineStr">
+      <c r="E24" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1183,7 +1186,7 @@
       <c r="F24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1193,17 +1196,17 @@
           <t>Dual-listed giant Capstone Copper flirts with $600m-plus carve-out</t>
         </is>
       </c>
-      <c r="C25" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D25" s="16" t="inlineStr">
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNcVh4blRkQnoyaG1TajhVV0lrOEJRaHdTZWtzUnJHaEdaSXNRWThGTHlVdGl4dGJ1cTMwZ2pLcVNzUXRYNlZzVzhvaXdkNGtVUG0wN0FrMHB0R1I2Ry1jcEgtSWUtajI0cTFMRTlfdzBuMWtrZmJOLVUtMkl5dW85dFp6dEhEOHhTNzdfOFNFSGtlT0MwQnRlY0VhcUZBNE9RYzhQcDdOQUFnYkgzd0V0N253SQ?oc=5</t>
         </is>
       </c>
-      <c r="E25" s="16" t="inlineStr">
+      <c r="E25" s="17" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1211,7 +1214,7 @@
       <c r="F25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1221,17 +1224,17 @@
           <t>Guzman y Gomez unveils a new menu under $4</t>
         </is>
       </c>
-      <c r="C26" s="16" t="inlineStr">
+      <c r="C26" s="17" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D26" s="16" t="inlineStr">
+      <c r="D26" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPMjRjRTV2a3BJc3AzdDNOQktoYjBvLVZSODVsc3lKQ3pET0lxUlpkc05NcVlKRlZITjVJbjkwLS1DUFJNMGJ1amJKTlp3S3VqMWJaU3YtUENEN01rUEJiV1FNZTRXYjcyV08zZzlxNDVOSlVOTlJDOGV3QzBQcUpKa2Zab1ItNlI3ajZVVTF3?oc=5</t>
         </is>
       </c>
-      <c r="E26" s="16" t="inlineStr">
+      <c r="E26" s="17" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1239,7 +1242,7 @@
       <c r="F26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1249,17 +1252,17 @@
           <t>Can Sydney’s burrito king conquer the $676b US fast food market?</t>
         </is>
       </c>
-      <c r="C27" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D27" s="16" t="inlineStr">
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNM0ZFcUpLN1dUZWUyaE1LMnNZVGlEbkNNQUQ4Wmd6QVFlTy0wZDVHdnlja1gzMEZTbVpKU1Ftb3VKZ2pzajcyWU16NUtUTmR0TlZMOVhMRUNqZXZiX2d2NWY0YlJDOFhhYUE0SkhMRUprNndXak8tWGdERU90cmMxTkFjcFFVSTd5VlZ3NFVKOXN3M255MFhzZThmbi1VUGMyQ3E4d2pYcFlJckY3QlVBdVJJeF9qUQ?oc=5</t>
         </is>
       </c>
-      <c r="E27" s="16" t="inlineStr">
+      <c r="E27" s="17" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1267,7 +1270,7 @@
       <c r="F27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1277,17 +1280,17 @@
           <t>Drone maker Innovaero prepares for ASX float, taps Euroz Hartleys</t>
         </is>
       </c>
-      <c r="C28" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D28" s="16" t="inlineStr">
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D28" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNU3JrejNRZ1VBZVNVV29NMkFPVmRsWE4yMVZPcjk2aUNUTHFJUGFyQ1VnZEZiZlIzQW9VVzRNNDNRR01jcHo3X0tqZjB4bzhMTTI0Y3BwYUh6OGRUUGt2REIxV09oRnJoVWlVelZWaUlWUmlPQ3dJdi1TejcyaXB1Z0x1MEJRSlB3SGMwVGdXaXJJNm9TVllPOG5JZC1feEV3TVhTeExGeHR2RHFIWlVCOXh3?oc=5</t>
         </is>
       </c>
-      <c r="E28" s="16" t="inlineStr">
+      <c r="E28" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1295,7 +1298,7 @@
       <c r="F28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1305,17 +1308,17 @@
           <t>Bain flaunts Estia 2.0 as IPO roadshow gets under way</t>
         </is>
       </c>
-      <c r="C29" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D29" s="16" t="inlineStr">
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNTEN1cGsxNDN2c1NqUzB6UmJ4TFl0NGZjZVN3U3oxMlVFWTF4WUZLQS13dUxMV0N2ek1XN2VURTNVWms1NjdXSm0waEdaTXQwdTdWY1MxZ1V3ZnpEcVJtczdOWGNNZ0RQNzRZLU1MTTgtRW5DZkctbXBGMmVXVXdPZW5pNThiRHEzWnB2eFZzTFZTb1ZkeW9LendkNDd0cXRid05ZSGZYbW9NZXdOLVZWODdZU3hVcTA?oc=5</t>
         </is>
       </c>
-      <c r="E29" s="16" t="inlineStr">
+      <c r="E29" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1323,7 +1326,7 @@
       <c r="F29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="inlineStr">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1333,17 +1336,17 @@
           <t>Carl’s Jr. Australia unveils nationwide freebies for Happiness Day</t>
         </is>
       </c>
-      <c r="C30" s="16" t="inlineStr">
+      <c r="C30" s="17" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D30" s="16" t="inlineStr">
+      <c r="D30" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNVWgwdjU1NDFWalBfMTFYX1dQOWNDbG1FVUdlcS1LTVlHZVRRTVBWTjhSMnpkTXRXNlFJdllGQUp5Mm5ObWpIazd1d0RJa3QtdFBZN1hOenBmVzBEU05wM0gtNUxPeWpsYkxyVnhWWFFOU2Y3R0tXcmNkeWhpWDh2eDZBdjNCMHhuc1lHYTZHblBPVkpfRXpKd051UWlNc1hm?oc=5</t>
         </is>
       </c>
-      <c r="E30" s="16" t="inlineStr">
+      <c r="E30" s="17" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1351,7 +1354,7 @@
       <c r="F30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1361,17 +1364,17 @@
           <t>BHP and Woodside appoint new CEOs in major mining shake-up</t>
         </is>
       </c>
-      <c r="C31" s="16" t="inlineStr">
+      <c r="C31" s="17" t="inlineStr">
         <is>
           <t>ABC News</t>
         </is>
       </c>
-      <c r="D31" s="16" t="inlineStr">
+      <c r="D31" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQbTg5VFJLbWJfcy1uV3ZReTJkTndzX01qZ2MxNWkzaWZRckNLZUR1Y1VsMVRNc2FySC13U0NzalFEb3k1R3BaUEhfcTV0N1M4Q1dpSlo0YXI0UFhrMGRab2RiYV9DQVNVX01ycFc5ZFZrZWZqc1VRZXoxLVEzSDJLclJLSWg5bzN3R1I0bG9lWjVDaHE4?oc=5</t>
         </is>
       </c>
-      <c r="E31" s="16" t="inlineStr">
+      <c r="E31" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1379,7 +1382,7 @@
       <c r="F31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1389,17 +1392,17 @@
           <t>Next Capital sells Enviropacific unit to French waste management giant</t>
         </is>
       </c>
-      <c r="C32" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D32" s="16" t="inlineStr">
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPR3lFbERLR2FtdmJUU3BDU2thZk00YmFHRFhXR2VBVXhQSURTeE5ONVJKczBwbzlFMnR5cmhxMnM0bzlJbWo4SXl1dHpqYWxxMUJBRjZHVUtab1RYZjZMTnpGc3FzMWQ2NjNEdGU3NTZwa0diM1lJS1haYllwTldLZlpZbXp0YzlxcDh0ekcwTy03dDdPcnk4b29HZVdqbHhZY2JPR2drM2puSVpjUzZkVjNpZUE4dVMwYlE?oc=5</t>
         </is>
       </c>
-      <c r="E32" s="16" t="inlineStr">
+      <c r="E32" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1407,7 +1410,7 @@
       <c r="F32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="16" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1417,17 +1420,17 @@
           <t>Future Fund private equity and real assets chiefs head for the door</t>
         </is>
       </c>
-      <c r="C33" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D33" s="16" t="inlineStr">
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPUHNHRFhFMVdwVld6RFRZUFd3QWNOd1kzeS1QdnJxMERFSnE5LTdZcDhDYlVGcWZMeWxlR0FSRWF6YkZoQVZrZU9TQ1E4YTEydUJnOFE3enV5Rmk5UnF5VEdYZ1FMUWpKVjdjMlZZUGFsU0tKcV9Vbl8zcHp5aVF5Z2JMOUZocHJqRXNRaEp4Nm5CbDM1WkdIMHdQS2xqQnE2Tnh3?oc=5</t>
         </is>
       </c>
-      <c r="E33" s="16" t="inlineStr">
+      <c r="E33" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1435,7 +1438,7 @@
       <c r="F33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1445,17 +1448,17 @@
           <t>‘I actually started to die’: the new billionaire’s epiphany</t>
         </is>
       </c>
-      <c r="C34" s="16" t="inlineStr">
+      <c r="C34" s="17" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D34" s="16" t="inlineStr">
+      <c r="D34" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxPblkxbHVrdnVKY1pqQzNyWGNMZm9UYmY3dzlPaGQ4Yi1tc0U1akhrVWdIaXBpM05aZXRwTXE1eDBITlZpbDkwRXNrWjJ2YXBzX0VCY2JSLWhrVmpjSTE5eE5rLWgtc2pRZEdXbmhhWU1KeFExZDBGS2pjSkIwV0FGbndBZVAyQkg4WFRsengzSGYyZkFfQnJsQ18tUHJGNDd2T0pzZElPSVJTQkl2Rm5QTExJNHhmU2dHOHJGdTdzU08yNHRtd1R3Q0cyOF8taDktQTZvVXVBVjN1d0NHMmtFOHBWZXBFcUFWa1IyWGNDTDZUT3lQSXJHOVhxTFQ3b3RH0gGGAkFVX3lxTFBZQ3BFQWl5dEwwLW5yVWJuMU8zcXBPdE9pamRVSWVkbWNyVzgydGVOaDBROUN6RlBDbjdld05DVmZyb0R1eEN0UERubzZRU2NiMTQtVV9XNS1wYmlvZ1paM3RaOUlrTzJka0tXVVJEamFESGlSdXg2bDk1aUdhUVhBcXpnN01fX0Y0cTNvcm5DdEFFLVVERDFKTWxKZFR0UzAyblJqVHBua2JoYUdzeUNMb053ZVczWUFQU1AtVHV1d3lSSDFfZFh2cEkxSGw2MEdicEVsb2pLQ1RuQmdaRl9xNUROS3pKR2s2T2wxTTZ5bEwtTUNQNU04djFHTHlPbXVLSW9YSUE?oc=5</t>
         </is>
       </c>
-      <c r="E34" s="16" t="inlineStr">
+      <c r="E34" s="17" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1463,7 +1466,7 @@
       <c r="F34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
+      <c r="A35" s="17" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1473,17 +1476,17 @@
           <t>Ironbark shuns private equity as it hunts for cash injection</t>
         </is>
       </c>
-      <c r="C35" s="16" t="inlineStr">
+      <c r="C35" s="17" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D35" s="16" t="inlineStr">
+      <c r="D35" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxQZWFaeVhldi00VkV5ZmEtS2tjcWdFWG55OGpCX3IyN25Rb3ZFV0ZKVm1aSE1WbThoYVY4ZEdfODVGX0RaUDV2Ul9HS1JQMDFCT05Fc2FaU0RINTMwbDRveWFsOFJSM2ZqTU9tVGxJSEl2ZmhhUHFHT3dqYkk5TUtvMUQySnZzTWw1MzFNWl9aVzhkSEZ4Q3YyWjRMUmpIdmJkdUVKWE54Nkt6bTd2dGFSUFoyNkgxTHh2TGVGak9ja0dFZ0xQM2g0S1lmQkZiWWtUcTVNdHhBdC1KeVRQcDA2dnpmeHRkWEnSAewBQVVfeXFMTWtYRDRSaHNULW1HanowRnpMdFF2VVMtZW1SV2ViZXlGaW02WlIwUzRZMGg5WDNrOUR4eDlGOEt5eGlqV0pfVDFhb0JEcS1faEJodWxyRnB3MkozOVJyT3NvM1I5MzdDcXNnUFNSdkRDamUzZTRQYlk0c1VIQUNMZ2ZzOWVCb2V2MC1aSTZLWkFkbW9GYk05b3RmN1htWENTeDh3SU1WYWJMcWx2eGUzZmwwVXF6czlnRGdXbE1vRElyVG0yM0ZzXzZ5TFh1YlRGNU9MQ1p3NnVZSFB0M0xBcGlueVZILXlVaXdqUkU?oc=5</t>
         </is>
       </c>
-      <c r="E35" s="16" t="inlineStr">
+      <c r="E35" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1491,7 +1494,7 @@
       <c r="F35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="16" t="inlineStr">
+      <c r="A36" s="17" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1501,17 +1504,17 @@
           <t>Minister leaps to fix food chain</t>
         </is>
       </c>
-      <c r="C36" s="16" t="inlineStr">
+      <c r="C36" s="17" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D36" s="16" t="inlineStr">
+      <c r="D36" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxOd2NqakVWRnQ4anFZNkl4Zy03MkloX08tUkktRTZqeEtQWFZJeVhkMUJIb0FxUjc2UjhCQ3MxbmNxczNxblJIZ09IeTBGNFM4Wkh4ZE1qNkhJMjIwU2RtX1JxcEV1Y0NjWXF6eHpVdTN4ZUlYMGIwcDJzMXZMTk94VzFlcjhpcVZVSTJFMjhsQjVGWEJQYTQ3aTFyNmNEZ1F1b3NGTWd5WnFJWmxXSTJ2NlRLcjJHNWkwaTZ2YVR6S0w5WVo1Vlg0VWdxcWZoa3VaTmcxY2NVcnR2bFRWNGNvZ1M2Tlg5NzlvVXZFZm9B0gHzAUFVX3lxTE1uNERoR3p2dXRIa0g0RXI2MWR6N0c5U3NGcjFDQVMtdEpyNDI2bk8yOS1qUnFOazdiODl0Ymo5R1pwRVJ0UFFVdzlhYjRDSUFCU0FRak4xcVVrTHphdTdxcHNIMnEyRVZud1FURmh5T0JLOHpRM3lFbDRuRnZMYmtaRnRFTXh3dkszTFhFUmZlRmoydnlEbW1fZTlmUzh4NXNyeTZTeUhOSktvclJVc0NTZTVYMkdJZEUyY2RmVC1kQ1hwVEloSEtVMEo5QnNTUXQyME5IN1BPd1NOS3oyR1JtMHBFVTZEbzhEQmdrWUk1ZnZVTQ?oc=5</t>
         </is>
       </c>
-      <c r="E36" s="16" t="inlineStr">
+      <c r="E36" s="17" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1519,7 +1522,7 @@
       <c r="F36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="16" t="inlineStr">
+      <c r="A37" s="17" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1529,17 +1532,17 @@
           <t>‘Brace for swings on every tweet’: Investors bamboozled by peace talks</t>
         </is>
       </c>
-      <c r="C37" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D37" s="16" t="inlineStr">
+      <c r="C37" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D37" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOczZHTWFmTW9FZ1ZwSnc5Z3ZacGpsVDQ3LWw1a1BFT0tjRkphek41MlhNOU84emYzZUVwNV9xM0hyc1FUR0NHck14Qnh6c2JvQks5ZE02ZTNLWDI0dy1STi1HbDFDWW9yMDhGQXVVVzdkMzFXcnNNMVZHVXFMUXUteGtsVGhPVmhLcVZPQzlhTWNoYVVRMHF0cFhybWxzek13Y3ZjcjlXWjZJM2VYbm0tTmk4NExLQzQzX1ZPMVlhcnJxQkZx?oc=5</t>
         </is>
       </c>
-      <c r="E37" s="16" t="inlineStr">
+      <c r="E37" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1547,7 +1550,7 @@
       <c r="F37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="16" t="inlineStr">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1557,17 +1560,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C38" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D38" s="16" t="inlineStr">
+      <c r="C38" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5</t>
         </is>
       </c>
-      <c r="E38" s="16" t="inlineStr">
+      <c r="E38" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1575,7 +1578,7 @@
       <c r="F38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="16" t="inlineStr">
+      <c r="A39" s="17" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1585,17 +1588,17 @@
           <t>Wirth’s Myer rescue mission is caught in the eye of the storm</t>
         </is>
       </c>
-      <c r="C39" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D39" s="16" t="inlineStr">
+      <c r="C39" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNTlQ4NDRnWE91VG1YNENpSTUxNnBjZkljOGdYaGV0aVB5dkVOaEJ6SjZ1bVA4NXE1S1hjV1NjcVhQTEVpWEVNV0UtbzhQTFZLOWxIenZiaF9QM3F6bmJYRy1lbXVMczZ3TnBHNy1aLUtVcnBDdkl4TE0zRGN4U0FwSjNPY1M5S3AtdUQ3UUNmR0x4MlU2YXRuUDJEUm01SmZWakx2UjFvY04zRHk4Smc?oc=5</t>
         </is>
       </c>
-      <c r="E39" s="16" t="inlineStr">
+      <c r="E39" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1603,7 +1606,7 @@
       <c r="F39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="16" t="inlineStr">
+      <c r="A40" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1613,17 +1616,17 @@
           <t>‘Darling, I’m not going anywhere’: The rise of at-home care</t>
         </is>
       </c>
-      <c r="C40" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D40" s="16" t="inlineStr">
+      <c r="C40" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D40" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQS2k0M2otaldpNVFXdHRTMVNtZVhyUDV4VTNIcE5FSnFRaHNubGNQQzBVbllnNTktNGhrZ1lndzV5V1FpUS01SklRaTZmZHJkRzVsQmlsdEVmenZ4U2x6U01NeXdIMktBUW94TUE3R3FoLUxVcVhsVFI0SjVQVUFaZldnd3prMWMyaVRWX2J4aUdfQ25KWHpaLUlqSnhvQmM2TTRRQldGbm8tclFYRDA0TVdnU2g3QQ?oc=5</t>
         </is>
       </c>
-      <c r="E40" s="16" t="inlineStr">
+      <c r="E40" s="17" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1631,7 +1634,7 @@
       <c r="F40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="16" t="inlineStr">
+      <c r="A41" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1641,17 +1644,17 @@
           <t>Iran targets Israel and Gulf states as Trump looks to calm markets</t>
         </is>
       </c>
-      <c r="C41" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D41" s="16" t="inlineStr">
+      <c r="C41" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPLXBITXU3WTRtc0NYdnhTZHFaUTBCSXdldTBuSHliTlY1dlJONW43Qkd6Nl9pNmY1eDhzaHZoX19xYjBxMXR5UEhkVUg2M2k1MmhuVEwyY0JxbnJyemxVYUZjbk5BbkN4ajhPbW9ZeDhlRDRYTW1hN3k2d084c2djMEJUZTV3NVdPbllKUmFlU2JsaDV3Zk9CVFF0VDFkV09JSloycWdOUlVrREptQTJfa25LUEx5djA2SjNMMFY0RjM?oc=5</t>
         </is>
       </c>
-      <c r="E41" s="16" t="inlineStr">
+      <c r="E41" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1659,7 +1662,7 @@
       <c r="F41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="16" t="inlineStr">
+      <c r="A42" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1669,17 +1672,17 @@
           <t>Meet Christian Louboutin, footwear’s most famous billionaire</t>
         </is>
       </c>
-      <c r="C42" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D42" s="16" t="inlineStr">
+      <c r="C42" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D42" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPcXdGd0tMckYxbjZ5TVJmQ0Q4NFl2RkhHMHdlZDZsdGZ6cVQ0cUpaLWJTNlVoc2ZOQmtXNlFTRnJVMnVDTGc1NFNZN2g1VnotQlNQbzhlM1BJV3ZwQktOcGtac3RwSHRLZkR0b2l0eGIyVVlYdHJrc2hpT0pJbDR3LURPTnowZk54LThObndtMVkwV2VWQkluNVlWY0p4QVJGbE1hSGMzOW8zdkJZOWdocEZQWFBhTllNR1ZBSEg1TWRXUWd3X0t6TVcyY05PM0pF?oc=5</t>
         </is>
       </c>
-      <c r="E42" s="16" t="inlineStr">
+      <c r="E42" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1687,7 +1690,7 @@
       <c r="F42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="16" t="inlineStr">
+      <c r="A43" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1697,17 +1700,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C43" s="16" t="inlineStr">
+      <c r="C43" s="17" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D43" s="16" t="inlineStr">
+      <c r="D43" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQbHdYM2pSM2xkdmZ3OHhQc2tVUmhzclJWaVJ0aEwtUkNBR0ZUd3p1emF1M21jbTF1ejlKSkdDMnotcVNjZE1CYUlKako3WXR4MTJhdWNlSXZMbTBYanlmTWFzRGFIandXRUQ3UjN6SEV1bThvZjN2bDY0eFdpaTdMODN6TGFTdE5rd05TUll3MmNfTDhkQldoNDIwVlpoSl85aVRwcTd5Ymh3TDl4enZhZ2p4OExGY1ZaOFNEWFBB?oc=5</t>
         </is>
       </c>
-      <c r="E43" s="16" t="inlineStr">
+      <c r="E43" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1715,7 +1718,7 @@
       <c r="F43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="16" t="inlineStr">
+      <c r="A44" s="17" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1725,17 +1728,17 @@
           <t>Sembcorp Picks Banks for $2 Billion Alinta Loan in Aussie Push</t>
         </is>
       </c>
-      <c r="C44" s="16" t="inlineStr">
+      <c r="C44" s="17" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D44" s="16" t="inlineStr">
+      <c r="D44" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOdS1aaXZjT2VnSDl2TDdzZ3NfRElDWXdUXzZQYjFQMEZJOGlpaE5CNGdQMlZ2UFVHbUtfOXF1ZVBReExrdF85M0RWLWlBY2Y5dlRtWVdXLWp0Y1VrRmF4UGQzVUhxaHA4UHd1SUdFV21QcVFITXFHRlhzekdSUS1PdHlYRjdUbUQydU8wSktKVHRJQ0NaWE9sU1l6YXhtSWtBd3RwTERacnV4VzB6YlFhUE1QcXNDVXVESFcyeWY3cGhHUkRJcDhrYUtpTEY2UQ?oc=5</t>
         </is>
       </c>
-      <c r="E44" s="16" t="inlineStr">
+      <c r="E44" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1743,7 +1746,7 @@
       <c r="F44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="16" t="inlineStr">
+      <c r="A45" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1753,17 +1756,17 @@
           <t>Navis targets June for $1bn-plus med-tech auction</t>
         </is>
       </c>
-      <c r="C45" s="16" t="inlineStr">
+      <c r="C45" s="17" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D45" s="16" t="inlineStr">
+      <c r="D45" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxPNHRXaU5tNUVkd2MtcTg5M0EyQllrM0owMkZobGxLaUJxYUN2MUg0ZkdKdzU2YmxfanR3QU53cHZzNDI1WXgzRUcxOE9EZlluNmtNRUUzTGJPRnpfVVVOeFM3bFRNQmp6VHFBdi1mTnU4UDBvOEpMaHZPNXFtdUIyTlhuRExIVElSeVRUMGxjU0k5VnVxaWFfd3htWngydlhuR2E5aTQ5VW1LS01ac05rMGZoVFdOZzVyTzFhUDVsYkNrc0VQZmhubERSaTNwelk3WEhYUjF5d2ptMktYeEhzOHpWazFQZXphd0xfUFdhbkVGMVR2Z1dtVtIB_gFBVV95cUxObEwzeHd6RmZtNUp2dXVVV0plOVQ4WlNqQXNJU0thd1BEWE8yWkxxVTZjTkpsVGxxWGxpQzN0OERZbk91ai1fZkdtc0JoM1h5NERLTVdDbVJ4Y2k4djdQcWlVcDF6NjMyVDQzZWMzUFZxWjVRWllMZHVSOF9jQ2U1REFfNUlhM2EwYloxb1MwSTJjODdWdlZwX2h2N0xiQWNhallHUTNPZEtLaXhsY3dBZy0xM1VITXhLUERXS1JxR0R3OUpBTVBPZ2dPZTRUTVpvbFBNMjFUSTJuWS1XLWdhUS11UTRzVTVqaEhfMDhqWHlTMlJGekU2QzJVcFdodw?oc=5</t>
         </is>
       </c>
-      <c r="E45" s="16" t="inlineStr">
+      <c r="E45" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1771,7 +1774,7 @@
       <c r="F45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="16" t="inlineStr">
+      <c r="A46" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1781,17 +1784,17 @@
           <t>ExxonMobil eyes New Zealand market exit</t>
         </is>
       </c>
-      <c r="C46" s="16" t="inlineStr">
+      <c r="C46" s="17" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D46" s="16" t="inlineStr">
+      <c r="D46" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxPanlvR1V1eVVpdmYxNVNGMnd6UjJFd0J6Zk9IU1lhOW1GbmVTcjY4QkJCYkl3Y3NOU25VRTBUekwtS3plV0NVdlZtOTZZRHJWZ0FVdDl3S05aMlFWeEZiYzdwYmQtVnJxZEw0NktHaFZMNlZkUC16empqRGxxMEhhZGwxRzVEek5FelB3aE9UWFhGQW42b21MRnJHUXV2ZGJYUXJIMnVFWGZsSnEwazNGNUdVcjVoekp0NEZCN1J3cTlaZldFa1pMUkJTbVZYeFljVkRqQmlZV1M2aXh0ZjI5dEI1NDB0UElPUERsbUljMlA3OHBnYmtJTXFWZWkyUdIBgwJBVV95cUxNWFBRQ05GUDdwTWJ2ZVFJUS00ZUh0QkpZQVNNcU9JYXRTN21sMS1VZTlOSTh2LVFuZHh6UVk2djlrdWFsd3MwcDFCNmhwUlVLTlpjVF8wSmt1YnBWRE9tNVpKQlk2YXJWdmwzZWlLX0xpaWxSMUpsX3ZjYXhmRmE2YlAtSFJGRG5pQnVmMnViQXlsVFV3OU1hZFVrY3ZITHQxcTR5UkZ5U1pReHVJMGZGM2FCZWliSFZQZmpVLThSdExWMW14OElodmVVSC05SUh1d1hBenJoY3BUZGxoM0NTbTExdERmM3pjZGd4VzgyV3BNOG11TElBQ3NsRGhtSEc3YzJz?oc=5</t>
         </is>
       </c>
-      <c r="E46" s="16" t="inlineStr">
+      <c r="E46" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1799,7 +1802,7 @@
       <c r="F46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="16" t="inlineStr">
+      <c r="A47" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1809,17 +1812,17 @@
           <t>PAC Capital’s Clayton Larcombe charged with assaulting wife</t>
         </is>
       </c>
-      <c r="C47" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D47" s="16" t="inlineStr">
+      <c r="C47" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D47" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOLXNDU2xjMWpyeEZwWGwtZkV0TjNSbGtWS3ZidUo3a0dvV1hrTnJiVXBXSkJNWlhXYXFHZkNTa3g4a1ZfMjRPM3BtWTZUNGg3S09kbGI2TTRGd0Jkc1A4WFAycjlpVC1URjFvNnBraWprRkhaT0VOWkh6N0xkUjNXNUw0dGx2N1JtTDVsREdtZDhraXVsSkxhR2ozamFUSGR5VHBBRm1Zcmx1c2RDaUIxQkVpeUpfWjFNeTRLWVRtYjluZ3ZncGZIMQ?oc=5</t>
         </is>
       </c>
-      <c r="E47" s="16" t="inlineStr">
+      <c r="E47" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1827,7 +1830,7 @@
       <c r="F47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="16" t="inlineStr">
+      <c r="A48" s="17" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1837,17 +1840,17 @@
           <t>China touts itself as ‘harbour of stability’ to global CEOs</t>
         </is>
       </c>
-      <c r="C48" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D48" s="16" t="inlineStr">
+      <c r="C48" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D48" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPUzBWeVk0elBOZ0l5QU44TUJvU0RvSmtPdmVyT2VuQTczaEdzbkktT25ZT2Y0Nzh0bVBhQW96TUhpWkdEOEJMVVk2UWxLOENKZGk3X2tQcDNsWGZtU0JkM2U0N3VfUWFBclhUSUZya0NwRTJOWmZJdWlhT3JtY1EtSkJ6TmlsV3dzOXpDaVFMNlBaa3RfRHBjc3Q0cjk0eVdPV2MwcjlHNA?oc=5</t>
         </is>
       </c>
-      <c r="E48" s="16" t="inlineStr">
+      <c r="E48" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1855,7 +1858,7 @@
       <c r="F48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="16" t="inlineStr">
+      <c r="A49" s="17" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1865,17 +1868,17 @@
           <t>Eyes on 3D Energi as oil and gas giant Conoco flexes buy-out rights</t>
         </is>
       </c>
-      <c r="C49" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D49" s="16" t="inlineStr">
+      <c r="C49" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D49" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWVU1QmhTUGFkYlpTQkw1WUFPTHhmbk5lbnE4T1haQUswSi1ITHlhVmhyM3ZYS3N4cVd6ZkwzdGdhT1lvM1JJek4yLXFpSWoxUnRtR2JRLTZWa2dlTDVTakE3b2xvazFWX0kzRHFZWVB4OUh0XzFFd3JVSVlfelpVa21qTldCVHdvcmJYcGNjZ1RrdElWS3Yzck9KYzRvbzloWkNqMnQ3dmtHbzNuc21ZSXNYeEFlZw?oc=5</t>
         </is>
       </c>
-      <c r="E49" s="16" t="inlineStr">
+      <c r="E49" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1883,7 +1886,7 @@
       <c r="F49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="16" t="inlineStr">
+      <c r="A50" s="17" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1893,17 +1896,17 @@
           <t>Blackstone tempted by $900m payday for Sydney’s JPMorgan tower</t>
         </is>
       </c>
-      <c r="C50" s="16" t="inlineStr">
+      <c r="C50" s="17" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D50" s="16" t="inlineStr">
+      <c r="D50" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxQNEZTZjY0S2YzcUxsb25RSDk2NHd1N1VOVlpMbi1JNGEzbUt5ajlYZFhvLWNBTkNQVXNuWERfTkl0Z2o4R1U0Zk5jVE1FTW5TTUJGZnNJc2NqMm1fT2dmYTVwRGU2TkZ0c3BjZVBGS29fWFJvZ2F0MWNLa0pYY0RNME5xYS1vOGZmMDVBcDBaLV9MWF9od0EwekFyb0ZCOEdkNTFaN3ZXckJwd25zS0FsdzU4OW1UODlueGNyZVBDSDZkeHQwelV5ZXVDVlcyUkhKWDZfVlRacEJHSElmNnhKSXk4ZHJHWHhPTEV5NGNkcmhyU0hjV3J4dVBXbnRGQdIBgwJBVV95cUxPME4ySFF5RWNrejVlWW1yeW56N244RGpyeVJUZEgyTjFNcE10YjVpMmJyeWsxTENzZFhPRlpsbl9pVXl0NGJvUlZFT216NE1KRFNwOHVZVXMzanNKNXFmWEdsMndsd1cza3NTTzUyUUZfaDEyWHJwZEtQbTdJRmkyU3A0RGh4QlAtT1lRVXk2SGoyaTI1NUpwVExYSkZJNmVFNjdXTDJTNURFOEh4Y1dnUDVGdjBpaDlWVWJtUHZiRDdGTmE5R1R6TDBwWFFnT2MwQ1lmT2w5bDF6eVU0R20tYnpnT3JCZlJod2s0UndyZTM5M2xLZC02a3E0NmJRdFV0Qkow?oc=5</t>
         </is>
       </c>
-      <c r="E50" s="16" t="inlineStr">
+      <c r="E50" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1911,7 +1914,7 @@
       <c r="F50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="16" t="inlineStr">
+      <c r="A51" s="17" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1921,17 +1924,17 @@
           <t>I-MED attracts mystery suitor as Permira weighs sale or IPO</t>
         </is>
       </c>
-      <c r="C51" s="16" t="inlineStr">
+      <c r="C51" s="17" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D51" s="16" t="inlineStr">
+      <c r="D51" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxNaGlwS3d5MGFMbEg2U2hnZUxMQmdqaWI4bS1lblNZOFhkSnRMcUotRkZMTjhFZkRUQWxUUDVtYml6TVAxUXkyZmx3SHRFb0gzVHRST2ZQUThKa25aWlhlcGprSU9tWktXZjZRaC12bFpkaVVWZHhIMERyeVNNWEswYTJ2ZHdnRFVRaFhod2U5N011TkQ0NG5MYVhoT3MwRUVZdVB2UVhKZExvdFIyXzNNUGt2SHJUanQxRkI3bXlLSlNJQTF4NXQ1YlZDaGVBM0EzNUhYQVp6NkFWRzU4bnRPWTgtXy1HVnB0ZlN0Uy1rY2FuWlNfN1U4WXVHQnRzVkNG0gGGAkFVX3lxTE1GaDJJdTJlOXFEZUtDTmdXMmsyLXlpaUxzQXpycHk4MTdHZng0dVczYWVwdWRzdFFCMlNLWkZpMm5Zd2RpN0Y0Zmo3Q1FOZFBZQlh5LVl6aVZ3X284UmpxM0pVRzZmMmpjaUdNWnJPZGV4V3lNai1CTllCcW5oUEVxaG0zejB5anc5YnJEZzZPT2d2QklCWjl2MjRBc25jUndqZkVadllKaUZScG12bEozT1NKUUJYR0pHTGtJZVc0ZHZLNHVSYlhzcTE0SkZmMXNlVGJ4YWJ1cThxcGlZTDMzRUMxLVM5VHh2OW5tRW1PT3VyRUhDbV8tRzUzVzRzVWZPZ2w1bnc?oc=5</t>
         </is>
       </c>
-      <c r="E51" s="16" t="inlineStr">
+      <c r="E51" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1939,7 +1942,7 @@
       <c r="F51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="16" t="inlineStr">
+      <c r="A52" s="17" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1949,17 +1952,17 @@
           <t>The stagflationary mix that has billionaire Solomon Lew worried</t>
         </is>
       </c>
-      <c r="C52" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D52" s="16" t="inlineStr">
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPWTh3S05XQWpTQm03WjhBT1pWc2cyOFRMd2ZraHhPUHlDRW1tWkZvdkhQWHE0MHVMRUpaOFRoX0JsYWhJV21nVkpIM2RBSmlZRUtEbFAydzZfOTh1S05oNEZPOGgyZDJRMS1uLThWYWRVT3VEVGhtYkVLN3J2OWsyX0VVdTUteFBCOVNKZ28xUTRPTk1SUkMxZ1NJc1B6NXRrUEEzOG01YnZOYjk2cWlFZA?oc=5</t>
         </is>
       </c>
-      <c r="E52" s="16" t="inlineStr">
+      <c r="E52" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1967,7 +1970,7 @@
       <c r="F52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="16" t="inlineStr">
+      <c r="A53" s="17" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1977,17 +1980,17 @@
           <t>Oliver Curtis on Firmus: From prison barber to AI billionaire</t>
         </is>
       </c>
-      <c r="C53" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D53" s="16" t="inlineStr">
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D53" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQek9VTlV1b2hVb2RoZ0Fya0REb3E3YlBCR2NYZldXcEh2VEY0LXg5bjd6RzlnZDI0OUJJd2cydTBwTm9tdHpiZ1lSMnhtcmJSYVRKbzJFMjdDaEJyZExSQVJVRDh1c00yMjFMaVlPdnRuV3VkTjNxdzFRbW1yeGltSF8tVXlJVXJzTEJXS2FTYkJTVkdKbmdPTTd6YzRtYV9nN0JzOVZNTzhUdUk?oc=5</t>
         </is>
       </c>
-      <c r="E53" s="16" t="inlineStr">
+      <c r="E53" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1995,7 +1998,7 @@
       <c r="F53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="16" t="inlineStr">
+      <c r="A54" s="17" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2005,17 +2008,17 @@
           <t>Three startups that raised $161 million this week</t>
         </is>
       </c>
-      <c r="C54" s="16" t="inlineStr">
+      <c r="C54" s="17" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D54" s="16" t="inlineStr">
+      <c r="D54" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNRGVZMF9DeGJjX29vN3B0blVoM3RKSlJJTllrMThKUDJNZzdPNFNnT2JyTElUOUYxMHlsUm9yM2dBQnZfaVNZblpqb3NzTXdHVlpQNkRqR3NBZHdzODdjN3RKMTZhSVRqUEM5d3JRc3F2OG9hWmZJdU5rakg4ck8wLXlMTnZSU0lNaERmQmswbkVGWW8?oc=5</t>
         </is>
       </c>
-      <c r="E54" s="16" t="inlineStr">
+      <c r="E54" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2023,7 +2026,7 @@
       <c r="F54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="16" t="inlineStr">
+      <c r="A55" s="17" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2033,17 +2036,17 @@
           <t>Iran eyes ‘plenty more’ vulnerable energy targets in costly war</t>
         </is>
       </c>
-      <c r="C55" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D55" s="16" t="inlineStr">
+      <c r="C55" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D55" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNLUN1MHlZaTNfVHhVX0RnTXp5QW83RmM4WVZkWW1PSnNaZF93VkY5ZF81anB3NDNmX0kyMkVSdkxNSURvSEh6enloWnRVcTlsR0JPTjVzNFR1YjRsSm52VnA1XzFFUlUtODJjYy15YWRRdWZZRkdjRXpCcEFSVURmV3VpSTFhTjVUb1d5bmw3NHNlT3VQZU9ieEYwM1J1TGEyZnlnWXNIWFJUMEtIOVZad0dxRWZBdw?oc=5</t>
         </is>
       </c>
-      <c r="E55" s="16" t="inlineStr">
+      <c r="E55" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2051,7 +2054,7 @@
       <c r="F55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="16" t="inlineStr">
+      <c r="A56" s="17" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2061,17 +2064,17 @@
           <t>Don’t take it personally: Bain Special Sits hits hurdle at Infinity</t>
         </is>
       </c>
-      <c r="C56" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D56" s="16" t="inlineStr">
+      <c r="C56" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D56" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQRjdwTk0xTHVIRHNkdG9tVk1EQ0hiQjJ6dGcxaWZRZ0hZV1U4YjJDU0tnTUlWSkQ1S2dUTHJVNk0tNWQ2cVd4dkw0M25leXRreWJtdlBKYTAtNzRocTJUazh1dnRzSVlYZThySTBNVjg5X0xYWUxCMC1SelltSHVSUEV5U3B1bTA2NjAzMGFZLW1CNkQ3aWU0S1JxS0d0YmZiZjBKQVRNVUpzYno5R1pvbTBsaTM?oc=5</t>
         </is>
       </c>
-      <c r="E56" s="16" t="inlineStr">
+      <c r="E56" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2079,7 +2082,7 @@
       <c r="F56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="16" t="inlineStr">
+      <c r="A57" s="17" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2089,17 +2092,17 @@
           <t>Drill, baby, drill: It’s boom time for mineral and petroleum explorers</t>
         </is>
       </c>
-      <c r="C57" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D57" s="16" t="inlineStr">
+      <c r="C57" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D57" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNdlFOWld5ZWhPVnFRa2xidWlUVzluQzkxUTgxR0t0Rmg2S1BzNjdINnhwS3VLRkNjRVJLX0RHU0h4VFVRY2RfSHBudEhfNVNjeE50ZUxQenJNSlJtWFRlcnNsZm1iLXlxM2RmVDViWEtjNDloaTBhUDVxYkNfOWFCTjV6cExEVlFCMzNfWnVwRDJHYWxWV0hOR2V2S0VlV2NyS2s5cWNmREtWXzlMMDRQNW1tVlBOblp3SHBEVg?oc=5</t>
         </is>
       </c>
-      <c r="E57" s="16" t="inlineStr">
+      <c r="E57" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2107,7 +2110,7 @@
       <c r="F57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="16" t="inlineStr">
+      <c r="A58" s="17" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2117,17 +2120,17 @@
           <t>‘Wake up’: Fury as farming crisis looms</t>
         </is>
       </c>
-      <c r="C58" s="16" t="inlineStr">
+      <c r="C58" s="17" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D58" s="16" t="inlineStr">
+      <c r="D58" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNelJvMXFPX3MwUVRMN2xqbzE1MWdvOF92Zy02YmIyZW9SQXRNQVZsS0xVVG9UdkFPaTV6ZC1tV05SZWNqblNFZ3Y1VGNaVVBaaEl6aFJqQ09ONDVkNUs4TzNvVjV5eHNjUk9xaDRFZTM0alpuYUdvWGtLRzRhYXN5alZ1QWdsZTEyODdQVnZoazkya29WeTJZVmpxLVBCdWxfY0dTN2Z3WFZlSy1sVW44RDlvZFAzYlhnQ0N6UWhKSU02eF9iZllIU3g5MWtSbkJzZGxWLUxHNERzdUlLTF9VYmpJSTRLY3U4NlVVaDhmc09uOWwtUGtlb0I2M05DR1dnRWxGSFV2NEJXaEF4c00tN9IBlgJBVV95cUxOSzZ5NXZMTTlZa3BSNjZyTUxUMjRhYWJhN0hMa3dDcW9CWGstNnI5MzV5U0hJSTdKLTFwa2E5YUItZnFRbW5RbzVuYW91MmZaYXN3R25hWVpUbW9oUU9fVktPRHROVDYyd2dSLXJVZWQtY016bkVxY0VPbkY3Zkgtb1liWGMxeEpyYmloS1V0TVJMMWZaeWRZX3FQRjBmVzJwdkkwMEVDSXV1MTdReUhGZ0Z3dENyMEFkLUl1aXhtRkFLRFFXcEdMZzFuT3NxRDFMOGVaY2YzeXBQc09fY3YwcFp4MVczRVN3d3dJZWJfTFFscjF0cUtRWHdzTUptaHowNDhYWXZXTHhYTHNTdlZGUmNlamRTdw?oc=5</t>
         </is>
       </c>
-      <c r="E58" s="16" t="inlineStr">
+      <c r="E58" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2135,7 +2138,7 @@
       <c r="F58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="16" t="inlineStr">
+      <c r="A59" s="17" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2145,17 +2148,17 @@
           <t>Construction giant FDC road tests IPO pitch</t>
         </is>
       </c>
-      <c r="C59" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D59" s="16" t="inlineStr">
+      <c r="C59" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D59" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxON3p5Y3VPM01XZFk4a3g0R3JnQkZXbHVGV3BKdDB6M3NRb0M0SEl3V0R5RmhCQ3dnaHB0ZHp5N2hCMUFsNU1ZNWZ4YWdNZWdETkUyZmdoeW81amwtTWNFZlc5WlNpMkJwRzk0QklORGhlLWNEalh2d0JCX0lhVHhhUF9ibVlxcHAwOW9ENndVOTY0enBYUWc?oc=5</t>
         </is>
       </c>
-      <c r="E59" s="16" t="inlineStr">
+      <c r="E59" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2163,7 +2166,7 @@
       <c r="F59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="16" t="inlineStr">
+      <c r="A60" s="17" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2173,17 +2176,17 @@
           <t>Austal suitor Arlington Capital Partners buys Eptec’s defence unit</t>
         </is>
       </c>
-      <c r="C60" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D60" s="16" t="inlineStr">
+      <c r="C60" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D60" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNM01qb1ZRZVBIdmp3cFc3R3RLaTdmZk1JOFo4anRtSm95Z1hJc0N0S3VranBTV29IdlViT0FkSm92eHdtbDBqdU5HTHNMaXo0dGRWMkpDdjk3LVRBVU1rZC1YejZJMkhyNmpZZFJodGoxWlB1dkRhYTJVRlljMlV0dUllQ3EtOHZkNFdSUWJLSW9Xemw1XzFzU2RHV1o0RTViOXp0bDZFQTZycWhpNElLU0FZQVI?oc=5</t>
         </is>
       </c>
-      <c r="E60" s="16" t="inlineStr">
+      <c r="E60" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2191,7 +2194,7 @@
       <c r="F60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="16" t="inlineStr">
+      <c r="A61" s="17" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2201,17 +2204,17 @@
           <t>Eyes on Tom Wallace as clock ticks on Adgemis pub deal</t>
         </is>
       </c>
-      <c r="C61" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D61" s="16" t="inlineStr">
+      <c r="C61" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D61" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxNSExQeDlENWlHb0prRnRldjZ5YWhKVUZ5eVdsYjZmbVRWRWQ0WnZXWkU3UHZJdElnQ21jMU9zNnhnc3JlNDczVGQ5Y0FGV2J3QUp3NXdZTXZMNm5tVC1vWDFtOFN3aS04QVJZb3FZV2VsUmJ2aVgwbUhTaFVGdHg0UjRyTXVVUnFhQmE5eFYwMGR6T1R2U3Q3WEdZclVKNWJiby1IRg?oc=5</t>
         </is>
       </c>
-      <c r="E61" s="16" t="inlineStr">
+      <c r="E61" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2219,7 +2222,7 @@
       <c r="F61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="16" t="inlineStr">
+      <c r="A62" s="17" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2229,17 +2232,17 @@
           <t>UBS names head of APAC leveraged capital markets</t>
         </is>
       </c>
-      <c r="C62" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D62" s="16" t="inlineStr">
+      <c r="C62" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D62" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNMm9WZ2ZKVFBvX2pYMk16VmY1WFZnZ2J5N0F2bHduTVM0Sjg4STVtTGFLQVdzeFloVHg3clRic0owTDMwYVpXdDVjdjFOWjQxdkdxdFY5MEY1Q1U2Q0R5dFBJWTNtUzgyd3RXcm9uM0hKdEZ3b3JjXzcwQ2VpRm5SS0hYT2gxSU9iVFRlR05Xd2EtM2JOQjBGUzlKdnE?oc=5</t>
         </is>
       </c>
-      <c r="E62" s="16" t="inlineStr">
+      <c r="E62" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2247,7 +2250,7 @@
       <c r="F62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="16" t="inlineStr">
+      <c r="A63" s="17" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2257,17 +2260,17 @@
           <t>BHP, Woodside rise after new CEOs named; Future Fund chiefs exit; Sandilands ‘doesn’t accept’ termination</t>
         </is>
       </c>
-      <c r="C63" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D63" s="16" t="inlineStr">
+      <c r="C63" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D63" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNUHhZeHNHemtiLW1IOHN1OTZXOGpsM0ZtUG1MVHRCT1hUT1k5S2lEOXlXRENWOXNlMEZadThQR18xSTJfTVlQM3BtX0ptX1J0bk80SzNLUVRtbkJITGgtb0lsSVdJTWt2S1E1WUlXdUdsbEV0V1RpNWlyRXBoc0dPVDl1OXRrSlM3SHlDazg2UlcxenVzNzlhQldhUGhfNE5IV2xrVmVBNzhhSE9qY042Z3pzMEVzd0VyVmZudXgxcTgwWGJXSWZKZ0FyNVhjcmhjTm5DYUVjLUdDRmxUQkZuTDFlUXVaV0ZoSWp5WHMyR3c?oc=5</t>
         </is>
       </c>
-      <c r="E63" s="16" t="inlineStr">
+      <c r="E63" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2275,7 +2278,7 @@
       <c r="F63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="16" t="inlineStr">
+      <c r="A64" s="17" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2285,17 +2288,17 @@
           <t>BHP’s new CEO will shift the Big Australian’s centre of gravity</t>
         </is>
       </c>
-      <c r="C64" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D64" s="16" t="inlineStr">
+      <c r="C64" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D64" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPQnZpWndNZzZvN1VsOHBmRDVLRHVTNkxLeDVDelpOMURjOTRDSDZfN2dPZlZqaW05WEZuZXMyRTJZeVZnV0poT2UxRkVfZ1RZSjdvUjVKblhoSU5Cd1plRTVNNTRaNWZmbm1yUGZkblVpYkctNzVRRkVQQm4zX1FtRG1KV2Y0djUtOURianJ3dElqeXBUMFp4aWFEWVFYelVjYTluSWpOM1FlbHpIaUxXdnBn?oc=5</t>
         </is>
       </c>
-      <c r="E64" s="16" t="inlineStr">
+      <c r="E64" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2303,7 +2306,7 @@
       <c r="F64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="16" t="inlineStr">
+      <c r="A65" s="17" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2313,17 +2316,17 @@
           <t>How philanthropy became the sandbox of succession</t>
         </is>
       </c>
-      <c r="C65" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D65" s="16" t="inlineStr">
+      <c r="C65" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D65" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxObnBPb2MzQ1RvSVVCbmNzYWFBMlFjU0dQRmpPakNfdkxtMWc1bFdVNXNlZmRKQnNlWEtUUDNSTHpTLVV4Skx0V2otbTZsTTdvT1VaUDhMZFZoMFFab1RoS2pCcno1WGlNQlY4eXQ0OFEtLXJTay1MUkFSSEJ2MVVScUpjUkhJOThISy1QbHIzTzFlWVhOc29fWWs0V19sQ25hRW9MSGhBVVNKWUp6dUo3NS1SWlk?oc=5</t>
         </is>
       </c>
-      <c r="E65" s="16" t="inlineStr">
+      <c r="E65" s="17" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2331,7 +2334,7 @@
       <c r="F65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="16" t="inlineStr">
+      <c r="A66" s="17" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2341,17 +2344,17 @@
           <t>Advanced Navigation raises $158 million Series C round with NRFC backing</t>
         </is>
       </c>
-      <c r="C66" s="16" t="inlineStr">
+      <c r="C66" s="17" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D66" s="16" t="inlineStr">
+      <c r="D66" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNTXhwVlVLUy1pWEpFdzFCazNTY0dkczd4WW9oeW14cUtTaDZRTGlVQXBPaHN4WTBkNW1zOGxvN0tVWl9JSFdVNXlQMzVxbk4zbDZFUjNOcUxSamNaSnFCckMzWEk1VlNoSHJHQ3VWdGltVWZCV0c0NmU4UlN6YU55Q0J2TkQtUzBzOW96UXRxem5Zb3M2SUljNURISlRkQmJD?oc=5</t>
         </is>
       </c>
-      <c r="E66" s="16" t="inlineStr">
+      <c r="E66" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2359,7 +2362,7 @@
       <c r="F66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="16" t="inlineStr">
+      <c r="A67" s="17" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2369,17 +2372,17 @@
           <t>Kal Somani-led consortium buys Rajasthan Royals for USD 1.63 billion</t>
         </is>
       </c>
-      <c r="C67" s="16" t="inlineStr">
+      <c r="C67" s="17" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D67" s="16" t="inlineStr">
+      <c r="D67" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOX3lmdG5aTmk4TEpBa3ROdWZ1aDJHUElBQXktVmlKaHFmTUhPX1QxX1dKLXZfaHRDQjBnWm9McTZjTjJtTWFETTRNMHgzN0tTTm1xY0JpMF84Q2lNaFQyZGVjaHN4bkVmcDN5Qy1ta3FtYnpMSVVyYm0ydWpTRUdZU1hoYXpaNkZUQzlPc1QycjZ6aG5QVHRqY213?oc=5</t>
         </is>
       </c>
-      <c r="E67" s="16" t="inlineStr">
+      <c r="E67" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2387,7 +2390,7 @@
       <c r="F67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="16" t="inlineStr">
+      <c r="A68" s="17" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2397,17 +2400,17 @@
           <t>KMD says Rip Curl demerger proposal delivers investors ‘no value’</t>
         </is>
       </c>
-      <c r="C68" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D68" s="16" t="inlineStr">
+      <c r="C68" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D68" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPTXhBdHByWE9EbllFdDA2OW1UTUZEMVJfV2xsNFdURFRKX2JrODJReVRuQlFoakpWbTBKcjhNLUVsNE9sdG5LUElLZlVrbFNERS1QZTN6bEZIWEhXZ1pTWG5GWEw3ZmNETTdDUDUzYzR5M0E3ZGVlTWpSUnVlVU56dDNFZUtZN3liZ1dKNzJhLWU1S0M1ZnlKd1JNWXlxSlkyU3pGS1lhS05hTUJPRkxucldabzFucGs?oc=5</t>
         </is>
       </c>
-      <c r="E68" s="16" t="inlineStr">
+      <c r="E68" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2415,7 +2418,7 @@
       <c r="F68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="16" t="inlineStr">
+      <c r="A69" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2425,17 +2428,17 @@
           <t>Ex-Macquarie banker drives mortgage broker roll-up Recludo towards IPO</t>
         </is>
       </c>
-      <c r="C69" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D69" s="16" t="inlineStr">
+      <c r="C69" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D69" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxNQms5X1F2aTNhOExDbW42TlZOLVJwVWxna1JYSW9vWF9Na1RZa1ViTFdZc0tCcXRZZkRudTlsTzNuZGgwSENyYi03Zjdfc0lZTXp0NmJRZnhzb2pWRXRIOUdJN2lQM2h3ZFFtTXlSWHVWOFBIaW1Na3FQMjBCck1nVlhUcmRkLW9LOHpKWXQwTm9LcWR5M2FfdjFiRW04TndoanR5NmJvMENGalNuUGNINy1Qc20xR1J4d21ncHNNSUZqa1BXNnI4STIxSUFkZXdU?oc=5</t>
         </is>
       </c>
-      <c r="E69" s="16" t="inlineStr">
+      <c r="E69" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2443,7 +2446,7 @@
       <c r="F69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="16" t="inlineStr">
+      <c r="A70" s="17" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2453,17 +2456,17 @@
           <t>Coles reviews truck fuel charges as crisis worsens</t>
         </is>
       </c>
-      <c r="C70" s="16" t="inlineStr">
+      <c r="C70" s="17" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D70" s="16" t="inlineStr">
+      <c r="D70" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxOSGpBM3RjLVJ3LVlmR1QydnY2dm50WlVxcG43ajRFZ25QS1hDNTBONU8tY3Z2TklzbUNla0ttZk1GZzFaLUZRakFjSUpUQWItQ0VqVTVwS1B0QS1ObVEzNzdRT1l6aU9pVm5jSlhna1N6QmFKT3k1RkhMZGNTVnVLcDVIcXZmRjdjLWRpYVlRQUVmcVRtM21BSjVhTGNaaThyZkhLS2NWdkNCSkZKTlloUVdtbzRnYjFKbllOZXhOd3lkcFZEYURwUFVNQzVnSWRyM1RlOGd2M1pMZXI3c0NIa0Y0MNIB6AFBVV95cUxNSjB3Z0hoTGxwOHJQQ09xb3BmRmhCYjBCc2E0OHA2elFDRE45UGpaTEVDc1Y2VnRvVmZQUzRHbng4QTMwNGZZNGpmaVlHRmV6bnhiZ0FReU50TnRiQ0NZMEtoM3dBZ0hXbFBZMVJQNXd4LVdXRDVyTDAxNS1zeVdvcFVvend2N3J5R2pLYmhxNVFfd19rUlRsNWNndlptMUVkcS1CaUN6UXRHVzByTU5BMW1TdktOZUJYck5xMEJucmR6czIySEMycDA5cmR1MXB0N25Xc0JDUG9zN29YWklVc1BUMzl3UVhn?oc=5</t>
         </is>
       </c>
-      <c r="E70" s="16" t="inlineStr">
+      <c r="E70" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2471,7 +2474,7 @@
       <c r="F70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="16" t="inlineStr">
+      <c r="A71" s="17" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2481,17 +2484,17 @@
           <t>Sam Arnaout’s Midas touch turns suburban pubs into pokie gold mines</t>
         </is>
       </c>
-      <c r="C71" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D71" s="16" t="inlineStr">
+      <c r="C71" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D71" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQV2xlTTdYOFpIMzNmVVRnMlJRbTdGTC1jelVCd1V3UjN5cHQ1VzhWZzhrNW1PNm1RX3FlZmU3UkRycjF4WDlQUzRMcVVYY1g3UTZqQ0hxRnl2Ti1IQ0owVmZjN3Jod1BFbmhPVUwxNjhsTGh6d0kzdU01N0hmempRZ044ZmZNUllnenhyc3djRGJOdEtrekx5UVFoaFFMWDdqMHMwdng1SFg4TzZHY1hQNFJNN3huZXpWYWFtQ0ZJakhkVFlQcl9SQlRfZkQ?oc=5</t>
         </is>
       </c>
-      <c r="E71" s="16" t="inlineStr">
+      <c r="E71" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2499,7 +2502,7 @@
       <c r="F71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="16" t="inlineStr">
+      <c r="A72" s="17" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2509,17 +2512,17 @@
           <t>Gentlemen at Melbourne’s exclusive The Australian Club sweat another election</t>
         </is>
       </c>
-      <c r="C72" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D72" s="16" t="inlineStr">
+      <c r="C72" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D72" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPcEwyU01BOXF4TzlmREhYbTFEWklxdWZqWmZybDVnOWtLQ2dTU2dNQ2t5M3BVT2stN08xYkFmazVkY29oT3RVc2xUZmZINFJURGtIRTg4RGsxOURBdWEybTUwU2NUODQ2eDNBbTdPT3QxeXRFNHlSc014T0g1aG4xZ1A0U0FWMTB1Wm1CSHlQU0ZJb3lMYkE?oc=5</t>
         </is>
       </c>
-      <c r="E72" s="16" t="inlineStr">
+      <c r="E72" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2527,7 +2530,7 @@
       <c r="F72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="16" t="inlineStr">
+      <c r="A73" s="17" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2537,17 +2540,17 @@
           <t>Inside Fortescue’s AI ‘hive’ that could save the mining giant billions</t>
         </is>
       </c>
-      <c r="C73" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D73" s="16" t="inlineStr">
+      <c r="C73" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D73" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOSVVCbGpzcVcxTGlZZ2dTUkxXdVVvVU1ONEtUS0t1R1VkWWRNeUF1UmlHbXd6clR3QVRuWGxrUGQwVG1OeUxZb2RqTzdYOEVGQ1N6eDFta3VOZDdHNThYbUEwWEVHZlZBVzNpZ1Foak1kLURZTWpJVzZLekczdzFrdHMtLVZwMUZnYmkxSVc0czFqWnFaSGZiT2pIVW5rdVZmdThreFlRZWVEU0xoa1VFOV9MTjE2UHFOcWhqUzVB?oc=5</t>
         </is>
       </c>
-      <c r="E73" s="16" t="inlineStr">
+      <c r="E73" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2555,7 +2558,7 @@
       <c r="F73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="16" t="inlineStr">
+      <c r="A74" s="17" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2565,17 +2568,17 @@
           <t>Tiny house maker Elsewhere Pods seeks cash after Bunnings debut</t>
         </is>
       </c>
-      <c r="C74" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D74" s="16" t="inlineStr">
+      <c r="C74" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D74" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM0ZpVnBTS21Ib25qa09CaU52Z29kZWhTU0FJLW5VR2JCLVFPTVlZTmpYX3lZVWdtMDVTYTJkWHlPUmhXa0Rua2ZXTTBWQU1VdmFrV21KOGlrdjJ3TTdxbGlvZVBUZUxUWE1uelpWMGxWWk04UndJTXVKQjBZUEtoX3lodmdpMWZKNUc1YTIxVFZLYkFKT1QwbS01WU01ZUZTTlczY2ZpLXlpTjNJTWpsUg?oc=5</t>
         </is>
       </c>
-      <c r="E74" s="16" t="inlineStr">
+      <c r="E74" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2583,7 +2586,7 @@
       <c r="F74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="16" t="inlineStr">
+      <c r="A75" s="17" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2593,17 +2596,17 @@
           <t>Chinese consortium emerges as dark horse in Made Group sale</t>
         </is>
       </c>
-      <c r="C75" s="16" t="inlineStr">
+      <c r="C75" s="17" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D75" s="16" t="inlineStr">
+      <c r="D75" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQYlpEY0hxNm5lalIxSTUzbDE4UEF5QTNpMTl4dWNPMkRrMU1yQnltZ25WcUkwOU13V2Y2RGItVW5QTXotSnBZRUJMdGJySGw0NVVxc3ZLZmVEcTlfU193Vkd5UVVuTFVYWFNtd185eGlVQW5RRElHdk5pMjhUR24wd1k0T0I3cW9qTG5Lcjg2bV9aNWsya0FYODRjeURyMW1EeHdYT05iZHZhLVFrUVNoV25idnZYZ2lpZEhta2JxOWFJb0M2SE9hbFF6NlVWYTM3QmF5anpWOEZackZiTDBfN2gtX1luQkxFOUxSSNIB8gFBVV95cUxOQklMYWl1ZkRqZGUwN0ppeXFubzZWNTNmeE5GY1BfcS13N2dFT096YW9JSndVX1EzTlBKdWZIemdKZnRIME9SQk5aT1M2WnRESjJxckFTaUdOSEd6eG9hRVBjdlhBbWQyWGpUS1kwQXJsdlpkLXJpXzJZX2xiUC1FSlNnNTFoVXQ4bF9JeUp3UGRWdUFOUVRrNUtsRzRxaUczb1p2LVVucFBNazhuZFNDaUZDR2ZQUVdObmVtTnBndGlkazZqeHVheVNzSE9RY3Bad0lrckxDSWY5QXBWS0hwVzZvSTZjaGEtNkNncW1RRE5uUQ?oc=5</t>
         </is>
       </c>
-      <c r="E75" s="16" t="inlineStr">
+      <c r="E75" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2611,7 +2614,7 @@
       <c r="F75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="16" t="inlineStr">
+      <c r="A76" s="17" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2621,17 +2624,17 @@
           <t>KMD faces uphill battle in capital raise as key shareholder baulks</t>
         </is>
       </c>
-      <c r="C76" s="16" t="inlineStr">
+      <c r="C76" s="17" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D76" s="16" t="inlineStr">
+      <c r="D76" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxOVTU0OGNfRURNcDdzYUtIcG8tR3N4OFFYalhKNWJBaUd6ZlQwNU5MZVZYbUZVSzB3WmdOOFdTZHlBOXBzSGdYUVV6eGt1UndHN296bENxZzNUM2NoaV93LXZaZFNNOXJ2YlA4RHNFS2FDb1ltNWpPWUdRR3VGMWoxaU5qYm9VSW9yUW5kS1NaN2RSc2YtcHZRSTB6aE9Zdkl3NG5nbVRzODRfQVYtelo5M3g4R2JEbnpraFpWbENOZzE2Qndla2t3MXRPWkU1dXg4NmZRME1jT3pOOHZOVlpTZGloNENUZllaSTFmWUV1Y2JLck02ZDhnTHJ5bUPSAYICQVVfeXFMUEFXR29tQjlTbTdMRVNDWUlGNFNOQjVhX0FiSkl0U2stbml5VHR4d1g3bDFqMUw2TzR1eHhYOU5ZUmJpZ2xBY2NzcmJRX3MwaEQ0YmpzMUFnV1BQNGxmcnlXUzVvbHpwNEo5dWFnZlduZ0Z2dGZGRFRKRTNCUzctZDNCd0FMNEkzTm84dmZOM2NKYk81RERsVnlZN1VZaXp5TW5QRVAzOHNXQTFWdVlKdGtFX0FmcU1EbElZSm52alBQeWx4VnlvOFRwNk1ia2lZYXlpemQ4cFdmckotMmMyRGE4ZXN0dThQYmxxUkpvMzAwRXBBcVJuRnp0QkZ3b2tqMWF3?oc=5</t>
         </is>
       </c>
-      <c r="E76" s="16" t="inlineStr">
+      <c r="E76" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2639,7 +2642,7 @@
       <c r="F76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="16" t="inlineStr">
+      <c r="A77" s="17" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2649,17 +2652,17 @@
           <t>AustralianSuper claims another listed M&amp;A kill with Pepper Money</t>
         </is>
       </c>
-      <c r="C77" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D77" s="16" t="inlineStr">
+      <c r="C77" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D77" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOY0RwcnpWZlhfOHA2MG13MkJUX1RDNF9wN2RxZGU2cEpzS1RKTjJDeUl0OERFOGhFRXJaSXNETEhHbW9PS0lua283RnFVbHJvTlRva0djQ2lRSGc2RENJYmt0OEsyYTRVSzFGeE9jWVhKMVRnd240WXVNTVdac2lOUGJSZlc4UVZ5RXo0OTlQbUd6NWRSek1HZG9fZGk2aDhDelhGVmk4YkRKeVV1M0VHZ2hZNmFVdXM?oc=5</t>
         </is>
       </c>
-      <c r="E77" s="16" t="inlineStr">
+      <c r="E77" s="17" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2667,7 +2670,7 @@
       <c r="F77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="16" t="inlineStr">
+      <c r="A78" s="17" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2677,17 +2680,17 @@
           <t>Apollo to Acquire Nippon Sheet Glass in $3.7 Billion Deal</t>
         </is>
       </c>
-      <c r="C78" s="16" t="inlineStr">
+      <c r="C78" s="17" t="inlineStr">
         <is>
           <t>Wall Street Journal</t>
         </is>
       </c>
-      <c r="D78" s="16" t="inlineStr">
+      <c r="D78" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOanpORVBremoyamJyZ2FqQWVOcDcxa2NpempBUmNYcktMLUl1Mzg5VDloWmlVbUdNUnplVk90WEUzXzJjNGxENk9LcGF0enVSdlFpWU9nd244YWNTS0ZHd1JTZEtlbjRQTmJUU0dzWmlDOVFhR1ZRSFJkNXN4a3FHdGozcUcwdHRseXpYMFREUzBNcXRmQ1VCN056SWlEa1l5VVE?oc=5</t>
         </is>
       </c>
-      <c r="E78" s="16" t="inlineStr">
+      <c r="E78" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2695,7 +2698,7 @@
       <c r="F78" s="3" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="16" t="inlineStr">
+      <c r="A79" s="17" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2705,17 +2708,17 @@
           <t>Estee Lauder in talks to combine with Jean Paul Gaultier owner Puig</t>
         </is>
       </c>
-      <c r="C79" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D79" s="16" t="inlineStr">
+      <c r="C79" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D79" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPSjN6QnFVbmdHWFoteURWaU5VaWZmRmpTT3QtYm1tZUFyNUZyLUdheGdfWlRBTlJyTlp4THIwVDA4U3BnWFNpT2FpZlZzX1lJSDV0MkRGVjYtNVc0b0lOQy1RSnFGTWhCTWE2ZFFPYlFQX05yaVlfZF9IUEN2ZWkzQ0VFMUxxdHF2ODNQY09xdWlqWEczSC1CZk5wYU9QQlAyaTMyelJnaVM0cmN4M0paNzlBdzM1RndoZE8yRHN4UnZqaXVhVmx5NFpqS3hmUHhUdlpF?oc=5</t>
         </is>
       </c>
-      <c r="E79" s="16" t="inlineStr">
+      <c r="E79" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2723,7 +2726,7 @@
       <c r="F79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="16" t="inlineStr">
+      <c r="A80" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2733,17 +2736,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C80" s="16" t="inlineStr">
+      <c r="C80" s="17" t="inlineStr">
         <is>
           <t>The Age</t>
         </is>
       </c>
-      <c r="D80" s="16" t="inlineStr">
+      <c r="D80" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPdUtyNWs5YmxJMXNsNWtaMi1WMm5SVHd6ci1ReURLajdYd1IzWGJMZmE2MzJsSzAxQWtSTm8xMUEwNTh4Vy1zTmFsWFBKTkJ0YXc3ZkcwOVk2a2VNRWVGUS0yQzZhSXlCWmpDYUx6RmpTTlNhS0xIQklyVFdIVXJRZTNPaVB4TG4yQ1R1ZWF2MWpmSG81TVRaRzdtMXpydWhBS2w0a3ZPZFI5MnFKOW5tN21oUDB3NkNtQmR4LVVBWW9BUQ?oc=5</t>
         </is>
       </c>
-      <c r="E80" s="16" t="inlineStr">
+      <c r="E80" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2751,7 +2754,7 @@
       <c r="F80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="16" t="inlineStr">
+      <c r="A81" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2761,17 +2764,17 @@
           <t>Australia’s new millionaire factory: Start-up to $1.6b in five years</t>
         </is>
       </c>
-      <c r="C81" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D81" s="16" t="inlineStr">
+      <c r="C81" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D81" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOVkl5N1NGWS1XWWZSc0pHXzE3MUNERmV5SUgyQ3o2MmJ3U3Y2YlNwUXNSTGlQenBwVFdnMWhoT2FrcDAwUHNVU0RQbjFHMjJiLU1TRC1nemdrX3hPTG93VWZUQUx3Wk9HT3lYd055Z2FtREFpOWRlYXFDb2hwV0cyWFMwaHpsLU0ta2VVQlpid1dlYks0ZHg5YTY3Ykt6Um5YaF9MR2tIRzd1Tk1IRnBrWVhxVjZNSUl1OE9iRlZzYmQ3QUVnZmhYVGxoOA?oc=5</t>
         </is>
       </c>
-      <c r="E81" s="16" t="inlineStr">
+      <c r="E81" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2779,7 +2782,7 @@
       <c r="F81" s="3" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="16" t="inlineStr">
+      <c r="A82" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2789,17 +2792,17 @@
           <t>Social Media Wrap: Genki Sushi Singapore's loyalty benefits; Dunkin Philippines launches new collectible; Burger King Malaysia unveils new Korean inspired burger</t>
         </is>
       </c>
-      <c r="C82" s="16" t="inlineStr">
+      <c r="C82" s="17" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D82" s="16" t="inlineStr">
+      <c r="D82" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxPbFR6eHVTRWZNcUw1TTBJdE1JTFpmbk5iWndKZnRoU3Fmc3cxcF80TnVhRERmY0poM09zTFpCaEVnMGo5aktxY0ExV1ZlZVpHYUtldXBoOUh6bm14SURHNmhnUE9tYnI5YlpXQ3pRZlp0Ni1wM2lYQmdxdjk4SDl0aFN0R1VBbGxpbFVzOHV0TFY3YjJZbDg4Vk1HMTBkQk5LRHd1ZEVpRnBsT1U0Nm1IbVFkZEUybmpabEhuLUNLOGhicUxXZG5UalRLOE5DSzcxRncyNjVRdk8zclhJNkVQcTRkQTZYSEdN?oc=5</t>
         </is>
       </c>
-      <c r="E82" s="16" t="inlineStr">
+      <c r="E82" s="17" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -2807,7 +2810,7 @@
       <c r="F82" s="3" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="16" t="inlineStr">
+      <c r="A83" s="17" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -2817,17 +2820,17 @@
           <t>Copyright ‘status quo’ not working in AI boom times, says Charlton</t>
         </is>
       </c>
-      <c r="C83" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D83" s="16" t="inlineStr">
+      <c r="C83" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D83" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNVVgwdEQ2YUt0eFo3THcxOXZHbUFYZ091VTFKZDZHX0szYWQ2dnZ1dkJma3VZcGk1LUM2SUtQSWhxMGpCUlFZVzdKNmdoSGEycm1oYlBUdEZ5R0ZlU2hrWHpFWXdSN1lCZnZzb3hZc2twVVlWdTNNVXhaR0Nza0FiaUNveXZWQWQ1ZE45MU1HbGNmWlU2aUdha2FyZllzNWdONEpsM2RrdGRFSFl2UlpJUnQ4WGpleGs?oc=5</t>
         </is>
       </c>
-      <c r="E83" s="16" t="inlineStr">
+      <c r="E83" s="17" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2835,7 +2838,7 @@
       <c r="F83" s="3" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="16" t="inlineStr">
+      <c r="A84" s="17" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -2845,17 +2848,17 @@
           <t>The unapologetically analogue 4WD for off-roaders with $120k to spare</t>
         </is>
       </c>
-      <c r="C84" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D84" s="16" t="inlineStr">
+      <c r="C84" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D84" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxPSFJ4ZnNLT3U1REp3MWI2WDFaQm5vZlp6QWN6c0hZamtYVU95WmpkUERwR1dwc0NQN1dEc0FNbHlaMTdLclVHb1JTc2VZNExENGYyUE9OR1BkQ244YXRVeWNwbkxia2VrckVqSy00WV9UNWlvZWJHOG9ibUthaTlpVmRBOGZjLWFzMU8yS2Q5Um05SWIzY2dKajhoMWFUcmFrbTMzai1CdVBNLWczTWRvbTBwSDRfUzNwOHhqQm5hTDdhM0xLWEpNQTRyRXZjU1FLdGhRMUxtOTg?oc=5</t>
         </is>
       </c>
-      <c r="E84" s="16" t="inlineStr">
+      <c r="E84" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2863,7 +2866,7 @@
       <c r="F84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="16" t="inlineStr">
+      <c r="A85" s="17" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2873,17 +2876,17 @@
           <t>Junk room to become jazz club with priceless Melbourne view</t>
         </is>
       </c>
-      <c r="C85" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D85" s="16" t="inlineStr">
+      <c r="C85" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D85" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQbHN4My1nOGtueVJQZWM0LXNjLTR3MmhuemRJMUEwN09FTUZhZk1lbV9MbnVWblgyUXFEMEl3LUtsOGVqdGUweFR0MXF0ZEo0XzNhWVRqb2pGRUdiNTlLc1dFcXFmdnctQU1wQkRSdHN0T3J6VGt3MU1iNENydGlsOEpsT0ttZmJVZ0FUZmFXSUd3alVzUTQxMzVmcEVXSlV2dWdQd3JsMUZ0d3ZZYlBHaGhKTm9rM01SUmdseE9hT1prbHZtMlhv?oc=5</t>
         </is>
       </c>
-      <c r="E85" s="16" t="inlineStr">
+      <c r="E85" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2891,7 +2894,7 @@
       <c r="F85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="16" t="inlineStr">
+      <c r="A86" s="17" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2901,17 +2904,17 @@
           <t>Zimmermann fashion label appoints new CEO Roberto Eggs to replace Chris Olliver</t>
         </is>
       </c>
-      <c r="C86" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D86" s="16" t="inlineStr">
+      <c r="C86" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D86" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM2M5QU1scVoyNHBmV2lwQ0VQS1Z6d2Qwa1ZkZ0M2WVIzdXR3QnZwVWhUSDRCUEdRZkc5QzFQSFFhNzZ4VE9lWXBTcGhpS01JdG12TlQxSHhValZfbWt3MUdFZGl3RlBtdnlrel83TjNjNFZ0SUpvSDNQbThpU3FLa3Atd0dNU04zQm9OSk5uNHpTVE84aWZpaVlKWkdOQjJjRTZSd1MwMEZ1b3pENkRCQQ?oc=5</t>
         </is>
       </c>
-      <c r="E86" s="16" t="inlineStr">
+      <c r="E86" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2919,7 +2922,7 @@
       <c r="F86" s="3" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="16" t="inlineStr">
+      <c r="A87" s="17" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2929,17 +2932,17 @@
           <t>Construction giant FDC road tests IPO pitch - AFR</t>
         </is>
       </c>
-      <c r="C87" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D87" s="16" t="inlineStr">
+      <c r="C87" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D87" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNTnRScHFhQlpkdEdSb2x1bExxQm96ZE5zSV9wTDNDV2pxYjFQdUtoYmNBell3SFlTTFEzMUhpeXlmNERSeDd6VGppM2szQ1NHVE9PY1R3MTN0SUZLWkF5em8tQ3IycUZ2RmswX0tnN1IwOHl1ZFo4UUtMUDlQbXRjTnRCWFB5cU1RZFhsdDdaWGpMZzh3d29CWWZvZGtnTjl0T1k5ZHFHSUg5XzFSSF9TSUxTYkU0QkFheFlLZUY3S2tCSWRLZWlBbUpxUjc3TXBQQ01V?oc=5</t>
         </is>
       </c>
-      <c r="E87" s="16" t="inlineStr">
+      <c r="E87" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2947,7 +2950,7 @@
       <c r="F87" s="3" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="16" t="inlineStr">
+      <c r="A88" s="17" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -2957,17 +2960,17 @@
           <t>David Jones is trying to defy retail gravity. It’s causing problems</t>
         </is>
       </c>
-      <c r="C88" s="16" t="inlineStr">
+      <c r="C88" s="17" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D88" s="16" t="inlineStr">
+      <c r="D88" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPZy14UldWZDRrSjI3R0lzdGlKamlkVnU1WWVjTWRUTlpya1ZpVW80WHlrT0FQTUUwMzkzM19xQWpwTnVLOF8zeTFXamhTZFRQVjl5TTlXbE1RRWY2NW03dlpmZ25qdkgyN1IwbDdjRlhxd1MzSGkxeG45M214OVlESWF5WWh5TjM0STQtOXdieWIyOUI2NzRsaDhiS0ROUU5YQ185aWtObUY2S0dOSTBROVlwSVB1VkNqTkZTTllkZmtMYmxjNVdlTA?oc=5</t>
         </is>
       </c>
-      <c r="E88" s="16" t="inlineStr">
+      <c r="E88" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2975,7 +2978,7 @@
       <c r="F88" s="3" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="16" t="inlineStr">
+      <c r="A89" s="17" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -2985,17 +2988,17 @@
           <t>Jefferies’ Australian ambitions in focus as Sumitomo circles</t>
         </is>
       </c>
-      <c r="C89" s="16" t="inlineStr">
+      <c r="C89" s="17" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D89" s="16" t="inlineStr">
+      <c r="D89" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxNUTd0LXFPQmZXSldrTmZHTkIwUWQ3MmlCUmFOUGRkcVVjRXV6YXZJUTcyMG5FV3I0dWY2NXh6MnduVjNxZmhJMHdDVGw5VzFxTEFzN2FBdlNvS1JGSDltQmlzVS1QRDdCeWdfSHZ2VlZDMlBnN1Y0d2JxbnlGejhWVjJpWGZLejdCTUt2Uk9ENmhyRkd4dDJjd0RlUnBlZXhOTmUtOG9ITE05VHJ3dTBRSWZneURuUW1NYkExVXpfWXlsMzZ1WUlyNE84SThQX1JJTFlXOHc4ZnB0aXRmdVhaaG1qSEJRZUhuU3RibHAzbHVNLWFLUF9NNTFoUXV3NGQzelcwcNIBigJBVV95cUxPMkhEeDJpNzg0NTlDZmF2LUFPSEs4cmZ5U2p6bWVZSTYwcXVUUGVIb0FLVnhZV0cta01CLVpfQzQzYzdvTWdxR0o4bGJDWDVBb1lnOGx0bWROdTdjcHhwLUpPMW9MQ0RVM2NUOUt6UGpTd05JYzhuVmgybGp2LVpORFF0SHpBTU5DUTJEUmZKUFBNajlQdHJ4WkdHVV9QMjVwOWVlNWliVkFaM20yWGZhOEc4bldHRERJak1BWXlmSE0zdno1VTVSc0FMck0wSE1BR1RVaVRMSEdzU2FvcWpMYmp5ZTVJTWcyUGdXanhqSUNZU0tzTkNYWVg2SXpVMEoyS184VkxOeWtSUQ?oc=5</t>
         </is>
       </c>
-      <c r="E89" s="16" t="inlineStr">
+      <c r="E89" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3003,7 +3006,7 @@
       <c r="F89" s="3" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="16" t="inlineStr">
+      <c r="A90" s="17" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3013,17 +3016,17 @@
           <t>Bain Gets Nearly $300 Million Loan for Australia Wealth Unit M&amp;A</t>
         </is>
       </c>
-      <c r="C90" s="16" t="inlineStr">
+      <c r="C90" s="17" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D90" s="16" t="inlineStr">
+      <c r="D90" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMUQ4WExYZFY1aFBwWENNR1JiVkw4OHFKWjY4NW4zQ3ZBalFiTU10Y2hic2p2VjFqOE1rMndNYmVoN0lPcnY0WmFOV1MtaEY5c2xvcW1PNGN2SzZVcThwc3ljWkYwV1Q4a2dIaUpBeXZpMkRUU3IxZzVBVkhydGU3OXEzNW1sdlVQeTRNRFY4bUJLOGpGYmJ0ZXpPc1YzY05TYWd2bF9oWVJ6Rks2dWlod1dGRU4?oc=5</t>
         </is>
       </c>
-      <c r="E90" s="16" t="inlineStr">
+      <c r="E90" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3031,7 +3034,7 @@
       <c r="F90" s="3" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="16" t="inlineStr">
+      <c r="A91" s="17" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3041,17 +3044,17 @@
           <t>Fund managers caught up in Aware, TelstraSuper $237b merger</t>
         </is>
       </c>
-      <c r="C91" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D91" s="16" t="inlineStr">
+      <c r="C91" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D91" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcFF4Q1A5X1VtNWFnYXZSVUlZX2JMRVoxaUJoeGhybmRrZkd4UlEzTURwMkx2d2I1Y1hMYmljbk05WUFzRl9JbF9JampqeDd2bXdYcUpHbVZYak1sYXFHS2VuUDJyTUhzSS1QTW15aVpfeHRuMGZHenlxOHJQRUdENkV0b2FMZXhOZWF1Yk5hR1lOYWFQc2Q0SEROUFNERXhKQUIzRkt6NTQ?oc=5</t>
         </is>
       </c>
-      <c r="E91" s="16" t="inlineStr">
+      <c r="E91" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3059,7 +3062,7 @@
       <c r="F91" s="3" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="16" t="inlineStr">
+      <c r="A92" s="17" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3069,17 +3072,17 @@
           <t>Soul Patts defies private credit jitters with 15pc returns</t>
         </is>
       </c>
-      <c r="C92" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D92" s="16" t="inlineStr">
+      <c r="C92" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D92" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPRkNINFJOai1NbUUtX3ZrcnJFS3EzRHZPbFRfVFE3SERudTVqbjIybWsyYUthOUJOUVFPb1U0UzlGTTRqbUxraFZfYlVtclQxeTBQU1M5YjJzMDVPU3RiX0cxbk8xOEd5YjV1R04zT0NNZjhNSi1meWo4RHM1ckFsUnNLd0JiQXFnZ0dtckNzdWxmanZoQUl3TEQ2a29nRkRDZ1lJd2Y5VGc2UWZHX0pkU1NObmRJTlZKS0E?oc=5</t>
         </is>
       </c>
-      <c r="E92" s="16" t="inlineStr">
+      <c r="E92" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3087,7 +3090,7 @@
       <c r="F92" s="3" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" s="16" t="inlineStr">
+      <c r="A93" s="17" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3097,17 +3100,17 @@
           <t>Ex-KKR China heads negotiate to buy Vitaco, owner of Musashi, Nutra-Life</t>
         </is>
       </c>
-      <c r="C93" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D93" s="16" t="inlineStr">
+      <c r="C93" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D93" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQRmlCdTlFeHdBUGkyOS1CeEFIYTRSREdZM1JOZ3IyZThnNmNMdm9QeXVwRWtMbzU0em1vcDAyM1hodDlvalVRdThtNVhLR2FsaE1vV0xuWjkwMkVCUDk5SmVka1BURFJZNkl2bURLeC1GdzI0V2hEaVhrNlJZejlvc2gwRmtnUjd1NDFlX2trbGk2aXJiQ2FrTWtmVVpiOXhBc05JSkNYY2xLX2JEQUpWY2dlY1pDZw?oc=5</t>
         </is>
       </c>
-      <c r="E93" s="16" t="inlineStr">
+      <c r="E93" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3115,7 +3118,7 @@
       <c r="F93" s="3" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="16" t="inlineStr">
+      <c r="A94" s="17" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3125,17 +3128,17 @@
           <t>Antipodes Global Investment Company</t>
         </is>
       </c>
-      <c r="C94" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D94" s="16" t="inlineStr">
+      <c r="C94" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D94" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE5mdkJzN19XLTFQc25LOUk0ZGJBMER6djB2VnFvbGVrS1hlemRBRmlNY2JmMGlPTzktU0RRS3NNUW8tRXhtUE1QdE1JLWdUNVhibmZPZi1MRkJOWk95NzM2bXplS3JzeG13UU5henhza1ozeGRZZmlBNTNR?oc=5</t>
         </is>
       </c>
-      <c r="E94" s="16" t="inlineStr">
+      <c r="E94" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3143,7 +3146,7 @@
       <c r="F94" s="3" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="16" t="inlineStr">
+      <c r="A95" s="17" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3153,17 +3156,17 @@
           <t>AusSuper to lift insurance premiums by up to 40pc</t>
         </is>
       </c>
-      <c r="C95" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D95" s="16" t="inlineStr">
+      <c r="C95" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D95" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQNEhYQkoyNnJFU2xBZG8wdXhEZWRSakRiWWNHOGZBTFhfaElxWkRsSWViaWxjenVjMF91cGdrbFZxSGJfbkR2SUZNdEJtYUVadlV6YVVrWU1VbVdsMWpyNUZ4bE13Mmo4cGQ3WWZlVFVrTTdyOGpSdkpUb0tkcjdQUFlsTnM0MnpOMDJNZlJ4YTlzZGpLS1QzMFluOFU2VUJya3lSclBLSnZkQ2Y0a2djNUpSYlo?oc=5</t>
         </is>
       </c>
-      <c r="E95" s="16" t="inlineStr">
+      <c r="E95" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3171,7 +3174,7 @@
       <c r="F95" s="3" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" s="16" t="inlineStr">
+      <c r="A96" s="17" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -3181,17 +3184,17 @@
           <t>Unions want inflation-plus minimum wage rise due to ‘Trump and RBA’</t>
         </is>
       </c>
-      <c r="C96" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D96" s="16" t="inlineStr">
+      <c r="C96" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D96" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNdzNhU0MzbFRFX2I3OVY4bFItd1h6OVE2Wnpqb01NM2tMYzNob21BeW02LTBfTFZIWnN6SG5DVnYxQTJGZWZaLTJpTXZGUnhmS3RPY3hQV01fd1RIYU9Ednc4a1hvalVRT19ESU5TX19sQjN4dVV3X29kQjliQjNFU19iaXFIS2l3blk5TWUwdHFrRmJtQ0JocDN0WEhWbXZOVUJzR3RaYnJPSHpIRFlYOVFObEtuT1d0TUo0MUVZTXdFZWR3WG1r?oc=5</t>
         </is>
       </c>
-      <c r="E96" s="16" t="inlineStr">
+      <c r="E96" s="17" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3199,7 +3202,7 @@
       <c r="F96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" s="16" t="inlineStr">
+      <c r="A97" s="17" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3209,17 +3212,17 @@
           <t>Firmus’ Oliver Curtis set for green light to run ASX-listed company</t>
         </is>
       </c>
-      <c r="C97" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D97" s="16" t="inlineStr">
+      <c r="C97" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D97" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNR3VmQW9vNmUyeU9WbVRvRG9tcTNMYVlvRUhCd29wTkRZaVlEcG50Z0hIN29XcE5GUmxkUy1yMm0yTm94Q1BXMmNCcXBpZDlqVTRlZFpMX1QyMWh5Ym5XQ3VjYW1ZdDFtYWNyOERCOURuWXM5ZTV4WGthMVVjNUZlcmVTQ3JBUjQzUXRXYXRLQjlNeHpBMkVCVWpsd2Z1Vk42TjJxSlRiQ0ZtaTkzOTZtNmRHQQ?oc=5</t>
         </is>
       </c>
-      <c r="E97" s="16" t="inlineStr">
+      <c r="E97" s="17" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3227,7 +3230,7 @@
       <c r="F97" s="3" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" s="16" t="inlineStr">
+      <c r="A98" s="17" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3237,17 +3240,17 @@
           <t>Crisis Hit David Jones Chasing Funding As Retail Markets Come Under Pressure</t>
         </is>
       </c>
-      <c r="C98" s="16" t="inlineStr">
+      <c r="C98" s="17" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D98" s="16" t="inlineStr">
+      <c r="D98" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNNjJSOUVQcTkwUmxXNXg4ZzljSGhnRlBJY0otSHRrX2ZIQXRqWmNDZlgxYW1jckhHd3BtdXJsUWhwTjQ5SGw2NUU3TnFtcmhYd2JVcThIR2VCLWJLU0h5RE8xaTV5TS03Mi1za19hcF9PcXRRSU9PX3ZxSktSV2FfY1ppcUFVV2w1TmF1UWVtZlBWSUhEcG9oRGlEVkEwR2ltQ2VMSTNlcENEYlY0?oc=5</t>
         </is>
       </c>
-      <c r="E98" s="16" t="inlineStr">
+      <c r="E98" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3255,7 +3258,7 @@
       <c r="F98" s="3" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" s="16" t="inlineStr">
+      <c r="A99" s="17" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3265,17 +3268,17 @@
           <t>Beirut Street Food eyes niche in Lebanese fast casual</t>
         </is>
       </c>
-      <c r="C99" s="16" t="inlineStr">
+      <c r="C99" s="17" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D99" s="16" t="inlineStr">
+      <c r="D99" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNVlZVeTNGcXVOSXV1eklvTnFxYk1hb1A2VTQtNHkwdUpvdFF0YnlYU2RSWkZNV2dGQkEyZjRVQzVJZ2Uwc3gtZ0F1TGlSQlVna01HRnZOTTJnVUFxaWtOam1vZ245Z05jdlRnQURqbnQxaGtEcnFYS20wWmtvSDV0MW15c18zUE5ZN2JJWUpLV0RsZE1LSm5fcUNNeVZNTmdMQ2c?oc=5</t>
         </is>
       </c>
-      <c r="E99" s="16" t="inlineStr">
+      <c r="E99" s="17" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3283,7 +3286,7 @@
       <c r="F99" s="3" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" s="16" t="inlineStr">
+      <c r="A100" s="17" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3293,17 +3296,17 @@
           <t>Gami Chicken credits chip design for cult following across Australia</t>
         </is>
       </c>
-      <c r="C100" s="16" t="inlineStr">
+      <c r="C100" s="17" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D100" s="16" t="inlineStr">
+      <c r="D100" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPTXg4T0dvQ1l4NFVxV25iUXQzY0F3MnFjYmE4X0NOcFdNZHgweUg4NmVZZjNJbTFMajNhNHBmVDE2MGNBZzhOTUJsaG5KejFZbk1Db0JyNTZJbUI2WnRZeVhXRFRMNXVBWVFMdGJ3WkN5dV85dEduQi1OVDhOSE9UOGVERXh3T2hCVmlDNVg5LTdLY2VHNEZJSzlrN3VuemhzX1B5blpYRGtwS0hrak5r?oc=5</t>
         </is>
       </c>
-      <c r="E100" s="16" t="inlineStr">
+      <c r="E100" s="17" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3311,7 +3314,7 @@
       <c r="F100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" s="16" t="inlineStr">
+      <c r="A101" s="17" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3321,17 +3324,17 @@
           <t>The great fake meat meltdown is taking plant-based burgers with it</t>
         </is>
       </c>
-      <c r="C101" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D101" s="16" t="inlineStr">
+      <c r="C101" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D101" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPRTVDNW5oaWJ5bHdKM21iYllEVnpJbHhSbWFzYy1RcEZCdnNGUlJOWVJCaDZacFVoRjlSUGpfa3N6ckQtMFYzZTNITW5tMy05Sk0tZmtlSWlESHdOMWIyUWpUbE5RQVlsTHp0VXg0cHJYM0lJVmw1ckRURkFPVHFabTRIUzlFX1FlbFNuYmQ5MVJwWHVOaVhVWTdPajZxdG1WOTliTE1qZ3k1dnFRbk9BNTZCcXRRSGlIXzJv?oc=5</t>
         </is>
       </c>
-      <c r="E101" s="16" t="inlineStr">
+      <c r="E101" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3339,7 +3342,7 @@
       <c r="F101" s="3" t="inlineStr"/>
     </row>
     <row r="102">
-      <c r="A102" s="16" t="inlineStr">
+      <c r="A102" s="17" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3349,17 +3352,17 @@
           <t>Solar for Cuba: How Xi is turning Trump’s war into a China win</t>
         </is>
       </c>
-      <c r="C102" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D102" s="16" t="inlineStr">
+      <c r="C102" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D102" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQOFlUUnNZUWo0MTJRaDFIZHp5dUJudERrOWxCZmY1WjZmeXRTVzJkbENEbUFhSkZFUWV6WjNGNUJIejVYRXFPcmRNZjFZeTkzTmtaeFNlb2V1OFFnMGtkV2JfTVRUN2FSV2xxcUpDUDJQeUpqWE9DRHRmT2kyc1dIZE9jeUM2eV9KQjd2RkJuTkxYeEdISDZDejhRbVo?oc=5</t>
         </is>
       </c>
-      <c r="E102" s="16" t="inlineStr">
+      <c r="E102" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3367,7 +3370,7 @@
       <c r="F102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" s="16" t="inlineStr">
+      <c r="A103" s="17" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3377,17 +3380,17 @@
           <t>Beer Sectoral Group appoints Nigerian Breweries CEO Thibaut Boidin as Chairman</t>
         </is>
       </c>
-      <c r="C103" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D103" s="16" t="inlineStr">
+      <c r="C103" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D103" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOamdsNTN1dkRUY19Yak0wUGxsdm9NZGhySUM0Vzc4blNCeldzdFBiRkxuSW1xbTlZQUJIWkNxdzI3Zi1zc3F3SmJvai1UVGlZdUhGTEJ0eF9mNHRwSGREbDktT2txWXA4OVBESTdPLXdxWmV2V3FPTEZaYjRWLTlMM1VaY1dCbGZudTczZlFEYzN1aE9HeWdObE1yZFduLUtNVXBheDNsUWlIcUxibml4YQ?oc=5</t>
         </is>
       </c>
-      <c r="E103" s="16" t="inlineStr">
+      <c r="E103" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3395,7 +3398,7 @@
       <c r="F103" s="3" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" s="16" t="inlineStr">
+      <c r="A104" s="17" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3405,17 +3408,17 @@
           <t>Hip pocket pain comes for shoppers – and for supermarket giants</t>
         </is>
       </c>
-      <c r="C104" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D104" s="16" t="inlineStr">
+      <c r="C104" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D104" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOeTdfN2dwYlBWSTdGbFo0SWRJcTNYelFFM2FBRnlORWRNcGd0WUVCbVdHVWZ6TFdZQzFpM2h6TkU2OEtqeE5OYlRrNmhsRU43a0E0UXhtZEZyTWZidzhMUEVxSVdiMlpTYXQ4ZVRaNl9BSi1Mb3JRaXhvM2hlMmNDcnk1aFBvVXFQSmlPbkN4Z3o2R2RzV0drQWpKaVZpbXR4dHppa08wRFd0dlNwcDc1alRDSXg?oc=5</t>
         </is>
       </c>
-      <c r="E104" s="16" t="inlineStr">
+      <c r="E104" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3423,7 +3426,7 @@
       <c r="F104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
-      <c r="A105" s="16" t="inlineStr">
+      <c r="A105" s="17" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3433,17 +3436,17 @@
           <t>RBA calls for co-ordinated effort to unlock digital asset markets</t>
         </is>
       </c>
-      <c r="C105" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D105" s="16" t="inlineStr">
+      <c r="C105" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D105" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOT3dEcEtwVUptWTZydTRYWFdCU1RhTjI1RkFWeU5HckRVZjBxc2lqRkNOT0stc1h2Q0E1YTkxTjk3NTB3TGxKZGIweGFQRGh2S05QWHRoVGNZRFR2SlI2bkEzWlRoY2t3WU16dDlhVEI4RTFWYzhKS25YbGYxSVRjdFpVQ2M0dVc5MFJuUExNMTJIMVJTYmZGbkNLR1BPeVFYSF95NkNnWEEzamg3NmRuRkx0U2NjbXlxY015UWljTzRWbXpKclAwUg?oc=5</t>
         </is>
       </c>
-      <c r="E105" s="16" t="inlineStr">
+      <c r="E105" s="17" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3451,7 +3454,7 @@
       <c r="F105" s="3" t="inlineStr"/>
     </row>
     <row r="106">
-      <c r="A106" s="16" t="inlineStr">
+      <c r="A106" s="17" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -3461,17 +3464,17 @@
           <t>Banks rebuff work from home calls as Wesfarmers pauses business travel</t>
         </is>
       </c>
-      <c r="C106" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D106" s="16" t="inlineStr">
+      <c r="C106" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D106" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOTjFLNnZUNXZHeE85a3kyaG1IX29sWjFvZ2NzS041UnYxNkkwUF9YU3ZFYXhtQmlxY3Rmd0lUSTJrdTl1Y0ZobWp0M1lrZnZhZE9OSzV3Ql9Hb2UtUEpqWC1McjM0S2pESDJQVWJKQkw4enF5THJfeXFWRDZiMk5KMmVrazVUMzBNTk1tOXRVX1ZzVU1IUHBVSlhENEdEWFJpQnFXUGkyNVJGUnhzdXgyNW1WZXRkRmRaaVloZnpaMFdqVmk3elpFSkZ6ZmotZw?oc=5</t>
         </is>
       </c>
-      <c r="E106" s="16" t="inlineStr">
+      <c r="E106" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3479,7 +3482,7 @@
       <c r="F106" s="3" t="inlineStr"/>
     </row>
     <row r="107">
-      <c r="A107" s="16" t="inlineStr">
+      <c r="A107" s="17" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -3489,17 +3492,17 @@
           <t>This mine was fast-tracked to boost Australian solar. It’s exporting to China instead</t>
         </is>
       </c>
-      <c r="C107" s="16" t="inlineStr">
+      <c r="C107" s="17" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D107" s="16" t="inlineStr">
+      <c r="D107" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAJBVV95cUxPN1ZSdEMzSXBhMno2YzNkSFFtdlBOTTRGV3UtbnZtRktEd3Q0MHdmZHp0SDN5S0FZYmVKUllicHRMRkxTdmxtbkMtT2ZVN3hsUXdBVzAxdzhWcGFWRkxVdFY3NURqTVV2QVJQT0ZUT193R3JLLU9aZUw4YzlucjVUN0xyTzdoZlNjYXdyR2VWeDZrbW53cTJoRGZDd2kxbkxzMHBQWkRJMTFPMkNlX19wYjI2LVBZbnVJOVNsRjF3Tm0xUUFpY0ctczFZdWJFcHQyLUhwdDNiSGVtdHQzVVRtbExpcHJZak1SNkhWd2s4a0RtYWFNN2J2Q3FobTF1N0hWLXA4YUtaMXBScjZsUWt3alVVTVpJdVl0WDF5RTJLM1BKUl85dnhUUktkb2VwMzFkUWZ1ctIBugJBVV95cUxOOENIa2JzQzdxekNYTnJNVmRzdm9KTFpndnBybEJfNjBUR3VNMk92ZnhGY0JwVGZLeFRpdHJLMTQ0NjRNOFg5b3FESzhPLWlub2hSeFdidW0yS1h6ZXlGMjh3X3FhaWo1dHdneUZxS2NsaUJ6dWtfT1R6VndwSk52bVVNN2I5VlNYazBIelcwUkVBZHFlM0hiQVJ1a2NGWFpmR0c5R3Bna2RZMmJuSXB5WkQ1Zl94VDFtcjVEd2x6amIwSWdXUWtQVVo1Q0hpWVBLRVFycDAyU1NJV3N4YktlUlBtMTlkY2VNZjc1QVZhbnRrQ01OQnZqNzI5dTNNZ1VlNVVJcURycXlDRFZDYVo1aC15RXpwUFlvZWxlMHFybWJiM1YxT05lRElXYlZsbkJWUnI4VV9Da1lIUQ?oc=5</t>
         </is>
       </c>
-      <c r="E107" s="16" t="inlineStr">
+      <c r="E107" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3507,7 +3510,7 @@
       <c r="F107" s="3" t="inlineStr"/>
     </row>
     <row r="108">
-      <c r="A108" s="16" t="inlineStr">
+      <c r="A108" s="17" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3517,17 +3520,17 @@
           <t>A $600m dream or a dangerous gamble for cricket?</t>
         </is>
       </c>
-      <c r="C108" s="16" t="inlineStr">
+      <c r="C108" s="17" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D108" s="16" t="inlineStr">
+      <c r="D108" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxOYnpVaTZiU3hGMWY1UVVmYk9nRTJaRTVFYUE2ZklLYmJIQkdXZzFMbWs3MVRJb0l4bUpPeThwRnhOSmh0bzNBdzhpeXpuS1RrZ0tNVVJ4eU8tRVIwR2FyYmUtNG1UVmN2OXRsZm1mVy1LZDVERkpXQURMUk1HRE9Hc3F3RWQzYmFvbHRCVGhFOTQ3M2xnVGcxTWxtT3cydW84NTNPc3BXQURodmY0azBOUllOQjhrbzJ6WmI3bjY5dk5RRzlDQ0JlYzg0VzRsdWtIblZJelRSamFyQnNweHdHLTRTMTFOcy1Jd3ZtQWFodEcxOThVeVVz0gH3AUFVX3lxTE5ielVpNmJTeEYxZjVRVWZiT2dFMlpFNUVhQTZmSUtiYkhCR1dnMUxtazcxVElvSXhtSk95OHBGeE5KaHRvM0F3OGl5em5LVGtnS01VUnh5Ty1FUjBHYXJiZS00bVRWY3Y5dGxmbWZXLUtkNURGSldBRExSTUdET0dzcXdFZDNiYW9sdEJUaEU5NDczbGdUZzFNbG1PdzJ1bzg1M09zcFdBRGh2ZjRrME5SWU5COGtvMnpaYjduNjl2TlFHOUNDQmVjODRXNGx1a0huVkl6VFJqYXJCc3B4d0ctNFMxMU5zLUl3dm1BYWh0RzE5OFV5VXM?oc=5</t>
         </is>
       </c>
-      <c r="E108" s="16" t="inlineStr">
+      <c r="E108" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3535,7 +3538,7 @@
       <c r="F108" s="3" t="inlineStr"/>
     </row>
     <row r="109">
-      <c r="A109" s="16" t="inlineStr">
+      <c r="A109" s="17" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3545,17 +3548,17 @@
           <t>Why these people decided to vote for One Nation</t>
         </is>
       </c>
-      <c r="C109" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D109" s="16" t="inlineStr">
+      <c r="C109" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D109" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOQmNaOHZXWEEwZzRmdTBVT2FiS2hsYUhFczgxaFJaeEQzMGlfSnRoUWo0ZXl3cWhhbTU2NDRLUjh1c2Jxd3ZoR2pJOHVNemI2cTFrdU9oVkFCNXN4WV94TER4VmtIX1JCblhKNTl4VHlMdFBDRHVBUFhkS1AtR05RMG5QVGJFaTlWaVpMZERIa3Ntbmh0V0xnVVhYNDdMWWlpSWc?oc=5</t>
         </is>
       </c>
-      <c r="E109" s="16" t="inlineStr">
+      <c r="E109" s="17" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3563,7 +3566,7 @@
       <c r="F109" s="3" t="inlineStr"/>
     </row>
     <row r="110">
-      <c r="A110" s="16" t="inlineStr">
+      <c r="A110" s="17" t="inlineStr">
         <is>
           <t>2026-03-28</t>
         </is>
@@ -3573,17 +3576,17 @@
           <t>The Right Amount to Pay for Sushi</t>
         </is>
       </c>
-      <c r="C110" s="16" t="inlineStr">
+      <c r="C110" s="17" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D110" s="16" t="inlineStr">
+      <c r="D110" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOLUljQ1FWeHk0N21FcnpCTzdNVW1WZmxfbDFucXRNYlBMSzR6aTh4WlNrdnFuT1VSWWpKWlJValZrbTE5RlllanJkcHNHeEVwVkxldnZSdjdLc2c1SHJTVG1hMHBKd2xtZXptV1FmcGZ0cXUwVXFMWjJiRFhhYTlKRkNBNHZQekVRcnRicXlNM2NQdXJaZkVRbTZta0hDRlV5YVN5NG9TYzltUFZucXNXc29Wc1Y?oc=5</t>
         </is>
       </c>
-      <c r="E110" s="16" t="inlineStr">
+      <c r="E110" s="17" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3591,7 +3594,7 @@
       <c r="F110" s="3" t="inlineStr"/>
     </row>
     <row r="111">
-      <c r="A111" s="16" t="inlineStr">
+      <c r="A111" s="17" t="inlineStr">
         <is>
           <t>2026-03-29</t>
         </is>
@@ -3601,17 +3604,17 @@
           <t>Blackstone-backed $2b Xpansiv kicks off raise</t>
         </is>
       </c>
-      <c r="C111" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D111" s="16" t="inlineStr">
+      <c r="C111" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D111" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOOGIxbEhpZjgwbk5XampWenBXbGZmbzFQbnJhUjU1Z2FtT1FGVk40SHExMUJBZHZoRDBRVXZHS3ZlR3o5RGU0c1o0Y0E2MXVKZ3U2ZFBBRm1NbVJPRk1pMGp3dV96ZTlMNERlMFBPRDNROXpNZlNmLV83VGV2QVNzWkhtV1kxY2x6TUQ3QkhlcVNPNTlyMUQ0?oc=5</t>
         </is>
       </c>
-      <c r="E111" s="16" t="inlineStr">
+      <c r="E111" s="17" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3619,7 +3622,7 @@
       <c r="F111" s="3" t="inlineStr"/>
     </row>
     <row r="112">
-      <c r="A112" s="16" t="inlineStr">
+      <c r="A112" s="17" t="inlineStr">
         <is>
           <t>2026-03-28</t>
         </is>
@@ -3629,17 +3632,17 @@
           <t>Elon Musk puts a $2.5 trillion rocket up Wall Street convention</t>
         </is>
       </c>
-      <c r="C112" s="16" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D112" s="16" t="inlineStr">
+      <c r="C112" s="17" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D112" s="17" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPeE52VS03NHBqZ3hvc1Q4V2laUElCcmxKem9SSzM0d1Uyd09ZSFl4SjZmUDl1Sl85WXp3TWtGX3hydFRwZG0xQmFlOVUtdEtaNmtYWFkzVDYyZGI0SWFZRWtYR2tGODdPVUNhLXBzVVpzYnVRYmZNZW8xbEpreGZMVzU5c1JrWDY1Nk9uWk53a3FCOHpQTDBCT0h6QllmbW1wc3FmVU4yTUlxSmRhTUdF?oc=5</t>
         </is>
       </c>
-      <c r="E112" s="16" t="inlineStr">
+      <c r="E112" s="17" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -4037,6 +4040,566 @@
         </is>
       </c>
       <c r="F126" s="3" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>RBA’s surcharge hit on the banks may miss bigger picture</t>
+        </is>
+      </c>
+      <c r="C127" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D127" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOdWl1NWlxN0dzeEdzWThmcDVkNkpyYjJaNnZBa2dBSWhpaHhXRktTR2VtRzdUSnB3VGtDOTFuMTZXc2xycHFYN3dnQm9SaThYUURCSjg0dVlhLU52Vlo5VnRVNl9SSXFSbWFPeXdVRmdlUVA5S3FZQXc5d2lDY19UU2tJNGdrUzc0UXFHU3BGV0NHVldJcWxTS2Zydy16eHQ3QUlLQVdjWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E127" s="18" t="inlineStr">
+        <is>
+          <t>Australian Economy &amp; Markets</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>The six best new places to dine in Australia this month</t>
+        </is>
+      </c>
+      <c r="C128" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D128" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxObFAyUFZmNFk4LWJ3QzFDZnpZZlRNTEgzbGt1S1BOVF9qa2V4NnR0Yy1pX0RVUFlaUDg5bmV6LTZ2VExkWVpyZmRmV1dxNExoWkdvQzdzMTNuT0UxekhITmZBQmNhWENzV0lMYnE5all1Nk1CczFpRmhlN2pxenE1NGtLQzlKb21pSnljMlhHQjR5SVVxaG9wM01ndUdMOGpuWDduQ00waTF6OVpJUTdFV2ZWNm1yVjYzcnR3?oc=5</t>
+        </is>
+      </c>
+      <c r="E128" s="18" t="inlineStr">
+        <is>
+          <t>Australian Economy &amp; Markets</t>
+        </is>
+      </c>
+      <c r="F128" s="3" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>Mesabi Metallics secures 520 million dollars from Breakwall Capital</t>
+        </is>
+      </c>
+      <c r="C129" s="18" t="inlineStr">
+        <is>
+          <t>News.com.au</t>
+        </is>
+      </c>
+      <c r="D129" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNbVRfWlRYc2U4bV9WUVRxWmxpQWY3UTZyVGhGMGZtbEV5UXR2OTZJdGVYdFRUNzNtSUZEUVhwSzBDVWlmbWE5bTJsbDlBVXdZR0IxUHkzSDBXVkNiY3paYnlZWXBoUm1iam5oNUh5ejU2M3ZaaVhqTjV5SlpFd250Ym5HY0FvdEJvS1JvUnFRa1pmdFpKUV9OZg?oc=5</t>
+        </is>
+      </c>
+      <c r="E129" s="18" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="F129" s="3" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>Fast food giant offloads Aussie stores in fire sale after costly flop</t>
+        </is>
+      </c>
+      <c r="C130" s="18" t="inlineStr">
+        <is>
+          <t>The Australian</t>
+        </is>
+      </c>
+      <c r="D130" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwJBVV95cUxNOXRhd0lOSkctZjVDaVRpcktmZzV1aEFJZGpsbHJHVU5Rdm9JM3U5Q3JBOEdFU2tMeDBnLUJ2WmxiOGZaRVF5RF8tS3R0R1dtQWFGaEJkbHV4VjdfSDRJSnFCYnQ2bXlhOE90N3V5THdCM1JnU0JjLU1Kb1U5YkxjU0N5bUpTYVJzX3l4X3ZHakpESmVrVWdWTk5RQlFZM1Awa25rWHVabzNlNWFqbENHdFhMX3hTWFBqNDlvVTJlcjlMeHRMWE8tRm1rTElTanB4RFl0THJTazJrVTdGYkh2OUxQaDdwSmx5bTkxNGJhQUIza1F1cjJCSGNQTDRDX3RaVzZBbDFhOXB5S0hSQ3U1ckVhRWNLUF9MVTA00gGgAkFVX3lxTE1RSE5Hb0FJRE1YWjRxa1RwZk5GUmhXa1MtcmM4NDB0ZWZxTWNtaEhDczZjZ1FUT0p2d2ZTcHZGd25vbC1mR2lGOF9NQnlGNEtWUFprdG5KM1hTRGFRb0VxdkxJU2E3NUFWLXBveUM2TktmeWRoSWlaaWpTbUFOSEVmZXJIQzFOVHNLUUVCSDgyLW8yWHRBN25vSkhYNy1vRnNOVkpXbXRQNVhpWXE0NVNTWjYxd2xXTGZqdWxWa0NsNHdLNEhMQTFNcFZzS0YyY0N3MDJhLUJKUGFVc05vQkZuUU5JUDhBazYzejVpYnZ3NjJzMEFPYVpDb3IzMzlLTWdNRFBscEVCQ1pDQTBoXzBfbnpuWTJTSmRNWnhiaExPeg?oc=5</t>
+        </is>
+      </c>
+      <c r="E130" s="18" t="inlineStr">
+        <is>
+          <t>QSR &amp; Franchising</t>
+        </is>
+      </c>
+      <c r="F130" s="3" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>Young QSR workers stand to gain over junior pay rates abolishment</t>
+        </is>
+      </c>
+      <c r="C131" s="18" t="inlineStr">
+        <is>
+          <t>QSR Media</t>
+        </is>
+      </c>
+      <c r="D131" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNcXN5UDZ5d3h6NTd5YTdqUkM0dXBmdjZ0WlQ4YjF3QUxsTzdEZUVicTRweTJHYVVfYVFsQndwaURnWVBPYlJUdVRUUThQVG9jQkgzRVFyMEdBN053MDdBUmlKNHp3X0NmYVc1OFBGT2paSTZsNG5zdE9uNm1BVXd4TFEzVmgxMnJVRzFpclRlZndDTDMxU2djcGc2WVhWM2VkLW9NVkdTSnpQOHM?oc=5</t>
+        </is>
+      </c>
+      <c r="E131" s="18" t="inlineStr">
+        <is>
+          <t>QSR &amp; Franchising</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>Bain presses ahead on Estia IPO, trade bids land in $2.2b-$2.7b range</t>
+        </is>
+      </c>
+      <c r="C132" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D132" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxONzVXcThuZjBBc3ZBQWg4bWU0Wmg0X3ZEdEZkeTFKa2U3RGRabC1Jem9nOGx4MWVwOFB2SFh6UjlIdVZuV2h4Zks0Y2pVV2pnVU9Rei1TX1Y4ZzVvVkh6MzRwTlZUS3NDZDNLZDVfZjB0NlRfTnBzWkFOSW5xbUc2bi01b2p1dHlaQ3pvZWV2YTR1dWdXZzZuX2FfM0pzSkxRck1OTEgydlB3SS1GTmpMZXhvMm4?oc=5</t>
+        </is>
+      </c>
+      <c r="E132" s="18" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F132" s="3" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>Challenger-backed emerging markets fund Ox Capital shuts its doors</t>
+        </is>
+      </c>
+      <c r="C133" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D133" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQalJpNmNjb1dtSDBtLTVEQjNodkJNTVdRNUhBVkxxR3lnQlhYSGY1YW1hdnZGTUhRRzR1QnhJN3pTdC1ablBwOWtydGZTLTNTaTJiZFFHanY3VTc2YTRqcDZUQTRvS21TNDF0YmljSzIxYkxxZzRMTHY0RzViWl9heS1xT2EzbUFmUkd0bHZkZzl4Zll4UzEwOHRhazgyWHN4VUw0WUFSLWRmLTJpZDltdjcyLXA?oc=5</t>
+        </is>
+      </c>
+      <c r="E133" s="18" t="inlineStr">
+        <is>
+          <t>Retail &amp; Consumer</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>Bosses send warning on 42pc junior pay spike</t>
+        </is>
+      </c>
+      <c r="C134" s="18" t="inlineStr">
+        <is>
+          <t>The Australian</t>
+        </is>
+      </c>
+      <c r="D134" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxNaVJ0aGJ3RE9zNlVJSTVzZE1zMlpEbmpIWHpSVFVUQkNYZWJ3R3NCbjQyM1JWQV9sdUs3MVNkWnVqUnRUQjlQNmZoUkVjTHVTRENuQmxRS1NfRmd5MTM5VXMxWU5ST2M3ZjVkU2hKN3NINmhQWkJwMUZSenBnM1RselBCdVVabGNjandnV2NlTkc2SjJucUR4cjBFblNrSmlLRngzN3dlbnhTS1NkaS02R1Zwc1hrUHl6MHR0a2NkSy1XRm9hZ1B6bklHaTF6VVlmdzNaNDRWcFRXYXFDSnFpXzMxZDBZZEtORHZfckx1eEM4UdIB9wFBVV95cUxPeGhqYjFsazdhaENpSk1rY3lYM2lJSmVqSU5BX3Y4VTBsb2pBNWtqbHNqblpsNzduZktWNmxhZDJ1UTZxYnp0bWdqRFlkTEZ2aWJ5TmM3QWtEaGRhZUltcjgzVFFsaXQ5ajg0VmRmTFNXSlM5dHh3SHlsRWZOSzN4TkxUYnl2cXg3VHdTaEI0TklnTFBFVVVCRUhHRXgyR3l1bWpEeHZmQVBFM2Q4RnZoYzRiaTNYNUFBQm5XS25HcE1JRzJUT25sbXNrWGJEajBWSHJSOXlGMWFiWHJMb2pZWUFUUHJuZ2VKellQUHpEaEZKQjVYaHI0?oc=5</t>
+        </is>
+      </c>
+      <c r="E134" s="18" t="inlineStr">
+        <is>
+          <t>Retail &amp; Consumer</t>
+        </is>
+      </c>
+      <c r="F134" s="3" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>Justin Ryan’s Glow Capital cleans up with new investment</t>
+        </is>
+      </c>
+      <c r="C135" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D135" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPRWlpNFBQUTVzOE5yejU5a0tGcUN4ZHJieTV6S21BXzIwbGRmNXluSi0yVUlmaHp5Y1BaZG5CT2lVblktM3BvSDBDdEZ4d1pHLTI3NVRzeHNDdjl6Tm1tYUVLSkdoUlNidGhXUFpwVHNSRXZBOWZjVk85LXVHLWRRUUEtWDZ5Mld0T1ZPMEZoMi1hcHBWRGZJaDNJVDQ4RWkxVk9lR0JDSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E135" s="18" t="inlineStr">
+        <is>
+          <t>Retail &amp; Consumer</t>
+        </is>
+      </c>
+      <c r="F135" s="3" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>RBA crackdown on fee rort is a raid on banking’s hollow log</t>
+        </is>
+      </c>
+      <c r="C136" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D136" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQSHhSOWlMSVlkVlVaZnUwZjBzWHJxSUcyamI4ZjkxNWluOU1NUHA1RjJFdWZFaFBHTTRuRndCd0xabFJtclhZeTZ3bC1aRG5UREg5UVFyWDdIODhtV2JSdFV5R3hKZlZOc24xQlhGOWNJRXdFZl83TjU3emJ2YjZkVmFtSEpPSDBoRUNTc2JCZVNkZk1sWjI3RWo0SXZOY1dMU2xicndqVGdUOVk?oc=5</t>
+        </is>
+      </c>
+      <c r="E136" s="18" t="inlineStr">
+        <is>
+          <t>Australian Economy &amp; Markets</t>
+        </is>
+      </c>
+      <c r="F136" s="3" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>Inside Project Taronga: Koala’s choppy run to the ASX boards</t>
+        </is>
+      </c>
+      <c r="C137" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D137" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQeHotX0dQdVN6YWlES2twNXJaUUtzOEdESGJrbUdacmwxOHBDaXh6SVViWXJkMUloTGtpN3h2anNTMm1XWWVqSU5uaFlLdDZKaFV5d1BYZ3lXUE9NN0ZxN0hMWlBRejVlTUNwMUIwY0hGMmlVcnltR21GREw3ekNSSzJFUkI3ZWRINU9oOU5TRTdmRVp2MVpBQ0pPVzJHTi1ZZTFDSnBtSWwwWjRVQmpGT0N0NjlELUo5Slk5VTBYUTh0Zw?oc=5</t>
+        </is>
+      </c>
+      <c r="E137" s="18" t="inlineStr">
+        <is>
+          <t>Australian Economy &amp; Markets</t>
+        </is>
+      </c>
+      <c r="F137" s="3" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>Spotlight retail billionaires weigh up Barbeques Galore purchase</t>
+        </is>
+      </c>
+      <c r="C138" s="18" t="inlineStr">
+        <is>
+          <t>The Australian</t>
+        </is>
+      </c>
+      <c r="D138" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxNVk9feFNXOE1feC0wX1ZHaW16bUR1SUpKRWtjTHdfMDk3Y3J6WjFjNGdYcGdzbmk0c2N2b1N4cXhGVXEtU0hjYzMxRVlZT3FYMGZkend2OGg0VkpxdS1tNWM0RHRMNk5GbUJfVVVfc1NhTmFsNDlvMThjQk9PcTVnNTBUeUw4ZXNybW1ES0dXdlYyb291V280MTFCdlZMYVRIUVQ2dmUwblZjdnQ5N2pzLXMxOTcya0V4bFREM05PZkZZOHhuSTAzTFpxZUg4MmlUaDMzVHRROGQzUFkzVUFwZlZidGJhVXRTV2dPLdIB8gFBVV95cUxPRFBhdmluUkZtRldxd21BSmdkSWJsR2xNc1BYY0VGUjdVN3kweWM5WjR1VUhuRDNKYmNJellHQUl0cVJBd1o0QkdObW1PMzBTLUJmdXBlQnNJcGx5Qk1DVndrSHhzR0E0ZVRsN2t5M0ZqV3ZJUVhLdkN2d0I1VkVHZkpVQ3dNTGZLWUV2RU9tbXRvRHhDMmZzRk9fWktodmYxckZXU0dTcWg4X3M5WFJ6OTBYbjdyd1BxRnBia3RuMWJNOWE1M0Nla29hMGVPRExQWW02TWhfbXRlZkxmZ0tYS0tldDdLM3ZCU2s5UVEzNVN5QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E138" s="18" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="F138" s="3" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>Chargrill Charlie’s opens in Redfern</t>
+        </is>
+      </c>
+      <c r="C139" s="18" t="inlineStr">
+        <is>
+          <t>QSR Media</t>
+        </is>
+      </c>
+      <c r="D139" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxOalVFNURyb3NER1J2SVpsazF0S195WUpTdFcwaHhvNG9Dblc3MEw5SS0yakJiaDJLeDRZLVBSZmw5SjdkOVpEeWFmaTN4Rnl2SkdJbHBDU2VXdjA3Sm9JU2drXzNxOU5sZER6eGp6MmljX2RMWmM0VjNXeVZsWFpqYW53?oc=5</t>
+        </is>
+      </c>
+      <c r="E139" s="18" t="inlineStr">
+        <is>
+          <t>QSR &amp; Franchising</t>
+        </is>
+      </c>
+      <c r="F139" s="3" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>Former KFC exec named new CMO of Pizza Hut Australia</t>
+        </is>
+      </c>
+      <c r="C140" s="18" t="inlineStr">
+        <is>
+          <t>QSR Media</t>
+        </is>
+      </c>
+      <c r="D140" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPaDJEelhoN2tnME1SazlhTTZpOVhaWnFnN3ozUTFkZmZ4LTFXdGtQSWZVcUN4aVdhSERUSFY5NDl3X2QtUDRjNWx0WElXV1M1bTVnNWRrMURkMFlwQmljMkRlc0tnbHVzZkdha21YNWFlWC1JX1dHX0hCYi1PRGFoVDdxWDk1OGtUeXI4RkMtbXUyUVdWbHlmbGN3?oc=5</t>
+        </is>
+      </c>
+      <c r="E140" s="18" t="inlineStr">
+        <is>
+          <t>QSR &amp; Franchising</t>
+        </is>
+      </c>
+      <c r="F140" s="3" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>Restaurant Brands New Zealand snaps up Taco Bell franchise from Collins Foods</t>
+        </is>
+      </c>
+      <c r="C141" s="18" t="inlineStr">
+        <is>
+          <t>QSR Media</t>
+        </is>
+      </c>
+      <c r="D141" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNak9JTVQ3ZUFpN3BYU3U3d1FwdVAwU3V6Z3VxREhqX2h3Q0tFalhDMHpqWFpfcUxuc3NMSjBsRi1QR21oNmg2NUt4dHFPV3ZDNjE1N01yT2JuSFBjU2dGeFl5SjVmSEZtSlpfZHVtTThTZmxrLWttZGxYZURvOTBRcjRMRVFIV08xUU1PUXNSMHJ3MV9LSVBMSzVIX1RkRFhZa1Q5cG12eWVJT1dCT3Nr?oc=5</t>
+        </is>
+      </c>
+      <c r="E141" s="18" t="inlineStr">
+        <is>
+          <t>QSR &amp; Franchising</t>
+        </is>
+      </c>
+      <c r="F141" s="3" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>Gelatissimo hits 60 outlets with Zetland opening</t>
+        </is>
+      </c>
+      <c r="C142" s="18" t="inlineStr">
+        <is>
+          <t>QSR Media</t>
+        </is>
+      </c>
+      <c r="D142" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxObVNNeU1EalQtaFRrbVIzdGRDcjIwampSckY5VlM4RzF1aXpmX3hweTFucmpxQ3gxUFhGZmVrck5GTzNyb3VxR1gtRVBwbXRVaFE5REJ3UWQ4U3hqd1RFU05kcVA5ZlVEUG80cUU1a1U0VWNtMXp2QmkzZ3F5X01pcEt5WkxvLUg2UTFzTw?oc=5</t>
+        </is>
+      </c>
+      <c r="E142" s="18" t="inlineStr">
+        <is>
+          <t>QSR &amp; Franchising</t>
+        </is>
+      </c>
+      <c r="F142" s="3" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>Investors flock to Koala as furniture retailer soars on ASX debut</t>
+        </is>
+      </c>
+      <c r="C143" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D143" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOWHFPQVY5MGg5dzRzeDNQVG5PM204dkUyQWtYNTVGQWpIY0NFWTUzTFZMV3VuV2FWTWZqSVpldmdNY0YzU2VTX2c5eXUtajJPWXJmSm5iRlRleWNRMVhmZUJxaXNDNENMNGV0RmZWNEkxTWZPTE95VGtDYWhwSzZGZzBNbGZ4OXZBM2FxbElnTU14WnpVbUhyYTJGaGZHdjd0Yk0tRDlacno?oc=5</t>
+        </is>
+      </c>
+      <c r="E143" s="18" t="inlineStr">
+        <is>
+          <t>Retail &amp; Consumer</t>
+        </is>
+      </c>
+      <c r="F143" s="3" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>Australia's Collins Foods to transfer 20 Taco Bell outlets to Yum Brands</t>
+        </is>
+      </c>
+      <c r="C144" s="18" t="inlineStr">
+        <is>
+          <t>Reuters</t>
+        </is>
+      </c>
+      <c r="D144" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOWnNHb0VCMjhOUTNrUS1WOUhmRlpnelpxMmtFZmxGY1poSzB4dHFWcjdNN3lWcVhyWUpSU1UwSjhpY2dUNlg1N1hQQ1pRVUFKcm5MSHV0TWYwSmtqTHF4a1FQX1MtdmhqUV8tZ1lJcC11c2J3TXJWWG5mVmtSUkFWTDBZaXc4QVcxeGhxeHVBQVJ4TVJ1Sm5scHlmNTFsSzJWcktEekp0dk1QeFJSdnVpd2Mtdklya3ZiQmJodw?oc=5</t>
+        </is>
+      </c>
+      <c r="E144" s="18" t="inlineStr">
+        <is>
+          <t>QSR &amp; Franchising</t>
+        </is>
+      </c>
+      <c r="F144" s="3" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>KFC operator Collins Foods offloads Taco Bell outlets</t>
+        </is>
+      </c>
+      <c r="C145" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D145" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQV2x0VTJWLWNLcGlYWDZCc1NpbTd3MnlvX09kMWpIeS1jMGQ0OF9sc0k2RHZFY0JudmVJdVJtNnF1Zk5vYTRDNG1aNDlVQmZMM0RLRFZWZFR6bUhJQVZlc1hDY2NCbDJVMzBCMVF0ZlhvNEpVOHNUV0Uyb0hCQU1ndzN5Vk5pMFlSQWxXaktmdTQycVctTGx2dGV1Um5ycDFFWmVkQ2puLWlTZw?oc=5</t>
+        </is>
+      </c>
+      <c r="E145" s="18" t="inlineStr">
+        <is>
+          <t>QSR &amp; Franchising</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="18" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>Count launches $40m capital raising for financial planning acquisition</t>
+        </is>
+      </c>
+      <c r="C146" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D146" s="18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQQl9MSkpfamt1UUxyeTVILVlKSThwOXVrUmxfdF9nMVIySC1pc3RLNXB0c1Y2X2ZRakw4dS1FLVB3YlJlQ1BkcXBRUGc1NXNKS0lMblVpQVhsZWZlNTdPRXFQMzdyUDNtTjlkeHQyRkdXaUtiQzZUVHpPV3p3a3hqYVdTaU1CdWFvYmhiTmhBeFVwZlozQjJnWHl3NTYzYTlTbkgxUi1OYXlLcS13eG05ZnBsQUthQ0E0?oc=5</t>
+        </is>
+      </c>
+      <c r="E146" s="18" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F146" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>

</xml_diff>

<commit_message>
Update news log — 2026-04-01
</commit_message>
<xml_diff>
--- a/news_log.xlsx
+++ b/news_log.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -87,6 +87,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -498,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F146"/>
+  <dimension ref="A1:F152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -542,7 +545,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="17" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -552,17 +555,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C2" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D2" s="17" t="inlineStr">
+      <c r="C2" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D2" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E2" s="17" t="inlineStr">
+      <c r="E2" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -570,7 +573,7 @@
       <c r="F2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -580,17 +583,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C3" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D3" s="17" t="inlineStr">
+      <c r="C3" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D3" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E3" s="17" t="inlineStr">
+      <c r="E3" s="18" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -598,7 +601,7 @@
       <c r="F3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -608,17 +611,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -626,7 +629,7 @@
       <c r="F4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -636,17 +639,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D5" s="17" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E5" s="17" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -654,7 +657,7 @@
       <c r="F5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -664,17 +667,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D6" s="17" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E6" s="17" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -682,7 +685,7 @@
       <c r="F6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -692,17 +695,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5</t>
         </is>
       </c>
-      <c r="E7" s="17" t="inlineStr">
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -710,7 +713,7 @@
       <c r="F7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -720,17 +723,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -738,7 +741,7 @@
       <c r="F8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -748,17 +751,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -766,7 +769,7 @@
       <c r="F9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -776,17 +779,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr">
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5</t>
         </is>
       </c>
-      <c r="E10" s="17" t="inlineStr">
+      <c r="E10" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -794,7 +797,7 @@
       <c r="F10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -804,17 +807,17 @@
           <t>Zarraffa’s Coffee celebrates 30 years, eyes nationwide growth</t>
         </is>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D11" s="17" t="inlineStr">
+      <c r="D11" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOcXNzUkRLemZEOWtOZjhvRUtzcUZrSTdzV0s0LUJTd2NGRk1Gb1NSLUR5Rlh3NUdWQUJkVWctb0toUFBRajlMcWV3VnNyTUtydy1PSUoyb1NCOGVtMUZqRVN0MzFkVkNlOUZNVXlHN2kzREhSdWJQUnJqa0pnUzExTVZSc1NCVFZSNlBSUWNfWnZ3MC01aUx0UWF5SkNOaHI3ZkE?oc=5</t>
         </is>
       </c>
-      <c r="E11" s="17" t="inlineStr">
+      <c r="E11" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -822,7 +825,7 @@
       <c r="F11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -832,17 +835,17 @@
           <t>Zarraffa’s Coffee eyes 200 outlets ahead of 2032 Olympics</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D12" s="17" t="inlineStr">
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPMUFjRTlGVFBqYzlPWXdzQ0dKVVlhWGxncUQxTDd1R0VHcThlV3ExVmo4SlBGSHVuUGZrMGNqSVo1YVpDWHViMm5KZWIxcHNMMHo0b1FQcmxUNElDR2lEeWRuLWZIN2lyQUV0VndEUWNkNU42Z3AzNXRlbm50NzhtTXZ0Q245dF9hNzBxOENuMXZsVlU4Z0JGVElR?oc=5</t>
         </is>
       </c>
-      <c r="E12" s="17" t="inlineStr">
+      <c r="E12" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -850,7 +853,7 @@
       <c r="F12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -860,17 +863,17 @@
           <t>Aware Super appoints new head of private equity</t>
         </is>
       </c>
-      <c r="C13" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D13" s="17" t="inlineStr">
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNVHJXNWEtdEZZUW1fZzdYMTB4RklBTUh6dUNKQ3BrTlpYUnBwRURIVGZjWTV0OUxScnhGMVNSczhLUjVqOEwzbkR2WWlEbmF4ZkNUdHNQY0J1djI0REctbHd2SVhUNlNCa2M5bFhOQ0JPU0RHOVVTQkEzRDdGMjRZbVFDOUdlTXNNczlmZWF6bXlfbEFGRE0xbkZQaw?oc=5</t>
         </is>
       </c>
-      <c r="E13" s="17" t="inlineStr">
+      <c r="E13" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -878,7 +881,7 @@
       <c r="F13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -888,17 +891,17 @@
           <t>Commission wrinkle over UP Education sale</t>
         </is>
       </c>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D14" s="17" t="inlineStr">
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxNSV9GMjhqM2ZSanI2X0w2OVlQVFRQTUoxYzAxaXVZMmU1REVTcHlUeEltdXJtaXZrcUJWdDZxNGpYTTZYSFE2TkZHeG9OaVRZakoxV0s1U01TVjJpWlhaSENfNVhucG5NVzFMbTVBY25zWGRSODBtRGtkS1owVTlJWnNfcTJ5alFnbVl1SU9aUDF1QWxJLTBSQ3kxUUFlZnpJMlVEQndFSGRGbDF6WVBUVHlCcDM5Qnh3R2xBMG9xN2FLckNzbUFOWDI1aVF1YV90d0twd0ZmMnUySDBMdG1R0gHkAUFVX3lxTE5EWVp6VzZWb01TRmlHSS0wMExldkJwSHJjdlZXdElsRlpBTEtVMkd6VzNQa1RpVDNsOFQzaGZ2VHpzUnBDYk82RmZGQWJuTmVQMXhxLXVmdVFxTVZOZTBsOHZ0V3cyVVVkNWUwVUxSc0xNSU92ZktpdFRfYnQ4WHBTX3A5bFhXZ1YwZXNrc1BSZEU4LVYybnNBd0dCdk92OFUwclJCMzdoU0ctX1pEdTAwY0JiTWQ4S01QRE00TW5EUEJwR2YtczZ0T005bTJnN1RDY2p6NFF1SndfLUo4QzJUWk1tRg?oc=5</t>
         </is>
       </c>
-      <c r="E14" s="17" t="inlineStr">
+      <c r="E14" s="18" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -906,7 +909,7 @@
       <c r="F14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -916,17 +919,17 @@
           <t>Gloria Jean’s owner has an angry shareholder on its case</t>
         </is>
       </c>
-      <c r="C15" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D15" s="17" t="inlineStr">
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPTnZwUVBCdTFJZWkwc0YtVmJqMkNPcUR5RktjMlVURmhROFZkYUpXM01iRUh3SnJEUElxRGlSNk9DQjZSdTdNdmZwWWpONjlmR1hoMl92cUNmd3M4cnJhVkNqc095MmN6WXBYUmdEblB0eERtVDdlUU4yNGFjXzVnT19rOERIRzVPNzY3VDNNRS1tVGVTX3pKMVRpTXZVR1ROLURBLWtJbVZhY0lSU09DNkE2NzFLbEFU?oc=5</t>
         </is>
       </c>
-      <c r="E15" s="17" t="inlineStr">
+      <c r="E15" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -934,7 +937,7 @@
       <c r="F15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -944,17 +947,17 @@
           <t>Oporto-owner Craveable Brands hires new CEO from Domino’s</t>
         </is>
       </c>
-      <c r="C16" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D16" s="17" t="inlineStr">
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNNmxfQVc2Umc4QWwzSTdsZTFvejRzTzZxXy1ScGlhXzh6bm5JS3IyX0xTNDVBNjh0cXpPbGhxNU5xUHhQN3EtRF9aV3FEc2JoSG5QTU1WeU1TLUJfZzVUT2N6dXloQXhZaHB5djB3dDFKN1llVmI3UVpKNjJTNlcyV0ZDcG9GdVdSdW41ZkN1b1N3SFFIUzcwRkQ3UHY2TmxERmZwTlA0RzU?oc=5</t>
         </is>
       </c>
-      <c r="E16" s="17" t="inlineStr">
+      <c r="E16" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -962,7 +965,7 @@
       <c r="F16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -972,17 +975,17 @@
           <t>Brookfield, BGH Capital rub shoulders in ScotPac’s data room</t>
         </is>
       </c>
-      <c r="C17" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D17" s="17" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPMVlxbzlQNnFXWnJFNU11Y1BhTTVqbjN4RG1nbkZuN0pkdDFFaUhJN0RaVnUtWDlZSGJWR1ozQXk5UUx6RVdOcjBPU2t5UzN4T0JvUFJISnNvVWxQemd3blNHZjRQVVVZQk1nZER0Y0JfY3VvQ0t1a09sM1RTS2c1YTJyUmdzYWh1WGRUNjl2dkdzYTJJeHVhMTdqR3Y5WVlHVEtSZHp1cmVYYmM?oc=5</t>
         </is>
       </c>
-      <c r="E17" s="17" t="inlineStr">
+      <c r="E17" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -990,7 +993,7 @@
       <c r="F17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1000,17 +1003,17 @@
           <t>Payments player Pay.com.au hits the road(show) for $850m IPO</t>
         </is>
       </c>
-      <c r="C18" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D18" s="17" t="inlineStr">
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOMFZleXZrbU53TzBlakI2ZmJKTjlrN3BoQlRaWjQ5cXFzTllKWmFoRm1UT2xDUHBtNC1QNTNiX1BwSzllMkRZdHIzRlAteDREaUczN1JTNTByTW1jNnR3d2NnR0RxUDBxeHYyWU1CSUs5MEZad2JqSGF6ZUxHZUNtZmFQaTJZZVJVZ1B4MkZ6V09QMWIxaUNHQmVzTDhvWVA1Ty1UbHgtQnRrQQ?oc=5</t>
         </is>
       </c>
-      <c r="E18" s="17" t="inlineStr">
+      <c r="E18" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1018,7 +1021,7 @@
       <c r="F18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1028,17 +1031,17 @@
           <t>Another year, another IPO cold shower for investors</t>
         </is>
       </c>
-      <c r="C19" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D19" s="17" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNeEhzYzQzdjR5MDJCWkd6Q2VLdEZzbzRoWnNOcXFlQjNfMlV4Q0NQRjExMlNhT2NPcnRBbW1sZUkteXo4N0dGaHNNeGZJOEZ2aXFvdmZiN2V2QzdOMzFteFRnY1RVRm1rQXltWmY5VFZOdFVNNVpudVp1dTlrcFM5b1k5SmlWQllDMVFXSjA4ZVpSZHgtV2JpWDJ4SkFRbVE?oc=5</t>
         </is>
       </c>
-      <c r="E19" s="17" t="inlineStr">
+      <c r="E19" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1046,7 +1049,7 @@
       <c r="F19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1056,17 +1059,17 @@
           <t>Priceline Pharmacy franchisee sale narrows to final four bidders</t>
         </is>
       </c>
-      <c r="C20" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D20" s="17" t="inlineStr">
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNR294am9sYWNiQ3FVT1B6YlV5ejMyeHAyT0FibTFVbU5pcjZyaVRyazEzbFkxd0lrcnpZNGpTYUx4Ykl1Xy1sZF93M2Nid19ydUFwbUJ3ZHozaURaNkRoOE9OMnRBRGZfQVdCVWZCaVhhNnZSRjlwYUdDVnp2WU9HUkJxbE1QMV8zdWxYRTNBQWktR0xSOFU4dmtXZWk0am9SSU92NWp6QUZmTVU5TzJEOEJNak5fQUtN?oc=5</t>
         </is>
       </c>
-      <c r="E20" s="17" t="inlineStr">
+      <c r="E20" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1074,7 +1077,7 @@
       <c r="F20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1084,17 +1087,17 @@
           <t>Private equity gets better image of Qscan</t>
         </is>
       </c>
-      <c r="C21" s="17" t="inlineStr">
+      <c r="C21" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D21" s="17" t="inlineStr">
+      <c r="D21" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxPRjVmT0hDRjZLblB1VHdPRmRGeXhKdDJHdWxDTzV4RDZ0VzdHaUFfOVlnZjRQMWhKcWMxby1oRDR6N2lQZkI1UDE1REppS3c4LTVmU3p5b2wtblRCWnhNajFnZGNHaGRJUHFMUGRtTHAyQmIxOHhNNTgwRWVSeWp6ZWRxbUY0WVhiUnhMRUpDLXNwS1RuelJldTk0Z1R0WHg0XzNXNTA5Rk5TRFZhU1RNVnN2TlZuaFE4OWtIYXQ5a2VGSW1UWmt5Rlc4Q2lIXzF3YlkwNVhfUzJDV0dQdVAxa2RKc08wRGR6TlB2Vi14QV9BdlhyaTZsM2pEVGZycTjSAYQCQVVfeXFMTWpnb0lWQmZ6MTFnRGhWNTNqczk1TWhTcUFEMVpDNnJ4ZWVxVlRUODhJXy03NHdGZVJlMmhyUHM0Nlh4NlZtTzRhQ0xxRDFLVHNzUVNfbWxhS3BLUEQteEMzZHRrc0F1eFRzYmxVNDZlSURyZDB5bF9wQTNRRU5yZEs1Z3pFRTdwcFBaMkNlN0JvT1NEYkFWVUJNcHJqcEM5RVJYa0JFUVl6cThyQXloaERzQjhkTUVPakJqb0hzNVlwSWxNS0dmZkNFSG9Gb3dNUnVvUnV0d3MxSmpzdFZKTHJ2RTQwRUoyMEVLLWMwT1NnOHdXVl9lRXNDWEFndzJFSDlZU0o?oc=5</t>
         </is>
       </c>
-      <c r="E21" s="17" t="inlineStr">
+      <c r="E21" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1102,7 +1105,7 @@
       <c r="F21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="18" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1112,17 +1115,17 @@
           <t>Oporto CEO’s first year reshapes brand and network strategy</t>
         </is>
       </c>
-      <c r="C22" s="17" t="inlineStr">
+      <c r="C22" s="18" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="D22" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPY25mNTJfT3FiVlBPZE5CcVNkR1UzR2xWaUtJSmxhU3EwcEMzQi1ISDFSajlCQWk1UUJpZVJ1Q19ZV3Jjd0Noc0l3OExpMXhSQUVVdHhCLTBlOXNoZzA3UXZBdkR1VHBvMmVsZkNhUFJndm1DdGpnX2w0ZVViU2phZ1RmYXY1SlhwUnhKSUxBQVZZUXpqNHQxQmo0Rk1iV0g0OW9qUS16eWRSNW5FaW1yQQ?oc=5</t>
         </is>
       </c>
-      <c r="E22" s="17" t="inlineStr">
+      <c r="E22" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1130,7 +1133,7 @@
       <c r="F22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="18" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1140,17 +1143,17 @@
           <t>The Melbourne restaurant our reviewer grew to love</t>
         </is>
       </c>
-      <c r="C23" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D23" s="17" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOc3YxQTljcHJXVWtRX2ZGM2lpM2pILWNwSFg0MFJrNmNWX0ZxRG9nV0J5N19qRWh4U0hPXzNmVVZwWk9wT2kzaFNrTlV3NEQ1Q3JpaXVIYlBHb216Q3VYVWdSRXMwdDl0SmYzdnRlSDFUYVRmRGJyZVlRZDJKTHpJOUctYlF1RDZSYjloY0hfZy13QmFTLU9UNjkwTHc1bjlGcGxoZ0ZLVU1GWTctZkdLZU9zSGhEZEpKbXJnaWJfZjd2OWs3?oc=5</t>
         </is>
       </c>
-      <c r="E23" s="17" t="inlineStr">
+      <c r="E23" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1158,7 +1161,7 @@
       <c r="F23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="inlineStr">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1168,17 +1171,17 @@
           <t>Crescent Capital strikes Benson Radiology deal for close to $400m</t>
         </is>
       </c>
-      <c r="C24" s="17" t="inlineStr">
+      <c r="C24" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D24" s="17" t="inlineStr">
+      <c r="D24" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOLTNrWG1ZZlFoU3pDZ3E2SEgwMlhzQkdtQUYzaHZTZmYwU3ZhMnE0dlkza005VkZmZ09NMExlWDVncnBmYVVISXJ6X1ZjNHhpM2RnSlprY1dnbndJNUczcDVtNXNRY3pVNW12bm5rUVdqVmR4R0JlVHFuN0RwTlFkR2xrbFFpSl9jcm5oSjk3aFM1clBSVDhnbkhoWUREeUhsbVpvQW90d05xOTdfOV9nbW5POFdmelJkVlpsUlRuYl9odmRNVUV2S0pCMFBMTS0tcVhGVGFYU0h2d9IB3wFBVV95cUxPWEs4R2pxdThPbHJHb0dBT183SkRHTTlXNzdWazcxdkd1eGx2VlAyM2VVbEtEbWxTZ1R0TlBFRmRMZTFoalgxSmVVRUJFR0c0RFYzZVJFODg3dWxicU9pOHppeFhjaVp0WWlyTnUzV1dyZXdkMHBDVHI4LUVQdjc0cWpheU55NTlvdWdCZmVoODB0Mm5fbGNCTmQwLUhMZ0psQVpzb3BEUnJpSkRnOUM0c0VCdUp5N3g5MkhaM01vTHJ3NWd0ay02UXZUUG9nVkxicVc1Z0xjWGhjUDRDVjlN?oc=5</t>
         </is>
       </c>
-      <c r="E24" s="17" t="inlineStr">
+      <c r="E24" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1186,7 +1189,7 @@
       <c r="F24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="inlineStr">
+      <c r="A25" s="18" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1196,17 +1199,17 @@
           <t>Dual-listed giant Capstone Copper flirts with $600m-plus carve-out</t>
         </is>
       </c>
-      <c r="C25" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D25" s="17" t="inlineStr">
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNcVh4blRkQnoyaG1TajhVV0lrOEJRaHdTZWtzUnJHaEdaSXNRWThGTHlVdGl4dGJ1cTMwZ2pLcVNzUXRYNlZzVzhvaXdkNGtVUG0wN0FrMHB0R1I2Ry1jcEgtSWUtajI0cTFMRTlfdzBuMWtrZmJOLVUtMkl5dW85dFp6dEhEOHhTNzdfOFNFSGtlT0MwQnRlY0VhcUZBNE9RYzhQcDdOQUFnYkgzd0V0N253SQ?oc=5</t>
         </is>
       </c>
-      <c r="E25" s="17" t="inlineStr">
+      <c r="E25" s="18" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1214,7 +1217,7 @@
       <c r="F25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="inlineStr">
+      <c r="A26" s="18" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1224,17 +1227,17 @@
           <t>Guzman y Gomez unveils a new menu under $4</t>
         </is>
       </c>
-      <c r="C26" s="17" t="inlineStr">
+      <c r="C26" s="18" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D26" s="17" t="inlineStr">
+      <c r="D26" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPMjRjRTV2a3BJc3AzdDNOQktoYjBvLVZSODVsc3lKQ3pET0lxUlpkc05NcVlKRlZITjVJbjkwLS1DUFJNMGJ1amJKTlp3S3VqMWJaU3YtUENEN01rUEJiV1FNZTRXYjcyV08zZzlxNDVOSlVOTlJDOGV3QzBQcUpKa2Zab1ItNlI3ajZVVTF3?oc=5</t>
         </is>
       </c>
-      <c r="E26" s="17" t="inlineStr">
+      <c r="E26" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1242,7 +1245,7 @@
       <c r="F26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="17" t="inlineStr">
+      <c r="A27" s="18" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1252,17 +1255,17 @@
           <t>Can Sydney’s burrito king conquer the $676b US fast food market?</t>
         </is>
       </c>
-      <c r="C27" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D27" s="17" t="inlineStr">
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNM0ZFcUpLN1dUZWUyaE1LMnNZVGlEbkNNQUQ4Wmd6QVFlTy0wZDVHdnlja1gzMEZTbVpKU1Ftb3VKZ2pzajcyWU16NUtUTmR0TlZMOVhMRUNqZXZiX2d2NWY0YlJDOFhhYUE0SkhMRUprNndXak8tWGdERU90cmMxTkFjcFFVSTd5VlZ3NFVKOXN3M255MFhzZThmbi1VUGMyQ3E4d2pYcFlJckY3QlVBdVJJeF9qUQ?oc=5</t>
         </is>
       </c>
-      <c r="E27" s="17" t="inlineStr">
+      <c r="E27" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1270,7 +1273,7 @@
       <c r="F27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="17" t="inlineStr">
+      <c r="A28" s="18" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1280,17 +1283,17 @@
           <t>Drone maker Innovaero prepares for ASX float, taps Euroz Hartleys</t>
         </is>
       </c>
-      <c r="C28" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D28" s="17" t="inlineStr">
+      <c r="C28" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNU3JrejNRZ1VBZVNVV29NMkFPVmRsWE4yMVZPcjk2aUNUTHFJUGFyQ1VnZEZiZlIzQW9VVzRNNDNRR01jcHo3X0tqZjB4bzhMTTI0Y3BwYUh6OGRUUGt2REIxV09oRnJoVWlVelZWaUlWUmlPQ3dJdi1TejcyaXB1Z0x1MEJRSlB3SGMwVGdXaXJJNm9TVllPOG5JZC1feEV3TVhTeExGeHR2RHFIWlVCOXh3?oc=5</t>
         </is>
       </c>
-      <c r="E28" s="17" t="inlineStr">
+      <c r="E28" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1298,7 +1301,7 @@
       <c r="F28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="17" t="inlineStr">
+      <c r="A29" s="18" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1308,17 +1311,17 @@
           <t>Bain flaunts Estia 2.0 as IPO roadshow gets under way</t>
         </is>
       </c>
-      <c r="C29" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D29" s="17" t="inlineStr">
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D29" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNTEN1cGsxNDN2c1NqUzB6UmJ4TFl0NGZjZVN3U3oxMlVFWTF4WUZLQS13dUxMV0N2ek1XN2VURTNVWms1NjdXSm0waEdaTXQwdTdWY1MxZ1V3ZnpEcVJtczdOWGNNZ0RQNzRZLU1MTTgtRW5DZkctbXBGMmVXVXdPZW5pNThiRHEzWnB2eFZzTFZTb1ZkeW9LendkNDd0cXRid05ZSGZYbW9NZXdOLVZWODdZU3hVcTA?oc=5</t>
         </is>
       </c>
-      <c r="E29" s="17" t="inlineStr">
+      <c r="E29" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1326,7 +1329,7 @@
       <c r="F29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="inlineStr">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1336,17 +1339,17 @@
           <t>Carl’s Jr. Australia unveils nationwide freebies for Happiness Day</t>
         </is>
       </c>
-      <c r="C30" s="17" t="inlineStr">
+      <c r="C30" s="18" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D30" s="17" t="inlineStr">
+      <c r="D30" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNVWgwdjU1NDFWalBfMTFYX1dQOWNDbG1FVUdlcS1LTVlHZVRRTVBWTjhSMnpkTXRXNlFJdllGQUp5Mm5ObWpIazd1d0RJa3QtdFBZN1hOenBmVzBEU05wM0gtNUxPeWpsYkxyVnhWWFFOU2Y3R0tXcmNkeWhpWDh2eDZBdjNCMHhuc1lHYTZHblBPVkpfRXpKd051UWlNc1hm?oc=5</t>
         </is>
       </c>
-      <c r="E30" s="17" t="inlineStr">
+      <c r="E30" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1354,7 +1357,7 @@
       <c r="F30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="inlineStr">
+      <c r="A31" s="18" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1364,17 +1367,17 @@
           <t>BHP and Woodside appoint new CEOs in major mining shake-up</t>
         </is>
       </c>
-      <c r="C31" s="17" t="inlineStr">
+      <c r="C31" s="18" t="inlineStr">
         <is>
           <t>ABC News</t>
         </is>
       </c>
-      <c r="D31" s="17" t="inlineStr">
+      <c r="D31" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQbTg5VFJLbWJfcy1uV3ZReTJkTndzX01qZ2MxNWkzaWZRckNLZUR1Y1VsMVRNc2FySC13U0NzalFEb3k1R3BaUEhfcTV0N1M4Q1dpSlo0YXI0UFhrMGRab2RiYV9DQVNVX01ycFc5ZFZrZWZqc1VRZXoxLVEzSDJLclJLSWg5bzN3R1I0bG9lWjVDaHE4?oc=5</t>
         </is>
       </c>
-      <c r="E31" s="17" t="inlineStr">
+      <c r="E31" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1382,7 +1385,7 @@
       <c r="F31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="17" t="inlineStr">
+      <c r="A32" s="18" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1392,17 +1395,17 @@
           <t>Next Capital sells Enviropacific unit to French waste management giant</t>
         </is>
       </c>
-      <c r="C32" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D32" s="17" t="inlineStr">
+      <c r="C32" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D32" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPR3lFbERLR2FtdmJUU3BDU2thZk00YmFHRFhXR2VBVXhQSURTeE5ONVJKczBwbzlFMnR5cmhxMnM0bzlJbWo4SXl1dHpqYWxxMUJBRjZHVUtab1RYZjZMTnpGc3FzMWQ2NjNEdGU3NTZwa0diM1lJS1haYllwTldLZlpZbXp0YzlxcDh0ekcwTy03dDdPcnk4b29HZVdqbHhZY2JPR2drM2puSVpjUzZkVjNpZUE4dVMwYlE?oc=5</t>
         </is>
       </c>
-      <c r="E32" s="17" t="inlineStr">
+      <c r="E32" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1410,7 +1413,7 @@
       <c r="F32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="17" t="inlineStr">
+      <c r="A33" s="18" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1420,17 +1423,17 @@
           <t>Future Fund private equity and real assets chiefs head for the door</t>
         </is>
       </c>
-      <c r="C33" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D33" s="17" t="inlineStr">
+      <c r="C33" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D33" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPUHNHRFhFMVdwVld6RFRZUFd3QWNOd1kzeS1QdnJxMERFSnE5LTdZcDhDYlVGcWZMeWxlR0FSRWF6YkZoQVZrZU9TQ1E4YTEydUJnOFE3enV5Rmk5UnF5VEdYZ1FMUWpKVjdjMlZZUGFsU0tKcV9Vbl8zcHp5aVF5Z2JMOUZocHJqRXNRaEp4Nm5CbDM1WkdIMHdQS2xqQnE2Tnh3?oc=5</t>
         </is>
       </c>
-      <c r="E33" s="17" t="inlineStr">
+      <c r="E33" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1438,7 +1441,7 @@
       <c r="F33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="17" t="inlineStr">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1448,17 +1451,17 @@
           <t>‘I actually started to die’: the new billionaire’s epiphany</t>
         </is>
       </c>
-      <c r="C34" s="17" t="inlineStr">
+      <c r="C34" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D34" s="17" t="inlineStr">
+      <c r="D34" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxPblkxbHVrdnVKY1pqQzNyWGNMZm9UYmY3dzlPaGQ4Yi1tc0U1akhrVWdIaXBpM05aZXRwTXE1eDBITlZpbDkwRXNrWjJ2YXBzX0VCY2JSLWhrVmpjSTE5eE5rLWgtc2pRZEdXbmhhWU1KeFExZDBGS2pjSkIwV0FGbndBZVAyQkg4WFRsengzSGYyZkFfQnJsQ18tUHJGNDd2T0pzZElPSVJTQkl2Rm5QTExJNHhmU2dHOHJGdTdzU08yNHRtd1R3Q0cyOF8taDktQTZvVXVBVjN1d0NHMmtFOHBWZXBFcUFWa1IyWGNDTDZUT3lQSXJHOVhxTFQ3b3RH0gGGAkFVX3lxTFBZQ3BFQWl5dEwwLW5yVWJuMU8zcXBPdE9pamRVSWVkbWNyVzgydGVOaDBROUN6RlBDbjdld05DVmZyb0R1eEN0UERubzZRU2NiMTQtVV9XNS1wYmlvZ1paM3RaOUlrTzJka0tXVVJEamFESGlSdXg2bDk1aUdhUVhBcXpnN01fX0Y0cTNvcm5DdEFFLVVERDFKTWxKZFR0UzAyblJqVHBua2JoYUdzeUNMb053ZVczWUFQU1AtVHV1d3lSSDFfZFh2cEkxSGw2MEdicEVsb2pLQ1RuQmdaRl9xNUROS3pKR2s2T2wxTTZ5bEwtTUNQNU04djFHTHlPbXVLSW9YSUE?oc=5</t>
         </is>
       </c>
-      <c r="E34" s="17" t="inlineStr">
+      <c r="E34" s="18" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1466,7 +1469,7 @@
       <c r="F34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="inlineStr">
+      <c r="A35" s="18" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1476,17 +1479,17 @@
           <t>Ironbark shuns private equity as it hunts for cash injection</t>
         </is>
       </c>
-      <c r="C35" s="17" t="inlineStr">
+      <c r="C35" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D35" s="17" t="inlineStr">
+      <c r="D35" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxQZWFaeVhldi00VkV5ZmEtS2tjcWdFWG55OGpCX3IyN25Rb3ZFV0ZKVm1aSE1WbThoYVY4ZEdfODVGX0RaUDV2Ul9HS1JQMDFCT05Fc2FaU0RINTMwbDRveWFsOFJSM2ZqTU9tVGxJSEl2ZmhhUHFHT3dqYkk5TUtvMUQySnZzTWw1MzFNWl9aVzhkSEZ4Q3YyWjRMUmpIdmJkdUVKWE54Nkt6bTd2dGFSUFoyNkgxTHh2TGVGak9ja0dFZ0xQM2g0S1lmQkZiWWtUcTVNdHhBdC1KeVRQcDA2dnpmeHRkWEnSAewBQVVfeXFMTWtYRDRSaHNULW1HanowRnpMdFF2VVMtZW1SV2ViZXlGaW02WlIwUzRZMGg5WDNrOUR4eDlGOEt5eGlqV0pfVDFhb0JEcS1faEJodWxyRnB3MkozOVJyT3NvM1I5MzdDcXNnUFNSdkRDamUzZTRQYlk0c1VIQUNMZ2ZzOWVCb2V2MC1aSTZLWkFkbW9GYk05b3RmN1htWENTeDh3SU1WYWJMcWx2eGUzZmwwVXF6czlnRGdXbE1vRElyVG0yM0ZzXzZ5TFh1YlRGNU9MQ1p3NnVZSFB0M0xBcGlueVZILXlVaXdqUkU?oc=5</t>
         </is>
       </c>
-      <c r="E35" s="17" t="inlineStr">
+      <c r="E35" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1494,7 +1497,7 @@
       <c r="F35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="17" t="inlineStr">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1504,17 +1507,17 @@
           <t>Minister leaps to fix food chain</t>
         </is>
       </c>
-      <c r="C36" s="17" t="inlineStr">
+      <c r="C36" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D36" s="17" t="inlineStr">
+      <c r="D36" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxOd2NqakVWRnQ4anFZNkl4Zy03MkloX08tUkktRTZqeEtQWFZJeVhkMUJIb0FxUjc2UjhCQ3MxbmNxczNxblJIZ09IeTBGNFM4Wkh4ZE1qNkhJMjIwU2RtX1JxcEV1Y0NjWXF6eHpVdTN4ZUlYMGIwcDJzMXZMTk94VzFlcjhpcVZVSTJFMjhsQjVGWEJQYTQ3aTFyNmNEZ1F1b3NGTWd5WnFJWmxXSTJ2NlRLcjJHNWkwaTZ2YVR6S0w5WVo1Vlg0VWdxcWZoa3VaTmcxY2NVcnR2bFRWNGNvZ1M2Tlg5NzlvVXZFZm9B0gHzAUFVX3lxTE1uNERoR3p2dXRIa0g0RXI2MWR6N0c5U3NGcjFDQVMtdEpyNDI2bk8yOS1qUnFOazdiODl0Ymo5R1pwRVJ0UFFVdzlhYjRDSUFCU0FRak4xcVVrTHphdTdxcHNIMnEyRVZud1FURmh5T0JLOHpRM3lFbDRuRnZMYmtaRnRFTXh3dkszTFhFUmZlRmoydnlEbW1fZTlmUzh4NXNyeTZTeUhOSktvclJVc0NTZTVYMkdJZEUyY2RmVC1kQ1hwVEloSEtVMEo5QnNTUXQyME5IN1BPd1NOS3oyR1JtMHBFVTZEbzhEQmdrWUk1ZnZVTQ?oc=5</t>
         </is>
       </c>
-      <c r="E36" s="17" t="inlineStr">
+      <c r="E36" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1522,7 +1525,7 @@
       <c r="F36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="17" t="inlineStr">
+      <c r="A37" s="18" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1532,17 +1535,17 @@
           <t>‘Brace for swings on every tweet’: Investors bamboozled by peace talks</t>
         </is>
       </c>
-      <c r="C37" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D37" s="17" t="inlineStr">
+      <c r="C37" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D37" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOczZHTWFmTW9FZ1ZwSnc5Z3ZacGpsVDQ3LWw1a1BFT0tjRkphek41MlhNOU84emYzZUVwNV9xM0hyc1FUR0NHck14Qnh6c2JvQks5ZE02ZTNLWDI0dy1STi1HbDFDWW9yMDhGQXVVVzdkMzFXcnNNMVZHVXFMUXUteGtsVGhPVmhLcVZPQzlhTWNoYVVRMHF0cFhybWxzek13Y3ZjcjlXWjZJM2VYbm0tTmk4NExLQzQzX1ZPMVlhcnJxQkZx?oc=5</t>
         </is>
       </c>
-      <c r="E37" s="17" t="inlineStr">
+      <c r="E37" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1550,7 +1553,7 @@
       <c r="F37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="17" t="inlineStr">
+      <c r="A38" s="18" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1560,17 +1563,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C38" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D38" s="17" t="inlineStr">
+      <c r="C38" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D38" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5</t>
         </is>
       </c>
-      <c r="E38" s="17" t="inlineStr">
+      <c r="E38" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1578,7 +1581,7 @@
       <c r="F38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="17" t="inlineStr">
+      <c r="A39" s="18" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1588,17 +1591,17 @@
           <t>Wirth’s Myer rescue mission is caught in the eye of the storm</t>
         </is>
       </c>
-      <c r="C39" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D39" s="17" t="inlineStr">
+      <c r="C39" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D39" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNTlQ4NDRnWE91VG1YNENpSTUxNnBjZkljOGdYaGV0aVB5dkVOaEJ6SjZ1bVA4NXE1S1hjV1NjcVhQTEVpWEVNV0UtbzhQTFZLOWxIenZiaF9QM3F6bmJYRy1lbXVMczZ3TnBHNy1aLUtVcnBDdkl4TE0zRGN4U0FwSjNPY1M5S3AtdUQ3UUNmR0x4MlU2YXRuUDJEUm01SmZWakx2UjFvY04zRHk4Smc?oc=5</t>
         </is>
       </c>
-      <c r="E39" s="17" t="inlineStr">
+      <c r="E39" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1606,7 +1609,7 @@
       <c r="F39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="17" t="inlineStr">
+      <c r="A40" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1616,17 +1619,17 @@
           <t>‘Darling, I’m not going anywhere’: The rise of at-home care</t>
         </is>
       </c>
-      <c r="C40" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D40" s="17" t="inlineStr">
+      <c r="C40" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D40" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQS2k0M2otaldpNVFXdHRTMVNtZVhyUDV4VTNIcE5FSnFRaHNubGNQQzBVbllnNTktNGhrZ1lndzV5V1FpUS01SklRaTZmZHJkRzVsQmlsdEVmenZ4U2x6U01NeXdIMktBUW94TUE3R3FoLUxVcVhsVFI0SjVQVUFaZldnd3prMWMyaVRWX2J4aUdfQ25KWHpaLUlqSnhvQmM2TTRRQldGbm8tclFYRDA0TVdnU2g3QQ?oc=5</t>
         </is>
       </c>
-      <c r="E40" s="17" t="inlineStr">
+      <c r="E40" s="18" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1634,7 +1637,7 @@
       <c r="F40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="17" t="inlineStr">
+      <c r="A41" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1644,17 +1647,17 @@
           <t>Iran targets Israel and Gulf states as Trump looks to calm markets</t>
         </is>
       </c>
-      <c r="C41" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D41" s="17" t="inlineStr">
+      <c r="C41" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D41" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPLXBITXU3WTRtc0NYdnhTZHFaUTBCSXdldTBuSHliTlY1dlJONW43Qkd6Nl9pNmY1eDhzaHZoX19xYjBxMXR5UEhkVUg2M2k1MmhuVEwyY0JxbnJyemxVYUZjbk5BbkN4ajhPbW9ZeDhlRDRYTW1hN3k2d084c2djMEJUZTV3NVdPbllKUmFlU2JsaDV3Zk9CVFF0VDFkV09JSloycWdOUlVrREptQTJfa25LUEx5djA2SjNMMFY0RjM?oc=5</t>
         </is>
       </c>
-      <c r="E41" s="17" t="inlineStr">
+      <c r="E41" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1662,7 +1665,7 @@
       <c r="F41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="17" t="inlineStr">
+      <c r="A42" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1672,17 +1675,17 @@
           <t>Meet Christian Louboutin, footwear’s most famous billionaire</t>
         </is>
       </c>
-      <c r="C42" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D42" s="17" t="inlineStr">
+      <c r="C42" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D42" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPcXdGd0tMckYxbjZ5TVJmQ0Q4NFl2RkhHMHdlZDZsdGZ6cVQ0cUpaLWJTNlVoc2ZOQmtXNlFTRnJVMnVDTGc1NFNZN2g1VnotQlNQbzhlM1BJV3ZwQktOcGtac3RwSHRLZkR0b2l0eGIyVVlYdHJrc2hpT0pJbDR3LURPTnowZk54LThObndtMVkwV2VWQkluNVlWY0p4QVJGbE1hSGMzOW8zdkJZOWdocEZQWFBhTllNR1ZBSEg1TWRXUWd3X0t6TVcyY05PM0pF?oc=5</t>
         </is>
       </c>
-      <c r="E42" s="17" t="inlineStr">
+      <c r="E42" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1690,7 +1693,7 @@
       <c r="F42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="17" t="inlineStr">
+      <c r="A43" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1700,17 +1703,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C43" s="17" t="inlineStr">
+      <c r="C43" s="18" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D43" s="17" t="inlineStr">
+      <c r="D43" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQbHdYM2pSM2xkdmZ3OHhQc2tVUmhzclJWaVJ0aEwtUkNBR0ZUd3p1emF1M21jbTF1ejlKSkdDMnotcVNjZE1CYUlKako3WXR4MTJhdWNlSXZMbTBYanlmTWFzRGFIandXRUQ3UjN6SEV1bThvZjN2bDY0eFdpaTdMODN6TGFTdE5rd05TUll3MmNfTDhkQldoNDIwVlpoSl85aVRwcTd5Ymh3TDl4enZhZ2p4OExGY1ZaOFNEWFBB?oc=5</t>
         </is>
       </c>
-      <c r="E43" s="17" t="inlineStr">
+      <c r="E43" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1718,7 +1721,7 @@
       <c r="F43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="17" t="inlineStr">
+      <c r="A44" s="18" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1728,17 +1731,17 @@
           <t>Sembcorp Picks Banks for $2 Billion Alinta Loan in Aussie Push</t>
         </is>
       </c>
-      <c r="C44" s="17" t="inlineStr">
+      <c r="C44" s="18" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D44" s="17" t="inlineStr">
+      <c r="D44" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOdS1aaXZjT2VnSDl2TDdzZ3NfRElDWXdUXzZQYjFQMEZJOGlpaE5CNGdQMlZ2UFVHbUtfOXF1ZVBReExrdF85M0RWLWlBY2Y5dlRtWVdXLWp0Y1VrRmF4UGQzVUhxaHA4UHd1SUdFV21QcVFITXFHRlhzekdSUS1PdHlYRjdUbUQydU8wSktKVHRJQ0NaWE9sU1l6YXhtSWtBd3RwTERacnV4VzB6YlFhUE1QcXNDVXVESFcyeWY3cGhHUkRJcDhrYUtpTEY2UQ?oc=5</t>
         </is>
       </c>
-      <c r="E44" s="17" t="inlineStr">
+      <c r="E44" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1746,7 +1749,7 @@
       <c r="F44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="17" t="inlineStr">
+      <c r="A45" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1756,17 +1759,17 @@
           <t>Navis targets June for $1bn-plus med-tech auction</t>
         </is>
       </c>
-      <c r="C45" s="17" t="inlineStr">
+      <c r="C45" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D45" s="17" t="inlineStr">
+      <c r="D45" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxPNHRXaU5tNUVkd2MtcTg5M0EyQllrM0owMkZobGxLaUJxYUN2MUg0ZkdKdzU2YmxfanR3QU53cHZzNDI1WXgzRUcxOE9EZlluNmtNRUUzTGJPRnpfVVVOeFM3bFRNQmp6VHFBdi1mTnU4UDBvOEpMaHZPNXFtdUIyTlhuRExIVElSeVRUMGxjU0k5VnVxaWFfd3htWngydlhuR2E5aTQ5VW1LS01ac05rMGZoVFdOZzVyTzFhUDVsYkNrc0VQZmhubERSaTNwelk3WEhYUjF5d2ptMktYeEhzOHpWazFQZXphd0xfUFdhbkVGMVR2Z1dtVtIB_gFBVV95cUxObEwzeHd6RmZtNUp2dXVVV0plOVQ4WlNqQXNJU0thd1BEWE8yWkxxVTZjTkpsVGxxWGxpQzN0OERZbk91ai1fZkdtc0JoM1h5NERLTVdDbVJ4Y2k4djdQcWlVcDF6NjMyVDQzZWMzUFZxWjVRWllMZHVSOF9jQ2U1REFfNUlhM2EwYloxb1MwSTJjODdWdlZwX2h2N0xiQWNhallHUTNPZEtLaXhsY3dBZy0xM1VITXhLUERXS1JxR0R3OUpBTVBPZ2dPZTRUTVpvbFBNMjFUSTJuWS1XLWdhUS11UTRzVTVqaEhfMDhqWHlTMlJGekU2QzJVcFdodw?oc=5</t>
         </is>
       </c>
-      <c r="E45" s="17" t="inlineStr">
+      <c r="E45" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1774,7 +1777,7 @@
       <c r="F45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="17" t="inlineStr">
+      <c r="A46" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1784,17 +1787,17 @@
           <t>ExxonMobil eyes New Zealand market exit</t>
         </is>
       </c>
-      <c r="C46" s="17" t="inlineStr">
+      <c r="C46" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D46" s="17" t="inlineStr">
+      <c r="D46" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxPanlvR1V1eVVpdmYxNVNGMnd6UjJFd0J6Zk9IU1lhOW1GbmVTcjY4QkJCYkl3Y3NOU25VRTBUekwtS3plV0NVdlZtOTZZRHJWZ0FVdDl3S05aMlFWeEZiYzdwYmQtVnJxZEw0NktHaFZMNlZkUC16empqRGxxMEhhZGwxRzVEek5FelB3aE9UWFhGQW42b21MRnJHUXV2ZGJYUXJIMnVFWGZsSnEwazNGNUdVcjVoekp0NEZCN1J3cTlaZldFa1pMUkJTbVZYeFljVkRqQmlZV1M2aXh0ZjI5dEI1NDB0UElPUERsbUljMlA3OHBnYmtJTXFWZWkyUdIBgwJBVV95cUxNWFBRQ05GUDdwTWJ2ZVFJUS00ZUh0QkpZQVNNcU9JYXRTN21sMS1VZTlOSTh2LVFuZHh6UVk2djlrdWFsd3MwcDFCNmhwUlVLTlpjVF8wSmt1YnBWRE9tNVpKQlk2YXJWdmwzZWlLX0xpaWxSMUpsX3ZjYXhmRmE2YlAtSFJGRG5pQnVmMnViQXlsVFV3OU1hZFVrY3ZITHQxcTR5UkZ5U1pReHVJMGZGM2FCZWliSFZQZmpVLThSdExWMW14OElodmVVSC05SUh1d1hBenJoY3BUZGxoM0NTbTExdERmM3pjZGd4VzgyV3BNOG11TElBQ3NsRGhtSEc3YzJz?oc=5</t>
         </is>
       </c>
-      <c r="E46" s="17" t="inlineStr">
+      <c r="E46" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1802,7 +1805,7 @@
       <c r="F46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="17" t="inlineStr">
+      <c r="A47" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1812,17 +1815,17 @@
           <t>PAC Capital’s Clayton Larcombe charged with assaulting wife</t>
         </is>
       </c>
-      <c r="C47" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D47" s="17" t="inlineStr">
+      <c r="C47" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D47" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOLXNDU2xjMWpyeEZwWGwtZkV0TjNSbGtWS3ZidUo3a0dvV1hrTnJiVXBXSkJNWlhXYXFHZkNTa3g4a1ZfMjRPM3BtWTZUNGg3S09kbGI2TTRGd0Jkc1A4WFAycjlpVC1URjFvNnBraWprRkhaT0VOWkh6N0xkUjNXNUw0dGx2N1JtTDVsREdtZDhraXVsSkxhR2ozamFUSGR5VHBBRm1Zcmx1c2RDaUIxQkVpeUpfWjFNeTRLWVRtYjluZ3ZncGZIMQ?oc=5</t>
         </is>
       </c>
-      <c r="E47" s="17" t="inlineStr">
+      <c r="E47" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1830,7 +1833,7 @@
       <c r="F47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="17" t="inlineStr">
+      <c r="A48" s="18" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1840,17 +1843,17 @@
           <t>China touts itself as ‘harbour of stability’ to global CEOs</t>
         </is>
       </c>
-      <c r="C48" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D48" s="17" t="inlineStr">
+      <c r="C48" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D48" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPUzBWeVk0elBOZ0l5QU44TUJvU0RvSmtPdmVyT2VuQTczaEdzbkktT25ZT2Y0Nzh0bVBhQW96TUhpWkdEOEJMVVk2UWxLOENKZGk3X2tQcDNsWGZtU0JkM2U0N3VfUWFBclhUSUZya0NwRTJOWmZJdWlhT3JtY1EtSkJ6TmlsV3dzOXpDaVFMNlBaa3RfRHBjc3Q0cjk0eVdPV2MwcjlHNA?oc=5</t>
         </is>
       </c>
-      <c r="E48" s="17" t="inlineStr">
+      <c r="E48" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1858,7 +1861,7 @@
       <c r="F48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="17" t="inlineStr">
+      <c r="A49" s="18" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1868,17 +1871,17 @@
           <t>Eyes on 3D Energi as oil and gas giant Conoco flexes buy-out rights</t>
         </is>
       </c>
-      <c r="C49" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D49" s="17" t="inlineStr">
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D49" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWVU1QmhTUGFkYlpTQkw1WUFPTHhmbk5lbnE4T1haQUswSi1ITHlhVmhyM3ZYS3N4cVd6ZkwzdGdhT1lvM1JJek4yLXFpSWoxUnRtR2JRLTZWa2dlTDVTakE3b2xvazFWX0kzRHFZWVB4OUh0XzFFd3JVSVlfelpVa21qTldCVHdvcmJYcGNjZ1RrdElWS3Yzck9KYzRvbzloWkNqMnQ3dmtHbzNuc21ZSXNYeEFlZw?oc=5</t>
         </is>
       </c>
-      <c r="E49" s="17" t="inlineStr">
+      <c r="E49" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1886,7 +1889,7 @@
       <c r="F49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="17" t="inlineStr">
+      <c r="A50" s="18" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1896,17 +1899,17 @@
           <t>Blackstone tempted by $900m payday for Sydney’s JPMorgan tower</t>
         </is>
       </c>
-      <c r="C50" s="17" t="inlineStr">
+      <c r="C50" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D50" s="17" t="inlineStr">
+      <c r="D50" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxQNEZTZjY0S2YzcUxsb25RSDk2NHd1N1VOVlpMbi1JNGEzbUt5ajlYZFhvLWNBTkNQVXNuWERfTkl0Z2o4R1U0Zk5jVE1FTW5TTUJGZnNJc2NqMm1fT2dmYTVwRGU2TkZ0c3BjZVBGS29fWFJvZ2F0MWNLa0pYY0RNME5xYS1vOGZmMDVBcDBaLV9MWF9od0EwekFyb0ZCOEdkNTFaN3ZXckJwd25zS0FsdzU4OW1UODlueGNyZVBDSDZkeHQwelV5ZXVDVlcyUkhKWDZfVlRacEJHSElmNnhKSXk4ZHJHWHhPTEV5NGNkcmhyU0hjV3J4dVBXbnRGQdIBgwJBVV95cUxPME4ySFF5RWNrejVlWW1yeW56N244RGpyeVJUZEgyTjFNcE10YjVpMmJyeWsxTENzZFhPRlpsbl9pVXl0NGJvUlZFT216NE1KRFNwOHVZVXMzanNKNXFmWEdsMndsd1cza3NTTzUyUUZfaDEyWHJwZEtQbTdJRmkyU3A0RGh4QlAtT1lRVXk2SGoyaTI1NUpwVExYSkZJNmVFNjdXTDJTNURFOEh4Y1dnUDVGdjBpaDlWVWJtUHZiRDdGTmE5R1R6TDBwWFFnT2MwQ1lmT2w5bDF6eVU0R20tYnpnT3JCZlJod2s0UndyZTM5M2xLZC02a3E0NmJRdFV0Qkow?oc=5</t>
         </is>
       </c>
-      <c r="E50" s="17" t="inlineStr">
+      <c r="E50" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1914,7 +1917,7 @@
       <c r="F50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="17" t="inlineStr">
+      <c r="A51" s="18" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1924,17 +1927,17 @@
           <t>I-MED attracts mystery suitor as Permira weighs sale or IPO</t>
         </is>
       </c>
-      <c r="C51" s="17" t="inlineStr">
+      <c r="C51" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D51" s="17" t="inlineStr">
+      <c r="D51" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxNaGlwS3d5MGFMbEg2U2hnZUxMQmdqaWI4bS1lblNZOFhkSnRMcUotRkZMTjhFZkRUQWxUUDVtYml6TVAxUXkyZmx3SHRFb0gzVHRST2ZQUThKa25aWlhlcGprSU9tWktXZjZRaC12bFpkaVVWZHhIMERyeVNNWEswYTJ2ZHdnRFVRaFhod2U5N011TkQ0NG5MYVhoT3MwRUVZdVB2UVhKZExvdFIyXzNNUGt2SHJUanQxRkI3bXlLSlNJQTF4NXQ1YlZDaGVBM0EzNUhYQVp6NkFWRzU4bnRPWTgtXy1HVnB0ZlN0Uy1rY2FuWlNfN1U4WXVHQnRzVkNG0gGGAkFVX3lxTE1GaDJJdTJlOXFEZUtDTmdXMmsyLXlpaUxzQXpycHk4MTdHZng0dVczYWVwdWRzdFFCMlNLWkZpMm5Zd2RpN0Y0Zmo3Q1FOZFBZQlh5LVl6aVZ3X284UmpxM0pVRzZmMmpjaUdNWnJPZGV4V3lNai1CTllCcW5oUEVxaG0zejB5anc5YnJEZzZPT2d2QklCWjl2MjRBc25jUndqZkVadllKaUZScG12bEozT1NKUUJYR0pHTGtJZVc0ZHZLNHVSYlhzcTE0SkZmMXNlVGJ4YWJ1cThxcGlZTDMzRUMxLVM5VHh2OW5tRW1PT3VyRUhDbV8tRzUzVzRzVWZPZ2w1bnc?oc=5</t>
         </is>
       </c>
-      <c r="E51" s="17" t="inlineStr">
+      <c r="E51" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1942,7 +1945,7 @@
       <c r="F51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="17" t="inlineStr">
+      <c r="A52" s="18" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1952,17 +1955,17 @@
           <t>The stagflationary mix that has billionaire Solomon Lew worried</t>
         </is>
       </c>
-      <c r="C52" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D52" s="17" t="inlineStr">
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D52" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPWTh3S05XQWpTQm03WjhBT1pWc2cyOFRMd2ZraHhPUHlDRW1tWkZvdkhQWHE0MHVMRUpaOFRoX0JsYWhJV21nVkpIM2RBSmlZRUtEbFAydzZfOTh1S05oNEZPOGgyZDJRMS1uLThWYWRVT3VEVGhtYkVLN3J2OWsyX0VVdTUteFBCOVNKZ28xUTRPTk1SUkMxZ1NJc1B6NXRrUEEzOG01YnZOYjk2cWlFZA?oc=5</t>
         </is>
       </c>
-      <c r="E52" s="17" t="inlineStr">
+      <c r="E52" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1970,7 +1973,7 @@
       <c r="F52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="17" t="inlineStr">
+      <c r="A53" s="18" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1980,17 +1983,17 @@
           <t>Oliver Curtis on Firmus: From prison barber to AI billionaire</t>
         </is>
       </c>
-      <c r="C53" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D53" s="17" t="inlineStr">
+      <c r="C53" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D53" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQek9VTlV1b2hVb2RoZ0Fya0REb3E3YlBCR2NYZldXcEh2VEY0LXg5bjd6RzlnZDI0OUJJd2cydTBwTm9tdHpiZ1lSMnhtcmJSYVRKbzJFMjdDaEJyZExSQVJVRDh1c00yMjFMaVlPdnRuV3VkTjNxdzFRbW1yeGltSF8tVXlJVXJzTEJXS2FTYkJTVkdKbmdPTTd6YzRtYV9nN0JzOVZNTzhUdUk?oc=5</t>
         </is>
       </c>
-      <c r="E53" s="17" t="inlineStr">
+      <c r="E53" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1998,7 +2001,7 @@
       <c r="F53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="17" t="inlineStr">
+      <c r="A54" s="18" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2008,17 +2011,17 @@
           <t>Three startups that raised $161 million this week</t>
         </is>
       </c>
-      <c r="C54" s="17" t="inlineStr">
+      <c r="C54" s="18" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D54" s="17" t="inlineStr">
+      <c r="D54" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNRGVZMF9DeGJjX29vN3B0blVoM3RKSlJJTllrMThKUDJNZzdPNFNnT2JyTElUOUYxMHlsUm9yM2dBQnZfaVNZblpqb3NzTXdHVlpQNkRqR3NBZHdzODdjN3RKMTZhSVRqUEM5d3JRc3F2OG9hWmZJdU5rakg4ck8wLXlMTnZSU0lNaERmQmswbkVGWW8?oc=5</t>
         </is>
       </c>
-      <c r="E54" s="17" t="inlineStr">
+      <c r="E54" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2026,7 +2029,7 @@
       <c r="F54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="17" t="inlineStr">
+      <c r="A55" s="18" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2036,17 +2039,17 @@
           <t>Iran eyes ‘plenty more’ vulnerable energy targets in costly war</t>
         </is>
       </c>
-      <c r="C55" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D55" s="17" t="inlineStr">
+      <c r="C55" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D55" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNLUN1MHlZaTNfVHhVX0RnTXp5QW83RmM4WVZkWW1PSnNaZF93VkY5ZF81anB3NDNmX0kyMkVSdkxNSURvSEh6enloWnRVcTlsR0JPTjVzNFR1YjRsSm52VnA1XzFFUlUtODJjYy15YWRRdWZZRkdjRXpCcEFSVURmV3VpSTFhTjVUb1d5bmw3NHNlT3VQZU9ieEYwM1J1TGEyZnlnWXNIWFJUMEtIOVZad0dxRWZBdw?oc=5</t>
         </is>
       </c>
-      <c r="E55" s="17" t="inlineStr">
+      <c r="E55" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2054,7 +2057,7 @@
       <c r="F55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="17" t="inlineStr">
+      <c r="A56" s="18" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2064,17 +2067,17 @@
           <t>Don’t take it personally: Bain Special Sits hits hurdle at Infinity</t>
         </is>
       </c>
-      <c r="C56" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D56" s="17" t="inlineStr">
+      <c r="C56" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D56" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQRjdwTk0xTHVIRHNkdG9tVk1EQ0hiQjJ6dGcxaWZRZ0hZV1U4YjJDU0tnTUlWSkQ1S2dUTHJVNk0tNWQ2cVd4dkw0M25leXRreWJtdlBKYTAtNzRocTJUazh1dnRzSVlYZThySTBNVjg5X0xYWUxCMC1SelltSHVSUEV5U3B1bTA2NjAzMGFZLW1CNkQ3aWU0S1JxS0d0YmZiZjBKQVRNVUpzYno5R1pvbTBsaTM?oc=5</t>
         </is>
       </c>
-      <c r="E56" s="17" t="inlineStr">
+      <c r="E56" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2082,7 +2085,7 @@
       <c r="F56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="17" t="inlineStr">
+      <c r="A57" s="18" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2092,17 +2095,17 @@
           <t>Drill, baby, drill: It’s boom time for mineral and petroleum explorers</t>
         </is>
       </c>
-      <c r="C57" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D57" s="17" t="inlineStr">
+      <c r="C57" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D57" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNdlFOWld5ZWhPVnFRa2xidWlUVzluQzkxUTgxR0t0Rmg2S1BzNjdINnhwS3VLRkNjRVJLX0RHU0h4VFVRY2RfSHBudEhfNVNjeE50ZUxQenJNSlJtWFRlcnNsZm1iLXlxM2RmVDViWEtjNDloaTBhUDVxYkNfOWFCTjV6cExEVlFCMzNfWnVwRDJHYWxWV0hOR2V2S0VlV2NyS2s5cWNmREtWXzlMMDRQNW1tVlBOblp3SHBEVg?oc=5</t>
         </is>
       </c>
-      <c r="E57" s="17" t="inlineStr">
+      <c r="E57" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2110,7 +2113,7 @@
       <c r="F57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="17" t="inlineStr">
+      <c r="A58" s="18" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2120,17 +2123,17 @@
           <t>‘Wake up’: Fury as farming crisis looms</t>
         </is>
       </c>
-      <c r="C58" s="17" t="inlineStr">
+      <c r="C58" s="18" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D58" s="17" t="inlineStr">
+      <c r="D58" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNelJvMXFPX3MwUVRMN2xqbzE1MWdvOF92Zy02YmIyZW9SQXRNQVZsS0xVVG9UdkFPaTV6ZC1tV05SZWNqblNFZ3Y1VGNaVVBaaEl6aFJqQ09ONDVkNUs4TzNvVjV5eHNjUk9xaDRFZTM0alpuYUdvWGtLRzRhYXN5alZ1QWdsZTEyODdQVnZoazkya29WeTJZVmpxLVBCdWxfY0dTN2Z3WFZlSy1sVW44RDlvZFAzYlhnQ0N6UWhKSU02eF9iZllIU3g5MWtSbkJzZGxWLUxHNERzdUlLTF9VYmpJSTRLY3U4NlVVaDhmc09uOWwtUGtlb0I2M05DR1dnRWxGSFV2NEJXaEF4c00tN9IBlgJBVV95cUxOSzZ5NXZMTTlZa3BSNjZyTUxUMjRhYWJhN0hMa3dDcW9CWGstNnI5MzV5U0hJSTdKLTFwa2E5YUItZnFRbW5RbzVuYW91MmZaYXN3R25hWVpUbW9oUU9fVktPRHROVDYyd2dSLXJVZWQtY016bkVxY0VPbkY3Zkgtb1liWGMxeEpyYmloS1V0TVJMMWZaeWRZX3FQRjBmVzJwdkkwMEVDSXV1MTdReUhGZ0Z3dENyMEFkLUl1aXhtRkFLRFFXcEdMZzFuT3NxRDFMOGVaY2YzeXBQc09fY3YwcFp4MVczRVN3d3dJZWJfTFFscjF0cUtRWHdzTUptaHowNDhYWXZXTHhYTHNTdlZGUmNlamRTdw?oc=5</t>
         </is>
       </c>
-      <c r="E58" s="17" t="inlineStr">
+      <c r="E58" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2138,7 +2141,7 @@
       <c r="F58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="17" t="inlineStr">
+      <c r="A59" s="18" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2148,17 +2151,17 @@
           <t>Construction giant FDC road tests IPO pitch</t>
         </is>
       </c>
-      <c r="C59" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D59" s="17" t="inlineStr">
+      <c r="C59" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D59" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxON3p5Y3VPM01XZFk4a3g0R3JnQkZXbHVGV3BKdDB6M3NRb0M0SEl3V0R5RmhCQ3dnaHB0ZHp5N2hCMUFsNU1ZNWZ4YWdNZWdETkUyZmdoeW81amwtTWNFZlc5WlNpMkJwRzk0QklORGhlLWNEalh2d0JCX0lhVHhhUF9ibVlxcHAwOW9ENndVOTY0enBYUWc?oc=5</t>
         </is>
       </c>
-      <c r="E59" s="17" t="inlineStr">
+      <c r="E59" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2166,7 +2169,7 @@
       <c r="F59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="17" t="inlineStr">
+      <c r="A60" s="18" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2176,17 +2179,17 @@
           <t>Austal suitor Arlington Capital Partners buys Eptec’s defence unit</t>
         </is>
       </c>
-      <c r="C60" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D60" s="17" t="inlineStr">
+      <c r="C60" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D60" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNM01qb1ZRZVBIdmp3cFc3R3RLaTdmZk1JOFo4anRtSm95Z1hJc0N0S3VranBTV29IdlViT0FkSm92eHdtbDBqdU5HTHNMaXo0dGRWMkpDdjk3LVRBVU1rZC1YejZJMkhyNmpZZFJodGoxWlB1dkRhYTJVRlljMlV0dUllQ3EtOHZkNFdSUWJLSW9Xemw1XzFzU2RHV1o0RTViOXp0bDZFQTZycWhpNElLU0FZQVI?oc=5</t>
         </is>
       </c>
-      <c r="E60" s="17" t="inlineStr">
+      <c r="E60" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2194,7 +2197,7 @@
       <c r="F60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="17" t="inlineStr">
+      <c r="A61" s="18" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2204,17 +2207,17 @@
           <t>Eyes on Tom Wallace as clock ticks on Adgemis pub deal</t>
         </is>
       </c>
-      <c r="C61" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D61" s="17" t="inlineStr">
+      <c r="C61" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D61" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxNSExQeDlENWlHb0prRnRldjZ5YWhKVUZ5eVdsYjZmbVRWRWQ0WnZXWkU3UHZJdElnQ21jMU9zNnhnc3JlNDczVGQ5Y0FGV2J3QUp3NXdZTXZMNm5tVC1vWDFtOFN3aS04QVJZb3FZV2VsUmJ2aVgwbUhTaFVGdHg0UjRyTXVVUnFhQmE5eFYwMGR6T1R2U3Q3WEdZclVKNWJiby1IRg?oc=5</t>
         </is>
       </c>
-      <c r="E61" s="17" t="inlineStr">
+      <c r="E61" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2222,7 +2225,7 @@
       <c r="F61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="17" t="inlineStr">
+      <c r="A62" s="18" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2232,17 +2235,17 @@
           <t>UBS names head of APAC leveraged capital markets</t>
         </is>
       </c>
-      <c r="C62" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D62" s="17" t="inlineStr">
+      <c r="C62" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D62" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNMm9WZ2ZKVFBvX2pYMk16VmY1WFZnZ2J5N0F2bHduTVM0Sjg4STVtTGFLQVdzeFloVHg3clRic0owTDMwYVpXdDVjdjFOWjQxdkdxdFY5MEY1Q1U2Q0R5dFBJWTNtUzgyd3RXcm9uM0hKdEZ3b3JjXzcwQ2VpRm5SS0hYT2gxSU9iVFRlR05Xd2EtM2JOQjBGUzlKdnE?oc=5</t>
         </is>
       </c>
-      <c r="E62" s="17" t="inlineStr">
+      <c r="E62" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2250,7 +2253,7 @@
       <c r="F62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="17" t="inlineStr">
+      <c r="A63" s="18" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2260,17 +2263,17 @@
           <t>BHP, Woodside rise after new CEOs named; Future Fund chiefs exit; Sandilands ‘doesn’t accept’ termination</t>
         </is>
       </c>
-      <c r="C63" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D63" s="17" t="inlineStr">
+      <c r="C63" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D63" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNUHhZeHNHemtiLW1IOHN1OTZXOGpsM0ZtUG1MVHRCT1hUT1k5S2lEOXlXRENWOXNlMEZadThQR18xSTJfTVlQM3BtX0ptX1J0bk80SzNLUVRtbkJITGgtb0lsSVdJTWt2S1E1WUlXdUdsbEV0V1RpNWlyRXBoc0dPVDl1OXRrSlM3SHlDazg2UlcxenVzNzlhQldhUGhfNE5IV2xrVmVBNzhhSE9qY042Z3pzMEVzd0VyVmZudXgxcTgwWGJXSWZKZ0FyNVhjcmhjTm5DYUVjLUdDRmxUQkZuTDFlUXVaV0ZoSWp5WHMyR3c?oc=5</t>
         </is>
       </c>
-      <c r="E63" s="17" t="inlineStr">
+      <c r="E63" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2278,7 +2281,7 @@
       <c r="F63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="17" t="inlineStr">
+      <c r="A64" s="18" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2288,17 +2291,17 @@
           <t>BHP’s new CEO will shift the Big Australian’s centre of gravity</t>
         </is>
       </c>
-      <c r="C64" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D64" s="17" t="inlineStr">
+      <c r="C64" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D64" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPQnZpWndNZzZvN1VsOHBmRDVLRHVTNkxLeDVDelpOMURjOTRDSDZfN2dPZlZqaW05WEZuZXMyRTJZeVZnV0poT2UxRkVfZ1RZSjdvUjVKblhoSU5Cd1plRTVNNTRaNWZmbm1yUGZkblVpYkctNzVRRkVQQm4zX1FtRG1KV2Y0djUtOURianJ3dElqeXBUMFp4aWFEWVFYelVjYTluSWpOM1FlbHpIaUxXdnBn?oc=5</t>
         </is>
       </c>
-      <c r="E64" s="17" t="inlineStr">
+      <c r="E64" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2306,7 +2309,7 @@
       <c r="F64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="17" t="inlineStr">
+      <c r="A65" s="18" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2316,17 +2319,17 @@
           <t>How philanthropy became the sandbox of succession</t>
         </is>
       </c>
-      <c r="C65" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D65" s="17" t="inlineStr">
+      <c r="C65" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D65" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxObnBPb2MzQ1RvSVVCbmNzYWFBMlFjU0dQRmpPakNfdkxtMWc1bFdVNXNlZmRKQnNlWEtUUDNSTHpTLVV4Skx0V2otbTZsTTdvT1VaUDhMZFZoMFFab1RoS2pCcno1WGlNQlY4eXQ0OFEtLXJTay1MUkFSSEJ2MVVScUpjUkhJOThISy1QbHIzTzFlWVhOc29fWWs0V19sQ25hRW9MSGhBVVNKWUp6dUo3NS1SWlk?oc=5</t>
         </is>
       </c>
-      <c r="E65" s="17" t="inlineStr">
+      <c r="E65" s="18" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2334,7 +2337,7 @@
       <c r="F65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="17" t="inlineStr">
+      <c r="A66" s="18" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2344,17 +2347,17 @@
           <t>Advanced Navigation raises $158 million Series C round with NRFC backing</t>
         </is>
       </c>
-      <c r="C66" s="17" t="inlineStr">
+      <c r="C66" s="18" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D66" s="17" t="inlineStr">
+      <c r="D66" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNTXhwVlVLUy1pWEpFdzFCazNTY0dkczd4WW9oeW14cUtTaDZRTGlVQXBPaHN4WTBkNW1zOGxvN0tVWl9JSFdVNXlQMzVxbk4zbDZFUjNOcUxSamNaSnFCckMzWEk1VlNoSHJHQ3VWdGltVWZCV0c0NmU4UlN6YU55Q0J2TkQtUzBzOW96UXRxem5Zb3M2SUljNURISlRkQmJD?oc=5</t>
         </is>
       </c>
-      <c r="E66" s="17" t="inlineStr">
+      <c r="E66" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2362,7 +2365,7 @@
       <c r="F66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="17" t="inlineStr">
+      <c r="A67" s="18" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2372,17 +2375,17 @@
           <t>Kal Somani-led consortium buys Rajasthan Royals for USD 1.63 billion</t>
         </is>
       </c>
-      <c r="C67" s="17" t="inlineStr">
+      <c r="C67" s="18" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D67" s="17" t="inlineStr">
+      <c r="D67" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOX3lmdG5aTmk4TEpBa3ROdWZ1aDJHUElBQXktVmlKaHFmTUhPX1QxX1dKLXZfaHRDQjBnWm9McTZjTjJtTWFETTRNMHgzN0tTTm1xY0JpMF84Q2lNaFQyZGVjaHN4bkVmcDN5Qy1ta3FtYnpMSVVyYm0ydWpTRUdZU1hoYXpaNkZUQzlPc1QycjZ6aG5QVHRqY213?oc=5</t>
         </is>
       </c>
-      <c r="E67" s="17" t="inlineStr">
+      <c r="E67" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2390,7 +2393,7 @@
       <c r="F67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="17" t="inlineStr">
+      <c r="A68" s="18" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2400,17 +2403,17 @@
           <t>KMD says Rip Curl demerger proposal delivers investors ‘no value’</t>
         </is>
       </c>
-      <c r="C68" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D68" s="17" t="inlineStr">
+      <c r="C68" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D68" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPTXhBdHByWE9EbllFdDA2OW1UTUZEMVJfV2xsNFdURFRKX2JrODJReVRuQlFoakpWbTBKcjhNLUVsNE9sdG5LUElLZlVrbFNERS1QZTN6bEZIWEhXZ1pTWG5GWEw3ZmNETTdDUDUzYzR5M0E3ZGVlTWpSUnVlVU56dDNFZUtZN3liZ1dKNzJhLWU1S0M1ZnlKd1JNWXlxSlkyU3pGS1lhS05hTUJPRkxucldabzFucGs?oc=5</t>
         </is>
       </c>
-      <c r="E68" s="17" t="inlineStr">
+      <c r="E68" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2418,7 +2421,7 @@
       <c r="F68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="17" t="inlineStr">
+      <c r="A69" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2428,17 +2431,17 @@
           <t>Ex-Macquarie banker drives mortgage broker roll-up Recludo towards IPO</t>
         </is>
       </c>
-      <c r="C69" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D69" s="17" t="inlineStr">
+      <c r="C69" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D69" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxNQms5X1F2aTNhOExDbW42TlZOLVJwVWxna1JYSW9vWF9Na1RZa1ViTFdZc0tCcXRZZkRudTlsTzNuZGgwSENyYi03Zjdfc0lZTXp0NmJRZnhzb2pWRXRIOUdJN2lQM2h3ZFFtTXlSWHVWOFBIaW1Na3FQMjBCck1nVlhUcmRkLW9LOHpKWXQwTm9LcWR5M2FfdjFiRW04TndoanR5NmJvMENGalNuUGNINy1Qc20xR1J4d21ncHNNSUZqa1BXNnI4STIxSUFkZXdU?oc=5</t>
         </is>
       </c>
-      <c r="E69" s="17" t="inlineStr">
+      <c r="E69" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2446,7 +2449,7 @@
       <c r="F69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="17" t="inlineStr">
+      <c r="A70" s="18" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2456,17 +2459,17 @@
           <t>Coles reviews truck fuel charges as crisis worsens</t>
         </is>
       </c>
-      <c r="C70" s="17" t="inlineStr">
+      <c r="C70" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D70" s="17" t="inlineStr">
+      <c r="D70" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxOSGpBM3RjLVJ3LVlmR1QydnY2dm50WlVxcG43ajRFZ25QS1hDNTBONU8tY3Z2TklzbUNla0ttZk1GZzFaLUZRakFjSUpUQWItQ0VqVTVwS1B0QS1ObVEzNzdRT1l6aU9pVm5jSlhna1N6QmFKT3k1RkhMZGNTVnVLcDVIcXZmRjdjLWRpYVlRQUVmcVRtM21BSjVhTGNaaThyZkhLS2NWdkNCSkZKTlloUVdtbzRnYjFKbllOZXhOd3lkcFZEYURwUFVNQzVnSWRyM1RlOGd2M1pMZXI3c0NIa0Y0MNIB6AFBVV95cUxNSjB3Z0hoTGxwOHJQQ09xb3BmRmhCYjBCc2E0OHA2elFDRE45UGpaTEVDc1Y2VnRvVmZQUzRHbng4QTMwNGZZNGpmaVlHRmV6bnhiZ0FReU50TnRiQ0NZMEtoM3dBZ0hXbFBZMVJQNXd4LVdXRDVyTDAxNS1zeVdvcFVvend2N3J5R2pLYmhxNVFfd19rUlRsNWNndlptMUVkcS1CaUN6UXRHVzByTU5BMW1TdktOZUJYck5xMEJucmR6czIySEMycDA5cmR1MXB0N25Xc0JDUG9zN29YWklVc1BUMzl3UVhn?oc=5</t>
         </is>
       </c>
-      <c r="E70" s="17" t="inlineStr">
+      <c r="E70" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2474,7 +2477,7 @@
       <c r="F70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="17" t="inlineStr">
+      <c r="A71" s="18" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2484,17 +2487,17 @@
           <t>Sam Arnaout’s Midas touch turns suburban pubs into pokie gold mines</t>
         </is>
       </c>
-      <c r="C71" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D71" s="17" t="inlineStr">
+      <c r="C71" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D71" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQV2xlTTdYOFpIMzNmVVRnMlJRbTdGTC1jelVCd1V3UjN5cHQ1VzhWZzhrNW1PNm1RX3FlZmU3UkRycjF4WDlQUzRMcVVYY1g3UTZqQ0hxRnl2Ti1IQ0owVmZjN3Jod1BFbmhPVUwxNjhsTGh6d0kzdU01N0hmempRZ044ZmZNUllnenhyc3djRGJOdEtrekx5UVFoaFFMWDdqMHMwdng1SFg4TzZHY1hQNFJNN3huZXpWYWFtQ0ZJakhkVFlQcl9SQlRfZkQ?oc=5</t>
         </is>
       </c>
-      <c r="E71" s="17" t="inlineStr">
+      <c r="E71" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2502,7 +2505,7 @@
       <c r="F71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="17" t="inlineStr">
+      <c r="A72" s="18" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2512,17 +2515,17 @@
           <t>Gentlemen at Melbourne’s exclusive The Australian Club sweat another election</t>
         </is>
       </c>
-      <c r="C72" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D72" s="17" t="inlineStr">
+      <c r="C72" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D72" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPcEwyU01BOXF4TzlmREhYbTFEWklxdWZqWmZybDVnOWtLQ2dTU2dNQ2t5M3BVT2stN08xYkFmazVkY29oT3RVc2xUZmZINFJURGtIRTg4RGsxOURBdWEybTUwU2NUODQ2eDNBbTdPT3QxeXRFNHlSc014T0g1aG4xZ1A0U0FWMTB1Wm1CSHlQU0ZJb3lMYkE?oc=5</t>
         </is>
       </c>
-      <c r="E72" s="17" t="inlineStr">
+      <c r="E72" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2530,7 +2533,7 @@
       <c r="F72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="17" t="inlineStr">
+      <c r="A73" s="18" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2540,17 +2543,17 @@
           <t>Inside Fortescue’s AI ‘hive’ that could save the mining giant billions</t>
         </is>
       </c>
-      <c r="C73" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D73" s="17" t="inlineStr">
+      <c r="C73" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D73" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOSVVCbGpzcVcxTGlZZ2dTUkxXdVVvVU1ONEtUS0t1R1VkWWRNeUF1UmlHbXd6clR3QVRuWGxrUGQwVG1OeUxZb2RqTzdYOEVGQ1N6eDFta3VOZDdHNThYbUEwWEVHZlZBVzNpZ1Foak1kLURZTWpJVzZLekczdzFrdHMtLVZwMUZnYmkxSVc0czFqWnFaSGZiT2pIVW5rdVZmdThreFlRZWVEU0xoa1VFOV9MTjE2UHFOcWhqUzVB?oc=5</t>
         </is>
       </c>
-      <c r="E73" s="17" t="inlineStr">
+      <c r="E73" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2558,7 +2561,7 @@
       <c r="F73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="17" t="inlineStr">
+      <c r="A74" s="18" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2568,17 +2571,17 @@
           <t>Tiny house maker Elsewhere Pods seeks cash after Bunnings debut</t>
         </is>
       </c>
-      <c r="C74" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D74" s="17" t="inlineStr">
+      <c r="C74" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D74" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM0ZpVnBTS21Ib25qa09CaU52Z29kZWhTU0FJLW5VR2JCLVFPTVlZTmpYX3lZVWdtMDVTYTJkWHlPUmhXa0Rua2ZXTTBWQU1VdmFrV21KOGlrdjJ3TTdxbGlvZVBUZUxUWE1uelpWMGxWWk04UndJTXVKQjBZUEtoX3lodmdpMWZKNUc1YTIxVFZLYkFKT1QwbS01WU01ZUZTTlczY2ZpLXlpTjNJTWpsUg?oc=5</t>
         </is>
       </c>
-      <c r="E74" s="17" t="inlineStr">
+      <c r="E74" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2586,7 +2589,7 @@
       <c r="F74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="17" t="inlineStr">
+      <c r="A75" s="18" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2596,17 +2599,17 @@
           <t>Chinese consortium emerges as dark horse in Made Group sale</t>
         </is>
       </c>
-      <c r="C75" s="17" t="inlineStr">
+      <c r="C75" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D75" s="17" t="inlineStr">
+      <c r="D75" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQYlpEY0hxNm5lalIxSTUzbDE4UEF5QTNpMTl4dWNPMkRrMU1yQnltZ25WcUkwOU13V2Y2RGItVW5QTXotSnBZRUJMdGJySGw0NVVxc3ZLZmVEcTlfU193Vkd5UVVuTFVYWFNtd185eGlVQW5RRElHdk5pMjhUR24wd1k0T0I3cW9qTG5Lcjg2bV9aNWsya0FYODRjeURyMW1EeHdYT05iZHZhLVFrUVNoV25idnZYZ2lpZEhta2JxOWFJb0M2SE9hbFF6NlVWYTM3QmF5anpWOEZackZiTDBfN2gtX1luQkxFOUxSSNIB8gFBVV95cUxOQklMYWl1ZkRqZGUwN0ppeXFubzZWNTNmeE5GY1BfcS13N2dFT096YW9JSndVX1EzTlBKdWZIemdKZnRIME9SQk5aT1M2WnRESjJxckFTaUdOSEd6eG9hRVBjdlhBbWQyWGpUS1kwQXJsdlpkLXJpXzJZX2xiUC1FSlNnNTFoVXQ4bF9JeUp3UGRWdUFOUVRrNUtsRzRxaUczb1p2LVVucFBNazhuZFNDaUZDR2ZQUVdObmVtTnBndGlkazZqeHVheVNzSE9RY3Bad0lrckxDSWY5QXBWS0hwVzZvSTZjaGEtNkNncW1RRE5uUQ?oc=5</t>
         </is>
       </c>
-      <c r="E75" s="17" t="inlineStr">
+      <c r="E75" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2614,7 +2617,7 @@
       <c r="F75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="17" t="inlineStr">
+      <c r="A76" s="18" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2624,17 +2627,17 @@
           <t>KMD faces uphill battle in capital raise as key shareholder baulks</t>
         </is>
       </c>
-      <c r="C76" s="17" t="inlineStr">
+      <c r="C76" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D76" s="17" t="inlineStr">
+      <c r="D76" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxOVTU0OGNfRURNcDdzYUtIcG8tR3N4OFFYalhKNWJBaUd6ZlQwNU5MZVZYbUZVSzB3WmdOOFdTZHlBOXBzSGdYUVV6eGt1UndHN296bENxZzNUM2NoaV93LXZaZFNNOXJ2YlA4RHNFS2FDb1ltNWpPWUdRR3VGMWoxaU5qYm9VSW9yUW5kS1NaN2RSc2YtcHZRSTB6aE9Zdkl3NG5nbVRzODRfQVYtelo5M3g4R2JEbnpraFpWbENOZzE2Qndla2t3MXRPWkU1dXg4NmZRME1jT3pOOHZOVlpTZGloNENUZllaSTFmWUV1Y2JLck02ZDhnTHJ5bUPSAYICQVVfeXFMUEFXR29tQjlTbTdMRVNDWUlGNFNOQjVhX0FiSkl0U2stbml5VHR4d1g3bDFqMUw2TzR1eHhYOU5ZUmJpZ2xBY2NzcmJRX3MwaEQ0YmpzMUFnV1BQNGxmcnlXUzVvbHpwNEo5dWFnZlduZ0Z2dGZGRFRKRTNCUzctZDNCd0FMNEkzTm84dmZOM2NKYk81RERsVnlZN1VZaXp5TW5QRVAzOHNXQTFWdVlKdGtFX0FmcU1EbElZSm52alBQeWx4VnlvOFRwNk1ia2lZYXlpemQ4cFdmckotMmMyRGE4ZXN0dThQYmxxUkpvMzAwRXBBcVJuRnp0QkZ3b2tqMWF3?oc=5</t>
         </is>
       </c>
-      <c r="E76" s="17" t="inlineStr">
+      <c r="E76" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2642,7 +2645,7 @@
       <c r="F76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="17" t="inlineStr">
+      <c r="A77" s="18" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2652,17 +2655,17 @@
           <t>AustralianSuper claims another listed M&amp;A kill with Pepper Money</t>
         </is>
       </c>
-      <c r="C77" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D77" s="17" t="inlineStr">
+      <c r="C77" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D77" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOY0RwcnpWZlhfOHA2MG13MkJUX1RDNF9wN2RxZGU2cEpzS1RKTjJDeUl0OERFOGhFRXJaSXNETEhHbW9PS0lua283RnFVbHJvTlRva0djQ2lRSGc2RENJYmt0OEsyYTRVSzFGeE9jWVhKMVRnd240WXVNTVdac2lOUGJSZlc4UVZ5RXo0OTlQbUd6NWRSek1HZG9fZGk2aDhDelhGVmk4YkRKeVV1M0VHZ2hZNmFVdXM?oc=5</t>
         </is>
       </c>
-      <c r="E77" s="17" t="inlineStr">
+      <c r="E77" s="18" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2670,7 +2673,7 @@
       <c r="F77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="17" t="inlineStr">
+      <c r="A78" s="18" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2680,17 +2683,17 @@
           <t>Apollo to Acquire Nippon Sheet Glass in $3.7 Billion Deal</t>
         </is>
       </c>
-      <c r="C78" s="17" t="inlineStr">
+      <c r="C78" s="18" t="inlineStr">
         <is>
           <t>Wall Street Journal</t>
         </is>
       </c>
-      <c r="D78" s="17" t="inlineStr">
+      <c r="D78" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOanpORVBremoyamJyZ2FqQWVOcDcxa2NpempBUmNYcktMLUl1Mzg5VDloWmlVbUdNUnplVk90WEUzXzJjNGxENk9LcGF0enVSdlFpWU9nd244YWNTS0ZHd1JTZEtlbjRQTmJUU0dzWmlDOVFhR1ZRSFJkNXN4a3FHdGozcUcwdHRseXpYMFREUzBNcXRmQ1VCN056SWlEa1l5VVE?oc=5</t>
         </is>
       </c>
-      <c r="E78" s="17" t="inlineStr">
+      <c r="E78" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2698,7 +2701,7 @@
       <c r="F78" s="3" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="17" t="inlineStr">
+      <c r="A79" s="18" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2708,17 +2711,17 @@
           <t>Estee Lauder in talks to combine with Jean Paul Gaultier owner Puig</t>
         </is>
       </c>
-      <c r="C79" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D79" s="17" t="inlineStr">
+      <c r="C79" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D79" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPSjN6QnFVbmdHWFoteURWaU5VaWZmRmpTT3QtYm1tZUFyNUZyLUdheGdfWlRBTlJyTlp4THIwVDA4U3BnWFNpT2FpZlZzX1lJSDV0MkRGVjYtNVc0b0lOQy1RSnFGTWhCTWE2ZFFPYlFQX05yaVlfZF9IUEN2ZWkzQ0VFMUxxdHF2ODNQY09xdWlqWEczSC1CZk5wYU9QQlAyaTMyelJnaVM0cmN4M0paNzlBdzM1RndoZE8yRHN4UnZqaXVhVmx5NFpqS3hmUHhUdlpF?oc=5</t>
         </is>
       </c>
-      <c r="E79" s="17" t="inlineStr">
+      <c r="E79" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2726,7 +2729,7 @@
       <c r="F79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="17" t="inlineStr">
+      <c r="A80" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2736,17 +2739,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C80" s="17" t="inlineStr">
+      <c r="C80" s="18" t="inlineStr">
         <is>
           <t>The Age</t>
         </is>
       </c>
-      <c r="D80" s="17" t="inlineStr">
+      <c r="D80" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPdUtyNWs5YmxJMXNsNWtaMi1WMm5SVHd6ci1ReURLajdYd1IzWGJMZmE2MzJsSzAxQWtSTm8xMUEwNTh4Vy1zTmFsWFBKTkJ0YXc3ZkcwOVk2a2VNRWVGUS0yQzZhSXlCWmpDYUx6RmpTTlNhS0xIQklyVFdIVXJRZTNPaVB4TG4yQ1R1ZWF2MWpmSG81TVRaRzdtMXpydWhBS2w0a3ZPZFI5MnFKOW5tN21oUDB3NkNtQmR4LVVBWW9BUQ?oc=5</t>
         </is>
       </c>
-      <c r="E80" s="17" t="inlineStr">
+      <c r="E80" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2754,7 +2757,7 @@
       <c r="F80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="17" t="inlineStr">
+      <c r="A81" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2764,17 +2767,17 @@
           <t>Australia’s new millionaire factory: Start-up to $1.6b in five years</t>
         </is>
       </c>
-      <c r="C81" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D81" s="17" t="inlineStr">
+      <c r="C81" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D81" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOVkl5N1NGWS1XWWZSc0pHXzE3MUNERmV5SUgyQ3o2MmJ3U3Y2YlNwUXNSTGlQenBwVFdnMWhoT2FrcDAwUHNVU0RQbjFHMjJiLU1TRC1nemdrX3hPTG93VWZUQUx3Wk9HT3lYd055Z2FtREFpOWRlYXFDb2hwV0cyWFMwaHpsLU0ta2VVQlpid1dlYks0ZHg5YTY3Ykt6Um5YaF9MR2tIRzd1Tk1IRnBrWVhxVjZNSUl1OE9iRlZzYmQ3QUVnZmhYVGxoOA?oc=5</t>
         </is>
       </c>
-      <c r="E81" s="17" t="inlineStr">
+      <c r="E81" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2782,7 +2785,7 @@
       <c r="F81" s="3" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="17" t="inlineStr">
+      <c r="A82" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2792,17 +2795,17 @@
           <t>Social Media Wrap: Genki Sushi Singapore's loyalty benefits; Dunkin Philippines launches new collectible; Burger King Malaysia unveils new Korean inspired burger</t>
         </is>
       </c>
-      <c r="C82" s="17" t="inlineStr">
+      <c r="C82" s="18" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D82" s="17" t="inlineStr">
+      <c r="D82" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxPbFR6eHVTRWZNcUw1TTBJdE1JTFpmbk5iWndKZnRoU3Fmc3cxcF80TnVhRERmY0poM09zTFpCaEVnMGo5aktxY0ExV1ZlZVpHYUtldXBoOUh6bm14SURHNmhnUE9tYnI5YlpXQ3pRZlp0Ni1wM2lYQmdxdjk4SDl0aFN0R1VBbGxpbFVzOHV0TFY3YjJZbDg4Vk1HMTBkQk5LRHd1ZEVpRnBsT1U0Nm1IbVFkZEUybmpabEhuLUNLOGhicUxXZG5UalRLOE5DSzcxRncyNjVRdk8zclhJNkVQcTRkQTZYSEdN?oc=5</t>
         </is>
       </c>
-      <c r="E82" s="17" t="inlineStr">
+      <c r="E82" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -2810,7 +2813,7 @@
       <c r="F82" s="3" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="17" t="inlineStr">
+      <c r="A83" s="18" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -2820,17 +2823,17 @@
           <t>Copyright ‘status quo’ not working in AI boom times, says Charlton</t>
         </is>
       </c>
-      <c r="C83" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D83" s="17" t="inlineStr">
+      <c r="C83" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D83" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNVVgwdEQ2YUt0eFo3THcxOXZHbUFYZ091VTFKZDZHX0szYWQ2dnZ1dkJma3VZcGk1LUM2SUtQSWhxMGpCUlFZVzdKNmdoSGEycm1oYlBUdEZ5R0ZlU2hrWHpFWXdSN1lCZnZzb3hZc2twVVlWdTNNVXhaR0Nza0FiaUNveXZWQWQ1ZE45MU1HbGNmWlU2aUdha2FyZllzNWdONEpsM2RrdGRFSFl2UlpJUnQ4WGpleGs?oc=5</t>
         </is>
       </c>
-      <c r="E83" s="17" t="inlineStr">
+      <c r="E83" s="18" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2838,7 +2841,7 @@
       <c r="F83" s="3" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="17" t="inlineStr">
+      <c r="A84" s="18" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -2848,17 +2851,17 @@
           <t>The unapologetically analogue 4WD for off-roaders with $120k to spare</t>
         </is>
       </c>
-      <c r="C84" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D84" s="17" t="inlineStr">
+      <c r="C84" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D84" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxPSFJ4ZnNLT3U1REp3MWI2WDFaQm5vZlp6QWN6c0hZamtYVU95WmpkUERwR1dwc0NQN1dEc0FNbHlaMTdLclVHb1JTc2VZNExENGYyUE9OR1BkQ244YXRVeWNwbkxia2VrckVqSy00WV9UNWlvZWJHOG9ibUthaTlpVmRBOGZjLWFzMU8yS2Q5Um05SWIzY2dKajhoMWFUcmFrbTMzai1CdVBNLWczTWRvbTBwSDRfUzNwOHhqQm5hTDdhM0xLWEpNQTRyRXZjU1FLdGhRMUxtOTg?oc=5</t>
         </is>
       </c>
-      <c r="E84" s="17" t="inlineStr">
+      <c r="E84" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2866,7 +2869,7 @@
       <c r="F84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="17" t="inlineStr">
+      <c r="A85" s="18" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2876,17 +2879,17 @@
           <t>Junk room to become jazz club with priceless Melbourne view</t>
         </is>
       </c>
-      <c r="C85" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D85" s="17" t="inlineStr">
+      <c r="C85" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D85" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQbHN4My1nOGtueVJQZWM0LXNjLTR3MmhuemRJMUEwN09FTUZhZk1lbV9MbnVWblgyUXFEMEl3LUtsOGVqdGUweFR0MXF0ZEo0XzNhWVRqb2pGRUdiNTlLc1dFcXFmdnctQU1wQkRSdHN0T3J6VGt3MU1iNENydGlsOEpsT0ttZmJVZ0FUZmFXSUd3alVzUTQxMzVmcEVXSlV2dWdQd3JsMUZ0d3ZZYlBHaGhKTm9rM01SUmdseE9hT1prbHZtMlhv?oc=5</t>
         </is>
       </c>
-      <c r="E85" s="17" t="inlineStr">
+      <c r="E85" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2894,7 +2897,7 @@
       <c r="F85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="17" t="inlineStr">
+      <c r="A86" s="18" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2904,17 +2907,17 @@
           <t>Zimmermann fashion label appoints new CEO Roberto Eggs to replace Chris Olliver</t>
         </is>
       </c>
-      <c r="C86" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D86" s="17" t="inlineStr">
+      <c r="C86" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D86" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM2M5QU1scVoyNHBmV2lwQ0VQS1Z6d2Qwa1ZkZ0M2WVIzdXR3QnZwVWhUSDRCUEdRZkc5QzFQSFFhNzZ4VE9lWXBTcGhpS01JdG12TlQxSHhValZfbWt3MUdFZGl3RlBtdnlrel83TjNjNFZ0SUpvSDNQbThpU3FLa3Atd0dNU04zQm9OSk5uNHpTVE84aWZpaVlKWkdOQjJjRTZSd1MwMEZ1b3pENkRCQQ?oc=5</t>
         </is>
       </c>
-      <c r="E86" s="17" t="inlineStr">
+      <c r="E86" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2922,7 +2925,7 @@
       <c r="F86" s="3" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="17" t="inlineStr">
+      <c r="A87" s="18" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2932,17 +2935,17 @@
           <t>Construction giant FDC road tests IPO pitch - AFR</t>
         </is>
       </c>
-      <c r="C87" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D87" s="17" t="inlineStr">
+      <c r="C87" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D87" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNTnRScHFhQlpkdEdSb2x1bExxQm96ZE5zSV9wTDNDV2pxYjFQdUtoYmNBell3SFlTTFEzMUhpeXlmNERSeDd6VGppM2szQ1NHVE9PY1R3MTN0SUZLWkF5em8tQ3IycUZ2RmswX0tnN1IwOHl1ZFo4UUtMUDlQbXRjTnRCWFB5cU1RZFhsdDdaWGpMZzh3d29CWWZvZGtnTjl0T1k5ZHFHSUg5XzFSSF9TSUxTYkU0QkFheFlLZUY3S2tCSWRLZWlBbUpxUjc3TXBQQ01V?oc=5</t>
         </is>
       </c>
-      <c r="E87" s="17" t="inlineStr">
+      <c r="E87" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2950,7 +2953,7 @@
       <c r="F87" s="3" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="17" t="inlineStr">
+      <c r="A88" s="18" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -2960,17 +2963,17 @@
           <t>David Jones is trying to defy retail gravity. It’s causing problems</t>
         </is>
       </c>
-      <c r="C88" s="17" t="inlineStr">
+      <c r="C88" s="18" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D88" s="17" t="inlineStr">
+      <c r="D88" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPZy14UldWZDRrSjI3R0lzdGlKamlkVnU1WWVjTWRUTlpya1ZpVW80WHlrT0FQTUUwMzkzM19xQWpwTnVLOF8zeTFXamhTZFRQVjl5TTlXbE1RRWY2NW03dlpmZ25qdkgyN1IwbDdjRlhxd1MzSGkxeG45M214OVlESWF5WWh5TjM0STQtOXdieWIyOUI2NzRsaDhiS0ROUU5YQ185aWtObUY2S0dOSTBROVlwSVB1VkNqTkZTTllkZmtMYmxjNVdlTA?oc=5</t>
         </is>
       </c>
-      <c r="E88" s="17" t="inlineStr">
+      <c r="E88" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2978,7 +2981,7 @@
       <c r="F88" s="3" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="17" t="inlineStr">
+      <c r="A89" s="18" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -2988,17 +2991,17 @@
           <t>Jefferies’ Australian ambitions in focus as Sumitomo circles</t>
         </is>
       </c>
-      <c r="C89" s="17" t="inlineStr">
+      <c r="C89" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D89" s="17" t="inlineStr">
+      <c r="D89" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxNUTd0LXFPQmZXSldrTmZHTkIwUWQ3MmlCUmFOUGRkcVVjRXV6YXZJUTcyMG5FV3I0dWY2NXh6MnduVjNxZmhJMHdDVGw5VzFxTEFzN2FBdlNvS1JGSDltQmlzVS1QRDdCeWdfSHZ2VlZDMlBnN1Y0d2JxbnlGejhWVjJpWGZLejdCTUt2Uk9ENmhyRkd4dDJjd0RlUnBlZXhOTmUtOG9ITE05VHJ3dTBRSWZneURuUW1NYkExVXpfWXlsMzZ1WUlyNE84SThQX1JJTFlXOHc4ZnB0aXRmdVhaaG1qSEJRZUhuU3RibHAzbHVNLWFLUF9NNTFoUXV3NGQzelcwcNIBigJBVV95cUxPMkhEeDJpNzg0NTlDZmF2LUFPSEs4cmZ5U2p6bWVZSTYwcXVUUGVIb0FLVnhZV0cta01CLVpfQzQzYzdvTWdxR0o4bGJDWDVBb1lnOGx0bWROdTdjcHhwLUpPMW9MQ0RVM2NUOUt6UGpTd05JYzhuVmgybGp2LVpORFF0SHpBTU5DUTJEUmZKUFBNajlQdHJ4WkdHVV9QMjVwOWVlNWliVkFaM20yWGZhOEc4bldHRERJak1BWXlmSE0zdno1VTVSc0FMck0wSE1BR1RVaVRMSEdzU2FvcWpMYmp5ZTVJTWcyUGdXanhqSUNZU0tzTkNYWVg2SXpVMEoyS184VkxOeWtSUQ?oc=5</t>
         </is>
       </c>
-      <c r="E89" s="17" t="inlineStr">
+      <c r="E89" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3006,7 +3009,7 @@
       <c r="F89" s="3" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="17" t="inlineStr">
+      <c r="A90" s="18" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3016,17 +3019,17 @@
           <t>Bain Gets Nearly $300 Million Loan for Australia Wealth Unit M&amp;A</t>
         </is>
       </c>
-      <c r="C90" s="17" t="inlineStr">
+      <c r="C90" s="18" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D90" s="17" t="inlineStr">
+      <c r="D90" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMUQ4WExYZFY1aFBwWENNR1JiVkw4OHFKWjY4NW4zQ3ZBalFiTU10Y2hic2p2VjFqOE1rMndNYmVoN0lPcnY0WmFOV1MtaEY5c2xvcW1PNGN2SzZVcThwc3ljWkYwV1Q4a2dIaUpBeXZpMkRUU3IxZzVBVkhydGU3OXEzNW1sdlVQeTRNRFY4bUJLOGpGYmJ0ZXpPc1YzY05TYWd2bF9oWVJ6Rks2dWlod1dGRU4?oc=5</t>
         </is>
       </c>
-      <c r="E90" s="17" t="inlineStr">
+      <c r="E90" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3034,7 +3037,7 @@
       <c r="F90" s="3" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="17" t="inlineStr">
+      <c r="A91" s="18" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3044,17 +3047,17 @@
           <t>Fund managers caught up in Aware, TelstraSuper $237b merger</t>
         </is>
       </c>
-      <c r="C91" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D91" s="17" t="inlineStr">
+      <c r="C91" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D91" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcFF4Q1A5X1VtNWFnYXZSVUlZX2JMRVoxaUJoeGhybmRrZkd4UlEzTURwMkx2d2I1Y1hMYmljbk05WUFzRl9JbF9JampqeDd2bXdYcUpHbVZYak1sYXFHS2VuUDJyTUhzSS1QTW15aVpfeHRuMGZHenlxOHJQRUdENkV0b2FMZXhOZWF1Yk5hR1lOYWFQc2Q0SEROUFNERXhKQUIzRkt6NTQ?oc=5</t>
         </is>
       </c>
-      <c r="E91" s="17" t="inlineStr">
+      <c r="E91" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3062,7 +3065,7 @@
       <c r="F91" s="3" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="17" t="inlineStr">
+      <c r="A92" s="18" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3072,17 +3075,17 @@
           <t>Soul Patts defies private credit jitters with 15pc returns</t>
         </is>
       </c>
-      <c r="C92" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D92" s="17" t="inlineStr">
+      <c r="C92" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D92" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPRkNINFJOai1NbUUtX3ZrcnJFS3EzRHZPbFRfVFE3SERudTVqbjIybWsyYUthOUJOUVFPb1U0UzlGTTRqbUxraFZfYlVtclQxeTBQU1M5YjJzMDVPU3RiX0cxbk8xOEd5YjV1R04zT0NNZjhNSi1meWo4RHM1ckFsUnNLd0JiQXFnZ0dtckNzdWxmanZoQUl3TEQ2a29nRkRDZ1lJd2Y5VGc2UWZHX0pkU1NObmRJTlZKS0E?oc=5</t>
         </is>
       </c>
-      <c r="E92" s="17" t="inlineStr">
+      <c r="E92" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3090,7 +3093,7 @@
       <c r="F92" s="3" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" s="17" t="inlineStr">
+      <c r="A93" s="18" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3100,17 +3103,17 @@
           <t>Ex-KKR China heads negotiate to buy Vitaco, owner of Musashi, Nutra-Life</t>
         </is>
       </c>
-      <c r="C93" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D93" s="17" t="inlineStr">
+      <c r="C93" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D93" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQRmlCdTlFeHdBUGkyOS1CeEFIYTRSREdZM1JOZ3IyZThnNmNMdm9QeXVwRWtMbzU0em1vcDAyM1hodDlvalVRdThtNVhLR2FsaE1vV0xuWjkwMkVCUDk5SmVka1BURFJZNkl2bURLeC1GdzI0V2hEaVhrNlJZejlvc2gwRmtnUjd1NDFlX2trbGk2aXJiQ2FrTWtmVVpiOXhBc05JSkNYY2xLX2JEQUpWY2dlY1pDZw?oc=5</t>
         </is>
       </c>
-      <c r="E93" s="17" t="inlineStr">
+      <c r="E93" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3118,7 +3121,7 @@
       <c r="F93" s="3" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="17" t="inlineStr">
+      <c r="A94" s="18" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3128,17 +3131,17 @@
           <t>Antipodes Global Investment Company</t>
         </is>
       </c>
-      <c r="C94" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D94" s="17" t="inlineStr">
+      <c r="C94" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D94" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE5mdkJzN19XLTFQc25LOUk0ZGJBMER6djB2VnFvbGVrS1hlemRBRmlNY2JmMGlPTzktU0RRS3NNUW8tRXhtUE1QdE1JLWdUNVhibmZPZi1MRkJOWk95NzM2bXplS3JzeG13UU5henhza1ozeGRZZmlBNTNR?oc=5</t>
         </is>
       </c>
-      <c r="E94" s="17" t="inlineStr">
+      <c r="E94" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3146,7 +3149,7 @@
       <c r="F94" s="3" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="17" t="inlineStr">
+      <c r="A95" s="18" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3156,17 +3159,17 @@
           <t>AusSuper to lift insurance premiums by up to 40pc</t>
         </is>
       </c>
-      <c r="C95" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D95" s="17" t="inlineStr">
+      <c r="C95" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D95" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQNEhYQkoyNnJFU2xBZG8wdXhEZWRSakRiWWNHOGZBTFhfaElxWkRsSWViaWxjenVjMF91cGdrbFZxSGJfbkR2SUZNdEJtYUVadlV6YVVrWU1VbVdsMWpyNUZ4bE13Mmo4cGQ3WWZlVFVrTTdyOGpSdkpUb0tkcjdQUFlsTnM0MnpOMDJNZlJ4YTlzZGpLS1QzMFluOFU2VUJya3lSclBLSnZkQ2Y0a2djNUpSYlo?oc=5</t>
         </is>
       </c>
-      <c r="E95" s="17" t="inlineStr">
+      <c r="E95" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3174,7 +3177,7 @@
       <c r="F95" s="3" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" s="17" t="inlineStr">
+      <c r="A96" s="18" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -3184,17 +3187,17 @@
           <t>Unions want inflation-plus minimum wage rise due to ‘Trump and RBA’</t>
         </is>
       </c>
-      <c r="C96" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D96" s="17" t="inlineStr">
+      <c r="C96" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D96" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNdzNhU0MzbFRFX2I3OVY4bFItd1h6OVE2Wnpqb01NM2tMYzNob21BeW02LTBfTFZIWnN6SG5DVnYxQTJGZWZaLTJpTXZGUnhmS3RPY3hQV01fd1RIYU9Ednc4a1hvalVRT19ESU5TX19sQjN4dVV3X29kQjliQjNFU19iaXFIS2l3blk5TWUwdHFrRmJtQ0JocDN0WEhWbXZOVUJzR3RaYnJPSHpIRFlYOVFObEtuT1d0TUo0MUVZTXdFZWR3WG1r?oc=5</t>
         </is>
       </c>
-      <c r="E96" s="17" t="inlineStr">
+      <c r="E96" s="18" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3202,7 +3205,7 @@
       <c r="F96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" s="17" t="inlineStr">
+      <c r="A97" s="18" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3212,17 +3215,17 @@
           <t>Firmus’ Oliver Curtis set for green light to run ASX-listed company</t>
         </is>
       </c>
-      <c r="C97" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D97" s="17" t="inlineStr">
+      <c r="C97" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D97" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNR3VmQW9vNmUyeU9WbVRvRG9tcTNMYVlvRUhCd29wTkRZaVlEcG50Z0hIN29XcE5GUmxkUy1yMm0yTm94Q1BXMmNCcXBpZDlqVTRlZFpMX1QyMWh5Ym5XQ3VjYW1ZdDFtYWNyOERCOURuWXM5ZTV4WGthMVVjNUZlcmVTQ3JBUjQzUXRXYXRLQjlNeHpBMkVCVWpsd2Z1Vk42TjJxSlRiQ0ZtaTkzOTZtNmRHQQ?oc=5</t>
         </is>
       </c>
-      <c r="E97" s="17" t="inlineStr">
+      <c r="E97" s="18" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3230,7 +3233,7 @@
       <c r="F97" s="3" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" s="17" t="inlineStr">
+      <c r="A98" s="18" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3240,17 +3243,17 @@
           <t>Crisis Hit David Jones Chasing Funding As Retail Markets Come Under Pressure</t>
         </is>
       </c>
-      <c r="C98" s="17" t="inlineStr">
+      <c r="C98" s="18" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D98" s="17" t="inlineStr">
+      <c r="D98" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNNjJSOUVQcTkwUmxXNXg4ZzljSGhnRlBJY0otSHRrX2ZIQXRqWmNDZlgxYW1jckhHd3BtdXJsUWhwTjQ5SGw2NUU3TnFtcmhYd2JVcThIR2VCLWJLU0h5RE8xaTV5TS03Mi1za19hcF9PcXRRSU9PX3ZxSktSV2FfY1ppcUFVV2w1TmF1UWVtZlBWSUhEcG9oRGlEVkEwR2ltQ2VMSTNlcENEYlY0?oc=5</t>
         </is>
       </c>
-      <c r="E98" s="17" t="inlineStr">
+      <c r="E98" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3258,7 +3261,7 @@
       <c r="F98" s="3" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" s="17" t="inlineStr">
+      <c r="A99" s="18" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3268,17 +3271,17 @@
           <t>Beirut Street Food eyes niche in Lebanese fast casual</t>
         </is>
       </c>
-      <c r="C99" s="17" t="inlineStr">
+      <c r="C99" s="18" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D99" s="17" t="inlineStr">
+      <c r="D99" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNVlZVeTNGcXVOSXV1eklvTnFxYk1hb1A2VTQtNHkwdUpvdFF0YnlYU2RSWkZNV2dGQkEyZjRVQzVJZ2Uwc3gtZ0F1TGlSQlVna01HRnZOTTJnVUFxaWtOam1vZ245Z05jdlRnQURqbnQxaGtEcnFYS20wWmtvSDV0MW15c18zUE5ZN2JJWUpLV0RsZE1LSm5fcUNNeVZNTmdMQ2c?oc=5</t>
         </is>
       </c>
-      <c r="E99" s="17" t="inlineStr">
+      <c r="E99" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3286,7 +3289,7 @@
       <c r="F99" s="3" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" s="17" t="inlineStr">
+      <c r="A100" s="18" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3296,17 +3299,17 @@
           <t>Gami Chicken credits chip design for cult following across Australia</t>
         </is>
       </c>
-      <c r="C100" s="17" t="inlineStr">
+      <c r="C100" s="18" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D100" s="17" t="inlineStr">
+      <c r="D100" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPTXg4T0dvQ1l4NFVxV25iUXQzY0F3MnFjYmE4X0NOcFdNZHgweUg4NmVZZjNJbTFMajNhNHBmVDE2MGNBZzhOTUJsaG5KejFZbk1Db0JyNTZJbUI2WnRZeVhXRFRMNXVBWVFMdGJ3WkN5dV85dEduQi1OVDhOSE9UOGVERXh3T2hCVmlDNVg5LTdLY2VHNEZJSzlrN3VuemhzX1B5blpYRGtwS0hrak5r?oc=5</t>
         </is>
       </c>
-      <c r="E100" s="17" t="inlineStr">
+      <c r="E100" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3314,7 +3317,7 @@
       <c r="F100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" s="17" t="inlineStr">
+      <c r="A101" s="18" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3324,17 +3327,17 @@
           <t>The great fake meat meltdown is taking plant-based burgers with it</t>
         </is>
       </c>
-      <c r="C101" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D101" s="17" t="inlineStr">
+      <c r="C101" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D101" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPRTVDNW5oaWJ5bHdKM21iYllEVnpJbHhSbWFzYy1RcEZCdnNGUlJOWVJCaDZacFVoRjlSUGpfa3N6ckQtMFYzZTNITW5tMy05Sk0tZmtlSWlESHdOMWIyUWpUbE5RQVlsTHp0VXg0cHJYM0lJVmw1ckRURkFPVHFabTRIUzlFX1FlbFNuYmQ5MVJwWHVOaVhVWTdPajZxdG1WOTliTE1qZ3k1dnFRbk9BNTZCcXRRSGlIXzJv?oc=5</t>
         </is>
       </c>
-      <c r="E101" s="17" t="inlineStr">
+      <c r="E101" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3342,7 +3345,7 @@
       <c r="F101" s="3" t="inlineStr"/>
     </row>
     <row r="102">
-      <c r="A102" s="17" t="inlineStr">
+      <c r="A102" s="18" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3352,17 +3355,17 @@
           <t>Solar for Cuba: How Xi is turning Trump’s war into a China win</t>
         </is>
       </c>
-      <c r="C102" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D102" s="17" t="inlineStr">
+      <c r="C102" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D102" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQOFlUUnNZUWo0MTJRaDFIZHp5dUJudERrOWxCZmY1WjZmeXRTVzJkbENEbUFhSkZFUWV6WjNGNUJIejVYRXFPcmRNZjFZeTkzTmtaeFNlb2V1OFFnMGtkV2JfTVRUN2FSV2xxcUpDUDJQeUpqWE9DRHRmT2kyc1dIZE9jeUM2eV9KQjd2RkJuTkxYeEdISDZDejhRbVo?oc=5</t>
         </is>
       </c>
-      <c r="E102" s="17" t="inlineStr">
+      <c r="E102" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3370,7 +3373,7 @@
       <c r="F102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" s="17" t="inlineStr">
+      <c r="A103" s="18" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3380,17 +3383,17 @@
           <t>Beer Sectoral Group appoints Nigerian Breweries CEO Thibaut Boidin as Chairman</t>
         </is>
       </c>
-      <c r="C103" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D103" s="17" t="inlineStr">
+      <c r="C103" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D103" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOamdsNTN1dkRUY19Yak0wUGxsdm9NZGhySUM0Vzc4blNCeldzdFBiRkxuSW1xbTlZQUJIWkNxdzI3Zi1zc3F3SmJvai1UVGlZdUhGTEJ0eF9mNHRwSGREbDktT2txWXA4OVBESTdPLXdxWmV2V3FPTEZaYjRWLTlMM1VaY1dCbGZudTczZlFEYzN1aE9HeWdObE1yZFduLUtNVXBheDNsUWlIcUxibml4YQ?oc=5</t>
         </is>
       </c>
-      <c r="E103" s="17" t="inlineStr">
+      <c r="E103" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3398,7 +3401,7 @@
       <c r="F103" s="3" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" s="17" t="inlineStr">
+      <c r="A104" s="18" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3408,17 +3411,17 @@
           <t>Hip pocket pain comes for shoppers – and for supermarket giants</t>
         </is>
       </c>
-      <c r="C104" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D104" s="17" t="inlineStr">
+      <c r="C104" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D104" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOeTdfN2dwYlBWSTdGbFo0SWRJcTNYelFFM2FBRnlORWRNcGd0WUVCbVdHVWZ6TFdZQzFpM2h6TkU2OEtqeE5OYlRrNmhsRU43a0E0UXhtZEZyTWZidzhMUEVxSVdiMlpTYXQ4ZVRaNl9BSi1Mb3JRaXhvM2hlMmNDcnk1aFBvVXFQSmlPbkN4Z3o2R2RzV0drQWpKaVZpbXR4dHppa08wRFd0dlNwcDc1alRDSXg?oc=5</t>
         </is>
       </c>
-      <c r="E104" s="17" t="inlineStr">
+      <c r="E104" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3426,7 +3429,7 @@
       <c r="F104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
-      <c r="A105" s="17" t="inlineStr">
+      <c r="A105" s="18" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3436,17 +3439,17 @@
           <t>RBA calls for co-ordinated effort to unlock digital asset markets</t>
         </is>
       </c>
-      <c r="C105" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D105" s="17" t="inlineStr">
+      <c r="C105" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D105" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOT3dEcEtwVUptWTZydTRYWFdCU1RhTjI1RkFWeU5HckRVZjBxc2lqRkNOT0stc1h2Q0E1YTkxTjk3NTB3TGxKZGIweGFQRGh2S05QWHRoVGNZRFR2SlI2bkEzWlRoY2t3WU16dDlhVEI4RTFWYzhKS25YbGYxSVRjdFpVQ2M0dVc5MFJuUExNMTJIMVJTYmZGbkNLR1BPeVFYSF95NkNnWEEzamg3NmRuRkx0U2NjbXlxY015UWljTzRWbXpKclAwUg?oc=5</t>
         </is>
       </c>
-      <c r="E105" s="17" t="inlineStr">
+      <c r="E105" s="18" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3454,7 +3457,7 @@
       <c r="F105" s="3" t="inlineStr"/>
     </row>
     <row r="106">
-      <c r="A106" s="17" t="inlineStr">
+      <c r="A106" s="18" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -3464,17 +3467,17 @@
           <t>Banks rebuff work from home calls as Wesfarmers pauses business travel</t>
         </is>
       </c>
-      <c r="C106" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D106" s="17" t="inlineStr">
+      <c r="C106" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D106" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOTjFLNnZUNXZHeE85a3kyaG1IX29sWjFvZ2NzS041UnYxNkkwUF9YU3ZFYXhtQmlxY3Rmd0lUSTJrdTl1Y0ZobWp0M1lrZnZhZE9OSzV3Ql9Hb2UtUEpqWC1McjM0S2pESDJQVWJKQkw4enF5THJfeXFWRDZiMk5KMmVrazVUMzBNTk1tOXRVX1ZzVU1IUHBVSlhENEdEWFJpQnFXUGkyNVJGUnhzdXgyNW1WZXRkRmRaaVloZnpaMFdqVmk3elpFSkZ6ZmotZw?oc=5</t>
         </is>
       </c>
-      <c r="E106" s="17" t="inlineStr">
+      <c r="E106" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3482,7 +3485,7 @@
       <c r="F106" s="3" t="inlineStr"/>
     </row>
     <row r="107">
-      <c r="A107" s="17" t="inlineStr">
+      <c r="A107" s="18" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -3492,17 +3495,17 @@
           <t>This mine was fast-tracked to boost Australian solar. It’s exporting to China instead</t>
         </is>
       </c>
-      <c r="C107" s="17" t="inlineStr">
+      <c r="C107" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D107" s="17" t="inlineStr">
+      <c r="D107" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAJBVV95cUxPN1ZSdEMzSXBhMno2YzNkSFFtdlBOTTRGV3UtbnZtRktEd3Q0MHdmZHp0SDN5S0FZYmVKUllicHRMRkxTdmxtbkMtT2ZVN3hsUXdBVzAxdzhWcGFWRkxVdFY3NURqTVV2QVJQT0ZUT193R3JLLU9aZUw4YzlucjVUN0xyTzdoZlNjYXdyR2VWeDZrbW53cTJoRGZDd2kxbkxzMHBQWkRJMTFPMkNlX19wYjI2LVBZbnVJOVNsRjF3Tm0xUUFpY0ctczFZdWJFcHQyLUhwdDNiSGVtdHQzVVRtbExpcHJZak1SNkhWd2s4a0RtYWFNN2J2Q3FobTF1N0hWLXA4YUtaMXBScjZsUWt3alVVTVpJdVl0WDF5RTJLM1BKUl85dnhUUktkb2VwMzFkUWZ1ctIBugJBVV95cUxOOENIa2JzQzdxekNYTnJNVmRzdm9KTFpndnBybEJfNjBUR3VNMk92ZnhGY0JwVGZLeFRpdHJLMTQ0NjRNOFg5b3FESzhPLWlub2hSeFdidW0yS1h6ZXlGMjh3X3FhaWo1dHdneUZxS2NsaUJ6dWtfT1R6VndwSk52bVVNN2I5VlNYazBIelcwUkVBZHFlM0hiQVJ1a2NGWFpmR0c5R3Bna2RZMmJuSXB5WkQ1Zl94VDFtcjVEd2x6amIwSWdXUWtQVVo1Q0hpWVBLRVFycDAyU1NJV3N4YktlUlBtMTlkY2VNZjc1QVZhbnRrQ01OQnZqNzI5dTNNZ1VlNVVJcURycXlDRFZDYVo1aC15RXpwUFlvZWxlMHFybWJiM1YxT05lRElXYlZsbkJWUnI4VV9Da1lIUQ?oc=5</t>
         </is>
       </c>
-      <c r="E107" s="17" t="inlineStr">
+      <c r="E107" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3510,7 +3513,7 @@
       <c r="F107" s="3" t="inlineStr"/>
     </row>
     <row r="108">
-      <c r="A108" s="17" t="inlineStr">
+      <c r="A108" s="18" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3520,17 +3523,17 @@
           <t>A $600m dream or a dangerous gamble for cricket?</t>
         </is>
       </c>
-      <c r="C108" s="17" t="inlineStr">
+      <c r="C108" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D108" s="17" t="inlineStr">
+      <c r="D108" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxOYnpVaTZiU3hGMWY1UVVmYk9nRTJaRTVFYUE2ZklLYmJIQkdXZzFMbWs3MVRJb0l4bUpPeThwRnhOSmh0bzNBdzhpeXpuS1RrZ0tNVVJ4eU8tRVIwR2FyYmUtNG1UVmN2OXRsZm1mVy1LZDVERkpXQURMUk1HRE9Hc3F3RWQzYmFvbHRCVGhFOTQ3M2xnVGcxTWxtT3cydW84NTNPc3BXQURodmY0azBOUllOQjhrbzJ6WmI3bjY5dk5RRzlDQ0JlYzg0VzRsdWtIblZJelRSamFyQnNweHdHLTRTMTFOcy1Jd3ZtQWFodEcxOThVeVVz0gH3AUFVX3lxTE5ielVpNmJTeEYxZjVRVWZiT2dFMlpFNUVhQTZmSUtiYkhCR1dnMUxtazcxVElvSXhtSk95OHBGeE5KaHRvM0F3OGl5em5LVGtnS01VUnh5Ty1FUjBHYXJiZS00bVRWY3Y5dGxmbWZXLUtkNURGSldBRExSTUdET0dzcXdFZDNiYW9sdEJUaEU5NDczbGdUZzFNbG1PdzJ1bzg1M09zcFdBRGh2ZjRrME5SWU5COGtvMnpaYjduNjl2TlFHOUNDQmVjODRXNGx1a0huVkl6VFJqYXJCc3B4d0ctNFMxMU5zLUl3dm1BYWh0RzE5OFV5VXM?oc=5</t>
         </is>
       </c>
-      <c r="E108" s="17" t="inlineStr">
+      <c r="E108" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3538,7 +3541,7 @@
       <c r="F108" s="3" t="inlineStr"/>
     </row>
     <row r="109">
-      <c r="A109" s="17" t="inlineStr">
+      <c r="A109" s="18" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3548,17 +3551,17 @@
           <t>Why these people decided to vote for One Nation</t>
         </is>
       </c>
-      <c r="C109" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D109" s="17" t="inlineStr">
+      <c r="C109" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D109" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOQmNaOHZXWEEwZzRmdTBVT2FiS2hsYUhFczgxaFJaeEQzMGlfSnRoUWo0ZXl3cWhhbTU2NDRLUjh1c2Jxd3ZoR2pJOHVNemI2cTFrdU9oVkFCNXN4WV94TER4VmtIX1JCblhKNTl4VHlMdFBDRHVBUFhkS1AtR05RMG5QVGJFaTlWaVpMZERIa3Ntbmh0V0xnVVhYNDdMWWlpSWc?oc=5</t>
         </is>
       </c>
-      <c r="E109" s="17" t="inlineStr">
+      <c r="E109" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3566,7 +3569,7 @@
       <c r="F109" s="3" t="inlineStr"/>
     </row>
     <row r="110">
-      <c r="A110" s="17" t="inlineStr">
+      <c r="A110" s="18" t="inlineStr">
         <is>
           <t>2026-03-28</t>
         </is>
@@ -3576,17 +3579,17 @@
           <t>The Right Amount to Pay for Sushi</t>
         </is>
       </c>
-      <c r="C110" s="17" t="inlineStr">
+      <c r="C110" s="18" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D110" s="17" t="inlineStr">
+      <c r="D110" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOLUljQ1FWeHk0N21FcnpCTzdNVW1WZmxfbDFucXRNYlBMSzR6aTh4WlNrdnFuT1VSWWpKWlJValZrbTE5RlllanJkcHNHeEVwVkxldnZSdjdLc2c1SHJTVG1hMHBKd2xtZXptV1FmcGZ0cXUwVXFMWjJiRFhhYTlKRkNBNHZQekVRcnRicXlNM2NQdXJaZkVRbTZta0hDRlV5YVN5NG9TYzltUFZucXNXc29Wc1Y?oc=5</t>
         </is>
       </c>
-      <c r="E110" s="17" t="inlineStr">
+      <c r="E110" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3594,7 +3597,7 @@
       <c r="F110" s="3" t="inlineStr"/>
     </row>
     <row r="111">
-      <c r="A111" s="17" t="inlineStr">
+      <c r="A111" s="18" t="inlineStr">
         <is>
           <t>2026-03-29</t>
         </is>
@@ -3604,17 +3607,17 @@
           <t>Blackstone-backed $2b Xpansiv kicks off raise</t>
         </is>
       </c>
-      <c r="C111" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D111" s="17" t="inlineStr">
+      <c r="C111" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D111" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOOGIxbEhpZjgwbk5XampWenBXbGZmbzFQbnJhUjU1Z2FtT1FGVk40SHExMUJBZHZoRDBRVXZHS3ZlR3o5RGU0c1o0Y0E2MXVKZ3U2ZFBBRm1NbVJPRk1pMGp3dV96ZTlMNERlMFBPRDNROXpNZlNmLV83VGV2QVNzWkhtV1kxY2x6TUQ3QkhlcVNPNTlyMUQ0?oc=5</t>
         </is>
       </c>
-      <c r="E111" s="17" t="inlineStr">
+      <c r="E111" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3622,7 +3625,7 @@
       <c r="F111" s="3" t="inlineStr"/>
     </row>
     <row r="112">
-      <c r="A112" s="17" t="inlineStr">
+      <c r="A112" s="18" t="inlineStr">
         <is>
           <t>2026-03-28</t>
         </is>
@@ -3632,17 +3635,17 @@
           <t>Elon Musk puts a $2.5 trillion rocket up Wall Street convention</t>
         </is>
       </c>
-      <c r="C112" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D112" s="17" t="inlineStr">
+      <c r="C112" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D112" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPeE52VS03NHBqZ3hvc1Q4V2laUElCcmxKem9SSzM0d1Uyd09ZSFl4SjZmUDl1Sl85WXp3TWtGX3hydFRwZG0xQmFlOVUtdEtaNmtYWFkzVDYyZGI0SWFZRWtYR2tGODdPVUNhLXBzVVpzYnVRYmZNZW8xbEpreGZMVzU5c1JrWDY1Nk9uWk53a3FCOHpQTDBCT0h6QllmbW1wc3FmVU4yTUlxSmRhTUdF?oc=5</t>
         </is>
       </c>
-      <c r="E112" s="17" t="inlineStr">
+      <c r="E112" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3650,7 +3653,7 @@
       <c r="F112" s="3" t="inlineStr"/>
     </row>
     <row r="113">
-      <c r="A113" s="17" t="inlineStr">
+      <c r="A113" s="18" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3660,17 +3663,17 @@
           <t>KMD Brands makes emergency capital raise, chairman David Kirk to exit</t>
         </is>
       </c>
-      <c r="C113" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D113" s="17" t="inlineStr">
+      <c r="C113" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D113" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNb1JhRUM4dDhXM1hoajdzQkNLQk12LURQbkp5LWdqQXpEczBxdVhySHphaUhiLVRiYVh1R25kbHRidy1TbjhCOEk0MXk5a2VWWlhHcUt5aXpfNjZWNnd6LVpQUkZNbFFXSWJHTmFaM2x2aS0tbG9TeXFxUWI1NF9uazJKa3BrZHFwclB1OVR3cWhXU2dJNFhaZmpVRVlwWUdiX2hrX0thQ3RDOWdFTF9BOGdHTG1JSlF6RVRZdnZn?oc=5</t>
         </is>
       </c>
-      <c r="E113" s="17" t="inlineStr">
+      <c r="E113" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3678,7 +3681,7 @@
       <c r="F113" s="3" t="inlineStr"/>
     </row>
     <row r="114">
-      <c r="A114" s="17" t="inlineStr">
+      <c r="A114" s="18" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3688,17 +3691,17 @@
           <t>RBA green lights credit card surcharge ban</t>
         </is>
       </c>
-      <c r="C114" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D114" s="17" t="inlineStr">
+      <c r="C114" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D114" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOcTB6SlhfdTQ5ZWdqNDExZVhOcVVybW5mbmxOVktCS3ljTndLY3ItWldSNDIyeEkwQmdBZ3p1X1o5S3ktZXI3MFM3eVkwWWc4cGtUTUw3aWM4azM3VGdrcGZjTjZMN1diWHZ0N3pna0tJZHZNU1FaN2VZbVNwMmozSFNBb253OUcya0duaEMtZnNQaFYwUFBhTGthaGhyTWY0NHpPTTFubmZOWEk?oc=5</t>
         </is>
       </c>
-      <c r="E114" s="17" t="inlineStr">
+      <c r="E114" s="18" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3706,7 +3709,7 @@
       <c r="F114" s="3" t="inlineStr"/>
     </row>
     <row r="115">
-      <c r="A115" s="17" t="inlineStr">
+      <c r="A115" s="18" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3716,17 +3719,17 @@
           <t>Constellation Brands to acquire Hop Wtr, expanding non-alcoholic beverage portfolio</t>
         </is>
       </c>
-      <c r="C115" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D115" s="17" t="inlineStr">
+      <c r="C115" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D115" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPcjdPYWlEWWF6dkY2Y3RPWUh6M0pXYUw1NFNabUdXTS01TVBMWGtBMUpxTXFRekJINGNFOE5oVEI0WjR4Z2kzTUR6emJHUUYxWjA0MGVlWFNPR25xNmJJWkN2RHIzcWNxUHRFQXcwdWN5cHNZRVVYV3JTdXRJUFg1MWJKODNOdjJ5UEd4dWZEbVFyWlNaRkJPcnlyQW5janktSDVwYWRVRGJqTFdPTEdUSUFvRXI4QQ?oc=5</t>
         </is>
       </c>
-      <c r="E115" s="17" t="inlineStr">
+      <c r="E115" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3734,7 +3737,7 @@
       <c r="F115" s="3" t="inlineStr"/>
     </row>
     <row r="116">
-      <c r="A116" s="17" t="inlineStr">
+      <c r="A116" s="18" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3744,17 +3747,17 @@
           <t>David Jones races to secure $150m survival deal</t>
         </is>
       </c>
-      <c r="C116" s="17" t="inlineStr">
+      <c r="C116" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D116" s="17" t="inlineStr">
+      <c r="D116" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxONHp5S2RtcFJkYWVxakc1ZDE4UzZUVWlHSlBMTHJqVnVaRHJrcEwyV3BHWk9TdXdkOUlocWY2ZlN4NklobGVuYWhRc1BvdWppWlNFTm9wcGZoMG1UMEtjLS1scmx4cVNhNkZQYWw0M1VUQTJfOTJrYWMtTlpJYnl0N01QTWxZZDZPOEpfcTM1dFRVMDBTOEthcFU2Z0U4WFFBaE1GM2V6VHJVb2Z5ekxJWmUwQlphbXRlTS02NWNJV2p1Ym5Ca2JxNS0xQWZpbHJ4UFVtbDBCXy1IV2NXMlFOY25HSVkzTjYxbXZB0gHwAUFVX3lxTFBDVlc2X3JNcnNNWjlUV2RkeEdtSFBJRFNtTXVHcmZERW1vZURfeDFvRGo0b1Z5SlVOVGNJTXB4MVc3d3hWY3FVOENwbEJ1MERBalhlc2EwNnktcUprSjZQLUxNTVlqYzc0enZtQ0FOUFVTWHBCZVF1SWs2Y0ZKRllXblI4MVRrXzZUMHNicmxqeFhUUld4VzM0TGNtcl9fTG4wbEJPWDg4RWpjMUdHOUxlczdEend1MkZLRTZuUjdkV0xGRlR6RVlXdVUxdUhndmozTHNtT2czTjJzRUs0bFc2QnMxS0V1X3QwcjVNeGVjcQ?oc=5</t>
         </is>
       </c>
-      <c r="E116" s="17" t="inlineStr">
+      <c r="E116" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3762,7 +3765,7 @@
       <c r="F116" s="3" t="inlineStr"/>
     </row>
     <row r="117">
-      <c r="A117" s="17" t="inlineStr">
+      <c r="A117" s="18" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3772,17 +3775,17 @@
           <t>Newly listed Advanced Innergy targets smaller rival</t>
         </is>
       </c>
-      <c r="C117" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D117" s="17" t="inlineStr">
+      <c r="C117" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D117" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPamkyYnZfT0NwamdES3JPYklaaXFYdUp5cHJPOTZUNklqcUlral9ObHFPY1VROHJSdm1tOS1KZlZJWFA0Q1l2UUZhOThleHFsWDJTSVdTUnhlbE1OeVhBTXVQQjVIdHZHTFBHOUxGOGx3MWc1UmVIWUV6Q3RhTDR6WHRfRy05a25VX01lcWZOV3BWX1JyQVI0WlQ3dTQwNHhxWXJCQmV0VQ?oc=5</t>
         </is>
       </c>
-      <c r="E117" s="17" t="inlineStr">
+      <c r="E117" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3790,7 +3793,7 @@
       <c r="F117" s="3" t="inlineStr"/>
     </row>
     <row r="118">
-      <c r="A118" s="17" t="inlineStr">
+      <c r="A118" s="18" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3800,17 +3803,17 @@
           <t>Aussie eyewear giant’s costly $20k mistake</t>
         </is>
       </c>
-      <c r="C118" s="17" t="inlineStr">
+      <c r="C118" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D118" s="17" t="inlineStr">
+      <c r="D118" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAJBVV95cUxOTmtzblUxcW5WbDZLeEJXSWVuVW5qVzdpRkc1Rkoxc1pVT0FIaHdmR0p4ZzljcVpST2tHdTBwVEdqbmF2TVhlV0VaMDFiMVk2ZEZkUTZMNFQ1a1lUbWRCdGwySkJtbmRfTXFmUy1VVU1tU1dzMldON3lEUFVVVFI4T000b2NJLVhobDBBUzQyLTRGLXNPT3ptZ2tlUU8wNG5nNFAyUVo1elpTeDd1TW01YzB4eUI2eE9YQjZxNTJBSVpLYy0yR1BzSVFiWWxib1g0YmlzREFGTEV0bkRucmNLa3U4dXhkTC1aRkhnUHN1d0hjVUFuZFlWWG9xVUtMT0hKMjhmNkZzLWpMS2MzYWp1OVN0cV9IYnBRZG5OdWwwcErSAaYCQVVfeXFMTzBFMkJ2TU5EZGZYLVF5WHBJanYzeFJqS1owbk5EUUNOZFNiam5PcEZ1aDBFelJ5MjFzM0E0NlZRdGI4Rjdnb1RYVmVSN1Z1OWd1SFdweVB0ZEY5akVqOHBsTHpJaXZKNnhUMmd2YVVxTzUtUEJKcWpOY0VHeHlTbXNCbHFDdnlndzJFT2ZDcnlZWXYxNUFNekVUZWU1UTFnOXZXUERMWjdjYl9wVVl6OURodW1JSUI2ejJDTktfaTRCY2xEeHVBRW9tNmM3YXBHU201WXpHYjFYbU1sYnB1MjlLNjI0eTRWVElXU2ZqMDNNRW5LMVQyS2M5Z2tPSHJneGlkUkxFYXhDdWM1MGtkUUExT1hBSlU1ZkgtRlM4YnV3b1hkM2NR?oc=5</t>
         </is>
       </c>
-      <c r="E118" s="17" t="inlineStr">
+      <c r="E118" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3818,7 +3821,7 @@
       <c r="F118" s="3" t="inlineStr"/>
     </row>
     <row r="119">
-      <c r="A119" s="17" t="inlineStr">
+      <c r="A119" s="18" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3828,17 +3831,17 @@
           <t>Rio Tinto bankers up for infrastructure sale; eyes on Pilbara power</t>
         </is>
       </c>
-      <c r="C119" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D119" s="17" t="inlineStr">
+      <c r="C119" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D119" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPQTRxenprUFZmM2JIMDNPZGVVV09IakN5STI4ZFJVQmEtemVQUlJCRjdtbGpKWEZFOWVRd2ZYZk4xNkNHclpMSEFZLUpBVHhKaFN5Q0Y2bmhRWERpc2N4NEhua0VSQnFpVmpxa29tSlFNOHJRaFROMS1mTHBGdzZ6UlhLaVpqaUJhOEs3Y0Iyc29KY01XUXR3R1gwOXJHQUp2QVpNYi03NTZhLVgxN3VlODY4T0E?oc=5</t>
         </is>
       </c>
-      <c r="E119" s="17" t="inlineStr">
+      <c r="E119" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3846,7 +3849,7 @@
       <c r="F119" s="3" t="inlineStr"/>
     </row>
     <row r="120">
-      <c r="A120" s="17" t="inlineStr">
+      <c r="A120" s="18" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3856,17 +3859,17 @@
           <t>Luke’s Bánh Mí launches budget mini meal deal</t>
         </is>
       </c>
-      <c r="C120" s="17" t="inlineStr">
+      <c r="C120" s="18" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D120" s="17" t="inlineStr">
+      <c r="D120" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPQmh4NzlPa29pOXFmeTlKVFVUenNqdTF0VGU2REVwaWRsR3dKSEs3NFlTcGlscFRhRWRtV1JtVmFNTzJCb1d4d1NrUm9mMzBKcDBmM2JBbWZPTEVNdWZ1ZlVZZW93bW14Ull1UTNLUDh6WlZ2RUdBTS1NZEg2dmRZc3BEd2dfTFRFUERwdERnZnZwMFRR?oc=5</t>
         </is>
       </c>
-      <c r="E120" s="17" t="inlineStr">
+      <c r="E120" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3874,7 +3877,7 @@
       <c r="F120" s="3" t="inlineStr"/>
     </row>
     <row r="121">
-      <c r="A121" s="17" t="inlineStr">
+      <c r="A121" s="18" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3884,17 +3887,17 @@
           <t>Zeus Street Greek sets sights on drive-thru as next phase of growth</t>
         </is>
       </c>
-      <c r="C121" s="17" t="inlineStr">
+      <c r="C121" s="18" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D121" s="17" t="inlineStr">
+      <c r="D121" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNTEEzZ2VJMDdRek9JdGZCVVpJRGZoSjNIWjNiN3h2OHR2RjUwUG42SzViRUpteXRURFZzbFBpR0Q4TFdianc0SjZkc09DU01MY0hMLWRNbXQyYUVNai1BMUxFM0pZRWJaT0cwcmFna3pRS253R1FUY3UxOURmRkcwN3Fmd0VfLWVONzJJXzBzX1U5TFBQTFMtSURtZUV0TDhu?oc=5</t>
         </is>
       </c>
-      <c r="E121" s="17" t="inlineStr">
+      <c r="E121" s="18" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3902,7 +3905,7 @@
       <c r="F121" s="3" t="inlineStr"/>
     </row>
     <row r="122">
-      <c r="A122" s="17" t="inlineStr">
+      <c r="A122" s="18" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3912,17 +3915,17 @@
           <t>From $5bn to $50bn: The end of an era at Blackstone</t>
         </is>
       </c>
-      <c r="C122" s="17" t="inlineStr">
+      <c r="C122" s="18" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D122" s="17" t="inlineStr">
+      <c r="D122" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijgJBVV95cUxQc251ZVp0SEY1TnpWc2g4WERmLU9INk5VTUJHa3RGWGRmbWYzLV9MQW9rZmQ3bjVTRVI3R3NDbVNPdW9GTksxNUdrdkk1eTk0VXNFZmR2V2FBQWtnZGRmZkVMbm5QTUo4dFUxSGlOS0FSRmZZcThBVnlqWTN0eEUwUjFPdjhFb29BTXFWTTdHODRYelQwWUNBbXdNOElkQ2UzRU51VjM3SC1HZmpEUlNJUFFKRmdPWnhqNlEtVkNUaUtCbEc3ZWo2NFVIVktNMTQyd21lekpHVjlXOGV5WEhIZWJrU0ZTTFlrSkZnYlUxOWdUYnhna2JZTlhGYlAwMmhDYlJfZ1o3bVVDTnppS1HSAZMCQVVfeXFMT2E5cHJhVE9FUlVLN3RPakxmMHZKN3JLVUEwM3FSdmlfR0o0X2tybDFQWTg3NmZsYkE5LVRjX1dQMHVhNHBXNkhVRl9kd3lGeFdIWUV2QVFyYVgzWXU1Z2dpLXd6OGtUR0Z5SkdZc2VVM0tDU2MydXZSbGZOZjhUOEg0YXlBN2EtVDk3Z2FUM3pGY2JkTXdGZ2I5U2otVkJ1S3NhTXRBVVNqS1FvYzdPeHdaY3dqNlJmdkhwWHZCdjVsMXNibEc3aDFBR3NkRkZpdVRzU3Nad3Y0N2gyaHRQWlY0cGV2SUh3T1NwdEJEZTh3T3laM1B6YXlzVHlRRXdHc09tOFVKUTFfYjU0aFpJMDRlSTQ?oc=5</t>
         </is>
       </c>
-      <c r="E122" s="17" t="inlineStr">
+      <c r="E122" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3930,7 +3933,7 @@
       <c r="F122" s="3" t="inlineStr"/>
     </row>
     <row r="123">
-      <c r="A123" s="17" t="inlineStr">
+      <c r="A123" s="18" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3940,17 +3943,17 @@
           <t>Starbucks opens first retail outlet at new Town Hall Station</t>
         </is>
       </c>
-      <c r="C123" s="17" t="inlineStr">
+      <c r="C123" s="18" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D123" s="17" t="inlineStr">
+      <c r="D123" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOTnJ1YVF6V1dqMm9HbmdUZEk3NlQtdjRxT28ya19fbjRKMlJRb3hsam5zdDg1cnEycHc4STRPdENPQnlMQldBbTh3NXlYb0tUNW9WS201NTZ0M0xvRE8zRkVYcFlNSmdOeVZvbXRMVzJMMkV6czFPX2djSFdKNlhWbUQtNUpMcnhFNnpfa1RPY3Q?oc=5</t>
         </is>
       </c>
-      <c r="E123" s="17" t="inlineStr">
+      <c r="E123" s="18" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3958,7 +3961,7 @@
       <c r="F123" s="3" t="inlineStr"/>
     </row>
     <row r="124">
-      <c r="A124" s="17" t="inlineStr">
+      <c r="A124" s="18" t="inlineStr">
         <is>
           <t>2026-03-29</t>
         </is>
@@ -3968,17 +3971,17 @@
           <t>The ex-Platinum quant who has won billionaire Kerr Neilson’s backing</t>
         </is>
       </c>
-      <c r="C124" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D124" s="17" t="inlineStr">
+      <c r="C124" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D124" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNMkpmVTVUVU1WZUZiRWlJUkRId3BhS1hqM09aM0FSODBFNE96SDlKWG11Qkw2bjVSNFFrc0oyWHBBVXNYclBYQklIdnZBNEZ3b2NvZzdHZWNrV1JhbWI5aUpBLXRqTjIwSnhRSlFtdUlTU3VUbVMxcmtYZzlnVEsxellFb0dwb1hhME9QbERGcU9aXy1rOEtyQ0pXZW9KcENIem5TMjhUZ1VydFlrVWI3cWN6aGJROGFwWUFlNjQweTdqYkptcHc?oc=5</t>
         </is>
       </c>
-      <c r="E124" s="17" t="inlineStr">
+      <c r="E124" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3986,7 +3989,7 @@
       <c r="F124" s="3" t="inlineStr"/>
     </row>
     <row r="125">
-      <c r="A125" s="17" t="inlineStr">
+      <c r="A125" s="18" t="inlineStr">
         <is>
           <t>2026-03-29</t>
         </is>
@@ -3996,17 +3999,17 @@
           <t>Media bosses: ‘Australia shouldn’t be held to ransom’ by AI giants</t>
         </is>
       </c>
-      <c r="C125" s="17" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D125" s="17" t="inlineStr">
+      <c r="C125" s="18" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D125" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPSGdRM3JDVld4OG5UWk5RdlVZVlU2LTFKUjdzVy1HejgyaUxMWHhmUlJnN1FrY2dSTTczczU0Tno2TUVPWDFiZk9TTjJTNlQ4Yi03MWpfdVEwWGFaQm9ydjJpaGFkekZHME1xNUswcWF4b2Y4TUxkOUpOa0dFTjlYVmhVMnFPMXlEcGJjeXZBR0tFaDZUa3Ixd1lIai1qcml5OE9SM1dTcUVkWW1HdFJTUFBJZUU0Nzg?oc=5</t>
         </is>
       </c>
-      <c r="E125" s="17" t="inlineStr">
+      <c r="E125" s="18" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -4014,7 +4017,7 @@
       <c r="F125" s="3" t="inlineStr"/>
     </row>
     <row r="126">
-      <c r="A126" s="17" t="inlineStr">
+      <c r="A126" s="18" t="inlineStr">
         <is>
           <t>2026-03-28</t>
         </is>
@@ -4024,17 +4027,17 @@
           <t>PLI scheme for food processing industries sees Rs 9,207 crore investment</t>
         </is>
       </c>
-      <c r="C126" s="17" t="inlineStr">
+      <c r="C126" s="18" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D126" s="17" t="inlineStr">
+      <c r="D126" s="18" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOcUwtamFxVTZ0YTdEOTBsN1gxNlphTV84aGJoRnFFTkFkZDhaT2VzVkFDT29hMU1Xa3BLeWFiRWlXT3Noc3VVVkg3WkphSFMwS3k2aWI4ZlhfcDN2LTV6Q3E0YnNXbEFVZFdUU3U0R293aEtlUmxlLXdFWXl5MHh0X2hWYnNvbU5MLUNCRm53aVpJa0E4OUxuNnN3X1FwUQ?oc=5</t>
         </is>
       </c>
-      <c r="E126" s="17" t="inlineStr">
+      <c r="E126" s="18" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -4600,6 +4603,174 @@
         </is>
       </c>
       <c r="F146" s="3" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="19" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>Inside the AI-fuelled fraud that deceived Australia’s biggest bank</t>
+        </is>
+      </c>
+      <c r="C147" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D147" s="19" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxPZWdmQklwRGlvLXBrbzVlNHVJZlJEVWMyWmVDUFd0eVFZNW91dUtBRXB6Q0s1bGpkTDZkUEpaTnNBZjhpTTBaTFRDc2NLb3JaVFNkUnVUd0NZQy1zVVN4WGxmbkFBQ1l5ZWFrUDJnejZRTXRhR3k4TGVXQy1TaFVLNlUyaWU3ZlhHMlhBdFJmQy1JdkRLSjlDWndWNEZpeW9QVEVpSGFWOXNKMW94ZUpRbWF6TFMxS3Vxd2M4QlBBYUNfMGJRVzNWa3lZYw?oc=5</t>
+        </is>
+      </c>
+      <c r="E147" s="19" t="inlineStr">
+        <is>
+          <t>Australian Economy &amp; Markets</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="19" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>Meet the winners of the Best Places to Work awards</t>
+        </is>
+      </c>
+      <c r="C148" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D148" s="19" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQQTYweEJveHFxWlZVUm5QUVQxOVU2QW15N0EwOW9aOEpXNGJ1TWExVUZpV25IMFVMVVRQTFlzYTlhN1NGM05JRDJCUmN1SVF4T0dmRGV5ZlRHdGY3bDA1Nzk3aWQwOFVwY3lRQjJvWUU2ZWtSZzQ3SWljVy04VW9FM3RGQWk1NmIxSUFGcS1paGJFQ0d3QW5ZWmJjRXZsakF3alNOTmItbXFFNHBsYk1zZkhNdw?oc=5</t>
+        </is>
+      </c>
+      <c r="E148" s="19" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F148" s="3" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="19" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>Healthscope landlords offer break-up deal with private equity</t>
+        </is>
+      </c>
+      <c r="C149" s="19" t="inlineStr">
+        <is>
+          <t>SMH</t>
+        </is>
+      </c>
+      <c r="D149" s="19" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNSEdKYllEUEZ0ME5KNkh4aUoyVUdudm9ROFJ2RDVuUGRNS3EtdnZVbXpJeGxFMklrYmhaTEVlUzh3cVhyTERCVDlSZGVkckg5cHNDRDl2VmYwNW5SZnZwbXVHbkpqSFZXU3luSkcySl8tUlZLODRFM05mRU5mdENUcE1SenlLVDFsYzVGYkUxR3lNcHBpdTd4MVJwcXU2M25GVkN3VzdvM3FadWNCT2lYVkN2WHlqa2dLU0oxWjBsWnFSZw?oc=5</t>
+        </is>
+      </c>
+      <c r="E149" s="19" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="19" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>TPG NewQuest gets its paws on Pemba’s Vets Central continuation fund</t>
+        </is>
+      </c>
+      <c r="C150" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D150" s="19" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNN3FVaGNQYzBnU3ZHWG9oN19YY3BERTdYcUZROEd1dVYyMWViYkpGMkpxNm5qQjViWHpWWS1wU3dFbFNWMzhUbFIzUDU1Z1puY21lRWN5VGl6cUVlMnBjb3hlYXA1QWcwaVhXZDVXbW4xTHpiUTluSmNNOEVzMUF1Mm5pVXRPRTVyZlRETnFGSzJqTFJWQXVmOVlrUUZ2aUdWSWFVNWNqcnFTcnRyT2UxYVF3?oc=5</t>
+        </is>
+      </c>
+      <c r="E150" s="19" t="inlineStr">
+        <is>
+          <t>Australian Economy &amp; Markets</t>
+        </is>
+      </c>
+      <c r="F150" s="3" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="19" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>Sushi Express Singapore launches limited-time collaborations with The Powerpuff Girls</t>
+        </is>
+      </c>
+      <c r="C151" s="19" t="inlineStr">
+        <is>
+          <t>QSR Media</t>
+        </is>
+      </c>
+      <c r="D151" s="19" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOHpNQ1NrdkFiNng1bV9lNVQ4WWxUOGVTQUpnMUVoMWsySmVTRXFGMXo2SEVFUzVJd3Vid3YtZ2VIb1dycEJwR0tGcGJ1ZEg2YkdUNkJQN1BMT1Utd2hpcEswbFhxYlJfUDhVSl96TjRLWnR2Z0JRbERJelZtZGlEUmFabkhHYTU3UVR6WVRFNXVHdmN0LTRIY0FjaVJjV0RTcUN4Ui12UUR1TUJMU3B0dE14MA?oc=5</t>
+        </is>
+      </c>
+      <c r="E151" s="19" t="inlineStr">
+        <is>
+          <t>QSR &amp; Franchising</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="19" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>Stocks are surging in early signs of huge short squeeze</t>
+        </is>
+      </c>
+      <c r="C152" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D152" s="19" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNRGFlZ2RyZ1Rla3ZZYzVVVkx0Q1ZtUHp2aldyQVJDZEVDWnY3V1dDYUhHMEtYN2dQck9sNEpQd2tOc2tkc3VaSjJIWmV4VXhoYTE3RkxSTFRGUDluSUVTbTRORkJrN0VlX3Z6d2VINVlyVDZhNkFteVJkYnZyci1oa1J4bW9ZN3BJZ2pzajVPdU0yOHUtdkxqdWpFUU9xWWVrMHBxTlRjdThCTHlaaUdON2Rua2txQlZn?oc=5</t>
+        </is>
+      </c>
+      <c r="E152" s="19" t="inlineStr">
+        <is>
+          <t>Australian Economy &amp; Markets</t>
+        </is>
+      </c>
+      <c r="F152" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>

</xml_diff>

<commit_message>
Update news log — 2026-04-02
</commit_message>
<xml_diff>
--- a/news_log.xlsx
+++ b/news_log.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -87,6 +87,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -501,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F152"/>
+  <dimension ref="A1:F155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -545,7 +548,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -555,17 +558,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C2" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D2" s="18" t="inlineStr">
+      <c r="C2" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D2" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E2" s="18" t="inlineStr">
+      <c r="E2" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -573,7 +576,7 @@
       <c r="F2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -583,17 +586,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C3" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D3" s="18" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D3" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E3" s="18" t="inlineStr">
+      <c r="E3" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -601,7 +604,7 @@
       <c r="F3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -611,17 +614,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -629,7 +632,7 @@
       <c r="F4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -639,17 +642,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -657,7 +660,7 @@
       <c r="F5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -667,17 +670,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -685,7 +688,7 @@
       <c r="F6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -695,17 +698,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -713,7 +716,7 @@
       <c r="F7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -723,17 +726,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5</t>
         </is>
       </c>
-      <c r="E8" s="18" t="inlineStr">
+      <c r="E8" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -741,7 +744,7 @@
       <c r="F8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -751,17 +754,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5</t>
         </is>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="E9" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -769,7 +772,7 @@
       <c r="F9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -779,17 +782,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C10" s="18" t="inlineStr">
+      <c r="C10" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D10" s="18" t="inlineStr">
+      <c r="D10" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5</t>
         </is>
       </c>
-      <c r="E10" s="18" t="inlineStr">
+      <c r="E10" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -797,7 +800,7 @@
       <c r="F10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -807,17 +810,17 @@
           <t>Zarraffa’s Coffee celebrates 30 years, eyes nationwide growth</t>
         </is>
       </c>
-      <c r="C11" s="18" t="inlineStr">
+      <c r="C11" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D11" s="18" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOcXNzUkRLemZEOWtOZjhvRUtzcUZrSTdzV0s0LUJTd2NGRk1Gb1NSLUR5Rlh3NUdWQUJkVWctb0toUFBRajlMcWV3VnNyTUtydy1PSUoyb1NCOGVtMUZqRVN0MzFkVkNlOUZNVXlHN2kzREhSdWJQUnJqa0pnUzExTVZSc1NCVFZSNlBSUWNfWnZ3MC01aUx0UWF5SkNOaHI3ZkE?oc=5</t>
         </is>
       </c>
-      <c r="E11" s="18" t="inlineStr">
+      <c r="E11" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -825,7 +828,7 @@
       <c r="F11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -835,17 +838,17 @@
           <t>Zarraffa’s Coffee eyes 200 outlets ahead of 2032 Olympics</t>
         </is>
       </c>
-      <c r="C12" s="18" t="inlineStr">
+      <c r="C12" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D12" s="18" t="inlineStr">
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPMUFjRTlGVFBqYzlPWXdzQ0dKVVlhWGxncUQxTDd1R0VHcThlV3ExVmo4SlBGSHVuUGZrMGNqSVo1YVpDWHViMm5KZWIxcHNMMHo0b1FQcmxUNElDR2lEeWRuLWZIN2lyQUV0VndEUWNkNU42Z3AzNXRlbm50NzhtTXZ0Q245dF9hNzBxOENuMXZsVlU4Z0JGVElR?oc=5</t>
         </is>
       </c>
-      <c r="E12" s="18" t="inlineStr">
+      <c r="E12" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -853,7 +856,7 @@
       <c r="F12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -863,17 +866,17 @@
           <t>Aware Super appoints new head of private equity</t>
         </is>
       </c>
-      <c r="C13" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNVHJXNWEtdEZZUW1fZzdYMTB4RklBTUh6dUNKQ3BrTlpYUnBwRURIVGZjWTV0OUxScnhGMVNSczhLUjVqOEwzbkR2WWlEbmF4ZkNUdHNQY0J1djI0REctbHd2SVhUNlNCa2M5bFhOQ0JPU0RHOVVTQkEzRDdGMjRZbVFDOUdlTXNNczlmZWF6bXlfbEFGRE0xbkZQaw?oc=5</t>
         </is>
       </c>
-      <c r="E13" s="18" t="inlineStr">
+      <c r="E13" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -881,7 +884,7 @@
       <c r="F13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -891,17 +894,17 @@
           <t>Commission wrinkle over UP Education sale</t>
         </is>
       </c>
-      <c r="C14" s="18" t="inlineStr">
+      <c r="C14" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D14" s="18" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxNSV9GMjhqM2ZSanI2X0w2OVlQVFRQTUoxYzAxaXVZMmU1REVTcHlUeEltdXJtaXZrcUJWdDZxNGpYTTZYSFE2TkZHeG9OaVRZakoxV0s1U01TVjJpWlhaSENfNVhucG5NVzFMbTVBY25zWGRSODBtRGtkS1owVTlJWnNfcTJ5alFnbVl1SU9aUDF1QWxJLTBSQ3kxUUFlZnpJMlVEQndFSGRGbDF6WVBUVHlCcDM5Qnh3R2xBMG9xN2FLckNzbUFOWDI1aVF1YV90d0twd0ZmMnUySDBMdG1R0gHkAUFVX3lxTE5EWVp6VzZWb01TRmlHSS0wMExldkJwSHJjdlZXdElsRlpBTEtVMkd6VzNQa1RpVDNsOFQzaGZ2VHpzUnBDYk82RmZGQWJuTmVQMXhxLXVmdVFxTVZOZTBsOHZ0V3cyVVVkNWUwVUxSc0xNSU92ZktpdFRfYnQ4WHBTX3A5bFhXZ1YwZXNrc1BSZEU4LVYybnNBd0dCdk92OFUwclJCMzdoU0ctX1pEdTAwY0JiTWQ4S01QRE00TW5EUEJwR2YtczZ0T005bTJnN1RDY2p6NFF1SndfLUo4QzJUWk1tRg?oc=5</t>
         </is>
       </c>
-      <c r="E14" s="18" t="inlineStr">
+      <c r="E14" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -909,7 +912,7 @@
       <c r="F14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -919,17 +922,17 @@
           <t>Gloria Jean’s owner has an angry shareholder on its case</t>
         </is>
       </c>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D15" s="18" t="inlineStr">
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPTnZwUVBCdTFJZWkwc0YtVmJqMkNPcUR5RktjMlVURmhROFZkYUpXM01iRUh3SnJEUElxRGlSNk9DQjZSdTdNdmZwWWpONjlmR1hoMl92cUNmd3M4cnJhVkNqc095MmN6WXBYUmdEblB0eERtVDdlUU4yNGFjXzVnT19rOERIRzVPNzY3VDNNRS1tVGVTX3pKMVRpTXZVR1ROLURBLWtJbVZhY0lSU09DNkE2NzFLbEFU?oc=5</t>
         </is>
       </c>
-      <c r="E15" s="18" t="inlineStr">
+      <c r="E15" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -937,7 +940,7 @@
       <c r="F15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -947,17 +950,17 @@
           <t>Oporto-owner Craveable Brands hires new CEO from Domino’s</t>
         </is>
       </c>
-      <c r="C16" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNNmxfQVc2Umc4QWwzSTdsZTFvejRzTzZxXy1ScGlhXzh6bm5JS3IyX0xTNDVBNjh0cXpPbGhxNU5xUHhQN3EtRF9aV3FEc2JoSG5QTU1WeU1TLUJfZzVUT2N6dXloQXhZaHB5djB3dDFKN1llVmI3UVpKNjJTNlcyV0ZDcG9GdVdSdW41ZkN1b1N3SFFIUzcwRkQ3UHY2TmxERmZwTlA0RzU?oc=5</t>
         </is>
       </c>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="E16" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -965,7 +968,7 @@
       <c r="F16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -975,17 +978,17 @@
           <t>Brookfield, BGH Capital rub shoulders in ScotPac’s data room</t>
         </is>
       </c>
-      <c r="C17" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D17" s="18" t="inlineStr">
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPMVlxbzlQNnFXWnJFNU11Y1BhTTVqbjN4RG1nbkZuN0pkdDFFaUhJN0RaVnUtWDlZSGJWR1ozQXk5UUx6RVdOcjBPU2t5UzN4T0JvUFJISnNvVWxQemd3blNHZjRQVVVZQk1nZER0Y0JfY3VvQ0t1a09sM1RTS2c1YTJyUmdzYWh1WGRUNjl2dkdzYTJJeHVhMTdqR3Y5WVlHVEtSZHp1cmVYYmM?oc=5</t>
         </is>
       </c>
-      <c r="E17" s="18" t="inlineStr">
+      <c r="E17" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -993,7 +996,7 @@
       <c r="F17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1003,17 +1006,17 @@
           <t>Payments player Pay.com.au hits the road(show) for $850m IPO</t>
         </is>
       </c>
-      <c r="C18" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOMFZleXZrbU53TzBlakI2ZmJKTjlrN3BoQlRaWjQ5cXFzTllKWmFoRm1UT2xDUHBtNC1QNTNiX1BwSzllMkRZdHIzRlAteDREaUczN1JTNTByTW1jNnR3d2NnR0RxUDBxeHYyWU1CSUs5MEZad2JqSGF6ZUxHZUNtZmFQaTJZZVJVZ1B4MkZ6V09QMWIxaUNHQmVzTDhvWVA1Ty1UbHgtQnRrQQ?oc=5</t>
         </is>
       </c>
-      <c r="E18" s="18" t="inlineStr">
+      <c r="E18" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1021,7 +1024,7 @@
       <c r="F18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1031,17 +1034,17 @@
           <t>Another year, another IPO cold shower for investors</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D19" s="18" t="inlineStr">
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNeEhzYzQzdjR5MDJCWkd6Q2VLdEZzbzRoWnNOcXFlQjNfMlV4Q0NQRjExMlNhT2NPcnRBbW1sZUkteXo4N0dGaHNNeGZJOEZ2aXFvdmZiN2V2QzdOMzFteFRnY1RVRm1rQXltWmY5VFZOdFVNNVpudVp1dTlrcFM5b1k5SmlWQllDMVFXSjA4ZVpSZHgtV2JpWDJ4SkFRbVE?oc=5</t>
         </is>
       </c>
-      <c r="E19" s="18" t="inlineStr">
+      <c r="E19" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1049,7 +1052,7 @@
       <c r="F19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1059,17 +1062,17 @@
           <t>Priceline Pharmacy franchisee sale narrows to final four bidders</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D20" s="18" t="inlineStr">
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNR294am9sYWNiQ3FVT1B6YlV5ejMyeHAyT0FibTFVbU5pcjZyaVRyazEzbFkxd0lrcnpZNGpTYUx4Ykl1Xy1sZF93M2Nid19ydUFwbUJ3ZHozaURaNkRoOE9OMnRBRGZfQVdCVWZCaVhhNnZSRjlwYUdDVnp2WU9HUkJxbE1QMV8zdWxYRTNBQWktR0xSOFU4dmtXZWk0am9SSU92NWp6QUZmTVU5TzJEOEJNak5fQUtN?oc=5</t>
         </is>
       </c>
-      <c r="E20" s="18" t="inlineStr">
+      <c r="E20" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1077,7 +1080,7 @@
       <c r="F20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1087,17 +1090,17 @@
           <t>Private equity gets better image of Qscan</t>
         </is>
       </c>
-      <c r="C21" s="18" t="inlineStr">
+      <c r="C21" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D21" s="18" t="inlineStr">
+      <c r="D21" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxPRjVmT0hDRjZLblB1VHdPRmRGeXhKdDJHdWxDTzV4RDZ0VzdHaUFfOVlnZjRQMWhKcWMxby1oRDR6N2lQZkI1UDE1REppS3c4LTVmU3p5b2wtblRCWnhNajFnZGNHaGRJUHFMUGRtTHAyQmIxOHhNNTgwRWVSeWp6ZWRxbUY0WVhiUnhMRUpDLXNwS1RuelJldTk0Z1R0WHg0XzNXNTA5Rk5TRFZhU1RNVnN2TlZuaFE4OWtIYXQ5a2VGSW1UWmt5Rlc4Q2lIXzF3YlkwNVhfUzJDV0dQdVAxa2RKc08wRGR6TlB2Vi14QV9BdlhyaTZsM2pEVGZycTjSAYQCQVVfeXFMTWpnb0lWQmZ6MTFnRGhWNTNqczk1TWhTcUFEMVpDNnJ4ZWVxVlRUODhJXy03NHdGZVJlMmhyUHM0Nlh4NlZtTzRhQ0xxRDFLVHNzUVNfbWxhS3BLUEQteEMzZHRrc0F1eFRzYmxVNDZlSURyZDB5bF9wQTNRRU5yZEs1Z3pFRTdwcFBaMkNlN0JvT1NEYkFWVUJNcHJqcEM5RVJYa0JFUVl6cThyQXloaERzQjhkTUVPakJqb0hzNVlwSWxNS0dmZkNFSG9Gb3dNUnVvUnV0d3MxSmpzdFZKTHJ2RTQwRUoyMEVLLWMwT1NnOHdXVl9lRXNDWEFndzJFSDlZU0o?oc=5</t>
         </is>
       </c>
-      <c r="E21" s="18" t="inlineStr">
+      <c r="E21" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1105,7 +1108,7 @@
       <c r="F21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1115,17 +1118,17 @@
           <t>Oporto CEO’s first year reshapes brand and network strategy</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
+      <c r="C22" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D22" s="18" t="inlineStr">
+      <c r="D22" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPY25mNTJfT3FiVlBPZE5CcVNkR1UzR2xWaUtJSmxhU3EwcEMzQi1ISDFSajlCQWk1UUJpZVJ1Q19ZV3Jjd0Noc0l3OExpMXhSQUVVdHhCLTBlOXNoZzA3UXZBdkR1VHBvMmVsZkNhUFJndm1DdGpnX2w0ZVViU2phZ1RmYXY1SlhwUnhKSUxBQVZZUXpqNHQxQmo0Rk1iV0g0OW9qUS16eWRSNW5FaW1yQQ?oc=5</t>
         </is>
       </c>
-      <c r="E22" s="18" t="inlineStr">
+      <c r="E22" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1133,7 +1136,7 @@
       <c r="F22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1143,17 +1146,17 @@
           <t>The Melbourne restaurant our reviewer grew to love</t>
         </is>
       </c>
-      <c r="C23" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D23" s="18" t="inlineStr">
+      <c r="C23" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOc3YxQTljcHJXVWtRX2ZGM2lpM2pILWNwSFg0MFJrNmNWX0ZxRG9nV0J5N19qRWh4U0hPXzNmVVZwWk9wT2kzaFNrTlV3NEQ1Q3JpaXVIYlBHb216Q3VYVWdSRXMwdDl0SmYzdnRlSDFUYVRmRGJyZVlRZDJKTHpJOUctYlF1RDZSYjloY0hfZy13QmFTLU9UNjkwTHc1bjlGcGxoZ0ZLVU1GWTctZkdLZU9zSGhEZEpKbXJnaWJfZjd2OWs3?oc=5</t>
         </is>
       </c>
-      <c r="E23" s="18" t="inlineStr">
+      <c r="E23" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1161,7 +1164,7 @@
       <c r="F23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1171,17 +1174,17 @@
           <t>Crescent Capital strikes Benson Radiology deal for close to $400m</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C24" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D24" s="18" t="inlineStr">
+      <c r="D24" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOLTNrWG1ZZlFoU3pDZ3E2SEgwMlhzQkdtQUYzaHZTZmYwU3ZhMnE0dlkza005VkZmZ09NMExlWDVncnBmYVVISXJ6X1ZjNHhpM2RnSlprY1dnbndJNUczcDVtNXNRY3pVNW12bm5rUVdqVmR4R0JlVHFuN0RwTlFkR2xrbFFpSl9jcm5oSjk3aFM1clBSVDhnbkhoWUREeUhsbVpvQW90d05xOTdfOV9nbW5POFdmelJkVlpsUlRuYl9odmRNVUV2S0pCMFBMTS0tcVhGVGFYU0h2d9IB3wFBVV95cUxPWEs4R2pxdThPbHJHb0dBT183SkRHTTlXNzdWazcxdkd1eGx2VlAyM2VVbEtEbWxTZ1R0TlBFRmRMZTFoalgxSmVVRUJFR0c0RFYzZVJFODg3dWxicU9pOHppeFhjaVp0WWlyTnUzV1dyZXdkMHBDVHI4LUVQdjc0cWpheU55NTlvdWdCZmVoODB0Mm5fbGNCTmQwLUhMZ0psQVpzb3BEUnJpSkRnOUM0c0VCdUp5N3g5MkhaM01vTHJ3NWd0ay02UXZUUG9nVkxicVc1Z0xjWGhjUDRDVjlN?oc=5</t>
         </is>
       </c>
-      <c r="E24" s="18" t="inlineStr">
+      <c r="E24" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1189,7 +1192,7 @@
       <c r="F24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="18" t="inlineStr">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1199,17 +1202,17 @@
           <t>Dual-listed giant Capstone Copper flirts with $600m-plus carve-out</t>
         </is>
       </c>
-      <c r="C25" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
+      <c r="C25" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNcVh4blRkQnoyaG1TajhVV0lrOEJRaHdTZWtzUnJHaEdaSXNRWThGTHlVdGl4dGJ1cTMwZ2pLcVNzUXRYNlZzVzhvaXdkNGtVUG0wN0FrMHB0R1I2Ry1jcEgtSWUtajI0cTFMRTlfdzBuMWtrZmJOLVUtMkl5dW85dFp6dEhEOHhTNzdfOFNFSGtlT0MwQnRlY0VhcUZBNE9RYzhQcDdOQUFnYkgzd0V0N253SQ?oc=5</t>
         </is>
       </c>
-      <c r="E25" s="18" t="inlineStr">
+      <c r="E25" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1217,7 +1220,7 @@
       <c r="F25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="18" t="inlineStr">
+      <c r="A26" s="19" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1227,17 +1230,17 @@
           <t>Guzman y Gomez unveils a new menu under $4</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C26" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D26" s="18" t="inlineStr">
+      <c r="D26" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPMjRjRTV2a3BJc3AzdDNOQktoYjBvLVZSODVsc3lKQ3pET0lxUlpkc05NcVlKRlZITjVJbjkwLS1DUFJNMGJ1amJKTlp3S3VqMWJaU3YtUENEN01rUEJiV1FNZTRXYjcyV08zZzlxNDVOSlVOTlJDOGV3QzBQcUpKa2Zab1ItNlI3ajZVVTF3?oc=5</t>
         </is>
       </c>
-      <c r="E26" s="18" t="inlineStr">
+      <c r="E26" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1245,7 +1248,7 @@
       <c r="F26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="18" t="inlineStr">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1255,17 +1258,17 @@
           <t>Can Sydney’s burrito king conquer the $676b US fast food market?</t>
         </is>
       </c>
-      <c r="C27" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D27" s="18" t="inlineStr">
+      <c r="C27" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D27" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNM0ZFcUpLN1dUZWUyaE1LMnNZVGlEbkNNQUQ4Wmd6QVFlTy0wZDVHdnlja1gzMEZTbVpKU1Ftb3VKZ2pzajcyWU16NUtUTmR0TlZMOVhMRUNqZXZiX2d2NWY0YlJDOFhhYUE0SkhMRUprNndXak8tWGdERU90cmMxTkFjcFFVSTd5VlZ3NFVKOXN3M255MFhzZThmbi1VUGMyQ3E4d2pYcFlJckY3QlVBdVJJeF9qUQ?oc=5</t>
         </is>
       </c>
-      <c r="E27" s="18" t="inlineStr">
+      <c r="E27" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1273,7 +1276,7 @@
       <c r="F27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="18" t="inlineStr">
+      <c r="A28" s="19" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1283,17 +1286,17 @@
           <t>Drone maker Innovaero prepares for ASX float, taps Euroz Hartleys</t>
         </is>
       </c>
-      <c r="C28" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
+      <c r="C28" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D28" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNU3JrejNRZ1VBZVNVV29NMkFPVmRsWE4yMVZPcjk2aUNUTHFJUGFyQ1VnZEZiZlIzQW9VVzRNNDNRR01jcHo3X0tqZjB4bzhMTTI0Y3BwYUh6OGRUUGt2REIxV09oRnJoVWlVelZWaUlWUmlPQ3dJdi1TejcyaXB1Z0x1MEJRSlB3SGMwVGdXaXJJNm9TVllPOG5JZC1feEV3TVhTeExGeHR2RHFIWlVCOXh3?oc=5</t>
         </is>
       </c>
-      <c r="E28" s="18" t="inlineStr">
+      <c r="E28" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1301,7 +1304,7 @@
       <c r="F28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="18" t="inlineStr">
+      <c r="A29" s="19" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1311,17 +1314,17 @@
           <t>Bain flaunts Estia 2.0 as IPO roadshow gets under way</t>
         </is>
       </c>
-      <c r="C29" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D29" s="18" t="inlineStr">
+      <c r="C29" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNTEN1cGsxNDN2c1NqUzB6UmJ4TFl0NGZjZVN3U3oxMlVFWTF4WUZLQS13dUxMV0N2ek1XN2VURTNVWms1NjdXSm0waEdaTXQwdTdWY1MxZ1V3ZnpEcVJtczdOWGNNZ0RQNzRZLU1MTTgtRW5DZkctbXBGMmVXVXdPZW5pNThiRHEzWnB2eFZzTFZTb1ZkeW9LendkNDd0cXRid05ZSGZYbW9NZXdOLVZWODdZU3hVcTA?oc=5</t>
         </is>
       </c>
-      <c r="E29" s="18" t="inlineStr">
+      <c r="E29" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1329,7 +1332,7 @@
       <c r="F29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="inlineStr">
+      <c r="A30" s="19" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1339,17 +1342,17 @@
           <t>Carl’s Jr. Australia unveils nationwide freebies for Happiness Day</t>
         </is>
       </c>
-      <c r="C30" s="18" t="inlineStr">
+      <c r="C30" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D30" s="18" t="inlineStr">
+      <c r="D30" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNVWgwdjU1NDFWalBfMTFYX1dQOWNDbG1FVUdlcS1LTVlHZVRRTVBWTjhSMnpkTXRXNlFJdllGQUp5Mm5ObWpIazd1d0RJa3QtdFBZN1hOenBmVzBEU05wM0gtNUxPeWpsYkxyVnhWWFFOU2Y3R0tXcmNkeWhpWDh2eDZBdjNCMHhuc1lHYTZHblBPVkpfRXpKd051UWlNc1hm?oc=5</t>
         </is>
       </c>
-      <c r="E30" s="18" t="inlineStr">
+      <c r="E30" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1357,7 +1360,7 @@
       <c r="F30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="18" t="inlineStr">
+      <c r="A31" s="19" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1367,17 +1370,17 @@
           <t>BHP and Woodside appoint new CEOs in major mining shake-up</t>
         </is>
       </c>
-      <c r="C31" s="18" t="inlineStr">
+      <c r="C31" s="19" t="inlineStr">
         <is>
           <t>ABC News</t>
         </is>
       </c>
-      <c r="D31" s="18" t="inlineStr">
+      <c r="D31" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQbTg5VFJLbWJfcy1uV3ZReTJkTndzX01qZ2MxNWkzaWZRckNLZUR1Y1VsMVRNc2FySC13U0NzalFEb3k1R3BaUEhfcTV0N1M4Q1dpSlo0YXI0UFhrMGRab2RiYV9DQVNVX01ycFc5ZFZrZWZqc1VRZXoxLVEzSDJLclJLSWg5bzN3R1I0bG9lWjVDaHE4?oc=5</t>
         </is>
       </c>
-      <c r="E31" s="18" t="inlineStr">
+      <c r="E31" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1385,7 +1388,7 @@
       <c r="F31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="18" t="inlineStr">
+      <c r="A32" s="19" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1395,17 +1398,17 @@
           <t>Next Capital sells Enviropacific unit to French waste management giant</t>
         </is>
       </c>
-      <c r="C32" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D32" s="18" t="inlineStr">
+      <c r="C32" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPR3lFbERLR2FtdmJUU3BDU2thZk00YmFHRFhXR2VBVXhQSURTeE5ONVJKczBwbzlFMnR5cmhxMnM0bzlJbWo4SXl1dHpqYWxxMUJBRjZHVUtab1RYZjZMTnpGc3FzMWQ2NjNEdGU3NTZwa0diM1lJS1haYllwTldLZlpZbXp0YzlxcDh0ekcwTy03dDdPcnk4b29HZVdqbHhZY2JPR2drM2puSVpjUzZkVjNpZUE4dVMwYlE?oc=5</t>
         </is>
       </c>
-      <c r="E32" s="18" t="inlineStr">
+      <c r="E32" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1413,7 +1416,7 @@
       <c r="F32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="18" t="inlineStr">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1423,17 +1426,17 @@
           <t>Future Fund private equity and real assets chiefs head for the door</t>
         </is>
       </c>
-      <c r="C33" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D33" s="18" t="inlineStr">
+      <c r="C33" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D33" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPUHNHRFhFMVdwVld6RFRZUFd3QWNOd1kzeS1QdnJxMERFSnE5LTdZcDhDYlVGcWZMeWxlR0FSRWF6YkZoQVZrZU9TQ1E4YTEydUJnOFE3enV5Rmk5UnF5VEdYZ1FMUWpKVjdjMlZZUGFsU0tKcV9Vbl8zcHp5aVF5Z2JMOUZocHJqRXNRaEp4Nm5CbDM1WkdIMHdQS2xqQnE2Tnh3?oc=5</t>
         </is>
       </c>
-      <c r="E33" s="18" t="inlineStr">
+      <c r="E33" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1441,7 +1444,7 @@
       <c r="F33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="inlineStr">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1451,17 +1454,17 @@
           <t>‘I actually started to die’: the new billionaire’s epiphany</t>
         </is>
       </c>
-      <c r="C34" s="18" t="inlineStr">
+      <c r="C34" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D34" s="18" t="inlineStr">
+      <c r="D34" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxPblkxbHVrdnVKY1pqQzNyWGNMZm9UYmY3dzlPaGQ4Yi1tc0U1akhrVWdIaXBpM05aZXRwTXE1eDBITlZpbDkwRXNrWjJ2YXBzX0VCY2JSLWhrVmpjSTE5eE5rLWgtc2pRZEdXbmhhWU1KeFExZDBGS2pjSkIwV0FGbndBZVAyQkg4WFRsengzSGYyZkFfQnJsQ18tUHJGNDd2T0pzZElPSVJTQkl2Rm5QTExJNHhmU2dHOHJGdTdzU08yNHRtd1R3Q0cyOF8taDktQTZvVXVBVjN1d0NHMmtFOHBWZXBFcUFWa1IyWGNDTDZUT3lQSXJHOVhxTFQ3b3RH0gGGAkFVX3lxTFBZQ3BFQWl5dEwwLW5yVWJuMU8zcXBPdE9pamRVSWVkbWNyVzgydGVOaDBROUN6RlBDbjdld05DVmZyb0R1eEN0UERubzZRU2NiMTQtVV9XNS1wYmlvZ1paM3RaOUlrTzJka0tXVVJEamFESGlSdXg2bDk1aUdhUVhBcXpnN01fX0Y0cTNvcm5DdEFFLVVERDFKTWxKZFR0UzAyblJqVHBua2JoYUdzeUNMb053ZVczWUFQU1AtVHV1d3lSSDFfZFh2cEkxSGw2MEdicEVsb2pLQ1RuQmdaRl9xNUROS3pKR2s2T2wxTTZ5bEwtTUNQNU04djFHTHlPbXVLSW9YSUE?oc=5</t>
         </is>
       </c>
-      <c r="E34" s="18" t="inlineStr">
+      <c r="E34" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1469,7 +1472,7 @@
       <c r="F34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="18" t="inlineStr">
+      <c r="A35" s="19" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1479,17 +1482,17 @@
           <t>Ironbark shuns private equity as it hunts for cash injection</t>
         </is>
       </c>
-      <c r="C35" s="18" t="inlineStr">
+      <c r="C35" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D35" s="18" t="inlineStr">
+      <c r="D35" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxQZWFaeVhldi00VkV5ZmEtS2tjcWdFWG55OGpCX3IyN25Rb3ZFV0ZKVm1aSE1WbThoYVY4ZEdfODVGX0RaUDV2Ul9HS1JQMDFCT05Fc2FaU0RINTMwbDRveWFsOFJSM2ZqTU9tVGxJSEl2ZmhhUHFHT3dqYkk5TUtvMUQySnZzTWw1MzFNWl9aVzhkSEZ4Q3YyWjRMUmpIdmJkdUVKWE54Nkt6bTd2dGFSUFoyNkgxTHh2TGVGak9ja0dFZ0xQM2g0S1lmQkZiWWtUcTVNdHhBdC1KeVRQcDA2dnpmeHRkWEnSAewBQVVfeXFMTWtYRDRSaHNULW1HanowRnpMdFF2VVMtZW1SV2ViZXlGaW02WlIwUzRZMGg5WDNrOUR4eDlGOEt5eGlqV0pfVDFhb0JEcS1faEJodWxyRnB3MkozOVJyT3NvM1I5MzdDcXNnUFNSdkRDamUzZTRQYlk0c1VIQUNMZ2ZzOWVCb2V2MC1aSTZLWkFkbW9GYk05b3RmN1htWENTeDh3SU1WYWJMcWx2eGUzZmwwVXF6czlnRGdXbE1vRElyVG0yM0ZzXzZ5TFh1YlRGNU9MQ1p3NnVZSFB0M0xBcGlueVZILXlVaXdqUkU?oc=5</t>
         </is>
       </c>
-      <c r="E35" s="18" t="inlineStr">
+      <c r="E35" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1497,7 +1500,7 @@
       <c r="F35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="18" t="inlineStr">
+      <c r="A36" s="19" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1507,17 +1510,17 @@
           <t>Minister leaps to fix food chain</t>
         </is>
       </c>
-      <c r="C36" s="18" t="inlineStr">
+      <c r="C36" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D36" s="18" t="inlineStr">
+      <c r="D36" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxOd2NqakVWRnQ4anFZNkl4Zy03MkloX08tUkktRTZqeEtQWFZJeVhkMUJIb0FxUjc2UjhCQ3MxbmNxczNxblJIZ09IeTBGNFM4Wkh4ZE1qNkhJMjIwU2RtX1JxcEV1Y0NjWXF6eHpVdTN4ZUlYMGIwcDJzMXZMTk94VzFlcjhpcVZVSTJFMjhsQjVGWEJQYTQ3aTFyNmNEZ1F1b3NGTWd5WnFJWmxXSTJ2NlRLcjJHNWkwaTZ2YVR6S0w5WVo1Vlg0VWdxcWZoa3VaTmcxY2NVcnR2bFRWNGNvZ1M2Tlg5NzlvVXZFZm9B0gHzAUFVX3lxTE1uNERoR3p2dXRIa0g0RXI2MWR6N0c5U3NGcjFDQVMtdEpyNDI2bk8yOS1qUnFOazdiODl0Ymo5R1pwRVJ0UFFVdzlhYjRDSUFCU0FRak4xcVVrTHphdTdxcHNIMnEyRVZud1FURmh5T0JLOHpRM3lFbDRuRnZMYmtaRnRFTXh3dkszTFhFUmZlRmoydnlEbW1fZTlmUzh4NXNyeTZTeUhOSktvclJVc0NTZTVYMkdJZEUyY2RmVC1kQ1hwVEloSEtVMEo5QnNTUXQyME5IN1BPd1NOS3oyR1JtMHBFVTZEbzhEQmdrWUk1ZnZVTQ?oc=5</t>
         </is>
       </c>
-      <c r="E36" s="18" t="inlineStr">
+      <c r="E36" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1525,7 +1528,7 @@
       <c r="F36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="18" t="inlineStr">
+      <c r="A37" s="19" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1535,17 +1538,17 @@
           <t>‘Brace for swings on every tweet’: Investors bamboozled by peace talks</t>
         </is>
       </c>
-      <c r="C37" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D37" s="18" t="inlineStr">
+      <c r="C37" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D37" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOczZHTWFmTW9FZ1ZwSnc5Z3ZacGpsVDQ3LWw1a1BFT0tjRkphek41MlhNOU84emYzZUVwNV9xM0hyc1FUR0NHck14Qnh6c2JvQks5ZE02ZTNLWDI0dy1STi1HbDFDWW9yMDhGQXVVVzdkMzFXcnNNMVZHVXFMUXUteGtsVGhPVmhLcVZPQzlhTWNoYVVRMHF0cFhybWxzek13Y3ZjcjlXWjZJM2VYbm0tTmk4NExLQzQzX1ZPMVlhcnJxQkZx?oc=5</t>
         </is>
       </c>
-      <c r="E37" s="18" t="inlineStr">
+      <c r="E37" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1553,7 +1556,7 @@
       <c r="F37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="18" t="inlineStr">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1563,17 +1566,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C38" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D38" s="18" t="inlineStr">
+      <c r="C38" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D38" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5</t>
         </is>
       </c>
-      <c r="E38" s="18" t="inlineStr">
+      <c r="E38" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1581,7 +1584,7 @@
       <c r="F38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="18" t="inlineStr">
+      <c r="A39" s="19" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1591,17 +1594,17 @@
           <t>Wirth’s Myer rescue mission is caught in the eye of the storm</t>
         </is>
       </c>
-      <c r="C39" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D39" s="18" t="inlineStr">
+      <c r="C39" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D39" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNTlQ4NDRnWE91VG1YNENpSTUxNnBjZkljOGdYaGV0aVB5dkVOaEJ6SjZ1bVA4NXE1S1hjV1NjcVhQTEVpWEVNV0UtbzhQTFZLOWxIenZiaF9QM3F6bmJYRy1lbXVMczZ3TnBHNy1aLUtVcnBDdkl4TE0zRGN4U0FwSjNPY1M5S3AtdUQ3UUNmR0x4MlU2YXRuUDJEUm01SmZWakx2UjFvY04zRHk4Smc?oc=5</t>
         </is>
       </c>
-      <c r="E39" s="18" t="inlineStr">
+      <c r="E39" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1609,7 +1612,7 @@
       <c r="F39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="18" t="inlineStr">
+      <c r="A40" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1619,17 +1622,17 @@
           <t>‘Darling, I’m not going anywhere’: The rise of at-home care</t>
         </is>
       </c>
-      <c r="C40" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D40" s="18" t="inlineStr">
+      <c r="C40" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D40" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQS2k0M2otaldpNVFXdHRTMVNtZVhyUDV4VTNIcE5FSnFRaHNubGNQQzBVbllnNTktNGhrZ1lndzV5V1FpUS01SklRaTZmZHJkRzVsQmlsdEVmenZ4U2x6U01NeXdIMktBUW94TUE3R3FoLUxVcVhsVFI0SjVQVUFaZldnd3prMWMyaVRWX2J4aUdfQ25KWHpaLUlqSnhvQmM2TTRRQldGbm8tclFYRDA0TVdnU2g3QQ?oc=5</t>
         </is>
       </c>
-      <c r="E40" s="18" t="inlineStr">
+      <c r="E40" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1637,7 +1640,7 @@
       <c r="F40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="18" t="inlineStr">
+      <c r="A41" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1647,17 +1650,17 @@
           <t>Iran targets Israel and Gulf states as Trump looks to calm markets</t>
         </is>
       </c>
-      <c r="C41" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D41" s="18" t="inlineStr">
+      <c r="C41" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D41" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPLXBITXU3WTRtc0NYdnhTZHFaUTBCSXdldTBuSHliTlY1dlJONW43Qkd6Nl9pNmY1eDhzaHZoX19xYjBxMXR5UEhkVUg2M2k1MmhuVEwyY0JxbnJyemxVYUZjbk5BbkN4ajhPbW9ZeDhlRDRYTW1hN3k2d084c2djMEJUZTV3NVdPbllKUmFlU2JsaDV3Zk9CVFF0VDFkV09JSloycWdOUlVrREptQTJfa25LUEx5djA2SjNMMFY0RjM?oc=5</t>
         </is>
       </c>
-      <c r="E41" s="18" t="inlineStr">
+      <c r="E41" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1665,7 +1668,7 @@
       <c r="F41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="18" t="inlineStr">
+      <c r="A42" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1675,17 +1678,17 @@
           <t>Meet Christian Louboutin, footwear’s most famous billionaire</t>
         </is>
       </c>
-      <c r="C42" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D42" s="18" t="inlineStr">
+      <c r="C42" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D42" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPcXdGd0tMckYxbjZ5TVJmQ0Q4NFl2RkhHMHdlZDZsdGZ6cVQ0cUpaLWJTNlVoc2ZOQmtXNlFTRnJVMnVDTGc1NFNZN2g1VnotQlNQbzhlM1BJV3ZwQktOcGtac3RwSHRLZkR0b2l0eGIyVVlYdHJrc2hpT0pJbDR3LURPTnowZk54LThObndtMVkwV2VWQkluNVlWY0p4QVJGbE1hSGMzOW8zdkJZOWdocEZQWFBhTllNR1ZBSEg1TWRXUWd3X0t6TVcyY05PM0pF?oc=5</t>
         </is>
       </c>
-      <c r="E42" s="18" t="inlineStr">
+      <c r="E42" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1693,7 +1696,7 @@
       <c r="F42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="18" t="inlineStr">
+      <c r="A43" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1703,17 +1706,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C43" s="18" t="inlineStr">
+      <c r="C43" s="19" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D43" s="18" t="inlineStr">
+      <c r="D43" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQbHdYM2pSM2xkdmZ3OHhQc2tVUmhzclJWaVJ0aEwtUkNBR0ZUd3p1emF1M21jbTF1ejlKSkdDMnotcVNjZE1CYUlKako3WXR4MTJhdWNlSXZMbTBYanlmTWFzRGFIandXRUQ3UjN6SEV1bThvZjN2bDY0eFdpaTdMODN6TGFTdE5rd05TUll3MmNfTDhkQldoNDIwVlpoSl85aVRwcTd5Ymh3TDl4enZhZ2p4OExGY1ZaOFNEWFBB?oc=5</t>
         </is>
       </c>
-      <c r="E43" s="18" t="inlineStr">
+      <c r="E43" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1721,7 +1724,7 @@
       <c r="F43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="18" t="inlineStr">
+      <c r="A44" s="19" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1731,17 +1734,17 @@
           <t>Sembcorp Picks Banks for $2 Billion Alinta Loan in Aussie Push</t>
         </is>
       </c>
-      <c r="C44" s="18" t="inlineStr">
+      <c r="C44" s="19" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D44" s="18" t="inlineStr">
+      <c r="D44" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOdS1aaXZjT2VnSDl2TDdzZ3NfRElDWXdUXzZQYjFQMEZJOGlpaE5CNGdQMlZ2UFVHbUtfOXF1ZVBReExrdF85M0RWLWlBY2Y5dlRtWVdXLWp0Y1VrRmF4UGQzVUhxaHA4UHd1SUdFV21QcVFITXFHRlhzekdSUS1PdHlYRjdUbUQydU8wSktKVHRJQ0NaWE9sU1l6YXhtSWtBd3RwTERacnV4VzB6YlFhUE1QcXNDVXVESFcyeWY3cGhHUkRJcDhrYUtpTEY2UQ?oc=5</t>
         </is>
       </c>
-      <c r="E44" s="18" t="inlineStr">
+      <c r="E44" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1749,7 +1752,7 @@
       <c r="F44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="18" t="inlineStr">
+      <c r="A45" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1759,17 +1762,17 @@
           <t>Navis targets June for $1bn-plus med-tech auction</t>
         </is>
       </c>
-      <c r="C45" s="18" t="inlineStr">
+      <c r="C45" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D45" s="18" t="inlineStr">
+      <c r="D45" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxPNHRXaU5tNUVkd2MtcTg5M0EyQllrM0owMkZobGxLaUJxYUN2MUg0ZkdKdzU2YmxfanR3QU53cHZzNDI1WXgzRUcxOE9EZlluNmtNRUUzTGJPRnpfVVVOeFM3bFRNQmp6VHFBdi1mTnU4UDBvOEpMaHZPNXFtdUIyTlhuRExIVElSeVRUMGxjU0k5VnVxaWFfd3htWngydlhuR2E5aTQ5VW1LS01ac05rMGZoVFdOZzVyTzFhUDVsYkNrc0VQZmhubERSaTNwelk3WEhYUjF5d2ptMktYeEhzOHpWazFQZXphd0xfUFdhbkVGMVR2Z1dtVtIB_gFBVV95cUxObEwzeHd6RmZtNUp2dXVVV0plOVQ4WlNqQXNJU0thd1BEWE8yWkxxVTZjTkpsVGxxWGxpQzN0OERZbk91ai1fZkdtc0JoM1h5NERLTVdDbVJ4Y2k4djdQcWlVcDF6NjMyVDQzZWMzUFZxWjVRWllMZHVSOF9jQ2U1REFfNUlhM2EwYloxb1MwSTJjODdWdlZwX2h2N0xiQWNhallHUTNPZEtLaXhsY3dBZy0xM1VITXhLUERXS1JxR0R3OUpBTVBPZ2dPZTRUTVpvbFBNMjFUSTJuWS1XLWdhUS11UTRzVTVqaEhfMDhqWHlTMlJGekU2QzJVcFdodw?oc=5</t>
         </is>
       </c>
-      <c r="E45" s="18" t="inlineStr">
+      <c r="E45" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1777,7 +1780,7 @@
       <c r="F45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="18" t="inlineStr">
+      <c r="A46" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1787,17 +1790,17 @@
           <t>ExxonMobil eyes New Zealand market exit</t>
         </is>
       </c>
-      <c r="C46" s="18" t="inlineStr">
+      <c r="C46" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D46" s="18" t="inlineStr">
+      <c r="D46" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxPanlvR1V1eVVpdmYxNVNGMnd6UjJFd0J6Zk9IU1lhOW1GbmVTcjY4QkJCYkl3Y3NOU25VRTBUekwtS3plV0NVdlZtOTZZRHJWZ0FVdDl3S05aMlFWeEZiYzdwYmQtVnJxZEw0NktHaFZMNlZkUC16empqRGxxMEhhZGwxRzVEek5FelB3aE9UWFhGQW42b21MRnJHUXV2ZGJYUXJIMnVFWGZsSnEwazNGNUdVcjVoekp0NEZCN1J3cTlaZldFa1pMUkJTbVZYeFljVkRqQmlZV1M2aXh0ZjI5dEI1NDB0UElPUERsbUljMlA3OHBnYmtJTXFWZWkyUdIBgwJBVV95cUxNWFBRQ05GUDdwTWJ2ZVFJUS00ZUh0QkpZQVNNcU9JYXRTN21sMS1VZTlOSTh2LVFuZHh6UVk2djlrdWFsd3MwcDFCNmhwUlVLTlpjVF8wSmt1YnBWRE9tNVpKQlk2YXJWdmwzZWlLX0xpaWxSMUpsX3ZjYXhmRmE2YlAtSFJGRG5pQnVmMnViQXlsVFV3OU1hZFVrY3ZITHQxcTR5UkZ5U1pReHVJMGZGM2FCZWliSFZQZmpVLThSdExWMW14OElodmVVSC05SUh1d1hBenJoY3BUZGxoM0NTbTExdERmM3pjZGd4VzgyV3BNOG11TElBQ3NsRGhtSEc3YzJz?oc=5</t>
         </is>
       </c>
-      <c r="E46" s="18" t="inlineStr">
+      <c r="E46" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1805,7 +1808,7 @@
       <c r="F46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="18" t="inlineStr">
+      <c r="A47" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1815,17 +1818,17 @@
           <t>PAC Capital’s Clayton Larcombe charged with assaulting wife</t>
         </is>
       </c>
-      <c r="C47" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D47" s="18" t="inlineStr">
+      <c r="C47" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D47" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOLXNDU2xjMWpyeEZwWGwtZkV0TjNSbGtWS3ZidUo3a0dvV1hrTnJiVXBXSkJNWlhXYXFHZkNTa3g4a1ZfMjRPM3BtWTZUNGg3S09kbGI2TTRGd0Jkc1A4WFAycjlpVC1URjFvNnBraWprRkhaT0VOWkh6N0xkUjNXNUw0dGx2N1JtTDVsREdtZDhraXVsSkxhR2ozamFUSGR5VHBBRm1Zcmx1c2RDaUIxQkVpeUpfWjFNeTRLWVRtYjluZ3ZncGZIMQ?oc=5</t>
         </is>
       </c>
-      <c r="E47" s="18" t="inlineStr">
+      <c r="E47" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1833,7 +1836,7 @@
       <c r="F47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="18" t="inlineStr">
+      <c r="A48" s="19" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1843,17 +1846,17 @@
           <t>China touts itself as ‘harbour of stability’ to global CEOs</t>
         </is>
       </c>
-      <c r="C48" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D48" s="18" t="inlineStr">
+      <c r="C48" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D48" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPUzBWeVk0elBOZ0l5QU44TUJvU0RvSmtPdmVyT2VuQTczaEdzbkktT25ZT2Y0Nzh0bVBhQW96TUhpWkdEOEJMVVk2UWxLOENKZGk3X2tQcDNsWGZtU0JkM2U0N3VfUWFBclhUSUZya0NwRTJOWmZJdWlhT3JtY1EtSkJ6TmlsV3dzOXpDaVFMNlBaa3RfRHBjc3Q0cjk0eVdPV2MwcjlHNA?oc=5</t>
         </is>
       </c>
-      <c r="E48" s="18" t="inlineStr">
+      <c r="E48" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1861,7 +1864,7 @@
       <c r="F48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="18" t="inlineStr">
+      <c r="A49" s="19" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1871,17 +1874,17 @@
           <t>Eyes on 3D Energi as oil and gas giant Conoco flexes buy-out rights</t>
         </is>
       </c>
-      <c r="C49" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D49" s="18" t="inlineStr">
+      <c r="C49" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D49" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWVU1QmhTUGFkYlpTQkw1WUFPTHhmbk5lbnE4T1haQUswSi1ITHlhVmhyM3ZYS3N4cVd6ZkwzdGdhT1lvM1JJek4yLXFpSWoxUnRtR2JRLTZWa2dlTDVTakE3b2xvazFWX0kzRHFZWVB4OUh0XzFFd3JVSVlfelpVa21qTldCVHdvcmJYcGNjZ1RrdElWS3Yzck9KYzRvbzloWkNqMnQ3dmtHbzNuc21ZSXNYeEFlZw?oc=5</t>
         </is>
       </c>
-      <c r="E49" s="18" t="inlineStr">
+      <c r="E49" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1889,7 +1892,7 @@
       <c r="F49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="18" t="inlineStr">
+      <c r="A50" s="19" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1899,17 +1902,17 @@
           <t>Blackstone tempted by $900m payday for Sydney’s JPMorgan tower</t>
         </is>
       </c>
-      <c r="C50" s="18" t="inlineStr">
+      <c r="C50" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D50" s="18" t="inlineStr">
+      <c r="D50" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxQNEZTZjY0S2YzcUxsb25RSDk2NHd1N1VOVlpMbi1JNGEzbUt5ajlYZFhvLWNBTkNQVXNuWERfTkl0Z2o4R1U0Zk5jVE1FTW5TTUJGZnNJc2NqMm1fT2dmYTVwRGU2TkZ0c3BjZVBGS29fWFJvZ2F0MWNLa0pYY0RNME5xYS1vOGZmMDVBcDBaLV9MWF9od0EwekFyb0ZCOEdkNTFaN3ZXckJwd25zS0FsdzU4OW1UODlueGNyZVBDSDZkeHQwelV5ZXVDVlcyUkhKWDZfVlRacEJHSElmNnhKSXk4ZHJHWHhPTEV5NGNkcmhyU0hjV3J4dVBXbnRGQdIBgwJBVV95cUxPME4ySFF5RWNrejVlWW1yeW56N244RGpyeVJUZEgyTjFNcE10YjVpMmJyeWsxTENzZFhPRlpsbl9pVXl0NGJvUlZFT216NE1KRFNwOHVZVXMzanNKNXFmWEdsMndsd1cza3NTTzUyUUZfaDEyWHJwZEtQbTdJRmkyU3A0RGh4QlAtT1lRVXk2SGoyaTI1NUpwVExYSkZJNmVFNjdXTDJTNURFOEh4Y1dnUDVGdjBpaDlWVWJtUHZiRDdGTmE5R1R6TDBwWFFnT2MwQ1lmT2w5bDF6eVU0R20tYnpnT3JCZlJod2s0UndyZTM5M2xLZC02a3E0NmJRdFV0Qkow?oc=5</t>
         </is>
       </c>
-      <c r="E50" s="18" t="inlineStr">
+      <c r="E50" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1917,7 +1920,7 @@
       <c r="F50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="18" t="inlineStr">
+      <c r="A51" s="19" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1927,17 +1930,17 @@
           <t>I-MED attracts mystery suitor as Permira weighs sale or IPO</t>
         </is>
       </c>
-      <c r="C51" s="18" t="inlineStr">
+      <c r="C51" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D51" s="18" t="inlineStr">
+      <c r="D51" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxNaGlwS3d5MGFMbEg2U2hnZUxMQmdqaWI4bS1lblNZOFhkSnRMcUotRkZMTjhFZkRUQWxUUDVtYml6TVAxUXkyZmx3SHRFb0gzVHRST2ZQUThKa25aWlhlcGprSU9tWktXZjZRaC12bFpkaVVWZHhIMERyeVNNWEswYTJ2ZHdnRFVRaFhod2U5N011TkQ0NG5MYVhoT3MwRUVZdVB2UVhKZExvdFIyXzNNUGt2SHJUanQxRkI3bXlLSlNJQTF4NXQ1YlZDaGVBM0EzNUhYQVp6NkFWRzU4bnRPWTgtXy1HVnB0ZlN0Uy1rY2FuWlNfN1U4WXVHQnRzVkNG0gGGAkFVX3lxTE1GaDJJdTJlOXFEZUtDTmdXMmsyLXlpaUxzQXpycHk4MTdHZng0dVczYWVwdWRzdFFCMlNLWkZpMm5Zd2RpN0Y0Zmo3Q1FOZFBZQlh5LVl6aVZ3X284UmpxM0pVRzZmMmpjaUdNWnJPZGV4V3lNai1CTllCcW5oUEVxaG0zejB5anc5YnJEZzZPT2d2QklCWjl2MjRBc25jUndqZkVadllKaUZScG12bEozT1NKUUJYR0pHTGtJZVc0ZHZLNHVSYlhzcTE0SkZmMXNlVGJ4YWJ1cThxcGlZTDMzRUMxLVM5VHh2OW5tRW1PT3VyRUhDbV8tRzUzVzRzVWZPZ2w1bnc?oc=5</t>
         </is>
       </c>
-      <c r="E51" s="18" t="inlineStr">
+      <c r="E51" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1945,7 +1948,7 @@
       <c r="F51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="18" t="inlineStr">
+      <c r="A52" s="19" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1955,17 +1958,17 @@
           <t>The stagflationary mix that has billionaire Solomon Lew worried</t>
         </is>
       </c>
-      <c r="C52" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D52" s="18" t="inlineStr">
+      <c r="C52" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D52" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPWTh3S05XQWpTQm03WjhBT1pWc2cyOFRMd2ZraHhPUHlDRW1tWkZvdkhQWHE0MHVMRUpaOFRoX0JsYWhJV21nVkpIM2RBSmlZRUtEbFAydzZfOTh1S05oNEZPOGgyZDJRMS1uLThWYWRVT3VEVGhtYkVLN3J2OWsyX0VVdTUteFBCOVNKZ28xUTRPTk1SUkMxZ1NJc1B6NXRrUEEzOG01YnZOYjk2cWlFZA?oc=5</t>
         </is>
       </c>
-      <c r="E52" s="18" t="inlineStr">
+      <c r="E52" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1973,7 +1976,7 @@
       <c r="F52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="18" t="inlineStr">
+      <c r="A53" s="19" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1983,17 +1986,17 @@
           <t>Oliver Curtis on Firmus: From prison barber to AI billionaire</t>
         </is>
       </c>
-      <c r="C53" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D53" s="18" t="inlineStr">
+      <c r="C53" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D53" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQek9VTlV1b2hVb2RoZ0Fya0REb3E3YlBCR2NYZldXcEh2VEY0LXg5bjd6RzlnZDI0OUJJd2cydTBwTm9tdHpiZ1lSMnhtcmJSYVRKbzJFMjdDaEJyZExSQVJVRDh1c00yMjFMaVlPdnRuV3VkTjNxdzFRbW1yeGltSF8tVXlJVXJzTEJXS2FTYkJTVkdKbmdPTTd6YzRtYV9nN0JzOVZNTzhUdUk?oc=5</t>
         </is>
       </c>
-      <c r="E53" s="18" t="inlineStr">
+      <c r="E53" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2001,7 +2004,7 @@
       <c r="F53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="18" t="inlineStr">
+      <c r="A54" s="19" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2011,17 +2014,17 @@
           <t>Three startups that raised $161 million this week</t>
         </is>
       </c>
-      <c r="C54" s="18" t="inlineStr">
+      <c r="C54" s="19" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D54" s="18" t="inlineStr">
+      <c r="D54" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNRGVZMF9DeGJjX29vN3B0blVoM3RKSlJJTllrMThKUDJNZzdPNFNnT2JyTElUOUYxMHlsUm9yM2dBQnZfaVNZblpqb3NzTXdHVlpQNkRqR3NBZHdzODdjN3RKMTZhSVRqUEM5d3JRc3F2OG9hWmZJdU5rakg4ck8wLXlMTnZSU0lNaERmQmswbkVGWW8?oc=5</t>
         </is>
       </c>
-      <c r="E54" s="18" t="inlineStr">
+      <c r="E54" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2029,7 +2032,7 @@
       <c r="F54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="18" t="inlineStr">
+      <c r="A55" s="19" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2039,17 +2042,17 @@
           <t>Iran eyes ‘plenty more’ vulnerable energy targets in costly war</t>
         </is>
       </c>
-      <c r="C55" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D55" s="18" t="inlineStr">
+      <c r="C55" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D55" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNLUN1MHlZaTNfVHhVX0RnTXp5QW83RmM4WVZkWW1PSnNaZF93VkY5ZF81anB3NDNmX0kyMkVSdkxNSURvSEh6enloWnRVcTlsR0JPTjVzNFR1YjRsSm52VnA1XzFFUlUtODJjYy15YWRRdWZZRkdjRXpCcEFSVURmV3VpSTFhTjVUb1d5bmw3NHNlT3VQZU9ieEYwM1J1TGEyZnlnWXNIWFJUMEtIOVZad0dxRWZBdw?oc=5</t>
         </is>
       </c>
-      <c r="E55" s="18" t="inlineStr">
+      <c r="E55" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2057,7 +2060,7 @@
       <c r="F55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="18" t="inlineStr">
+      <c r="A56" s="19" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2067,17 +2070,17 @@
           <t>Don’t take it personally: Bain Special Sits hits hurdle at Infinity</t>
         </is>
       </c>
-      <c r="C56" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D56" s="18" t="inlineStr">
+      <c r="C56" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D56" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQRjdwTk0xTHVIRHNkdG9tVk1EQ0hiQjJ6dGcxaWZRZ0hZV1U4YjJDU0tnTUlWSkQ1S2dUTHJVNk0tNWQ2cVd4dkw0M25leXRreWJtdlBKYTAtNzRocTJUazh1dnRzSVlYZThySTBNVjg5X0xYWUxCMC1SelltSHVSUEV5U3B1bTA2NjAzMGFZLW1CNkQ3aWU0S1JxS0d0YmZiZjBKQVRNVUpzYno5R1pvbTBsaTM?oc=5</t>
         </is>
       </c>
-      <c r="E56" s="18" t="inlineStr">
+      <c r="E56" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2085,7 +2088,7 @@
       <c r="F56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="18" t="inlineStr">
+      <c r="A57" s="19" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2095,17 +2098,17 @@
           <t>Drill, baby, drill: It’s boom time for mineral and petroleum explorers</t>
         </is>
       </c>
-      <c r="C57" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D57" s="18" t="inlineStr">
+      <c r="C57" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D57" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNdlFOWld5ZWhPVnFRa2xidWlUVzluQzkxUTgxR0t0Rmg2S1BzNjdINnhwS3VLRkNjRVJLX0RHU0h4VFVRY2RfSHBudEhfNVNjeE50ZUxQenJNSlJtWFRlcnNsZm1iLXlxM2RmVDViWEtjNDloaTBhUDVxYkNfOWFCTjV6cExEVlFCMzNfWnVwRDJHYWxWV0hOR2V2S0VlV2NyS2s5cWNmREtWXzlMMDRQNW1tVlBOblp3SHBEVg?oc=5</t>
         </is>
       </c>
-      <c r="E57" s="18" t="inlineStr">
+      <c r="E57" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2113,7 +2116,7 @@
       <c r="F57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="18" t="inlineStr">
+      <c r="A58" s="19" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2123,17 +2126,17 @@
           <t>‘Wake up’: Fury as farming crisis looms</t>
         </is>
       </c>
-      <c r="C58" s="18" t="inlineStr">
+      <c r="C58" s="19" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D58" s="18" t="inlineStr">
+      <c r="D58" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNelJvMXFPX3MwUVRMN2xqbzE1MWdvOF92Zy02YmIyZW9SQXRNQVZsS0xVVG9UdkFPaTV6ZC1tV05SZWNqblNFZ3Y1VGNaVVBaaEl6aFJqQ09ONDVkNUs4TzNvVjV5eHNjUk9xaDRFZTM0alpuYUdvWGtLRzRhYXN5alZ1QWdsZTEyODdQVnZoazkya29WeTJZVmpxLVBCdWxfY0dTN2Z3WFZlSy1sVW44RDlvZFAzYlhnQ0N6UWhKSU02eF9iZllIU3g5MWtSbkJzZGxWLUxHNERzdUlLTF9VYmpJSTRLY3U4NlVVaDhmc09uOWwtUGtlb0I2M05DR1dnRWxGSFV2NEJXaEF4c00tN9IBlgJBVV95cUxOSzZ5NXZMTTlZa3BSNjZyTUxUMjRhYWJhN0hMa3dDcW9CWGstNnI5MzV5U0hJSTdKLTFwa2E5YUItZnFRbW5RbzVuYW91MmZaYXN3R25hWVpUbW9oUU9fVktPRHROVDYyd2dSLXJVZWQtY016bkVxY0VPbkY3Zkgtb1liWGMxeEpyYmloS1V0TVJMMWZaeWRZX3FQRjBmVzJwdkkwMEVDSXV1MTdReUhGZ0Z3dENyMEFkLUl1aXhtRkFLRFFXcEdMZzFuT3NxRDFMOGVaY2YzeXBQc09fY3YwcFp4MVczRVN3d3dJZWJfTFFscjF0cUtRWHdzTUptaHowNDhYWXZXTHhYTHNTdlZGUmNlamRTdw?oc=5</t>
         </is>
       </c>
-      <c r="E58" s="18" t="inlineStr">
+      <c r="E58" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2141,7 +2144,7 @@
       <c r="F58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="18" t="inlineStr">
+      <c r="A59" s="19" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2151,17 +2154,17 @@
           <t>Construction giant FDC road tests IPO pitch</t>
         </is>
       </c>
-      <c r="C59" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D59" s="18" t="inlineStr">
+      <c r="C59" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D59" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxON3p5Y3VPM01XZFk4a3g0R3JnQkZXbHVGV3BKdDB6M3NRb0M0SEl3V0R5RmhCQ3dnaHB0ZHp5N2hCMUFsNU1ZNWZ4YWdNZWdETkUyZmdoeW81amwtTWNFZlc5WlNpMkJwRzk0QklORGhlLWNEalh2d0JCX0lhVHhhUF9ibVlxcHAwOW9ENndVOTY0enBYUWc?oc=5</t>
         </is>
       </c>
-      <c r="E59" s="18" t="inlineStr">
+      <c r="E59" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2169,7 +2172,7 @@
       <c r="F59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="18" t="inlineStr">
+      <c r="A60" s="19" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2179,17 +2182,17 @@
           <t>Austal suitor Arlington Capital Partners buys Eptec’s defence unit</t>
         </is>
       </c>
-      <c r="C60" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D60" s="18" t="inlineStr">
+      <c r="C60" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D60" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNM01qb1ZRZVBIdmp3cFc3R3RLaTdmZk1JOFo4anRtSm95Z1hJc0N0S3VranBTV29IdlViT0FkSm92eHdtbDBqdU5HTHNMaXo0dGRWMkpDdjk3LVRBVU1rZC1YejZJMkhyNmpZZFJodGoxWlB1dkRhYTJVRlljMlV0dUllQ3EtOHZkNFdSUWJLSW9Xemw1XzFzU2RHV1o0RTViOXp0bDZFQTZycWhpNElLU0FZQVI?oc=5</t>
         </is>
       </c>
-      <c r="E60" s="18" t="inlineStr">
+      <c r="E60" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2197,7 +2200,7 @@
       <c r="F60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="18" t="inlineStr">
+      <c r="A61" s="19" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2207,17 +2210,17 @@
           <t>Eyes on Tom Wallace as clock ticks on Adgemis pub deal</t>
         </is>
       </c>
-      <c r="C61" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D61" s="18" t="inlineStr">
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxNSExQeDlENWlHb0prRnRldjZ5YWhKVUZ5eVdsYjZmbVRWRWQ0WnZXWkU3UHZJdElnQ21jMU9zNnhnc3JlNDczVGQ5Y0FGV2J3QUp3NXdZTXZMNm5tVC1vWDFtOFN3aS04QVJZb3FZV2VsUmJ2aVgwbUhTaFVGdHg0UjRyTXVVUnFhQmE5eFYwMGR6T1R2U3Q3WEdZclVKNWJiby1IRg?oc=5</t>
         </is>
       </c>
-      <c r="E61" s="18" t="inlineStr">
+      <c r="E61" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2225,7 +2228,7 @@
       <c r="F61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="18" t="inlineStr">
+      <c r="A62" s="19" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2235,17 +2238,17 @@
           <t>UBS names head of APAC leveraged capital markets</t>
         </is>
       </c>
-      <c r="C62" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D62" s="18" t="inlineStr">
+      <c r="C62" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D62" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNMm9WZ2ZKVFBvX2pYMk16VmY1WFZnZ2J5N0F2bHduTVM0Sjg4STVtTGFLQVdzeFloVHg3clRic0owTDMwYVpXdDVjdjFOWjQxdkdxdFY5MEY1Q1U2Q0R5dFBJWTNtUzgyd3RXcm9uM0hKdEZ3b3JjXzcwQ2VpRm5SS0hYT2gxSU9iVFRlR05Xd2EtM2JOQjBGUzlKdnE?oc=5</t>
         </is>
       </c>
-      <c r="E62" s="18" t="inlineStr">
+      <c r="E62" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2253,7 +2256,7 @@
       <c r="F62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="18" t="inlineStr">
+      <c r="A63" s="19" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2263,17 +2266,17 @@
           <t>BHP, Woodside rise after new CEOs named; Future Fund chiefs exit; Sandilands ‘doesn’t accept’ termination</t>
         </is>
       </c>
-      <c r="C63" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D63" s="18" t="inlineStr">
+      <c r="C63" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNUHhZeHNHemtiLW1IOHN1OTZXOGpsM0ZtUG1MVHRCT1hUT1k5S2lEOXlXRENWOXNlMEZadThQR18xSTJfTVlQM3BtX0ptX1J0bk80SzNLUVRtbkJITGgtb0lsSVdJTWt2S1E1WUlXdUdsbEV0V1RpNWlyRXBoc0dPVDl1OXRrSlM3SHlDazg2UlcxenVzNzlhQldhUGhfNE5IV2xrVmVBNzhhSE9qY042Z3pzMEVzd0VyVmZudXgxcTgwWGJXSWZKZ0FyNVhjcmhjTm5DYUVjLUdDRmxUQkZuTDFlUXVaV0ZoSWp5WHMyR3c?oc=5</t>
         </is>
       </c>
-      <c r="E63" s="18" t="inlineStr">
+      <c r="E63" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2281,7 +2284,7 @@
       <c r="F63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="18" t="inlineStr">
+      <c r="A64" s="19" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2291,17 +2294,17 @@
           <t>BHP’s new CEO will shift the Big Australian’s centre of gravity</t>
         </is>
       </c>
-      <c r="C64" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D64" s="18" t="inlineStr">
+      <c r="C64" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D64" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPQnZpWndNZzZvN1VsOHBmRDVLRHVTNkxLeDVDelpOMURjOTRDSDZfN2dPZlZqaW05WEZuZXMyRTJZeVZnV0poT2UxRkVfZ1RZSjdvUjVKblhoSU5Cd1plRTVNNTRaNWZmbm1yUGZkblVpYkctNzVRRkVQQm4zX1FtRG1KV2Y0djUtOURianJ3dElqeXBUMFp4aWFEWVFYelVjYTluSWpOM1FlbHpIaUxXdnBn?oc=5</t>
         </is>
       </c>
-      <c r="E64" s="18" t="inlineStr">
+      <c r="E64" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2309,7 +2312,7 @@
       <c r="F64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="18" t="inlineStr">
+      <c r="A65" s="19" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2319,17 +2322,17 @@
           <t>How philanthropy became the sandbox of succession</t>
         </is>
       </c>
-      <c r="C65" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D65" s="18" t="inlineStr">
+      <c r="C65" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D65" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxObnBPb2MzQ1RvSVVCbmNzYWFBMlFjU0dQRmpPakNfdkxtMWc1bFdVNXNlZmRKQnNlWEtUUDNSTHpTLVV4Skx0V2otbTZsTTdvT1VaUDhMZFZoMFFab1RoS2pCcno1WGlNQlY4eXQ0OFEtLXJTay1MUkFSSEJ2MVVScUpjUkhJOThISy1QbHIzTzFlWVhOc29fWWs0V19sQ25hRW9MSGhBVVNKWUp6dUo3NS1SWlk?oc=5</t>
         </is>
       </c>
-      <c r="E65" s="18" t="inlineStr">
+      <c r="E65" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2337,7 +2340,7 @@
       <c r="F65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="18" t="inlineStr">
+      <c r="A66" s="19" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2347,17 +2350,17 @@
           <t>Advanced Navigation raises $158 million Series C round with NRFC backing</t>
         </is>
       </c>
-      <c r="C66" s="18" t="inlineStr">
+      <c r="C66" s="19" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D66" s="18" t="inlineStr">
+      <c r="D66" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNTXhwVlVLUy1pWEpFdzFCazNTY0dkczd4WW9oeW14cUtTaDZRTGlVQXBPaHN4WTBkNW1zOGxvN0tVWl9JSFdVNXlQMzVxbk4zbDZFUjNOcUxSamNaSnFCckMzWEk1VlNoSHJHQ3VWdGltVWZCV0c0NmU4UlN6YU55Q0J2TkQtUzBzOW96UXRxem5Zb3M2SUljNURISlRkQmJD?oc=5</t>
         </is>
       </c>
-      <c r="E66" s="18" t="inlineStr">
+      <c r="E66" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2365,7 +2368,7 @@
       <c r="F66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="18" t="inlineStr">
+      <c r="A67" s="19" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2375,17 +2378,17 @@
           <t>Kal Somani-led consortium buys Rajasthan Royals for USD 1.63 billion</t>
         </is>
       </c>
-      <c r="C67" s="18" t="inlineStr">
+      <c r="C67" s="19" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D67" s="18" t="inlineStr">
+      <c r="D67" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOX3lmdG5aTmk4TEpBa3ROdWZ1aDJHUElBQXktVmlKaHFmTUhPX1QxX1dKLXZfaHRDQjBnWm9McTZjTjJtTWFETTRNMHgzN0tTTm1xY0JpMF84Q2lNaFQyZGVjaHN4bkVmcDN5Qy1ta3FtYnpMSVVyYm0ydWpTRUdZU1hoYXpaNkZUQzlPc1QycjZ6aG5QVHRqY213?oc=5</t>
         </is>
       </c>
-      <c r="E67" s="18" t="inlineStr">
+      <c r="E67" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2393,7 +2396,7 @@
       <c r="F67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="18" t="inlineStr">
+      <c r="A68" s="19" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2403,17 +2406,17 @@
           <t>KMD says Rip Curl demerger proposal delivers investors ‘no value’</t>
         </is>
       </c>
-      <c r="C68" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D68" s="18" t="inlineStr">
+      <c r="C68" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D68" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPTXhBdHByWE9EbllFdDA2OW1UTUZEMVJfV2xsNFdURFRKX2JrODJReVRuQlFoakpWbTBKcjhNLUVsNE9sdG5LUElLZlVrbFNERS1QZTN6bEZIWEhXZ1pTWG5GWEw3ZmNETTdDUDUzYzR5M0E3ZGVlTWpSUnVlVU56dDNFZUtZN3liZ1dKNzJhLWU1S0M1ZnlKd1JNWXlxSlkyU3pGS1lhS05hTUJPRkxucldabzFucGs?oc=5</t>
         </is>
       </c>
-      <c r="E68" s="18" t="inlineStr">
+      <c r="E68" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2421,7 +2424,7 @@
       <c r="F68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="18" t="inlineStr">
+      <c r="A69" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2431,17 +2434,17 @@
           <t>Ex-Macquarie banker drives mortgage broker roll-up Recludo towards IPO</t>
         </is>
       </c>
-      <c r="C69" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D69" s="18" t="inlineStr">
+      <c r="C69" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D69" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxNQms5X1F2aTNhOExDbW42TlZOLVJwVWxna1JYSW9vWF9Na1RZa1ViTFdZc0tCcXRZZkRudTlsTzNuZGgwSENyYi03Zjdfc0lZTXp0NmJRZnhzb2pWRXRIOUdJN2lQM2h3ZFFtTXlSWHVWOFBIaW1Na3FQMjBCck1nVlhUcmRkLW9LOHpKWXQwTm9LcWR5M2FfdjFiRW04TndoanR5NmJvMENGalNuUGNINy1Qc20xR1J4d21ncHNNSUZqa1BXNnI4STIxSUFkZXdU?oc=5</t>
         </is>
       </c>
-      <c r="E69" s="18" t="inlineStr">
+      <c r="E69" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2449,7 +2452,7 @@
       <c r="F69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="18" t="inlineStr">
+      <c r="A70" s="19" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2459,17 +2462,17 @@
           <t>Coles reviews truck fuel charges as crisis worsens</t>
         </is>
       </c>
-      <c r="C70" s="18" t="inlineStr">
+      <c r="C70" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D70" s="18" t="inlineStr">
+      <c r="D70" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxOSGpBM3RjLVJ3LVlmR1QydnY2dm50WlVxcG43ajRFZ25QS1hDNTBONU8tY3Z2TklzbUNla0ttZk1GZzFaLUZRakFjSUpUQWItQ0VqVTVwS1B0QS1ObVEzNzdRT1l6aU9pVm5jSlhna1N6QmFKT3k1RkhMZGNTVnVLcDVIcXZmRjdjLWRpYVlRQUVmcVRtM21BSjVhTGNaaThyZkhLS2NWdkNCSkZKTlloUVdtbzRnYjFKbllOZXhOd3lkcFZEYURwUFVNQzVnSWRyM1RlOGd2M1pMZXI3c0NIa0Y0MNIB6AFBVV95cUxNSjB3Z0hoTGxwOHJQQ09xb3BmRmhCYjBCc2E0OHA2elFDRE45UGpaTEVDc1Y2VnRvVmZQUzRHbng4QTMwNGZZNGpmaVlHRmV6bnhiZ0FReU50TnRiQ0NZMEtoM3dBZ0hXbFBZMVJQNXd4LVdXRDVyTDAxNS1zeVdvcFVvend2N3J5R2pLYmhxNVFfd19rUlRsNWNndlptMUVkcS1CaUN6UXRHVzByTU5BMW1TdktOZUJYck5xMEJucmR6czIySEMycDA5cmR1MXB0N25Xc0JDUG9zN29YWklVc1BUMzl3UVhn?oc=5</t>
         </is>
       </c>
-      <c r="E70" s="18" t="inlineStr">
+      <c r="E70" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2477,7 +2480,7 @@
       <c r="F70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="18" t="inlineStr">
+      <c r="A71" s="19" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2487,17 +2490,17 @@
           <t>Sam Arnaout’s Midas touch turns suburban pubs into pokie gold mines</t>
         </is>
       </c>
-      <c r="C71" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D71" s="18" t="inlineStr">
+      <c r="C71" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D71" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQV2xlTTdYOFpIMzNmVVRnMlJRbTdGTC1jelVCd1V3UjN5cHQ1VzhWZzhrNW1PNm1RX3FlZmU3UkRycjF4WDlQUzRMcVVYY1g3UTZqQ0hxRnl2Ti1IQ0owVmZjN3Jod1BFbmhPVUwxNjhsTGh6d0kzdU01N0hmempRZ044ZmZNUllnenhyc3djRGJOdEtrekx5UVFoaFFMWDdqMHMwdng1SFg4TzZHY1hQNFJNN3huZXpWYWFtQ0ZJakhkVFlQcl9SQlRfZkQ?oc=5</t>
         </is>
       </c>
-      <c r="E71" s="18" t="inlineStr">
+      <c r="E71" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2505,7 +2508,7 @@
       <c r="F71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="18" t="inlineStr">
+      <c r="A72" s="19" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2515,17 +2518,17 @@
           <t>Gentlemen at Melbourne’s exclusive The Australian Club sweat another election</t>
         </is>
       </c>
-      <c r="C72" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D72" s="18" t="inlineStr">
+      <c r="C72" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D72" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPcEwyU01BOXF4TzlmREhYbTFEWklxdWZqWmZybDVnOWtLQ2dTU2dNQ2t5M3BVT2stN08xYkFmazVkY29oT3RVc2xUZmZINFJURGtIRTg4RGsxOURBdWEybTUwU2NUODQ2eDNBbTdPT3QxeXRFNHlSc014T0g1aG4xZ1A0U0FWMTB1Wm1CSHlQU0ZJb3lMYkE?oc=5</t>
         </is>
       </c>
-      <c r="E72" s="18" t="inlineStr">
+      <c r="E72" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2533,7 +2536,7 @@
       <c r="F72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="18" t="inlineStr">
+      <c r="A73" s="19" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2543,17 +2546,17 @@
           <t>Inside Fortescue’s AI ‘hive’ that could save the mining giant billions</t>
         </is>
       </c>
-      <c r="C73" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D73" s="18" t="inlineStr">
+      <c r="C73" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D73" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOSVVCbGpzcVcxTGlZZ2dTUkxXdVVvVU1ONEtUS0t1R1VkWWRNeUF1UmlHbXd6clR3QVRuWGxrUGQwVG1OeUxZb2RqTzdYOEVGQ1N6eDFta3VOZDdHNThYbUEwWEVHZlZBVzNpZ1Foak1kLURZTWpJVzZLekczdzFrdHMtLVZwMUZnYmkxSVc0czFqWnFaSGZiT2pIVW5rdVZmdThreFlRZWVEU0xoa1VFOV9MTjE2UHFOcWhqUzVB?oc=5</t>
         </is>
       </c>
-      <c r="E73" s="18" t="inlineStr">
+      <c r="E73" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2561,7 +2564,7 @@
       <c r="F73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="18" t="inlineStr">
+      <c r="A74" s="19" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2571,17 +2574,17 @@
           <t>Tiny house maker Elsewhere Pods seeks cash after Bunnings debut</t>
         </is>
       </c>
-      <c r="C74" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D74" s="18" t="inlineStr">
+      <c r="C74" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D74" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM0ZpVnBTS21Ib25qa09CaU52Z29kZWhTU0FJLW5VR2JCLVFPTVlZTmpYX3lZVWdtMDVTYTJkWHlPUmhXa0Rua2ZXTTBWQU1VdmFrV21KOGlrdjJ3TTdxbGlvZVBUZUxUWE1uelpWMGxWWk04UndJTXVKQjBZUEtoX3lodmdpMWZKNUc1YTIxVFZLYkFKT1QwbS01WU01ZUZTTlczY2ZpLXlpTjNJTWpsUg?oc=5</t>
         </is>
       </c>
-      <c r="E74" s="18" t="inlineStr">
+      <c r="E74" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2589,7 +2592,7 @@
       <c r="F74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="18" t="inlineStr">
+      <c r="A75" s="19" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2599,17 +2602,17 @@
           <t>Chinese consortium emerges as dark horse in Made Group sale</t>
         </is>
       </c>
-      <c r="C75" s="18" t="inlineStr">
+      <c r="C75" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D75" s="18" t="inlineStr">
+      <c r="D75" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQYlpEY0hxNm5lalIxSTUzbDE4UEF5QTNpMTl4dWNPMkRrMU1yQnltZ25WcUkwOU13V2Y2RGItVW5QTXotSnBZRUJMdGJySGw0NVVxc3ZLZmVEcTlfU193Vkd5UVVuTFVYWFNtd185eGlVQW5RRElHdk5pMjhUR24wd1k0T0I3cW9qTG5Lcjg2bV9aNWsya0FYODRjeURyMW1EeHdYT05iZHZhLVFrUVNoV25idnZYZ2lpZEhta2JxOWFJb0M2SE9hbFF6NlVWYTM3QmF5anpWOEZackZiTDBfN2gtX1luQkxFOUxSSNIB8gFBVV95cUxOQklMYWl1ZkRqZGUwN0ppeXFubzZWNTNmeE5GY1BfcS13N2dFT096YW9JSndVX1EzTlBKdWZIemdKZnRIME9SQk5aT1M2WnRESjJxckFTaUdOSEd6eG9hRVBjdlhBbWQyWGpUS1kwQXJsdlpkLXJpXzJZX2xiUC1FSlNnNTFoVXQ4bF9JeUp3UGRWdUFOUVRrNUtsRzRxaUczb1p2LVVucFBNazhuZFNDaUZDR2ZQUVdObmVtTnBndGlkazZqeHVheVNzSE9RY3Bad0lrckxDSWY5QXBWS0hwVzZvSTZjaGEtNkNncW1RRE5uUQ?oc=5</t>
         </is>
       </c>
-      <c r="E75" s="18" t="inlineStr">
+      <c r="E75" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2617,7 +2620,7 @@
       <c r="F75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="18" t="inlineStr">
+      <c r="A76" s="19" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2627,17 +2630,17 @@
           <t>KMD faces uphill battle in capital raise as key shareholder baulks</t>
         </is>
       </c>
-      <c r="C76" s="18" t="inlineStr">
+      <c r="C76" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D76" s="18" t="inlineStr">
+      <c r="D76" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxOVTU0OGNfRURNcDdzYUtIcG8tR3N4OFFYalhKNWJBaUd6ZlQwNU5MZVZYbUZVSzB3WmdOOFdTZHlBOXBzSGdYUVV6eGt1UndHN296bENxZzNUM2NoaV93LXZaZFNNOXJ2YlA4RHNFS2FDb1ltNWpPWUdRR3VGMWoxaU5qYm9VSW9yUW5kS1NaN2RSc2YtcHZRSTB6aE9Zdkl3NG5nbVRzODRfQVYtelo5M3g4R2JEbnpraFpWbENOZzE2Qndla2t3MXRPWkU1dXg4NmZRME1jT3pOOHZOVlpTZGloNENUZllaSTFmWUV1Y2JLck02ZDhnTHJ5bUPSAYICQVVfeXFMUEFXR29tQjlTbTdMRVNDWUlGNFNOQjVhX0FiSkl0U2stbml5VHR4d1g3bDFqMUw2TzR1eHhYOU5ZUmJpZ2xBY2NzcmJRX3MwaEQ0YmpzMUFnV1BQNGxmcnlXUzVvbHpwNEo5dWFnZlduZ0Z2dGZGRFRKRTNCUzctZDNCd0FMNEkzTm84dmZOM2NKYk81RERsVnlZN1VZaXp5TW5QRVAzOHNXQTFWdVlKdGtFX0FmcU1EbElZSm52alBQeWx4VnlvOFRwNk1ia2lZYXlpemQ4cFdmckotMmMyRGE4ZXN0dThQYmxxUkpvMzAwRXBBcVJuRnp0QkZ3b2tqMWF3?oc=5</t>
         </is>
       </c>
-      <c r="E76" s="18" t="inlineStr">
+      <c r="E76" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2645,7 +2648,7 @@
       <c r="F76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="18" t="inlineStr">
+      <c r="A77" s="19" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2655,17 +2658,17 @@
           <t>AustralianSuper claims another listed M&amp;A kill with Pepper Money</t>
         </is>
       </c>
-      <c r="C77" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D77" s="18" t="inlineStr">
+      <c r="C77" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D77" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOY0RwcnpWZlhfOHA2MG13MkJUX1RDNF9wN2RxZGU2cEpzS1RKTjJDeUl0OERFOGhFRXJaSXNETEhHbW9PS0lua283RnFVbHJvTlRva0djQ2lRSGc2RENJYmt0OEsyYTRVSzFGeE9jWVhKMVRnd240WXVNTVdac2lOUGJSZlc4UVZ5RXo0OTlQbUd6NWRSek1HZG9fZGk2aDhDelhGVmk4YkRKeVV1M0VHZ2hZNmFVdXM?oc=5</t>
         </is>
       </c>
-      <c r="E77" s="18" t="inlineStr">
+      <c r="E77" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2673,7 +2676,7 @@
       <c r="F77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="18" t="inlineStr">
+      <c r="A78" s="19" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2683,17 +2686,17 @@
           <t>Apollo to Acquire Nippon Sheet Glass in $3.7 Billion Deal</t>
         </is>
       </c>
-      <c r="C78" s="18" t="inlineStr">
+      <c r="C78" s="19" t="inlineStr">
         <is>
           <t>Wall Street Journal</t>
         </is>
       </c>
-      <c r="D78" s="18" t="inlineStr">
+      <c r="D78" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOanpORVBremoyamJyZ2FqQWVOcDcxa2NpempBUmNYcktMLUl1Mzg5VDloWmlVbUdNUnplVk90WEUzXzJjNGxENk9LcGF0enVSdlFpWU9nd244YWNTS0ZHd1JTZEtlbjRQTmJUU0dzWmlDOVFhR1ZRSFJkNXN4a3FHdGozcUcwdHRseXpYMFREUzBNcXRmQ1VCN056SWlEa1l5VVE?oc=5</t>
         </is>
       </c>
-      <c r="E78" s="18" t="inlineStr">
+      <c r="E78" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2701,7 +2704,7 @@
       <c r="F78" s="3" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="18" t="inlineStr">
+      <c r="A79" s="19" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2711,17 +2714,17 @@
           <t>Estee Lauder in talks to combine with Jean Paul Gaultier owner Puig</t>
         </is>
       </c>
-      <c r="C79" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D79" s="18" t="inlineStr">
+      <c r="C79" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D79" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPSjN6QnFVbmdHWFoteURWaU5VaWZmRmpTT3QtYm1tZUFyNUZyLUdheGdfWlRBTlJyTlp4THIwVDA4U3BnWFNpT2FpZlZzX1lJSDV0MkRGVjYtNVc0b0lOQy1RSnFGTWhCTWE2ZFFPYlFQX05yaVlfZF9IUEN2ZWkzQ0VFMUxxdHF2ODNQY09xdWlqWEczSC1CZk5wYU9QQlAyaTMyelJnaVM0cmN4M0paNzlBdzM1RndoZE8yRHN4UnZqaXVhVmx5NFpqS3hmUHhUdlpF?oc=5</t>
         </is>
       </c>
-      <c r="E79" s="18" t="inlineStr">
+      <c r="E79" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2729,7 +2732,7 @@
       <c r="F79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="18" t="inlineStr">
+      <c r="A80" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2739,17 +2742,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C80" s="18" t="inlineStr">
+      <c r="C80" s="19" t="inlineStr">
         <is>
           <t>The Age</t>
         </is>
       </c>
-      <c r="D80" s="18" t="inlineStr">
+      <c r="D80" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPdUtyNWs5YmxJMXNsNWtaMi1WMm5SVHd6ci1ReURLajdYd1IzWGJMZmE2MzJsSzAxQWtSTm8xMUEwNTh4Vy1zTmFsWFBKTkJ0YXc3ZkcwOVk2a2VNRWVGUS0yQzZhSXlCWmpDYUx6RmpTTlNhS0xIQklyVFdIVXJRZTNPaVB4TG4yQ1R1ZWF2MWpmSG81TVRaRzdtMXpydWhBS2w0a3ZPZFI5MnFKOW5tN21oUDB3NkNtQmR4LVVBWW9BUQ?oc=5</t>
         </is>
       </c>
-      <c r="E80" s="18" t="inlineStr">
+      <c r="E80" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2757,7 +2760,7 @@
       <c r="F80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="18" t="inlineStr">
+      <c r="A81" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2767,17 +2770,17 @@
           <t>Australia’s new millionaire factory: Start-up to $1.6b in five years</t>
         </is>
       </c>
-      <c r="C81" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D81" s="18" t="inlineStr">
+      <c r="C81" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D81" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOVkl5N1NGWS1XWWZSc0pHXzE3MUNERmV5SUgyQ3o2MmJ3U3Y2YlNwUXNSTGlQenBwVFdnMWhoT2FrcDAwUHNVU0RQbjFHMjJiLU1TRC1nemdrX3hPTG93VWZUQUx3Wk9HT3lYd055Z2FtREFpOWRlYXFDb2hwV0cyWFMwaHpsLU0ta2VVQlpid1dlYks0ZHg5YTY3Ykt6Um5YaF9MR2tIRzd1Tk1IRnBrWVhxVjZNSUl1OE9iRlZzYmQ3QUVnZmhYVGxoOA?oc=5</t>
         </is>
       </c>
-      <c r="E81" s="18" t="inlineStr">
+      <c r="E81" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2785,7 +2788,7 @@
       <c r="F81" s="3" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="18" t="inlineStr">
+      <c r="A82" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2795,17 +2798,17 @@
           <t>Social Media Wrap: Genki Sushi Singapore's loyalty benefits; Dunkin Philippines launches new collectible; Burger King Malaysia unveils new Korean inspired burger</t>
         </is>
       </c>
-      <c r="C82" s="18" t="inlineStr">
+      <c r="C82" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D82" s="18" t="inlineStr">
+      <c r="D82" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxPbFR6eHVTRWZNcUw1TTBJdE1JTFpmbk5iWndKZnRoU3Fmc3cxcF80TnVhRERmY0poM09zTFpCaEVnMGo5aktxY0ExV1ZlZVpHYUtldXBoOUh6bm14SURHNmhnUE9tYnI5YlpXQ3pRZlp0Ni1wM2lYQmdxdjk4SDl0aFN0R1VBbGxpbFVzOHV0TFY3YjJZbDg4Vk1HMTBkQk5LRHd1ZEVpRnBsT1U0Nm1IbVFkZEUybmpabEhuLUNLOGhicUxXZG5UalRLOE5DSzcxRncyNjVRdk8zclhJNkVQcTRkQTZYSEdN?oc=5</t>
         </is>
       </c>
-      <c r="E82" s="18" t="inlineStr">
+      <c r="E82" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -2813,7 +2816,7 @@
       <c r="F82" s="3" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="18" t="inlineStr">
+      <c r="A83" s="19" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -2823,17 +2826,17 @@
           <t>Copyright ‘status quo’ not working in AI boom times, says Charlton</t>
         </is>
       </c>
-      <c r="C83" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D83" s="18" t="inlineStr">
+      <c r="C83" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D83" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNVVgwdEQ2YUt0eFo3THcxOXZHbUFYZ091VTFKZDZHX0szYWQ2dnZ1dkJma3VZcGk1LUM2SUtQSWhxMGpCUlFZVzdKNmdoSGEycm1oYlBUdEZ5R0ZlU2hrWHpFWXdSN1lCZnZzb3hZc2twVVlWdTNNVXhaR0Nza0FiaUNveXZWQWQ1ZE45MU1HbGNmWlU2aUdha2FyZllzNWdONEpsM2RrdGRFSFl2UlpJUnQ4WGpleGs?oc=5</t>
         </is>
       </c>
-      <c r="E83" s="18" t="inlineStr">
+      <c r="E83" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2841,7 +2844,7 @@
       <c r="F83" s="3" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="18" t="inlineStr">
+      <c r="A84" s="19" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -2851,17 +2854,17 @@
           <t>The unapologetically analogue 4WD for off-roaders with $120k to spare</t>
         </is>
       </c>
-      <c r="C84" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D84" s="18" t="inlineStr">
+      <c r="C84" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D84" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxPSFJ4ZnNLT3U1REp3MWI2WDFaQm5vZlp6QWN6c0hZamtYVU95WmpkUERwR1dwc0NQN1dEc0FNbHlaMTdLclVHb1JTc2VZNExENGYyUE9OR1BkQ244YXRVeWNwbkxia2VrckVqSy00WV9UNWlvZWJHOG9ibUthaTlpVmRBOGZjLWFzMU8yS2Q5Um05SWIzY2dKajhoMWFUcmFrbTMzai1CdVBNLWczTWRvbTBwSDRfUzNwOHhqQm5hTDdhM0xLWEpNQTRyRXZjU1FLdGhRMUxtOTg?oc=5</t>
         </is>
       </c>
-      <c r="E84" s="18" t="inlineStr">
+      <c r="E84" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2869,7 +2872,7 @@
       <c r="F84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="18" t="inlineStr">
+      <c r="A85" s="19" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2879,17 +2882,17 @@
           <t>Junk room to become jazz club with priceless Melbourne view</t>
         </is>
       </c>
-      <c r="C85" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D85" s="18" t="inlineStr">
+      <c r="C85" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D85" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQbHN4My1nOGtueVJQZWM0LXNjLTR3MmhuemRJMUEwN09FTUZhZk1lbV9MbnVWblgyUXFEMEl3LUtsOGVqdGUweFR0MXF0ZEo0XzNhWVRqb2pGRUdiNTlLc1dFcXFmdnctQU1wQkRSdHN0T3J6VGt3MU1iNENydGlsOEpsT0ttZmJVZ0FUZmFXSUd3alVzUTQxMzVmcEVXSlV2dWdQd3JsMUZ0d3ZZYlBHaGhKTm9rM01SUmdseE9hT1prbHZtMlhv?oc=5</t>
         </is>
       </c>
-      <c r="E85" s="18" t="inlineStr">
+      <c r="E85" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2897,7 +2900,7 @@
       <c r="F85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="18" t="inlineStr">
+      <c r="A86" s="19" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2907,17 +2910,17 @@
           <t>Zimmermann fashion label appoints new CEO Roberto Eggs to replace Chris Olliver</t>
         </is>
       </c>
-      <c r="C86" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D86" s="18" t="inlineStr">
+      <c r="C86" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D86" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM2M5QU1scVoyNHBmV2lwQ0VQS1Z6d2Qwa1ZkZ0M2WVIzdXR3QnZwVWhUSDRCUEdRZkc5QzFQSFFhNzZ4VE9lWXBTcGhpS01JdG12TlQxSHhValZfbWt3MUdFZGl3RlBtdnlrel83TjNjNFZ0SUpvSDNQbThpU3FLa3Atd0dNU04zQm9OSk5uNHpTVE84aWZpaVlKWkdOQjJjRTZSd1MwMEZ1b3pENkRCQQ?oc=5</t>
         </is>
       </c>
-      <c r="E86" s="18" t="inlineStr">
+      <c r="E86" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2925,7 +2928,7 @@
       <c r="F86" s="3" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="18" t="inlineStr">
+      <c r="A87" s="19" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2935,17 +2938,17 @@
           <t>Construction giant FDC road tests IPO pitch - AFR</t>
         </is>
       </c>
-      <c r="C87" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D87" s="18" t="inlineStr">
+      <c r="C87" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D87" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNTnRScHFhQlpkdEdSb2x1bExxQm96ZE5zSV9wTDNDV2pxYjFQdUtoYmNBell3SFlTTFEzMUhpeXlmNERSeDd6VGppM2szQ1NHVE9PY1R3MTN0SUZLWkF5em8tQ3IycUZ2RmswX0tnN1IwOHl1ZFo4UUtMUDlQbXRjTnRCWFB5cU1RZFhsdDdaWGpMZzh3d29CWWZvZGtnTjl0T1k5ZHFHSUg5XzFSSF9TSUxTYkU0QkFheFlLZUY3S2tCSWRLZWlBbUpxUjc3TXBQQ01V?oc=5</t>
         </is>
       </c>
-      <c r="E87" s="18" t="inlineStr">
+      <c r="E87" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2953,7 +2956,7 @@
       <c r="F87" s="3" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="18" t="inlineStr">
+      <c r="A88" s="19" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -2963,17 +2966,17 @@
           <t>David Jones is trying to defy retail gravity. It’s causing problems</t>
         </is>
       </c>
-      <c r="C88" s="18" t="inlineStr">
+      <c r="C88" s="19" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D88" s="18" t="inlineStr">
+      <c r="D88" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPZy14UldWZDRrSjI3R0lzdGlKamlkVnU1WWVjTWRUTlpya1ZpVW80WHlrT0FQTUUwMzkzM19xQWpwTnVLOF8zeTFXamhTZFRQVjl5TTlXbE1RRWY2NW03dlpmZ25qdkgyN1IwbDdjRlhxd1MzSGkxeG45M214OVlESWF5WWh5TjM0STQtOXdieWIyOUI2NzRsaDhiS0ROUU5YQ185aWtObUY2S0dOSTBROVlwSVB1VkNqTkZTTllkZmtMYmxjNVdlTA?oc=5</t>
         </is>
       </c>
-      <c r="E88" s="18" t="inlineStr">
+      <c r="E88" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2981,7 +2984,7 @@
       <c r="F88" s="3" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="18" t="inlineStr">
+      <c r="A89" s="19" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -2991,17 +2994,17 @@
           <t>Jefferies’ Australian ambitions in focus as Sumitomo circles</t>
         </is>
       </c>
-      <c r="C89" s="18" t="inlineStr">
+      <c r="C89" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D89" s="18" t="inlineStr">
+      <c r="D89" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxNUTd0LXFPQmZXSldrTmZHTkIwUWQ3MmlCUmFOUGRkcVVjRXV6YXZJUTcyMG5FV3I0dWY2NXh6MnduVjNxZmhJMHdDVGw5VzFxTEFzN2FBdlNvS1JGSDltQmlzVS1QRDdCeWdfSHZ2VlZDMlBnN1Y0d2JxbnlGejhWVjJpWGZLejdCTUt2Uk9ENmhyRkd4dDJjd0RlUnBlZXhOTmUtOG9ITE05VHJ3dTBRSWZneURuUW1NYkExVXpfWXlsMzZ1WUlyNE84SThQX1JJTFlXOHc4ZnB0aXRmdVhaaG1qSEJRZUhuU3RibHAzbHVNLWFLUF9NNTFoUXV3NGQzelcwcNIBigJBVV95cUxPMkhEeDJpNzg0NTlDZmF2LUFPSEs4cmZ5U2p6bWVZSTYwcXVUUGVIb0FLVnhZV0cta01CLVpfQzQzYzdvTWdxR0o4bGJDWDVBb1lnOGx0bWROdTdjcHhwLUpPMW9MQ0RVM2NUOUt6UGpTd05JYzhuVmgybGp2LVpORFF0SHpBTU5DUTJEUmZKUFBNajlQdHJ4WkdHVV9QMjVwOWVlNWliVkFaM20yWGZhOEc4bldHRERJak1BWXlmSE0zdno1VTVSc0FMck0wSE1BR1RVaVRMSEdzU2FvcWpMYmp5ZTVJTWcyUGdXanhqSUNZU0tzTkNYWVg2SXpVMEoyS184VkxOeWtSUQ?oc=5</t>
         </is>
       </c>
-      <c r="E89" s="18" t="inlineStr">
+      <c r="E89" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3009,7 +3012,7 @@
       <c r="F89" s="3" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="18" t="inlineStr">
+      <c r="A90" s="19" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3019,17 +3022,17 @@
           <t>Bain Gets Nearly $300 Million Loan for Australia Wealth Unit M&amp;A</t>
         </is>
       </c>
-      <c r="C90" s="18" t="inlineStr">
+      <c r="C90" s="19" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D90" s="18" t="inlineStr">
+      <c r="D90" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMUQ4WExYZFY1aFBwWENNR1JiVkw4OHFKWjY4NW4zQ3ZBalFiTU10Y2hic2p2VjFqOE1rMndNYmVoN0lPcnY0WmFOV1MtaEY5c2xvcW1PNGN2SzZVcThwc3ljWkYwV1Q4a2dIaUpBeXZpMkRUU3IxZzVBVkhydGU3OXEzNW1sdlVQeTRNRFY4bUJLOGpGYmJ0ZXpPc1YzY05TYWd2bF9oWVJ6Rks2dWlod1dGRU4?oc=5</t>
         </is>
       </c>
-      <c r="E90" s="18" t="inlineStr">
+      <c r="E90" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3037,7 +3040,7 @@
       <c r="F90" s="3" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="18" t="inlineStr">
+      <c r="A91" s="19" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3047,17 +3050,17 @@
           <t>Fund managers caught up in Aware, TelstraSuper $237b merger</t>
         </is>
       </c>
-      <c r="C91" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D91" s="18" t="inlineStr">
+      <c r="C91" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D91" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcFF4Q1A5X1VtNWFnYXZSVUlZX2JMRVoxaUJoeGhybmRrZkd4UlEzTURwMkx2d2I1Y1hMYmljbk05WUFzRl9JbF9JampqeDd2bXdYcUpHbVZYak1sYXFHS2VuUDJyTUhzSS1QTW15aVpfeHRuMGZHenlxOHJQRUdENkV0b2FMZXhOZWF1Yk5hR1lOYWFQc2Q0SEROUFNERXhKQUIzRkt6NTQ?oc=5</t>
         </is>
       </c>
-      <c r="E91" s="18" t="inlineStr">
+      <c r="E91" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3065,7 +3068,7 @@
       <c r="F91" s="3" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="18" t="inlineStr">
+      <c r="A92" s="19" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3075,17 +3078,17 @@
           <t>Soul Patts defies private credit jitters with 15pc returns</t>
         </is>
       </c>
-      <c r="C92" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D92" s="18" t="inlineStr">
+      <c r="C92" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D92" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPRkNINFJOai1NbUUtX3ZrcnJFS3EzRHZPbFRfVFE3SERudTVqbjIybWsyYUthOUJOUVFPb1U0UzlGTTRqbUxraFZfYlVtclQxeTBQU1M5YjJzMDVPU3RiX0cxbk8xOEd5YjV1R04zT0NNZjhNSi1meWo4RHM1ckFsUnNLd0JiQXFnZ0dtckNzdWxmanZoQUl3TEQ2a29nRkRDZ1lJd2Y5VGc2UWZHX0pkU1NObmRJTlZKS0E?oc=5</t>
         </is>
       </c>
-      <c r="E92" s="18" t="inlineStr">
+      <c r="E92" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3093,7 +3096,7 @@
       <c r="F92" s="3" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" s="18" t="inlineStr">
+      <c r="A93" s="19" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3103,17 +3106,17 @@
           <t>Ex-KKR China heads negotiate to buy Vitaco, owner of Musashi, Nutra-Life</t>
         </is>
       </c>
-      <c r="C93" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D93" s="18" t="inlineStr">
+      <c r="C93" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D93" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQRmlCdTlFeHdBUGkyOS1CeEFIYTRSREdZM1JOZ3IyZThnNmNMdm9QeXVwRWtMbzU0em1vcDAyM1hodDlvalVRdThtNVhLR2FsaE1vV0xuWjkwMkVCUDk5SmVka1BURFJZNkl2bURLeC1GdzI0V2hEaVhrNlJZejlvc2gwRmtnUjd1NDFlX2trbGk2aXJiQ2FrTWtmVVpiOXhBc05JSkNYY2xLX2JEQUpWY2dlY1pDZw?oc=5</t>
         </is>
       </c>
-      <c r="E93" s="18" t="inlineStr">
+      <c r="E93" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3121,7 +3124,7 @@
       <c r="F93" s="3" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="18" t="inlineStr">
+      <c r="A94" s="19" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3131,17 +3134,17 @@
           <t>Antipodes Global Investment Company</t>
         </is>
       </c>
-      <c r="C94" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D94" s="18" t="inlineStr">
+      <c r="C94" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D94" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE5mdkJzN19XLTFQc25LOUk0ZGJBMER6djB2VnFvbGVrS1hlemRBRmlNY2JmMGlPTzktU0RRS3NNUW8tRXhtUE1QdE1JLWdUNVhibmZPZi1MRkJOWk95NzM2bXplS3JzeG13UU5henhza1ozeGRZZmlBNTNR?oc=5</t>
         </is>
       </c>
-      <c r="E94" s="18" t="inlineStr">
+      <c r="E94" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3149,7 +3152,7 @@
       <c r="F94" s="3" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="18" t="inlineStr">
+      <c r="A95" s="19" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3159,17 +3162,17 @@
           <t>AusSuper to lift insurance premiums by up to 40pc</t>
         </is>
       </c>
-      <c r="C95" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D95" s="18" t="inlineStr">
+      <c r="C95" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D95" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQNEhYQkoyNnJFU2xBZG8wdXhEZWRSakRiWWNHOGZBTFhfaElxWkRsSWViaWxjenVjMF91cGdrbFZxSGJfbkR2SUZNdEJtYUVadlV6YVVrWU1VbVdsMWpyNUZ4bE13Mmo4cGQ3WWZlVFVrTTdyOGpSdkpUb0tkcjdQUFlsTnM0MnpOMDJNZlJ4YTlzZGpLS1QzMFluOFU2VUJya3lSclBLSnZkQ2Y0a2djNUpSYlo?oc=5</t>
         </is>
       </c>
-      <c r="E95" s="18" t="inlineStr">
+      <c r="E95" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3177,7 +3180,7 @@
       <c r="F95" s="3" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" s="18" t="inlineStr">
+      <c r="A96" s="19" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -3187,17 +3190,17 @@
           <t>Unions want inflation-plus minimum wage rise due to ‘Trump and RBA’</t>
         </is>
       </c>
-      <c r="C96" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D96" s="18" t="inlineStr">
+      <c r="C96" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D96" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNdzNhU0MzbFRFX2I3OVY4bFItd1h6OVE2Wnpqb01NM2tMYzNob21BeW02LTBfTFZIWnN6SG5DVnYxQTJGZWZaLTJpTXZGUnhmS3RPY3hQV01fd1RIYU9Ednc4a1hvalVRT19ESU5TX19sQjN4dVV3X29kQjliQjNFU19iaXFIS2l3blk5TWUwdHFrRmJtQ0JocDN0WEhWbXZOVUJzR3RaYnJPSHpIRFlYOVFObEtuT1d0TUo0MUVZTXdFZWR3WG1r?oc=5</t>
         </is>
       </c>
-      <c r="E96" s="18" t="inlineStr">
+      <c r="E96" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3205,7 +3208,7 @@
       <c r="F96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" s="18" t="inlineStr">
+      <c r="A97" s="19" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3215,17 +3218,17 @@
           <t>Firmus’ Oliver Curtis set for green light to run ASX-listed company</t>
         </is>
       </c>
-      <c r="C97" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D97" s="18" t="inlineStr">
+      <c r="C97" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D97" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNR3VmQW9vNmUyeU9WbVRvRG9tcTNMYVlvRUhCd29wTkRZaVlEcG50Z0hIN29XcE5GUmxkUy1yMm0yTm94Q1BXMmNCcXBpZDlqVTRlZFpMX1QyMWh5Ym5XQ3VjYW1ZdDFtYWNyOERCOURuWXM5ZTV4WGthMVVjNUZlcmVTQ3JBUjQzUXRXYXRLQjlNeHpBMkVCVWpsd2Z1Vk42TjJxSlRiQ0ZtaTkzOTZtNmRHQQ?oc=5</t>
         </is>
       </c>
-      <c r="E97" s="18" t="inlineStr">
+      <c r="E97" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3233,7 +3236,7 @@
       <c r="F97" s="3" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" s="18" t="inlineStr">
+      <c r="A98" s="19" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3243,17 +3246,17 @@
           <t>Crisis Hit David Jones Chasing Funding As Retail Markets Come Under Pressure</t>
         </is>
       </c>
-      <c r="C98" s="18" t="inlineStr">
+      <c r="C98" s="19" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D98" s="18" t="inlineStr">
+      <c r="D98" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNNjJSOUVQcTkwUmxXNXg4ZzljSGhnRlBJY0otSHRrX2ZIQXRqWmNDZlgxYW1jckhHd3BtdXJsUWhwTjQ5SGw2NUU3TnFtcmhYd2JVcThIR2VCLWJLU0h5RE8xaTV5TS03Mi1za19hcF9PcXRRSU9PX3ZxSktSV2FfY1ppcUFVV2w1TmF1UWVtZlBWSUhEcG9oRGlEVkEwR2ltQ2VMSTNlcENEYlY0?oc=5</t>
         </is>
       </c>
-      <c r="E98" s="18" t="inlineStr">
+      <c r="E98" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3261,7 +3264,7 @@
       <c r="F98" s="3" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" s="18" t="inlineStr">
+      <c r="A99" s="19" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3271,17 +3274,17 @@
           <t>Beirut Street Food eyes niche in Lebanese fast casual</t>
         </is>
       </c>
-      <c r="C99" s="18" t="inlineStr">
+      <c r="C99" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D99" s="18" t="inlineStr">
+      <c r="D99" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNVlZVeTNGcXVOSXV1eklvTnFxYk1hb1A2VTQtNHkwdUpvdFF0YnlYU2RSWkZNV2dGQkEyZjRVQzVJZ2Uwc3gtZ0F1TGlSQlVna01HRnZOTTJnVUFxaWtOam1vZ245Z05jdlRnQURqbnQxaGtEcnFYS20wWmtvSDV0MW15c18zUE5ZN2JJWUpLV0RsZE1LSm5fcUNNeVZNTmdMQ2c?oc=5</t>
         </is>
       </c>
-      <c r="E99" s="18" t="inlineStr">
+      <c r="E99" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3289,7 +3292,7 @@
       <c r="F99" s="3" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" s="18" t="inlineStr">
+      <c r="A100" s="19" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3299,17 +3302,17 @@
           <t>Gami Chicken credits chip design for cult following across Australia</t>
         </is>
       </c>
-      <c r="C100" s="18" t="inlineStr">
+      <c r="C100" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D100" s="18" t="inlineStr">
+      <c r="D100" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPTXg4T0dvQ1l4NFVxV25iUXQzY0F3MnFjYmE4X0NOcFdNZHgweUg4NmVZZjNJbTFMajNhNHBmVDE2MGNBZzhOTUJsaG5KejFZbk1Db0JyNTZJbUI2WnRZeVhXRFRMNXVBWVFMdGJ3WkN5dV85dEduQi1OVDhOSE9UOGVERXh3T2hCVmlDNVg5LTdLY2VHNEZJSzlrN3VuemhzX1B5blpYRGtwS0hrak5r?oc=5</t>
         </is>
       </c>
-      <c r="E100" s="18" t="inlineStr">
+      <c r="E100" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3317,7 +3320,7 @@
       <c r="F100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" s="18" t="inlineStr">
+      <c r="A101" s="19" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3327,17 +3330,17 @@
           <t>The great fake meat meltdown is taking plant-based burgers with it</t>
         </is>
       </c>
-      <c r="C101" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D101" s="18" t="inlineStr">
+      <c r="C101" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D101" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPRTVDNW5oaWJ5bHdKM21iYllEVnpJbHhSbWFzYy1RcEZCdnNGUlJOWVJCaDZacFVoRjlSUGpfa3N6ckQtMFYzZTNITW5tMy05Sk0tZmtlSWlESHdOMWIyUWpUbE5RQVlsTHp0VXg0cHJYM0lJVmw1ckRURkFPVHFabTRIUzlFX1FlbFNuYmQ5MVJwWHVOaVhVWTdPajZxdG1WOTliTE1qZ3k1dnFRbk9BNTZCcXRRSGlIXzJv?oc=5</t>
         </is>
       </c>
-      <c r="E101" s="18" t="inlineStr">
+      <c r="E101" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3345,7 +3348,7 @@
       <c r="F101" s="3" t="inlineStr"/>
     </row>
     <row r="102">
-      <c r="A102" s="18" t="inlineStr">
+      <c r="A102" s="19" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3355,17 +3358,17 @@
           <t>Solar for Cuba: How Xi is turning Trump’s war into a China win</t>
         </is>
       </c>
-      <c r="C102" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D102" s="18" t="inlineStr">
+      <c r="C102" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D102" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQOFlUUnNZUWo0MTJRaDFIZHp5dUJudERrOWxCZmY1WjZmeXRTVzJkbENEbUFhSkZFUWV6WjNGNUJIejVYRXFPcmRNZjFZeTkzTmtaeFNlb2V1OFFnMGtkV2JfTVRUN2FSV2xxcUpDUDJQeUpqWE9DRHRmT2kyc1dIZE9jeUM2eV9KQjd2RkJuTkxYeEdISDZDejhRbVo?oc=5</t>
         </is>
       </c>
-      <c r="E102" s="18" t="inlineStr">
+      <c r="E102" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3373,7 +3376,7 @@
       <c r="F102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" s="18" t="inlineStr">
+      <c r="A103" s="19" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3383,17 +3386,17 @@
           <t>Beer Sectoral Group appoints Nigerian Breweries CEO Thibaut Boidin as Chairman</t>
         </is>
       </c>
-      <c r="C103" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D103" s="18" t="inlineStr">
+      <c r="C103" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D103" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOamdsNTN1dkRUY19Yak0wUGxsdm9NZGhySUM0Vzc4blNCeldzdFBiRkxuSW1xbTlZQUJIWkNxdzI3Zi1zc3F3SmJvai1UVGlZdUhGTEJ0eF9mNHRwSGREbDktT2txWXA4OVBESTdPLXdxWmV2V3FPTEZaYjRWLTlMM1VaY1dCbGZudTczZlFEYzN1aE9HeWdObE1yZFduLUtNVXBheDNsUWlIcUxibml4YQ?oc=5</t>
         </is>
       </c>
-      <c r="E103" s="18" t="inlineStr">
+      <c r="E103" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3401,7 +3404,7 @@
       <c r="F103" s="3" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" s="18" t="inlineStr">
+      <c r="A104" s="19" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3411,17 +3414,17 @@
           <t>Hip pocket pain comes for shoppers – and for supermarket giants</t>
         </is>
       </c>
-      <c r="C104" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D104" s="18" t="inlineStr">
+      <c r="C104" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D104" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOeTdfN2dwYlBWSTdGbFo0SWRJcTNYelFFM2FBRnlORWRNcGd0WUVCbVdHVWZ6TFdZQzFpM2h6TkU2OEtqeE5OYlRrNmhsRU43a0E0UXhtZEZyTWZidzhMUEVxSVdiMlpTYXQ4ZVRaNl9BSi1Mb3JRaXhvM2hlMmNDcnk1aFBvVXFQSmlPbkN4Z3o2R2RzV0drQWpKaVZpbXR4dHppa08wRFd0dlNwcDc1alRDSXg?oc=5</t>
         </is>
       </c>
-      <c r="E104" s="18" t="inlineStr">
+      <c r="E104" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3429,7 +3432,7 @@
       <c r="F104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
-      <c r="A105" s="18" t="inlineStr">
+      <c r="A105" s="19" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3439,17 +3442,17 @@
           <t>RBA calls for co-ordinated effort to unlock digital asset markets</t>
         </is>
       </c>
-      <c r="C105" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D105" s="18" t="inlineStr">
+      <c r="C105" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D105" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOT3dEcEtwVUptWTZydTRYWFdCU1RhTjI1RkFWeU5HckRVZjBxc2lqRkNOT0stc1h2Q0E1YTkxTjk3NTB3TGxKZGIweGFQRGh2S05QWHRoVGNZRFR2SlI2bkEzWlRoY2t3WU16dDlhVEI4RTFWYzhKS25YbGYxSVRjdFpVQ2M0dVc5MFJuUExNMTJIMVJTYmZGbkNLR1BPeVFYSF95NkNnWEEzamg3NmRuRkx0U2NjbXlxY015UWljTzRWbXpKclAwUg?oc=5</t>
         </is>
       </c>
-      <c r="E105" s="18" t="inlineStr">
+      <c r="E105" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3457,7 +3460,7 @@
       <c r="F105" s="3" t="inlineStr"/>
     </row>
     <row r="106">
-      <c r="A106" s="18" t="inlineStr">
+      <c r="A106" s="19" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -3467,17 +3470,17 @@
           <t>Banks rebuff work from home calls as Wesfarmers pauses business travel</t>
         </is>
       </c>
-      <c r="C106" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D106" s="18" t="inlineStr">
+      <c r="C106" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D106" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOTjFLNnZUNXZHeE85a3kyaG1IX29sWjFvZ2NzS041UnYxNkkwUF9YU3ZFYXhtQmlxY3Rmd0lUSTJrdTl1Y0ZobWp0M1lrZnZhZE9OSzV3Ql9Hb2UtUEpqWC1McjM0S2pESDJQVWJKQkw4enF5THJfeXFWRDZiMk5KMmVrazVUMzBNTk1tOXRVX1ZzVU1IUHBVSlhENEdEWFJpQnFXUGkyNVJGUnhzdXgyNW1WZXRkRmRaaVloZnpaMFdqVmk3elpFSkZ6ZmotZw?oc=5</t>
         </is>
       </c>
-      <c r="E106" s="18" t="inlineStr">
+      <c r="E106" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3485,7 +3488,7 @@
       <c r="F106" s="3" t="inlineStr"/>
     </row>
     <row r="107">
-      <c r="A107" s="18" t="inlineStr">
+      <c r="A107" s="19" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -3495,17 +3498,17 @@
           <t>This mine was fast-tracked to boost Australian solar. It’s exporting to China instead</t>
         </is>
       </c>
-      <c r="C107" s="18" t="inlineStr">
+      <c r="C107" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D107" s="18" t="inlineStr">
+      <c r="D107" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAJBVV95cUxPN1ZSdEMzSXBhMno2YzNkSFFtdlBOTTRGV3UtbnZtRktEd3Q0MHdmZHp0SDN5S0FZYmVKUllicHRMRkxTdmxtbkMtT2ZVN3hsUXdBVzAxdzhWcGFWRkxVdFY3NURqTVV2QVJQT0ZUT193R3JLLU9aZUw4YzlucjVUN0xyTzdoZlNjYXdyR2VWeDZrbW53cTJoRGZDd2kxbkxzMHBQWkRJMTFPMkNlX19wYjI2LVBZbnVJOVNsRjF3Tm0xUUFpY0ctczFZdWJFcHQyLUhwdDNiSGVtdHQzVVRtbExpcHJZak1SNkhWd2s4a0RtYWFNN2J2Q3FobTF1N0hWLXA4YUtaMXBScjZsUWt3alVVTVpJdVl0WDF5RTJLM1BKUl85dnhUUktkb2VwMzFkUWZ1ctIBugJBVV95cUxOOENIa2JzQzdxekNYTnJNVmRzdm9KTFpndnBybEJfNjBUR3VNMk92ZnhGY0JwVGZLeFRpdHJLMTQ0NjRNOFg5b3FESzhPLWlub2hSeFdidW0yS1h6ZXlGMjh3X3FhaWo1dHdneUZxS2NsaUJ6dWtfT1R6VndwSk52bVVNN2I5VlNYazBIelcwUkVBZHFlM0hiQVJ1a2NGWFpmR0c5R3Bna2RZMmJuSXB5WkQ1Zl94VDFtcjVEd2x6amIwSWdXUWtQVVo1Q0hpWVBLRVFycDAyU1NJV3N4YktlUlBtMTlkY2VNZjc1QVZhbnRrQ01OQnZqNzI5dTNNZ1VlNVVJcURycXlDRFZDYVo1aC15RXpwUFlvZWxlMHFybWJiM1YxT05lRElXYlZsbkJWUnI4VV9Da1lIUQ?oc=5</t>
         </is>
       </c>
-      <c r="E107" s="18" t="inlineStr">
+      <c r="E107" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3513,7 +3516,7 @@
       <c r="F107" s="3" t="inlineStr"/>
     </row>
     <row r="108">
-      <c r="A108" s="18" t="inlineStr">
+      <c r="A108" s="19" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3523,17 +3526,17 @@
           <t>A $600m dream or a dangerous gamble for cricket?</t>
         </is>
       </c>
-      <c r="C108" s="18" t="inlineStr">
+      <c r="C108" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D108" s="18" t="inlineStr">
+      <c r="D108" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxOYnpVaTZiU3hGMWY1UVVmYk9nRTJaRTVFYUE2ZklLYmJIQkdXZzFMbWs3MVRJb0l4bUpPeThwRnhOSmh0bzNBdzhpeXpuS1RrZ0tNVVJ4eU8tRVIwR2FyYmUtNG1UVmN2OXRsZm1mVy1LZDVERkpXQURMUk1HRE9Hc3F3RWQzYmFvbHRCVGhFOTQ3M2xnVGcxTWxtT3cydW84NTNPc3BXQURodmY0azBOUllOQjhrbzJ6WmI3bjY5dk5RRzlDQ0JlYzg0VzRsdWtIblZJelRSamFyQnNweHdHLTRTMTFOcy1Jd3ZtQWFodEcxOThVeVVz0gH3AUFVX3lxTE5ielVpNmJTeEYxZjVRVWZiT2dFMlpFNUVhQTZmSUtiYkhCR1dnMUxtazcxVElvSXhtSk95OHBGeE5KaHRvM0F3OGl5em5LVGtnS01VUnh5Ty1FUjBHYXJiZS00bVRWY3Y5dGxmbWZXLUtkNURGSldBRExSTUdET0dzcXdFZDNiYW9sdEJUaEU5NDczbGdUZzFNbG1PdzJ1bzg1M09zcFdBRGh2ZjRrME5SWU5COGtvMnpaYjduNjl2TlFHOUNDQmVjODRXNGx1a0huVkl6VFJqYXJCc3B4d0ctNFMxMU5zLUl3dm1BYWh0RzE5OFV5VXM?oc=5</t>
         </is>
       </c>
-      <c r="E108" s="18" t="inlineStr">
+      <c r="E108" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3541,7 +3544,7 @@
       <c r="F108" s="3" t="inlineStr"/>
     </row>
     <row r="109">
-      <c r="A109" s="18" t="inlineStr">
+      <c r="A109" s="19" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3551,17 +3554,17 @@
           <t>Why these people decided to vote for One Nation</t>
         </is>
       </c>
-      <c r="C109" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D109" s="18" t="inlineStr">
+      <c r="C109" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D109" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOQmNaOHZXWEEwZzRmdTBVT2FiS2hsYUhFczgxaFJaeEQzMGlfSnRoUWo0ZXl3cWhhbTU2NDRLUjh1c2Jxd3ZoR2pJOHVNemI2cTFrdU9oVkFCNXN4WV94TER4VmtIX1JCblhKNTl4VHlMdFBDRHVBUFhkS1AtR05RMG5QVGJFaTlWaVpMZERIa3Ntbmh0V0xnVVhYNDdMWWlpSWc?oc=5</t>
         </is>
       </c>
-      <c r="E109" s="18" t="inlineStr">
+      <c r="E109" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3569,7 +3572,7 @@
       <c r="F109" s="3" t="inlineStr"/>
     </row>
     <row r="110">
-      <c r="A110" s="18" t="inlineStr">
+      <c r="A110" s="19" t="inlineStr">
         <is>
           <t>2026-03-28</t>
         </is>
@@ -3579,17 +3582,17 @@
           <t>The Right Amount to Pay for Sushi</t>
         </is>
       </c>
-      <c r="C110" s="18" t="inlineStr">
+      <c r="C110" s="19" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D110" s="18" t="inlineStr">
+      <c r="D110" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOLUljQ1FWeHk0N21FcnpCTzdNVW1WZmxfbDFucXRNYlBMSzR6aTh4WlNrdnFuT1VSWWpKWlJValZrbTE5RlllanJkcHNHeEVwVkxldnZSdjdLc2c1SHJTVG1hMHBKd2xtZXptV1FmcGZ0cXUwVXFMWjJiRFhhYTlKRkNBNHZQekVRcnRicXlNM2NQdXJaZkVRbTZta0hDRlV5YVN5NG9TYzltUFZucXNXc29Wc1Y?oc=5</t>
         </is>
       </c>
-      <c r="E110" s="18" t="inlineStr">
+      <c r="E110" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3597,7 +3600,7 @@
       <c r="F110" s="3" t="inlineStr"/>
     </row>
     <row r="111">
-      <c r="A111" s="18" t="inlineStr">
+      <c r="A111" s="19" t="inlineStr">
         <is>
           <t>2026-03-29</t>
         </is>
@@ -3607,17 +3610,17 @@
           <t>Blackstone-backed $2b Xpansiv kicks off raise</t>
         </is>
       </c>
-      <c r="C111" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D111" s="18" t="inlineStr">
+      <c r="C111" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D111" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOOGIxbEhpZjgwbk5XampWenBXbGZmbzFQbnJhUjU1Z2FtT1FGVk40SHExMUJBZHZoRDBRVXZHS3ZlR3o5RGU0c1o0Y0E2MXVKZ3U2ZFBBRm1NbVJPRk1pMGp3dV96ZTlMNERlMFBPRDNROXpNZlNmLV83VGV2QVNzWkhtV1kxY2x6TUQ3QkhlcVNPNTlyMUQ0?oc=5</t>
         </is>
       </c>
-      <c r="E111" s="18" t="inlineStr">
+      <c r="E111" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3625,7 +3628,7 @@
       <c r="F111" s="3" t="inlineStr"/>
     </row>
     <row r="112">
-      <c r="A112" s="18" t="inlineStr">
+      <c r="A112" s="19" t="inlineStr">
         <is>
           <t>2026-03-28</t>
         </is>
@@ -3635,17 +3638,17 @@
           <t>Elon Musk puts a $2.5 trillion rocket up Wall Street convention</t>
         </is>
       </c>
-      <c r="C112" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D112" s="18" t="inlineStr">
+      <c r="C112" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D112" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPeE52VS03NHBqZ3hvc1Q4V2laUElCcmxKem9SSzM0d1Uyd09ZSFl4SjZmUDl1Sl85WXp3TWtGX3hydFRwZG0xQmFlOVUtdEtaNmtYWFkzVDYyZGI0SWFZRWtYR2tGODdPVUNhLXBzVVpzYnVRYmZNZW8xbEpreGZMVzU5c1JrWDY1Nk9uWk53a3FCOHpQTDBCT0h6QllmbW1wc3FmVU4yTUlxSmRhTUdF?oc=5</t>
         </is>
       </c>
-      <c r="E112" s="18" t="inlineStr">
+      <c r="E112" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3653,7 +3656,7 @@
       <c r="F112" s="3" t="inlineStr"/>
     </row>
     <row r="113">
-      <c r="A113" s="18" t="inlineStr">
+      <c r="A113" s="19" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3663,17 +3666,17 @@
           <t>KMD Brands makes emergency capital raise, chairman David Kirk to exit</t>
         </is>
       </c>
-      <c r="C113" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D113" s="18" t="inlineStr">
+      <c r="C113" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D113" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNb1JhRUM4dDhXM1hoajdzQkNLQk12LURQbkp5LWdqQXpEczBxdVhySHphaUhiLVRiYVh1R25kbHRidy1TbjhCOEk0MXk5a2VWWlhHcUt5aXpfNjZWNnd6LVpQUkZNbFFXSWJHTmFaM2x2aS0tbG9TeXFxUWI1NF9uazJKa3BrZHFwclB1OVR3cWhXU2dJNFhaZmpVRVlwWUdiX2hrX0thQ3RDOWdFTF9BOGdHTG1JSlF6RVRZdnZn?oc=5</t>
         </is>
       </c>
-      <c r="E113" s="18" t="inlineStr">
+      <c r="E113" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3681,7 +3684,7 @@
       <c r="F113" s="3" t="inlineStr"/>
     </row>
     <row r="114">
-      <c r="A114" s="18" t="inlineStr">
+      <c r="A114" s="19" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3691,17 +3694,17 @@
           <t>RBA green lights credit card surcharge ban</t>
         </is>
       </c>
-      <c r="C114" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D114" s="18" t="inlineStr">
+      <c r="C114" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D114" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOcTB6SlhfdTQ5ZWdqNDExZVhOcVVybW5mbmxOVktCS3ljTndLY3ItWldSNDIyeEkwQmdBZ3p1X1o5S3ktZXI3MFM3eVkwWWc4cGtUTUw3aWM4azM3VGdrcGZjTjZMN1diWHZ0N3pna0tJZHZNU1FaN2VZbVNwMmozSFNBb253OUcya0duaEMtZnNQaFYwUFBhTGthaGhyTWY0NHpPTTFubmZOWEk?oc=5</t>
         </is>
       </c>
-      <c r="E114" s="18" t="inlineStr">
+      <c r="E114" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3709,7 +3712,7 @@
       <c r="F114" s="3" t="inlineStr"/>
     </row>
     <row r="115">
-      <c r="A115" s="18" t="inlineStr">
+      <c r="A115" s="19" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3719,17 +3722,17 @@
           <t>Constellation Brands to acquire Hop Wtr, expanding non-alcoholic beverage portfolio</t>
         </is>
       </c>
-      <c r="C115" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D115" s="18" t="inlineStr">
+      <c r="C115" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D115" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPcjdPYWlEWWF6dkY2Y3RPWUh6M0pXYUw1NFNabUdXTS01TVBMWGtBMUpxTXFRekJINGNFOE5oVEI0WjR4Z2kzTUR6emJHUUYxWjA0MGVlWFNPR25xNmJJWkN2RHIzcWNxUHRFQXcwdWN5cHNZRVVYV3JTdXRJUFg1MWJKODNOdjJ5UEd4dWZEbVFyWlNaRkJPcnlyQW5janktSDVwYWRVRGJqTFdPTEdUSUFvRXI4QQ?oc=5</t>
         </is>
       </c>
-      <c r="E115" s="18" t="inlineStr">
+      <c r="E115" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3737,7 +3740,7 @@
       <c r="F115" s="3" t="inlineStr"/>
     </row>
     <row r="116">
-      <c r="A116" s="18" t="inlineStr">
+      <c r="A116" s="19" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3747,17 +3750,17 @@
           <t>David Jones races to secure $150m survival deal</t>
         </is>
       </c>
-      <c r="C116" s="18" t="inlineStr">
+      <c r="C116" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D116" s="18" t="inlineStr">
+      <c r="D116" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxONHp5S2RtcFJkYWVxakc1ZDE4UzZUVWlHSlBMTHJqVnVaRHJrcEwyV3BHWk9TdXdkOUlocWY2ZlN4NklobGVuYWhRc1BvdWppWlNFTm9wcGZoMG1UMEtjLS1scmx4cVNhNkZQYWw0M1VUQTJfOTJrYWMtTlpJYnl0N01QTWxZZDZPOEpfcTM1dFRVMDBTOEthcFU2Z0U4WFFBaE1GM2V6VHJVb2Z5ekxJWmUwQlphbXRlTS02NWNJV2p1Ym5Ca2JxNS0xQWZpbHJ4UFVtbDBCXy1IV2NXMlFOY25HSVkzTjYxbXZB0gHwAUFVX3lxTFBDVlc2X3JNcnNNWjlUV2RkeEdtSFBJRFNtTXVHcmZERW1vZURfeDFvRGo0b1Z5SlVOVGNJTXB4MVc3d3hWY3FVOENwbEJ1MERBalhlc2EwNnktcUprSjZQLUxNTVlqYzc0enZtQ0FOUFVTWHBCZVF1SWs2Y0ZKRllXblI4MVRrXzZUMHNicmxqeFhUUld4VzM0TGNtcl9fTG4wbEJPWDg4RWpjMUdHOUxlczdEend1MkZLRTZuUjdkV0xGRlR6RVlXdVUxdUhndmozTHNtT2czTjJzRUs0bFc2QnMxS0V1X3QwcjVNeGVjcQ?oc=5</t>
         </is>
       </c>
-      <c r="E116" s="18" t="inlineStr">
+      <c r="E116" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3765,7 +3768,7 @@
       <c r="F116" s="3" t="inlineStr"/>
     </row>
     <row r="117">
-      <c r="A117" s="18" t="inlineStr">
+      <c r="A117" s="19" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3775,17 +3778,17 @@
           <t>Newly listed Advanced Innergy targets smaller rival</t>
         </is>
       </c>
-      <c r="C117" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D117" s="18" t="inlineStr">
+      <c r="C117" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D117" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPamkyYnZfT0NwamdES3JPYklaaXFYdUp5cHJPOTZUNklqcUlral9ObHFPY1VROHJSdm1tOS1KZlZJWFA0Q1l2UUZhOThleHFsWDJTSVdTUnhlbE1OeVhBTXVQQjVIdHZHTFBHOUxGOGx3MWc1UmVIWUV6Q3RhTDR6WHRfRy05a25VX01lcWZOV3BWX1JyQVI0WlQ3dTQwNHhxWXJCQmV0VQ?oc=5</t>
         </is>
       </c>
-      <c r="E117" s="18" t="inlineStr">
+      <c r="E117" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3793,7 +3796,7 @@
       <c r="F117" s="3" t="inlineStr"/>
     </row>
     <row r="118">
-      <c r="A118" s="18" t="inlineStr">
+      <c r="A118" s="19" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3803,17 +3806,17 @@
           <t>Aussie eyewear giant’s costly $20k mistake</t>
         </is>
       </c>
-      <c r="C118" s="18" t="inlineStr">
+      <c r="C118" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D118" s="18" t="inlineStr">
+      <c r="D118" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAJBVV95cUxOTmtzblUxcW5WbDZLeEJXSWVuVW5qVzdpRkc1Rkoxc1pVT0FIaHdmR0p4ZzljcVpST2tHdTBwVEdqbmF2TVhlV0VaMDFiMVk2ZEZkUTZMNFQ1a1lUbWRCdGwySkJtbmRfTXFmUy1VVU1tU1dzMldON3lEUFVVVFI4T000b2NJLVhobDBBUzQyLTRGLXNPT3ptZ2tlUU8wNG5nNFAyUVo1elpTeDd1TW01YzB4eUI2eE9YQjZxNTJBSVpLYy0yR1BzSVFiWWxib1g0YmlzREFGTEV0bkRucmNLa3U4dXhkTC1aRkhnUHN1d0hjVUFuZFlWWG9xVUtMT0hKMjhmNkZzLWpMS2MzYWp1OVN0cV9IYnBRZG5OdWwwcErSAaYCQVVfeXFMTzBFMkJ2TU5EZGZYLVF5WHBJanYzeFJqS1owbk5EUUNOZFNiam5PcEZ1aDBFelJ5MjFzM0E0NlZRdGI4Rjdnb1RYVmVSN1Z1OWd1SFdweVB0ZEY5akVqOHBsTHpJaXZKNnhUMmd2YVVxTzUtUEJKcWpOY0VHeHlTbXNCbHFDdnlndzJFT2ZDcnlZWXYxNUFNekVUZWU1UTFnOXZXUERMWjdjYl9wVVl6OURodW1JSUI2ejJDTktfaTRCY2xEeHVBRW9tNmM3YXBHU201WXpHYjFYbU1sYnB1MjlLNjI0eTRWVElXU2ZqMDNNRW5LMVQyS2M5Z2tPSHJneGlkUkxFYXhDdWM1MGtkUUExT1hBSlU1ZkgtRlM4YnV3b1hkM2NR?oc=5</t>
         </is>
       </c>
-      <c r="E118" s="18" t="inlineStr">
+      <c r="E118" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3821,7 +3824,7 @@
       <c r="F118" s="3" t="inlineStr"/>
     </row>
     <row r="119">
-      <c r="A119" s="18" t="inlineStr">
+      <c r="A119" s="19" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3831,17 +3834,17 @@
           <t>Rio Tinto bankers up for infrastructure sale; eyes on Pilbara power</t>
         </is>
       </c>
-      <c r="C119" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D119" s="18" t="inlineStr">
+      <c r="C119" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D119" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPQTRxenprUFZmM2JIMDNPZGVVV09IakN5STI4ZFJVQmEtemVQUlJCRjdtbGpKWEZFOWVRd2ZYZk4xNkNHclpMSEFZLUpBVHhKaFN5Q0Y2bmhRWERpc2N4NEhua0VSQnFpVmpxa29tSlFNOHJRaFROMS1mTHBGdzZ6UlhLaVpqaUJhOEs3Y0Iyc29KY01XUXR3R1gwOXJHQUp2QVpNYi03NTZhLVgxN3VlODY4T0E?oc=5</t>
         </is>
       </c>
-      <c r="E119" s="18" t="inlineStr">
+      <c r="E119" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3849,7 +3852,7 @@
       <c r="F119" s="3" t="inlineStr"/>
     </row>
     <row r="120">
-      <c r="A120" s="18" t="inlineStr">
+      <c r="A120" s="19" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3859,17 +3862,17 @@
           <t>Luke’s Bánh Mí launches budget mini meal deal</t>
         </is>
       </c>
-      <c r="C120" s="18" t="inlineStr">
+      <c r="C120" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D120" s="18" t="inlineStr">
+      <c r="D120" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPQmh4NzlPa29pOXFmeTlKVFVUenNqdTF0VGU2REVwaWRsR3dKSEs3NFlTcGlscFRhRWRtV1JtVmFNTzJCb1d4d1NrUm9mMzBKcDBmM2JBbWZPTEVNdWZ1ZlVZZW93bW14Ull1UTNLUDh6WlZ2RUdBTS1NZEg2dmRZc3BEd2dfTFRFUERwdERnZnZwMFRR?oc=5</t>
         </is>
       </c>
-      <c r="E120" s="18" t="inlineStr">
+      <c r="E120" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3877,7 +3880,7 @@
       <c r="F120" s="3" t="inlineStr"/>
     </row>
     <row r="121">
-      <c r="A121" s="18" t="inlineStr">
+      <c r="A121" s="19" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3887,17 +3890,17 @@
           <t>Zeus Street Greek sets sights on drive-thru as next phase of growth</t>
         </is>
       </c>
-      <c r="C121" s="18" t="inlineStr">
+      <c r="C121" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D121" s="18" t="inlineStr">
+      <c r="D121" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNTEEzZ2VJMDdRek9JdGZCVVpJRGZoSjNIWjNiN3h2OHR2RjUwUG42SzViRUpteXRURFZzbFBpR0Q4TFdianc0SjZkc09DU01MY0hMLWRNbXQyYUVNai1BMUxFM0pZRWJaT0cwcmFna3pRS253R1FUY3UxOURmRkcwN3Fmd0VfLWVONzJJXzBzX1U5TFBQTFMtSURtZUV0TDhu?oc=5</t>
         </is>
       </c>
-      <c r="E121" s="18" t="inlineStr">
+      <c r="E121" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3905,7 +3908,7 @@
       <c r="F121" s="3" t="inlineStr"/>
     </row>
     <row r="122">
-      <c r="A122" s="18" t="inlineStr">
+      <c r="A122" s="19" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3915,17 +3918,17 @@
           <t>From $5bn to $50bn: The end of an era at Blackstone</t>
         </is>
       </c>
-      <c r="C122" s="18" t="inlineStr">
+      <c r="C122" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D122" s="18" t="inlineStr">
+      <c r="D122" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijgJBVV95cUxQc251ZVp0SEY1TnpWc2g4WERmLU9INk5VTUJHa3RGWGRmbWYzLV9MQW9rZmQ3bjVTRVI3R3NDbVNPdW9GTksxNUdrdkk1eTk0VXNFZmR2V2FBQWtnZGRmZkVMbm5QTUo4dFUxSGlOS0FSRmZZcThBVnlqWTN0eEUwUjFPdjhFb29BTXFWTTdHODRYelQwWUNBbXdNOElkQ2UzRU51VjM3SC1HZmpEUlNJUFFKRmdPWnhqNlEtVkNUaUtCbEc3ZWo2NFVIVktNMTQyd21lekpHVjlXOGV5WEhIZWJrU0ZTTFlrSkZnYlUxOWdUYnhna2JZTlhGYlAwMmhDYlJfZ1o3bVVDTnppS1HSAZMCQVVfeXFMT2E5cHJhVE9FUlVLN3RPakxmMHZKN3JLVUEwM3FSdmlfR0o0X2tybDFQWTg3NmZsYkE5LVRjX1dQMHVhNHBXNkhVRl9kd3lGeFdIWUV2QVFyYVgzWXU1Z2dpLXd6OGtUR0Z5SkdZc2VVM0tDU2MydXZSbGZOZjhUOEg0YXlBN2EtVDk3Z2FUM3pGY2JkTXdGZ2I5U2otVkJ1S3NhTXRBVVNqS1FvYzdPeHdaY3dqNlJmdkhwWHZCdjVsMXNibEc3aDFBR3NkRkZpdVRzU3Nad3Y0N2gyaHRQWlY0cGV2SUh3T1NwdEJEZTh3T3laM1B6YXlzVHlRRXdHc09tOFVKUTFfYjU0aFpJMDRlSTQ?oc=5</t>
         </is>
       </c>
-      <c r="E122" s="18" t="inlineStr">
+      <c r="E122" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3933,7 +3936,7 @@
       <c r="F122" s="3" t="inlineStr"/>
     </row>
     <row r="123">
-      <c r="A123" s="18" t="inlineStr">
+      <c r="A123" s="19" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3943,17 +3946,17 @@
           <t>Starbucks opens first retail outlet at new Town Hall Station</t>
         </is>
       </c>
-      <c r="C123" s="18" t="inlineStr">
+      <c r="C123" s="19" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D123" s="18" t="inlineStr">
+      <c r="D123" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOTnJ1YVF6V1dqMm9HbmdUZEk3NlQtdjRxT28ya19fbjRKMlJRb3hsam5zdDg1cnEycHc4STRPdENPQnlMQldBbTh3NXlYb0tUNW9WS201NTZ0M0xvRE8zRkVYcFlNSmdOeVZvbXRMVzJMMkV6czFPX2djSFdKNlhWbUQtNUpMcnhFNnpfa1RPY3Q?oc=5</t>
         </is>
       </c>
-      <c r="E123" s="18" t="inlineStr">
+      <c r="E123" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3961,7 +3964,7 @@
       <c r="F123" s="3" t="inlineStr"/>
     </row>
     <row r="124">
-      <c r="A124" s="18" t="inlineStr">
+      <c r="A124" s="19" t="inlineStr">
         <is>
           <t>2026-03-29</t>
         </is>
@@ -3971,17 +3974,17 @@
           <t>The ex-Platinum quant who has won billionaire Kerr Neilson’s backing</t>
         </is>
       </c>
-      <c r="C124" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D124" s="18" t="inlineStr">
+      <c r="C124" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D124" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNMkpmVTVUVU1WZUZiRWlJUkRId3BhS1hqM09aM0FSODBFNE96SDlKWG11Qkw2bjVSNFFrc0oyWHBBVXNYclBYQklIdnZBNEZ3b2NvZzdHZWNrV1JhbWI5aUpBLXRqTjIwSnhRSlFtdUlTU3VUbVMxcmtYZzlnVEsxellFb0dwb1hhME9QbERGcU9aXy1rOEtyQ0pXZW9KcENIem5TMjhUZ1VydFlrVWI3cWN6aGJROGFwWUFlNjQweTdqYkptcHc?oc=5</t>
         </is>
       </c>
-      <c r="E124" s="18" t="inlineStr">
+      <c r="E124" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3989,7 +3992,7 @@
       <c r="F124" s="3" t="inlineStr"/>
     </row>
     <row r="125">
-      <c r="A125" s="18" t="inlineStr">
+      <c r="A125" s="19" t="inlineStr">
         <is>
           <t>2026-03-29</t>
         </is>
@@ -3999,17 +4002,17 @@
           <t>Media bosses: ‘Australia shouldn’t be held to ransom’ by AI giants</t>
         </is>
       </c>
-      <c r="C125" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D125" s="18" t="inlineStr">
+      <c r="C125" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D125" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPSGdRM3JDVld4OG5UWk5RdlVZVlU2LTFKUjdzVy1HejgyaUxMWHhmUlJnN1FrY2dSTTczczU0Tno2TUVPWDFiZk9TTjJTNlQ4Yi03MWpfdVEwWGFaQm9ydjJpaGFkekZHME1xNUswcWF4b2Y4TUxkOUpOa0dFTjlYVmhVMnFPMXlEcGJjeXZBR0tFaDZUa3Ixd1lIai1qcml5OE9SM1dTcUVkWW1HdFJTUFBJZUU0Nzg?oc=5</t>
         </is>
       </c>
-      <c r="E125" s="18" t="inlineStr">
+      <c r="E125" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -4017,7 +4020,7 @@
       <c r="F125" s="3" t="inlineStr"/>
     </row>
     <row r="126">
-      <c r="A126" s="18" t="inlineStr">
+      <c r="A126" s="19" t="inlineStr">
         <is>
           <t>2026-03-28</t>
         </is>
@@ -4027,17 +4030,17 @@
           <t>PLI scheme for food processing industries sees Rs 9,207 crore investment</t>
         </is>
       </c>
-      <c r="C126" s="18" t="inlineStr">
+      <c r="C126" s="19" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D126" s="18" t="inlineStr">
+      <c r="D126" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOcUwtamFxVTZ0YTdEOTBsN1gxNlphTV84aGJoRnFFTkFkZDhaT2VzVkFDT29hMU1Xa3BLeWFiRWlXT3Noc3VVVkg3WkphSFMwS3k2aWI4ZlhfcDN2LTV6Q3E0YnNXbEFVZFdUU3U0R293aEtlUmxlLXdFWXl5MHh0X2hWYnNvbU5MLUNCRm53aVpJa0E4OUxuNnN3X1FwUQ?oc=5</t>
         </is>
       </c>
-      <c r="E126" s="18" t="inlineStr">
+      <c r="E126" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -4045,7 +4048,7 @@
       <c r="F126" s="3" t="inlineStr"/>
     </row>
     <row r="127">
-      <c r="A127" s="18" t="inlineStr">
+      <c r="A127" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4055,17 +4058,17 @@
           <t>RBA’s surcharge hit on the banks may miss bigger picture</t>
         </is>
       </c>
-      <c r="C127" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D127" s="18" t="inlineStr">
+      <c r="C127" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D127" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOdWl1NWlxN0dzeEdzWThmcDVkNkpyYjJaNnZBa2dBSWhpaHhXRktTR2VtRzdUSnB3VGtDOTFuMTZXc2xycHFYN3dnQm9SaThYUURCSjg0dVlhLU52Vlo5VnRVNl9SSXFSbWFPeXdVRmdlUVA5S3FZQXc5d2lDY19UU2tJNGdrUzc0UXFHU3BGV0NHVldJcWxTS2Zydy16eHQ3QUlLQVdjWQ?oc=5</t>
         </is>
       </c>
-      <c r="E127" s="18" t="inlineStr">
+      <c r="E127" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -4073,7 +4076,7 @@
       <c r="F127" s="3" t="inlineStr"/>
     </row>
     <row r="128">
-      <c r="A128" s="18" t="inlineStr">
+      <c r="A128" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4083,17 +4086,17 @@
           <t>The six best new places to dine in Australia this month</t>
         </is>
       </c>
-      <c r="C128" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D128" s="18" t="inlineStr">
+      <c r="C128" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D128" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxObFAyUFZmNFk4LWJ3QzFDZnpZZlRNTEgzbGt1S1BOVF9qa2V4NnR0Yy1pX0RVUFlaUDg5bmV6LTZ2VExkWVpyZmRmV1dxNExoWkdvQzdzMTNuT0UxekhITmZBQmNhWENzV0lMYnE5all1Nk1CczFpRmhlN2pxenE1NGtLQzlKb21pSnljMlhHQjR5SVVxaG9wM01ndUdMOGpuWDduQ00waTF6OVpJUTdFV2ZWNm1yVjYzcnR3?oc=5</t>
         </is>
       </c>
-      <c r="E128" s="18" t="inlineStr">
+      <c r="E128" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -4101,7 +4104,7 @@
       <c r="F128" s="3" t="inlineStr"/>
     </row>
     <row r="129">
-      <c r="A129" s="18" t="inlineStr">
+      <c r="A129" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4111,17 +4114,17 @@
           <t>Mesabi Metallics secures 520 million dollars from Breakwall Capital</t>
         </is>
       </c>
-      <c r="C129" s="18" t="inlineStr">
+      <c r="C129" s="19" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D129" s="18" t="inlineStr">
+      <c r="D129" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNbVRfWlRYc2U4bV9WUVRxWmxpQWY3UTZyVGhGMGZtbEV5UXR2OTZJdGVYdFRUNzNtSUZEUVhwSzBDVWlmbWE5bTJsbDlBVXdZR0IxUHkzSDBXVkNiY3paYnlZWXBoUm1iam5oNUh5ejU2M3ZaaVhqTjV5SlpFd250Ym5HY0FvdEJvS1JvUnFRa1pmdFpKUV9OZg?oc=5</t>
         </is>
       </c>
-      <c r="E129" s="18" t="inlineStr">
+      <c r="E129" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -4129,7 +4132,7 @@
       <c r="F129" s="3" t="inlineStr"/>
     </row>
     <row r="130">
-      <c r="A130" s="18" t="inlineStr">
+      <c r="A130" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4139,17 +4142,17 @@
           <t>Fast food giant offloads Aussie stores in fire sale after costly flop</t>
         </is>
       </c>
-      <c r="C130" s="18" t="inlineStr">
+      <c r="C130" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D130" s="18" t="inlineStr">
+      <c r="D130" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimwJBVV95cUxNOXRhd0lOSkctZjVDaVRpcktmZzV1aEFJZGpsbHJHVU5Rdm9JM3U5Q3JBOEdFU2tMeDBnLUJ2WmxiOGZaRVF5RF8tS3R0R1dtQWFGaEJkbHV4VjdfSDRJSnFCYnQ2bXlhOE90N3V5THdCM1JnU0JjLU1Kb1U5YkxjU0N5bUpTYVJzX3l4X3ZHakpESmVrVWdWTk5RQlFZM1Awa25rWHVabzNlNWFqbENHdFhMX3hTWFBqNDlvVTJlcjlMeHRMWE8tRm1rTElTanB4RFl0THJTazJrVTdGYkh2OUxQaDdwSmx5bTkxNGJhQUIza1F1cjJCSGNQTDRDX3RaVzZBbDFhOXB5S0hSQ3U1ckVhRWNLUF9MVTA00gGgAkFVX3lxTE1RSE5Hb0FJRE1YWjRxa1RwZk5GUmhXa1MtcmM4NDB0ZWZxTWNtaEhDczZjZ1FUT0p2d2ZTcHZGd25vbC1mR2lGOF9NQnlGNEtWUFprdG5KM1hTRGFRb0VxdkxJU2E3NUFWLXBveUM2TktmeWRoSWlaaWpTbUFOSEVmZXJIQzFOVHNLUUVCSDgyLW8yWHRBN25vSkhYNy1vRnNOVkpXbXRQNVhpWXE0NVNTWjYxd2xXTGZqdWxWa0NsNHdLNEhMQTFNcFZzS0YyY0N3MDJhLUJKUGFVc05vQkZuUU5JUDhBazYzejVpYnZ3NjJzMEFPYVpDb3IzMzlLTWdNRFBscEVCQ1pDQTBoXzBfbnpuWTJTSmRNWnhiaExPeg?oc=5</t>
         </is>
       </c>
-      <c r="E130" s="18" t="inlineStr">
+      <c r="E130" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4157,7 +4160,7 @@
       <c r="F130" s="3" t="inlineStr"/>
     </row>
     <row r="131">
-      <c r="A131" s="18" t="inlineStr">
+      <c r="A131" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4167,17 +4170,17 @@
           <t>Young QSR workers stand to gain over junior pay rates abolishment</t>
         </is>
       </c>
-      <c r="C131" s="18" t="inlineStr">
+      <c r="C131" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D131" s="18" t="inlineStr">
+      <c r="D131" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNcXN5UDZ5d3h6NTd5YTdqUkM0dXBmdjZ0WlQ4YjF3QUxsTzdEZUVicTRweTJHYVVfYVFsQndwaURnWVBPYlJUdVRUUThQVG9jQkgzRVFyMEdBN053MDdBUmlKNHp3X0NmYVc1OFBGT2paSTZsNG5zdE9uNm1BVXd4TFEzVmgxMnJVRzFpclRlZndDTDMxU2djcGc2WVhWM2VkLW9NVkdTSnpQOHM?oc=5</t>
         </is>
       </c>
-      <c r="E131" s="18" t="inlineStr">
+      <c r="E131" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4185,7 +4188,7 @@
       <c r="F131" s="3" t="inlineStr"/>
     </row>
     <row r="132">
-      <c r="A132" s="18" t="inlineStr">
+      <c r="A132" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4195,17 +4198,17 @@
           <t>Bain presses ahead on Estia IPO, trade bids land in $2.2b-$2.7b range</t>
         </is>
       </c>
-      <c r="C132" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D132" s="18" t="inlineStr">
+      <c r="C132" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D132" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxONzVXcThuZjBBc3ZBQWg4bWU0Wmg0X3ZEdEZkeTFKa2U3RGRabC1Jem9nOGx4MWVwOFB2SFh6UjlIdVZuV2h4Zks0Y2pVV2pnVU9Rei1TX1Y4ZzVvVkh6MzRwTlZUS3NDZDNLZDVfZjB0NlRfTnBzWkFOSW5xbUc2bi01b2p1dHlaQ3pvZWV2YTR1dWdXZzZuX2FfM0pzSkxRck1OTEgydlB3SS1GTmpMZXhvMm4?oc=5</t>
         </is>
       </c>
-      <c r="E132" s="18" t="inlineStr">
+      <c r="E132" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -4213,7 +4216,7 @@
       <c r="F132" s="3" t="inlineStr"/>
     </row>
     <row r="133">
-      <c r="A133" s="18" t="inlineStr">
+      <c r="A133" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4223,17 +4226,17 @@
           <t>Challenger-backed emerging markets fund Ox Capital shuts its doors</t>
         </is>
       </c>
-      <c r="C133" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D133" s="18" t="inlineStr">
+      <c r="C133" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D133" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQalJpNmNjb1dtSDBtLTVEQjNodkJNTVdRNUhBVkxxR3lnQlhYSGY1YW1hdnZGTUhRRzR1QnhJN3pTdC1ablBwOWtydGZTLTNTaTJiZFFHanY3VTc2YTRqcDZUQTRvS21TNDF0YmljSzIxYkxxZzRMTHY0RzViWl9heS1xT2EzbUFmUkd0bHZkZzl4Zll4UzEwOHRhazgyWHN4VUw0WUFSLWRmLTJpZDltdjcyLXA?oc=5</t>
         </is>
       </c>
-      <c r="E133" s="18" t="inlineStr">
+      <c r="E133" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -4241,7 +4244,7 @@
       <c r="F133" s="3" t="inlineStr"/>
     </row>
     <row r="134">
-      <c r="A134" s="18" t="inlineStr">
+      <c r="A134" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4251,17 +4254,17 @@
           <t>Bosses send warning on 42pc junior pay spike</t>
         </is>
       </c>
-      <c r="C134" s="18" t="inlineStr">
+      <c r="C134" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D134" s="18" t="inlineStr">
+      <c r="D134" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxNaVJ0aGJ3RE9zNlVJSTVzZE1zMlpEbmpIWHpSVFVUQkNYZWJ3R3NCbjQyM1JWQV9sdUs3MVNkWnVqUnRUQjlQNmZoUkVjTHVTRENuQmxRS1NfRmd5MTM5VXMxWU5ST2M3ZjVkU2hKN3NINmhQWkJwMUZSenBnM1RselBCdVVabGNjandnV2NlTkc2SjJucUR4cjBFblNrSmlLRngzN3dlbnhTS1NkaS02R1Zwc1hrUHl6MHR0a2NkSy1XRm9hZ1B6bklHaTF6VVlmdzNaNDRWcFRXYXFDSnFpXzMxZDBZZEtORHZfckx1eEM4UdIB9wFBVV95cUxPeGhqYjFsazdhaENpSk1rY3lYM2lJSmVqSU5BX3Y4VTBsb2pBNWtqbHNqblpsNzduZktWNmxhZDJ1UTZxYnp0bWdqRFlkTEZ2aWJ5TmM3QWtEaGRhZUltcjgzVFFsaXQ5ajg0VmRmTFNXSlM5dHh3SHlsRWZOSzN4TkxUYnl2cXg3VHdTaEI0TklnTFBFVVVCRUhHRXgyR3l1bWpEeHZmQVBFM2Q4RnZoYzRiaTNYNUFBQm5XS25HcE1JRzJUT25sbXNrWGJEajBWSHJSOXlGMWFiWHJMb2pZWUFUUHJuZ2VKellQUHpEaEZKQjVYaHI0?oc=5</t>
         </is>
       </c>
-      <c r="E134" s="18" t="inlineStr">
+      <c r="E134" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -4269,7 +4272,7 @@
       <c r="F134" s="3" t="inlineStr"/>
     </row>
     <row r="135">
-      <c r="A135" s="18" t="inlineStr">
+      <c r="A135" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4279,17 +4282,17 @@
           <t>Justin Ryan’s Glow Capital cleans up with new investment</t>
         </is>
       </c>
-      <c r="C135" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D135" s="18" t="inlineStr">
+      <c r="C135" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D135" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPRWlpNFBQUTVzOE5yejU5a0tGcUN4ZHJieTV6S21BXzIwbGRmNXluSi0yVUlmaHp5Y1BaZG5CT2lVblktM3BvSDBDdEZ4d1pHLTI3NVRzeHNDdjl6Tm1tYUVLSkdoUlNidGhXUFpwVHNSRXZBOWZjVk85LXVHLWRRUUEtWDZ5Mld0T1ZPMEZoMi1hcHBWRGZJaDNJVDQ4RWkxVk9lR0JDSQ?oc=5</t>
         </is>
       </c>
-      <c r="E135" s="18" t="inlineStr">
+      <c r="E135" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -4297,7 +4300,7 @@
       <c r="F135" s="3" t="inlineStr"/>
     </row>
     <row r="136">
-      <c r="A136" s="18" t="inlineStr">
+      <c r="A136" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4307,17 +4310,17 @@
           <t>RBA crackdown on fee rort is a raid on banking’s hollow log</t>
         </is>
       </c>
-      <c r="C136" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D136" s="18" t="inlineStr">
+      <c r="C136" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D136" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQSHhSOWlMSVlkVlVaZnUwZjBzWHJxSUcyamI4ZjkxNWluOU1NUHA1RjJFdWZFaFBHTTRuRndCd0xabFJtclhZeTZ3bC1aRG5UREg5UVFyWDdIODhtV2JSdFV5R3hKZlZOc24xQlhGOWNJRXdFZl83TjU3emJ2YjZkVmFtSEpPSDBoRUNTc2JCZVNkZk1sWjI3RWo0SXZOY1dMU2xicndqVGdUOVk?oc=5</t>
         </is>
       </c>
-      <c r="E136" s="18" t="inlineStr">
+      <c r="E136" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -4325,7 +4328,7 @@
       <c r="F136" s="3" t="inlineStr"/>
     </row>
     <row r="137">
-      <c r="A137" s="18" t="inlineStr">
+      <c r="A137" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4335,17 +4338,17 @@
           <t>Inside Project Taronga: Koala’s choppy run to the ASX boards</t>
         </is>
       </c>
-      <c r="C137" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D137" s="18" t="inlineStr">
+      <c r="C137" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D137" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQeHotX0dQdVN6YWlES2twNXJaUUtzOEdESGJrbUdacmwxOHBDaXh6SVViWXJkMUloTGtpN3h2anNTMm1XWWVqSU5uaFlLdDZKaFV5d1BYZ3lXUE9NN0ZxN0hMWlBRejVlTUNwMUIwY0hGMmlVcnltR21GREw3ekNSSzJFUkI3ZWRINU9oOU5TRTdmRVp2MVpBQ0pPVzJHTi1ZZTFDSnBtSWwwWjRVQmpGT0N0NjlELUo5Slk5VTBYUTh0Zw?oc=5</t>
         </is>
       </c>
-      <c r="E137" s="18" t="inlineStr">
+      <c r="E137" s="19" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -4353,7 +4356,7 @@
       <c r="F137" s="3" t="inlineStr"/>
     </row>
     <row r="138">
-      <c r="A138" s="18" t="inlineStr">
+      <c r="A138" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4363,17 +4366,17 @@
           <t>Spotlight retail billionaires weigh up Barbeques Galore purchase</t>
         </is>
       </c>
-      <c r="C138" s="18" t="inlineStr">
+      <c r="C138" s="19" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D138" s="18" t="inlineStr">
+      <c r="D138" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxNVk9feFNXOE1feC0wX1ZHaW16bUR1SUpKRWtjTHdfMDk3Y3J6WjFjNGdYcGdzbmk0c2N2b1N4cXhGVXEtU0hjYzMxRVlZT3FYMGZkend2OGg0VkpxdS1tNWM0RHRMNk5GbUJfVVVfc1NhTmFsNDlvMThjQk9PcTVnNTBUeUw4ZXNybW1ES0dXdlYyb291V280MTFCdlZMYVRIUVQ2dmUwblZjdnQ5N2pzLXMxOTcya0V4bFREM05PZkZZOHhuSTAzTFpxZUg4MmlUaDMzVHRROGQzUFkzVUFwZlZidGJhVXRTV2dPLdIB8gFBVV95cUxPRFBhdmluUkZtRldxd21BSmdkSWJsR2xNc1BYY0VGUjdVN3kweWM5WjR1VUhuRDNKYmNJellHQUl0cVJBd1o0QkdObW1PMzBTLUJmdXBlQnNJcGx5Qk1DVndrSHhzR0E0ZVRsN2t5M0ZqV3ZJUVhLdkN2d0I1VkVHZkpVQ3dNTGZLWUV2RU9tbXRvRHhDMmZzRk9fWktodmYxckZXU0dTcWg4X3M5WFJ6OTBYbjdyd1BxRnBia3RuMWJNOWE1M0Nla29hMGVPRExQWW02TWhfbXRlZkxmZ0tYS0tldDdLM3ZCU2s5UVEzNVN5QQ?oc=5</t>
         </is>
       </c>
-      <c r="E138" s="18" t="inlineStr">
+      <c r="E138" s="19" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -4381,7 +4384,7 @@
       <c r="F138" s="3" t="inlineStr"/>
     </row>
     <row r="139">
-      <c r="A139" s="18" t="inlineStr">
+      <c r="A139" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4391,17 +4394,17 @@
           <t>Chargrill Charlie’s opens in Redfern</t>
         </is>
       </c>
-      <c r="C139" s="18" t="inlineStr">
+      <c r="C139" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D139" s="18" t="inlineStr">
+      <c r="D139" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxOalVFNURyb3NER1J2SVpsazF0S195WUpTdFcwaHhvNG9Dblc3MEw5SS0yakJiaDJLeDRZLVBSZmw5SjdkOVpEeWFmaTN4Rnl2SkdJbHBDU2VXdjA3Sm9JU2drXzNxOU5sZER6eGp6MmljX2RMWmM0VjNXeVZsWFpqYW53?oc=5</t>
         </is>
       </c>
-      <c r="E139" s="18" t="inlineStr">
+      <c r="E139" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4409,7 +4412,7 @@
       <c r="F139" s="3" t="inlineStr"/>
     </row>
     <row r="140">
-      <c r="A140" s="18" t="inlineStr">
+      <c r="A140" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4419,17 +4422,17 @@
           <t>Former KFC exec named new CMO of Pizza Hut Australia</t>
         </is>
       </c>
-      <c r="C140" s="18" t="inlineStr">
+      <c r="C140" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D140" s="18" t="inlineStr">
+      <c r="D140" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPaDJEelhoN2tnME1SazlhTTZpOVhaWnFnN3ozUTFkZmZ4LTFXdGtQSWZVcUN4aVdhSERUSFY5NDl3X2QtUDRjNWx0WElXV1M1bTVnNWRrMURkMFlwQmljMkRlc0tnbHVzZkdha21YNWFlWC1JX1dHX0hCYi1PRGFoVDdxWDk1OGtUeXI4RkMtbXUyUVdWbHlmbGN3?oc=5</t>
         </is>
       </c>
-      <c r="E140" s="18" t="inlineStr">
+      <c r="E140" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4437,7 +4440,7 @@
       <c r="F140" s="3" t="inlineStr"/>
     </row>
     <row r="141">
-      <c r="A141" s="18" t="inlineStr">
+      <c r="A141" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4447,17 +4450,17 @@
           <t>Restaurant Brands New Zealand snaps up Taco Bell franchise from Collins Foods</t>
         </is>
       </c>
-      <c r="C141" s="18" t="inlineStr">
+      <c r="C141" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D141" s="18" t="inlineStr">
+      <c r="D141" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNak9JTVQ3ZUFpN3BYU3U3d1FwdVAwU3V6Z3VxREhqX2h3Q0tFalhDMHpqWFpfcUxuc3NMSjBsRi1QR21oNmg2NUt4dHFPV3ZDNjE1N01yT2JuSFBjU2dGeFl5SjVmSEZtSlpfZHVtTThTZmxrLWttZGxYZURvOTBRcjRMRVFIV08xUU1PUXNSMHJ3MV9LSVBMSzVIX1RkRFhZa1Q5cG12eWVJT1dCT3Nr?oc=5</t>
         </is>
       </c>
-      <c r="E141" s="18" t="inlineStr">
+      <c r="E141" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4465,7 +4468,7 @@
       <c r="F141" s="3" t="inlineStr"/>
     </row>
     <row r="142">
-      <c r="A142" s="18" t="inlineStr">
+      <c r="A142" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4475,17 +4478,17 @@
           <t>Gelatissimo hits 60 outlets with Zetland opening</t>
         </is>
       </c>
-      <c r="C142" s="18" t="inlineStr">
+      <c r="C142" s="19" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D142" s="18" t="inlineStr">
+      <c r="D142" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxObVNNeU1EalQtaFRrbVIzdGRDcjIwampSckY5VlM4RzF1aXpmX3hweTFucmpxQ3gxUFhGZmVrck5GTzNyb3VxR1gtRVBwbXRVaFE5REJ3UWQ4U3hqd1RFU05kcVA5ZlVEUG80cUU1a1U0VWNtMXp2QmkzZ3F5X01pcEt5WkxvLUg2UTFzTw?oc=5</t>
         </is>
       </c>
-      <c r="E142" s="18" t="inlineStr">
+      <c r="E142" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4493,7 +4496,7 @@
       <c r="F142" s="3" t="inlineStr"/>
     </row>
     <row r="143">
-      <c r="A143" s="18" t="inlineStr">
+      <c r="A143" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4503,17 +4506,17 @@
           <t>Investors flock to Koala as furniture retailer soars on ASX debut</t>
         </is>
       </c>
-      <c r="C143" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D143" s="18" t="inlineStr">
+      <c r="C143" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D143" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOWHFPQVY5MGg5dzRzeDNQVG5PM204dkUyQWtYNTVGQWpIY0NFWTUzTFZMV3VuV2FWTWZqSVpldmdNY0YzU2VTX2c5eXUtajJPWXJmSm5iRlRleWNRMVhmZUJxaXNDNENMNGV0RmZWNEkxTWZPTE95VGtDYWhwSzZGZzBNbGZ4OXZBM2FxbElnTU14WnpVbUhyYTJGaGZHdjd0Yk0tRDlacno?oc=5</t>
         </is>
       </c>
-      <c r="E143" s="18" t="inlineStr">
+      <c r="E143" s="19" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -4521,7 +4524,7 @@
       <c r="F143" s="3" t="inlineStr"/>
     </row>
     <row r="144">
-      <c r="A144" s="18" t="inlineStr">
+      <c r="A144" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4531,17 +4534,17 @@
           <t>Australia's Collins Foods to transfer 20 Taco Bell outlets to Yum Brands</t>
         </is>
       </c>
-      <c r="C144" s="18" t="inlineStr">
+      <c r="C144" s="19" t="inlineStr">
         <is>
           <t>Reuters</t>
         </is>
       </c>
-      <c r="D144" s="18" t="inlineStr">
+      <c r="D144" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOWnNHb0VCMjhOUTNrUS1WOUhmRlpnelpxMmtFZmxGY1poSzB4dHFWcjdNN3lWcVhyWUpSU1UwSjhpY2dUNlg1N1hQQ1pRVUFKcm5MSHV0TWYwSmtqTHF4a1FQX1MtdmhqUV8tZ1lJcC11c2J3TXJWWG5mVmtSUkFWTDBZaXc4QVcxeGhxeHVBQVJ4TVJ1Sm5scHlmNTFsSzJWcktEekp0dk1QeFJSdnVpd2Mtdklya3ZiQmJodw?oc=5</t>
         </is>
       </c>
-      <c r="E144" s="18" t="inlineStr">
+      <c r="E144" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4549,7 +4552,7 @@
       <c r="F144" s="3" t="inlineStr"/>
     </row>
     <row r="145">
-      <c r="A145" s="18" t="inlineStr">
+      <c r="A145" s="19" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4559,17 +4562,17 @@
           <t>KFC operator Collins Foods offloads Taco Bell outlets</t>
         </is>
       </c>
-      <c r="C145" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D145" s="18" t="inlineStr">
+      <c r="C145" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D145" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQV2x0VTJWLWNLcGlYWDZCc1NpbTd3MnlvX09kMWpIeS1jMGQ0OF9sc0k2RHZFY0JudmVJdVJtNnF1Zk5vYTRDNG1aNDlVQmZMM0RLRFZWZFR6bUhJQVZlc1hDY2NCbDJVMzBCMVF0ZlhvNEpVOHNUV0Uyb0hCQU1ndzN5Vk5pMFlSQWxXaktmdTQycVctTGx2dGV1Um5ycDFFWmVkQ2puLWlTZw?oc=5</t>
         </is>
       </c>
-      <c r="E145" s="18" t="inlineStr">
+      <c r="E145" s="19" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4577,7 +4580,7 @@
       <c r="F145" s="3" t="inlineStr"/>
     </row>
     <row r="146">
-      <c r="A146" s="18" t="inlineStr">
+      <c r="A146" s="19" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -4587,17 +4590,17 @@
           <t>Count launches $40m capital raising for financial planning acquisition</t>
         </is>
       </c>
-      <c r="C146" s="18" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D146" s="18" t="inlineStr">
+      <c r="C146" s="19" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D146" s="19" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQQl9MSkpfamt1UUxyeTVILVlKSThwOXVrUmxfdF9nMVIySC1pc3RLNXB0c1Y2X2ZRakw4dS1FLVB3YlJlQ1BkcXBRUGc1NXNKS0lMblVpQVhsZWZlNTdPRXFQMzdyUDNtTjlkeHQyRkdXaUtiQzZUVHpPV3p3a3hqYVdTaU1CdWFvYmhiTmhBeFVwZlozQjJnWHl3NTYzYTlTbkgxUi1OYXlLcS13eG05ZnBsQUthQ0E0?oc=5</t>
         </is>
       </c>
-      <c r="E146" s="18" t="inlineStr">
+      <c r="E146" s="19" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -4771,6 +4774,90 @@
         </is>
       </c>
       <c r="F152" s="3" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="20" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>Luna Park owners buy Bankstown’s grim looking pub in $54m deal</t>
+        </is>
+      </c>
+      <c r="C153" s="20" t="inlineStr">
+        <is>
+          <t>SMH</t>
+        </is>
+      </c>
+      <c r="D153" s="20" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxNamwxcmFfNUsyQmlaVUdLcFA0MXg2enBINTBEazRPNHp3Rm0tQmRHZWhBdHNwMHJ1M3M4b2VTaHptUV94TDlOMzBqV0dlRnVfM0VzVkxrelBTZGQ2TGQ5OEx6TGpZOTZzQTV4bVhudWRPUTBFTVBPd3RuUHpSQmNzX3NndGcwaVNaS2w4MlBrNW91TGZwSnlLN29Fd0haY0ZUZ1paVUJVNWR1aEt2TUktNmVVTE8xTUpBdUZ4WlZ3OGR6WWR1cWY0Uw?oc=5</t>
+        </is>
+      </c>
+      <c r="E153" s="20" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="F153" s="3" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="20" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>First Guardian boss grilled over chef’s loans and missing millions</t>
+        </is>
+      </c>
+      <c r="C154" s="20" t="inlineStr">
+        <is>
+          <t>The Australian</t>
+        </is>
+      </c>
+      <c r="D154" s="20" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingJBVV95cUxQNmxSS1NQQ1VMeGNpQm9YejFjOTRjR2dzdGs1RnFmWENiaWZ6RHltNC1uZW9wRmpPLVVUeTRtRS03VnlwRUVNOEhqams4Q2I1V0o2SGpaZERlQW1CeEkxWGF1cmJsVnVVekJldkVacXFhNkcxTjdHN093TGpCMXZzZHJlUmQ1ZlBjR3paaHZSNmoxN1htdnA5SExLalpPTkp5ZjN4Mm8wUUJUU0ZmOG4wNEt6UW13anY5R19tb0VOdEZjVFRwMWJ1d1hHRjE5VVp2eFlJTTJPYlVPTmZIaGtKdkpWS1hmaHM2VDFmcXU2RHV0bkxfUmxNQWd6N2pJLUp2ME1HRnkzX2N3b0hsR204RGtuTGJDeXUyQURFM2V30gGjAkFVX3lxTE8yWXRQT2NCRkcweXlsM2FDOTcwMzJpSURadzQ4aGJKemkyOTN4VWNVcFNHdS13bFd4VS1UWWRfcWI3LVpqSHZSTFZSNkFHRlN5aUNkc2VkVjhzb0VlVmg3UUk0T0ZINHN0NTR0ZFdmaVlTREV2SUJ3Z29mbzlEYzZjVTMzX01Eb3Q1VXFTYmdJNjhsQ2xfczNNTkJsd2dQWGJzT2FJbDI5bHh6dVI3T192NC1sVUtoNnNZOVBBWS1GSDc5ZzJJRGNiUXBQTjh1R2k0OE12VXdMWWFpNWVzVG5WOG5idXR6c0UyZTJQY29IMFUtTlE2UUxDdzFLY3FPbVV4TUdRSDdXbXZxeXNJcmhVWlBYX1FFQXg3a0V3RDFOLUtidw?oc=5</t>
+        </is>
+      </c>
+      <c r="E154" s="20" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage</t>
+        </is>
+      </c>
+      <c r="F154" s="3" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="20" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>Wham, bam, ASX finally gets slammed</t>
+        </is>
+      </c>
+      <c r="C155" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D155" s="20" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxORjBOYnVQcS1SOUFpaWlmd2ZYRlIzM1pUUHFWeFhEV1EyLU5NNmd3WmdQNUhOUzUzVWRIUGFNTngzc04ydWRKU2gxS0hveVV2di1acnBpenRyVGFhY0Zpb2ZKbXozV00zNjI4Z2xrV2tNa19uSU9uUjBZSDhERWNSU0xMWFROOE1I?oc=5</t>
+        </is>
+      </c>
+      <c r="E155" s="20" t="inlineStr">
+        <is>
+          <t>Australian Economy &amp; Markets</t>
+        </is>
+      </c>
+      <c r="F155" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>

</xml_diff>

<commit_message>
Update news log — 2026-04-03
</commit_message>
<xml_diff>
--- a/news_log.xlsx
+++ b/news_log.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -87,6 +87,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -504,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F155"/>
+  <dimension ref="A1:F156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -548,7 +551,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -558,17 +561,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C2" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D2" s="19" t="inlineStr">
+      <c r="C2" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D2" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E2" s="19" t="inlineStr">
+      <c r="E2" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -576,7 +579,7 @@
       <c r="F2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -586,17 +589,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E3" s="19" t="inlineStr">
+      <c r="E3" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -604,7 +607,7 @@
       <c r="F3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -614,17 +617,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -632,7 +635,7 @@
       <c r="F4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -642,17 +645,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D5" s="19" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E5" s="19" t="inlineStr">
+      <c r="E5" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -660,7 +663,7 @@
       <c r="F5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -670,17 +673,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D6" s="19" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
-      <c r="E6" s="19" t="inlineStr">
+      <c r="E6" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -688,7 +691,7 @@
       <c r="F6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -698,17 +701,17 @@
           <t>Firmus tees up non-deal roadshow around the globe ahead of IPO</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D7" s="19" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQaFNqUElYdTEzaXhfNjhmemdmbVhoNk90MDh0SlJaVU1OWnZwZG13N2JiYmRtaTdWazJyODA1SlRaVWphU01IVlZ0NWt0ZkgxNXZxMHNrRjBEclZ1T2pNUG9icnNBb2xFQ3JweDQtcXB1VU10ckE4Z1NqLXZiRTl3Y3FnanB0cGFqd2p0LVVOQ1JuRkdqX3NYSm94V3lZUzlUdHdweTgyZURiSVBnMFdV?oc=5</t>
         </is>
       </c>
-      <c r="E7" s="19" t="inlineStr">
+      <c r="E7" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -716,7 +719,7 @@
       <c r="F7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -726,17 +729,17 @@
           <t>Auckland’s BlackBull charges at dual listing; BJ, UBS tee up roadshow</t>
         </is>
       </c>
-      <c r="C8" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOSldYQUoxbkR2TnRkbGpzZ29USEZhazRwbUpZeC1BQVJkMGl2WTduQlFSd21xUGdCNFZmYk00WEZLVXlkalBybGtzcmVnVWdtY3lsb1hGMVVGMlJreS1lWXQycjZZOGhXd2VKcDh0UXQwaG1VM1AwQ25md1VaTHlhNFJiRk1VT1VhSERKbjc3U1dZUnN4NmhzMkFiMjFza0s3bXFEYzExNXZWOHc2eHY4UVd4eGhKUQ?oc=5</t>
         </is>
       </c>
-      <c r="E8" s="19" t="inlineStr">
+      <c r="E8" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -744,7 +747,7 @@
       <c r="F8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -754,17 +757,17 @@
           <t>Biotech HaemaLogiX prepares for ASX debut; taps Ord Minnett, Canaccord</t>
         </is>
       </c>
-      <c r="C9" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D9" s="19" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNVA5RnV3SldDejg5M044VUVsMmpxdkxqTl83QlRYNmFseUUzTFJScEJRZEhtSW1CSmN3WjY5TmVud0tjTWdxSmd3UWZDUnVQYVB1QWdzQUFvVXVMM194RFFBdURENi02eHdrTkFXWURxWHNxR1d1VWxQYmtRR3p4MVc4NGdWZVhkQU54X3JyYmJhbnk2R25LdXNBRlBRUktUdm9qTkQwektJSW51eEQxSGJWY2MzUXc?oc=5</t>
         </is>
       </c>
-      <c r="E9" s="19" t="inlineStr">
+      <c r="E9" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -772,7 +775,7 @@
       <c r="F9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -782,17 +785,17 @@
           <t>Craveable Brands taps Josh Kilimnik as Group CEO</t>
         </is>
       </c>
-      <c r="C10" s="19" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D10" s="19" t="inlineStr">
+      <c r="D10" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPOExiR2M2NERiQWotTk9wLUNoX1owa0RBdnhvUEVrX242NTFaZFdZQ1pkNFAyQmUxRGFKYzZZZEN2TXg5T00tQXEtZUNxOXN0S0F2QXlXMHV6NVJUeFJ2ZkFTUW1WWTlqc1kzX1VrQlhTblE4ZTdVTG83Q0Q5MGd5dVRnYUtybHpBRmFVeW5nNmUtR3Zy?oc=5</t>
         </is>
       </c>
-      <c r="E10" s="19" t="inlineStr">
+      <c r="E10" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -800,7 +803,7 @@
       <c r="F10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -810,17 +813,17 @@
           <t>Zarraffa’s Coffee celebrates 30 years, eyes nationwide growth</t>
         </is>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D11" s="19" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOcXNzUkRLemZEOWtOZjhvRUtzcUZrSTdzV0s0LUJTd2NGRk1Gb1NSLUR5Rlh3NUdWQUJkVWctb0toUFBRajlMcWV3VnNyTUtydy1PSUoyb1NCOGVtMUZqRVN0MzFkVkNlOUZNVXlHN2kzREhSdWJQUnJqa0pnUzExTVZSc1NCVFZSNlBSUWNfWnZ3MC01aUx0UWF5SkNOaHI3ZkE?oc=5</t>
         </is>
       </c>
-      <c r="E11" s="19" t="inlineStr">
+      <c r="E11" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -828,7 +831,7 @@
       <c r="F11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -838,17 +841,17 @@
           <t>Zarraffa’s Coffee eyes 200 outlets ahead of 2032 Olympics</t>
         </is>
       </c>
-      <c r="C12" s="19" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D12" s="19" t="inlineStr">
+      <c r="D12" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPMUFjRTlGVFBqYzlPWXdzQ0dKVVlhWGxncUQxTDd1R0VHcThlV3ExVmo4SlBGSHVuUGZrMGNqSVo1YVpDWHViMm5KZWIxcHNMMHo0b1FQcmxUNElDR2lEeWRuLWZIN2lyQUV0VndEUWNkNU42Z3AzNXRlbm50NzhtTXZ0Q245dF9hNzBxOENuMXZsVlU4Z0JGVElR?oc=5</t>
         </is>
       </c>
-      <c r="E12" s="19" t="inlineStr">
+      <c r="E12" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -856,7 +859,7 @@
       <c r="F12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -866,17 +869,17 @@
           <t>Aware Super appoints new head of private equity</t>
         </is>
       </c>
-      <c r="C13" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D13" s="19" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNVHJXNWEtdEZZUW1fZzdYMTB4RklBTUh6dUNKQ3BrTlpYUnBwRURIVGZjWTV0OUxScnhGMVNSczhLUjVqOEwzbkR2WWlEbmF4ZkNUdHNQY0J1djI0REctbHd2SVhUNlNCa2M5bFhOQ0JPU0RHOVVTQkEzRDdGMjRZbVFDOUdlTXNNczlmZWF6bXlfbEFGRE0xbkZQaw?oc=5</t>
         </is>
       </c>
-      <c r="E13" s="19" t="inlineStr">
+      <c r="E13" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -884,7 +887,7 @@
       <c r="F13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -894,17 +897,17 @@
           <t>Commission wrinkle over UP Education sale</t>
         </is>
       </c>
-      <c r="C14" s="19" t="inlineStr">
+      <c r="C14" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D14" s="19" t="inlineStr">
+      <c r="D14" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxNSV9GMjhqM2ZSanI2X0w2OVlQVFRQTUoxYzAxaXVZMmU1REVTcHlUeEltdXJtaXZrcUJWdDZxNGpYTTZYSFE2TkZHeG9OaVRZakoxV0s1U01TVjJpWlhaSENfNVhucG5NVzFMbTVBY25zWGRSODBtRGtkS1owVTlJWnNfcTJ5alFnbVl1SU9aUDF1QWxJLTBSQ3kxUUFlZnpJMlVEQndFSGRGbDF6WVBUVHlCcDM5Qnh3R2xBMG9xN2FLckNzbUFOWDI1aVF1YV90d0twd0ZmMnUySDBMdG1R0gHkAUFVX3lxTE5EWVp6VzZWb01TRmlHSS0wMExldkJwSHJjdlZXdElsRlpBTEtVMkd6VzNQa1RpVDNsOFQzaGZ2VHpzUnBDYk82RmZGQWJuTmVQMXhxLXVmdVFxTVZOZTBsOHZ0V3cyVVVkNWUwVUxSc0xNSU92ZktpdFRfYnQ4WHBTX3A5bFhXZ1YwZXNrc1BSZEU4LVYybnNBd0dCdk92OFUwclJCMzdoU0ctX1pEdTAwY0JiTWQ4S01QRE00TW5EUEJwR2YtczZ0T005bTJnN1RDY2p6NFF1SndfLUo4QzJUWk1tRg?oc=5</t>
         </is>
       </c>
-      <c r="E14" s="19" t="inlineStr">
+      <c r="E14" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -912,7 +915,7 @@
       <c r="F14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -922,17 +925,17 @@
           <t>Gloria Jean’s owner has an angry shareholder on its case</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D15" s="19" t="inlineStr">
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D15" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPTnZwUVBCdTFJZWkwc0YtVmJqMkNPcUR5RktjMlVURmhROFZkYUpXM01iRUh3SnJEUElxRGlSNk9DQjZSdTdNdmZwWWpONjlmR1hoMl92cUNmd3M4cnJhVkNqc095MmN6WXBYUmdEblB0eERtVDdlUU4yNGFjXzVnT19rOERIRzVPNzY3VDNNRS1tVGVTX3pKMVRpTXZVR1ROLURBLWtJbVZhY0lSU09DNkE2NzFLbEFU?oc=5</t>
         </is>
       </c>
-      <c r="E15" s="19" t="inlineStr">
+      <c r="E15" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -940,7 +943,7 @@
       <c r="F15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -950,17 +953,17 @@
           <t>Oporto-owner Craveable Brands hires new CEO from Domino’s</t>
         </is>
       </c>
-      <c r="C16" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D16" s="19" t="inlineStr">
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D16" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNNmxfQVc2Umc4QWwzSTdsZTFvejRzTzZxXy1ScGlhXzh6bm5JS3IyX0xTNDVBNjh0cXpPbGhxNU5xUHhQN3EtRF9aV3FEc2JoSG5QTU1WeU1TLUJfZzVUT2N6dXloQXhZaHB5djB3dDFKN1llVmI3UVpKNjJTNlcyV0ZDcG9GdVdSdW41ZkN1b1N3SFFIUzcwRkQ3UHY2TmxERmZwTlA0RzU?oc=5</t>
         </is>
       </c>
-      <c r="E16" s="19" t="inlineStr">
+      <c r="E16" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -968,7 +971,7 @@
       <c r="F16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -978,17 +981,17 @@
           <t>Brookfield, BGH Capital rub shoulders in ScotPac’s data room</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D17" s="19" t="inlineStr">
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D17" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPMVlxbzlQNnFXWnJFNU11Y1BhTTVqbjN4RG1nbkZuN0pkdDFFaUhJN0RaVnUtWDlZSGJWR1ozQXk5UUx6RVdOcjBPU2t5UzN4T0JvUFJISnNvVWxQemd3blNHZjRQVVVZQk1nZER0Y0JfY3VvQ0t1a09sM1RTS2c1YTJyUmdzYWh1WGRUNjl2dkdzYTJJeHVhMTdqR3Y5WVlHVEtSZHp1cmVYYmM?oc=5</t>
         </is>
       </c>
-      <c r="E17" s="19" t="inlineStr">
+      <c r="E17" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -996,7 +999,7 @@
       <c r="F17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1006,17 +1009,17 @@
           <t>Payments player Pay.com.au hits the road(show) for $850m IPO</t>
         </is>
       </c>
-      <c r="C18" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D18" s="19" t="inlineStr">
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D18" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOMFZleXZrbU53TzBlakI2ZmJKTjlrN3BoQlRaWjQ5cXFzTllKWmFoRm1UT2xDUHBtNC1QNTNiX1BwSzllMkRZdHIzRlAteDREaUczN1JTNTByTW1jNnR3d2NnR0RxUDBxeHYyWU1CSUs5MEZad2JqSGF6ZUxHZUNtZmFQaTJZZVJVZ1B4MkZ6V09QMWIxaUNHQmVzTDhvWVA1Ty1UbHgtQnRrQQ?oc=5</t>
         </is>
       </c>
-      <c r="E18" s="19" t="inlineStr">
+      <c r="E18" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1024,7 +1027,7 @@
       <c r="F18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1034,17 +1037,17 @@
           <t>Another year, another IPO cold shower for investors</t>
         </is>
       </c>
-      <c r="C19" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D19" s="19" t="inlineStr">
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D19" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNeEhzYzQzdjR5MDJCWkd6Q2VLdEZzbzRoWnNOcXFlQjNfMlV4Q0NQRjExMlNhT2NPcnRBbW1sZUkteXo4N0dGaHNNeGZJOEZ2aXFvdmZiN2V2QzdOMzFteFRnY1RVRm1rQXltWmY5VFZOdFVNNVpudVp1dTlrcFM5b1k5SmlWQllDMVFXSjA4ZVpSZHgtV2JpWDJ4SkFRbVE?oc=5</t>
         </is>
       </c>
-      <c r="E19" s="19" t="inlineStr">
+      <c r="E19" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1052,7 +1055,7 @@
       <c r="F19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1062,17 +1065,17 @@
           <t>Priceline Pharmacy franchisee sale narrows to final four bidders</t>
         </is>
       </c>
-      <c r="C20" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D20" s="19" t="inlineStr">
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D20" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNR294am9sYWNiQ3FVT1B6YlV5ejMyeHAyT0FibTFVbU5pcjZyaVRyazEzbFkxd0lrcnpZNGpTYUx4Ykl1Xy1sZF93M2Nid19ydUFwbUJ3ZHozaURaNkRoOE9OMnRBRGZfQVdCVWZCaVhhNnZSRjlwYUdDVnp2WU9HUkJxbE1QMV8zdWxYRTNBQWktR0xSOFU4dmtXZWk0am9SSU92NWp6QUZmTVU5TzJEOEJNak5fQUtN?oc=5</t>
         </is>
       </c>
-      <c r="E20" s="19" t="inlineStr">
+      <c r="E20" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1080,7 +1083,7 @@
       <c r="F20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="inlineStr">
+      <c r="A21" s="20" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1090,17 +1093,17 @@
           <t>Private equity gets better image of Qscan</t>
         </is>
       </c>
-      <c r="C21" s="19" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D21" s="19" t="inlineStr">
+      <c r="D21" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxPRjVmT0hDRjZLblB1VHdPRmRGeXhKdDJHdWxDTzV4RDZ0VzdHaUFfOVlnZjRQMWhKcWMxby1oRDR6N2lQZkI1UDE1REppS3c4LTVmU3p5b2wtblRCWnhNajFnZGNHaGRJUHFMUGRtTHAyQmIxOHhNNTgwRWVSeWp6ZWRxbUY0WVhiUnhMRUpDLXNwS1RuelJldTk0Z1R0WHg0XzNXNTA5Rk5TRFZhU1RNVnN2TlZuaFE4OWtIYXQ5a2VGSW1UWmt5Rlc4Q2lIXzF3YlkwNVhfUzJDV0dQdVAxa2RKc08wRGR6TlB2Vi14QV9BdlhyaTZsM2pEVGZycTjSAYQCQVVfeXFMTWpnb0lWQmZ6MTFnRGhWNTNqczk1TWhTcUFEMVpDNnJ4ZWVxVlRUODhJXy03NHdGZVJlMmhyUHM0Nlh4NlZtTzRhQ0xxRDFLVHNzUVNfbWxhS3BLUEQteEMzZHRrc0F1eFRzYmxVNDZlSURyZDB5bF9wQTNRRU5yZEs1Z3pFRTdwcFBaMkNlN0JvT1NEYkFWVUJNcHJqcEM5RVJYa0JFUVl6cThyQXloaERzQjhkTUVPakJqb0hzNVlwSWxNS0dmZkNFSG9Gb3dNUnVvUnV0d3MxSmpzdFZKTHJ2RTQwRUoyMEVLLWMwT1NnOHdXVl9lRXNDWEFndzJFSDlZU0o?oc=5</t>
         </is>
       </c>
-      <c r="E21" s="19" t="inlineStr">
+      <c r="E21" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1108,7 +1111,7 @@
       <c r="F21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1118,17 +1121,17 @@
           <t>Oporto CEO’s first year reshapes brand and network strategy</t>
         </is>
       </c>
-      <c r="C22" s="19" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D22" s="19" t="inlineStr">
+      <c r="D22" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPY25mNTJfT3FiVlBPZE5CcVNkR1UzR2xWaUtJSmxhU3EwcEMzQi1ISDFSajlCQWk1UUJpZVJ1Q19ZV3Jjd0Noc0l3OExpMXhSQUVVdHhCLTBlOXNoZzA3UXZBdkR1VHBvMmVsZkNhUFJndm1DdGpnX2w0ZVViU2phZ1RmYXY1SlhwUnhKSUxBQVZZUXpqNHQxQmo0Rk1iV0g0OW9qUS16eWRSNW5FaW1yQQ?oc=5</t>
         </is>
       </c>
-      <c r="E22" s="19" t="inlineStr">
+      <c r="E22" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1136,7 +1139,7 @@
       <c r="F22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1146,17 +1149,17 @@
           <t>The Melbourne restaurant our reviewer grew to love</t>
         </is>
       </c>
-      <c r="C23" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D23" s="19" t="inlineStr">
+      <c r="C23" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D23" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOc3YxQTljcHJXVWtRX2ZGM2lpM2pILWNwSFg0MFJrNmNWX0ZxRG9nV0J5N19qRWh4U0hPXzNmVVZwWk9wT2kzaFNrTlV3NEQ1Q3JpaXVIYlBHb216Q3VYVWdSRXMwdDl0SmYzdnRlSDFUYVRmRGJyZVlRZDJKTHpJOUctYlF1RDZSYjloY0hfZy13QmFTLU9UNjkwTHc1bjlGcGxoZ0ZLVU1GWTctZkdLZU9zSGhEZEpKbXJnaWJfZjd2OWs3?oc=5</t>
         </is>
       </c>
-      <c r="E23" s="19" t="inlineStr">
+      <c r="E23" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1164,7 +1167,7 @@
       <c r="F23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="inlineStr">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1174,17 +1177,17 @@
           <t>Crescent Capital strikes Benson Radiology deal for close to $400m</t>
         </is>
       </c>
-      <c r="C24" s="19" t="inlineStr">
+      <c r="C24" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D24" s="19" t="inlineStr">
+      <c r="D24" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOLTNrWG1ZZlFoU3pDZ3E2SEgwMlhzQkdtQUYzaHZTZmYwU3ZhMnE0dlkza005VkZmZ09NMExlWDVncnBmYVVISXJ6X1ZjNHhpM2RnSlprY1dnbndJNUczcDVtNXNRY3pVNW12bm5rUVdqVmR4R0JlVHFuN0RwTlFkR2xrbFFpSl9jcm5oSjk3aFM1clBSVDhnbkhoWUREeUhsbVpvQW90d05xOTdfOV9nbW5POFdmelJkVlpsUlRuYl9odmRNVUV2S0pCMFBMTS0tcVhGVGFYU0h2d9IB3wFBVV95cUxPWEs4R2pxdThPbHJHb0dBT183SkRHTTlXNzdWazcxdkd1eGx2VlAyM2VVbEtEbWxTZ1R0TlBFRmRMZTFoalgxSmVVRUJFR0c0RFYzZVJFODg3dWxicU9pOHppeFhjaVp0WWlyTnUzV1dyZXdkMHBDVHI4LUVQdjc0cWpheU55NTlvdWdCZmVoODB0Mm5fbGNCTmQwLUhMZ0psQVpzb3BEUnJpSkRnOUM0c0VCdUp5N3g5MkhaM01vTHJ3NWd0ay02UXZUUG9nVkxicVc1Z0xjWGhjUDRDVjlN?oc=5</t>
         </is>
       </c>
-      <c r="E24" s="19" t="inlineStr">
+      <c r="E24" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1192,7 +1195,7 @@
       <c r="F24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
+      <c r="A25" s="20" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1202,17 +1205,17 @@
           <t>Dual-listed giant Capstone Copper flirts with $600m-plus carve-out</t>
         </is>
       </c>
-      <c r="C25" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D25" s="19" t="inlineStr">
+      <c r="C25" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNcVh4blRkQnoyaG1TajhVV0lrOEJRaHdTZWtzUnJHaEdaSXNRWThGTHlVdGl4dGJ1cTMwZ2pLcVNzUXRYNlZzVzhvaXdkNGtVUG0wN0FrMHB0R1I2Ry1jcEgtSWUtajI0cTFMRTlfdzBuMWtrZmJOLVUtMkl5dW85dFp6dEhEOHhTNzdfOFNFSGtlT0MwQnRlY0VhcUZBNE9RYzhQcDdOQUFnYkgzd0V0N253SQ?oc=5</t>
         </is>
       </c>
-      <c r="E25" s="19" t="inlineStr">
+      <c r="E25" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1220,7 +1223,7 @@
       <c r="F25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="inlineStr">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1230,17 +1233,17 @@
           <t>Guzman y Gomez unveils a new menu under $4</t>
         </is>
       </c>
-      <c r="C26" s="19" t="inlineStr">
+      <c r="C26" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D26" s="19" t="inlineStr">
+      <c r="D26" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPMjRjRTV2a3BJc3AzdDNOQktoYjBvLVZSODVsc3lKQ3pET0lxUlpkc05NcVlKRlZITjVJbjkwLS1DUFJNMGJ1amJKTlp3S3VqMWJaU3YtUENEN01rUEJiV1FNZTRXYjcyV08zZzlxNDVOSlVOTlJDOGV3QzBQcUpKa2Zab1ItNlI3ajZVVTF3?oc=5</t>
         </is>
       </c>
-      <c r="E26" s="19" t="inlineStr">
+      <c r="E26" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1248,7 +1251,7 @@
       <c r="F26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="A27" s="20" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1258,17 +1261,17 @@
           <t>Can Sydney’s burrito king conquer the $676b US fast food market?</t>
         </is>
       </c>
-      <c r="C27" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D27" s="19" t="inlineStr">
+      <c r="C27" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D27" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNM0ZFcUpLN1dUZWUyaE1LMnNZVGlEbkNNQUQ4Wmd6QVFlTy0wZDVHdnlja1gzMEZTbVpKU1Ftb3VKZ2pzajcyWU16NUtUTmR0TlZMOVhMRUNqZXZiX2d2NWY0YlJDOFhhYUE0SkhMRUprNndXak8tWGdERU90cmMxTkFjcFFVSTd5VlZ3NFVKOXN3M255MFhzZThmbi1VUGMyQ3E4d2pYcFlJckY3QlVBdVJJeF9qUQ?oc=5</t>
         </is>
       </c>
-      <c r="E27" s="19" t="inlineStr">
+      <c r="E27" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1276,7 +1279,7 @@
       <c r="F27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="inlineStr">
+      <c r="A28" s="20" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1286,17 +1289,17 @@
           <t>Drone maker Innovaero prepares for ASX float, taps Euroz Hartleys</t>
         </is>
       </c>
-      <c r="C28" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D28" s="19" t="inlineStr">
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNU3JrejNRZ1VBZVNVV29NMkFPVmRsWE4yMVZPcjk2aUNUTHFJUGFyQ1VnZEZiZlIzQW9VVzRNNDNRR01jcHo3X0tqZjB4bzhMTTI0Y3BwYUh6OGRUUGt2REIxV09oRnJoVWlVelZWaUlWUmlPQ3dJdi1TejcyaXB1Z0x1MEJRSlB3SGMwVGdXaXJJNm9TVllPOG5JZC1feEV3TVhTeExGeHR2RHFIWlVCOXh3?oc=5</t>
         </is>
       </c>
-      <c r="E28" s="19" t="inlineStr">
+      <c r="E28" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1304,7 +1307,7 @@
       <c r="F28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="inlineStr">
+      <c r="A29" s="20" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1314,17 +1317,17 @@
           <t>Bain flaunts Estia 2.0 as IPO roadshow gets under way</t>
         </is>
       </c>
-      <c r="C29" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D29" s="19" t="inlineStr">
+      <c r="C29" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNTEN1cGsxNDN2c1NqUzB6UmJ4TFl0NGZjZVN3U3oxMlVFWTF4WUZLQS13dUxMV0N2ek1XN2VURTNVWms1NjdXSm0waEdaTXQwdTdWY1MxZ1V3ZnpEcVJtczdOWGNNZ0RQNzRZLU1MTTgtRW5DZkctbXBGMmVXVXdPZW5pNThiRHEzWnB2eFZzTFZTb1ZkeW9LendkNDd0cXRid05ZSGZYbW9NZXdOLVZWODdZU3hVcTA?oc=5</t>
         </is>
       </c>
-      <c r="E29" s="19" t="inlineStr">
+      <c r="E29" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1332,7 +1335,7 @@
       <c r="F29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="inlineStr">
+      <c r="A30" s="20" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1342,17 +1345,17 @@
           <t>Carl’s Jr. Australia unveils nationwide freebies for Happiness Day</t>
         </is>
       </c>
-      <c r="C30" s="19" t="inlineStr">
+      <c r="C30" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D30" s="19" t="inlineStr">
+      <c r="D30" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNVWgwdjU1NDFWalBfMTFYX1dQOWNDbG1FVUdlcS1LTVlHZVRRTVBWTjhSMnpkTXRXNlFJdllGQUp5Mm5ObWpIazd1d0RJa3QtdFBZN1hOenBmVzBEU05wM0gtNUxPeWpsYkxyVnhWWFFOU2Y3R0tXcmNkeWhpWDh2eDZBdjNCMHhuc1lHYTZHblBPVkpfRXpKd051UWlNc1hm?oc=5</t>
         </is>
       </c>
-      <c r="E30" s="19" t="inlineStr">
+      <c r="E30" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1360,7 +1363,7 @@
       <c r="F30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="inlineStr">
+      <c r="A31" s="20" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -1370,17 +1373,17 @@
           <t>BHP and Woodside appoint new CEOs in major mining shake-up</t>
         </is>
       </c>
-      <c r="C31" s="19" t="inlineStr">
+      <c r="C31" s="20" t="inlineStr">
         <is>
           <t>ABC News</t>
         </is>
       </c>
-      <c r="D31" s="19" t="inlineStr">
+      <c r="D31" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQbTg5VFJLbWJfcy1uV3ZReTJkTndzX01qZ2MxNWkzaWZRckNLZUR1Y1VsMVRNc2FySC13U0NzalFEb3k1R3BaUEhfcTV0N1M4Q1dpSlo0YXI0UFhrMGRab2RiYV9DQVNVX01ycFc5ZFZrZWZqc1VRZXoxLVEzSDJLclJLSWg5bzN3R1I0bG9lWjVDaHE4?oc=5</t>
         </is>
       </c>
-      <c r="E31" s="19" t="inlineStr">
+      <c r="E31" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1388,7 +1391,7 @@
       <c r="F31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="19" t="inlineStr">
+      <c r="A32" s="20" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1398,17 +1401,17 @@
           <t>Next Capital sells Enviropacific unit to French waste management giant</t>
         </is>
       </c>
-      <c r="C32" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D32" s="19" t="inlineStr">
+      <c r="C32" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D32" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPR3lFbERLR2FtdmJUU3BDU2thZk00YmFHRFhXR2VBVXhQSURTeE5ONVJKczBwbzlFMnR5cmhxMnM0bzlJbWo4SXl1dHpqYWxxMUJBRjZHVUtab1RYZjZMTnpGc3FzMWQ2NjNEdGU3NTZwa0diM1lJS1haYllwTldLZlpZbXp0YzlxcDh0ekcwTy03dDdPcnk4b29HZVdqbHhZY2JPR2drM2puSVpjUzZkVjNpZUE4dVMwYlE?oc=5</t>
         </is>
       </c>
-      <c r="E32" s="19" t="inlineStr">
+      <c r="E32" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1416,7 +1419,7 @@
       <c r="F32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="19" t="inlineStr">
+      <c r="A33" s="20" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1426,17 +1429,17 @@
           <t>Future Fund private equity and real assets chiefs head for the door</t>
         </is>
       </c>
-      <c r="C33" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D33" s="19" t="inlineStr">
+      <c r="C33" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D33" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPUHNHRFhFMVdwVld6RFRZUFd3QWNOd1kzeS1QdnJxMERFSnE5LTdZcDhDYlVGcWZMeWxlR0FSRWF6YkZoQVZrZU9TQ1E4YTEydUJnOFE3enV5Rmk5UnF5VEdYZ1FMUWpKVjdjMlZZUGFsU0tKcV9Vbl8zcHp5aVF5Z2JMOUZocHJqRXNRaEp4Nm5CbDM1WkdIMHdQS2xqQnE2Tnh3?oc=5</t>
         </is>
       </c>
-      <c r="E33" s="19" t="inlineStr">
+      <c r="E33" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1444,7 +1447,7 @@
       <c r="F33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="19" t="inlineStr">
+      <c r="A34" s="20" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1454,17 +1457,17 @@
           <t>‘I actually started to die’: the new billionaire’s epiphany</t>
         </is>
       </c>
-      <c r="C34" s="19" t="inlineStr">
+      <c r="C34" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D34" s="19" t="inlineStr">
+      <c r="D34" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxPblkxbHVrdnVKY1pqQzNyWGNMZm9UYmY3dzlPaGQ4Yi1tc0U1akhrVWdIaXBpM05aZXRwTXE1eDBITlZpbDkwRXNrWjJ2YXBzX0VCY2JSLWhrVmpjSTE5eE5rLWgtc2pRZEdXbmhhWU1KeFExZDBGS2pjSkIwV0FGbndBZVAyQkg4WFRsengzSGYyZkFfQnJsQ18tUHJGNDd2T0pzZElPSVJTQkl2Rm5QTExJNHhmU2dHOHJGdTdzU08yNHRtd1R3Q0cyOF8taDktQTZvVXVBVjN1d0NHMmtFOHBWZXBFcUFWa1IyWGNDTDZUT3lQSXJHOVhxTFQ3b3RH0gGGAkFVX3lxTFBZQ3BFQWl5dEwwLW5yVWJuMU8zcXBPdE9pamRVSWVkbWNyVzgydGVOaDBROUN6RlBDbjdld05DVmZyb0R1eEN0UERubzZRU2NiMTQtVV9XNS1wYmlvZ1paM3RaOUlrTzJka0tXVVJEamFESGlSdXg2bDk1aUdhUVhBcXpnN01fX0Y0cTNvcm5DdEFFLVVERDFKTWxKZFR0UzAyblJqVHBua2JoYUdzeUNMb053ZVczWUFQU1AtVHV1d3lSSDFfZFh2cEkxSGw2MEdicEVsb2pLQ1RuQmdaRl9xNUROS3pKR2s2T2wxTTZ5bEwtTUNQNU04djFHTHlPbXVLSW9YSUE?oc=5</t>
         </is>
       </c>
-      <c r="E34" s="19" t="inlineStr">
+      <c r="E34" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1472,7 +1475,7 @@
       <c r="F34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="19" t="inlineStr">
+      <c r="A35" s="20" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1482,17 +1485,17 @@
           <t>Ironbark shuns private equity as it hunts for cash injection</t>
         </is>
       </c>
-      <c r="C35" s="19" t="inlineStr">
+      <c r="C35" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D35" s="19" t="inlineStr">
+      <c r="D35" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxQZWFaeVhldi00VkV5ZmEtS2tjcWdFWG55OGpCX3IyN25Rb3ZFV0ZKVm1aSE1WbThoYVY4ZEdfODVGX0RaUDV2Ul9HS1JQMDFCT05Fc2FaU0RINTMwbDRveWFsOFJSM2ZqTU9tVGxJSEl2ZmhhUHFHT3dqYkk5TUtvMUQySnZzTWw1MzFNWl9aVzhkSEZ4Q3YyWjRMUmpIdmJkdUVKWE54Nkt6bTd2dGFSUFoyNkgxTHh2TGVGak9ja0dFZ0xQM2g0S1lmQkZiWWtUcTVNdHhBdC1KeVRQcDA2dnpmeHRkWEnSAewBQVVfeXFMTWtYRDRSaHNULW1HanowRnpMdFF2VVMtZW1SV2ViZXlGaW02WlIwUzRZMGg5WDNrOUR4eDlGOEt5eGlqV0pfVDFhb0JEcS1faEJodWxyRnB3MkozOVJyT3NvM1I5MzdDcXNnUFNSdkRDamUzZTRQYlk0c1VIQUNMZ2ZzOWVCb2V2MC1aSTZLWkFkbW9GYk05b3RmN1htWENTeDh3SU1WYWJMcWx2eGUzZmwwVXF6czlnRGdXbE1vRElyVG0yM0ZzXzZ5TFh1YlRGNU9MQ1p3NnVZSFB0M0xBcGlueVZILXlVaXdqUkU?oc=5</t>
         </is>
       </c>
-      <c r="E35" s="19" t="inlineStr">
+      <c r="E35" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1500,7 +1503,7 @@
       <c r="F35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="19" t="inlineStr">
+      <c r="A36" s="20" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -1510,17 +1513,17 @@
           <t>Minister leaps to fix food chain</t>
         </is>
       </c>
-      <c r="C36" s="19" t="inlineStr">
+      <c r="C36" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D36" s="19" t="inlineStr">
+      <c r="D36" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxOd2NqakVWRnQ4anFZNkl4Zy03MkloX08tUkktRTZqeEtQWFZJeVhkMUJIb0FxUjc2UjhCQ3MxbmNxczNxblJIZ09IeTBGNFM4Wkh4ZE1qNkhJMjIwU2RtX1JxcEV1Y0NjWXF6eHpVdTN4ZUlYMGIwcDJzMXZMTk94VzFlcjhpcVZVSTJFMjhsQjVGWEJQYTQ3aTFyNmNEZ1F1b3NGTWd5WnFJWmxXSTJ2NlRLcjJHNWkwaTZ2YVR6S0w5WVo1Vlg0VWdxcWZoa3VaTmcxY2NVcnR2bFRWNGNvZ1M2Tlg5NzlvVXZFZm9B0gHzAUFVX3lxTE1uNERoR3p2dXRIa0g0RXI2MWR6N0c5U3NGcjFDQVMtdEpyNDI2bk8yOS1qUnFOazdiODl0Ymo5R1pwRVJ0UFFVdzlhYjRDSUFCU0FRak4xcVVrTHphdTdxcHNIMnEyRVZud1FURmh5T0JLOHpRM3lFbDRuRnZMYmtaRnRFTXh3dkszTFhFUmZlRmoydnlEbW1fZTlmUzh4NXNyeTZTeUhOSktvclJVc0NTZTVYMkdJZEUyY2RmVC1kQ1hwVEloSEtVMEo5QnNTUXQyME5IN1BPd1NOS3oyR1JtMHBFVTZEbzhEQmdrWUk1ZnZVTQ?oc=5</t>
         </is>
       </c>
-      <c r="E36" s="19" t="inlineStr">
+      <c r="E36" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -1528,7 +1531,7 @@
       <c r="F36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="19" t="inlineStr">
+      <c r="A37" s="20" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1538,17 +1541,17 @@
           <t>‘Brace for swings on every tweet’: Investors bamboozled by peace talks</t>
         </is>
       </c>
-      <c r="C37" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D37" s="19" t="inlineStr">
+      <c r="C37" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D37" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOczZHTWFmTW9FZ1ZwSnc5Z3ZacGpsVDQ3LWw1a1BFT0tjRkphek41MlhNOU84emYzZUVwNV9xM0hyc1FUR0NHck14Qnh6c2JvQks5ZE02ZTNLWDI0dy1STi1HbDFDWW9yMDhGQXVVVzdkMzFXcnNNMVZHVXFMUXUteGtsVGhPVmhLcVZPQzlhTWNoYVVRMHF0cFhybWxzek13Y3ZjcjlXWjZJM2VYbm0tTmk4NExLQzQzX1ZPMVlhcnJxQkZx?oc=5</t>
         </is>
       </c>
-      <c r="E37" s="19" t="inlineStr">
+      <c r="E37" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1556,7 +1559,7 @@
       <c r="F37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="19" t="inlineStr">
+      <c r="A38" s="20" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1566,17 +1569,17 @@
           <t>Just Jeans revamp emerges as bright spot in disappointing Myer result</t>
         </is>
       </c>
-      <c r="C38" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D38" s="19" t="inlineStr">
+      <c r="C38" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D38" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOa0xia0ctWjQ4MFhmRE05R21QSWhpOWFqa1Y1S3hNRUYyRjdnZGpZY3BwWTZPb2FFLWpDSnFrY0tia3VBemRGY1g1aHZHZ05zcWZweVNfb3BHd1h4ZUc4V1VFSmFFMHVJX3BGLWlwMXg0RjhDTVd6Y1Zld0lCcVZ2UGRqb3Z1cktmTl9uNVNjVFRUbFloaVVIWmo1RGVCQ2VWMFNycE9aamR1Uk11U21Hc2o2aw?oc=5</t>
         </is>
       </c>
-      <c r="E38" s="19" t="inlineStr">
+      <c r="E38" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1584,7 +1587,7 @@
       <c r="F38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="19" t="inlineStr">
+      <c r="A39" s="20" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1594,17 +1597,17 @@
           <t>Wirth’s Myer rescue mission is caught in the eye of the storm</t>
         </is>
       </c>
-      <c r="C39" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D39" s="19" t="inlineStr">
+      <c r="C39" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D39" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNTlQ4NDRnWE91VG1YNENpSTUxNnBjZkljOGdYaGV0aVB5dkVOaEJ6SjZ1bVA4NXE1S1hjV1NjcVhQTEVpWEVNV0UtbzhQTFZLOWxIenZiaF9QM3F6bmJYRy1lbXVMczZ3TnBHNy1aLUtVcnBDdkl4TE0zRGN4U0FwSjNPY1M5S3AtdUQ3UUNmR0x4MlU2YXRuUDJEUm01SmZWakx2UjFvY04zRHk4Smc?oc=5</t>
         </is>
       </c>
-      <c r="E39" s="19" t="inlineStr">
+      <c r="E39" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1612,7 +1615,7 @@
       <c r="F39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="19" t="inlineStr">
+      <c r="A40" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1622,17 +1625,17 @@
           <t>‘Darling, I’m not going anywhere’: The rise of at-home care</t>
         </is>
       </c>
-      <c r="C40" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D40" s="19" t="inlineStr">
+      <c r="C40" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D40" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQS2k0M2otaldpNVFXdHRTMVNtZVhyUDV4VTNIcE5FSnFRaHNubGNQQzBVbllnNTktNGhrZ1lndzV5V1FpUS01SklRaTZmZHJkRzVsQmlsdEVmenZ4U2x6U01NeXdIMktBUW94TUE3R3FoLUxVcVhsVFI0SjVQVUFaZldnd3prMWMyaVRWX2J4aUdfQ25KWHpaLUlqSnhvQmM2TTRRQldGbm8tclFYRDA0TVdnU2g3QQ?oc=5</t>
         </is>
       </c>
-      <c r="E40" s="19" t="inlineStr">
+      <c r="E40" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -1640,7 +1643,7 @@
       <c r="F40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="19" t="inlineStr">
+      <c r="A41" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1650,17 +1653,17 @@
           <t>Iran targets Israel and Gulf states as Trump looks to calm markets</t>
         </is>
       </c>
-      <c r="C41" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D41" s="19" t="inlineStr">
+      <c r="C41" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D41" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPLXBITXU3WTRtc0NYdnhTZHFaUTBCSXdldTBuSHliTlY1dlJONW43Qkd6Nl9pNmY1eDhzaHZoX19xYjBxMXR5UEhkVUg2M2k1MmhuVEwyY0JxbnJyemxVYUZjbk5BbkN4ajhPbW9ZeDhlRDRYTW1hN3k2d084c2djMEJUZTV3NVdPbllKUmFlU2JsaDV3Zk9CVFF0VDFkV09JSloycWdOUlVrREptQTJfa25LUEx5djA2SjNMMFY0RjM?oc=5</t>
         </is>
       </c>
-      <c r="E41" s="19" t="inlineStr">
+      <c r="E41" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1668,7 +1671,7 @@
       <c r="F41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="19" t="inlineStr">
+      <c r="A42" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1678,17 +1681,17 @@
           <t>Meet Christian Louboutin, footwear’s most famous billionaire</t>
         </is>
       </c>
-      <c r="C42" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D42" s="19" t="inlineStr">
+      <c r="C42" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D42" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPcXdGd0tMckYxbjZ5TVJmQ0Q4NFl2RkhHMHdlZDZsdGZ6cVQ0cUpaLWJTNlVoc2ZOQmtXNlFTRnJVMnVDTGc1NFNZN2g1VnotQlNQbzhlM1BJV3ZwQktOcGtac3RwSHRLZkR0b2l0eGIyVVlYdHJrc2hpT0pJbDR3LURPTnowZk54LThObndtMVkwV2VWQkluNVlWY0p4QVJGbE1hSGMzOW8zdkJZOWdocEZQWFBhTllNR1ZBSEg1TWRXUWd3X0t6TVcyY05PM0pF?oc=5</t>
         </is>
       </c>
-      <c r="E42" s="19" t="inlineStr">
+      <c r="E42" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1696,7 +1699,7 @@
       <c r="F42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="19" t="inlineStr">
+      <c r="A43" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1706,17 +1709,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C43" s="19" t="inlineStr">
+      <c r="C43" s="20" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D43" s="19" t="inlineStr">
+      <c r="D43" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQbHdYM2pSM2xkdmZ3OHhQc2tVUmhzclJWaVJ0aEwtUkNBR0ZUd3p1emF1M21jbTF1ejlKSkdDMnotcVNjZE1CYUlKako3WXR4MTJhdWNlSXZMbTBYanlmTWFzRGFIandXRUQ3UjN6SEV1bThvZjN2bDY0eFdpaTdMODN6TGFTdE5rd05TUll3MmNfTDhkQldoNDIwVlpoSl85aVRwcTd5Ymh3TDl4enZhZ2p4OExGY1ZaOFNEWFBB?oc=5</t>
         </is>
       </c>
-      <c r="E43" s="19" t="inlineStr">
+      <c r="E43" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1724,7 +1727,7 @@
       <c r="F43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="19" t="inlineStr">
+      <c r="A44" s="20" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -1734,17 +1737,17 @@
           <t>Sembcorp Picks Banks for $2 Billion Alinta Loan in Aussie Push</t>
         </is>
       </c>
-      <c r="C44" s="19" t="inlineStr">
+      <c r="C44" s="20" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D44" s="19" t="inlineStr">
+      <c r="D44" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOdS1aaXZjT2VnSDl2TDdzZ3NfRElDWXdUXzZQYjFQMEZJOGlpaE5CNGdQMlZ2UFVHbUtfOXF1ZVBReExrdF85M0RWLWlBY2Y5dlRtWVdXLWp0Y1VrRmF4UGQzVUhxaHA4UHd1SUdFV21QcVFITXFHRlhzekdSUS1PdHlYRjdUbUQydU8wSktKVHRJQ0NaWE9sU1l6YXhtSWtBd3RwTERacnV4VzB6YlFhUE1QcXNDVXVESFcyeWY3cGhHUkRJcDhrYUtpTEY2UQ?oc=5</t>
         </is>
       </c>
-      <c r="E44" s="19" t="inlineStr">
+      <c r="E44" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1752,7 +1755,7 @@
       <c r="F44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="19" t="inlineStr">
+      <c r="A45" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1762,17 +1765,17 @@
           <t>Navis targets June for $1bn-plus med-tech auction</t>
         </is>
       </c>
-      <c r="C45" s="19" t="inlineStr">
+      <c r="C45" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D45" s="19" t="inlineStr">
+      <c r="D45" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxPNHRXaU5tNUVkd2MtcTg5M0EyQllrM0owMkZobGxLaUJxYUN2MUg0ZkdKdzU2YmxfanR3QU53cHZzNDI1WXgzRUcxOE9EZlluNmtNRUUzTGJPRnpfVVVOeFM3bFRNQmp6VHFBdi1mTnU4UDBvOEpMaHZPNXFtdUIyTlhuRExIVElSeVRUMGxjU0k5VnVxaWFfd3htWngydlhuR2E5aTQ5VW1LS01ac05rMGZoVFdOZzVyTzFhUDVsYkNrc0VQZmhubERSaTNwelk3WEhYUjF5d2ptMktYeEhzOHpWazFQZXphd0xfUFdhbkVGMVR2Z1dtVtIB_gFBVV95cUxObEwzeHd6RmZtNUp2dXVVV0plOVQ4WlNqQXNJU0thd1BEWE8yWkxxVTZjTkpsVGxxWGxpQzN0OERZbk91ai1fZkdtc0JoM1h5NERLTVdDbVJ4Y2k4djdQcWlVcDF6NjMyVDQzZWMzUFZxWjVRWllMZHVSOF9jQ2U1REFfNUlhM2EwYloxb1MwSTJjODdWdlZwX2h2N0xiQWNhallHUTNPZEtLaXhsY3dBZy0xM1VITXhLUERXS1JxR0R3OUpBTVBPZ2dPZTRUTVpvbFBNMjFUSTJuWS1XLWdhUS11UTRzVTVqaEhfMDhqWHlTMlJGekU2QzJVcFdodw?oc=5</t>
         </is>
       </c>
-      <c r="E45" s="19" t="inlineStr">
+      <c r="E45" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1780,7 +1783,7 @@
       <c r="F45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="19" t="inlineStr">
+      <c r="A46" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1790,17 +1793,17 @@
           <t>ExxonMobil eyes New Zealand market exit</t>
         </is>
       </c>
-      <c r="C46" s="19" t="inlineStr">
+      <c r="C46" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D46" s="19" t="inlineStr">
+      <c r="D46" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxPanlvR1V1eVVpdmYxNVNGMnd6UjJFd0J6Zk9IU1lhOW1GbmVTcjY4QkJCYkl3Y3NOU25VRTBUekwtS3plV0NVdlZtOTZZRHJWZ0FVdDl3S05aMlFWeEZiYzdwYmQtVnJxZEw0NktHaFZMNlZkUC16empqRGxxMEhhZGwxRzVEek5FelB3aE9UWFhGQW42b21MRnJHUXV2ZGJYUXJIMnVFWGZsSnEwazNGNUdVcjVoekp0NEZCN1J3cTlaZldFa1pMUkJTbVZYeFljVkRqQmlZV1M2aXh0ZjI5dEI1NDB0UElPUERsbUljMlA3OHBnYmtJTXFWZWkyUdIBgwJBVV95cUxNWFBRQ05GUDdwTWJ2ZVFJUS00ZUh0QkpZQVNNcU9JYXRTN21sMS1VZTlOSTh2LVFuZHh6UVk2djlrdWFsd3MwcDFCNmhwUlVLTlpjVF8wSmt1YnBWRE9tNVpKQlk2YXJWdmwzZWlLX0xpaWxSMUpsX3ZjYXhmRmE2YlAtSFJGRG5pQnVmMnViQXlsVFV3OU1hZFVrY3ZITHQxcTR5UkZ5U1pReHVJMGZGM2FCZWliSFZQZmpVLThSdExWMW14OElodmVVSC05SUh1d1hBenJoY3BUZGxoM0NTbTExdERmM3pjZGd4VzgyV3BNOG11TElBQ3NsRGhtSEc3YzJz?oc=5</t>
         </is>
       </c>
-      <c r="E46" s="19" t="inlineStr">
+      <c r="E46" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1808,7 +1811,7 @@
       <c r="F46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="19" t="inlineStr">
+      <c r="A47" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -1818,17 +1821,17 @@
           <t>PAC Capital’s Clayton Larcombe charged with assaulting wife</t>
         </is>
       </c>
-      <c r="C47" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D47" s="19" t="inlineStr">
+      <c r="C47" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D47" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOLXNDU2xjMWpyeEZwWGwtZkV0TjNSbGtWS3ZidUo3a0dvV1hrTnJiVXBXSkJNWlhXYXFHZkNTa3g4a1ZfMjRPM3BtWTZUNGg3S09kbGI2TTRGd0Jkc1A4WFAycjlpVC1URjFvNnBraWprRkhaT0VOWkh6N0xkUjNXNUw0dGx2N1JtTDVsREdtZDhraXVsSkxhR2ozamFUSGR5VHBBRm1Zcmx1c2RDaUIxQkVpeUpfWjFNeTRLWVRtYjluZ3ZncGZIMQ?oc=5</t>
         </is>
       </c>
-      <c r="E47" s="19" t="inlineStr">
+      <c r="E47" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -1836,7 +1839,7 @@
       <c r="F47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="19" t="inlineStr">
+      <c r="A48" s="20" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1846,17 +1849,17 @@
           <t>China touts itself as ‘harbour of stability’ to global CEOs</t>
         </is>
       </c>
-      <c r="C48" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D48" s="19" t="inlineStr">
+      <c r="C48" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D48" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPUzBWeVk0elBOZ0l5QU44TUJvU0RvSmtPdmVyT2VuQTczaEdzbkktT25ZT2Y0Nzh0bVBhQW96TUhpWkdEOEJMVVk2UWxLOENKZGk3X2tQcDNsWGZtU0JkM2U0N3VfUWFBclhUSUZya0NwRTJOWmZJdWlhT3JtY1EtSkJ6TmlsV3dzOXpDaVFMNlBaa3RfRHBjc3Q0cjk0eVdPV2MwcjlHNA?oc=5</t>
         </is>
       </c>
-      <c r="E48" s="19" t="inlineStr">
+      <c r="E48" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1864,7 +1867,7 @@
       <c r="F48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="19" t="inlineStr">
+      <c r="A49" s="20" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1874,17 +1877,17 @@
           <t>Eyes on 3D Energi as oil and gas giant Conoco flexes buy-out rights</t>
         </is>
       </c>
-      <c r="C49" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D49" s="19" t="inlineStr">
+      <c r="C49" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D49" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWVU1QmhTUGFkYlpTQkw1WUFPTHhmbk5lbnE4T1haQUswSi1ITHlhVmhyM3ZYS3N4cVd6ZkwzdGdhT1lvM1JJek4yLXFpSWoxUnRtR2JRLTZWa2dlTDVTakE3b2xvazFWX0kzRHFZWVB4OUh0XzFFd3JVSVlfelpVa21qTldCVHdvcmJYcGNjZ1RrdElWS3Yzck9KYzRvbzloWkNqMnQ3dmtHbzNuc21ZSXNYeEFlZw?oc=5</t>
         </is>
       </c>
-      <c r="E49" s="19" t="inlineStr">
+      <c r="E49" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1892,7 +1895,7 @@
       <c r="F49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="19" t="inlineStr">
+      <c r="A50" s="20" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -1902,17 +1905,17 @@
           <t>Blackstone tempted by $900m payday for Sydney’s JPMorgan tower</t>
         </is>
       </c>
-      <c r="C50" s="19" t="inlineStr">
+      <c r="C50" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D50" s="19" t="inlineStr">
+      <c r="D50" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxQNEZTZjY0S2YzcUxsb25RSDk2NHd1N1VOVlpMbi1JNGEzbUt5ajlYZFhvLWNBTkNQVXNuWERfTkl0Z2o4R1U0Zk5jVE1FTW5TTUJGZnNJc2NqMm1fT2dmYTVwRGU2TkZ0c3BjZVBGS29fWFJvZ2F0MWNLa0pYY0RNME5xYS1vOGZmMDVBcDBaLV9MWF9od0EwekFyb0ZCOEdkNTFaN3ZXckJwd25zS0FsdzU4OW1UODlueGNyZVBDSDZkeHQwelV5ZXVDVlcyUkhKWDZfVlRacEJHSElmNnhKSXk4ZHJHWHhPTEV5NGNkcmhyU0hjV3J4dVBXbnRGQdIBgwJBVV95cUxPME4ySFF5RWNrejVlWW1yeW56N244RGpyeVJUZEgyTjFNcE10YjVpMmJyeWsxTENzZFhPRlpsbl9pVXl0NGJvUlZFT216NE1KRFNwOHVZVXMzanNKNXFmWEdsMndsd1cza3NTTzUyUUZfaDEyWHJwZEtQbTdJRmkyU3A0RGh4QlAtT1lRVXk2SGoyaTI1NUpwVExYSkZJNmVFNjdXTDJTNURFOEh4Y1dnUDVGdjBpaDlWVWJtUHZiRDdGTmE5R1R6TDBwWFFnT2MwQ1lmT2w5bDF6eVU0R20tYnpnT3JCZlJod2s0UndyZTM5M2xLZC02a3E0NmJRdFV0Qkow?oc=5</t>
         </is>
       </c>
-      <c r="E50" s="19" t="inlineStr">
+      <c r="E50" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1920,7 +1923,7 @@
       <c r="F50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="19" t="inlineStr">
+      <c r="A51" s="20" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1930,17 +1933,17 @@
           <t>I-MED attracts mystery suitor as Permira weighs sale or IPO</t>
         </is>
       </c>
-      <c r="C51" s="19" t="inlineStr">
+      <c r="C51" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D51" s="19" t="inlineStr">
+      <c r="D51" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxNaGlwS3d5MGFMbEg2U2hnZUxMQmdqaWI4bS1lblNZOFhkSnRMcUotRkZMTjhFZkRUQWxUUDVtYml6TVAxUXkyZmx3SHRFb0gzVHRST2ZQUThKa25aWlhlcGprSU9tWktXZjZRaC12bFpkaVVWZHhIMERyeVNNWEswYTJ2ZHdnRFVRaFhod2U5N011TkQ0NG5MYVhoT3MwRUVZdVB2UVhKZExvdFIyXzNNUGt2SHJUanQxRkI3bXlLSlNJQTF4NXQ1YlZDaGVBM0EzNUhYQVp6NkFWRzU4bnRPWTgtXy1HVnB0ZlN0Uy1rY2FuWlNfN1U4WXVHQnRzVkNG0gGGAkFVX3lxTE1GaDJJdTJlOXFEZUtDTmdXMmsyLXlpaUxzQXpycHk4MTdHZng0dVczYWVwdWRzdFFCMlNLWkZpMm5Zd2RpN0Y0Zmo3Q1FOZFBZQlh5LVl6aVZ3X284UmpxM0pVRzZmMmpjaUdNWnJPZGV4V3lNai1CTllCcW5oUEVxaG0zejB5anc5YnJEZzZPT2d2QklCWjl2MjRBc25jUndqZkVadllKaUZScG12bEozT1NKUUJYR0pHTGtJZVc0ZHZLNHVSYlhzcTE0SkZmMXNlVGJ4YWJ1cThxcGlZTDMzRUMxLVM5VHh2OW5tRW1PT3VyRUhDbV8tRzUzVzRzVWZPZ2w1bnc?oc=5</t>
         </is>
       </c>
-      <c r="E51" s="19" t="inlineStr">
+      <c r="E51" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -1948,7 +1951,7 @@
       <c r="F51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="19" t="inlineStr">
+      <c r="A52" s="20" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1958,17 +1961,17 @@
           <t>The stagflationary mix that has billionaire Solomon Lew worried</t>
         </is>
       </c>
-      <c r="C52" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D52" s="19" t="inlineStr">
+      <c r="C52" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D52" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPWTh3S05XQWpTQm03WjhBT1pWc2cyOFRMd2ZraHhPUHlDRW1tWkZvdkhQWHE0MHVMRUpaOFRoX0JsYWhJV21nVkpIM2RBSmlZRUtEbFAydzZfOTh1S05oNEZPOGgyZDJRMS1uLThWYWRVT3VEVGhtYkVLN3J2OWsyX0VVdTUteFBCOVNKZ28xUTRPTk1SUkMxZ1NJc1B6NXRrUEEzOG01YnZOYjk2cWlFZA?oc=5</t>
         </is>
       </c>
-      <c r="E52" s="19" t="inlineStr">
+      <c r="E52" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -1976,7 +1979,7 @@
       <c r="F52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="19" t="inlineStr">
+      <c r="A53" s="20" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -1986,17 +1989,17 @@
           <t>Oliver Curtis on Firmus: From prison barber to AI billionaire</t>
         </is>
       </c>
-      <c r="C53" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D53" s="19" t="inlineStr">
+      <c r="C53" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D53" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQek9VTlV1b2hVb2RoZ0Fya0REb3E3YlBCR2NYZldXcEh2VEY0LXg5bjd6RzlnZDI0OUJJd2cydTBwTm9tdHpiZ1lSMnhtcmJSYVRKbzJFMjdDaEJyZExSQVJVRDh1c00yMjFMaVlPdnRuV3VkTjNxdzFRbW1yeGltSF8tVXlJVXJzTEJXS2FTYkJTVkdKbmdPTTd6YzRtYV9nN0JzOVZNTzhUdUk?oc=5</t>
         </is>
       </c>
-      <c r="E53" s="19" t="inlineStr">
+      <c r="E53" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2004,7 +2007,7 @@
       <c r="F53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="19" t="inlineStr">
+      <c r="A54" s="20" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2014,17 +2017,17 @@
           <t>Three startups that raised $161 million this week</t>
         </is>
       </c>
-      <c r="C54" s="19" t="inlineStr">
+      <c r="C54" s="20" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D54" s="19" t="inlineStr">
+      <c r="D54" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNRGVZMF9DeGJjX29vN3B0blVoM3RKSlJJTllrMThKUDJNZzdPNFNnT2JyTElUOUYxMHlsUm9yM2dBQnZfaVNZblpqb3NzTXdHVlpQNkRqR3NBZHdzODdjN3RKMTZhSVRqUEM5d3JRc3F2OG9hWmZJdU5rakg4ck8wLXlMTnZSU0lNaERmQmswbkVGWW8?oc=5</t>
         </is>
       </c>
-      <c r="E54" s="19" t="inlineStr">
+      <c r="E54" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2032,7 +2035,7 @@
       <c r="F54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="19" t="inlineStr">
+      <c r="A55" s="20" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2042,17 +2045,17 @@
           <t>Iran eyes ‘plenty more’ vulnerable energy targets in costly war</t>
         </is>
       </c>
-      <c r="C55" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D55" s="19" t="inlineStr">
+      <c r="C55" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D55" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNLUN1MHlZaTNfVHhVX0RnTXp5QW83RmM4WVZkWW1PSnNaZF93VkY5ZF81anB3NDNmX0kyMkVSdkxNSURvSEh6enloWnRVcTlsR0JPTjVzNFR1YjRsSm52VnA1XzFFUlUtODJjYy15YWRRdWZZRkdjRXpCcEFSVURmV3VpSTFhTjVUb1d5bmw3NHNlT3VQZU9ieEYwM1J1TGEyZnlnWXNIWFJUMEtIOVZad0dxRWZBdw?oc=5</t>
         </is>
       </c>
-      <c r="E55" s="19" t="inlineStr">
+      <c r="E55" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2060,7 +2063,7 @@
       <c r="F55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="19" t="inlineStr">
+      <c r="A56" s="20" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2070,17 +2073,17 @@
           <t>Don’t take it personally: Bain Special Sits hits hurdle at Infinity</t>
         </is>
       </c>
-      <c r="C56" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D56" s="19" t="inlineStr">
+      <c r="C56" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D56" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQRjdwTk0xTHVIRHNkdG9tVk1EQ0hiQjJ6dGcxaWZRZ0hZV1U4YjJDU0tnTUlWSkQ1S2dUTHJVNk0tNWQ2cVd4dkw0M25leXRreWJtdlBKYTAtNzRocTJUazh1dnRzSVlYZThySTBNVjg5X0xYWUxCMC1SelltSHVSUEV5U3B1bTA2NjAzMGFZLW1CNkQ3aWU0S1JxS0d0YmZiZjBKQVRNVUpzYno5R1pvbTBsaTM?oc=5</t>
         </is>
       </c>
-      <c r="E56" s="19" t="inlineStr">
+      <c r="E56" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2088,7 +2091,7 @@
       <c r="F56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="19" t="inlineStr">
+      <c r="A57" s="20" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2098,17 +2101,17 @@
           <t>Drill, baby, drill: It’s boom time for mineral and petroleum explorers</t>
         </is>
       </c>
-      <c r="C57" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D57" s="19" t="inlineStr">
+      <c r="C57" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D57" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNdlFOWld5ZWhPVnFRa2xidWlUVzluQzkxUTgxR0t0Rmg2S1BzNjdINnhwS3VLRkNjRVJLX0RHU0h4VFVRY2RfSHBudEhfNVNjeE50ZUxQenJNSlJtWFRlcnNsZm1iLXlxM2RmVDViWEtjNDloaTBhUDVxYkNfOWFCTjV6cExEVlFCMzNfWnVwRDJHYWxWV0hOR2V2S0VlV2NyS2s5cWNmREtWXzlMMDRQNW1tVlBOblp3SHBEVg?oc=5</t>
         </is>
       </c>
-      <c r="E57" s="19" t="inlineStr">
+      <c r="E57" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2116,7 +2119,7 @@
       <c r="F57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="19" t="inlineStr">
+      <c r="A58" s="20" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2126,17 +2129,17 @@
           <t>‘Wake up’: Fury as farming crisis looms</t>
         </is>
       </c>
-      <c r="C58" s="19" t="inlineStr">
+      <c r="C58" s="20" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D58" s="19" t="inlineStr">
+      <c r="D58" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNelJvMXFPX3MwUVRMN2xqbzE1MWdvOF92Zy02YmIyZW9SQXRNQVZsS0xVVG9UdkFPaTV6ZC1tV05SZWNqblNFZ3Y1VGNaVVBaaEl6aFJqQ09ONDVkNUs4TzNvVjV5eHNjUk9xaDRFZTM0alpuYUdvWGtLRzRhYXN5alZ1QWdsZTEyODdQVnZoazkya29WeTJZVmpxLVBCdWxfY0dTN2Z3WFZlSy1sVW44RDlvZFAzYlhnQ0N6UWhKSU02eF9iZllIU3g5MWtSbkJzZGxWLUxHNERzdUlLTF9VYmpJSTRLY3U4NlVVaDhmc09uOWwtUGtlb0I2M05DR1dnRWxGSFV2NEJXaEF4c00tN9IBlgJBVV95cUxOSzZ5NXZMTTlZa3BSNjZyTUxUMjRhYWJhN0hMa3dDcW9CWGstNnI5MzV5U0hJSTdKLTFwa2E5YUItZnFRbW5RbzVuYW91MmZaYXN3R25hWVpUbW9oUU9fVktPRHROVDYyd2dSLXJVZWQtY016bkVxY0VPbkY3Zkgtb1liWGMxeEpyYmloS1V0TVJMMWZaeWRZX3FQRjBmVzJwdkkwMEVDSXV1MTdReUhGZ0Z3dENyMEFkLUl1aXhtRkFLRFFXcEdMZzFuT3NxRDFMOGVaY2YzeXBQc09fY3YwcFp4MVczRVN3d3dJZWJfTFFscjF0cUtRWHdzTUptaHowNDhYWXZXTHhYTHNTdlZGUmNlamRTdw?oc=5</t>
         </is>
       </c>
-      <c r="E58" s="19" t="inlineStr">
+      <c r="E58" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2144,7 +2147,7 @@
       <c r="F58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="19" t="inlineStr">
+      <c r="A59" s="20" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2154,17 +2157,17 @@
           <t>Construction giant FDC road tests IPO pitch</t>
         </is>
       </c>
-      <c r="C59" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D59" s="19" t="inlineStr">
+      <c r="C59" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D59" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxON3p5Y3VPM01XZFk4a3g0R3JnQkZXbHVGV3BKdDB6M3NRb0M0SEl3V0R5RmhCQ3dnaHB0ZHp5N2hCMUFsNU1ZNWZ4YWdNZWdETkUyZmdoeW81amwtTWNFZlc5WlNpMkJwRzk0QklORGhlLWNEalh2d0JCX0lhVHhhUF9ibVlxcHAwOW9ENndVOTY0enBYUWc?oc=5</t>
         </is>
       </c>
-      <c r="E59" s="19" t="inlineStr">
+      <c r="E59" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2172,7 +2175,7 @@
       <c r="F59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="19" t="inlineStr">
+      <c r="A60" s="20" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2182,17 +2185,17 @@
           <t>Austal suitor Arlington Capital Partners buys Eptec’s defence unit</t>
         </is>
       </c>
-      <c r="C60" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D60" s="19" t="inlineStr">
+      <c r="C60" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D60" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNM01qb1ZRZVBIdmp3cFc3R3RLaTdmZk1JOFo4anRtSm95Z1hJc0N0S3VranBTV29IdlViT0FkSm92eHdtbDBqdU5HTHNMaXo0dGRWMkpDdjk3LVRBVU1rZC1YejZJMkhyNmpZZFJodGoxWlB1dkRhYTJVRlljMlV0dUllQ3EtOHZkNFdSUWJLSW9Xemw1XzFzU2RHV1o0RTViOXp0bDZFQTZycWhpNElLU0FZQVI?oc=5</t>
         </is>
       </c>
-      <c r="E60" s="19" t="inlineStr">
+      <c r="E60" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2200,7 +2203,7 @@
       <c r="F60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="19" t="inlineStr">
+      <c r="A61" s="20" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2210,17 +2213,17 @@
           <t>Eyes on Tom Wallace as clock ticks on Adgemis pub deal</t>
         </is>
       </c>
-      <c r="C61" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D61" s="19" t="inlineStr">
+      <c r="C61" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D61" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxNSExQeDlENWlHb0prRnRldjZ5YWhKVUZ5eVdsYjZmbVRWRWQ0WnZXWkU3UHZJdElnQ21jMU9zNnhnc3JlNDczVGQ5Y0FGV2J3QUp3NXdZTXZMNm5tVC1vWDFtOFN3aS04QVJZb3FZV2VsUmJ2aVgwbUhTaFVGdHg0UjRyTXVVUnFhQmE5eFYwMGR6T1R2U3Q3WEdZclVKNWJiby1IRg?oc=5</t>
         </is>
       </c>
-      <c r="E61" s="19" t="inlineStr">
+      <c r="E61" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2228,7 +2231,7 @@
       <c r="F61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="19" t="inlineStr">
+      <c r="A62" s="20" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2238,17 +2241,17 @@
           <t>UBS names head of APAC leveraged capital markets</t>
         </is>
       </c>
-      <c r="C62" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D62" s="19" t="inlineStr">
+      <c r="C62" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D62" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNMm9WZ2ZKVFBvX2pYMk16VmY1WFZnZ2J5N0F2bHduTVM0Sjg4STVtTGFLQVdzeFloVHg3clRic0owTDMwYVpXdDVjdjFOWjQxdkdxdFY5MEY1Q1U2Q0R5dFBJWTNtUzgyd3RXcm9uM0hKdEZ3b3JjXzcwQ2VpRm5SS0hYT2gxSU9iVFRlR05Xd2EtM2JOQjBGUzlKdnE?oc=5</t>
         </is>
       </c>
-      <c r="E62" s="19" t="inlineStr">
+      <c r="E62" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2256,7 +2259,7 @@
       <c r="F62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="19" t="inlineStr">
+      <c r="A63" s="20" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2266,17 +2269,17 @@
           <t>BHP, Woodside rise after new CEOs named; Future Fund chiefs exit; Sandilands ‘doesn’t accept’ termination</t>
         </is>
       </c>
-      <c r="C63" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D63" s="19" t="inlineStr">
+      <c r="C63" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D63" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNUHhZeHNHemtiLW1IOHN1OTZXOGpsM0ZtUG1MVHRCT1hUT1k5S2lEOXlXRENWOXNlMEZadThQR18xSTJfTVlQM3BtX0ptX1J0bk80SzNLUVRtbkJITGgtb0lsSVdJTWt2S1E1WUlXdUdsbEV0V1RpNWlyRXBoc0dPVDl1OXRrSlM3SHlDazg2UlcxenVzNzlhQldhUGhfNE5IV2xrVmVBNzhhSE9qY042Z3pzMEVzd0VyVmZudXgxcTgwWGJXSWZKZ0FyNVhjcmhjTm5DYUVjLUdDRmxUQkZuTDFlUXVaV0ZoSWp5WHMyR3c?oc=5</t>
         </is>
       </c>
-      <c r="E63" s="19" t="inlineStr">
+      <c r="E63" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2284,7 +2287,7 @@
       <c r="F63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="19" t="inlineStr">
+      <c r="A64" s="20" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
@@ -2294,17 +2297,17 @@
           <t>BHP’s new CEO will shift the Big Australian’s centre of gravity</t>
         </is>
       </c>
-      <c r="C64" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D64" s="19" t="inlineStr">
+      <c r="C64" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D64" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPQnZpWndNZzZvN1VsOHBmRDVLRHVTNkxLeDVDelpOMURjOTRDSDZfN2dPZlZqaW05WEZuZXMyRTJZeVZnV0poT2UxRkVfZ1RZSjdvUjVKblhoSU5Cd1plRTVNNTRaNWZmbm1yUGZkblVpYkctNzVRRkVQQm4zX1FtRG1KV2Y0djUtOURianJ3dElqeXBUMFp4aWFEWVFYelVjYTluSWpOM1FlbHpIaUxXdnBn?oc=5</t>
         </is>
       </c>
-      <c r="E64" s="19" t="inlineStr">
+      <c r="E64" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2312,7 +2315,7 @@
       <c r="F64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="19" t="inlineStr">
+      <c r="A65" s="20" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2322,17 +2325,17 @@
           <t>How philanthropy became the sandbox of succession</t>
         </is>
       </c>
-      <c r="C65" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D65" s="19" t="inlineStr">
+      <c r="C65" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D65" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxObnBPb2MzQ1RvSVVCbmNzYWFBMlFjU0dQRmpPakNfdkxtMWc1bFdVNXNlZmRKQnNlWEtUUDNSTHpTLVV4Skx0V2otbTZsTTdvT1VaUDhMZFZoMFFab1RoS2pCcno1WGlNQlY4eXQ0OFEtLXJTay1MUkFSSEJ2MVVScUpjUkhJOThISy1QbHIzTzFlWVhOc29fWWs0V19sQ25hRW9MSGhBVVNKWUp6dUo3NS1SWlk?oc=5</t>
         </is>
       </c>
-      <c r="E65" s="19" t="inlineStr">
+      <c r="E65" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2340,7 +2343,7 @@
       <c r="F65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="19" t="inlineStr">
+      <c r="A66" s="20" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -2350,17 +2353,17 @@
           <t>Advanced Navigation raises $158 million Series C round with NRFC backing</t>
         </is>
       </c>
-      <c r="C66" s="19" t="inlineStr">
+      <c r="C66" s="20" t="inlineStr">
         <is>
           <t>SmartCompany</t>
         </is>
       </c>
-      <c r="D66" s="19" t="inlineStr">
+      <c r="D66" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNTXhwVlVLUy1pWEpFdzFCazNTY0dkczd4WW9oeW14cUtTaDZRTGlVQXBPaHN4WTBkNW1zOGxvN0tVWl9JSFdVNXlQMzVxbk4zbDZFUjNOcUxSamNaSnFCckMzWEk1VlNoSHJHQ3VWdGltVWZCV0c0NmU4UlN6YU55Q0J2TkQtUzBzOW96UXRxem5Zb3M2SUljNURISlRkQmJD?oc=5</t>
         </is>
       </c>
-      <c r="E66" s="19" t="inlineStr">
+      <c r="E66" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2368,7 +2371,7 @@
       <c r="F66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="19" t="inlineStr">
+      <c r="A67" s="20" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2378,17 +2381,17 @@
           <t>Kal Somani-led consortium buys Rajasthan Royals for USD 1.63 billion</t>
         </is>
       </c>
-      <c r="C67" s="19" t="inlineStr">
+      <c r="C67" s="20" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D67" s="19" t="inlineStr">
+      <c r="D67" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOX3lmdG5aTmk4TEpBa3ROdWZ1aDJHUElBQXktVmlKaHFmTUhPX1QxX1dKLXZfaHRDQjBnWm9McTZjTjJtTWFETTRNMHgzN0tTTm1xY0JpMF84Q2lNaFQyZGVjaHN4bkVmcDN5Qy1ta3FtYnpMSVVyYm0ydWpTRUdZU1hoYXpaNkZUQzlPc1QycjZ6aG5QVHRqY213?oc=5</t>
         </is>
       </c>
-      <c r="E67" s="19" t="inlineStr">
+      <c r="E67" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2396,7 +2399,7 @@
       <c r="F67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="19" t="inlineStr">
+      <c r="A68" s="20" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2406,17 +2409,17 @@
           <t>KMD says Rip Curl demerger proposal delivers investors ‘no value’</t>
         </is>
       </c>
-      <c r="C68" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D68" s="19" t="inlineStr">
+      <c r="C68" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D68" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPTXhBdHByWE9EbllFdDA2OW1UTUZEMVJfV2xsNFdURFRKX2JrODJReVRuQlFoakpWbTBKcjhNLUVsNE9sdG5LUElLZlVrbFNERS1QZTN6bEZIWEhXZ1pTWG5GWEw3ZmNETTdDUDUzYzR5M0E3ZGVlTWpSUnVlVU56dDNFZUtZN3liZ1dKNzJhLWU1S0M1ZnlKd1JNWXlxSlkyU3pGS1lhS05hTUJPRkxucldabzFucGs?oc=5</t>
         </is>
       </c>
-      <c r="E68" s="19" t="inlineStr">
+      <c r="E68" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2424,7 +2427,7 @@
       <c r="F68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="19" t="inlineStr">
+      <c r="A69" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2434,17 +2437,17 @@
           <t>Ex-Macquarie banker drives mortgage broker roll-up Recludo towards IPO</t>
         </is>
       </c>
-      <c r="C69" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D69" s="19" t="inlineStr">
+      <c r="C69" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D69" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxNQms5X1F2aTNhOExDbW42TlZOLVJwVWxna1JYSW9vWF9Na1RZa1ViTFdZc0tCcXRZZkRudTlsTzNuZGgwSENyYi03Zjdfc0lZTXp0NmJRZnhzb2pWRXRIOUdJN2lQM2h3ZFFtTXlSWHVWOFBIaW1Na3FQMjBCck1nVlhUcmRkLW9LOHpKWXQwTm9LcWR5M2FfdjFiRW04TndoanR5NmJvMENGalNuUGNINy1Qc20xR1J4d21ncHNNSUZqa1BXNnI4STIxSUFkZXdU?oc=5</t>
         </is>
       </c>
-      <c r="E69" s="19" t="inlineStr">
+      <c r="E69" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2452,7 +2455,7 @@
       <c r="F69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="19" t="inlineStr">
+      <c r="A70" s="20" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2462,17 +2465,17 @@
           <t>Coles reviews truck fuel charges as crisis worsens</t>
         </is>
       </c>
-      <c r="C70" s="19" t="inlineStr">
+      <c r="C70" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D70" s="19" t="inlineStr">
+      <c r="D70" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxOSGpBM3RjLVJ3LVlmR1QydnY2dm50WlVxcG43ajRFZ25QS1hDNTBONU8tY3Z2TklzbUNla0ttZk1GZzFaLUZRakFjSUpUQWItQ0VqVTVwS1B0QS1ObVEzNzdRT1l6aU9pVm5jSlhna1N6QmFKT3k1RkhMZGNTVnVLcDVIcXZmRjdjLWRpYVlRQUVmcVRtM21BSjVhTGNaaThyZkhLS2NWdkNCSkZKTlloUVdtbzRnYjFKbllOZXhOd3lkcFZEYURwUFVNQzVnSWRyM1RlOGd2M1pMZXI3c0NIa0Y0MNIB6AFBVV95cUxNSjB3Z0hoTGxwOHJQQ09xb3BmRmhCYjBCc2E0OHA2elFDRE45UGpaTEVDc1Y2VnRvVmZQUzRHbng4QTMwNGZZNGpmaVlHRmV6bnhiZ0FReU50TnRiQ0NZMEtoM3dBZ0hXbFBZMVJQNXd4LVdXRDVyTDAxNS1zeVdvcFVvend2N3J5R2pLYmhxNVFfd19rUlRsNWNndlptMUVkcS1CaUN6UXRHVzByTU5BMW1TdktOZUJYck5xMEJucmR6czIySEMycDA5cmR1MXB0N25Xc0JDUG9zN29YWklVc1BUMzl3UVhn?oc=5</t>
         </is>
       </c>
-      <c r="E70" s="19" t="inlineStr">
+      <c r="E70" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2480,7 +2483,7 @@
       <c r="F70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="19" t="inlineStr">
+      <c r="A71" s="20" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2490,17 +2493,17 @@
           <t>Sam Arnaout’s Midas touch turns suburban pubs into pokie gold mines</t>
         </is>
       </c>
-      <c r="C71" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D71" s="19" t="inlineStr">
+      <c r="C71" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D71" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQV2xlTTdYOFpIMzNmVVRnMlJRbTdGTC1jelVCd1V3UjN5cHQ1VzhWZzhrNW1PNm1RX3FlZmU3UkRycjF4WDlQUzRMcVVYY1g3UTZqQ0hxRnl2Ti1IQ0owVmZjN3Jod1BFbmhPVUwxNjhsTGh6d0kzdU01N0hmempRZ044ZmZNUllnenhyc3djRGJOdEtrekx5UVFoaFFMWDdqMHMwdng1SFg4TzZHY1hQNFJNN3huZXpWYWFtQ0ZJakhkVFlQcl9SQlRfZkQ?oc=5</t>
         </is>
       </c>
-      <c r="E71" s="19" t="inlineStr">
+      <c r="E71" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2508,7 +2511,7 @@
       <c r="F71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="19" t="inlineStr">
+      <c r="A72" s="20" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2518,17 +2521,17 @@
           <t>Gentlemen at Melbourne’s exclusive The Australian Club sweat another election</t>
         </is>
       </c>
-      <c r="C72" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D72" s="19" t="inlineStr">
+      <c r="C72" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D72" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPcEwyU01BOXF4TzlmREhYbTFEWklxdWZqWmZybDVnOWtLQ2dTU2dNQ2t5M3BVT2stN08xYkFmazVkY29oT3RVc2xUZmZINFJURGtIRTg4RGsxOURBdWEybTUwU2NUODQ2eDNBbTdPT3QxeXRFNHlSc014T0g1aG4xZ1A0U0FWMTB1Wm1CSHlQU0ZJb3lMYkE?oc=5</t>
         </is>
       </c>
-      <c r="E72" s="19" t="inlineStr">
+      <c r="E72" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2536,7 +2539,7 @@
       <c r="F72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="19" t="inlineStr">
+      <c r="A73" s="20" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2546,17 +2549,17 @@
           <t>Inside Fortescue’s AI ‘hive’ that could save the mining giant billions</t>
         </is>
       </c>
-      <c r="C73" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D73" s="19" t="inlineStr">
+      <c r="C73" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D73" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOSVVCbGpzcVcxTGlZZ2dTUkxXdVVvVU1ONEtUS0t1R1VkWWRNeUF1UmlHbXd6clR3QVRuWGxrUGQwVG1OeUxZb2RqTzdYOEVGQ1N6eDFta3VOZDdHNThYbUEwWEVHZlZBVzNpZ1Foak1kLURZTWpJVzZLekczdzFrdHMtLVZwMUZnYmkxSVc0czFqWnFaSGZiT2pIVW5rdVZmdThreFlRZWVEU0xoa1VFOV9MTjE2UHFOcWhqUzVB?oc=5</t>
         </is>
       </c>
-      <c r="E73" s="19" t="inlineStr">
+      <c r="E73" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2564,7 +2567,7 @@
       <c r="F73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="19" t="inlineStr">
+      <c r="A74" s="20" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2574,17 +2577,17 @@
           <t>Tiny house maker Elsewhere Pods seeks cash after Bunnings debut</t>
         </is>
       </c>
-      <c r="C74" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D74" s="19" t="inlineStr">
+      <c r="C74" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D74" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM0ZpVnBTS21Ib25qa09CaU52Z29kZWhTU0FJLW5VR2JCLVFPTVlZTmpYX3lZVWdtMDVTYTJkWHlPUmhXa0Rua2ZXTTBWQU1VdmFrV21KOGlrdjJ3TTdxbGlvZVBUZUxUWE1uelpWMGxWWk04UndJTXVKQjBZUEtoX3lodmdpMWZKNUc1YTIxVFZLYkFKT1QwbS01WU01ZUZTTlczY2ZpLXlpTjNJTWpsUg?oc=5</t>
         </is>
       </c>
-      <c r="E74" s="19" t="inlineStr">
+      <c r="E74" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2592,7 +2595,7 @@
       <c r="F74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="19" t="inlineStr">
+      <c r="A75" s="20" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2602,17 +2605,17 @@
           <t>Chinese consortium emerges as dark horse in Made Group sale</t>
         </is>
       </c>
-      <c r="C75" s="19" t="inlineStr">
+      <c r="C75" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D75" s="19" t="inlineStr">
+      <c r="D75" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxQYlpEY0hxNm5lalIxSTUzbDE4UEF5QTNpMTl4dWNPMkRrMU1yQnltZ25WcUkwOU13V2Y2RGItVW5QTXotSnBZRUJMdGJySGw0NVVxc3ZLZmVEcTlfU193Vkd5UVVuTFVYWFNtd185eGlVQW5RRElHdk5pMjhUR24wd1k0T0I3cW9qTG5Lcjg2bV9aNWsya0FYODRjeURyMW1EeHdYT05iZHZhLVFrUVNoV25idnZYZ2lpZEhta2JxOWFJb0M2SE9hbFF6NlVWYTM3QmF5anpWOEZackZiTDBfN2gtX1luQkxFOUxSSNIB8gFBVV95cUxOQklMYWl1ZkRqZGUwN0ppeXFubzZWNTNmeE5GY1BfcS13N2dFT096YW9JSndVX1EzTlBKdWZIemdKZnRIME9SQk5aT1M2WnRESjJxckFTaUdOSEd6eG9hRVBjdlhBbWQyWGpUS1kwQXJsdlpkLXJpXzJZX2xiUC1FSlNnNTFoVXQ4bF9JeUp3UGRWdUFOUVRrNUtsRzRxaUczb1p2LVVucFBNazhuZFNDaUZDR2ZQUVdObmVtTnBndGlkazZqeHVheVNzSE9RY3Bad0lrckxDSWY5QXBWS0hwVzZvSTZjaGEtNkNncW1RRE5uUQ?oc=5</t>
         </is>
       </c>
-      <c r="E75" s="19" t="inlineStr">
+      <c r="E75" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2620,7 +2623,7 @@
       <c r="F75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="19" t="inlineStr">
+      <c r="A76" s="20" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -2630,17 +2633,17 @@
           <t>KMD faces uphill battle in capital raise as key shareholder baulks</t>
         </is>
       </c>
-      <c r="C76" s="19" t="inlineStr">
+      <c r="C76" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D76" s="19" t="inlineStr">
+      <c r="D76" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxOVTU0OGNfRURNcDdzYUtIcG8tR3N4OFFYalhKNWJBaUd6ZlQwNU5MZVZYbUZVSzB3WmdOOFdTZHlBOXBzSGdYUVV6eGt1UndHN296bENxZzNUM2NoaV93LXZaZFNNOXJ2YlA4RHNFS2FDb1ltNWpPWUdRR3VGMWoxaU5qYm9VSW9yUW5kS1NaN2RSc2YtcHZRSTB6aE9Zdkl3NG5nbVRzODRfQVYtelo5M3g4R2JEbnpraFpWbENOZzE2Qndla2t3MXRPWkU1dXg4NmZRME1jT3pOOHZOVlpTZGloNENUZllaSTFmWUV1Y2JLck02ZDhnTHJ5bUPSAYICQVVfeXFMUEFXR29tQjlTbTdMRVNDWUlGNFNOQjVhX0FiSkl0U2stbml5VHR4d1g3bDFqMUw2TzR1eHhYOU5ZUmJpZ2xBY2NzcmJRX3MwaEQ0YmpzMUFnV1BQNGxmcnlXUzVvbHpwNEo5dWFnZlduZ0Z2dGZGRFRKRTNCUzctZDNCd0FMNEkzTm84dmZOM2NKYk81RERsVnlZN1VZaXp5TW5QRVAzOHNXQTFWdVlKdGtFX0FmcU1EbElZSm52alBQeWx4VnlvOFRwNk1ia2lZYXlpemQ4cFdmckotMmMyRGE4ZXN0dThQYmxxUkpvMzAwRXBBcVJuRnp0QkZ3b2tqMWF3?oc=5</t>
         </is>
       </c>
-      <c r="E76" s="19" t="inlineStr">
+      <c r="E76" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2648,7 +2651,7 @@
       <c r="F76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="19" t="inlineStr">
+      <c r="A77" s="20" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2658,17 +2661,17 @@
           <t>AustralianSuper claims another listed M&amp;A kill with Pepper Money</t>
         </is>
       </c>
-      <c r="C77" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D77" s="19" t="inlineStr">
+      <c r="C77" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D77" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOY0RwcnpWZlhfOHA2MG13MkJUX1RDNF9wN2RxZGU2cEpzS1RKTjJDeUl0OERFOGhFRXJaSXNETEhHbW9PS0lua283RnFVbHJvTlRva0djQ2lRSGc2RENJYmt0OEsyYTRVSzFGeE9jWVhKMVRnd240WXVNTVdac2lOUGJSZlc4UVZ5RXo0OTlQbUd6NWRSek1HZG9fZGk2aDhDelhGVmk4YkRKeVV1M0VHZ2hZNmFVdXM?oc=5</t>
         </is>
       </c>
-      <c r="E77" s="19" t="inlineStr">
+      <c r="E77" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2676,7 +2679,7 @@
       <c r="F77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="19" t="inlineStr">
+      <c r="A78" s="20" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2686,17 +2689,17 @@
           <t>Apollo to Acquire Nippon Sheet Glass in $3.7 Billion Deal</t>
         </is>
       </c>
-      <c r="C78" s="19" t="inlineStr">
+      <c r="C78" s="20" t="inlineStr">
         <is>
           <t>Wall Street Journal</t>
         </is>
       </c>
-      <c r="D78" s="19" t="inlineStr">
+      <c r="D78" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOanpORVBremoyamJyZ2FqQWVOcDcxa2NpempBUmNYcktMLUl1Mzg5VDloWmlVbUdNUnplVk90WEUzXzJjNGxENk9LcGF0enVSdlFpWU9nd244YWNTS0ZHd1JTZEtlbjRQTmJUU0dzWmlDOVFhR1ZRSFJkNXN4a3FHdGozcUcwdHRseXpYMFREUzBNcXRmQ1VCN056SWlEa1l5VVE?oc=5</t>
         </is>
       </c>
-      <c r="E78" s="19" t="inlineStr">
+      <c r="E78" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2704,7 +2707,7 @@
       <c r="F78" s="3" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="19" t="inlineStr">
+      <c r="A79" s="20" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -2714,17 +2717,17 @@
           <t>Estee Lauder in talks to combine with Jean Paul Gaultier owner Puig</t>
         </is>
       </c>
-      <c r="C79" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D79" s="19" t="inlineStr">
+      <c r="C79" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D79" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPSjN6QnFVbmdHWFoteURWaU5VaWZmRmpTT3QtYm1tZUFyNUZyLUdheGdfWlRBTlJyTlp4THIwVDA4U3BnWFNpT2FpZlZzX1lJSDV0MkRGVjYtNVc0b0lOQy1RSnFGTWhCTWE2ZFFPYlFQX05yaVlfZF9IUEN2ZWkzQ0VFMUxxdHF2ODNQY09xdWlqWEczSC1CZk5wYU9QQlAyaTMyelJnaVM0cmN4M0paNzlBdzM1RndoZE8yRHN4UnZqaXVhVmx5NFpqS3hmUHhUdlpF?oc=5</t>
         </is>
       </c>
-      <c r="E79" s="19" t="inlineStr">
+      <c r="E79" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2732,7 +2735,7 @@
       <c r="F79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="19" t="inlineStr">
+      <c r="A80" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2742,17 +2745,17 @@
           <t>David Jones accused of squeezing suppliers as losses mount</t>
         </is>
       </c>
-      <c r="C80" s="19" t="inlineStr">
+      <c r="C80" s="20" t="inlineStr">
         <is>
           <t>The Age</t>
         </is>
       </c>
-      <c r="D80" s="19" t="inlineStr">
+      <c r="D80" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPdUtyNWs5YmxJMXNsNWtaMi1WMm5SVHd6ci1ReURLajdYd1IzWGJMZmE2MzJsSzAxQWtSTm8xMUEwNTh4Vy1zTmFsWFBKTkJ0YXc3ZkcwOVk2a2VNRWVGUS0yQzZhSXlCWmpDYUx6RmpTTlNhS0xIQklyVFdIVXJRZTNPaVB4TG4yQ1R1ZWF2MWpmSG81TVRaRzdtMXpydWhBS2w0a3ZPZFI5MnFKOW5tN21oUDB3NkNtQmR4LVVBWW9BUQ?oc=5</t>
         </is>
       </c>
-      <c r="E80" s="19" t="inlineStr">
+      <c r="E80" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2760,7 +2763,7 @@
       <c r="F80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="19" t="inlineStr">
+      <c r="A81" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2770,17 +2773,17 @@
           <t>Australia’s new millionaire factory: Start-up to $1.6b in five years</t>
         </is>
       </c>
-      <c r="C81" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D81" s="19" t="inlineStr">
+      <c r="C81" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D81" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOVkl5N1NGWS1XWWZSc0pHXzE3MUNERmV5SUgyQ3o2MmJ3U3Y2YlNwUXNSTGlQenBwVFdnMWhoT2FrcDAwUHNVU0RQbjFHMjJiLU1TRC1nemdrX3hPTG93VWZUQUx3Wk9HT3lYd055Z2FtREFpOWRlYXFDb2hwV0cyWFMwaHpsLU0ta2VVQlpid1dlYks0ZHg5YTY3Ykt6Um5YaF9MR2tIRzd1Tk1IRnBrWVhxVjZNSUl1OE9iRlZzYmQ3QUVnZmhYVGxoOA?oc=5</t>
         </is>
       </c>
-      <c r="E81" s="19" t="inlineStr">
+      <c r="E81" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -2788,7 +2791,7 @@
       <c r="F81" s="3" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="19" t="inlineStr">
+      <c r="A82" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -2798,17 +2801,17 @@
           <t>Social Media Wrap: Genki Sushi Singapore's loyalty benefits; Dunkin Philippines launches new collectible; Burger King Malaysia unveils new Korean inspired burger</t>
         </is>
       </c>
-      <c r="C82" s="19" t="inlineStr">
+      <c r="C82" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D82" s="19" t="inlineStr">
+      <c r="D82" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxPbFR6eHVTRWZNcUw1TTBJdE1JTFpmbk5iWndKZnRoU3Fmc3cxcF80TnVhRERmY0poM09zTFpCaEVnMGo5aktxY0ExV1ZlZVpHYUtldXBoOUh6bm14SURHNmhnUE9tYnI5YlpXQ3pRZlp0Ni1wM2lYQmdxdjk4SDl0aFN0R1VBbGxpbFVzOHV0TFY3YjJZbDg4Vk1HMTBkQk5LRHd1ZEVpRnBsT1U0Nm1IbVFkZEUybmpabEhuLUNLOGhicUxXZG5UalRLOE5DSzcxRncyNjVRdk8zclhJNkVQcTRkQTZYSEdN?oc=5</t>
         </is>
       </c>
-      <c r="E82" s="19" t="inlineStr">
+      <c r="E82" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -2816,7 +2819,7 @@
       <c r="F82" s="3" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="19" t="inlineStr">
+      <c r="A83" s="20" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -2826,17 +2829,17 @@
           <t>Copyright ‘status quo’ not working in AI boom times, says Charlton</t>
         </is>
       </c>
-      <c r="C83" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D83" s="19" t="inlineStr">
+      <c r="C83" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D83" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNVVgwdEQ2YUt0eFo3THcxOXZHbUFYZ091VTFKZDZHX0szYWQ2dnZ1dkJma3VZcGk1LUM2SUtQSWhxMGpCUlFZVzdKNmdoSGEycm1oYlBUdEZ5R0ZlU2hrWHpFWXdSN1lCZnZzb3hZc2twVVlWdTNNVXhaR0Nza0FiaUNveXZWQWQ1ZE45MU1HbGNmWlU2aUdha2FyZllzNWdONEpsM2RrdGRFSFl2UlpJUnQ4WGpleGs?oc=5</t>
         </is>
       </c>
-      <c r="E83" s="19" t="inlineStr">
+      <c r="E83" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -2844,7 +2847,7 @@
       <c r="F83" s="3" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="19" t="inlineStr">
+      <c r="A84" s="20" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -2854,17 +2857,17 @@
           <t>The unapologetically analogue 4WD for off-roaders with $120k to spare</t>
         </is>
       </c>
-      <c r="C84" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D84" s="19" t="inlineStr">
+      <c r="C84" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D84" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxPSFJ4ZnNLT3U1REp3MWI2WDFaQm5vZlp6QWN6c0hZamtYVU95WmpkUERwR1dwc0NQN1dEc0FNbHlaMTdLclVHb1JTc2VZNExENGYyUE9OR1BkQ244YXRVeWNwbkxia2VrckVqSy00WV9UNWlvZWJHOG9ibUthaTlpVmRBOGZjLWFzMU8yS2Q5Um05SWIzY2dKajhoMWFUcmFrbTMzai1CdVBNLWczTWRvbTBwSDRfUzNwOHhqQm5hTDdhM0xLWEpNQTRyRXZjU1FLdGhRMUxtOTg?oc=5</t>
         </is>
       </c>
-      <c r="E84" s="19" t="inlineStr">
+      <c r="E84" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2872,7 +2875,7 @@
       <c r="F84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="19" t="inlineStr">
+      <c r="A85" s="20" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2882,17 +2885,17 @@
           <t>Junk room to become jazz club with priceless Melbourne view</t>
         </is>
       </c>
-      <c r="C85" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D85" s="19" t="inlineStr">
+      <c r="C85" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D85" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQbHN4My1nOGtueVJQZWM0LXNjLTR3MmhuemRJMUEwN09FTUZhZk1lbV9MbnVWblgyUXFEMEl3LUtsOGVqdGUweFR0MXF0ZEo0XzNhWVRqb2pGRUdiNTlLc1dFcXFmdnctQU1wQkRSdHN0T3J6VGt3MU1iNENydGlsOEpsT0ttZmJVZ0FUZmFXSUd3alVzUTQxMzVmcEVXSlV2dWdQd3JsMUZ0d3ZZYlBHaGhKTm9rM01SUmdseE9hT1prbHZtMlhv?oc=5</t>
         </is>
       </c>
-      <c r="E85" s="19" t="inlineStr">
+      <c r="E85" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2900,7 +2903,7 @@
       <c r="F85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="19" t="inlineStr">
+      <c r="A86" s="20" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
@@ -2910,17 +2913,17 @@
           <t>Zimmermann fashion label appoints new CEO Roberto Eggs to replace Chris Olliver</t>
         </is>
       </c>
-      <c r="C86" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D86" s="19" t="inlineStr">
+      <c r="C86" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D86" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQM2M5QU1scVoyNHBmV2lwQ0VQS1Z6d2Qwa1ZkZ0M2WVIzdXR3QnZwVWhUSDRCUEdRZkc5QzFQSFFhNzZ4VE9lWXBTcGhpS01JdG12TlQxSHhValZfbWt3MUdFZGl3RlBtdnlrel83TjNjNFZ0SUpvSDNQbThpU3FLa3Atd0dNU04zQm9OSk5uNHpTVE84aWZpaVlKWkdOQjJjRTZSd1MwMEZ1b3pENkRCQQ?oc=5</t>
         </is>
       </c>
-      <c r="E86" s="19" t="inlineStr">
+      <c r="E86" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2928,7 +2931,7 @@
       <c r="F86" s="3" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="19" t="inlineStr">
+      <c r="A87" s="20" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -2938,17 +2941,17 @@
           <t>Construction giant FDC road tests IPO pitch - AFR</t>
         </is>
       </c>
-      <c r="C87" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D87" s="19" t="inlineStr">
+      <c r="C87" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D87" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNTnRScHFhQlpkdEdSb2x1bExxQm96ZE5zSV9wTDNDV2pxYjFQdUtoYmNBell3SFlTTFEzMUhpeXlmNERSeDd6VGppM2szQ1NHVE9PY1R3MTN0SUZLWkF5em8tQ3IycUZ2RmswX0tnN1IwOHl1ZFo4UUtMUDlQbXRjTnRCWFB5cU1RZFhsdDdaWGpMZzh3d29CWWZvZGtnTjl0T1k5ZHFHSUg5XzFSSF9TSUxTYkU0QkFheFlLZUY3S2tCSWRLZWlBbUpxUjc3TXBQQ01V?oc=5</t>
         </is>
       </c>
-      <c r="E87" s="19" t="inlineStr">
+      <c r="E87" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -2956,7 +2959,7 @@
       <c r="F87" s="3" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="19" t="inlineStr">
+      <c r="A88" s="20" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -2966,17 +2969,17 @@
           <t>David Jones is trying to defy retail gravity. It’s causing problems</t>
         </is>
       </c>
-      <c r="C88" s="19" t="inlineStr">
+      <c r="C88" s="20" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D88" s="19" t="inlineStr">
+      <c r="D88" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPZy14UldWZDRrSjI3R0lzdGlKamlkVnU1WWVjTWRUTlpya1ZpVW80WHlrT0FQTUUwMzkzM19xQWpwTnVLOF8zeTFXamhTZFRQVjl5TTlXbE1RRWY2NW03dlpmZ25qdkgyN1IwbDdjRlhxd1MzSGkxeG45M214OVlESWF5WWh5TjM0STQtOXdieWIyOUI2NzRsaDhiS0ROUU5YQ185aWtObUY2S0dOSTBROVlwSVB1VkNqTkZTTllkZmtMYmxjNVdlTA?oc=5</t>
         </is>
       </c>
-      <c r="E88" s="19" t="inlineStr">
+      <c r="E88" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -2984,7 +2987,7 @@
       <c r="F88" s="3" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="19" t="inlineStr">
+      <c r="A89" s="20" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -2994,17 +2997,17 @@
           <t>Jefferies’ Australian ambitions in focus as Sumitomo circles</t>
         </is>
       </c>
-      <c r="C89" s="19" t="inlineStr">
+      <c r="C89" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D89" s="19" t="inlineStr">
+      <c r="D89" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxNUTd0LXFPQmZXSldrTmZHTkIwUWQ3MmlCUmFOUGRkcVVjRXV6YXZJUTcyMG5FV3I0dWY2NXh6MnduVjNxZmhJMHdDVGw5VzFxTEFzN2FBdlNvS1JGSDltQmlzVS1QRDdCeWdfSHZ2VlZDMlBnN1Y0d2JxbnlGejhWVjJpWGZLejdCTUt2Uk9ENmhyRkd4dDJjd0RlUnBlZXhOTmUtOG9ITE05VHJ3dTBRSWZneURuUW1NYkExVXpfWXlsMzZ1WUlyNE84SThQX1JJTFlXOHc4ZnB0aXRmdVhaaG1qSEJRZUhuU3RibHAzbHVNLWFLUF9NNTFoUXV3NGQzelcwcNIBigJBVV95cUxPMkhEeDJpNzg0NTlDZmF2LUFPSEs4cmZ5U2p6bWVZSTYwcXVUUGVIb0FLVnhZV0cta01CLVpfQzQzYzdvTWdxR0o4bGJDWDVBb1lnOGx0bWROdTdjcHhwLUpPMW9MQ0RVM2NUOUt6UGpTd05JYzhuVmgybGp2LVpORFF0SHpBTU5DUTJEUmZKUFBNajlQdHJ4WkdHVV9QMjVwOWVlNWliVkFaM20yWGZhOEc4bldHRERJak1BWXlmSE0zdno1VTVSc0FMck0wSE1BR1RVaVRMSEdzU2FvcWpMYmp5ZTVJTWcyUGdXanhqSUNZU0tzTkNYWVg2SXpVMEoyS184VkxOeWtSUQ?oc=5</t>
         </is>
       </c>
-      <c r="E89" s="19" t="inlineStr">
+      <c r="E89" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3012,7 +3015,7 @@
       <c r="F89" s="3" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="19" t="inlineStr">
+      <c r="A90" s="20" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3022,17 +3025,17 @@
           <t>Bain Gets Nearly $300 Million Loan for Australia Wealth Unit M&amp;A</t>
         </is>
       </c>
-      <c r="C90" s="19" t="inlineStr">
+      <c r="C90" s="20" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D90" s="19" t="inlineStr">
+      <c r="D90" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOMUQ4WExYZFY1aFBwWENNR1JiVkw4OHFKWjY4NW4zQ3ZBalFiTU10Y2hic2p2VjFqOE1rMndNYmVoN0lPcnY0WmFOV1MtaEY5c2xvcW1PNGN2SzZVcThwc3ljWkYwV1Q4a2dIaUpBeXZpMkRUU3IxZzVBVkhydGU3OXEzNW1sdlVQeTRNRFY4bUJLOGpGYmJ0ZXpPc1YzY05TYWd2bF9oWVJ6Rks2dWlod1dGRU4?oc=5</t>
         </is>
       </c>
-      <c r="E90" s="19" t="inlineStr">
+      <c r="E90" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3040,7 +3043,7 @@
       <c r="F90" s="3" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="19" t="inlineStr">
+      <c r="A91" s="20" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3050,17 +3053,17 @@
           <t>Fund managers caught up in Aware, TelstraSuper $237b merger</t>
         </is>
       </c>
-      <c r="C91" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D91" s="19" t="inlineStr">
+      <c r="C91" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D91" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPcFF4Q1A5X1VtNWFnYXZSVUlZX2JMRVoxaUJoeGhybmRrZkd4UlEzTURwMkx2d2I1Y1hMYmljbk05WUFzRl9JbF9JampqeDd2bXdYcUpHbVZYak1sYXFHS2VuUDJyTUhzSS1QTW15aVpfeHRuMGZHenlxOHJQRUdENkV0b2FMZXhOZWF1Yk5hR1lOYWFQc2Q0SEROUFNERXhKQUIzRkt6NTQ?oc=5</t>
         </is>
       </c>
-      <c r="E91" s="19" t="inlineStr">
+      <c r="E91" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3068,7 +3071,7 @@
       <c r="F91" s="3" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="19" t="inlineStr">
+      <c r="A92" s="20" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3078,17 +3081,17 @@
           <t>Soul Patts defies private credit jitters with 15pc returns</t>
         </is>
       </c>
-      <c r="C92" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D92" s="19" t="inlineStr">
+      <c r="C92" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D92" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPRkNINFJOai1NbUUtX3ZrcnJFS3EzRHZPbFRfVFE3SERudTVqbjIybWsyYUthOUJOUVFPb1U0UzlGTTRqbUxraFZfYlVtclQxeTBQU1M5YjJzMDVPU3RiX0cxbk8xOEd5YjV1R04zT0NNZjhNSi1meWo4RHM1ckFsUnNLd0JiQXFnZ0dtckNzdWxmanZoQUl3TEQ2a29nRkRDZ1lJd2Y5VGc2UWZHX0pkU1NObmRJTlZKS0E?oc=5</t>
         </is>
       </c>
-      <c r="E92" s="19" t="inlineStr">
+      <c r="E92" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3096,7 +3099,7 @@
       <c r="F92" s="3" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" s="19" t="inlineStr">
+      <c r="A93" s="20" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3106,17 +3109,17 @@
           <t>Ex-KKR China heads negotiate to buy Vitaco, owner of Musashi, Nutra-Life</t>
         </is>
       </c>
-      <c r="C93" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D93" s="19" t="inlineStr">
+      <c r="C93" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D93" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQRmlCdTlFeHdBUGkyOS1CeEFIYTRSREdZM1JOZ3IyZThnNmNMdm9QeXVwRWtMbzU0em1vcDAyM1hodDlvalVRdThtNVhLR2FsaE1vV0xuWjkwMkVCUDk5SmVka1BURFJZNkl2bURLeC1GdzI0V2hEaVhrNlJZejlvc2gwRmtnUjd1NDFlX2trbGk2aXJiQ2FrTWtmVVpiOXhBc05JSkNYY2xLX2JEQUpWY2dlY1pDZw?oc=5</t>
         </is>
       </c>
-      <c r="E93" s="19" t="inlineStr">
+      <c r="E93" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3124,7 +3127,7 @@
       <c r="F93" s="3" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="19" t="inlineStr">
+      <c r="A94" s="20" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3134,17 +3137,17 @@
           <t>Antipodes Global Investment Company</t>
         </is>
       </c>
-      <c r="C94" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D94" s="19" t="inlineStr">
+      <c r="C94" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D94" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE5mdkJzN19XLTFQc25LOUk0ZGJBMER6djB2VnFvbGVrS1hlemRBRmlNY2JmMGlPTzktU0RRS3NNUW8tRXhtUE1QdE1JLWdUNVhibmZPZi1MRkJOWk95NzM2bXplS3JzeG13UU5henhza1ozeGRZZmlBNTNR?oc=5</t>
         </is>
       </c>
-      <c r="E94" s="19" t="inlineStr">
+      <c r="E94" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3152,7 +3155,7 @@
       <c r="F94" s="3" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="19" t="inlineStr">
+      <c r="A95" s="20" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3162,17 +3165,17 @@
           <t>AusSuper to lift insurance premiums by up to 40pc</t>
         </is>
       </c>
-      <c r="C95" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D95" s="19" t="inlineStr">
+      <c r="C95" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D95" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQNEhYQkoyNnJFU2xBZG8wdXhEZWRSakRiWWNHOGZBTFhfaElxWkRsSWViaWxjenVjMF91cGdrbFZxSGJfbkR2SUZNdEJtYUVadlV6YVVrWU1VbVdsMWpyNUZ4bE13Mmo4cGQ3WWZlVFVrTTdyOGpSdkpUb0tkcjdQUFlsTnM0MnpOMDJNZlJ4YTlzZGpLS1QzMFluOFU2VUJya3lSclBLSnZkQ2Y0a2djNUpSYlo?oc=5</t>
         </is>
       </c>
-      <c r="E95" s="19" t="inlineStr">
+      <c r="E95" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3180,7 +3183,7 @@
       <c r="F95" s="3" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" s="19" t="inlineStr">
+      <c r="A96" s="20" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -3190,17 +3193,17 @@
           <t>Unions want inflation-plus minimum wage rise due to ‘Trump and RBA’</t>
         </is>
       </c>
-      <c r="C96" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D96" s="19" t="inlineStr">
+      <c r="C96" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D96" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNdzNhU0MzbFRFX2I3OVY4bFItd1h6OVE2Wnpqb01NM2tMYzNob21BeW02LTBfTFZIWnN6SG5DVnYxQTJGZWZaLTJpTXZGUnhmS3RPY3hQV01fd1RIYU9Ednc4a1hvalVRT19ESU5TX19sQjN4dVV3X29kQjliQjNFU19iaXFIS2l3blk5TWUwdHFrRmJtQ0JocDN0WEhWbXZOVUJzR3RaYnJPSHpIRFlYOVFObEtuT1d0TUo0MUVZTXdFZWR3WG1r?oc=5</t>
         </is>
       </c>
-      <c r="E96" s="19" t="inlineStr">
+      <c r="E96" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3208,7 +3211,7 @@
       <c r="F96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" s="19" t="inlineStr">
+      <c r="A97" s="20" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3218,17 +3221,17 @@
           <t>Firmus’ Oliver Curtis set for green light to run ASX-listed company</t>
         </is>
       </c>
-      <c r="C97" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D97" s="19" t="inlineStr">
+      <c r="C97" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D97" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNR3VmQW9vNmUyeU9WbVRvRG9tcTNMYVlvRUhCd29wTkRZaVlEcG50Z0hIN29XcE5GUmxkUy1yMm0yTm94Q1BXMmNCcXBpZDlqVTRlZFpMX1QyMWh5Ym5XQ3VjYW1ZdDFtYWNyOERCOURuWXM5ZTV4WGthMVVjNUZlcmVTQ3JBUjQzUXRXYXRLQjlNeHpBMkVCVWpsd2Z1Vk42TjJxSlRiQ0ZtaTkzOTZtNmRHQQ?oc=5</t>
         </is>
       </c>
-      <c r="E97" s="19" t="inlineStr">
+      <c r="E97" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3236,7 +3239,7 @@
       <c r="F97" s="3" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" s="19" t="inlineStr">
+      <c r="A98" s="20" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3246,17 +3249,17 @@
           <t>Crisis Hit David Jones Chasing Funding As Retail Markets Come Under Pressure</t>
         </is>
       </c>
-      <c r="C98" s="19" t="inlineStr">
+      <c r="C98" s="20" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D98" s="19" t="inlineStr">
+      <c r="D98" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNNjJSOUVQcTkwUmxXNXg4ZzljSGhnRlBJY0otSHRrX2ZIQXRqWmNDZlgxYW1jckhHd3BtdXJsUWhwTjQ5SGw2NUU3TnFtcmhYd2JVcThIR2VCLWJLU0h5RE8xaTV5TS03Mi1za19hcF9PcXRRSU9PX3ZxSktSV2FfY1ppcUFVV2w1TmF1UWVtZlBWSUhEcG9oRGlEVkEwR2ltQ2VMSTNlcENEYlY0?oc=5</t>
         </is>
       </c>
-      <c r="E98" s="19" t="inlineStr">
+      <c r="E98" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3264,7 +3267,7 @@
       <c r="F98" s="3" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" s="19" t="inlineStr">
+      <c r="A99" s="20" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3274,17 +3277,17 @@
           <t>Beirut Street Food eyes niche in Lebanese fast casual</t>
         </is>
       </c>
-      <c r="C99" s="19" t="inlineStr">
+      <c r="C99" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D99" s="19" t="inlineStr">
+      <c r="D99" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNVlZVeTNGcXVOSXV1eklvTnFxYk1hb1A2VTQtNHkwdUpvdFF0YnlYU2RSWkZNV2dGQkEyZjRVQzVJZ2Uwc3gtZ0F1TGlSQlVna01HRnZOTTJnVUFxaWtOam1vZ245Z05jdlRnQURqbnQxaGtEcnFYS20wWmtvSDV0MW15c18zUE5ZN2JJWUpLV0RsZE1LSm5fcUNNeVZNTmdMQ2c?oc=5</t>
         </is>
       </c>
-      <c r="E99" s="19" t="inlineStr">
+      <c r="E99" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3292,7 +3295,7 @@
       <c r="F99" s="3" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" s="19" t="inlineStr">
+      <c r="A100" s="20" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3302,17 +3305,17 @@
           <t>Gami Chicken credits chip design for cult following across Australia</t>
         </is>
       </c>
-      <c r="C100" s="19" t="inlineStr">
+      <c r="C100" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D100" s="19" t="inlineStr">
+      <c r="D100" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPTXg4T0dvQ1l4NFVxV25iUXQzY0F3MnFjYmE4X0NOcFdNZHgweUg4NmVZZjNJbTFMajNhNHBmVDE2MGNBZzhOTUJsaG5KejFZbk1Db0JyNTZJbUI2WnRZeVhXRFRMNXVBWVFMdGJ3WkN5dV85dEduQi1OVDhOSE9UOGVERXh3T2hCVmlDNVg5LTdLY2VHNEZJSzlrN3VuemhzX1B5blpYRGtwS0hrak5r?oc=5</t>
         </is>
       </c>
-      <c r="E100" s="19" t="inlineStr">
+      <c r="E100" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3320,7 +3323,7 @@
       <c r="F100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" s="19" t="inlineStr">
+      <c r="A101" s="20" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3330,17 +3333,17 @@
           <t>The great fake meat meltdown is taking plant-based burgers with it</t>
         </is>
       </c>
-      <c r="C101" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D101" s="19" t="inlineStr">
+      <c r="C101" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D101" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPRTVDNW5oaWJ5bHdKM21iYllEVnpJbHhSbWFzYy1RcEZCdnNGUlJOWVJCaDZacFVoRjlSUGpfa3N6ckQtMFYzZTNITW5tMy05Sk0tZmtlSWlESHdOMWIyUWpUbE5RQVlsTHp0VXg0cHJYM0lJVmw1ckRURkFPVHFabTRIUzlFX1FlbFNuYmQ5MVJwWHVOaVhVWTdPajZxdG1WOTliTE1qZ3k1dnFRbk9BNTZCcXRRSGlIXzJv?oc=5</t>
         </is>
       </c>
-      <c r="E101" s="19" t="inlineStr">
+      <c r="E101" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3348,7 +3351,7 @@
       <c r="F101" s="3" t="inlineStr"/>
     </row>
     <row r="102">
-      <c r="A102" s="19" t="inlineStr">
+      <c r="A102" s="20" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -3358,17 +3361,17 @@
           <t>Solar for Cuba: How Xi is turning Trump’s war into a China win</t>
         </is>
       </c>
-      <c r="C102" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D102" s="19" t="inlineStr">
+      <c r="C102" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D102" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQOFlUUnNZUWo0MTJRaDFIZHp5dUJudERrOWxCZmY1WjZmeXRTVzJkbENEbUFhSkZFUWV6WjNGNUJIejVYRXFPcmRNZjFZeTkzTmtaeFNlb2V1OFFnMGtkV2JfTVRUN2FSV2xxcUpDUDJQeUpqWE9DRHRmT2kyc1dIZE9jeUM2eV9KQjd2RkJuTkxYeEdISDZDejhRbVo?oc=5</t>
         </is>
       </c>
-      <c r="E102" s="19" t="inlineStr">
+      <c r="E102" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3376,7 +3379,7 @@
       <c r="F102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" s="19" t="inlineStr">
+      <c r="A103" s="20" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3386,17 +3389,17 @@
           <t>Beer Sectoral Group appoints Nigerian Breweries CEO Thibaut Boidin as Chairman</t>
         </is>
       </c>
-      <c r="C103" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D103" s="19" t="inlineStr">
+      <c r="C103" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D103" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOamdsNTN1dkRUY19Yak0wUGxsdm9NZGhySUM0Vzc4blNCeldzdFBiRkxuSW1xbTlZQUJIWkNxdzI3Zi1zc3F3SmJvai1UVGlZdUhGTEJ0eF9mNHRwSGREbDktT2txWXA4OVBESTdPLXdxWmV2V3FPTEZaYjRWLTlMM1VaY1dCbGZudTczZlFEYzN1aE9HeWdObE1yZFduLUtNVXBheDNsUWlIcUxibml4YQ?oc=5</t>
         </is>
       </c>
-      <c r="E103" s="19" t="inlineStr">
+      <c r="E103" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3404,7 +3407,7 @@
       <c r="F103" s="3" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" s="19" t="inlineStr">
+      <c r="A104" s="20" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3414,17 +3417,17 @@
           <t>Hip pocket pain comes for shoppers – and for supermarket giants</t>
         </is>
       </c>
-      <c r="C104" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D104" s="19" t="inlineStr">
+      <c r="C104" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D104" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOeTdfN2dwYlBWSTdGbFo0SWRJcTNYelFFM2FBRnlORWRNcGd0WUVCbVdHVWZ6TFdZQzFpM2h6TkU2OEtqeE5OYlRrNmhsRU43a0E0UXhtZEZyTWZidzhMUEVxSVdiMlpTYXQ4ZVRaNl9BSi1Mb3JRaXhvM2hlMmNDcnk1aFBvVXFQSmlPbkN4Z3o2R2RzV0drQWpKaVZpbXR4dHppa08wRFd0dlNwcDc1alRDSXg?oc=5</t>
         </is>
       </c>
-      <c r="E104" s="19" t="inlineStr">
+      <c r="E104" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3432,7 +3435,7 @@
       <c r="F104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
-      <c r="A105" s="19" t="inlineStr">
+      <c r="A105" s="20" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
@@ -3442,17 +3445,17 @@
           <t>RBA calls for co-ordinated effort to unlock digital asset markets</t>
         </is>
       </c>
-      <c r="C105" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D105" s="19" t="inlineStr">
+      <c r="C105" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D105" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOT3dEcEtwVUptWTZydTRYWFdCU1RhTjI1RkFWeU5HckRVZjBxc2lqRkNOT0stc1h2Q0E1YTkxTjk3NTB3TGxKZGIweGFQRGh2S05QWHRoVGNZRFR2SlI2bkEzWlRoY2t3WU16dDlhVEI4RTFWYzhKS25YbGYxSVRjdFpVQ2M0dVc5MFJuUExNMTJIMVJTYmZGbkNLR1BPeVFYSF95NkNnWEEzamg3NmRuRkx0U2NjbXlxY015UWljTzRWbXpKclAwUg?oc=5</t>
         </is>
       </c>
-      <c r="E105" s="19" t="inlineStr">
+      <c r="E105" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3460,7 +3463,7 @@
       <c r="F105" s="3" t="inlineStr"/>
     </row>
     <row r="106">
-      <c r="A106" s="19" t="inlineStr">
+      <c r="A106" s="20" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
@@ -3470,17 +3473,17 @@
           <t>Banks rebuff work from home calls as Wesfarmers pauses business travel</t>
         </is>
       </c>
-      <c r="C106" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D106" s="19" t="inlineStr">
+      <c r="C106" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D106" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOTjFLNnZUNXZHeE85a3kyaG1IX29sWjFvZ2NzS041UnYxNkkwUF9YU3ZFYXhtQmlxY3Rmd0lUSTJrdTl1Y0ZobWp0M1lrZnZhZE9OSzV3Ql9Hb2UtUEpqWC1McjM0S2pESDJQVWJKQkw4enF5THJfeXFWRDZiMk5KMmVrazVUMzBNTk1tOXRVX1ZzVU1IUHBVSlhENEdEWFJpQnFXUGkyNVJGUnhzdXgyNW1WZXRkRmRaaVloZnpaMFdqVmk3elpFSkZ6ZmotZw?oc=5</t>
         </is>
       </c>
-      <c r="E106" s="19" t="inlineStr">
+      <c r="E106" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3488,7 +3491,7 @@
       <c r="F106" s="3" t="inlineStr"/>
     </row>
     <row r="107">
-      <c r="A107" s="19" t="inlineStr">
+      <c r="A107" s="20" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -3498,17 +3501,17 @@
           <t>This mine was fast-tracked to boost Australian solar. It’s exporting to China instead</t>
         </is>
       </c>
-      <c r="C107" s="19" t="inlineStr">
+      <c r="C107" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D107" s="19" t="inlineStr">
+      <c r="D107" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAJBVV95cUxPN1ZSdEMzSXBhMno2YzNkSFFtdlBOTTRGV3UtbnZtRktEd3Q0MHdmZHp0SDN5S0FZYmVKUllicHRMRkxTdmxtbkMtT2ZVN3hsUXdBVzAxdzhWcGFWRkxVdFY3NURqTVV2QVJQT0ZUT193R3JLLU9aZUw4YzlucjVUN0xyTzdoZlNjYXdyR2VWeDZrbW53cTJoRGZDd2kxbkxzMHBQWkRJMTFPMkNlX19wYjI2LVBZbnVJOVNsRjF3Tm0xUUFpY0ctczFZdWJFcHQyLUhwdDNiSGVtdHQzVVRtbExpcHJZak1SNkhWd2s4a0RtYWFNN2J2Q3FobTF1N0hWLXA4YUtaMXBScjZsUWt3alVVTVpJdVl0WDF5RTJLM1BKUl85dnhUUktkb2VwMzFkUWZ1ctIBugJBVV95cUxOOENIa2JzQzdxekNYTnJNVmRzdm9KTFpndnBybEJfNjBUR3VNMk92ZnhGY0JwVGZLeFRpdHJLMTQ0NjRNOFg5b3FESzhPLWlub2hSeFdidW0yS1h6ZXlGMjh3X3FhaWo1dHdneUZxS2NsaUJ6dWtfT1R6VndwSk52bVVNN2I5VlNYazBIelcwUkVBZHFlM0hiQVJ1a2NGWFpmR0c5R3Bna2RZMmJuSXB5WkQ1Zl94VDFtcjVEd2x6amIwSWdXUWtQVVo1Q0hpWVBLRVFycDAyU1NJV3N4YktlUlBtMTlkY2VNZjc1QVZhbnRrQ01OQnZqNzI5dTNNZ1VlNVVJcURycXlDRFZDYVo1aC15RXpwUFlvZWxlMHFybWJiM1YxT05lRElXYlZsbkJWUnI4VV9Da1lIUQ?oc=5</t>
         </is>
       </c>
-      <c r="E107" s="19" t="inlineStr">
+      <c r="E107" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3516,7 +3519,7 @@
       <c r="F107" s="3" t="inlineStr"/>
     </row>
     <row r="108">
-      <c r="A108" s="19" t="inlineStr">
+      <c r="A108" s="20" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3526,17 +3529,17 @@
           <t>A $600m dream or a dangerous gamble for cricket?</t>
         </is>
       </c>
-      <c r="C108" s="19" t="inlineStr">
+      <c r="C108" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D108" s="19" t="inlineStr">
+      <c r="D108" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxOYnpVaTZiU3hGMWY1UVVmYk9nRTJaRTVFYUE2ZklLYmJIQkdXZzFMbWs3MVRJb0l4bUpPeThwRnhOSmh0bzNBdzhpeXpuS1RrZ0tNVVJ4eU8tRVIwR2FyYmUtNG1UVmN2OXRsZm1mVy1LZDVERkpXQURMUk1HRE9Hc3F3RWQzYmFvbHRCVGhFOTQ3M2xnVGcxTWxtT3cydW84NTNPc3BXQURodmY0azBOUllOQjhrbzJ6WmI3bjY5dk5RRzlDQ0JlYzg0VzRsdWtIblZJelRSamFyQnNweHdHLTRTMTFOcy1Jd3ZtQWFodEcxOThVeVVz0gH3AUFVX3lxTE5ielVpNmJTeEYxZjVRVWZiT2dFMlpFNUVhQTZmSUtiYkhCR1dnMUxtazcxVElvSXhtSk95OHBGeE5KaHRvM0F3OGl5em5LVGtnS01VUnh5Ty1FUjBHYXJiZS00bVRWY3Y5dGxmbWZXLUtkNURGSldBRExSTUdET0dzcXdFZDNiYW9sdEJUaEU5NDczbGdUZzFNbG1PdzJ1bzg1M09zcFdBRGh2ZjRrME5SWU5COGtvMnpaYjduNjl2TlFHOUNDQmVjODRXNGx1a0huVkl6VFJqYXJCc3B4d0ctNFMxMU5zLUl3dm1BYWh0RzE5OFV5VXM?oc=5</t>
         </is>
       </c>
-      <c r="E108" s="19" t="inlineStr">
+      <c r="E108" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3544,7 +3547,7 @@
       <c r="F108" s="3" t="inlineStr"/>
     </row>
     <row r="109">
-      <c r="A109" s="19" t="inlineStr">
+      <c r="A109" s="20" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
@@ -3554,17 +3557,17 @@
           <t>Why these people decided to vote for One Nation</t>
         </is>
       </c>
-      <c r="C109" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D109" s="19" t="inlineStr">
+      <c r="C109" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D109" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOQmNaOHZXWEEwZzRmdTBVT2FiS2hsYUhFczgxaFJaeEQzMGlfSnRoUWo0ZXl3cWhhbTU2NDRLUjh1c2Jxd3ZoR2pJOHVNemI2cTFrdU9oVkFCNXN4WV94TER4VmtIX1JCblhKNTl4VHlMdFBDRHVBUFhkS1AtR05RMG5QVGJFaTlWaVpMZERIa3Ntbmh0V0xnVVhYNDdMWWlpSWc?oc=5</t>
         </is>
       </c>
-      <c r="E109" s="19" t="inlineStr">
+      <c r="E109" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3572,7 +3575,7 @@
       <c r="F109" s="3" t="inlineStr"/>
     </row>
     <row r="110">
-      <c r="A110" s="19" t="inlineStr">
+      <c r="A110" s="20" t="inlineStr">
         <is>
           <t>2026-03-28</t>
         </is>
@@ -3582,17 +3585,17 @@
           <t>The Right Amount to Pay for Sushi</t>
         </is>
       </c>
-      <c r="C110" s="19" t="inlineStr">
+      <c r="C110" s="20" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="D110" s="19" t="inlineStr">
+      <c r="D110" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOLUljQ1FWeHk0N21FcnpCTzdNVW1WZmxfbDFucXRNYlBMSzR6aTh4WlNrdnFuT1VSWWpKWlJValZrbTE5RlllanJkcHNHeEVwVkxldnZSdjdLc2c1SHJTVG1hMHBKd2xtZXptV1FmcGZ0cXUwVXFMWjJiRFhhYTlKRkNBNHZQekVRcnRicXlNM2NQdXJaZkVRbTZta0hDRlV5YVN5NG9TYzltUFZucXNXc29Wc1Y?oc=5</t>
         </is>
       </c>
-      <c r="E110" s="19" t="inlineStr">
+      <c r="E110" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3600,7 +3603,7 @@
       <c r="F110" s="3" t="inlineStr"/>
     </row>
     <row r="111">
-      <c r="A111" s="19" t="inlineStr">
+      <c r="A111" s="20" t="inlineStr">
         <is>
           <t>2026-03-29</t>
         </is>
@@ -3610,17 +3613,17 @@
           <t>Blackstone-backed $2b Xpansiv kicks off raise</t>
         </is>
       </c>
-      <c r="C111" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D111" s="19" t="inlineStr">
+      <c r="C111" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D111" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOOGIxbEhpZjgwbk5XampWenBXbGZmbzFQbnJhUjU1Z2FtT1FGVk40SHExMUJBZHZoRDBRVXZHS3ZlR3o5RGU0c1o0Y0E2MXVKZ3U2ZFBBRm1NbVJPRk1pMGp3dV96ZTlMNERlMFBPRDNROXpNZlNmLV83VGV2QVNzWkhtV1kxY2x6TUQ3QkhlcVNPNTlyMUQ0?oc=5</t>
         </is>
       </c>
-      <c r="E111" s="19" t="inlineStr">
+      <c r="E111" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3628,7 +3631,7 @@
       <c r="F111" s="3" t="inlineStr"/>
     </row>
     <row r="112">
-      <c r="A112" s="19" t="inlineStr">
+      <c r="A112" s="20" t="inlineStr">
         <is>
           <t>2026-03-28</t>
         </is>
@@ -3638,17 +3641,17 @@
           <t>Elon Musk puts a $2.5 trillion rocket up Wall Street convention</t>
         </is>
       </c>
-      <c r="C112" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D112" s="19" t="inlineStr">
+      <c r="C112" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D112" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPeE52VS03NHBqZ3hvc1Q4V2laUElCcmxKem9SSzM0d1Uyd09ZSFl4SjZmUDl1Sl85WXp3TWtGX3hydFRwZG0xQmFlOVUtdEtaNmtYWFkzVDYyZGI0SWFZRWtYR2tGODdPVUNhLXBzVVpzYnVRYmZNZW8xbEpreGZMVzU5c1JrWDY1Nk9uWk53a3FCOHpQTDBCT0h6QllmbW1wc3FmVU4yTUlxSmRhTUdF?oc=5</t>
         </is>
       </c>
-      <c r="E112" s="19" t="inlineStr">
+      <c r="E112" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3656,7 +3659,7 @@
       <c r="F112" s="3" t="inlineStr"/>
     </row>
     <row r="113">
-      <c r="A113" s="19" t="inlineStr">
+      <c r="A113" s="20" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3666,17 +3669,17 @@
           <t>KMD Brands makes emergency capital raise, chairman David Kirk to exit</t>
         </is>
       </c>
-      <c r="C113" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D113" s="19" t="inlineStr">
+      <c r="C113" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D113" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNb1JhRUM4dDhXM1hoajdzQkNLQk12LURQbkp5LWdqQXpEczBxdVhySHphaUhiLVRiYVh1R25kbHRidy1TbjhCOEk0MXk5a2VWWlhHcUt5aXpfNjZWNnd6LVpQUkZNbFFXSWJHTmFaM2x2aS0tbG9TeXFxUWI1NF9uazJKa3BrZHFwclB1OVR3cWhXU2dJNFhaZmpVRVlwWUdiX2hrX0thQ3RDOWdFTF9BOGdHTG1JSlF6RVRZdnZn?oc=5</t>
         </is>
       </c>
-      <c r="E113" s="19" t="inlineStr">
+      <c r="E113" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3684,7 +3687,7 @@
       <c r="F113" s="3" t="inlineStr"/>
     </row>
     <row r="114">
-      <c r="A114" s="19" t="inlineStr">
+      <c r="A114" s="20" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3694,17 +3697,17 @@
           <t>RBA green lights credit card surcharge ban</t>
         </is>
       </c>
-      <c r="C114" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D114" s="19" t="inlineStr">
+      <c r="C114" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D114" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOcTB6SlhfdTQ5ZWdqNDExZVhOcVVybW5mbmxOVktCS3ljTndLY3ItWldSNDIyeEkwQmdBZ3p1X1o5S3ktZXI3MFM3eVkwWWc4cGtUTUw3aWM4azM3VGdrcGZjTjZMN1diWHZ0N3pna0tJZHZNU1FaN2VZbVNwMmozSFNBb253OUcya0duaEMtZnNQaFYwUFBhTGthaGhyTWY0NHpPTTFubmZOWEk?oc=5</t>
         </is>
       </c>
-      <c r="E114" s="19" t="inlineStr">
+      <c r="E114" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -3712,7 +3715,7 @@
       <c r="F114" s="3" t="inlineStr"/>
     </row>
     <row r="115">
-      <c r="A115" s="19" t="inlineStr">
+      <c r="A115" s="20" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3722,17 +3725,17 @@
           <t>Constellation Brands to acquire Hop Wtr, expanding non-alcoholic beverage portfolio</t>
         </is>
       </c>
-      <c r="C115" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D115" s="19" t="inlineStr">
+      <c r="C115" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D115" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPcjdPYWlEWWF6dkY2Y3RPWUh6M0pXYUw1NFNabUdXTS01TVBMWGtBMUpxTXFRekJINGNFOE5oVEI0WjR4Z2kzTUR6emJHUUYxWjA0MGVlWFNPR25xNmJJWkN2RHIzcWNxUHRFQXcwdWN5cHNZRVVYV3JTdXRJUFg1MWJKODNOdjJ5UEd4dWZEbVFyWlNaRkJPcnlyQW5janktSDVwYWRVRGJqTFdPTEdUSUFvRXI4QQ?oc=5</t>
         </is>
       </c>
-      <c r="E115" s="19" t="inlineStr">
+      <c r="E115" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3740,7 +3743,7 @@
       <c r="F115" s="3" t="inlineStr"/>
     </row>
     <row r="116">
-      <c r="A116" s="19" t="inlineStr">
+      <c r="A116" s="20" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3750,17 +3753,17 @@
           <t>David Jones races to secure $150m survival deal</t>
         </is>
       </c>
-      <c r="C116" s="19" t="inlineStr">
+      <c r="C116" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D116" s="19" t="inlineStr">
+      <c r="D116" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxONHp5S2RtcFJkYWVxakc1ZDE4UzZUVWlHSlBMTHJqVnVaRHJrcEwyV3BHWk9TdXdkOUlocWY2ZlN4NklobGVuYWhRc1BvdWppWlNFTm9wcGZoMG1UMEtjLS1scmx4cVNhNkZQYWw0M1VUQTJfOTJrYWMtTlpJYnl0N01QTWxZZDZPOEpfcTM1dFRVMDBTOEthcFU2Z0U4WFFBaE1GM2V6VHJVb2Z5ekxJWmUwQlphbXRlTS02NWNJV2p1Ym5Ca2JxNS0xQWZpbHJ4UFVtbDBCXy1IV2NXMlFOY25HSVkzTjYxbXZB0gHwAUFVX3lxTFBDVlc2X3JNcnNNWjlUV2RkeEdtSFBJRFNtTXVHcmZERW1vZURfeDFvRGo0b1Z5SlVOVGNJTXB4MVc3d3hWY3FVOENwbEJ1MERBalhlc2EwNnktcUprSjZQLUxNTVlqYzc0enZtQ0FOUFVTWHBCZVF1SWs2Y0ZKRllXblI4MVRrXzZUMHNicmxqeFhUUld4VzM0TGNtcl9fTG4wbEJPWDg4RWpjMUdHOUxlczdEend1MkZLRTZuUjdkV0xGRlR6RVlXdVUxdUhndmozTHNtT2czTjJzRUs0bFc2QnMxS0V1X3QwcjVNeGVjcQ?oc=5</t>
         </is>
       </c>
-      <c r="E116" s="19" t="inlineStr">
+      <c r="E116" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3768,7 +3771,7 @@
       <c r="F116" s="3" t="inlineStr"/>
     </row>
     <row r="117">
-      <c r="A117" s="19" t="inlineStr">
+      <c r="A117" s="20" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3778,17 +3781,17 @@
           <t>Newly listed Advanced Innergy targets smaller rival</t>
         </is>
       </c>
-      <c r="C117" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D117" s="19" t="inlineStr">
+      <c r="C117" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D117" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPamkyYnZfT0NwamdES3JPYklaaXFYdUp5cHJPOTZUNklqcUlral9ObHFPY1VROHJSdm1tOS1KZlZJWFA0Q1l2UUZhOThleHFsWDJTSVdTUnhlbE1OeVhBTXVQQjVIdHZHTFBHOUxGOGx3MWc1UmVIWUV6Q3RhTDR6WHRfRy05a25VX01lcWZOV3BWX1JyQVI0WlQ3dTQwNHhxWXJCQmV0VQ?oc=5</t>
         </is>
       </c>
-      <c r="E117" s="19" t="inlineStr">
+      <c r="E117" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3796,7 +3799,7 @@
       <c r="F117" s="3" t="inlineStr"/>
     </row>
     <row r="118">
-      <c r="A118" s="19" t="inlineStr">
+      <c r="A118" s="20" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3806,17 +3809,17 @@
           <t>Aussie eyewear giant’s costly $20k mistake</t>
         </is>
       </c>
-      <c r="C118" s="19" t="inlineStr">
+      <c r="C118" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D118" s="19" t="inlineStr">
+      <c r="D118" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAJBVV95cUxOTmtzblUxcW5WbDZLeEJXSWVuVW5qVzdpRkc1Rkoxc1pVT0FIaHdmR0p4ZzljcVpST2tHdTBwVEdqbmF2TVhlV0VaMDFiMVk2ZEZkUTZMNFQ1a1lUbWRCdGwySkJtbmRfTXFmUy1VVU1tU1dzMldON3lEUFVVVFI4T000b2NJLVhobDBBUzQyLTRGLXNPT3ptZ2tlUU8wNG5nNFAyUVo1elpTeDd1TW01YzB4eUI2eE9YQjZxNTJBSVpLYy0yR1BzSVFiWWxib1g0YmlzREFGTEV0bkRucmNLa3U4dXhkTC1aRkhnUHN1d0hjVUFuZFlWWG9xVUtMT0hKMjhmNkZzLWpMS2MzYWp1OVN0cV9IYnBRZG5OdWwwcErSAaYCQVVfeXFMTzBFMkJ2TU5EZGZYLVF5WHBJanYzeFJqS1owbk5EUUNOZFNiam5PcEZ1aDBFelJ5MjFzM0E0NlZRdGI4Rjdnb1RYVmVSN1Z1OWd1SFdweVB0ZEY5akVqOHBsTHpJaXZKNnhUMmd2YVVxTzUtUEJKcWpOY0VHeHlTbXNCbHFDdnlndzJFT2ZDcnlZWXYxNUFNekVUZWU1UTFnOXZXUERMWjdjYl9wVVl6OURodW1JSUI2ejJDTktfaTRCY2xEeHVBRW9tNmM3YXBHU201WXpHYjFYbU1sYnB1MjlLNjI0eTRWVElXU2ZqMDNNRW5LMVQyS2M5Z2tPSHJneGlkUkxFYXhDdWM1MGtkUUExT1hBSlU1ZkgtRlM4YnV3b1hkM2NR?oc=5</t>
         </is>
       </c>
-      <c r="E118" s="19" t="inlineStr">
+      <c r="E118" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3824,7 +3827,7 @@
       <c r="F118" s="3" t="inlineStr"/>
     </row>
     <row r="119">
-      <c r="A119" s="19" t="inlineStr">
+      <c r="A119" s="20" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3834,17 +3837,17 @@
           <t>Rio Tinto bankers up for infrastructure sale; eyes on Pilbara power</t>
         </is>
       </c>
-      <c r="C119" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D119" s="19" t="inlineStr">
+      <c r="C119" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D119" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPQTRxenprUFZmM2JIMDNPZGVVV09IakN5STI4ZFJVQmEtemVQUlJCRjdtbGpKWEZFOWVRd2ZYZk4xNkNHclpMSEFZLUpBVHhKaFN5Q0Y2bmhRWERpc2N4NEhua0VSQnFpVmpxa29tSlFNOHJRaFROMS1mTHBGdzZ6UlhLaVpqaUJhOEs3Y0Iyc29KY01XUXR3R1gwOXJHQUp2QVpNYi03NTZhLVgxN3VlODY4T0E?oc=5</t>
         </is>
       </c>
-      <c r="E119" s="19" t="inlineStr">
+      <c r="E119" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3852,7 +3855,7 @@
       <c r="F119" s="3" t="inlineStr"/>
     </row>
     <row r="120">
-      <c r="A120" s="19" t="inlineStr">
+      <c r="A120" s="20" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3862,17 +3865,17 @@
           <t>Luke’s Bánh Mí launches budget mini meal deal</t>
         </is>
       </c>
-      <c r="C120" s="19" t="inlineStr">
+      <c r="C120" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D120" s="19" t="inlineStr">
+      <c r="D120" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPQmh4NzlPa29pOXFmeTlKVFVUenNqdTF0VGU2REVwaWRsR3dKSEs3NFlTcGlscFRhRWRtV1JtVmFNTzJCb1d4d1NrUm9mMzBKcDBmM2JBbWZPTEVNdWZ1ZlVZZW93bW14Ull1UTNLUDh6WlZ2RUdBTS1NZEg2dmRZc3BEd2dfTFRFUERwdERnZnZwMFRR?oc=5</t>
         </is>
       </c>
-      <c r="E120" s="19" t="inlineStr">
+      <c r="E120" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3880,7 +3883,7 @@
       <c r="F120" s="3" t="inlineStr"/>
     </row>
     <row r="121">
-      <c r="A121" s="19" t="inlineStr">
+      <c r="A121" s="20" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3890,17 +3893,17 @@
           <t>Zeus Street Greek sets sights on drive-thru as next phase of growth</t>
         </is>
       </c>
-      <c r="C121" s="19" t="inlineStr">
+      <c r="C121" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D121" s="19" t="inlineStr">
+      <c r="D121" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNTEEzZ2VJMDdRek9JdGZCVVpJRGZoSjNIWjNiN3h2OHR2RjUwUG42SzViRUpteXRURFZzbFBpR0Q4TFdianc0SjZkc09DU01MY0hMLWRNbXQyYUVNai1BMUxFM0pZRWJaT0cwcmFna3pRS253R1FUY3UxOURmRkcwN3Fmd0VfLWVONzJJXzBzX1U5TFBQTFMtSURtZUV0TDhu?oc=5</t>
         </is>
       </c>
-      <c r="E121" s="19" t="inlineStr">
+      <c r="E121" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -3908,7 +3911,7 @@
       <c r="F121" s="3" t="inlineStr"/>
     </row>
     <row r="122">
-      <c r="A122" s="19" t="inlineStr">
+      <c r="A122" s="20" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3918,17 +3921,17 @@
           <t>From $5bn to $50bn: The end of an era at Blackstone</t>
         </is>
       </c>
-      <c r="C122" s="19" t="inlineStr">
+      <c r="C122" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D122" s="19" t="inlineStr">
+      <c r="D122" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijgJBVV95cUxQc251ZVp0SEY1TnpWc2g4WERmLU9INk5VTUJHa3RGWGRmbWYzLV9MQW9rZmQ3bjVTRVI3R3NDbVNPdW9GTksxNUdrdkk1eTk0VXNFZmR2V2FBQWtnZGRmZkVMbm5QTUo4dFUxSGlOS0FSRmZZcThBVnlqWTN0eEUwUjFPdjhFb29BTXFWTTdHODRYelQwWUNBbXdNOElkQ2UzRU51VjM3SC1HZmpEUlNJUFFKRmdPWnhqNlEtVkNUaUtCbEc3ZWo2NFVIVktNMTQyd21lekpHVjlXOGV5WEhIZWJrU0ZTTFlrSkZnYlUxOWdUYnhna2JZTlhGYlAwMmhDYlJfZ1o3bVVDTnppS1HSAZMCQVVfeXFMT2E5cHJhVE9FUlVLN3RPakxmMHZKN3JLVUEwM3FSdmlfR0o0X2tybDFQWTg3NmZsYkE5LVRjX1dQMHVhNHBXNkhVRl9kd3lGeFdIWUV2QVFyYVgzWXU1Z2dpLXd6OGtUR0Z5SkdZc2VVM0tDU2MydXZSbGZOZjhUOEg0YXlBN2EtVDk3Z2FUM3pGY2JkTXdGZ2I5U2otVkJ1S3NhTXRBVVNqS1FvYzdPeHdaY3dqNlJmdkhwWHZCdjVsMXNibEc3aDFBR3NkRkZpdVRzU3Nad3Y0N2gyaHRQWlY0cGV2SUh3T1NwdEJEZTh3T3laM1B6YXlzVHlRRXdHc09tOFVKUTFfYjU0aFpJMDRlSTQ?oc=5</t>
         </is>
       </c>
-      <c r="E122" s="19" t="inlineStr">
+      <c r="E122" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -3936,7 +3939,7 @@
       <c r="F122" s="3" t="inlineStr"/>
     </row>
     <row r="123">
-      <c r="A123" s="19" t="inlineStr">
+      <c r="A123" s="20" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -3946,17 +3949,17 @@
           <t>Starbucks opens first retail outlet at new Town Hall Station</t>
         </is>
       </c>
-      <c r="C123" s="19" t="inlineStr">
+      <c r="C123" s="20" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D123" s="19" t="inlineStr">
+      <c r="D123" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOTnJ1YVF6V1dqMm9HbmdUZEk3NlQtdjRxT28ya19fbjRKMlJRb3hsam5zdDg1cnEycHc4STRPdENPQnlMQldBbTh3NXlYb0tUNW9WS201NTZ0M0xvRE8zRkVYcFlNSmdOeVZvbXRMVzJMMkV6czFPX2djSFdKNlhWbUQtNUpMcnhFNnpfa1RPY3Q?oc=5</t>
         </is>
       </c>
-      <c r="E123" s="19" t="inlineStr">
+      <c r="E123" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -3964,7 +3967,7 @@
       <c r="F123" s="3" t="inlineStr"/>
     </row>
     <row r="124">
-      <c r="A124" s="19" t="inlineStr">
+      <c r="A124" s="20" t="inlineStr">
         <is>
           <t>2026-03-29</t>
         </is>
@@ -3974,17 +3977,17 @@
           <t>The ex-Platinum quant who has won billionaire Kerr Neilson’s backing</t>
         </is>
       </c>
-      <c r="C124" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D124" s="19" t="inlineStr">
+      <c r="C124" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D124" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNMkpmVTVUVU1WZUZiRWlJUkRId3BhS1hqM09aM0FSODBFNE96SDlKWG11Qkw2bjVSNFFrc0oyWHBBVXNYclBYQklIdnZBNEZ3b2NvZzdHZWNrV1JhbWI5aUpBLXRqTjIwSnhRSlFtdUlTU3VUbVMxcmtYZzlnVEsxellFb0dwb1hhME9QbERGcU9aXy1rOEtyQ0pXZW9KcENIem5TMjhUZ1VydFlrVWI3cWN6aGJROGFwWUFlNjQweTdqYkptcHc?oc=5</t>
         </is>
       </c>
-      <c r="E124" s="19" t="inlineStr">
+      <c r="E124" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -3992,7 +3995,7 @@
       <c r="F124" s="3" t="inlineStr"/>
     </row>
     <row r="125">
-      <c r="A125" s="19" t="inlineStr">
+      <c r="A125" s="20" t="inlineStr">
         <is>
           <t>2026-03-29</t>
         </is>
@@ -4002,17 +4005,17 @@
           <t>Media bosses: ‘Australia shouldn’t be held to ransom’ by AI giants</t>
         </is>
       </c>
-      <c r="C125" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D125" s="19" t="inlineStr">
+      <c r="C125" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D125" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPSGdRM3JDVld4OG5UWk5RdlVZVlU2LTFKUjdzVy1HejgyaUxMWHhmUlJnN1FrY2dSTTczczU0Tno2TUVPWDFiZk9TTjJTNlQ4Yi03MWpfdVEwWGFaQm9ydjJpaGFkekZHME1xNUswcWF4b2Y4TUxkOUpOa0dFTjlYVmhVMnFPMXlEcGJjeXZBR0tFaDZUa3Ixd1lIai1qcml5OE9SM1dTcUVkWW1HdFJTUFBJZUU0Nzg?oc=5</t>
         </is>
       </c>
-      <c r="E125" s="19" t="inlineStr">
+      <c r="E125" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -4020,7 +4023,7 @@
       <c r="F125" s="3" t="inlineStr"/>
     </row>
     <row r="126">
-      <c r="A126" s="19" t="inlineStr">
+      <c r="A126" s="20" t="inlineStr">
         <is>
           <t>2026-03-28</t>
         </is>
@@ -4030,17 +4033,17 @@
           <t>PLI scheme for food processing industries sees Rs 9,207 crore investment</t>
         </is>
       </c>
-      <c r="C126" s="19" t="inlineStr">
+      <c r="C126" s="20" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D126" s="19" t="inlineStr">
+      <c r="D126" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOcUwtamFxVTZ0YTdEOTBsN1gxNlphTV84aGJoRnFFTkFkZDhaT2VzVkFDT29hMU1Xa3BLeWFiRWlXT3Noc3VVVkg3WkphSFMwS3k2aWI4ZlhfcDN2LTV6Q3E0YnNXbEFVZFdUU3U0R293aEtlUmxlLXdFWXl5MHh0X2hWYnNvbU5MLUNCRm53aVpJa0E4OUxuNnN3X1FwUQ?oc=5</t>
         </is>
       </c>
-      <c r="E126" s="19" t="inlineStr">
+      <c r="E126" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -4048,7 +4051,7 @@
       <c r="F126" s="3" t="inlineStr"/>
     </row>
     <row r="127">
-      <c r="A127" s="19" t="inlineStr">
+      <c r="A127" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4058,17 +4061,17 @@
           <t>RBA’s surcharge hit on the banks may miss bigger picture</t>
         </is>
       </c>
-      <c r="C127" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D127" s="19" t="inlineStr">
+      <c r="C127" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D127" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOdWl1NWlxN0dzeEdzWThmcDVkNkpyYjJaNnZBa2dBSWhpaHhXRktTR2VtRzdUSnB3VGtDOTFuMTZXc2xycHFYN3dnQm9SaThYUURCSjg0dVlhLU52Vlo5VnRVNl9SSXFSbWFPeXdVRmdlUVA5S3FZQXc5d2lDY19UU2tJNGdrUzc0UXFHU3BGV0NHVldJcWxTS2Zydy16eHQ3QUlLQVdjWQ?oc=5</t>
         </is>
       </c>
-      <c r="E127" s="19" t="inlineStr">
+      <c r="E127" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -4076,7 +4079,7 @@
       <c r="F127" s="3" t="inlineStr"/>
     </row>
     <row r="128">
-      <c r="A128" s="19" t="inlineStr">
+      <c r="A128" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4086,17 +4089,17 @@
           <t>The six best new places to dine in Australia this month</t>
         </is>
       </c>
-      <c r="C128" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D128" s="19" t="inlineStr">
+      <c r="C128" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D128" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxObFAyUFZmNFk4LWJ3QzFDZnpZZlRNTEgzbGt1S1BOVF9qa2V4NnR0Yy1pX0RVUFlaUDg5bmV6LTZ2VExkWVpyZmRmV1dxNExoWkdvQzdzMTNuT0UxekhITmZBQmNhWENzV0lMYnE5all1Nk1CczFpRmhlN2pxenE1NGtLQzlKb21pSnljMlhHQjR5SVVxaG9wM01ndUdMOGpuWDduQ00waTF6OVpJUTdFV2ZWNm1yVjYzcnR3?oc=5</t>
         </is>
       </c>
-      <c r="E128" s="19" t="inlineStr">
+      <c r="E128" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -4104,7 +4107,7 @@
       <c r="F128" s="3" t="inlineStr"/>
     </row>
     <row r="129">
-      <c r="A129" s="19" t="inlineStr">
+      <c r="A129" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4114,17 +4117,17 @@
           <t>Mesabi Metallics secures 520 million dollars from Breakwall Capital</t>
         </is>
       </c>
-      <c r="C129" s="19" t="inlineStr">
+      <c r="C129" s="20" t="inlineStr">
         <is>
           <t>News.com.au</t>
         </is>
       </c>
-      <c r="D129" s="19" t="inlineStr">
+      <c r="D129" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNbVRfWlRYc2U4bV9WUVRxWmxpQWY3UTZyVGhGMGZtbEV5UXR2OTZJdGVYdFRUNzNtSUZEUVhwSzBDVWlmbWE5bTJsbDlBVXdZR0IxUHkzSDBXVkNiY3paYnlZWXBoUm1iam5oNUh5ejU2M3ZaaVhqTjV5SlpFd250Ym5HY0FvdEJvS1JvUnFRa1pmdFpKUV9OZg?oc=5</t>
         </is>
       </c>
-      <c r="E129" s="19" t="inlineStr">
+      <c r="E129" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -4132,7 +4135,7 @@
       <c r="F129" s="3" t="inlineStr"/>
     </row>
     <row r="130">
-      <c r="A130" s="19" t="inlineStr">
+      <c r="A130" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4142,17 +4145,17 @@
           <t>Fast food giant offloads Aussie stores in fire sale after costly flop</t>
         </is>
       </c>
-      <c r="C130" s="19" t="inlineStr">
+      <c r="C130" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D130" s="19" t="inlineStr">
+      <c r="D130" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimwJBVV95cUxNOXRhd0lOSkctZjVDaVRpcktmZzV1aEFJZGpsbHJHVU5Rdm9JM3U5Q3JBOEdFU2tMeDBnLUJ2WmxiOGZaRVF5RF8tS3R0R1dtQWFGaEJkbHV4VjdfSDRJSnFCYnQ2bXlhOE90N3V5THdCM1JnU0JjLU1Kb1U5YkxjU0N5bUpTYVJzX3l4X3ZHakpESmVrVWdWTk5RQlFZM1Awa25rWHVabzNlNWFqbENHdFhMX3hTWFBqNDlvVTJlcjlMeHRMWE8tRm1rTElTanB4RFl0THJTazJrVTdGYkh2OUxQaDdwSmx5bTkxNGJhQUIza1F1cjJCSGNQTDRDX3RaVzZBbDFhOXB5S0hSQ3U1ckVhRWNLUF9MVTA00gGgAkFVX3lxTE1RSE5Hb0FJRE1YWjRxa1RwZk5GUmhXa1MtcmM4NDB0ZWZxTWNtaEhDczZjZ1FUT0p2d2ZTcHZGd25vbC1mR2lGOF9NQnlGNEtWUFprdG5KM1hTRGFRb0VxdkxJU2E3NUFWLXBveUM2TktmeWRoSWlaaWpTbUFOSEVmZXJIQzFOVHNLUUVCSDgyLW8yWHRBN25vSkhYNy1vRnNOVkpXbXRQNVhpWXE0NVNTWjYxd2xXTGZqdWxWa0NsNHdLNEhMQTFNcFZzS0YyY0N3MDJhLUJKUGFVc05vQkZuUU5JUDhBazYzejVpYnZ3NjJzMEFPYVpDb3IzMzlLTWdNRFBscEVCQ1pDQTBoXzBfbnpuWTJTSmRNWnhiaExPeg?oc=5</t>
         </is>
       </c>
-      <c r="E130" s="19" t="inlineStr">
+      <c r="E130" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4160,7 +4163,7 @@
       <c r="F130" s="3" t="inlineStr"/>
     </row>
     <row r="131">
-      <c r="A131" s="19" t="inlineStr">
+      <c r="A131" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4170,17 +4173,17 @@
           <t>Young QSR workers stand to gain over junior pay rates abolishment</t>
         </is>
       </c>
-      <c r="C131" s="19" t="inlineStr">
+      <c r="C131" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D131" s="19" t="inlineStr">
+      <c r="D131" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNcXN5UDZ5d3h6NTd5YTdqUkM0dXBmdjZ0WlQ4YjF3QUxsTzdEZUVicTRweTJHYVVfYVFsQndwaURnWVBPYlJUdVRUUThQVG9jQkgzRVFyMEdBN053MDdBUmlKNHp3X0NmYVc1OFBGT2paSTZsNG5zdE9uNm1BVXd4TFEzVmgxMnJVRzFpclRlZndDTDMxU2djcGc2WVhWM2VkLW9NVkdTSnpQOHM?oc=5</t>
         </is>
       </c>
-      <c r="E131" s="19" t="inlineStr">
+      <c r="E131" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4188,7 +4191,7 @@
       <c r="F131" s="3" t="inlineStr"/>
     </row>
     <row r="132">
-      <c r="A132" s="19" t="inlineStr">
+      <c r="A132" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4198,17 +4201,17 @@
           <t>Bain presses ahead on Estia IPO, trade bids land in $2.2b-$2.7b range</t>
         </is>
       </c>
-      <c r="C132" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D132" s="19" t="inlineStr">
+      <c r="C132" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D132" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxONzVXcThuZjBBc3ZBQWg4bWU0Wmg0X3ZEdEZkeTFKa2U3RGRabC1Jem9nOGx4MWVwOFB2SFh6UjlIdVZuV2h4Zks0Y2pVV2pnVU9Rei1TX1Y4ZzVvVkh6MzRwTlZUS3NDZDNLZDVfZjB0NlRfTnBzWkFOSW5xbUc2bi01b2p1dHlaQ3pvZWV2YTR1dWdXZzZuX2FfM0pzSkxRck1OTEgydlB3SS1GTmpMZXhvMm4?oc=5</t>
         </is>
       </c>
-      <c r="E132" s="19" t="inlineStr">
+      <c r="E132" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -4216,7 +4219,7 @@
       <c r="F132" s="3" t="inlineStr"/>
     </row>
     <row r="133">
-      <c r="A133" s="19" t="inlineStr">
+      <c r="A133" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4226,17 +4229,17 @@
           <t>Challenger-backed emerging markets fund Ox Capital shuts its doors</t>
         </is>
       </c>
-      <c r="C133" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D133" s="19" t="inlineStr">
+      <c r="C133" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D133" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQalJpNmNjb1dtSDBtLTVEQjNodkJNTVdRNUhBVkxxR3lnQlhYSGY1YW1hdnZGTUhRRzR1QnhJN3pTdC1ablBwOWtydGZTLTNTaTJiZFFHanY3VTc2YTRqcDZUQTRvS21TNDF0YmljSzIxYkxxZzRMTHY0RzViWl9heS1xT2EzbUFmUkd0bHZkZzl4Zll4UzEwOHRhazgyWHN4VUw0WUFSLWRmLTJpZDltdjcyLXA?oc=5</t>
         </is>
       </c>
-      <c r="E133" s="19" t="inlineStr">
+      <c r="E133" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -4244,7 +4247,7 @@
       <c r="F133" s="3" t="inlineStr"/>
     </row>
     <row r="134">
-      <c r="A134" s="19" t="inlineStr">
+      <c r="A134" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4254,17 +4257,17 @@
           <t>Bosses send warning on 42pc junior pay spike</t>
         </is>
       </c>
-      <c r="C134" s="19" t="inlineStr">
+      <c r="C134" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D134" s="19" t="inlineStr">
+      <c r="D134" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxNaVJ0aGJ3RE9zNlVJSTVzZE1zMlpEbmpIWHpSVFVUQkNYZWJ3R3NCbjQyM1JWQV9sdUs3MVNkWnVqUnRUQjlQNmZoUkVjTHVTRENuQmxRS1NfRmd5MTM5VXMxWU5ST2M3ZjVkU2hKN3NINmhQWkJwMUZSenBnM1RselBCdVVabGNjandnV2NlTkc2SjJucUR4cjBFblNrSmlLRngzN3dlbnhTS1NkaS02R1Zwc1hrUHl6MHR0a2NkSy1XRm9hZ1B6bklHaTF6VVlmdzNaNDRWcFRXYXFDSnFpXzMxZDBZZEtORHZfckx1eEM4UdIB9wFBVV95cUxPeGhqYjFsazdhaENpSk1rY3lYM2lJSmVqSU5BX3Y4VTBsb2pBNWtqbHNqblpsNzduZktWNmxhZDJ1UTZxYnp0bWdqRFlkTEZ2aWJ5TmM3QWtEaGRhZUltcjgzVFFsaXQ5ajg0VmRmTFNXSlM5dHh3SHlsRWZOSzN4TkxUYnl2cXg3VHdTaEI0TklnTFBFVVVCRUhHRXgyR3l1bWpEeHZmQVBFM2Q4RnZoYzRiaTNYNUFBQm5XS25HcE1JRzJUT25sbXNrWGJEajBWSHJSOXlGMWFiWHJMb2pZWUFUUHJuZ2VKellQUHpEaEZKQjVYaHI0?oc=5</t>
         </is>
       </c>
-      <c r="E134" s="19" t="inlineStr">
+      <c r="E134" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -4272,7 +4275,7 @@
       <c r="F134" s="3" t="inlineStr"/>
     </row>
     <row r="135">
-      <c r="A135" s="19" t="inlineStr">
+      <c r="A135" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4282,17 +4285,17 @@
           <t>Justin Ryan’s Glow Capital cleans up with new investment</t>
         </is>
       </c>
-      <c r="C135" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D135" s="19" t="inlineStr">
+      <c r="C135" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D135" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPRWlpNFBQUTVzOE5yejU5a0tGcUN4ZHJieTV6S21BXzIwbGRmNXluSi0yVUlmaHp5Y1BaZG5CT2lVblktM3BvSDBDdEZ4d1pHLTI3NVRzeHNDdjl6Tm1tYUVLSkdoUlNidGhXUFpwVHNSRXZBOWZjVk85LXVHLWRRUUEtWDZ5Mld0T1ZPMEZoMi1hcHBWRGZJaDNJVDQ4RWkxVk9lR0JDSQ?oc=5</t>
         </is>
       </c>
-      <c r="E135" s="19" t="inlineStr">
+      <c r="E135" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -4300,7 +4303,7 @@
       <c r="F135" s="3" t="inlineStr"/>
     </row>
     <row r="136">
-      <c r="A136" s="19" t="inlineStr">
+      <c r="A136" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4310,17 +4313,17 @@
           <t>RBA crackdown on fee rort is a raid on banking’s hollow log</t>
         </is>
       </c>
-      <c r="C136" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D136" s="19" t="inlineStr">
+      <c r="C136" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D136" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQSHhSOWlMSVlkVlVaZnUwZjBzWHJxSUcyamI4ZjkxNWluOU1NUHA1RjJFdWZFaFBHTTRuRndCd0xabFJtclhZeTZ3bC1aRG5UREg5UVFyWDdIODhtV2JSdFV5R3hKZlZOc24xQlhGOWNJRXdFZl83TjU3emJ2YjZkVmFtSEpPSDBoRUNTc2JCZVNkZk1sWjI3RWo0SXZOY1dMU2xicndqVGdUOVk?oc=5</t>
         </is>
       </c>
-      <c r="E136" s="19" t="inlineStr">
+      <c r="E136" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -4328,7 +4331,7 @@
       <c r="F136" s="3" t="inlineStr"/>
     </row>
     <row r="137">
-      <c r="A137" s="19" t="inlineStr">
+      <c r="A137" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4338,17 +4341,17 @@
           <t>Inside Project Taronga: Koala’s choppy run to the ASX boards</t>
         </is>
       </c>
-      <c r="C137" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D137" s="19" t="inlineStr">
+      <c r="C137" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D137" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQeHotX0dQdVN6YWlES2twNXJaUUtzOEdESGJrbUdacmwxOHBDaXh6SVViWXJkMUloTGtpN3h2anNTMm1XWWVqSU5uaFlLdDZKaFV5d1BYZ3lXUE9NN0ZxN0hMWlBRejVlTUNwMUIwY0hGMmlVcnltR21GREw3ekNSSzJFUkI3ZWRINU9oOU5TRTdmRVp2MVpBQ0pPVzJHTi1ZZTFDSnBtSWwwWjRVQmpGT0N0NjlELUo5Slk5VTBYUTh0Zw?oc=5</t>
         </is>
       </c>
-      <c r="E137" s="19" t="inlineStr">
+      <c r="E137" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -4356,7 +4359,7 @@
       <c r="F137" s="3" t="inlineStr"/>
     </row>
     <row r="138">
-      <c r="A138" s="19" t="inlineStr">
+      <c r="A138" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4366,17 +4369,17 @@
           <t>Spotlight retail billionaires weigh up Barbeques Galore purchase</t>
         </is>
       </c>
-      <c r="C138" s="19" t="inlineStr">
+      <c r="C138" s="20" t="inlineStr">
         <is>
           <t>The Australian</t>
         </is>
       </c>
-      <c r="D138" s="19" t="inlineStr">
+      <c r="D138" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxNVk9feFNXOE1feC0wX1ZHaW16bUR1SUpKRWtjTHdfMDk3Y3J6WjFjNGdYcGdzbmk0c2N2b1N4cXhGVXEtU0hjYzMxRVlZT3FYMGZkend2OGg0VkpxdS1tNWM0RHRMNk5GbUJfVVVfc1NhTmFsNDlvMThjQk9PcTVnNTBUeUw4ZXNybW1ES0dXdlYyb291V280MTFCdlZMYVRIUVQ2dmUwblZjdnQ5N2pzLXMxOTcya0V4bFREM05PZkZZOHhuSTAzTFpxZUg4MmlUaDMzVHRROGQzUFkzVUFwZlZidGJhVXRTV2dPLdIB8gFBVV95cUxPRFBhdmluUkZtRldxd21BSmdkSWJsR2xNc1BYY0VGUjdVN3kweWM5WjR1VUhuRDNKYmNJellHQUl0cVJBd1o0QkdObW1PMzBTLUJmdXBlQnNJcGx5Qk1DVndrSHhzR0E0ZVRsN2t5M0ZqV3ZJUVhLdkN2d0I1VkVHZkpVQ3dNTGZLWUV2RU9tbXRvRHhDMmZzRk9fWktodmYxckZXU0dTcWg4X3M5WFJ6OTBYbjdyd1BxRnBia3RuMWJNOWE1M0Nla29hMGVPRExQWW02TWhfbXRlZkxmZ0tYS0tldDdLM3ZCU2s5UVEzNVN5QQ?oc=5</t>
         </is>
       </c>
-      <c r="E138" s="19" t="inlineStr">
+      <c r="E138" s="20" t="inlineStr">
         <is>
           <t>Food &amp; Beverage</t>
         </is>
@@ -4384,7 +4387,7 @@
       <c r="F138" s="3" t="inlineStr"/>
     </row>
     <row r="139">
-      <c r="A139" s="19" t="inlineStr">
+      <c r="A139" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4394,17 +4397,17 @@
           <t>Chargrill Charlie’s opens in Redfern</t>
         </is>
       </c>
-      <c r="C139" s="19" t="inlineStr">
+      <c r="C139" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D139" s="19" t="inlineStr">
+      <c r="D139" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxOalVFNURyb3NER1J2SVpsazF0S195WUpTdFcwaHhvNG9Dblc3MEw5SS0yakJiaDJLeDRZLVBSZmw5SjdkOVpEeWFmaTN4Rnl2SkdJbHBDU2VXdjA3Sm9JU2drXzNxOU5sZER6eGp6MmljX2RMWmM0VjNXeVZsWFpqYW53?oc=5</t>
         </is>
       </c>
-      <c r="E139" s="19" t="inlineStr">
+      <c r="E139" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4412,7 +4415,7 @@
       <c r="F139" s="3" t="inlineStr"/>
     </row>
     <row r="140">
-      <c r="A140" s="19" t="inlineStr">
+      <c r="A140" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4422,17 +4425,17 @@
           <t>Former KFC exec named new CMO of Pizza Hut Australia</t>
         </is>
       </c>
-      <c r="C140" s="19" t="inlineStr">
+      <c r="C140" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D140" s="19" t="inlineStr">
+      <c r="D140" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPaDJEelhoN2tnME1SazlhTTZpOVhaWnFnN3ozUTFkZmZ4LTFXdGtQSWZVcUN4aVdhSERUSFY5NDl3X2QtUDRjNWx0WElXV1M1bTVnNWRrMURkMFlwQmljMkRlc0tnbHVzZkdha21YNWFlWC1JX1dHX0hCYi1PRGFoVDdxWDk1OGtUeXI4RkMtbXUyUVdWbHlmbGN3?oc=5</t>
         </is>
       </c>
-      <c r="E140" s="19" t="inlineStr">
+      <c r="E140" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4440,7 +4443,7 @@
       <c r="F140" s="3" t="inlineStr"/>
     </row>
     <row r="141">
-      <c r="A141" s="19" t="inlineStr">
+      <c r="A141" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4450,17 +4453,17 @@
           <t>Restaurant Brands New Zealand snaps up Taco Bell franchise from Collins Foods</t>
         </is>
       </c>
-      <c r="C141" s="19" t="inlineStr">
+      <c r="C141" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D141" s="19" t="inlineStr">
+      <c r="D141" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNak9JTVQ3ZUFpN3BYU3U3d1FwdVAwU3V6Z3VxREhqX2h3Q0tFalhDMHpqWFpfcUxuc3NMSjBsRi1QR21oNmg2NUt4dHFPV3ZDNjE1N01yT2JuSFBjU2dGeFl5SjVmSEZtSlpfZHVtTThTZmxrLWttZGxYZURvOTBRcjRMRVFIV08xUU1PUXNSMHJ3MV9LSVBMSzVIX1RkRFhZa1Q5cG12eWVJT1dCT3Nr?oc=5</t>
         </is>
       </c>
-      <c r="E141" s="19" t="inlineStr">
+      <c r="E141" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4468,7 +4471,7 @@
       <c r="F141" s="3" t="inlineStr"/>
     </row>
     <row r="142">
-      <c r="A142" s="19" t="inlineStr">
+      <c r="A142" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4478,17 +4481,17 @@
           <t>Gelatissimo hits 60 outlets with Zetland opening</t>
         </is>
       </c>
-      <c r="C142" s="19" t="inlineStr">
+      <c r="C142" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D142" s="19" t="inlineStr">
+      <c r="D142" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxObVNNeU1EalQtaFRrbVIzdGRDcjIwampSckY5VlM4RzF1aXpmX3hweTFucmpxQ3gxUFhGZmVrck5GTzNyb3VxR1gtRVBwbXRVaFE5REJ3UWQ4U3hqd1RFU05kcVA5ZlVEUG80cUU1a1U0VWNtMXp2QmkzZ3F5X01pcEt5WkxvLUg2UTFzTw?oc=5</t>
         </is>
       </c>
-      <c r="E142" s="19" t="inlineStr">
+      <c r="E142" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4496,7 +4499,7 @@
       <c r="F142" s="3" t="inlineStr"/>
     </row>
     <row r="143">
-      <c r="A143" s="19" t="inlineStr">
+      <c r="A143" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4506,17 +4509,17 @@
           <t>Investors flock to Koala as furniture retailer soars on ASX debut</t>
         </is>
       </c>
-      <c r="C143" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D143" s="19" t="inlineStr">
+      <c r="C143" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D143" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOWHFPQVY5MGg5dzRzeDNQVG5PM204dkUyQWtYNTVGQWpIY0NFWTUzTFZMV3VuV2FWTWZqSVpldmdNY0YzU2VTX2c5eXUtajJPWXJmSm5iRlRleWNRMVhmZUJxaXNDNENMNGV0RmZWNEkxTWZPTE95VGtDYWhwSzZGZzBNbGZ4OXZBM2FxbElnTU14WnpVbUhyYTJGaGZHdjd0Yk0tRDlacno?oc=5</t>
         </is>
       </c>
-      <c r="E143" s="19" t="inlineStr">
+      <c r="E143" s="20" t="inlineStr">
         <is>
           <t>Retail &amp; Consumer</t>
         </is>
@@ -4524,7 +4527,7 @@
       <c r="F143" s="3" t="inlineStr"/>
     </row>
     <row r="144">
-      <c r="A144" s="19" t="inlineStr">
+      <c r="A144" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4534,17 +4537,17 @@
           <t>Australia's Collins Foods to transfer 20 Taco Bell outlets to Yum Brands</t>
         </is>
       </c>
-      <c r="C144" s="19" t="inlineStr">
+      <c r="C144" s="20" t="inlineStr">
         <is>
           <t>Reuters</t>
         </is>
       </c>
-      <c r="D144" s="19" t="inlineStr">
+      <c r="D144" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOWnNHb0VCMjhOUTNrUS1WOUhmRlpnelpxMmtFZmxGY1poSzB4dHFWcjdNN3lWcVhyWUpSU1UwSjhpY2dUNlg1N1hQQ1pRVUFKcm5MSHV0TWYwSmtqTHF4a1FQX1MtdmhqUV8tZ1lJcC11c2J3TXJWWG5mVmtSUkFWTDBZaXc4QVcxeGhxeHVBQVJ4TVJ1Sm5scHlmNTFsSzJWcktEekp0dk1QeFJSdnVpd2Mtdklya3ZiQmJodw?oc=5</t>
         </is>
       </c>
-      <c r="E144" s="19" t="inlineStr">
+      <c r="E144" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4552,7 +4555,7 @@
       <c r="F144" s="3" t="inlineStr"/>
     </row>
     <row r="145">
-      <c r="A145" s="19" t="inlineStr">
+      <c r="A145" s="20" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
@@ -4562,17 +4565,17 @@
           <t>KFC operator Collins Foods offloads Taco Bell outlets</t>
         </is>
       </c>
-      <c r="C145" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D145" s="19" t="inlineStr">
+      <c r="C145" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D145" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQV2x0VTJWLWNLcGlYWDZCc1NpbTd3MnlvX09kMWpIeS1jMGQ0OF9sc0k2RHZFY0JudmVJdVJtNnF1Zk5vYTRDNG1aNDlVQmZMM0RLRFZWZFR6bUhJQVZlc1hDY2NCbDJVMzBCMVF0ZlhvNEpVOHNUV0Uyb0hCQU1ndzN5Vk5pMFlSQWxXaktmdTQycVctTGx2dGV1Um5ycDFFWmVkQ2puLWlTZw?oc=5</t>
         </is>
       </c>
-      <c r="E145" s="19" t="inlineStr">
+      <c r="E145" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4580,7 +4583,7 @@
       <c r="F145" s="3" t="inlineStr"/>
     </row>
     <row r="146">
-      <c r="A146" s="19" t="inlineStr">
+      <c r="A146" s="20" t="inlineStr">
         <is>
           <t>2026-03-30</t>
         </is>
@@ -4590,17 +4593,17 @@
           <t>Count launches $40m capital raising for financial planning acquisition</t>
         </is>
       </c>
-      <c r="C146" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D146" s="19" t="inlineStr">
+      <c r="C146" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D146" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQQl9MSkpfamt1UUxyeTVILVlKSThwOXVrUmxfdF9nMVIySC1pc3RLNXB0c1Y2X2ZRakw4dS1FLVB3YlJlQ1BkcXBRUGc1NXNKS0lMblVpQVhsZWZlNTdPRXFQMzdyUDNtTjlkeHQyRkdXaUtiQzZUVHpPV3p3a3hqYVdTaU1CdWFvYmhiTmhBeFVwZlozQjJnWHl3NTYzYTlTbkgxUi1OYXlLcS13eG05ZnBsQUthQ0E0?oc=5</t>
         </is>
       </c>
-      <c r="E146" s="19" t="inlineStr">
+      <c r="E146" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -4608,7 +4611,7 @@
       <c r="F146" s="3" t="inlineStr"/>
     </row>
     <row r="147">
-      <c r="A147" s="19" t="inlineStr">
+      <c r="A147" s="20" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
@@ -4618,17 +4621,17 @@
           <t>Inside the AI-fuelled fraud that deceived Australia’s biggest bank</t>
         </is>
       </c>
-      <c r="C147" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D147" s="19" t="inlineStr">
+      <c r="C147" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D147" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxPZWdmQklwRGlvLXBrbzVlNHVJZlJEVWMyWmVDUFd0eVFZNW91dUtBRXB6Q0s1bGpkTDZkUEpaTnNBZjhpTTBaTFRDc2NLb3JaVFNkUnVUd0NZQy1zVVN4WGxmbkFBQ1l5ZWFrUDJnejZRTXRhR3k4TGVXQy1TaFVLNlUyaWU3ZlhHMlhBdFJmQy1JdkRLSjlDWndWNEZpeW9QVEVpSGFWOXNKMW94ZUpRbWF6TFMxS3Vxd2M4QlBBYUNfMGJRVzNWa3lZYw?oc=5</t>
         </is>
       </c>
-      <c r="E147" s="19" t="inlineStr">
+      <c r="E147" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -4636,7 +4639,7 @@
       <c r="F147" s="3" t="inlineStr"/>
     </row>
     <row r="148">
-      <c r="A148" s="19" t="inlineStr">
+      <c r="A148" s="20" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
@@ -4646,17 +4649,17 @@
           <t>Meet the winners of the Best Places to Work awards</t>
         </is>
       </c>
-      <c r="C148" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D148" s="19" t="inlineStr">
+      <c r="C148" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D148" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQQTYweEJveHFxWlZVUm5QUVQxOVU2QW15N0EwOW9aOEpXNGJ1TWExVUZpV25IMFVMVVRQTFlzYTlhN1NGM05JRDJCUmN1SVF4T0dmRGV5ZlRHdGY3bDA1Nzk3aWQwOFVwY3lRQjJvWUU2ZWtSZzQ3SWljVy04VW9FM3RGQWk1NmIxSUFGcS1paGJFQ0d3QW5ZWmJjRXZsakF3alNOTmItbXFFNHBsYk1zZkhNdw?oc=5</t>
         </is>
       </c>
-      <c r="E148" s="19" t="inlineStr">
+      <c r="E148" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -4664,7 +4667,7 @@
       <c r="F148" s="3" t="inlineStr"/>
     </row>
     <row r="149">
-      <c r="A149" s="19" t="inlineStr">
+      <c r="A149" s="20" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
@@ -4674,17 +4677,17 @@
           <t>Healthscope landlords offer break-up deal with private equity</t>
         </is>
       </c>
-      <c r="C149" s="19" t="inlineStr">
+      <c r="C149" s="20" t="inlineStr">
         <is>
           <t>SMH</t>
         </is>
       </c>
-      <c r="D149" s="19" t="inlineStr">
+      <c r="D149" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNSEdKYllEUEZ0ME5KNkh4aUoyVUdudm9ROFJ2RDVuUGRNS3EtdnZVbXpJeGxFMklrYmhaTEVlUzh3cVhyTERCVDlSZGVkckg5cHNDRDl2VmYwNW5SZnZwbXVHbkpqSFZXU3luSkcySl8tUlZLODRFM05mRU5mdENUcE1SenlLVDFsYzVGYkUxR3lNcHBpdTd4MVJwcXU2M25GVkN3VzdvM3FadWNCT2lYVkN2WHlqa2dLU0oxWjBsWnFSZw?oc=5</t>
         </is>
       </c>
-      <c r="E149" s="19" t="inlineStr">
+      <c r="E149" s="20" t="inlineStr">
         <is>
           <t>Private Equity &amp; M&amp;A</t>
         </is>
@@ -4692,7 +4695,7 @@
       <c r="F149" s="3" t="inlineStr"/>
     </row>
     <row r="150">
-      <c r="A150" s="19" t="inlineStr">
+      <c r="A150" s="20" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
@@ -4702,17 +4705,17 @@
           <t>TPG NewQuest gets its paws on Pemba’s Vets Central continuation fund</t>
         </is>
       </c>
-      <c r="C150" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D150" s="19" t="inlineStr">
+      <c r="C150" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D150" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNN3FVaGNQYzBnU3ZHWG9oN19YY3BERTdYcUZROEd1dVYyMWViYkpGMkpxNm5qQjViWHpWWS1wU3dFbFNWMzhUbFIzUDU1Z1puY21lRWN5VGl6cUVlMnBjb3hlYXA1QWcwaVhXZDVXbW4xTHpiUTluSmNNOEVzMUF1Mm5pVXRPRTVyZlRETnFGSzJqTFJWQXVmOVlrUUZ2aUdWSWFVNWNqcnFTcnRyT2UxYVF3?oc=5</t>
         </is>
       </c>
-      <c r="E150" s="19" t="inlineStr">
+      <c r="E150" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -4720,7 +4723,7 @@
       <c r="F150" s="3" t="inlineStr"/>
     </row>
     <row r="151">
-      <c r="A151" s="19" t="inlineStr">
+      <c r="A151" s="20" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
@@ -4730,17 +4733,17 @@
           <t>Sushi Express Singapore launches limited-time collaborations with The Powerpuff Girls</t>
         </is>
       </c>
-      <c r="C151" s="19" t="inlineStr">
+      <c r="C151" s="20" t="inlineStr">
         <is>
           <t>QSR Media</t>
         </is>
       </c>
-      <c r="D151" s="19" t="inlineStr">
+      <c r="D151" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQOHpNQ1NrdkFiNng1bV9lNVQ4WWxUOGVTQUpnMUVoMWsySmVTRXFGMXo2SEVFUzVJd3Vid3YtZ2VIb1dycEJwR0tGcGJ1ZEg2YkdUNkJQN1BMT1Utd2hpcEswbFhxYlJfUDhVSl96TjRLWnR2Z0JRbERJelZtZGlEUmFabkhHYTU3UVR6WVRFNXVHdmN0LTRIY0FjaVJjV0RTcUN4Ui12UUR1TUJMU3B0dE14MA?oc=5</t>
         </is>
       </c>
-      <c r="E151" s="19" t="inlineStr">
+      <c r="E151" s="20" t="inlineStr">
         <is>
           <t>QSR &amp; Franchising</t>
         </is>
@@ -4748,7 +4751,7 @@
       <c r="F151" s="3" t="inlineStr"/>
     </row>
     <row r="152">
-      <c r="A152" s="19" t="inlineStr">
+      <c r="A152" s="20" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
@@ -4758,17 +4761,17 @@
           <t>Stocks are surging in early signs of huge short squeeze</t>
         </is>
       </c>
-      <c r="C152" s="19" t="inlineStr">
-        <is>
-          <t>AFR</t>
-        </is>
-      </c>
-      <c r="D152" s="19" t="inlineStr">
+      <c r="C152" s="20" t="inlineStr">
+        <is>
+          <t>AFR</t>
+        </is>
+      </c>
+      <c r="D152" s="20" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNRGFlZ2RyZ1Rla3ZZYzVVVkx0Q1ZtUHp2aldyQVJDZEVDWnY3V1dDYUhHMEtYN2dQck9sNEpQd2tOc2tkc3VaSjJIWmV4VXhoYTE3RkxSTFRGUDluSUVTbTRORkJrN0VlX3Z6d2VINVlyVDZhNkFteVJkYnZyci1oa1J4bW9ZN3BJZ2pzajVPdU0yOHUtdkxqdWpFUU9xWWVrMHBxTlRjdThCTHlaaUdON2Rua2txQlZn?oc=5</t>
         </is>
       </c>
-      <c r="E152" s="19" t="inlineStr">
+      <c r="E152" s="20" t="inlineStr">
         <is>
           <t>Australian Economy &amp; Markets</t>
         </is>
@@ -4858,6 +4861,34 @@
         </is>
       </c>
       <c r="F155" s="3" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>Bain Capital’s Managing Partner on Private Credit, Alts, and More</t>
+        </is>
+      </c>
+      <c r="C156" s="21" t="inlineStr">
+        <is>
+          <t>The Australian</t>
+        </is>
+      </c>
+      <c r="D156" s="21" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxQWFRCSzhzdi1SS19NLUVJcDB6ejhUR1pxY0wxVEI2dHRQdmxlbVpiX01PMmZiNm1JOFc3NUg4TmRwSG9VNHBrMlROZmVfa3VCYUJtZTlSbFViZldzcWE0dS1wRlV1X2lCUEpNVWtPU081RmpBdnQwRUhKQ0cwN1JLdm12NVlsZTJYZl9iX3pfZVFTMkNGYXU1NVNRMWNYZ2dwUTdmaXNSWk5UeEpZY2pGSUdBczVNRHBES0t1V0VjSGZXQTlfajhTMDZObHdMVnNFUjVqN2VnUUFTcjFoR2piQtIB4AFBVV95cUxQWFRCSzhzdi1SS19NLUVJcDB6ejhUR1pxY0wxVEI2dHRQdmxlbVpiX01PMmZiNm1JOFc3NUg4TmRwSG9VNHBrMlROZmVfa3VCYUJtZTlSbFViZldzcWE0dS1wRlV1X2lCUEpNVWtPU081RmpBdnQwRUhKQ0cwN1JLdm12NVlsZTJYZl9iX3pfZVFTMkNGYXU1NVNRMWNYZ2dwUTdmaXNSWk5UeEpZY2pGSUdBczVNRHBES0t1V0VjSGZXQTlfajhTMDZObHdMVnNFUjVqN2VnUUFTcjFoR2piQg?oc=5</t>
+        </is>
+      </c>
+      <c r="E156" s="21" t="inlineStr">
+        <is>
+          <t>Private Equity &amp; M&amp;A</t>
+        </is>
+      </c>
+      <c r="F156" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>

</xml_diff>